<commit_message>
Data update — 2026-09-14 candle + results refresh
</commit_message>
<xml_diff>
--- a/results/strategy_pnl_simple.xlsx
+++ b/results/strategy_pnl_simple.xlsx
@@ -1473,7 +1473,7 @@
         <v/>
       </c>
       <c r="J4" s="4" t="n">
-        <v>571.8200000000001</v>
+        <v>571.8</v>
       </c>
       <c r="K4" s="21">
         <f>IF(OR($B4="",$I4=""),"",$I4-IF($J4="",0,$J4))</f>
@@ -1524,7 +1524,7 @@
         <v/>
       </c>
       <c r="J5" s="4" t="n">
-        <v>688.91</v>
+        <v>688.92</v>
       </c>
       <c r="K5" s="21">
         <f>IF(OR($B5="",$I5=""),"",$I5-IF($J5="",0,$J5))</f>
@@ -1575,7 +1575,7 @@
         <v/>
       </c>
       <c r="J6" s="4" t="n">
-        <v>570.67</v>
+        <v>570.65</v>
       </c>
       <c r="K6" s="21">
         <f>IF(OR($B6="",$I6=""),"",$I6-IF($J6="",0,$J6))</f>
@@ -1626,7 +1626,7 @@
         <v/>
       </c>
       <c r="J7" s="4" t="n">
-        <v>663.08</v>
+        <v>663.05</v>
       </c>
       <c r="K7" s="21">
         <f>IF(OR($B7="",$I7=""),"",$I7-IF($J7="",0,$J7))</f>
@@ -1677,7 +1677,7 @@
         <v/>
       </c>
       <c r="J8" s="4" t="n">
-        <v>590.67</v>
+        <v>590.75</v>
       </c>
       <c r="K8" s="21">
         <f>IF(OR($B8="",$I8=""),"",$I8-IF($J8="",0,$J8))</f>
@@ -1779,7 +1779,7 @@
         <v/>
       </c>
       <c r="J10" s="4" t="n">
-        <v>398.64</v>
+        <v>398.62</v>
       </c>
       <c r="K10" s="21">
         <f>IF(OR($B10="",$I10=""),"",$I10-IF($J10="",0,$J10))</f>
@@ -1881,7 +1881,7 @@
         <v/>
       </c>
       <c r="J12" s="4" t="n">
-        <v>414.18</v>
+        <v>414.17</v>
       </c>
       <c r="K12" s="21">
         <f>IF(OR($B12="",$I12=""),"",$I12-IF($J12="",0,$J12))</f>
@@ -1932,7 +1932,7 @@
         <v/>
       </c>
       <c r="J13" s="4" t="n">
-        <v>345.09</v>
+        <v>345.08</v>
       </c>
       <c r="K13" s="21">
         <f>IF(OR($B13="",$I13=""),"",$I13-IF($J13="",0,$J13))</f>
@@ -1983,7 +1983,7 @@
         <v/>
       </c>
       <c r="J14" s="4" t="n">
-        <v>414.51</v>
+        <v>414.5</v>
       </c>
       <c r="K14" s="21">
         <f>IF(OR($B14="",$I14=""),"",$I14-IF($J14="",0,$J14))</f>
@@ -2034,7 +2034,7 @@
         <v/>
       </c>
       <c r="J15" s="4" t="n">
-        <v>380.28</v>
+        <v>380.31</v>
       </c>
       <c r="K15" s="21">
         <f>IF(OR($B15="",$I15=""),"",$I15-IF($J15="",0,$J15))</f>
@@ -2187,7 +2187,7 @@
         <v/>
       </c>
       <c r="J18" s="4" t="n">
-        <v>413.94</v>
+        <v>413.93</v>
       </c>
       <c r="K18" s="21">
         <f>IF(OR($B18="",$I18=""),"",$I18-IF($J18="",0,$J18))</f>
@@ -2238,7 +2238,7 @@
         <v/>
       </c>
       <c r="J19" s="4" t="n">
-        <v>406.47</v>
+        <v>406.46</v>
       </c>
       <c r="K19" s="21">
         <f>IF(OR($B19="",$I19=""),"",$I19-IF($J19="",0,$J19))</f>
@@ -2697,7 +2697,7 @@
         <v/>
       </c>
       <c r="J28" s="4" t="n">
-        <v>870.3200000000001</v>
+        <v>870.51</v>
       </c>
       <c r="K28" s="21">
         <f>IF(OR($B28="",$I28=""),"",$I28-IF($J28="",0,$J28))</f>
@@ -2850,7 +2850,7 @@
         <v/>
       </c>
       <c r="J31" s="4" t="n">
-        <v>391.16</v>
+        <v>391.15</v>
       </c>
       <c r="K31" s="21">
         <f>IF(OR($B31="",$I31=""),"",$I31-IF($J31="",0,$J31))</f>
@@ -2901,7 +2901,7 @@
         <v/>
       </c>
       <c r="J32" s="4" t="n">
-        <v>349.78</v>
+        <v>349.77</v>
       </c>
       <c r="K32" s="21">
         <f>IF(OR($B32="",$I32=""),"",$I32-IF($J32="",0,$J32))</f>
@@ -3003,7 +3003,7 @@
         <v/>
       </c>
       <c r="J34" s="4" t="n">
-        <v>349.89</v>
+        <v>349.93</v>
       </c>
       <c r="K34" s="21">
         <f>IF(OR($B34="",$I34=""),"",$I34-IF($J34="",0,$J34))</f>
@@ -3054,7 +3054,7 @@
         <v/>
       </c>
       <c r="J35" s="4" t="n">
-        <v>386.38</v>
+        <v>386.08</v>
       </c>
       <c r="K35" s="21">
         <f>IF(OR($B35="",$I35=""),"",$I35-IF($J35="",0,$J35))</f>
@@ -3564,7 +3564,7 @@
         <v/>
       </c>
       <c r="J45" s="4" t="n">
-        <v>599.6900000000001</v>
+        <v>599.6799999999999</v>
       </c>
       <c r="K45" s="21">
         <f>IF(OR($B45="",$I45=""),"",$I45-IF($J45="",0,$J45))</f>
@@ -3615,7 +3615,7 @@
         <v/>
       </c>
       <c r="J46" s="4" t="n">
-        <v>600.8</v>
+        <v>600.78</v>
       </c>
       <c r="K46" s="21">
         <f>IF(OR($B46="",$I46=""),"",$I46-IF($J46="",0,$J46))</f>
@@ -3666,7 +3666,7 @@
         <v/>
       </c>
       <c r="J47" s="4" t="n">
-        <v>678.54</v>
+        <v>678.63</v>
       </c>
       <c r="K47" s="21">
         <f>IF(OR($B47="",$I47=""),"",$I47-IF($J47="",0,$J47))</f>
@@ -3717,7 +3717,7 @@
         <v/>
       </c>
       <c r="J48" s="4" t="n">
-        <v>672.47</v>
+        <v>672.62</v>
       </c>
       <c r="K48" s="21">
         <f>IF(OR($B48="",$I48=""),"",$I48-IF($J48="",0,$J48))</f>
@@ -3768,7 +3768,7 @@
         <v/>
       </c>
       <c r="J49" s="4" t="n">
-        <v>538.67</v>
+        <v>538.66</v>
       </c>
       <c r="K49" s="21">
         <f>IF(OR($B49="",$I49=""),"",$I49-IF($J49="",0,$J49))</f>
@@ -3819,7 +3819,7 @@
         <v/>
       </c>
       <c r="J50" s="4" t="n">
-        <v>627.83</v>
+        <v>627.89</v>
       </c>
       <c r="K50" s="21">
         <f>IF(OR($B50="",$I50=""),"",$I50-IF($J50="",0,$J50))</f>
@@ -4023,7 +4023,7 @@
         <v/>
       </c>
       <c r="J54" s="4" t="n">
-        <v>619.1</v>
+        <v>619.12</v>
       </c>
       <c r="K54" s="21">
         <f>IF(OR($B54="",$I54=""),"",$I54-IF($J54="",0,$J54))</f>
@@ -4431,7 +4431,7 @@
         <v/>
       </c>
       <c r="J62" s="4" t="n">
-        <v>615.86</v>
+        <v>615.91</v>
       </c>
       <c r="K62" s="21">
         <f>IF(OR($B62="",$I62=""),"",$I62-IF($J62="",0,$J62))</f>
@@ -4533,7 +4533,7 @@
         <v/>
       </c>
       <c r="J64" s="4" t="n">
-        <v>440.62</v>
+        <v>440.52</v>
       </c>
       <c r="K64" s="21">
         <f>IF(OR($B64="",$I64=""),"",$I64-IF($J64="",0,$J64))</f>
@@ -5196,7 +5196,7 @@
         <v/>
       </c>
       <c r="J77" s="4" t="n">
-        <v>375.06</v>
+        <v>375.07</v>
       </c>
       <c r="K77" s="21">
         <f>IF(OR($B77="",$I77=""),"",$I77-IF($J77="",0,$J77))</f>
@@ -7185,7 +7185,7 @@
         <v/>
       </c>
       <c r="J116" s="4" t="n">
-        <v>394.17</v>
+        <v>394.18</v>
       </c>
       <c r="K116" s="21">
         <f>IF(OR($B116="",$I116=""),"",$I116-IF($J116="",0,$J116))</f>
@@ -7389,7 +7389,7 @@
         <v/>
       </c>
       <c r="J120" s="4" t="n">
-        <v>391.34</v>
+        <v>391.36</v>
       </c>
       <c r="K120" s="21">
         <f>IF(OR($B120="",$I120=""),"",$I120-IF($J120="",0,$J120))</f>
@@ -7746,7 +7746,7 @@
         <v/>
       </c>
       <c r="J127" s="4" t="n">
-        <v>814.21</v>
+        <v>587.9400000000001</v>
       </c>
       <c r="K127" s="21">
         <f>IF(OR($B127="",$I127=""),"",$I127-IF($J127="",0,$J127))</f>
@@ -7848,7 +7848,7 @@
         <v/>
       </c>
       <c r="J129" s="4" t="n">
-        <v>801.76</v>
+        <v>583.85</v>
       </c>
       <c r="K129" s="21">
         <f>IF(OR($B129="",$I129=""),"",$I129-IF($J129="",0,$J129))</f>
@@ -7950,7 +7950,7 @@
         <v/>
       </c>
       <c r="J131" s="4" t="n">
-        <v>807.52</v>
+        <v>592.84</v>
       </c>
       <c r="K131" s="21">
         <f>IF(OR($B131="",$I131=""),"",$I131-IF($J131="",0,$J131))</f>
@@ -8052,7 +8052,7 @@
         <v/>
       </c>
       <c r="J133" s="4" t="n">
-        <v>801.97</v>
+        <v>509.91</v>
       </c>
       <c r="K133" s="21">
         <f>IF(OR($B133="",$I133=""),"",$I133-IF($J133="",0,$J133))</f>
@@ -8103,7 +8103,7 @@
         <v/>
       </c>
       <c r="J134" s="4" t="n">
-        <v>794.09</v>
+        <v>578.39</v>
       </c>
       <c r="K134" s="21">
         <f>IF(OR($B134="",$I134=""),"",$I134-IF($J134="",0,$J134))</f>
@@ -8150,7 +8150,7 @@
         <v/>
       </c>
       <c r="J135" s="4" t="n">
-        <v>289.29</v>
+        <v>401.03</v>
       </c>
       <c r="K135" s="21">
         <f>IF(OR($B135="",$I135=""),"",$I135-IF($J135="",0,$J135))</f>
@@ -8248,7 +8248,7 @@
         <v/>
       </c>
       <c r="J137" s="4" t="n">
-        <v>154.28</v>
+        <v>357.16</v>
       </c>
       <c r="K137" s="21">
         <f>IF(OR($B137="",$I137=""),"",$I137-IF($J137="",0,$J137))</f>
@@ -8295,7 +8295,7 @@
         <v/>
       </c>
       <c r="J138" s="4" t="n">
-        <v>287.3</v>
+        <v>398.02</v>
       </c>
       <c r="K138" s="21">
         <f>IF(OR($B138="",$I138=""),"",$I138-IF($J138="",0,$J138))</f>
@@ -8346,7 +8346,7 @@
         <v/>
       </c>
       <c r="J139" s="4" t="n">
-        <v>149.94</v>
+        <v>342.92</v>
       </c>
       <c r="K139" s="21">
         <f>IF(OR($B139="",$I139=""),"",$I139-IF($J139="",0,$J139))</f>
@@ -8393,7 +8393,7 @@
         <v/>
       </c>
       <c r="J140" s="4" t="n">
-        <v>288.16</v>
+        <v>404.66</v>
       </c>
       <c r="K140" s="21">
         <f>IF(OR($B140="",$I140=""),"",$I140-IF($J140="",0,$J140))</f>
@@ -8440,7 +8440,7 @@
         <v/>
       </c>
       <c r="J141" s="4" t="n">
-        <v>289.27</v>
+        <v>396.69</v>
       </c>
       <c r="K141" s="21">
         <f>IF(OR($B141="",$I141=""),"",$I141-IF($J141="",0,$J141))</f>
@@ -8487,7 +8487,7 @@
         <v/>
       </c>
       <c r="J142" s="4" t="n">
-        <v>288.59</v>
+        <v>381.4</v>
       </c>
       <c r="K142" s="21">
         <f>IF(OR($B142="",$I142=""),"",$I142-IF($J142="",0,$J142))</f>
@@ -8538,7 +8538,7 @@
         <v/>
       </c>
       <c r="J143" s="4" t="n">
-        <v>148.6</v>
+        <v>339.3</v>
       </c>
       <c r="K143" s="21">
         <f>IF(OR($B143="",$I143=""),"",$I143-IF($J143="",0,$J143))</f>
@@ -8585,7 +8585,7 @@
         <v/>
       </c>
       <c r="J144" s="4" t="n">
-        <v>121.89</v>
+        <v>121.9</v>
       </c>
       <c r="K144" s="21">
         <f>IF(OR($B144="",$I144=""),"",$I144-IF($J144="",0,$J144))</f>
@@ -8632,7 +8632,7 @@
         <v/>
       </c>
       <c r="J145" s="4" t="n">
-        <v>288.47</v>
+        <v>405.65</v>
       </c>
       <c r="K145" s="21">
         <f>IF(OR($B145="",$I145=""),"",$I145-IF($J145="",0,$J145))</f>
@@ -8683,7 +8683,7 @@
         <v/>
       </c>
       <c r="J146" s="4" t="n">
-        <v>150.9</v>
+        <v>421.14</v>
       </c>
       <c r="K146" s="21">
         <f>IF(OR($B146="",$I146=""),"",$I146-IF($J146="",0,$J146))</f>
@@ -8734,7 +8734,7 @@
         <v/>
       </c>
       <c r="J147" s="4" t="n">
-        <v>149.67</v>
+        <v>343.65</v>
       </c>
       <c r="K147" s="21">
         <f>IF(OR($B147="",$I147=""),"",$I147-IF($J147="",0,$J147))</f>

</xml_diff>

<commit_message>
Data update — 2026-09-15 candle + results refresh
</commit_message>
<xml_diff>
--- a/results/strategy_pnl_simple.xlsx
+++ b/results/strategy_pnl_simple.xlsx
@@ -8143,14 +8143,18 @@
       <c r="F135" s="26" t="n">
         <v>618</v>
       </c>
-      <c r="G135" s="24" t="inlineStr"/>
-      <c r="H135" s="25" t="inlineStr"/>
+      <c r="G135" s="24" t="n">
+        <v>46280</v>
+      </c>
+      <c r="H135" s="25" t="n">
+        <v>281.0708</v>
+      </c>
       <c r="I135" s="21">
         <f>IF(OR($B135="",$H135=""),"",IF($C135="LONG",($H135-$E135)*$F135,($E135-$H135)*$F135))</f>
         <v/>
       </c>
       <c r="J135" s="4" t="n">
-        <v>401.03</v>
+        <v>642.08</v>
       </c>
       <c r="K135" s="21">
         <f>IF(OR($B135="",$I135=""),"",$I135-IF($J135="",0,$J135))</f>
@@ -8190,14 +8194,18 @@
       <c r="F136" s="26" t="n">
         <v>1042</v>
       </c>
-      <c r="G136" s="24" t="inlineStr"/>
-      <c r="H136" s="25" t="inlineStr"/>
+      <c r="G136" s="24" t="n">
+        <v>46280</v>
+      </c>
+      <c r="H136" s="25" t="n">
+        <v>87.90260000000001</v>
+      </c>
       <c r="I136" s="21">
         <f>IF(OR($B136="",$H136=""),"",IF($C136="LONG",($H136-$E136)*$F136,($E136-$H136)*$F136))</f>
         <v/>
       </c>
       <c r="J136" s="4" t="n">
-        <v>122.79</v>
+        <v>217.81</v>
       </c>
       <c r="K136" s="21">
         <f>IF(OR($B136="",$I136=""),"",$I136-IF($J136="",0,$J136))</f>
@@ -8288,14 +8296,18 @@
       <c r="F138" s="26" t="n">
         <v>47</v>
       </c>
-      <c r="G138" s="24" t="inlineStr"/>
-      <c r="H138" s="25" t="inlineStr"/>
+      <c r="G138" s="24" t="n">
+        <v>46280</v>
+      </c>
+      <c r="H138" s="25" t="n">
+        <v>3905.0383</v>
+      </c>
       <c r="I138" s="21">
         <f>IF(OR($B138="",$H138=""),"",IF($C138="LONG",($H138-$E138)*$F138,($E138-$H138)*$F138))</f>
         <v/>
       </c>
       <c r="J138" s="4" t="n">
-        <v>398.02</v>
+        <v>648.9299999999999</v>
       </c>
       <c r="K138" s="21">
         <f>IF(OR($B138="",$I138=""),"",$I138-IF($J138="",0,$J138))</f>
@@ -8386,14 +8398,18 @@
       <c r="F140" s="26" t="n">
         <v>860</v>
       </c>
-      <c r="G140" s="24" t="inlineStr"/>
-      <c r="H140" s="25" t="inlineStr"/>
+      <c r="G140" s="24" t="n">
+        <v>46280</v>
+      </c>
+      <c r="H140" s="25" t="n">
+        <v>204.1101</v>
+      </c>
       <c r="I140" s="21">
         <f>IF(OR($B140="",$H140=""),"",IF($C140="LONG",($H140-$E140)*$F140,($E140-$H140)*$F140))</f>
         <v/>
       </c>
       <c r="J140" s="4" t="n">
-        <v>404.66</v>
+        <v>649.1900000000001</v>
       </c>
       <c r="K140" s="21">
         <f>IF(OR($B140="",$I140=""),"",$I140-IF($J140="",0,$J140))</f>
@@ -8433,14 +8449,18 @@
       <c r="F141" s="26" t="n">
         <v>377</v>
       </c>
-      <c r="G141" s="24" t="inlineStr"/>
-      <c r="H141" s="25" t="inlineStr"/>
+      <c r="G141" s="24" t="n">
+        <v>46280</v>
+      </c>
+      <c r="H141" s="25" t="n">
+        <v>497.2753</v>
+      </c>
       <c r="I141" s="21">
         <f>IF(OR($B141="",$H141=""),"",IF($C141="LONG",($H141-$E141)*$F141,($E141-$H141)*$F141))</f>
         <v/>
       </c>
       <c r="J141" s="4" t="n">
-        <v>396.69</v>
+        <v>650.54</v>
       </c>
       <c r="K141" s="21">
         <f>IF(OR($B141="",$I141=""),"",$I141-IF($J141="",0,$J141))</f>
@@ -8480,14 +8500,18 @@
       <c r="F142" s="26" t="n">
         <v>103</v>
       </c>
-      <c r="G142" s="24" t="inlineStr"/>
-      <c r="H142" s="25" t="inlineStr"/>
+      <c r="G142" s="24" t="n">
+        <v>46280</v>
+      </c>
+      <c r="H142" s="25" t="n">
+        <v>1775.6097</v>
+      </c>
       <c r="I142" s="21">
         <f>IF(OR($B142="",$H142=""),"",IF($C142="LONG",($H142-$E142)*$F142,($E142-$H142)*$F142))</f>
         <v/>
       </c>
       <c r="J142" s="4" t="n">
-        <v>381.4</v>
+        <v>625.67</v>
       </c>
       <c r="K142" s="21">
         <f>IF(OR($B142="",$I142=""),"",$I142-IF($J142="",0,$J142))</f>
@@ -8578,14 +8602,18 @@
       <c r="F144" s="26" t="n">
         <v>83</v>
       </c>
-      <c r="G144" s="24" t="inlineStr"/>
-      <c r="H144" s="25" t="inlineStr"/>
+      <c r="G144" s="24" t="n">
+        <v>46280</v>
+      </c>
+      <c r="H144" s="25" t="n">
+        <v>1035.862</v>
+      </c>
       <c r="I144" s="21">
         <f>IF(OR($B144="",$H144=""),"",IF($C144="LONG",($H144-$E144)*$F144,($E144-$H144)*$F144))</f>
         <v/>
       </c>
       <c r="J144" s="4" t="n">
-        <v>121.9</v>
+        <v>211.09</v>
       </c>
       <c r="K144" s="21">
         <f>IF(OR($B144="",$I144=""),"",$I144-IF($J144="",0,$J144))</f>
@@ -8625,14 +8653,18 @@
       <c r="F145" s="26" t="n">
         <v>391</v>
       </c>
-      <c r="G145" s="24" t="inlineStr"/>
-      <c r="H145" s="25" t="inlineStr"/>
+      <c r="G145" s="24" t="n">
+        <v>46280</v>
+      </c>
+      <c r="H145" s="25" t="n">
+        <v>409.8205</v>
+      </c>
       <c r="I145" s="21">
         <f>IF(OR($B145="",$H145=""),"",IF($C145="LONG",($H145-$E145)*$F145,($E145-$H145)*$F145))</f>
         <v/>
       </c>
       <c r="J145" s="4" t="n">
-        <v>405.65</v>
+        <v>634.54</v>
       </c>
       <c r="K145" s="21">
         <f>IF(OR($B145="",$I145=""),"",$I145-IF($J145="",0,$J145))</f>
@@ -8750,19 +8782,43 @@
       </c>
     </row>
     <row r="148">
-      <c r="A148" s="23" t="n"/>
-      <c r="B148" s="23" t="n"/>
-      <c r="C148" s="23" t="n"/>
-      <c r="D148" s="24" t="n"/>
-      <c r="E148" s="25" t="n"/>
-      <c r="F148" s="26" t="n"/>
-      <c r="G148" s="24" t="n"/>
-      <c r="H148" s="25" t="n"/>
+      <c r="A148" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-221260915461009</t>
+        </is>
+      </c>
+      <c r="B148" s="23" t="inlineStr">
+        <is>
+          <t>AWFIS</t>
+        </is>
+      </c>
+      <c r="C148" s="23" t="inlineStr">
+        <is>
+          <t>SHORT</t>
+        </is>
+      </c>
+      <c r="D148" s="24" t="n">
+        <v>46280</v>
+      </c>
+      <c r="E148" s="25" t="n">
+        <v>280.9703</v>
+      </c>
+      <c r="F148" s="26" t="n">
+        <v>618</v>
+      </c>
+      <c r="G148" s="24" t="n">
+        <v>46280</v>
+      </c>
+      <c r="H148" s="25" t="n">
+        <v>274.7952</v>
+      </c>
       <c r="I148" s="21">
         <f>IF(OR($B148="",$H148=""),"",IF($C148="LONG",($H148-$E148)*$F148,($E148-$H148)*$F148))</f>
         <v/>
       </c>
-      <c r="J148" s="4" t="n"/>
+      <c r="J148" s="4" t="n">
+        <v>108.55</v>
+      </c>
       <c r="K148" s="21">
         <f>IF(OR($B148="",$I148=""),"",$I148-IF($J148="",0,$J148))</f>
         <v/>
@@ -8777,19 +8833,43 @@
       </c>
     </row>
     <row r="149">
-      <c r="A149" s="23" t="n"/>
-      <c r="B149" s="23" t="n"/>
-      <c r="C149" s="23" t="n"/>
-      <c r="D149" s="24" t="n"/>
-      <c r="E149" s="25" t="n"/>
-      <c r="F149" s="26" t="n"/>
-      <c r="G149" s="24" t="n"/>
-      <c r="H149" s="25" t="n"/>
+      <c r="A149" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-23126091516209</t>
+        </is>
+      </c>
+      <c r="B149" s="23" t="inlineStr">
+        <is>
+          <t>FILATEX</t>
+        </is>
+      </c>
+      <c r="C149" s="23" t="inlineStr">
+        <is>
+          <t>SHORT</t>
+        </is>
+      </c>
+      <c r="D149" s="24" t="n">
+        <v>46280</v>
+      </c>
+      <c r="E149" s="25" t="n">
+        <v>87.81999999999999</v>
+      </c>
+      <c r="F149" s="26" t="n">
+        <v>1042</v>
+      </c>
+      <c r="G149" s="24" t="n">
+        <v>46280</v>
+      </c>
+      <c r="H149" s="25" t="n">
+        <v>83.43000000000001</v>
+      </c>
       <c r="I149" s="21">
         <f>IF(OR($B149="",$H149=""),"",IF($C149="LONG",($H149-$E149)*$F149,($E149-$H149)*$F149))</f>
         <v/>
       </c>
-      <c r="J149" s="4" t="n"/>
+      <c r="J149" s="4" t="n">
+        <v>79.36</v>
+      </c>
       <c r="K149" s="21">
         <f>IF(OR($B149="",$I149=""),"",$I149-IF($J149="",0,$J149))</f>
         <v/>
@@ -8804,19 +8884,43 @@
       </c>
     </row>
     <row r="150">
-      <c r="A150" s="23" t="n"/>
-      <c r="B150" s="23" t="n"/>
-      <c r="C150" s="23" t="n"/>
-      <c r="D150" s="24" t="n"/>
-      <c r="E150" s="25" t="n"/>
-      <c r="F150" s="26" t="n"/>
-      <c r="G150" s="24" t="n"/>
-      <c r="H150" s="25" t="n"/>
+      <c r="A150" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-23126091516309</t>
+        </is>
+      </c>
+      <c r="B150" s="23" t="inlineStr">
+        <is>
+          <t>KIRLOSIND</t>
+        </is>
+      </c>
+      <c r="C150" s="23" t="inlineStr">
+        <is>
+          <t>SHORT</t>
+        </is>
+      </c>
+      <c r="D150" s="24" t="n">
+        <v>46280</v>
+      </c>
+      <c r="E150" s="25" t="n">
+        <v>3900.0042</v>
+      </c>
+      <c r="F150" s="26" t="n">
+        <v>47</v>
+      </c>
+      <c r="G150" s="24" t="n">
+        <v>46280</v>
+      </c>
+      <c r="H150" s="25" t="n">
+        <v>3823.1084</v>
+      </c>
       <c r="I150" s="21">
         <f>IF(OR($B150="",$H150=""),"",IF($C150="LONG",($H150-$E150)*$F150,($E150-$H150)*$F150))</f>
         <v/>
       </c>
-      <c r="J150" s="4" t="n"/>
+      <c r="J150" s="4" t="n">
+        <v>111.99</v>
+      </c>
       <c r="K150" s="21">
         <f>IF(OR($B150="",$I150=""),"",$I150-IF($J150="",0,$J150))</f>
         <v/>
@@ -8831,19 +8935,43 @@
       </c>
     </row>
     <row r="151">
-      <c r="A151" s="23" t="n"/>
-      <c r="B151" s="23" t="n"/>
-      <c r="C151" s="23" t="n"/>
-      <c r="D151" s="24" t="n"/>
-      <c r="E151" s="25" t="n"/>
-      <c r="F151" s="26" t="n"/>
-      <c r="G151" s="24" t="n"/>
-      <c r="H151" s="25" t="n"/>
+      <c r="A151" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-221260915460909</t>
+        </is>
+      </c>
+      <c r="B151" s="23" t="inlineStr">
+        <is>
+          <t>MOBIKWIK</t>
+        </is>
+      </c>
+      <c r="C151" s="23" t="inlineStr">
+        <is>
+          <t>SHORT</t>
+        </is>
+      </c>
+      <c r="D151" s="24" t="n">
+        <v>46280</v>
+      </c>
+      <c r="E151" s="25" t="n">
+        <v>204.3287</v>
+      </c>
+      <c r="F151" s="26" t="n">
+        <v>860</v>
+      </c>
+      <c r="G151" s="24" t="n">
+        <v>46280</v>
+      </c>
+      <c r="H151" s="25" t="n">
+        <v>205.9936</v>
+      </c>
       <c r="I151" s="21">
         <f>IF(OR($B151="",$H151=""),"",IF($C151="LONG",($H151-$E151)*$F151,($E151-$H151)*$F151))</f>
         <v/>
       </c>
-      <c r="J151" s="4" t="n"/>
+      <c r="J151" s="4" t="n">
+        <v>109.64</v>
+      </c>
       <c r="K151" s="21">
         <f>IF(OR($B151="",$I151=""),"",$I151-IF($J151="",0,$J151))</f>
         <v/>
@@ -8858,19 +8986,43 @@
       </c>
     </row>
     <row r="152">
-      <c r="A152" s="23" t="n"/>
-      <c r="B152" s="23" t="n"/>
-      <c r="C152" s="23" t="n"/>
-      <c r="D152" s="24" t="n"/>
-      <c r="E152" s="25" t="n"/>
-      <c r="F152" s="26" t="n"/>
-      <c r="G152" s="24" t="n"/>
-      <c r="H152" s="25" t="n"/>
+      <c r="A152" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-34126091550709</t>
+        </is>
+      </c>
+      <c r="B152" s="23" t="inlineStr">
+        <is>
+          <t>QUADFUTURE</t>
+        </is>
+      </c>
+      <c r="C152" s="23" t="inlineStr">
+        <is>
+          <t>SHORT</t>
+        </is>
+      </c>
+      <c r="D152" s="24" t="n">
+        <v>46280</v>
+      </c>
+      <c r="E152" s="25" t="n">
+        <v>496.9672</v>
+      </c>
+      <c r="F152" s="26" t="n">
+        <v>377</v>
+      </c>
+      <c r="G152" s="24" t="n">
+        <v>46280</v>
+      </c>
+      <c r="H152" s="25" t="n">
+        <v>490</v>
+      </c>
       <c r="I152" s="21">
         <f>IF(OR($B152="",$H152=""),"",IF($C152="LONG",($H152-$E152)*$F152,($E152-$H152)*$F152))</f>
         <v/>
       </c>
-      <c r="J152" s="4" t="n"/>
+      <c r="J152" s="4" t="n">
+        <v>113.5</v>
+      </c>
       <c r="K152" s="21">
         <f>IF(OR($B152="",$I152=""),"",$I152-IF($J152="",0,$J152))</f>
         <v/>
@@ -8885,19 +9037,43 @@
       </c>
     </row>
     <row r="153">
-      <c r="A153" s="23" t="n"/>
-      <c r="B153" s="23" t="n"/>
-      <c r="C153" s="23" t="n"/>
-      <c r="D153" s="24" t="n"/>
-      <c r="E153" s="25" t="n"/>
-      <c r="F153" s="26" t="n"/>
-      <c r="G153" s="24" t="n"/>
-      <c r="H153" s="25" t="n"/>
+      <c r="A153" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-34126091518009</t>
+        </is>
+      </c>
+      <c r="B153" s="23" t="inlineStr">
+        <is>
+          <t>RACLGEAR</t>
+        </is>
+      </c>
+      <c r="C153" s="23" t="inlineStr">
+        <is>
+          <t>SHORT</t>
+        </is>
+      </c>
+      <c r="D153" s="24" t="n">
+        <v>46280</v>
+      </c>
+      <c r="E153" s="25" t="n">
+        <v>1779.6</v>
+      </c>
+      <c r="F153" s="26" t="n">
+        <v>103</v>
+      </c>
+      <c r="G153" s="24" t="n">
+        <v>46280</v>
+      </c>
+      <c r="H153" s="25" t="n">
+        <v>1690.6</v>
+      </c>
       <c r="I153" s="21">
         <f>IF(OR($B153="",$H153=""),"",IF($C153="LONG",($H153-$E153)*$F153,($E153-$H153)*$F153))</f>
         <v/>
       </c>
-      <c r="J153" s="4" t="n"/>
+      <c r="J153" s="4" t="n">
+        <v>111.62</v>
+      </c>
       <c r="K153" s="21">
         <f>IF(OR($B153="",$I153=""),"",$I153-IF($J153="",0,$J153))</f>
         <v/>
@@ -8912,19 +9088,43 @@
       </c>
     </row>
     <row r="154">
-      <c r="A154" s="23" t="n"/>
-      <c r="B154" s="23" t="n"/>
-      <c r="C154" s="23" t="n"/>
-      <c r="D154" s="24" t="n"/>
-      <c r="E154" s="25" t="n"/>
-      <c r="F154" s="26" t="n"/>
-      <c r="G154" s="24" t="n"/>
-      <c r="H154" s="25" t="n"/>
+      <c r="A154" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-23126091546509</t>
+        </is>
+      </c>
+      <c r="B154" s="23" t="inlineStr">
+        <is>
+          <t>SIKA</t>
+        </is>
+      </c>
+      <c r="C154" s="23" t="inlineStr">
+        <is>
+          <t>SHORT</t>
+        </is>
+      </c>
+      <c r="D154" s="24" t="n">
+        <v>46280</v>
+      </c>
+      <c r="E154" s="25" t="n">
+        <v>1034.3916</v>
+      </c>
+      <c r="F154" s="26" t="n">
+        <v>83</v>
+      </c>
+      <c r="G154" s="24" t="n">
+        <v>46280</v>
+      </c>
+      <c r="H154" s="25" t="n">
+        <v>1044.0566</v>
+      </c>
       <c r="I154" s="21">
         <f>IF(OR($B154="",$H154=""),"",IF($C154="LONG",($H154-$E154)*$F154,($E154-$H154)*$F154))</f>
         <v/>
       </c>
-      <c r="J154" s="4" t="n"/>
+      <c r="J154" s="4" t="n">
+        <v>77.72</v>
+      </c>
       <c r="K154" s="21">
         <f>IF(OR($B154="",$I154=""),"",$I154-IF($J154="",0,$J154))</f>
         <v/>
@@ -8939,19 +9139,43 @@
       </c>
     </row>
     <row r="155">
-      <c r="A155" s="23" t="n"/>
-      <c r="B155" s="23" t="n"/>
-      <c r="C155" s="23" t="n"/>
-      <c r="D155" s="24" t="n"/>
-      <c r="E155" s="25" t="n"/>
-      <c r="F155" s="26" t="n"/>
-      <c r="G155" s="24" t="n"/>
-      <c r="H155" s="25" t="n"/>
+      <c r="A155" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-34126091550609</t>
+        </is>
+      </c>
+      <c r="B155" s="23" t="inlineStr">
+        <is>
+          <t>SMSPHARMA</t>
+        </is>
+      </c>
+      <c r="C155" s="23" t="inlineStr">
+        <is>
+          <t>SHORT</t>
+        </is>
+      </c>
+      <c r="D155" s="24" t="n">
+        <v>46280</v>
+      </c>
+      <c r="E155" s="25" t="n">
+        <v>409.8</v>
+      </c>
+      <c r="F155" s="26" t="n">
+        <v>391</v>
+      </c>
+      <c r="G155" s="24" t="n">
+        <v>46280</v>
+      </c>
+      <c r="H155" s="25" t="n">
+        <v>407.7166</v>
+      </c>
       <c r="I155" s="21">
         <f>IF(OR($B155="",$H155=""),"",IF($C155="LONG",($H155-$E155)*$F155,($E155-$H155)*$F155))</f>
         <v/>
       </c>
-      <c r="J155" s="4" t="n"/>
+      <c r="J155" s="4" t="n">
+        <v>104</v>
+      </c>
       <c r="K155" s="21">
         <f>IF(OR($B155="",$I155=""),"",$I155-IF($J155="",0,$J155))</f>
         <v/>

</xml_diff>

<commit_message>
Data update — 2026-09-16 candle + results refresh
</commit_message>
<xml_diff>
--- a/results/strategy_pnl_simple.xlsx
+++ b/results/strategy_pnl_simple.xlsx
@@ -1473,7 +1473,7 @@
         <v/>
       </c>
       <c r="J4" s="4" t="n">
-        <v>571.8</v>
+        <v>571.85</v>
       </c>
       <c r="K4" s="21">
         <f>IF(OR($B4="",$I4=""),"",$I4-IF($J4="",0,$J4))</f>
@@ -1524,7 +1524,7 @@
         <v/>
       </c>
       <c r="J5" s="4" t="n">
-        <v>688.92</v>
+        <v>688.88</v>
       </c>
       <c r="K5" s="21">
         <f>IF(OR($B5="",$I5=""),"",$I5-IF($J5="",0,$J5))</f>
@@ -1575,7 +1575,7 @@
         <v/>
       </c>
       <c r="J6" s="4" t="n">
-        <v>570.65</v>
+        <v>570.6900000000001</v>
       </c>
       <c r="K6" s="21">
         <f>IF(OR($B6="",$I6=""),"",$I6-IF($J6="",0,$J6))</f>
@@ -1626,7 +1626,7 @@
         <v/>
       </c>
       <c r="J7" s="4" t="n">
-        <v>663.05</v>
+        <v>663.11</v>
       </c>
       <c r="K7" s="21">
         <f>IF(OR($B7="",$I7=""),"",$I7-IF($J7="",0,$J7))</f>
@@ -1677,7 +1677,7 @@
         <v/>
       </c>
       <c r="J8" s="4" t="n">
-        <v>590.75</v>
+        <v>590.76</v>
       </c>
       <c r="K8" s="21">
         <f>IF(OR($B8="",$I8=""),"",$I8-IF($J8="",0,$J8))</f>
@@ -1779,7 +1779,7 @@
         <v/>
       </c>
       <c r="J10" s="4" t="n">
-        <v>398.62</v>
+        <v>398.65</v>
       </c>
       <c r="K10" s="21">
         <f>IF(OR($B10="",$I10=""),"",$I10-IF($J10="",0,$J10))</f>
@@ -1881,7 +1881,7 @@
         <v/>
       </c>
       <c r="J12" s="4" t="n">
-        <v>414.17</v>
+        <v>414.2</v>
       </c>
       <c r="K12" s="21">
         <f>IF(OR($B12="",$I12=""),"",$I12-IF($J12="",0,$J12))</f>
@@ -1932,7 +1932,7 @@
         <v/>
       </c>
       <c r="J13" s="4" t="n">
-        <v>345.08</v>
+        <v>345.09</v>
       </c>
       <c r="K13" s="21">
         <f>IF(OR($B13="",$I13=""),"",$I13-IF($J13="",0,$J13))</f>
@@ -1983,7 +1983,7 @@
         <v/>
       </c>
       <c r="J14" s="4" t="n">
-        <v>414.5</v>
+        <v>414.53</v>
       </c>
       <c r="K14" s="21">
         <f>IF(OR($B14="",$I14=""),"",$I14-IF($J14="",0,$J14))</f>
@@ -2034,7 +2034,7 @@
         <v/>
       </c>
       <c r="J15" s="4" t="n">
-        <v>380.31</v>
+        <v>380.34</v>
       </c>
       <c r="K15" s="21">
         <f>IF(OR($B15="",$I15=""),"",$I15-IF($J15="",0,$J15))</f>
@@ -2187,7 +2187,7 @@
         <v/>
       </c>
       <c r="J18" s="4" t="n">
-        <v>413.93</v>
+        <v>413.96</v>
       </c>
       <c r="K18" s="21">
         <f>IF(OR($B18="",$I18=""),"",$I18-IF($J18="",0,$J18))</f>
@@ -2238,7 +2238,7 @@
         <v/>
       </c>
       <c r="J19" s="4" t="n">
-        <v>406.46</v>
+        <v>406.49</v>
       </c>
       <c r="K19" s="21">
         <f>IF(OR($B19="",$I19=""),"",$I19-IF($J19="",0,$J19))</f>
@@ -2697,7 +2697,7 @@
         <v/>
       </c>
       <c r="J28" s="4" t="n">
-        <v>870.51</v>
+        <v>870.13</v>
       </c>
       <c r="K28" s="21">
         <f>IF(OR($B28="",$I28=""),"",$I28-IF($J28="",0,$J28))</f>
@@ -2850,7 +2850,7 @@
         <v/>
       </c>
       <c r="J31" s="4" t="n">
-        <v>391.15</v>
+        <v>391.16</v>
       </c>
       <c r="K31" s="21">
         <f>IF(OR($B31="",$I31=""),"",$I31-IF($J31="",0,$J31))</f>
@@ -2901,7 +2901,7 @@
         <v/>
       </c>
       <c r="J32" s="4" t="n">
-        <v>349.77</v>
+        <v>349.78</v>
       </c>
       <c r="K32" s="21">
         <f>IF(OR($B32="",$I32=""),"",$I32-IF($J32="",0,$J32))</f>
@@ -3003,7 +3003,7 @@
         <v/>
       </c>
       <c r="J34" s="4" t="n">
-        <v>349.93</v>
+        <v>349.78</v>
       </c>
       <c r="K34" s="21">
         <f>IF(OR($B34="",$I34=""),"",$I34-IF($J34="",0,$J34))</f>
@@ -3054,7 +3054,7 @@
         <v/>
       </c>
       <c r="J35" s="4" t="n">
-        <v>386.08</v>
+        <v>386.15</v>
       </c>
       <c r="K35" s="21">
         <f>IF(OR($B35="",$I35=""),"",$I35-IF($J35="",0,$J35))</f>
@@ -3411,7 +3411,7 @@
         <v/>
       </c>
       <c r="J42" s="4" t="n">
-        <v>978.27</v>
+        <v>978.29</v>
       </c>
       <c r="K42" s="21">
         <f>IF(OR($B42="",$I42=""),"",$I42-IF($J42="",0,$J42))</f>
@@ -3462,7 +3462,7 @@
         <v/>
       </c>
       <c r="J43" s="4" t="n">
-        <v>957.67</v>
+        <v>957.6799999999999</v>
       </c>
       <c r="K43" s="21">
         <f>IF(OR($B43="",$I43=""),"",$I43-IF($J43="",0,$J43))</f>
@@ -3513,7 +3513,7 @@
         <v/>
       </c>
       <c r="J44" s="4" t="n">
-        <v>992.26</v>
+        <v>992.28</v>
       </c>
       <c r="K44" s="21">
         <f>IF(OR($B44="",$I44=""),"",$I44-IF($J44="",0,$J44))</f>
@@ -3564,7 +3564,7 @@
         <v/>
       </c>
       <c r="J45" s="4" t="n">
-        <v>599.6799999999999</v>
+        <v>599.71</v>
       </c>
       <c r="K45" s="21">
         <f>IF(OR($B45="",$I45=""),"",$I45-IF($J45="",0,$J45))</f>
@@ -3615,7 +3615,7 @@
         <v/>
       </c>
       <c r="J46" s="4" t="n">
-        <v>600.78</v>
+        <v>600.8200000000001</v>
       </c>
       <c r="K46" s="21">
         <f>IF(OR($B46="",$I46=""),"",$I46-IF($J46="",0,$J46))</f>
@@ -3666,7 +3666,7 @@
         <v/>
       </c>
       <c r="J47" s="4" t="n">
-        <v>678.63</v>
+        <v>678.75</v>
       </c>
       <c r="K47" s="21">
         <f>IF(OR($B47="",$I47=""),"",$I47-IF($J47="",0,$J47))</f>
@@ -3717,7 +3717,7 @@
         <v/>
       </c>
       <c r="J48" s="4" t="n">
-        <v>672.62</v>
+        <v>672.49</v>
       </c>
       <c r="K48" s="21">
         <f>IF(OR($B48="",$I48=""),"",$I48-IF($J48="",0,$J48))</f>
@@ -3768,7 +3768,7 @@
         <v/>
       </c>
       <c r="J49" s="4" t="n">
-        <v>538.66</v>
+        <v>538.6799999999999</v>
       </c>
       <c r="K49" s="21">
         <f>IF(OR($B49="",$I49=""),"",$I49-IF($J49="",0,$J49))</f>
@@ -3819,7 +3819,7 @@
         <v/>
       </c>
       <c r="J50" s="4" t="n">
-        <v>627.89</v>
+        <v>627.98</v>
       </c>
       <c r="K50" s="21">
         <f>IF(OR($B50="",$I50=""),"",$I50-IF($J50="",0,$J50))</f>
@@ -4023,7 +4023,7 @@
         <v/>
       </c>
       <c r="J54" s="4" t="n">
-        <v>619.12</v>
+        <v>619.13</v>
       </c>
       <c r="K54" s="21">
         <f>IF(OR($B54="",$I54=""),"",$I54-IF($J54="",0,$J54))</f>
@@ -4176,7 +4176,7 @@
         <v/>
       </c>
       <c r="J57" s="4" t="n">
-        <v>612.2</v>
+        <v>612.27</v>
       </c>
       <c r="K57" s="21">
         <f>IF(OR($B57="",$I57=""),"",$I57-IF($J57="",0,$J57))</f>
@@ -4380,7 +4380,7 @@
         <v/>
       </c>
       <c r="J61" s="4" t="n">
-        <v>691.97</v>
+        <v>692.09</v>
       </c>
       <c r="K61" s="21">
         <f>IF(OR($B61="",$I61=""),"",$I61-IF($J61="",0,$J61))</f>
@@ -4431,7 +4431,7 @@
         <v/>
       </c>
       <c r="J62" s="4" t="n">
-        <v>615.91</v>
+        <v>615.39</v>
       </c>
       <c r="K62" s="21">
         <f>IF(OR($B62="",$I62=""),"",$I62-IF($J62="",0,$J62))</f>
@@ -4533,7 +4533,7 @@
         <v/>
       </c>
       <c r="J64" s="4" t="n">
-        <v>440.52</v>
+        <v>440.45</v>
       </c>
       <c r="K64" s="21">
         <f>IF(OR($B64="",$I64=""),"",$I64-IF($J64="",0,$J64))</f>
@@ -4584,7 +4584,7 @@
         <v/>
       </c>
       <c r="J65" s="4" t="n">
-        <v>386.52</v>
+        <v>386.59</v>
       </c>
       <c r="K65" s="21">
         <f>IF(OR($B65="",$I65=""),"",$I65-IF($J65="",0,$J65))</f>
@@ -4839,7 +4839,7 @@
         <v/>
       </c>
       <c r="J70" s="4" t="n">
-        <v>385.13</v>
+        <v>385.19</v>
       </c>
       <c r="K70" s="21">
         <f>IF(OR($B70="",$I70=""),"",$I70-IF($J70="",0,$J70))</f>
@@ -4890,7 +4890,7 @@
         <v/>
       </c>
       <c r="J71" s="4" t="n">
-        <v>434.2</v>
+        <v>434.27</v>
       </c>
       <c r="K71" s="21">
         <f>IF(OR($B71="",$I71=""),"",$I71-IF($J71="",0,$J71))</f>
@@ -4941,7 +4941,7 @@
         <v/>
       </c>
       <c r="J72" s="4" t="n">
-        <v>376.86</v>
+        <v>376.89</v>
       </c>
       <c r="K72" s="21">
         <f>IF(OR($B72="",$I72=""),"",$I72-IF($J72="",0,$J72))</f>
@@ -5043,7 +5043,7 @@
         <v/>
       </c>
       <c r="J74" s="4" t="n">
-        <v>327.29</v>
+        <v>327.31</v>
       </c>
       <c r="K74" s="21">
         <f>IF(OR($B74="",$I74=""),"",$I74-IF($J74="",0,$J74))</f>
@@ -5094,7 +5094,7 @@
         <v/>
       </c>
       <c r="J75" s="4" t="n">
-        <v>330.13</v>
+        <v>330.16</v>
       </c>
       <c r="K75" s="21">
         <f>IF(OR($B75="",$I75=""),"",$I75-IF($J75="",0,$J75))</f>
@@ -5196,7 +5196,7 @@
         <v/>
       </c>
       <c r="J77" s="4" t="n">
-        <v>375.07</v>
+        <v>375.06</v>
       </c>
       <c r="K77" s="21">
         <f>IF(OR($B77="",$I77=""),"",$I77-IF($J77="",0,$J77))</f>
@@ -5298,7 +5298,7 @@
         <v/>
       </c>
       <c r="J79" s="4" t="n">
-        <v>323.33</v>
+        <v>323.35</v>
       </c>
       <c r="K79" s="21">
         <f>IF(OR($B79="",$I79=""),"",$I79-IF($J79="",0,$J79))</f>
@@ -5349,7 +5349,7 @@
         <v/>
       </c>
       <c r="J80" s="4" t="n">
-        <v>324.62</v>
+        <v>324.64</v>
       </c>
       <c r="K80" s="21">
         <f>IF(OR($B80="",$I80=""),"",$I80-IF($J80="",0,$J80))</f>
@@ -6063,7 +6063,7 @@
         <v/>
       </c>
       <c r="J94" s="4" t="n">
-        <v>433.66</v>
+        <v>433.63</v>
       </c>
       <c r="K94" s="21">
         <f>IF(OR($B94="",$I94=""),"",$I94-IF($J94="",0,$J94))</f>
@@ -6879,7 +6879,7 @@
         <v/>
       </c>
       <c r="J110" s="4" t="n">
-        <v>437.61</v>
+        <v>437.57</v>
       </c>
       <c r="K110" s="21">
         <f>IF(OR($B110="",$I110=""),"",$I110-IF($J110="",0,$J110))</f>
@@ -7185,7 +7185,7 @@
         <v/>
       </c>
       <c r="J116" s="4" t="n">
-        <v>394.18</v>
+        <v>394.12</v>
       </c>
       <c r="K116" s="21">
         <f>IF(OR($B116="",$I116=""),"",$I116-IF($J116="",0,$J116))</f>
@@ -7389,7 +7389,7 @@
         <v/>
       </c>
       <c r="J120" s="4" t="n">
-        <v>391.36</v>
+        <v>391.21</v>
       </c>
       <c r="K120" s="21">
         <f>IF(OR($B120="",$I120=""),"",$I120-IF($J120="",0,$J120))</f>
@@ -7950,7 +7950,7 @@
         <v/>
       </c>
       <c r="J131" s="4" t="n">
-        <v>592.84</v>
+        <v>592.8200000000001</v>
       </c>
       <c r="K131" s="21">
         <f>IF(OR($B131="",$I131=""),"",$I131-IF($J131="",0,$J131))</f>
@@ -8154,7 +8154,7 @@
         <v/>
       </c>
       <c r="J135" s="4" t="n">
-        <v>642.08</v>
+        <v>468.38</v>
       </c>
       <c r="K135" s="21">
         <f>IF(OR($B135="",$I135=""),"",$I135-IF($J135="",0,$J135))</f>
@@ -8205,7 +8205,7 @@
         <v/>
       </c>
       <c r="J136" s="4" t="n">
-        <v>217.81</v>
+        <v>149.82</v>
       </c>
       <c r="K136" s="21">
         <f>IF(OR($B136="",$I136=""),"",$I136-IF($J136="",0,$J136))</f>
@@ -8307,7 +8307,7 @@
         <v/>
       </c>
       <c r="J138" s="4" t="n">
-        <v>648.9299999999999</v>
+        <v>465.39</v>
       </c>
       <c r="K138" s="21">
         <f>IF(OR($B138="",$I138=""),"",$I138-IF($J138="",0,$J138))</f>
@@ -8409,7 +8409,7 @@
         <v/>
       </c>
       <c r="J140" s="4" t="n">
-        <v>649.1900000000001</v>
+        <v>473.51</v>
       </c>
       <c r="K140" s="21">
         <f>IF(OR($B140="",$I140=""),"",$I140-IF($J140="",0,$J140))</f>
@@ -8460,7 +8460,7 @@
         <v/>
       </c>
       <c r="J141" s="4" t="n">
-        <v>650.54</v>
+        <v>463.24</v>
       </c>
       <c r="K141" s="21">
         <f>IF(OR($B141="",$I141=""),"",$I141-IF($J141="",0,$J141))</f>
@@ -8511,7 +8511,7 @@
         <v/>
       </c>
       <c r="J142" s="4" t="n">
-        <v>625.67</v>
+        <v>442.78</v>
       </c>
       <c r="K142" s="21">
         <f>IF(OR($B142="",$I142=""),"",$I142-IF($J142="",0,$J142))</f>
@@ -8613,7 +8613,7 @@
         <v/>
       </c>
       <c r="J144" s="4" t="n">
-        <v>211.09</v>
+        <v>148.71</v>
       </c>
       <c r="K144" s="21">
         <f>IF(OR($B144="",$I144=""),"",$I144-IF($J144="",0,$J144))</f>
@@ -8664,7 +8664,7 @@
         <v/>
       </c>
       <c r="J145" s="4" t="n">
-        <v>634.54</v>
+        <v>512.21</v>
       </c>
       <c r="K145" s="21">
         <f>IF(OR($B145="",$I145=""),"",$I145-IF($J145="",0,$J145))</f>
@@ -8817,7 +8817,7 @@
         <v/>
       </c>
       <c r="J148" s="4" t="n">
-        <v>108.55</v>
+        <v>257.03</v>
       </c>
       <c r="K148" s="21">
         <f>IF(OR($B148="",$I148=""),"",$I148-IF($J148="",0,$J148))</f>
@@ -8868,7 +8868,7 @@
         <v/>
       </c>
       <c r="J149" s="4" t="n">
-        <v>79.36</v>
+        <v>145.39</v>
       </c>
       <c r="K149" s="21">
         <f>IF(OR($B149="",$I149=""),"",$I149-IF($J149="",0,$J149))</f>
@@ -8919,7 +8919,7 @@
         <v/>
       </c>
       <c r="J150" s="4" t="n">
-        <v>111.99</v>
+        <v>270.28</v>
       </c>
       <c r="K150" s="21">
         <f>IF(OR($B150="",$I150=""),"",$I150-IF($J150="",0,$J150))</f>
@@ -8970,7 +8970,7 @@
         <v/>
       </c>
       <c r="J151" s="4" t="n">
-        <v>109.64</v>
+        <v>262.28</v>
       </c>
       <c r="K151" s="21">
         <f>IF(OR($B151="",$I151=""),"",$I151-IF($J151="",0,$J151))</f>
@@ -9021,7 +9021,7 @@
         <v/>
       </c>
       <c r="J152" s="4" t="n">
-        <v>113.5</v>
+        <v>276.22</v>
       </c>
       <c r="K152" s="21">
         <f>IF(OR($B152="",$I152=""),"",$I152-IF($J152="",0,$J152))</f>
@@ -9072,7 +9072,7 @@
         <v/>
       </c>
       <c r="J153" s="4" t="n">
-        <v>111.62</v>
+        <v>266.93</v>
       </c>
       <c r="K153" s="21">
         <f>IF(OR($B153="",$I153=""),"",$I153-IF($J153="",0,$J153))</f>
@@ -9123,7 +9123,7 @@
         <v/>
       </c>
       <c r="J154" s="4" t="n">
-        <v>77.72</v>
+        <v>140.35</v>
       </c>
       <c r="K154" s="21">
         <f>IF(OR($B154="",$I154=""),"",$I154-IF($J154="",0,$J154))</f>
@@ -9174,7 +9174,7 @@
         <v/>
       </c>
       <c r="J155" s="4" t="n">
-        <v>104</v>
+        <v>200.3</v>
       </c>
       <c r="K155" s="21">
         <f>IF(OR($B155="",$I155=""),"",$I155-IF($J155="",0,$J155))</f>
@@ -9190,19 +9190,39 @@
       </c>
     </row>
     <row r="156">
-      <c r="A156" s="23" t="n"/>
-      <c r="B156" s="23" t="n"/>
-      <c r="C156" s="23" t="n"/>
-      <c r="D156" s="24" t="n"/>
-      <c r="E156" s="25" t="n"/>
-      <c r="F156" s="26" t="n"/>
-      <c r="G156" s="24" t="n"/>
-      <c r="H156" s="25" t="n"/>
+      <c r="A156" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-23126091659109</t>
+        </is>
+      </c>
+      <c r="B156" s="23" t="inlineStr">
+        <is>
+          <t>EMUDHRA</t>
+        </is>
+      </c>
+      <c r="C156" s="23" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="D156" s="24" t="n">
+        <v>46281</v>
+      </c>
+      <c r="E156" s="25" t="n">
+        <v>635.303</v>
+      </c>
+      <c r="F156" s="26" t="n">
+        <v>395</v>
+      </c>
+      <c r="G156" s="24" t="inlineStr"/>
+      <c r="H156" s="25" t="inlineStr"/>
       <c r="I156" s="21">
         <f>IF(OR($B156="",$H156=""),"",IF($C156="LONG",($H156-$E156)*$F156,($E156-$H156)*$F156))</f>
         <v/>
       </c>
-      <c r="J156" s="4" t="n"/>
+      <c r="J156" s="4" t="n">
+        <v>371.72</v>
+      </c>
       <c r="K156" s="21">
         <f>IF(OR($B156="",$I156=""),"",$I156-IF($J156="",0,$J156))</f>
         <v/>
@@ -9217,19 +9237,39 @@
       </c>
     </row>
     <row r="157">
-      <c r="A157" s="23" t="n"/>
-      <c r="B157" s="23" t="n"/>
-      <c r="C157" s="23" t="n"/>
-      <c r="D157" s="24" t="n"/>
-      <c r="E157" s="25" t="n"/>
-      <c r="F157" s="26" t="n"/>
-      <c r="G157" s="24" t="n"/>
-      <c r="H157" s="25" t="n"/>
+      <c r="A157" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-34126091663709</t>
+        </is>
+      </c>
+      <c r="B157" s="23" t="inlineStr">
+        <is>
+          <t>FOSECOIND</t>
+        </is>
+      </c>
+      <c r="C157" s="23" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="D157" s="24" t="n">
+        <v>46281</v>
+      </c>
+      <c r="E157" s="25" t="n">
+        <v>6778.811</v>
+      </c>
+      <c r="F157" s="26" t="n">
+        <v>37</v>
+      </c>
+      <c r="G157" s="24" t="inlineStr"/>
+      <c r="H157" s="25" t="inlineStr"/>
       <c r="I157" s="21">
         <f>IF(OR($B157="",$H157=""),"",IF($C157="LONG",($H157-$E157)*$F157,($E157-$H157)*$F157))</f>
         <v/>
       </c>
-      <c r="J157" s="4" t="n"/>
+      <c r="J157" s="4" t="n">
+        <v>371.57</v>
+      </c>
       <c r="K157" s="21">
         <f>IF(OR($B157="",$I157=""),"",$I157-IF($J157="",0,$J157))</f>
         <v/>
@@ -9244,19 +9284,39 @@
       </c>
     </row>
     <row r="158">
-      <c r="A158" s="23" t="n"/>
-      <c r="B158" s="23" t="n"/>
-      <c r="C158" s="23" t="n"/>
-      <c r="D158" s="24" t="n"/>
-      <c r="E158" s="25" t="n"/>
-      <c r="F158" s="26" t="n"/>
-      <c r="G158" s="24" t="n"/>
-      <c r="H158" s="25" t="n"/>
+      <c r="A158" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-221260916649209</t>
+        </is>
+      </c>
+      <c r="B158" s="23" t="inlineStr">
+        <is>
+          <t>IPL</t>
+        </is>
+      </c>
+      <c r="C158" s="23" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="D158" s="24" t="n">
+        <v>46281</v>
+      </c>
+      <c r="E158" s="25" t="n">
+        <v>136.1157</v>
+      </c>
+      <c r="F158" s="26" t="n">
+        <v>1842</v>
+      </c>
+      <c r="G158" s="24" t="inlineStr"/>
+      <c r="H158" s="25" t="inlineStr"/>
       <c r="I158" s="21">
         <f>IF(OR($B158="",$H158=""),"",IF($C158="LONG",($H158-$E158)*$F158,($E158-$H158)*$F158))</f>
         <v/>
       </c>
-      <c r="J158" s="4" t="n"/>
+      <c r="J158" s="4" t="n">
+        <v>371.46</v>
+      </c>
       <c r="K158" s="21">
         <f>IF(OR($B158="",$I158=""),"",$I158-IF($J158="",0,$J158))</f>
         <v/>
@@ -9271,19 +9331,39 @@
       </c>
     </row>
     <row r="159">
-      <c r="A159" s="23" t="n"/>
-      <c r="B159" s="23" t="n"/>
-      <c r="C159" s="23" t="n"/>
-      <c r="D159" s="24" t="n"/>
-      <c r="E159" s="25" t="n"/>
-      <c r="F159" s="26" t="n"/>
-      <c r="G159" s="24" t="n"/>
-      <c r="H159" s="25" t="n"/>
+      <c r="A159" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-221260916649109</t>
+        </is>
+      </c>
+      <c r="B159" s="23" t="inlineStr">
+        <is>
+          <t>NPST</t>
+        </is>
+      </c>
+      <c r="C159" s="23" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="D159" s="24" t="n">
+        <v>46281</v>
+      </c>
+      <c r="E159" s="25" t="n">
+        <v>1848.2214</v>
+      </c>
+      <c r="F159" s="26" t="n">
+        <v>135</v>
+      </c>
+      <c r="G159" s="24" t="inlineStr"/>
+      <c r="H159" s="25" t="inlineStr"/>
       <c r="I159" s="21">
         <f>IF(OR($B159="",$H159=""),"",IF($C159="LONG",($H159-$E159)*$F159,($E159-$H159)*$F159))</f>
         <v/>
       </c>
-      <c r="J159" s="4" t="n"/>
+      <c r="J159" s="4" t="n">
+        <v>370.02</v>
+      </c>
       <c r="K159" s="21">
         <f>IF(OR($B159="",$I159=""),"",$I159-IF($J159="",0,$J159))</f>
         <v/>
@@ -9298,19 +9378,39 @@
       </c>
     </row>
     <row r="160">
-      <c r="A160" s="23" t="n"/>
-      <c r="B160" s="23" t="n"/>
-      <c r="C160" s="23" t="n"/>
-      <c r="D160" s="24" t="n"/>
-      <c r="E160" s="25" t="n"/>
-      <c r="F160" s="26" t="n"/>
-      <c r="G160" s="24" t="n"/>
-      <c r="H160" s="25" t="n"/>
+      <c r="A160" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-34126091663809</t>
+        </is>
+      </c>
+      <c r="B160" s="23" t="inlineStr">
+        <is>
+          <t>ROSSTECH</t>
+        </is>
+      </c>
+      <c r="C160" s="23" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="D160" s="24" t="n">
+        <v>46281</v>
+      </c>
+      <c r="E160" s="25" t="n">
+        <v>1340.8882</v>
+      </c>
+      <c r="F160" s="26" t="n">
+        <v>186</v>
+      </c>
+      <c r="G160" s="24" t="inlineStr"/>
+      <c r="H160" s="25" t="inlineStr"/>
       <c r="I160" s="21">
         <f>IF(OR($B160="",$H160=""),"",IF($C160="LONG",($H160-$E160)*$F160,($E160-$H160)*$F160))</f>
         <v/>
       </c>
-      <c r="J160" s="4" t="n"/>
+      <c r="J160" s="4" t="n">
+        <v>369.89</v>
+      </c>
       <c r="K160" s="21">
         <f>IF(OR($B160="",$I160=""),"",$I160-IF($J160="",0,$J160))</f>
         <v/>
@@ -9325,19 +9425,39 @@
       </c>
     </row>
     <row r="161">
-      <c r="A161" s="23" t="n"/>
-      <c r="B161" s="23" t="n"/>
-      <c r="C161" s="23" t="n"/>
-      <c r="D161" s="24" t="n"/>
-      <c r="E161" s="25" t="n"/>
-      <c r="F161" s="26" t="n"/>
-      <c r="G161" s="24" t="n"/>
-      <c r="H161" s="25" t="n"/>
+      <c r="A161" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-221260916649309</t>
+        </is>
+      </c>
+      <c r="B161" s="23" t="inlineStr">
+        <is>
+          <t>SAATVIKGL</t>
+        </is>
+      </c>
+      <c r="C161" s="23" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="D161" s="24" t="n">
+        <v>46281</v>
+      </c>
+      <c r="E161" s="25" t="n">
+        <v>414.316</v>
+      </c>
+      <c r="F161" s="26" t="n">
+        <v>603</v>
+      </c>
+      <c r="G161" s="24" t="inlineStr"/>
+      <c r="H161" s="25" t="inlineStr"/>
       <c r="I161" s="21">
         <f>IF(OR($B161="",$H161=""),"",IF($C161="LONG",($H161-$E161)*$F161,($E161-$H161)*$F161))</f>
         <v/>
       </c>
-      <c r="J161" s="4" t="n"/>
+      <c r="J161" s="4" t="n">
+        <v>370.4</v>
+      </c>
       <c r="K161" s="21">
         <f>IF(OR($B161="",$I161=""),"",$I161-IF($J161="",0,$J161))</f>
         <v/>
@@ -32516,7 +32636,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J76"/>
+  <dimension ref="A1:J82"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -33073,7 +33193,7 @@
     <row r="15">
       <c r="A15" s="27" t="inlineStr">
         <is>
-          <t>FILATEX</t>
+          <t>EMUDHRA</t>
         </is>
       </c>
       <c r="B15" s="20">
@@ -33116,7 +33236,7 @@
     <row r="16">
       <c r="A16" s="27" t="inlineStr">
         <is>
-          <t>FMGOETZE</t>
+          <t>FILATEX</t>
         </is>
       </c>
       <c r="B16" s="20">
@@ -33159,7 +33279,7 @@
     <row r="17">
       <c r="A17" s="27" t="inlineStr">
         <is>
-          <t>GKENERGY</t>
+          <t>FMGOETZE</t>
         </is>
       </c>
       <c r="B17" s="20">
@@ -33202,7 +33322,7 @@
     <row r="18">
       <c r="A18" s="27" t="inlineStr">
         <is>
-          <t>GNRL</t>
+          <t>FOSECOIND</t>
         </is>
       </c>
       <c r="B18" s="20">
@@ -33245,7 +33365,7 @@
     <row r="19">
       <c r="A19" s="27" t="inlineStr">
         <is>
-          <t>GOCLCORP</t>
+          <t>GKENERGY</t>
         </is>
       </c>
       <c r="B19" s="20">
@@ -33288,7 +33408,7 @@
     <row r="20">
       <c r="A20" s="27" t="inlineStr">
         <is>
-          <t>GOPAL</t>
+          <t>GNRL</t>
         </is>
       </c>
       <c r="B20" s="20">
@@ -33331,7 +33451,7 @@
     <row r="21">
       <c r="A21" s="27" t="inlineStr">
         <is>
-          <t>GUJTHEM</t>
+          <t>GOCLCORP</t>
         </is>
       </c>
       <c r="B21" s="20">
@@ -33374,7 +33494,7 @@
     <row r="22">
       <c r="A22" s="27" t="inlineStr">
         <is>
-          <t>HERITGFOOD</t>
+          <t>GOPAL</t>
         </is>
       </c>
       <c r="B22" s="20">
@@ -33417,7 +33537,7 @@
     <row r="23">
       <c r="A23" s="27" t="inlineStr">
         <is>
-          <t>HIKAL</t>
+          <t>GUJTHEM</t>
         </is>
       </c>
       <c r="B23" s="20">
@@ -33460,7 +33580,7 @@
     <row r="24">
       <c r="A24" s="27" t="inlineStr">
         <is>
-          <t>HINDOILEXP</t>
+          <t>HERITGFOOD</t>
         </is>
       </c>
       <c r="B24" s="20">
@@ -33503,7 +33623,7 @@
     <row r="25">
       <c r="A25" s="27" t="inlineStr">
         <is>
-          <t>HUBTOWN</t>
+          <t>HIKAL</t>
         </is>
       </c>
       <c r="B25" s="20">
@@ -33546,7 +33666,7 @@
     <row r="26">
       <c r="A26" s="27" t="inlineStr">
         <is>
-          <t>INDNIPPON</t>
+          <t>HINDOILEXP</t>
         </is>
       </c>
       <c r="B26" s="20">
@@ -33589,7 +33709,7 @@
     <row r="27">
       <c r="A27" s="27" t="inlineStr">
         <is>
-          <t>INDOCO</t>
+          <t>HUBTOWN</t>
         </is>
       </c>
       <c r="B27" s="20">
@@ -33632,7 +33752,7 @@
     <row r="28">
       <c r="A28" s="27" t="inlineStr">
         <is>
-          <t>INDORAMA</t>
+          <t>INDNIPPON</t>
         </is>
       </c>
       <c r="B28" s="20">
@@ -33675,7 +33795,7 @@
     <row r="29">
       <c r="A29" s="27" t="inlineStr">
         <is>
-          <t>JGCHEM</t>
+          <t>INDOCO</t>
         </is>
       </c>
       <c r="B29" s="20">
@@ -33718,7 +33838,7 @@
     <row r="30">
       <c r="A30" s="27" t="inlineStr">
         <is>
-          <t>KCP</t>
+          <t>INDORAMA</t>
         </is>
       </c>
       <c r="B30" s="20">
@@ -33761,7 +33881,7 @@
     <row r="31">
       <c r="A31" s="27" t="inlineStr">
         <is>
-          <t>KIRIINDUS</t>
+          <t>IPL</t>
         </is>
       </c>
       <c r="B31" s="20">
@@ -33804,7 +33924,7 @@
     <row r="32">
       <c r="A32" s="27" t="inlineStr">
         <is>
-          <t>KIRLOSIND</t>
+          <t>JGCHEM</t>
         </is>
       </c>
       <c r="B32" s="20">
@@ -33847,7 +33967,7 @@
     <row r="33">
       <c r="A33" s="27" t="inlineStr">
         <is>
-          <t>KLBRENG-B</t>
+          <t>KCP</t>
         </is>
       </c>
       <c r="B33" s="20">
@@ -33890,7 +34010,7 @@
     <row r="34">
       <c r="A34" s="27" t="inlineStr">
         <is>
-          <t>KSL</t>
+          <t>KIRIINDUS</t>
         </is>
       </c>
       <c r="B34" s="20">
@@ -33933,7 +34053,7 @@
     <row r="35">
       <c r="A35" s="27" t="inlineStr">
         <is>
-          <t>MAITHANALL</t>
+          <t>KIRLOSIND</t>
         </is>
       </c>
       <c r="B35" s="20">
@@ -33976,7 +34096,7 @@
     <row r="36">
       <c r="A36" s="27" t="inlineStr">
         <is>
-          <t>MANGLMCEM</t>
+          <t>KLBRENG-B</t>
         </is>
       </c>
       <c r="B36" s="20">
@@ -34019,7 +34139,7 @@
     <row r="37">
       <c r="A37" s="27" t="inlineStr">
         <is>
-          <t>MASTEK</t>
+          <t>KSL</t>
         </is>
       </c>
       <c r="B37" s="20">
@@ -34062,7 +34182,7 @@
     <row r="38">
       <c r="A38" s="27" t="inlineStr">
         <is>
-          <t>MOBIKWIK</t>
+          <t>MAITHANALL</t>
         </is>
       </c>
       <c r="B38" s="20">
@@ -34105,7 +34225,7 @@
     <row r="39">
       <c r="A39" s="27" t="inlineStr">
         <is>
-          <t>NETWORK18</t>
+          <t>MANGLMCEM</t>
         </is>
       </c>
       <c r="B39" s="20">
@@ -34148,7 +34268,7 @@
     <row r="40">
       <c r="A40" s="27" t="inlineStr">
         <is>
-          <t>NILKAMAL</t>
+          <t>MASTEK</t>
         </is>
       </c>
       <c r="B40" s="20">
@@ -34191,7 +34311,7 @@
     <row r="41">
       <c r="A41" s="27" t="inlineStr">
         <is>
-          <t>NORTHARC</t>
+          <t>MOBIKWIK</t>
         </is>
       </c>
       <c r="B41" s="20">
@@ -34234,7 +34354,7 @@
     <row r="42">
       <c r="A42" s="27" t="inlineStr">
         <is>
-          <t>NOVARTIND</t>
+          <t>NETWORK18</t>
         </is>
       </c>
       <c r="B42" s="20">
@@ -34277,7 +34397,7 @@
     <row r="43">
       <c r="A43" s="27" t="inlineStr">
         <is>
-          <t>OMAXE</t>
+          <t>NILKAMAL</t>
         </is>
       </c>
       <c r="B43" s="20">
@@ -34320,7 +34440,7 @@
     <row r="44">
       <c r="A44" s="27" t="inlineStr">
         <is>
-          <t>OPTIEMUS</t>
+          <t>NORTHARC</t>
         </is>
       </c>
       <c r="B44" s="20">
@@ -34363,7 +34483,7 @@
     <row r="45">
       <c r="A45" s="27" t="inlineStr">
         <is>
-          <t>ORIENTHOT</t>
+          <t>NOVARTIND</t>
         </is>
       </c>
       <c r="B45" s="20">
@@ -34406,7 +34526,7 @@
     <row r="46">
       <c r="A46" s="27" t="inlineStr">
         <is>
-          <t>PITTIENG</t>
+          <t>NPST</t>
         </is>
       </c>
       <c r="B46" s="20">
@@ -34449,7 +34569,7 @@
     <row r="47">
       <c r="A47" s="27" t="inlineStr">
         <is>
-          <t>QUADFUTURE</t>
+          <t>OMAXE</t>
         </is>
       </c>
       <c r="B47" s="20">
@@ -34492,7 +34612,7 @@
     <row r="48">
       <c r="A48" s="27" t="inlineStr">
         <is>
-          <t>RACLGEAR</t>
+          <t>OPTIEMUS</t>
         </is>
       </c>
       <c r="B48" s="20">
@@ -34535,7 +34655,7 @@
     <row r="49">
       <c r="A49" s="27" t="inlineStr">
         <is>
-          <t>RAMRAT</t>
+          <t>ORIENTHOT</t>
         </is>
       </c>
       <c r="B49" s="20">
@@ -34578,7 +34698,7 @@
     <row r="50">
       <c r="A50" s="27" t="inlineStr">
         <is>
-          <t>RAYMOND</t>
+          <t>PITTIENG</t>
         </is>
       </c>
       <c r="B50" s="20">
@@ -34621,7 +34741,7 @@
     <row r="51">
       <c r="A51" s="27" t="inlineStr">
         <is>
-          <t>RESPONIND</t>
+          <t>QUADFUTURE</t>
         </is>
       </c>
       <c r="B51" s="20">
@@ -34664,7 +34784,7 @@
     <row r="52">
       <c r="A52" s="27" t="inlineStr">
         <is>
-          <t>RML</t>
+          <t>RACLGEAR</t>
         </is>
       </c>
       <c r="B52" s="20">
@@ -34707,7 +34827,7 @@
     <row r="53">
       <c r="A53" s="27" t="inlineStr">
         <is>
-          <t>SAKAR</t>
+          <t>RAMRAT</t>
         </is>
       </c>
       <c r="B53" s="20">
@@ -34750,7 +34870,7 @@
     <row r="54">
       <c r="A54" s="27" t="inlineStr">
         <is>
-          <t>SAMHI</t>
+          <t>RAYMOND</t>
         </is>
       </c>
       <c r="B54" s="20">
@@ -34793,7 +34913,7 @@
     <row r="55">
       <c r="A55" s="27" t="inlineStr">
         <is>
-          <t>SHAREINDIA</t>
+          <t>RESPONIND</t>
         </is>
       </c>
       <c r="B55" s="20">
@@ -34836,7 +34956,7 @@
     <row r="56">
       <c r="A56" s="27" t="inlineStr">
         <is>
-          <t>SIKA</t>
+          <t>RML</t>
         </is>
       </c>
       <c r="B56" s="20">
@@ -34879,7 +34999,7 @@
     <row r="57">
       <c r="A57" s="27" t="inlineStr">
         <is>
-          <t>SINDHUTRAD</t>
+          <t>ROSSTECH</t>
         </is>
       </c>
       <c r="B57" s="20">
@@ -34922,7 +35042,7 @@
     <row r="58">
       <c r="A58" s="27" t="inlineStr">
         <is>
-          <t>SMSPHARMA</t>
+          <t>SAATVIKGL</t>
         </is>
       </c>
       <c r="B58" s="20">
@@ -34965,7 +35085,7 @@
     <row r="59">
       <c r="A59" s="27" t="inlineStr">
         <is>
-          <t>SOLARA</t>
+          <t>SAKAR</t>
         </is>
       </c>
       <c r="B59" s="20">
@@ -35008,7 +35128,7 @@
     <row r="60">
       <c r="A60" s="27" t="inlineStr">
         <is>
-          <t>SOTL</t>
+          <t>SAMHI</t>
         </is>
       </c>
       <c r="B60" s="20">
@@ -35051,7 +35171,7 @@
     <row r="61">
       <c r="A61" s="27" t="inlineStr">
         <is>
-          <t>SSWL</t>
+          <t>SHAREINDIA</t>
         </is>
       </c>
       <c r="B61" s="20">
@@ -35094,7 +35214,7 @@
     <row r="62">
       <c r="A62" s="27" t="inlineStr">
         <is>
-          <t>SYMPHONY</t>
+          <t>SIKA</t>
         </is>
       </c>
       <c r="B62" s="20">
@@ -35137,7 +35257,7 @@
     <row r="63">
       <c r="A63" s="27" t="inlineStr">
         <is>
-          <t>SYNCOMF</t>
+          <t>SINDHUTRAD</t>
         </is>
       </c>
       <c r="B63" s="20">
@@ -35180,7 +35300,7 @@
     <row r="64">
       <c r="A64" s="27" t="inlineStr">
         <is>
-          <t>TALBROAUTO</t>
+          <t>SMSPHARMA</t>
         </is>
       </c>
       <c r="B64" s="20">
@@ -35223,7 +35343,7 @@
     <row r="65">
       <c r="A65" s="27" t="inlineStr">
         <is>
-          <t>TBZ</t>
+          <t>SOLARA</t>
         </is>
       </c>
       <c r="B65" s="20">
@@ -35266,7 +35386,7 @@
     <row r="66">
       <c r="A66" s="27" t="inlineStr">
         <is>
-          <t>THOMASCOOK</t>
+          <t>SOTL</t>
         </is>
       </c>
       <c r="B66" s="20">
@@ -35309,7 +35429,7 @@
     <row r="67">
       <c r="A67" s="27" t="inlineStr">
         <is>
-          <t>VENKEYS</t>
+          <t>SSWL</t>
         </is>
       </c>
       <c r="B67" s="20">
@@ -35352,7 +35472,7 @@
     <row r="68">
       <c r="A68" s="27" t="inlineStr">
         <is>
-          <t>VENUSPIPES</t>
+          <t>SYMPHONY</t>
         </is>
       </c>
       <c r="B68" s="20">
@@ -35395,7 +35515,7 @@
     <row r="69">
       <c r="A69" s="27" t="inlineStr">
         <is>
-          <t>VERANDA</t>
+          <t>SYNCOMF</t>
         </is>
       </c>
       <c r="B69" s="20">
@@ -35438,7 +35558,7 @@
     <row r="70">
       <c r="A70" s="27" t="inlineStr">
         <is>
-          <t>VSSL</t>
+          <t>TALBROAUTO</t>
         </is>
       </c>
       <c r="B70" s="20">
@@ -35481,7 +35601,7 @@
     <row r="71">
       <c r="A71" s="27" t="inlineStr">
         <is>
-          <t>WELSPLSOL</t>
+          <t>TBZ</t>
         </is>
       </c>
       <c r="B71" s="20">
@@ -35524,7 +35644,7 @@
     <row r="72">
       <c r="A72" s="27" t="inlineStr">
         <is>
-          <t>WENDT</t>
+          <t>THOMASCOOK</t>
         </is>
       </c>
       <c r="B72" s="20">
@@ -35567,7 +35687,7 @@
     <row r="73">
       <c r="A73" s="27" t="inlineStr">
         <is>
-          <t>WINDLAS</t>
+          <t>VENKEYS</t>
         </is>
       </c>
       <c r="B73" s="20">
@@ -35610,7 +35730,7 @@
     <row r="74">
       <c r="A74" s="27" t="inlineStr">
         <is>
-          <t>XPROINDIA</t>
+          <t>VENUSPIPES</t>
         </is>
       </c>
       <c r="B74" s="20">
@@ -35653,7 +35773,7 @@
     <row r="75">
       <c r="A75" s="27" t="inlineStr">
         <is>
-          <t>ZAGGLE</t>
+          <t>VERANDA</t>
         </is>
       </c>
       <c r="B75" s="20">
@@ -35694,37 +35814,295 @@
       </c>
     </row>
     <row r="76">
-      <c r="A76" s="3" t="inlineStr">
+      <c r="A76" s="27" t="inlineStr">
+        <is>
+          <t>VSSL</t>
+        </is>
+      </c>
+      <c r="B76" s="20">
+        <f>COUNTIF('Trade Log'!$B$4:$B$503,$A76)</f>
+        <v/>
+      </c>
+      <c r="C76" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A76,'Trade Log'!$K$4:$K$503,"&gt;0")</f>
+        <v/>
+      </c>
+      <c r="D76" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A76,'Trade Log'!$K$4:$K$503,"&lt;0")</f>
+        <v/>
+      </c>
+      <c r="E76" s="29">
+        <f>IFERROR($C76/$B76,"")</f>
+        <v/>
+      </c>
+      <c r="F76" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A76,'Trade Log'!$I$4:$I$503)</f>
+        <v/>
+      </c>
+      <c r="G76" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A76,'Trade Log'!$K$4:$K$503)</f>
+        <v/>
+      </c>
+      <c r="H76" s="21">
+        <f>IFERROR($G76/$B76,"")</f>
+        <v/>
+      </c>
+      <c r="I76" s="21">
+        <f>IFERROR(_xlfn.MAXIFS('Trade Log'!$K$4:$K$503,'Trade Log'!$B$4:$B$503,$A76),"")</f>
+        <v/>
+      </c>
+      <c r="J76" s="21">
+        <f>IFERROR(_xlfn.MINIFS('Trade Log'!$K$4:$K$503,'Trade Log'!$B$4:$B$503,$A76),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="27" t="inlineStr">
+        <is>
+          <t>WELSPLSOL</t>
+        </is>
+      </c>
+      <c r="B77" s="20">
+        <f>COUNTIF('Trade Log'!$B$4:$B$503,$A77)</f>
+        <v/>
+      </c>
+      <c r="C77" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A77,'Trade Log'!$K$4:$K$503,"&gt;0")</f>
+        <v/>
+      </c>
+      <c r="D77" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A77,'Trade Log'!$K$4:$K$503,"&lt;0")</f>
+        <v/>
+      </c>
+      <c r="E77" s="29">
+        <f>IFERROR($C77/$B77,"")</f>
+        <v/>
+      </c>
+      <c r="F77" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A77,'Trade Log'!$I$4:$I$503)</f>
+        <v/>
+      </c>
+      <c r="G77" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A77,'Trade Log'!$K$4:$K$503)</f>
+        <v/>
+      </c>
+      <c r="H77" s="21">
+        <f>IFERROR($G77/$B77,"")</f>
+        <v/>
+      </c>
+      <c r="I77" s="21">
+        <f>IFERROR(_xlfn.MAXIFS('Trade Log'!$K$4:$K$503,'Trade Log'!$B$4:$B$503,$A77),"")</f>
+        <v/>
+      </c>
+      <c r="J77" s="21">
+        <f>IFERROR(_xlfn.MINIFS('Trade Log'!$K$4:$K$503,'Trade Log'!$B$4:$B$503,$A77),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="27" t="inlineStr">
+        <is>
+          <t>WENDT</t>
+        </is>
+      </c>
+      <c r="B78" s="20">
+        <f>COUNTIF('Trade Log'!$B$4:$B$503,$A78)</f>
+        <v/>
+      </c>
+      <c r="C78" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A78,'Trade Log'!$K$4:$K$503,"&gt;0")</f>
+        <v/>
+      </c>
+      <c r="D78" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A78,'Trade Log'!$K$4:$K$503,"&lt;0")</f>
+        <v/>
+      </c>
+      <c r="E78" s="29">
+        <f>IFERROR($C78/$B78,"")</f>
+        <v/>
+      </c>
+      <c r="F78" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A78,'Trade Log'!$I$4:$I$503)</f>
+        <v/>
+      </c>
+      <c r="G78" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A78,'Trade Log'!$K$4:$K$503)</f>
+        <v/>
+      </c>
+      <c r="H78" s="21">
+        <f>IFERROR($G78/$B78,"")</f>
+        <v/>
+      </c>
+      <c r="I78" s="21">
+        <f>IFERROR(_xlfn.MAXIFS('Trade Log'!$K$4:$K$503,'Trade Log'!$B$4:$B$503,$A78),"")</f>
+        <v/>
+      </c>
+      <c r="J78" s="21">
+        <f>IFERROR(_xlfn.MINIFS('Trade Log'!$K$4:$K$503,'Trade Log'!$B$4:$B$503,$A78),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="27" t="inlineStr">
+        <is>
+          <t>WINDLAS</t>
+        </is>
+      </c>
+      <c r="B79" s="20">
+        <f>COUNTIF('Trade Log'!$B$4:$B$503,$A79)</f>
+        <v/>
+      </c>
+      <c r="C79" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A79,'Trade Log'!$K$4:$K$503,"&gt;0")</f>
+        <v/>
+      </c>
+      <c r="D79" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A79,'Trade Log'!$K$4:$K$503,"&lt;0")</f>
+        <v/>
+      </c>
+      <c r="E79" s="29">
+        <f>IFERROR($C79/$B79,"")</f>
+        <v/>
+      </c>
+      <c r="F79" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A79,'Trade Log'!$I$4:$I$503)</f>
+        <v/>
+      </c>
+      <c r="G79" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A79,'Trade Log'!$K$4:$K$503)</f>
+        <v/>
+      </c>
+      <c r="H79" s="21">
+        <f>IFERROR($G79/$B79,"")</f>
+        <v/>
+      </c>
+      <c r="I79" s="21">
+        <f>IFERROR(_xlfn.MAXIFS('Trade Log'!$K$4:$K$503,'Trade Log'!$B$4:$B$503,$A79),"")</f>
+        <v/>
+      </c>
+      <c r="J79" s="21">
+        <f>IFERROR(_xlfn.MINIFS('Trade Log'!$K$4:$K$503,'Trade Log'!$B$4:$B$503,$A79),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="27" t="inlineStr">
+        <is>
+          <t>XPROINDIA</t>
+        </is>
+      </c>
+      <c r="B80" s="20">
+        <f>COUNTIF('Trade Log'!$B$4:$B$503,$A80)</f>
+        <v/>
+      </c>
+      <c r="C80" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A80,'Trade Log'!$K$4:$K$503,"&gt;0")</f>
+        <v/>
+      </c>
+      <c r="D80" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A80,'Trade Log'!$K$4:$K$503,"&lt;0")</f>
+        <v/>
+      </c>
+      <c r="E80" s="29">
+        <f>IFERROR($C80/$B80,"")</f>
+        <v/>
+      </c>
+      <c r="F80" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A80,'Trade Log'!$I$4:$I$503)</f>
+        <v/>
+      </c>
+      <c r="G80" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A80,'Trade Log'!$K$4:$K$503)</f>
+        <v/>
+      </c>
+      <c r="H80" s="21">
+        <f>IFERROR($G80/$B80,"")</f>
+        <v/>
+      </c>
+      <c r="I80" s="21">
+        <f>IFERROR(_xlfn.MAXIFS('Trade Log'!$K$4:$K$503,'Trade Log'!$B$4:$B$503,$A80),"")</f>
+        <v/>
+      </c>
+      <c r="J80" s="21">
+        <f>IFERROR(_xlfn.MINIFS('Trade Log'!$K$4:$K$503,'Trade Log'!$B$4:$B$503,$A80),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="27" t="inlineStr">
+        <is>
+          <t>ZAGGLE</t>
+        </is>
+      </c>
+      <c r="B81" s="20">
+        <f>COUNTIF('Trade Log'!$B$4:$B$503,$A81)</f>
+        <v/>
+      </c>
+      <c r="C81" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A81,'Trade Log'!$K$4:$K$503,"&gt;0")</f>
+        <v/>
+      </c>
+      <c r="D81" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A81,'Trade Log'!$K$4:$K$503,"&lt;0")</f>
+        <v/>
+      </c>
+      <c r="E81" s="29">
+        <f>IFERROR($C81/$B81,"")</f>
+        <v/>
+      </c>
+      <c r="F81" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A81,'Trade Log'!$I$4:$I$503)</f>
+        <v/>
+      </c>
+      <c r="G81" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A81,'Trade Log'!$K$4:$K$503)</f>
+        <v/>
+      </c>
+      <c r="H81" s="21">
+        <f>IFERROR($G81/$B81,"")</f>
+        <v/>
+      </c>
+      <c r="I81" s="21">
+        <f>IFERROR(_xlfn.MAXIFS('Trade Log'!$K$4:$K$503,'Trade Log'!$B$4:$B$503,$A81),"")</f>
+        <v/>
+      </c>
+      <c r="J81" s="21">
+        <f>IFERROR(_xlfn.MINIFS('Trade Log'!$K$4:$K$503,'Trade Log'!$B$4:$B$503,$A81),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="3" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="B76" s="30">
-        <f>SUM(B4:B75)</f>
-        <v/>
-      </c>
-      <c r="C76" s="30">
-        <f>SUM(C4:C75)</f>
-        <v/>
-      </c>
-      <c r="D76" s="30">
-        <f>SUM(D4:D75)</f>
-        <v/>
-      </c>
-      <c r="E76" s="31">
-        <f>IFERROR(C76/B76,"")</f>
-        <v/>
-      </c>
-      <c r="F76" s="32">
-        <f>SUM(F4:F75)</f>
-        <v/>
-      </c>
-      <c r="G76" s="32">
-        <f>SUM(G4:G75)</f>
-        <v/>
-      </c>
-      <c r="H76" s="32">
-        <f>IFERROR(G76/B76,"")</f>
+      <c r="B82" s="30">
+        <f>SUM(B4:B81)</f>
+        <v/>
+      </c>
+      <c r="C82" s="30">
+        <f>SUM(C4:C81)</f>
+        <v/>
+      </c>
+      <c r="D82" s="30">
+        <f>SUM(D4:D81)</f>
+        <v/>
+      </c>
+      <c r="E82" s="31">
+        <f>IFERROR(C82/B82,"")</f>
+        <v/>
+      </c>
+      <c r="F82" s="32">
+        <f>SUM(F4:F81)</f>
+        <v/>
+      </c>
+      <c r="G82" s="32">
+        <f>SUM(G4:G81)</f>
+        <v/>
+      </c>
+      <c r="H82" s="32">
+        <f>IFERROR(G82/B82,"")</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Drop estimated leg-charge fallback, use real trade-book API only
Charges without a real broker figure now report 0.0/"pending" instead of
a rate-card estimate, so P&L never shows a guessed number as if it were
final. Also abandons the Google Sheets sync experiment (script,
credentials, gitignore rules, and the run_trades.py hook) — reverting
to xlsx-only output.
</commit_message>
<xml_diff>
--- a/results/strategy_pnl_simple.xlsx
+++ b/results/strategy_pnl_simple.xlsx
@@ -9221,7 +9221,7 @@
         <v/>
       </c>
       <c r="J156" s="4" t="n">
-        <v>371.72</v>
+        <v>50.15</v>
       </c>
       <c r="K156" s="21">
         <f>IF(OR($B156="",$I156=""),"",$I156-IF($J156="",0,$J156))</f>
@@ -9268,7 +9268,7 @@
         <v/>
       </c>
       <c r="J157" s="4" t="n">
-        <v>371.57</v>
+        <v>50.15</v>
       </c>
       <c r="K157" s="21">
         <f>IF(OR($B157="",$I157=""),"",$I157-IF($J157="",0,$J157))</f>
@@ -9315,7 +9315,7 @@
         <v/>
       </c>
       <c r="J158" s="4" t="n">
-        <v>371.46</v>
+        <v>50.15</v>
       </c>
       <c r="K158" s="21">
         <f>IF(OR($B158="",$I158=""),"",$I158-IF($J158="",0,$J158))</f>
@@ -9362,7 +9362,7 @@
         <v/>
       </c>
       <c r="J159" s="4" t="n">
-        <v>370.02</v>
+        <v>50.15</v>
       </c>
       <c r="K159" s="21">
         <f>IF(OR($B159="",$I159=""),"",$I159-IF($J159="",0,$J159))</f>
@@ -9409,7 +9409,7 @@
         <v/>
       </c>
       <c r="J160" s="4" t="n">
-        <v>369.89</v>
+        <v>50.15</v>
       </c>
       <c r="K160" s="21">
         <f>IF(OR($B160="",$I160=""),"",$I160-IF($J160="",0,$J160))</f>
@@ -9456,7 +9456,7 @@
         <v/>
       </c>
       <c r="J161" s="4" t="n">
-        <v>370.4</v>
+        <v>50.15</v>
       </c>
       <c r="K161" s="21">
         <f>IF(OR($B161="",$I161=""),"",$I161-IF($J161="",0,$J161))</f>

</xml_diff>

<commit_message>
Data update — 2026-09-17 candle + results refresh
</commit_message>
<xml_diff>
--- a/results/strategy_pnl_simple.xlsx
+++ b/results/strategy_pnl_simple.xlsx
@@ -1473,7 +1473,7 @@
         <v/>
       </c>
       <c r="J4" s="4" t="n">
-        <v>571.85</v>
+        <v>571.8200000000001</v>
       </c>
       <c r="K4" s="21">
         <f>IF(OR($B4="",$I4=""),"",$I4-IF($J4="",0,$J4))</f>
@@ -1524,7 +1524,7 @@
         <v/>
       </c>
       <c r="J5" s="4" t="n">
-        <v>688.88</v>
+        <v>688.84</v>
       </c>
       <c r="K5" s="21">
         <f>IF(OR($B5="",$I5=""),"",$I5-IF($J5="",0,$J5))</f>
@@ -1575,7 +1575,7 @@
         <v/>
       </c>
       <c r="J6" s="4" t="n">
-        <v>570.6900000000001</v>
+        <v>570.67</v>
       </c>
       <c r="K6" s="21">
         <f>IF(OR($B6="",$I6=""),"",$I6-IF($J6="",0,$J6))</f>
@@ -1626,7 +1626,7 @@
         <v/>
       </c>
       <c r="J7" s="4" t="n">
-        <v>663.11</v>
+        <v>663.08</v>
       </c>
       <c r="K7" s="21">
         <f>IF(OR($B7="",$I7=""),"",$I7-IF($J7="",0,$J7))</f>
@@ -1677,7 +1677,7 @@
         <v/>
       </c>
       <c r="J8" s="4" t="n">
-        <v>590.76</v>
+        <v>590.88</v>
       </c>
       <c r="K8" s="21">
         <f>IF(OR($B8="",$I8=""),"",$I8-IF($J8="",0,$J8))</f>
@@ -1779,7 +1779,7 @@
         <v/>
       </c>
       <c r="J10" s="4" t="n">
-        <v>398.65</v>
+        <v>398.63</v>
       </c>
       <c r="K10" s="21">
         <f>IF(OR($B10="",$I10=""),"",$I10-IF($J10="",0,$J10))</f>
@@ -1881,7 +1881,7 @@
         <v/>
       </c>
       <c r="J12" s="4" t="n">
-        <v>414.2</v>
+        <v>414.18</v>
       </c>
       <c r="K12" s="21">
         <f>IF(OR($B12="",$I12=""),"",$I12-IF($J12="",0,$J12))</f>
@@ -1932,7 +1932,7 @@
         <v/>
       </c>
       <c r="J13" s="4" t="n">
-        <v>345.09</v>
+        <v>345.08</v>
       </c>
       <c r="K13" s="21">
         <f>IF(OR($B13="",$I13=""),"",$I13-IF($J13="",0,$J13))</f>
@@ -1983,7 +1983,7 @@
         <v/>
       </c>
       <c r="J14" s="4" t="n">
-        <v>414.53</v>
+        <v>414.51</v>
       </c>
       <c r="K14" s="21">
         <f>IF(OR($B14="",$I14=""),"",$I14-IF($J14="",0,$J14))</f>
@@ -2034,7 +2034,7 @@
         <v/>
       </c>
       <c r="J15" s="4" t="n">
-        <v>380.34</v>
+        <v>380.37</v>
       </c>
       <c r="K15" s="21">
         <f>IF(OR($B15="",$I15=""),"",$I15-IF($J15="",0,$J15))</f>
@@ -2187,7 +2187,7 @@
         <v/>
       </c>
       <c r="J18" s="4" t="n">
-        <v>413.96</v>
+        <v>413.94</v>
       </c>
       <c r="K18" s="21">
         <f>IF(OR($B18="",$I18=""),"",$I18-IF($J18="",0,$J18))</f>
@@ -2238,7 +2238,7 @@
         <v/>
       </c>
       <c r="J19" s="4" t="n">
-        <v>406.49</v>
+        <v>406.47</v>
       </c>
       <c r="K19" s="21">
         <f>IF(OR($B19="",$I19=""),"",$I19-IF($J19="",0,$J19))</f>
@@ -2697,7 +2697,7 @@
         <v/>
       </c>
       <c r="J28" s="4" t="n">
-        <v>870.13</v>
+        <v>870.25</v>
       </c>
       <c r="K28" s="21">
         <f>IF(OR($B28="",$I28=""),"",$I28-IF($J28="",0,$J28))</f>
@@ -2850,7 +2850,7 @@
         <v/>
       </c>
       <c r="J31" s="4" t="n">
-        <v>391.16</v>
+        <v>391.15</v>
       </c>
       <c r="K31" s="21">
         <f>IF(OR($B31="",$I31=""),"",$I31-IF($J31="",0,$J31))</f>
@@ -2901,7 +2901,7 @@
         <v/>
       </c>
       <c r="J32" s="4" t="n">
-        <v>349.78</v>
+        <v>349.77</v>
       </c>
       <c r="K32" s="21">
         <f>IF(OR($B32="",$I32=""),"",$I32-IF($J32="",0,$J32))</f>
@@ -3003,7 +3003,7 @@
         <v/>
       </c>
       <c r="J34" s="4" t="n">
-        <v>349.78</v>
+        <v>349.8</v>
       </c>
       <c r="K34" s="21">
         <f>IF(OR($B34="",$I34=""),"",$I34-IF($J34="",0,$J34))</f>
@@ -3054,7 +3054,7 @@
         <v/>
       </c>
       <c r="J35" s="4" t="n">
-        <v>386.15</v>
+        <v>386.17</v>
       </c>
       <c r="K35" s="21">
         <f>IF(OR($B35="",$I35=""),"",$I35-IF($J35="",0,$J35))</f>
@@ -3411,7 +3411,7 @@
         <v/>
       </c>
       <c r="J42" s="4" t="n">
-        <v>978.29</v>
+        <v>978.26</v>
       </c>
       <c r="K42" s="21">
         <f>IF(OR($B42="",$I42=""),"",$I42-IF($J42="",0,$J42))</f>
@@ -3462,7 +3462,7 @@
         <v/>
       </c>
       <c r="J43" s="4" t="n">
-        <v>957.6799999999999</v>
+        <v>957.66</v>
       </c>
       <c r="K43" s="21">
         <f>IF(OR($B43="",$I43=""),"",$I43-IF($J43="",0,$J43))</f>
@@ -3513,7 +3513,7 @@
         <v/>
       </c>
       <c r="J44" s="4" t="n">
-        <v>992.28</v>
+        <v>992.26</v>
       </c>
       <c r="K44" s="21">
         <f>IF(OR($B44="",$I44=""),"",$I44-IF($J44="",0,$J44))</f>
@@ -3564,7 +3564,7 @@
         <v/>
       </c>
       <c r="J45" s="4" t="n">
-        <v>599.71</v>
+        <v>599.67</v>
       </c>
       <c r="K45" s="21">
         <f>IF(OR($B45="",$I45=""),"",$I45-IF($J45="",0,$J45))</f>
@@ -3615,7 +3615,7 @@
         <v/>
       </c>
       <c r="J46" s="4" t="n">
-        <v>600.8200000000001</v>
+        <v>600.78</v>
       </c>
       <c r="K46" s="21">
         <f>IF(OR($B46="",$I46=""),"",$I46-IF($J46="",0,$J46))</f>
@@ -3666,7 +3666,7 @@
         <v/>
       </c>
       <c r="J47" s="4" t="n">
-        <v>678.75</v>
+        <v>678.8099999999999</v>
       </c>
       <c r="K47" s="21">
         <f>IF(OR($B47="",$I47=""),"",$I47-IF($J47="",0,$J47))</f>
@@ -3717,7 +3717,7 @@
         <v/>
       </c>
       <c r="J48" s="4" t="n">
-        <v>672.49</v>
+        <v>672.53</v>
       </c>
       <c r="K48" s="21">
         <f>IF(OR($B48="",$I48=""),"",$I48-IF($J48="",0,$J48))</f>
@@ -3768,7 +3768,7 @@
         <v/>
       </c>
       <c r="J49" s="4" t="n">
-        <v>538.6799999999999</v>
+        <v>538.66</v>
       </c>
       <c r="K49" s="21">
         <f>IF(OR($B49="",$I49=""),"",$I49-IF($J49="",0,$J49))</f>
@@ -3819,7 +3819,7 @@
         <v/>
       </c>
       <c r="J50" s="4" t="n">
-        <v>627.98</v>
+        <v>627.97</v>
       </c>
       <c r="K50" s="21">
         <f>IF(OR($B50="",$I50=""),"",$I50-IF($J50="",0,$J50))</f>
@@ -4023,7 +4023,7 @@
         <v/>
       </c>
       <c r="J54" s="4" t="n">
-        <v>619.13</v>
+        <v>619.1900000000001</v>
       </c>
       <c r="K54" s="21">
         <f>IF(OR($B54="",$I54=""),"",$I54-IF($J54="",0,$J54))</f>
@@ -4176,7 +4176,7 @@
         <v/>
       </c>
       <c r="J57" s="4" t="n">
-        <v>612.27</v>
+        <v>612.26</v>
       </c>
       <c r="K57" s="21">
         <f>IF(OR($B57="",$I57=""),"",$I57-IF($J57="",0,$J57))</f>
@@ -4380,7 +4380,7 @@
         <v/>
       </c>
       <c r="J61" s="4" t="n">
-        <v>692.09</v>
+        <v>692.1</v>
       </c>
       <c r="K61" s="21">
         <f>IF(OR($B61="",$I61=""),"",$I61-IF($J61="",0,$J61))</f>
@@ -4431,7 +4431,7 @@
         <v/>
       </c>
       <c r="J62" s="4" t="n">
-        <v>615.39</v>
+        <v>615.37</v>
       </c>
       <c r="K62" s="21">
         <f>IF(OR($B62="",$I62=""),"",$I62-IF($J62="",0,$J62))</f>
@@ -4533,7 +4533,7 @@
         <v/>
       </c>
       <c r="J64" s="4" t="n">
-        <v>440.45</v>
+        <v>440.41</v>
       </c>
       <c r="K64" s="21">
         <f>IF(OR($B64="",$I64=""),"",$I64-IF($J64="",0,$J64))</f>
@@ -4839,7 +4839,7 @@
         <v/>
       </c>
       <c r="J70" s="4" t="n">
-        <v>385.19</v>
+        <v>385.2</v>
       </c>
       <c r="K70" s="21">
         <f>IF(OR($B70="",$I70=""),"",$I70-IF($J70="",0,$J70))</f>
@@ -4941,7 +4941,7 @@
         <v/>
       </c>
       <c r="J72" s="4" t="n">
-        <v>376.89</v>
+        <v>411.19</v>
       </c>
       <c r="K72" s="21">
         <f>IF(OR($B72="",$I72=""),"",$I72-IF($J72="",0,$J72))</f>
@@ -5043,7 +5043,7 @@
         <v/>
       </c>
       <c r="J74" s="4" t="n">
-        <v>327.31</v>
+        <v>355.76</v>
       </c>
       <c r="K74" s="21">
         <f>IF(OR($B74="",$I74=""),"",$I74-IF($J74="",0,$J74))</f>
@@ -5094,7 +5094,7 @@
         <v/>
       </c>
       <c r="J75" s="4" t="n">
-        <v>330.16</v>
+        <v>364.28</v>
       </c>
       <c r="K75" s="21">
         <f>IF(OR($B75="",$I75=""),"",$I75-IF($J75="",0,$J75))</f>
@@ -5196,7 +5196,7 @@
         <v/>
       </c>
       <c r="J77" s="4" t="n">
-        <v>375.06</v>
+        <v>411.38</v>
       </c>
       <c r="K77" s="21">
         <f>IF(OR($B77="",$I77=""),"",$I77-IF($J77="",0,$J77))</f>
@@ -5298,7 +5298,7 @@
         <v/>
       </c>
       <c r="J79" s="4" t="n">
-        <v>323.35</v>
+        <v>343.87</v>
       </c>
       <c r="K79" s="21">
         <f>IF(OR($B79="",$I79=""),"",$I79-IF($J79="",0,$J79))</f>
@@ -5349,7 +5349,7 @@
         <v/>
       </c>
       <c r="J80" s="4" t="n">
-        <v>324.64</v>
+        <v>345.31</v>
       </c>
       <c r="K80" s="21">
         <f>IF(OR($B80="",$I80=""),"",$I80-IF($J80="",0,$J80))</f>
@@ -5859,7 +5859,7 @@
         <v/>
       </c>
       <c r="J90" s="4" t="n">
-        <v>833.8200000000001</v>
+        <v>891.79</v>
       </c>
       <c r="K90" s="21">
         <f>IF(OR($B90="",$I90=""),"",$I90-IF($J90="",0,$J90))</f>
@@ -5961,7 +5961,7 @@
         <v/>
       </c>
       <c r="J92" s="4" t="n">
-        <v>739.8200000000001</v>
+        <v>797.8099999999999</v>
       </c>
       <c r="K92" s="21">
         <f>IF(OR($B92="",$I92=""),"",$I92-IF($J92="",0,$J92))</f>
@@ -6012,7 +6012,7 @@
         <v/>
       </c>
       <c r="J93" s="4" t="n">
-        <v>766.78</v>
+        <v>825.14</v>
       </c>
       <c r="K93" s="21">
         <f>IF(OR($B93="",$I93=""),"",$I93-IF($J93="",0,$J93))</f>
@@ -6063,7 +6063,7 @@
         <v/>
       </c>
       <c r="J94" s="4" t="n">
-        <v>433.63</v>
+        <v>479.75</v>
       </c>
       <c r="K94" s="21">
         <f>IF(OR($B94="",$I94=""),"",$I94-IF($J94="",0,$J94))</f>
@@ -6165,7 +6165,7 @@
         <v/>
       </c>
       <c r="J96" s="4" t="n">
-        <v>430.76</v>
+        <v>474.02</v>
       </c>
       <c r="K96" s="21">
         <f>IF(OR($B96="",$I96=""),"",$I96-IF($J96="",0,$J96))</f>
@@ -6267,7 +6267,7 @@
         <v/>
       </c>
       <c r="J98" s="4" t="n">
-        <v>487.6</v>
+        <v>530.8</v>
       </c>
       <c r="K98" s="21">
         <f>IF(OR($B98="",$I98=""),"",$I98-IF($J98="",0,$J98))</f>
@@ -6471,7 +6471,7 @@
         <v/>
       </c>
       <c r="J102" s="4" t="n">
-        <v>487.69</v>
+        <v>531.01</v>
       </c>
       <c r="K102" s="21">
         <f>IF(OR($B102="",$I102=""),"",$I102-IF($J102="",0,$J102))</f>
@@ -6879,7 +6879,7 @@
         <v/>
       </c>
       <c r="J110" s="4" t="n">
-        <v>437.57</v>
+        <v>480.3</v>
       </c>
       <c r="K110" s="21">
         <f>IF(OR($B110="",$I110=""),"",$I110-IF($J110="",0,$J110))</f>
@@ -6981,7 +6981,7 @@
         <v/>
       </c>
       <c r="J112" s="4" t="n">
-        <v>382.63</v>
+        <v>419.66</v>
       </c>
       <c r="K112" s="21">
         <f>IF(OR($B112="",$I112=""),"",$I112-IF($J112="",0,$J112))</f>
@@ -7185,7 +7185,7 @@
         <v/>
       </c>
       <c r="J116" s="4" t="n">
-        <v>394.12</v>
+        <v>428.12</v>
       </c>
       <c r="K116" s="21">
         <f>IF(OR($B116="",$I116=""),"",$I116-IF($J116="",0,$J116))</f>
@@ -7236,7 +7236,7 @@
         <v/>
       </c>
       <c r="J117" s="4" t="n">
-        <v>494.15</v>
+        <v>545.67</v>
       </c>
       <c r="K117" s="21">
         <f>IF(OR($B117="",$I117=""),"",$I117-IF($J117="",0,$J117))</f>
@@ -7389,7 +7389,7 @@
         <v/>
       </c>
       <c r="J120" s="4" t="n">
-        <v>391.21</v>
+        <v>424.36</v>
       </c>
       <c r="K120" s="21">
         <f>IF(OR($B120="",$I120=""),"",$I120-IF($J120="",0,$J120))</f>
@@ -7440,7 +7440,7 @@
         <v/>
       </c>
       <c r="J121" s="4" t="n">
-        <v>343.5</v>
+        <v>371.23</v>
       </c>
       <c r="K121" s="21">
         <f>IF(OR($B121="",$I121=""),"",$I121-IF($J121="",0,$J121))</f>
@@ -7746,7 +7746,7 @@
         <v/>
       </c>
       <c r="J127" s="4" t="n">
-        <v>587.9400000000001</v>
+        <v>641.8</v>
       </c>
       <c r="K127" s="21">
         <f>IF(OR($B127="",$I127=""),"",$I127-IF($J127="",0,$J127))</f>
@@ -7848,7 +7848,7 @@
         <v/>
       </c>
       <c r="J129" s="4" t="n">
-        <v>583.85</v>
+        <v>637.65</v>
       </c>
       <c r="K129" s="21">
         <f>IF(OR($B129="",$I129=""),"",$I129-IF($J129="",0,$J129))</f>
@@ -7950,7 +7950,7 @@
         <v/>
       </c>
       <c r="J131" s="4" t="n">
-        <v>592.8200000000001</v>
+        <v>653.3099999999999</v>
       </c>
       <c r="K131" s="21">
         <f>IF(OR($B131="",$I131=""),"",$I131-IF($J131="",0,$J131))</f>
@@ -8052,7 +8052,7 @@
         <v/>
       </c>
       <c r="J133" s="4" t="n">
-        <v>509.91</v>
+        <v>563.48</v>
       </c>
       <c r="K133" s="21">
         <f>IF(OR($B133="",$I133=""),"",$I133-IF($J133="",0,$J133))</f>
@@ -8103,7 +8103,7 @@
         <v/>
       </c>
       <c r="J134" s="4" t="n">
-        <v>578.39</v>
+        <v>631.45</v>
       </c>
       <c r="K134" s="21">
         <f>IF(OR($B134="",$I134=""),"",$I134-IF($J134="",0,$J134))</f>
@@ -8154,7 +8154,7 @@
         <v/>
       </c>
       <c r="J135" s="4" t="n">
-        <v>468.38</v>
+        <v>496.78</v>
       </c>
       <c r="K135" s="21">
         <f>IF(OR($B135="",$I135=""),"",$I135-IF($J135="",0,$J135))</f>
@@ -8307,7 +8307,7 @@
         <v/>
       </c>
       <c r="J138" s="4" t="n">
-        <v>465.39</v>
+        <v>493.54</v>
       </c>
       <c r="K138" s="21">
         <f>IF(OR($B138="",$I138=""),"",$I138-IF($J138="",0,$J138))</f>
@@ -8409,7 +8409,7 @@
         <v/>
       </c>
       <c r="J140" s="4" t="n">
-        <v>473.51</v>
+        <v>503.24</v>
       </c>
       <c r="K140" s="21">
         <f>IF(OR($B140="",$I140=""),"",$I140-IF($J140="",0,$J140))</f>
@@ -8460,7 +8460,7 @@
         <v/>
       </c>
       <c r="J141" s="4" t="n">
-        <v>463.24</v>
+        <v>490.69</v>
       </c>
       <c r="K141" s="21">
         <f>IF(OR($B141="",$I141=""),"",$I141-IF($J141="",0,$J141))</f>
@@ -8511,7 +8511,7 @@
         <v/>
       </c>
       <c r="J142" s="4" t="n">
-        <v>442.78</v>
+        <v>466.38</v>
       </c>
       <c r="K142" s="21">
         <f>IF(OR($B142="",$I142=""),"",$I142-IF($J142="",0,$J142))</f>
@@ -8664,7 +8664,7 @@
         <v/>
       </c>
       <c r="J145" s="4" t="n">
-        <v>512.21</v>
+        <v>541.72</v>
       </c>
       <c r="K145" s="21">
         <f>IF(OR($B145="",$I145=""),"",$I145-IF($J145="",0,$J145))</f>
@@ -9214,14 +9214,18 @@
       <c r="F156" s="26" t="n">
         <v>395</v>
       </c>
-      <c r="G156" s="24" t="inlineStr"/>
-      <c r="H156" s="25" t="inlineStr"/>
+      <c r="G156" s="24" t="n">
+        <v>46282</v>
+      </c>
+      <c r="H156" s="25" t="n">
+        <v>634</v>
+      </c>
       <c r="I156" s="21">
         <f>IF(OR($B156="",$H156=""),"",IF($C156="LONG",($H156-$E156)*$F156,($E156-$H156)*$F156))</f>
         <v/>
       </c>
       <c r="J156" s="4" t="n">
-        <v>50.15</v>
+        <v>427.11</v>
       </c>
       <c r="K156" s="21">
         <f>IF(OR($B156="",$I156=""),"",$I156-IF($J156="",0,$J156))</f>
@@ -9261,14 +9265,18 @@
       <c r="F157" s="26" t="n">
         <v>37</v>
       </c>
-      <c r="G157" s="24" t="inlineStr"/>
-      <c r="H157" s="25" t="inlineStr"/>
+      <c r="G157" s="24" t="n">
+        <v>46282</v>
+      </c>
+      <c r="H157" s="25" t="n">
+        <v>6992.324</v>
+      </c>
       <c r="I157" s="21">
         <f>IF(OR($B157="",$H157=""),"",IF($C157="LONG",($H157-$E157)*$F157,($E157-$H157)*$F157))</f>
         <v/>
       </c>
       <c r="J157" s="4" t="n">
-        <v>50.15</v>
+        <v>427.33</v>
       </c>
       <c r="K157" s="21">
         <f>IF(OR($B157="",$I157=""),"",$I157-IF($J157="",0,$J157))</f>
@@ -9308,14 +9316,18 @@
       <c r="F158" s="26" t="n">
         <v>1842</v>
       </c>
-      <c r="G158" s="24" t="inlineStr"/>
-      <c r="H158" s="25" t="inlineStr"/>
+      <c r="G158" s="24" t="n">
+        <v>46282</v>
+      </c>
+      <c r="H158" s="25" t="n">
+        <v>136.6183</v>
+      </c>
       <c r="I158" s="21">
         <f>IF(OR($B158="",$H158=""),"",IF($C158="LONG",($H158-$E158)*$F158,($E158-$H158)*$F158))</f>
         <v/>
       </c>
       <c r="J158" s="4" t="n">
-        <v>50.15</v>
+        <v>422.92</v>
       </c>
       <c r="K158" s="21">
         <f>IF(OR($B158="",$I158=""),"",$I158-IF($J158="",0,$J158))</f>
@@ -9355,14 +9367,18 @@
       <c r="F159" s="26" t="n">
         <v>135</v>
       </c>
-      <c r="G159" s="24" t="inlineStr"/>
-      <c r="H159" s="25" t="inlineStr"/>
+      <c r="G159" s="24" t="n">
+        <v>46282</v>
+      </c>
+      <c r="H159" s="25" t="n">
+        <v>1877.0074</v>
+      </c>
       <c r="I159" s="21">
         <f>IF(OR($B159="",$H159=""),"",IF($C159="LONG",($H159-$E159)*$F159,($E159-$H159)*$F159))</f>
         <v/>
       </c>
       <c r="J159" s="4" t="n">
-        <v>50.15</v>
+        <v>421.22</v>
       </c>
       <c r="K159" s="21">
         <f>IF(OR($B159="",$I159=""),"",$I159-IF($J159="",0,$J159))</f>
@@ -9402,14 +9418,18 @@
       <c r="F160" s="26" t="n">
         <v>186</v>
       </c>
-      <c r="G160" s="24" t="inlineStr"/>
-      <c r="H160" s="25" t="inlineStr"/>
+      <c r="G160" s="24" t="n">
+        <v>46282</v>
+      </c>
+      <c r="H160" s="25" t="n">
+        <v>1364.2269</v>
+      </c>
       <c r="I160" s="21">
         <f>IF(OR($B160="",$H160=""),"",IF($C160="LONG",($H160-$E160)*$F160,($E160-$H160)*$F160))</f>
         <v/>
       </c>
       <c r="J160" s="4" t="n">
-        <v>50.15</v>
+        <v>412.55</v>
       </c>
       <c r="K160" s="21">
         <f>IF(OR($B160="",$I160=""),"",$I160-IF($J160="",0,$J160))</f>
@@ -9449,14 +9469,18 @@
       <c r="F161" s="26" t="n">
         <v>603</v>
       </c>
-      <c r="G161" s="24" t="inlineStr"/>
-      <c r="H161" s="25" t="inlineStr"/>
+      <c r="G161" s="24" t="n">
+        <v>46282</v>
+      </c>
+      <c r="H161" s="25" t="n">
+        <v>407.7921</v>
+      </c>
       <c r="I161" s="21">
         <f>IF(OR($B161="",$H161=""),"",IF($C161="LONG",($H161-$E161)*$F161,($E161-$H161)*$F161))</f>
         <v/>
       </c>
       <c r="J161" s="4" t="n">
-        <v>50.15</v>
+        <v>429.01</v>
       </c>
       <c r="K161" s="21">
         <f>IF(OR($B161="",$I161=""),"",$I161-IF($J161="",0,$J161))</f>
@@ -9472,19 +9496,43 @@
       </c>
     </row>
     <row r="162">
-      <c r="A162" s="23" t="n"/>
-      <c r="B162" s="23" t="n"/>
-      <c r="C162" s="23" t="n"/>
-      <c r="D162" s="24" t="n"/>
-      <c r="E162" s="25" t="n"/>
-      <c r="F162" s="26" t="n"/>
-      <c r="G162" s="24" t="n"/>
-      <c r="H162" s="25" t="n"/>
+      <c r="A162" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-23126091746909</t>
+        </is>
+      </c>
+      <c r="B162" s="23" t="inlineStr">
+        <is>
+          <t>EMUDHRA</t>
+        </is>
+      </c>
+      <c r="C162" s="23" t="inlineStr">
+        <is>
+          <t>SHORT</t>
+        </is>
+      </c>
+      <c r="D162" s="24" t="n">
+        <v>46282</v>
+      </c>
+      <c r="E162" s="25" t="n">
+        <v>633.678</v>
+      </c>
+      <c r="F162" s="26" t="n">
+        <v>395</v>
+      </c>
+      <c r="G162" s="24" t="n">
+        <v>46282</v>
+      </c>
+      <c r="H162" s="25" t="n">
+        <v>648.2501999999999</v>
+      </c>
       <c r="I162" s="21">
         <f>IF(OR($B162="",$H162=""),"",IF($C162="LONG",($H162-$E162)*$F162,($E162-$H162)*$F162))</f>
         <v/>
       </c>
-      <c r="J162" s="4" t="n"/>
+      <c r="J162" s="4" t="n">
+        <v>0</v>
+      </c>
       <c r="K162" s="21">
         <f>IF(OR($B162="",$I162=""),"",$I162-IF($J162="",0,$J162))</f>
         <v/>
@@ -9499,19 +9547,43 @@
       </c>
     </row>
     <row r="163">
-      <c r="A163" s="23" t="n"/>
-      <c r="B163" s="23" t="n"/>
-      <c r="C163" s="23" t="n"/>
-      <c r="D163" s="24" t="n"/>
-      <c r="E163" s="25" t="n"/>
-      <c r="F163" s="26" t="n"/>
-      <c r="G163" s="24" t="n"/>
-      <c r="H163" s="25" t="n"/>
+      <c r="A163" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-23126091718009</t>
+        </is>
+      </c>
+      <c r="B163" s="23" t="inlineStr">
+        <is>
+          <t>FOSECOIND</t>
+        </is>
+      </c>
+      <c r="C163" s="23" t="inlineStr">
+        <is>
+          <t>SHORT</t>
+        </is>
+      </c>
+      <c r="D163" s="24" t="n">
+        <v>46282</v>
+      </c>
+      <c r="E163" s="25" t="n">
+        <v>6984.243</v>
+      </c>
+      <c r="F163" s="26" t="n">
+        <v>37</v>
+      </c>
+      <c r="G163" s="24" t="n">
+        <v>46282</v>
+      </c>
+      <c r="H163" s="25" t="n">
+        <v>6814.2974</v>
+      </c>
       <c r="I163" s="21">
         <f>IF(OR($B163="",$H163=""),"",IF($C163="LONG",($H163-$E163)*$F163,($E163-$H163)*$F163))</f>
         <v/>
       </c>
-      <c r="J163" s="4" t="n"/>
+      <c r="J163" s="4" t="n">
+        <v>0</v>
+      </c>
       <c r="K163" s="21">
         <f>IF(OR($B163="",$I163=""),"",$I163-IF($J163="",0,$J163))</f>
         <v/>
@@ -9526,19 +9598,43 @@
       </c>
     </row>
     <row r="164">
-      <c r="A164" s="23" t="n"/>
-      <c r="B164" s="23" t="n"/>
-      <c r="C164" s="23" t="n"/>
-      <c r="D164" s="24" t="n"/>
-      <c r="E164" s="25" t="n"/>
-      <c r="F164" s="26" t="n"/>
-      <c r="G164" s="24" t="n"/>
-      <c r="H164" s="25" t="n"/>
+      <c r="A164" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-34126091721009</t>
+        </is>
+      </c>
+      <c r="B164" s="23" t="inlineStr">
+        <is>
+          <t>IPL</t>
+        </is>
+      </c>
+      <c r="C164" s="23" t="inlineStr">
+        <is>
+          <t>SHORT</t>
+        </is>
+      </c>
+      <c r="D164" s="24" t="n">
+        <v>46282</v>
+      </c>
+      <c r="E164" s="25" t="n">
+        <v>136.5789</v>
+      </c>
+      <c r="F164" s="26" t="n">
+        <v>1842</v>
+      </c>
+      <c r="G164" s="24" t="n">
+        <v>46282</v>
+      </c>
+      <c r="H164" s="25" t="n">
+        <v>138.1175</v>
+      </c>
       <c r="I164" s="21">
         <f>IF(OR($B164="",$H164=""),"",IF($C164="LONG",($H164-$E164)*$F164,($E164-$H164)*$F164))</f>
         <v/>
       </c>
-      <c r="J164" s="4" t="n"/>
+      <c r="J164" s="4" t="n">
+        <v>0</v>
+      </c>
       <c r="K164" s="21">
         <f>IF(OR($B164="",$I164=""),"",$I164-IF($J164="",0,$J164))</f>
         <v/>
@@ -9553,19 +9649,43 @@
       </c>
     </row>
     <row r="165">
-      <c r="A165" s="23" t="n"/>
-      <c r="B165" s="23" t="n"/>
-      <c r="C165" s="23" t="n"/>
-      <c r="D165" s="24" t="n"/>
-      <c r="E165" s="25" t="n"/>
-      <c r="F165" s="26" t="n"/>
-      <c r="G165" s="24" t="n"/>
-      <c r="H165" s="25" t="n"/>
+      <c r="A165" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-22126091785509</t>
+        </is>
+      </c>
+      <c r="B165" s="23" t="inlineStr">
+        <is>
+          <t>NPST</t>
+        </is>
+      </c>
+      <c r="C165" s="23" t="inlineStr">
+        <is>
+          <t>SHORT</t>
+        </is>
+      </c>
+      <c r="D165" s="24" t="n">
+        <v>46282</v>
+      </c>
+      <c r="E165" s="25" t="n">
+        <v>1880.0497</v>
+      </c>
+      <c r="F165" s="26" t="n">
+        <v>135</v>
+      </c>
+      <c r="G165" s="24" t="n">
+        <v>46282</v>
+      </c>
+      <c r="H165" s="25" t="n">
+        <v>1855.7349</v>
+      </c>
       <c r="I165" s="21">
         <f>IF(OR($B165="",$H165=""),"",IF($C165="LONG",($H165-$E165)*$F165,($E165-$H165)*$F165))</f>
         <v/>
       </c>
-      <c r="J165" s="4" t="n"/>
+      <c r="J165" s="4" t="n">
+        <v>0</v>
+      </c>
       <c r="K165" s="21">
         <f>IF(OR($B165="",$I165=""),"",$I165-IF($J165="",0,$J165))</f>
         <v/>
@@ -9580,19 +9700,43 @@
       </c>
     </row>
     <row r="166">
-      <c r="A166" s="23" t="n"/>
-      <c r="B166" s="23" t="n"/>
-      <c r="C166" s="23" t="n"/>
-      <c r="D166" s="24" t="n"/>
-      <c r="E166" s="25" t="n"/>
-      <c r="F166" s="26" t="n"/>
-      <c r="G166" s="24" t="n"/>
-      <c r="H166" s="25" t="n"/>
+      <c r="A166" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-22126091785609</t>
+        </is>
+      </c>
+      <c r="B166" s="23" t="inlineStr">
+        <is>
+          <t>ROSSTECH</t>
+        </is>
+      </c>
+      <c r="C166" s="23" t="inlineStr">
+        <is>
+          <t>SHORT</t>
+        </is>
+      </c>
+      <c r="D166" s="24" t="n">
+        <v>46282</v>
+      </c>
+      <c r="E166" s="25" t="n">
+        <v>1366.5123</v>
+      </c>
+      <c r="F166" s="26" t="n">
+        <v>186</v>
+      </c>
+      <c r="G166" s="24" t="n">
+        <v>46282</v>
+      </c>
+      <c r="H166" s="25" t="n">
+        <v>1364.1118</v>
+      </c>
       <c r="I166" s="21">
         <f>IF(OR($B166="",$H166=""),"",IF($C166="LONG",($H166-$E166)*$F166,($E166-$H166)*$F166))</f>
         <v/>
       </c>
-      <c r="J166" s="4" t="n"/>
+      <c r="J166" s="4" t="n">
+        <v>0</v>
+      </c>
       <c r="K166" s="21">
         <f>IF(OR($B166="",$I166=""),"",$I166-IF($J166="",0,$J166))</f>
         <v/>
@@ -9607,19 +9751,43 @@
       </c>
     </row>
     <row r="167">
-      <c r="A167" s="23" t="n"/>
-      <c r="B167" s="23" t="n"/>
-      <c r="C167" s="23" t="n"/>
-      <c r="D167" s="24" t="n"/>
-      <c r="E167" s="25" t="n"/>
-      <c r="F167" s="26" t="n"/>
-      <c r="G167" s="24" t="n"/>
-      <c r="H167" s="25" t="n"/>
+      <c r="A167" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-221260917413309</t>
+        </is>
+      </c>
+      <c r="B167" s="23" t="inlineStr">
+        <is>
+          <t>SAATVIKGL</t>
+        </is>
+      </c>
+      <c r="C167" s="23" t="inlineStr">
+        <is>
+          <t>SHORT</t>
+        </is>
+      </c>
+      <c r="D167" s="24" t="n">
+        <v>46282</v>
+      </c>
+      <c r="E167" s="25" t="n">
+        <v>407.1779</v>
+      </c>
+      <c r="F167" s="26" t="n">
+        <v>603</v>
+      </c>
+      <c r="G167" s="24" t="n">
+        <v>46282</v>
+      </c>
+      <c r="H167" s="25" t="n">
+        <v>404.5646</v>
+      </c>
       <c r="I167" s="21">
         <f>IF(OR($B167="",$H167=""),"",IF($C167="LONG",($H167-$E167)*$F167,($E167-$H167)*$F167))</f>
         <v/>
       </c>
-      <c r="J167" s="4" t="n"/>
+      <c r="J167" s="4" t="n">
+        <v>0</v>
+      </c>
       <c r="K167" s="21">
         <f>IF(OR($B167="",$I167=""),"",$I167-IF($J167="",0,$J167))</f>
         <v/>
@@ -9634,19 +9802,39 @@
       </c>
     </row>
     <row r="168">
-      <c r="A168" s="23" t="n"/>
-      <c r="B168" s="23" t="n"/>
-      <c r="C168" s="23" t="n"/>
-      <c r="D168" s="24" t="n"/>
-      <c r="E168" s="25" t="n"/>
-      <c r="F168" s="26" t="n"/>
-      <c r="G168" s="24" t="n"/>
-      <c r="H168" s="25" t="n"/>
+      <c r="A168" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-221260917656409</t>
+        </is>
+      </c>
+      <c r="B168" s="23" t="inlineStr">
+        <is>
+          <t>SHAREINDIA</t>
+        </is>
+      </c>
+      <c r="C168" s="23" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="D168" s="24" t="n">
+        <v>46282</v>
+      </c>
+      <c r="E168" s="25" t="n">
+        <v>219.5</v>
+      </c>
+      <c r="F168" s="26" t="n">
+        <v>1722</v>
+      </c>
+      <c r="G168" s="24" t="inlineStr"/>
+      <c r="H168" s="25" t="inlineStr"/>
       <c r="I168" s="21">
         <f>IF(OR($B168="",$H168=""),"",IF($C168="LONG",($H168-$E168)*$F168,($E168-$H168)*$F168))</f>
         <v/>
       </c>
-      <c r="J168" s="4" t="n"/>
+      <c r="J168" s="4" t="n">
+        <v>50.15</v>
+      </c>
       <c r="K168" s="21">
         <f>IF(OR($B168="",$I168=""),"",$I168-IF($J168="",0,$J168))</f>
         <v/>
@@ -9661,19 +9849,39 @@
       </c>
     </row>
     <row r="169">
-      <c r="A169" s="23" t="n"/>
-      <c r="B169" s="23" t="n"/>
-      <c r="C169" s="23" t="n"/>
-      <c r="D169" s="24" t="n"/>
-      <c r="E169" s="25" t="n"/>
-      <c r="F169" s="26" t="n"/>
-      <c r="G169" s="24" t="n"/>
-      <c r="H169" s="25" t="n"/>
+      <c r="A169" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-321260917609709</t>
+        </is>
+      </c>
+      <c r="B169" s="23" t="inlineStr">
+        <is>
+          <t>VENUSPIPES</t>
+        </is>
+      </c>
+      <c r="C169" s="23" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="D169" s="24" t="n">
+        <v>46282</v>
+      </c>
+      <c r="E169" s="25" t="n">
+        <v>2134.6694</v>
+      </c>
+      <c r="F169" s="26" t="n">
+        <v>176</v>
+      </c>
+      <c r="G169" s="24" t="inlineStr"/>
+      <c r="H169" s="25" t="inlineStr"/>
       <c r="I169" s="21">
         <f>IF(OR($B169="",$H169=""),"",IF($C169="LONG",($H169-$E169)*$F169,($E169-$H169)*$F169))</f>
         <v/>
       </c>
-      <c r="J169" s="4" t="n"/>
+      <c r="J169" s="4" t="n">
+        <v>50.15</v>
+      </c>
       <c r="K169" s="21">
         <f>IF(OR($B169="",$I169=""),"",$I169-IF($J169="",0,$J169))</f>
         <v/>

</xml_diff>

<commit_message>
Fix exit-leg charge lookup for legacy exited_925 positions
Today's check_exit_925 -> check_exit_916 rename dropped "exited_925" from
dhan/charges.py's status-keyed exit-field tables, silently zeroing the
exit-leg charge (and misdating MTF interest cutoffs to today) for all 44
historical positions still carrying the old status string. Keep both keys
so legacy data resolves correctly alongside new exits going forward.
Regenerated strategy_pnl_simple.xlsx with the fix applied.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/results/strategy_pnl_simple.xlsx
+++ b/results/strategy_pnl_simple.xlsx
@@ -1473,7 +1473,7 @@
         <v/>
       </c>
       <c r="J4" s="4" t="n">
-        <v>571.8200000000001</v>
+        <v>571.79</v>
       </c>
       <c r="K4" s="21">
         <f>IF(OR($B4="",$I4=""),"",$I4-IF($J4="",0,$J4))</f>
@@ -1524,7 +1524,7 @@
         <v/>
       </c>
       <c r="J5" s="4" t="n">
-        <v>688.84</v>
+        <v>688.87</v>
       </c>
       <c r="K5" s="21">
         <f>IF(OR($B5="",$I5=""),"",$I5-IF($J5="",0,$J5))</f>
@@ -1575,7 +1575,7 @@
         <v/>
       </c>
       <c r="J6" s="4" t="n">
-        <v>570.67</v>
+        <v>570.64</v>
       </c>
       <c r="K6" s="21">
         <f>IF(OR($B6="",$I6=""),"",$I6-IF($J6="",0,$J6))</f>
@@ -1626,7 +1626,7 @@
         <v/>
       </c>
       <c r="J7" s="4" t="n">
-        <v>663.08</v>
+        <v>663.04</v>
       </c>
       <c r="K7" s="21">
         <f>IF(OR($B7="",$I7=""),"",$I7-IF($J7="",0,$J7))</f>
@@ -1677,7 +1677,7 @@
         <v/>
       </c>
       <c r="J8" s="4" t="n">
-        <v>590.88</v>
+        <v>590.95</v>
       </c>
       <c r="K8" s="21">
         <f>IF(OR($B8="",$I8=""),"",$I8-IF($J8="",0,$J8))</f>
@@ -1779,7 +1779,7 @@
         <v/>
       </c>
       <c r="J10" s="4" t="n">
-        <v>398.63</v>
+        <v>398.62</v>
       </c>
       <c r="K10" s="21">
         <f>IF(OR($B10="",$I10=""),"",$I10-IF($J10="",0,$J10))</f>
@@ -1881,7 +1881,7 @@
         <v/>
       </c>
       <c r="J12" s="4" t="n">
-        <v>414.18</v>
+        <v>414.16</v>
       </c>
       <c r="K12" s="21">
         <f>IF(OR($B12="",$I12=""),"",$I12-IF($J12="",0,$J12))</f>
@@ -1932,7 +1932,7 @@
         <v/>
       </c>
       <c r="J13" s="4" t="n">
-        <v>345.08</v>
+        <v>345.07</v>
       </c>
       <c r="K13" s="21">
         <f>IF(OR($B13="",$I13=""),"",$I13-IF($J13="",0,$J13))</f>
@@ -1983,7 +1983,7 @@
         <v/>
       </c>
       <c r="J14" s="4" t="n">
-        <v>414.51</v>
+        <v>414.49</v>
       </c>
       <c r="K14" s="21">
         <f>IF(OR($B14="",$I14=""),"",$I14-IF($J14="",0,$J14))</f>
@@ -2034,7 +2034,7 @@
         <v/>
       </c>
       <c r="J15" s="4" t="n">
-        <v>380.37</v>
+        <v>380.4</v>
       </c>
       <c r="K15" s="21">
         <f>IF(OR($B15="",$I15=""),"",$I15-IF($J15="",0,$J15))</f>
@@ -2187,7 +2187,7 @@
         <v/>
       </c>
       <c r="J18" s="4" t="n">
-        <v>413.94</v>
+        <v>413.92</v>
       </c>
       <c r="K18" s="21">
         <f>IF(OR($B18="",$I18=""),"",$I18-IF($J18="",0,$J18))</f>
@@ -2238,7 +2238,7 @@
         <v/>
       </c>
       <c r="J19" s="4" t="n">
-        <v>406.47</v>
+        <v>406.46</v>
       </c>
       <c r="K19" s="21">
         <f>IF(OR($B19="",$I19=""),"",$I19-IF($J19="",0,$J19))</f>
@@ -2697,7 +2697,7 @@
         <v/>
       </c>
       <c r="J28" s="4" t="n">
-        <v>870.25</v>
+        <v>870.39</v>
       </c>
       <c r="K28" s="21">
         <f>IF(OR($B28="",$I28=""),"",$I28-IF($J28="",0,$J28))</f>
@@ -2850,7 +2850,7 @@
         <v/>
       </c>
       <c r="J31" s="4" t="n">
-        <v>391.15</v>
+        <v>391.16</v>
       </c>
       <c r="K31" s="21">
         <f>IF(OR($B31="",$I31=""),"",$I31-IF($J31="",0,$J31))</f>
@@ -2901,7 +2901,7 @@
         <v/>
       </c>
       <c r="J32" s="4" t="n">
-        <v>349.77</v>
+        <v>349.78</v>
       </c>
       <c r="K32" s="21">
         <f>IF(OR($B32="",$I32=""),"",$I32-IF($J32="",0,$J32))</f>
@@ -3003,7 +3003,7 @@
         <v/>
       </c>
       <c r="J34" s="4" t="n">
-        <v>349.8</v>
+        <v>349.81</v>
       </c>
       <c r="K34" s="21">
         <f>IF(OR($B34="",$I34=""),"",$I34-IF($J34="",0,$J34))</f>
@@ -3054,7 +3054,7 @@
         <v/>
       </c>
       <c r="J35" s="4" t="n">
-        <v>386.17</v>
+        <v>386.1</v>
       </c>
       <c r="K35" s="21">
         <f>IF(OR($B35="",$I35=""),"",$I35-IF($J35="",0,$J35))</f>
@@ -3411,7 +3411,7 @@
         <v/>
       </c>
       <c r="J42" s="4" t="n">
-        <v>978.26</v>
+        <v>978.27</v>
       </c>
       <c r="K42" s="21">
         <f>IF(OR($B42="",$I42=""),"",$I42-IF($J42="",0,$J42))</f>
@@ -3462,7 +3462,7 @@
         <v/>
       </c>
       <c r="J43" s="4" t="n">
-        <v>957.66</v>
+        <v>957.67</v>
       </c>
       <c r="K43" s="21">
         <f>IF(OR($B43="",$I43=""),"",$I43-IF($J43="",0,$J43))</f>
@@ -3564,7 +3564,7 @@
         <v/>
       </c>
       <c r="J45" s="4" t="n">
-        <v>599.67</v>
+        <v>599.6900000000001</v>
       </c>
       <c r="K45" s="21">
         <f>IF(OR($B45="",$I45=""),"",$I45-IF($J45="",0,$J45))</f>
@@ -3615,7 +3615,7 @@
         <v/>
       </c>
       <c r="J46" s="4" t="n">
-        <v>600.78</v>
+        <v>600.8</v>
       </c>
       <c r="K46" s="21">
         <f>IF(OR($B46="",$I46=""),"",$I46-IF($J46="",0,$J46))</f>
@@ -3666,7 +3666,7 @@
         <v/>
       </c>
       <c r="J47" s="4" t="n">
-        <v>678.8099999999999</v>
+        <v>678.96</v>
       </c>
       <c r="K47" s="21">
         <f>IF(OR($B47="",$I47=""),"",$I47-IF($J47="",0,$J47))</f>
@@ -3717,7 +3717,7 @@
         <v/>
       </c>
       <c r="J48" s="4" t="n">
-        <v>672.53</v>
+        <v>672.39</v>
       </c>
       <c r="K48" s="21">
         <f>IF(OR($B48="",$I48=""),"",$I48-IF($J48="",0,$J48))</f>
@@ -3768,7 +3768,7 @@
         <v/>
       </c>
       <c r="J49" s="4" t="n">
-        <v>538.66</v>
+        <v>538.67</v>
       </c>
       <c r="K49" s="21">
         <f>IF(OR($B49="",$I49=""),"",$I49-IF($J49="",0,$J49))</f>
@@ -3819,7 +3819,7 @@
         <v/>
       </c>
       <c r="J50" s="4" t="n">
-        <v>627.97</v>
+        <v>628.03</v>
       </c>
       <c r="K50" s="21">
         <f>IF(OR($B50="",$I50=""),"",$I50-IF($J50="",0,$J50))</f>
@@ -4023,7 +4023,7 @@
         <v/>
       </c>
       <c r="J54" s="4" t="n">
-        <v>619.1900000000001</v>
+        <v>619</v>
       </c>
       <c r="K54" s="21">
         <f>IF(OR($B54="",$I54=""),"",$I54-IF($J54="",0,$J54))</f>
@@ -4380,7 +4380,7 @@
         <v/>
       </c>
       <c r="J61" s="4" t="n">
-        <v>692.1</v>
+        <v>692.09</v>
       </c>
       <c r="K61" s="21">
         <f>IF(OR($B61="",$I61=""),"",$I61-IF($J61="",0,$J61))</f>
@@ -4431,7 +4431,7 @@
         <v/>
       </c>
       <c r="J62" s="4" t="n">
-        <v>615.37</v>
+        <v>615.42</v>
       </c>
       <c r="K62" s="21">
         <f>IF(OR($B62="",$I62=""),"",$I62-IF($J62="",0,$J62))</f>
@@ -4533,7 +4533,7 @@
         <v/>
       </c>
       <c r="J64" s="4" t="n">
-        <v>440.41</v>
+        <v>440.42</v>
       </c>
       <c r="K64" s="21">
         <f>IF(OR($B64="",$I64=""),"",$I64-IF($J64="",0,$J64))</f>
@@ -4839,7 +4839,7 @@
         <v/>
       </c>
       <c r="J70" s="4" t="n">
-        <v>385.2</v>
+        <v>385.19</v>
       </c>
       <c r="K70" s="21">
         <f>IF(OR($B70="",$I70=""),"",$I70-IF($J70="",0,$J70))</f>
@@ -5196,7 +5196,7 @@
         <v/>
       </c>
       <c r="J77" s="4" t="n">
-        <v>411.38</v>
+        <v>411.42</v>
       </c>
       <c r="K77" s="21">
         <f>IF(OR($B77="",$I77=""),"",$I77-IF($J77="",0,$J77))</f>
@@ -6012,7 +6012,7 @@
         <v/>
       </c>
       <c r="J93" s="4" t="n">
-        <v>825.14</v>
+        <v>825.13</v>
       </c>
       <c r="K93" s="21">
         <f>IF(OR($B93="",$I93=""),"",$I93-IF($J93="",0,$J93))</f>
@@ -6063,7 +6063,7 @@
         <v/>
       </c>
       <c r="J94" s="4" t="n">
-        <v>479.75</v>
+        <v>479.81</v>
       </c>
       <c r="K94" s="21">
         <f>IF(OR($B94="",$I94=""),"",$I94-IF($J94="",0,$J94))</f>
@@ -6879,7 +6879,7 @@
         <v/>
       </c>
       <c r="J110" s="4" t="n">
-        <v>480.3</v>
+        <v>480.27</v>
       </c>
       <c r="K110" s="21">
         <f>IF(OR($B110="",$I110=""),"",$I110-IF($J110="",0,$J110))</f>
@@ -7185,7 +7185,7 @@
         <v/>
       </c>
       <c r="J116" s="4" t="n">
-        <v>428.12</v>
+        <v>428.14</v>
       </c>
       <c r="K116" s="21">
         <f>IF(OR($B116="",$I116=""),"",$I116-IF($J116="",0,$J116))</f>
@@ -7389,7 +7389,7 @@
         <v/>
       </c>
       <c r="J120" s="4" t="n">
-        <v>424.36</v>
+        <v>424.42</v>
       </c>
       <c r="K120" s="21">
         <f>IF(OR($B120="",$I120=""),"",$I120-IF($J120="",0,$J120))</f>
@@ -8409,7 +8409,7 @@
         <v/>
       </c>
       <c r="J140" s="4" t="n">
-        <v>503.24</v>
+        <v>503.39</v>
       </c>
       <c r="K140" s="21">
         <f>IF(OR($B140="",$I140=""),"",$I140-IF($J140="",0,$J140))</f>
@@ -8460,7 +8460,7 @@
         <v/>
       </c>
       <c r="J141" s="4" t="n">
-        <v>490.69</v>
+        <v>490.4</v>
       </c>
       <c r="K141" s="21">
         <f>IF(OR($B141="",$I141=""),"",$I141-IF($J141="",0,$J141))</f>
@@ -8664,7 +8664,7 @@
         <v/>
       </c>
       <c r="J145" s="4" t="n">
-        <v>541.72</v>
+        <v>541.75</v>
       </c>
       <c r="K145" s="21">
         <f>IF(OR($B145="",$I145=""),"",$I145-IF($J145="",0,$J145))</f>
@@ -9225,7 +9225,7 @@
         <v/>
       </c>
       <c r="J156" s="4" t="n">
-        <v>427.11</v>
+        <v>427.14</v>
       </c>
       <c r="K156" s="21">
         <f>IF(OR($B156="",$I156=""),"",$I156-IF($J156="",0,$J156))</f>
@@ -9833,7 +9833,7 @@
         <v/>
       </c>
       <c r="J168" s="4" t="n">
-        <v>50.15</v>
+        <v>116.08</v>
       </c>
       <c r="K168" s="21">
         <f>IF(OR($B168="",$I168=""),"",$I168-IF($J168="",0,$J168))</f>
@@ -9880,7 +9880,7 @@
         <v/>
       </c>
       <c r="J169" s="4" t="n">
-        <v>50.15</v>
+        <v>127.24</v>
       </c>
       <c r="K169" s="21">
         <f>IF(OR($B169="",$I169=""),"",$I169-IF($J169="",0,$J169))</f>

</xml_diff>

<commit_message>
Data update — 2026-09-18 candle + results refresh
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/results/strategy_pnl_simple.xlsx
+++ b/results/strategy_pnl_simple.xlsx
@@ -9225,7 +9225,7 @@
         <v/>
       </c>
       <c r="J156" s="4" t="n">
-        <v>427.14</v>
+        <v>460.1</v>
       </c>
       <c r="K156" s="21">
         <f>IF(OR($B156="",$I156=""),"",$I156-IF($J156="",0,$J156))</f>
@@ -9276,7 +9276,7 @@
         <v/>
       </c>
       <c r="J157" s="4" t="n">
-        <v>427.33</v>
+        <v>524.72</v>
       </c>
       <c r="K157" s="21">
         <f>IF(OR($B157="",$I157=""),"",$I157-IF($J157="",0,$J157))</f>
@@ -9327,7 +9327,7 @@
         <v/>
       </c>
       <c r="J158" s="4" t="n">
-        <v>422.92</v>
+        <v>519.0599999999999</v>
       </c>
       <c r="K158" s="21">
         <f>IF(OR($B158="",$I158=""),"",$I158-IF($J158="",0,$J158))</f>
@@ -9378,7 +9378,7 @@
         <v/>
       </c>
       <c r="J159" s="4" t="n">
-        <v>421.22</v>
+        <v>517.4400000000001</v>
       </c>
       <c r="K159" s="21">
         <f>IF(OR($B159="",$I159=""),"",$I159-IF($J159="",0,$J159))</f>
@@ -9429,7 +9429,7 @@
         <v/>
       </c>
       <c r="J160" s="4" t="n">
-        <v>412.55</v>
+        <v>445.64</v>
       </c>
       <c r="K160" s="21">
         <f>IF(OR($B160="",$I160=""),"",$I160-IF($J160="",0,$J160))</f>
@@ -9480,7 +9480,7 @@
         <v/>
       </c>
       <c r="J161" s="4" t="n">
-        <v>429.01</v>
+        <v>461.81</v>
       </c>
       <c r="K161" s="21">
         <f>IF(OR($B161="",$I161=""),"",$I161-IF($J161="",0,$J161))</f>
@@ -9531,7 +9531,7 @@
         <v/>
       </c>
       <c r="J162" s="4" t="n">
-        <v>0</v>
+        <v>365.55</v>
       </c>
       <c r="K162" s="21">
         <f>IF(OR($B162="",$I162=""),"",$I162-IF($J162="",0,$J162))</f>
@@ -9582,7 +9582,7 @@
         <v/>
       </c>
       <c r="J163" s="4" t="n">
-        <v>0</v>
+        <v>306.98</v>
       </c>
       <c r="K163" s="21">
         <f>IF(OR($B163="",$I163=""),"",$I163-IF($J163="",0,$J163))</f>
@@ -9633,7 +9633,7 @@
         <v/>
       </c>
       <c r="J164" s="4" t="n">
-        <v>0</v>
+        <v>302.7</v>
       </c>
       <c r="K164" s="21">
         <f>IF(OR($B164="",$I164=""),"",$I164-IF($J164="",0,$J164))</f>
@@ -9684,7 +9684,7 @@
         <v/>
       </c>
       <c r="J165" s="4" t="n">
-        <v>0</v>
+        <v>302.56</v>
       </c>
       <c r="K165" s="21">
         <f>IF(OR($B165="",$I165=""),"",$I165-IF($J165="",0,$J165))</f>
@@ -9735,7 +9735,7 @@
         <v/>
       </c>
       <c r="J166" s="4" t="n">
-        <v>0</v>
+        <v>367.56</v>
       </c>
       <c r="K166" s="21">
         <f>IF(OR($B166="",$I166=""),"",$I166-IF($J166="",0,$J166))</f>
@@ -9786,7 +9786,7 @@
         <v/>
       </c>
       <c r="J167" s="4" t="n">
-        <v>0</v>
+        <v>355.64</v>
       </c>
       <c r="K167" s="21">
         <f>IF(OR($B167="",$I167=""),"",$I167-IF($J167="",0,$J167))</f>
@@ -9826,14 +9826,18 @@
       <c r="F168" s="26" t="n">
         <v>1722</v>
       </c>
-      <c r="G168" s="24" t="inlineStr"/>
-      <c r="H168" s="25" t="inlineStr"/>
+      <c r="G168" s="24" t="n">
+        <v>46283</v>
+      </c>
+      <c r="H168" s="25" t="n">
+        <v>222.63</v>
+      </c>
       <c r="I168" s="21">
         <f>IF(OR($B168="",$H168=""),"",IF($C168="LONG",($H168-$E168)*$F168,($E168-$H168)*$F168))</f>
         <v/>
       </c>
       <c r="J168" s="4" t="n">
-        <v>116.08</v>
+        <v>588.5</v>
       </c>
       <c r="K168" s="21">
         <f>IF(OR($B168="",$I168=""),"",$I168-IF($J168="",0,$J168))</f>
@@ -9873,14 +9877,18 @@
       <c r="F169" s="26" t="n">
         <v>176</v>
       </c>
-      <c r="G169" s="24" t="inlineStr"/>
-      <c r="H169" s="25" t="inlineStr"/>
+      <c r="G169" s="24" t="n">
+        <v>46283</v>
+      </c>
+      <c r="H169" s="25" t="n">
+        <v>2164.58</v>
+      </c>
       <c r="I169" s="21">
         <f>IF(OR($B169="",$H169=""),"",IF($C169="LONG",($H169-$E169)*$F169,($E169-$H169)*$F169))</f>
         <v/>
       </c>
       <c r="J169" s="4" t="n">
-        <v>127.24</v>
+        <v>596.58</v>
       </c>
       <c r="K169" s="21">
         <f>IF(OR($B169="",$I169=""),"",$I169-IF($J169="",0,$J169))</f>
@@ -9896,19 +9904,39 @@
       </c>
     </row>
     <row r="170">
-      <c r="A170" s="23" t="n"/>
-      <c r="B170" s="23" t="n"/>
-      <c r="C170" s="23" t="n"/>
-      <c r="D170" s="24" t="n"/>
-      <c r="E170" s="25" t="n"/>
-      <c r="F170" s="26" t="n"/>
-      <c r="G170" s="24" t="n"/>
-      <c r="H170" s="25" t="n"/>
+      <c r="A170" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-34126091813609</t>
+        </is>
+      </c>
+      <c r="B170" s="23" t="inlineStr">
+        <is>
+          <t>SHAREINDIA</t>
+        </is>
+      </c>
+      <c r="C170" s="23" t="inlineStr">
+        <is>
+          <t>SHORT</t>
+        </is>
+      </c>
+      <c r="D170" s="24" t="n">
+        <v>46283</v>
+      </c>
+      <c r="E170" s="25" t="n">
+        <v>223.51</v>
+      </c>
+      <c r="F170" s="26" t="n">
+        <v>1722</v>
+      </c>
+      <c r="G170" s="24" t="inlineStr"/>
+      <c r="H170" s="25" t="inlineStr"/>
       <c r="I170" s="21">
         <f>IF(OR($B170="",$H170=""),"",IF($C170="LONG",($H170-$E170)*$F170,($E170-$H170)*$F170))</f>
         <v/>
       </c>
-      <c r="J170" s="4" t="n"/>
+      <c r="J170" s="4" t="n">
+        <v>0</v>
+      </c>
       <c r="K170" s="21">
         <f>IF(OR($B170="",$I170=""),"",$I170-IF($J170="",0,$J170))</f>
         <v/>
@@ -9923,19 +9951,39 @@
       </c>
     </row>
     <row r="171">
-      <c r="A171" s="23" t="n"/>
-      <c r="B171" s="23" t="n"/>
-      <c r="C171" s="23" t="n"/>
-      <c r="D171" s="24" t="n"/>
-      <c r="E171" s="25" t="n"/>
-      <c r="F171" s="26" t="n"/>
-      <c r="G171" s="24" t="n"/>
-      <c r="H171" s="25" t="n"/>
+      <c r="A171" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-22126091853309</t>
+        </is>
+      </c>
+      <c r="B171" s="23" t="inlineStr">
+        <is>
+          <t>VENUSPIPES</t>
+        </is>
+      </c>
+      <c r="C171" s="23" t="inlineStr">
+        <is>
+          <t>SHORT</t>
+        </is>
+      </c>
+      <c r="D171" s="24" t="n">
+        <v>46283</v>
+      </c>
+      <c r="E171" s="25" t="n">
+        <v>2168.7</v>
+      </c>
+      <c r="F171" s="26" t="n">
+        <v>176</v>
+      </c>
+      <c r="G171" s="24" t="inlineStr"/>
+      <c r="H171" s="25" t="inlineStr"/>
       <c r="I171" s="21">
         <f>IF(OR($B171="",$H171=""),"",IF($C171="LONG",($H171-$E171)*$F171,($E171-$H171)*$F171))</f>
         <v/>
       </c>
-      <c r="J171" s="4" t="n"/>
+      <c r="J171" s="4" t="n">
+        <v>0</v>
+      </c>
       <c r="K171" s="21">
         <f>IF(OR($B171="",$I171=""),"",$I171-IF($J171="",0,$J171))</f>
         <v/>

</xml_diff>

<commit_message>
Data update — 2026-09-21 candle + results refresh
</commit_message>
<xml_diff>
--- a/results/strategy_pnl_simple.xlsx
+++ b/results/strategy_pnl_simple.xlsx
@@ -1473,7 +1473,7 @@
         <v/>
       </c>
       <c r="J4" s="4" t="n">
-        <v>571.79</v>
+        <v>571.78</v>
       </c>
       <c r="K4" s="21">
         <f>IF(OR($B4="",$I4=""),"",$I4-IF($J4="",0,$J4))</f>
@@ -1575,7 +1575,7 @@
         <v/>
       </c>
       <c r="J6" s="4" t="n">
-        <v>570.64</v>
+        <v>570.63</v>
       </c>
       <c r="K6" s="21">
         <f>IF(OR($B6="",$I6=""),"",$I6-IF($J6="",0,$J6))</f>
@@ -1626,7 +1626,7 @@
         <v/>
       </c>
       <c r="J7" s="4" t="n">
-        <v>663.04</v>
+        <v>663.03</v>
       </c>
       <c r="K7" s="21">
         <f>IF(OR($B7="",$I7=""),"",$I7-IF($J7="",0,$J7))</f>
@@ -1677,7 +1677,7 @@
         <v/>
       </c>
       <c r="J8" s="4" t="n">
-        <v>590.95</v>
+        <v>591.04</v>
       </c>
       <c r="K8" s="21">
         <f>IF(OR($B8="",$I8=""),"",$I8-IF($J8="",0,$J8))</f>
@@ -1779,7 +1779,7 @@
         <v/>
       </c>
       <c r="J10" s="4" t="n">
-        <v>398.62</v>
+        <v>398.61</v>
       </c>
       <c r="K10" s="21">
         <f>IF(OR($B10="",$I10=""),"",$I10-IF($J10="",0,$J10))</f>
@@ -1881,7 +1881,7 @@
         <v/>
       </c>
       <c r="J12" s="4" t="n">
-        <v>414.16</v>
+        <v>414.15</v>
       </c>
       <c r="K12" s="21">
         <f>IF(OR($B12="",$I12=""),"",$I12-IF($J12="",0,$J12))</f>
@@ -1983,7 +1983,7 @@
         <v/>
       </c>
       <c r="J14" s="4" t="n">
-        <v>414.49</v>
+        <v>414.48</v>
       </c>
       <c r="K14" s="21">
         <f>IF(OR($B14="",$I14=""),"",$I14-IF($J14="",0,$J14))</f>
@@ -2034,7 +2034,7 @@
         <v/>
       </c>
       <c r="J15" s="4" t="n">
-        <v>380.4</v>
+        <v>380.41</v>
       </c>
       <c r="K15" s="21">
         <f>IF(OR($B15="",$I15=""),"",$I15-IF($J15="",0,$J15))</f>
@@ -2187,7 +2187,7 @@
         <v/>
       </c>
       <c r="J18" s="4" t="n">
-        <v>413.92</v>
+        <v>413.91</v>
       </c>
       <c r="K18" s="21">
         <f>IF(OR($B18="",$I18=""),"",$I18-IF($J18="",0,$J18))</f>
@@ -2238,7 +2238,7 @@
         <v/>
       </c>
       <c r="J19" s="4" t="n">
-        <v>406.46</v>
+        <v>406.45</v>
       </c>
       <c r="K19" s="21">
         <f>IF(OR($B19="",$I19=""),"",$I19-IF($J19="",0,$J19))</f>
@@ -2697,7 +2697,7 @@
         <v/>
       </c>
       <c r="J28" s="4" t="n">
-        <v>870.39</v>
+        <v>870.41</v>
       </c>
       <c r="K28" s="21">
         <f>IF(OR($B28="",$I28=""),"",$I28-IF($J28="",0,$J28))</f>
@@ -2901,7 +2901,7 @@
         <v/>
       </c>
       <c r="J32" s="4" t="n">
-        <v>349.78</v>
+        <v>349.77</v>
       </c>
       <c r="K32" s="21">
         <f>IF(OR($B32="",$I32=""),"",$I32-IF($J32="",0,$J32))</f>
@@ -3003,7 +3003,7 @@
         <v/>
       </c>
       <c r="J34" s="4" t="n">
-        <v>349.81</v>
+        <v>349.8</v>
       </c>
       <c r="K34" s="21">
         <f>IF(OR($B34="",$I34=""),"",$I34-IF($J34="",0,$J34))</f>
@@ -3054,7 +3054,7 @@
         <v/>
       </c>
       <c r="J35" s="4" t="n">
-        <v>386.1</v>
+        <v>386.15</v>
       </c>
       <c r="K35" s="21">
         <f>IF(OR($B35="",$I35=""),"",$I35-IF($J35="",0,$J35))</f>
@@ -3564,7 +3564,7 @@
         <v/>
       </c>
       <c r="J45" s="4" t="n">
-        <v>599.6900000000001</v>
+        <v>599.6799999999999</v>
       </c>
       <c r="K45" s="21">
         <f>IF(OR($B45="",$I45=""),"",$I45-IF($J45="",0,$J45))</f>
@@ -3615,7 +3615,7 @@
         <v/>
       </c>
       <c r="J46" s="4" t="n">
-        <v>600.8</v>
+        <v>600.79</v>
       </c>
       <c r="K46" s="21">
         <f>IF(OR($B46="",$I46=""),"",$I46-IF($J46="",0,$J46))</f>
@@ -3666,7 +3666,7 @@
         <v/>
       </c>
       <c r="J47" s="4" t="n">
-        <v>678.96</v>
+        <v>678.95</v>
       </c>
       <c r="K47" s="21">
         <f>IF(OR($B47="",$I47=""),"",$I47-IF($J47="",0,$J47))</f>
@@ -3717,7 +3717,7 @@
         <v/>
       </c>
       <c r="J48" s="4" t="n">
-        <v>672.39</v>
+        <v>672.4299999999999</v>
       </c>
       <c r="K48" s="21">
         <f>IF(OR($B48="",$I48=""),"",$I48-IF($J48="",0,$J48))</f>
@@ -3819,7 +3819,7 @@
         <v/>
       </c>
       <c r="J50" s="4" t="n">
-        <v>628.03</v>
+        <v>627.9400000000001</v>
       </c>
       <c r="K50" s="21">
         <f>IF(OR($B50="",$I50=""),"",$I50-IF($J50="",0,$J50))</f>
@@ -4023,7 +4023,7 @@
         <v/>
       </c>
       <c r="J54" s="4" t="n">
-        <v>619</v>
+        <v>619.09</v>
       </c>
       <c r="K54" s="21">
         <f>IF(OR($B54="",$I54=""),"",$I54-IF($J54="",0,$J54))</f>
@@ -4176,7 +4176,7 @@
         <v/>
       </c>
       <c r="J57" s="4" t="n">
-        <v>612.26</v>
+        <v>612.28</v>
       </c>
       <c r="K57" s="21">
         <f>IF(OR($B57="",$I57=""),"",$I57-IF($J57="",0,$J57))</f>
@@ -4380,7 +4380,7 @@
         <v/>
       </c>
       <c r="J61" s="4" t="n">
-        <v>692.09</v>
+        <v>692.14</v>
       </c>
       <c r="K61" s="21">
         <f>IF(OR($B61="",$I61=""),"",$I61-IF($J61="",0,$J61))</f>
@@ -4431,7 +4431,7 @@
         <v/>
       </c>
       <c r="J62" s="4" t="n">
-        <v>615.42</v>
+        <v>615.15</v>
       </c>
       <c r="K62" s="21">
         <f>IF(OR($B62="",$I62=""),"",$I62-IF($J62="",0,$J62))</f>
@@ -4533,7 +4533,7 @@
         <v/>
       </c>
       <c r="J64" s="4" t="n">
-        <v>440.42</v>
+        <v>440.43</v>
       </c>
       <c r="K64" s="21">
         <f>IF(OR($B64="",$I64=""),"",$I64-IF($J64="",0,$J64))</f>
@@ -4584,7 +4584,7 @@
         <v/>
       </c>
       <c r="J65" s="4" t="n">
-        <v>386.59</v>
+        <v>386.62</v>
       </c>
       <c r="K65" s="21">
         <f>IF(OR($B65="",$I65=""),"",$I65-IF($J65="",0,$J65))</f>
@@ -4839,7 +4839,7 @@
         <v/>
       </c>
       <c r="J70" s="4" t="n">
-        <v>385.19</v>
+        <v>385.22</v>
       </c>
       <c r="K70" s="21">
         <f>IF(OR($B70="",$I70=""),"",$I70-IF($J70="",0,$J70))</f>
@@ -4890,7 +4890,7 @@
         <v/>
       </c>
       <c r="J71" s="4" t="n">
-        <v>434.27</v>
+        <v>434.29</v>
       </c>
       <c r="K71" s="21">
         <f>IF(OR($B71="",$I71=""),"",$I71-IF($J71="",0,$J71))</f>
@@ -4941,7 +4941,7 @@
         <v/>
       </c>
       <c r="J72" s="4" t="n">
-        <v>411.48</v>
+        <v>376.9</v>
       </c>
       <c r="K72" s="21">
         <f>IF(OR($B72="",$I72=""),"",$I72-IF($J72="",0,$J72))</f>
@@ -5043,7 +5043,7 @@
         <v/>
       </c>
       <c r="J74" s="4" t="n">
-        <v>327.31</v>
+        <v>356.06</v>
       </c>
       <c r="K74" s="21">
         <f>IF(OR($B74="",$I74=""),"",$I74-IF($J74="",0,$J74))</f>
@@ -5094,7 +5094,7 @@
         <v/>
       </c>
       <c r="J75" s="4" t="n">
-        <v>364.56</v>
+        <v>364.64</v>
       </c>
       <c r="K75" s="21">
         <f>IF(OR($B75="",$I75=""),"",$I75-IF($J75="",0,$J75))</f>
@@ -5196,7 +5196,7 @@
         <v/>
       </c>
       <c r="J77" s="4" t="n">
-        <v>411.72</v>
+        <v>411.85</v>
       </c>
       <c r="K77" s="21">
         <f>IF(OR($B77="",$I77=""),"",$I77-IF($J77="",0,$J77))</f>
@@ -5298,7 +5298,7 @@
         <v/>
       </c>
       <c r="J79" s="4" t="n">
-        <v>344.04</v>
+        <v>344.09</v>
       </c>
       <c r="K79" s="21">
         <f>IF(OR($B79="",$I79=""),"",$I79-IF($J79="",0,$J79))</f>
@@ -5349,7 +5349,7 @@
         <v/>
       </c>
       <c r="J80" s="4" t="n">
-        <v>345.48</v>
+        <v>345.53</v>
       </c>
       <c r="K80" s="21">
         <f>IF(OR($B80="",$I80=""),"",$I80-IF($J80="",0,$J80))</f>
@@ -5859,7 +5859,7 @@
         <v/>
       </c>
       <c r="J90" s="4" t="n">
-        <v>894.05</v>
+        <v>894.61</v>
       </c>
       <c r="K90" s="21">
         <f>IF(OR($B90="",$I90=""),"",$I90-IF($J90="",0,$J90))</f>
@@ -5961,7 +5961,7 @@
         <v/>
       </c>
       <c r="J92" s="4" t="n">
-        <v>800.0700000000001</v>
+        <v>800.62</v>
       </c>
       <c r="K92" s="21">
         <f>IF(OR($B92="",$I92=""),"",$I92-IF($J92="",0,$J92))</f>
@@ -6012,7 +6012,7 @@
         <v/>
       </c>
       <c r="J93" s="4" t="n">
-        <v>827.41</v>
+        <v>827.97</v>
       </c>
       <c r="K93" s="21">
         <f>IF(OR($B93="",$I93=""),"",$I93-IF($J93="",0,$J93))</f>
@@ -6063,7 +6063,7 @@
         <v/>
       </c>
       <c r="J94" s="4" t="n">
-        <v>480.62</v>
+        <v>480.84</v>
       </c>
       <c r="K94" s="21">
         <f>IF(OR($B94="",$I94=""),"",$I94-IF($J94="",0,$J94))</f>
@@ -6165,7 +6165,7 @@
         <v/>
       </c>
       <c r="J96" s="4" t="n">
-        <v>474.78</v>
+        <v>474.96</v>
       </c>
       <c r="K96" s="21">
         <f>IF(OR($B96="",$I96=""),"",$I96-IF($J96="",0,$J96))</f>
@@ -6267,7 +6267,7 @@
         <v/>
       </c>
       <c r="J98" s="4" t="n">
-        <v>531.55</v>
+        <v>531.74</v>
       </c>
       <c r="K98" s="21">
         <f>IF(OR($B98="",$I98=""),"",$I98-IF($J98="",0,$J98))</f>
@@ -6471,7 +6471,7 @@
         <v/>
       </c>
       <c r="J102" s="4" t="n">
-        <v>531.77</v>
+        <v>531.95</v>
       </c>
       <c r="K102" s="21">
         <f>IF(OR($B102="",$I102=""),"",$I102-IF($J102="",0,$J102))</f>
@@ -6879,7 +6879,7 @@
         <v/>
       </c>
       <c r="J110" s="4" t="n">
-        <v>481.01</v>
+        <v>481.18</v>
       </c>
       <c r="K110" s="21">
         <f>IF(OR($B110="",$I110=""),"",$I110-IF($J110="",0,$J110))</f>
@@ -6981,7 +6981,7 @@
         <v/>
       </c>
       <c r="J112" s="4" t="n">
-        <v>420.31</v>
+        <v>420.46</v>
       </c>
       <c r="K112" s="21">
         <f>IF(OR($B112="",$I112=""),"",$I112-IF($J112="",0,$J112))</f>
@@ -7185,7 +7185,7 @@
         <v/>
       </c>
       <c r="J116" s="4" t="n">
-        <v>428.73</v>
+        <v>428.94</v>
       </c>
       <c r="K116" s="21">
         <f>IF(OR($B116="",$I116=""),"",$I116-IF($J116="",0,$J116))</f>
@@ -7236,7 +7236,7 @@
         <v/>
       </c>
       <c r="J117" s="4" t="n">
-        <v>546.5599999999999</v>
+        <v>546.78</v>
       </c>
       <c r="K117" s="21">
         <f>IF(OR($B117="",$I117=""),"",$I117-IF($J117="",0,$J117))</f>
@@ -7389,7 +7389,7 @@
         <v/>
       </c>
       <c r="J120" s="4" t="n">
-        <v>425</v>
+        <v>425.16</v>
       </c>
       <c r="K120" s="21">
         <f>IF(OR($B120="",$I120=""),"",$I120-IF($J120="",0,$J120))</f>
@@ -7440,7 +7440,7 @@
         <v/>
       </c>
       <c r="J121" s="4" t="n">
-        <v>371.71</v>
+        <v>371.83</v>
       </c>
       <c r="K121" s="21">
         <f>IF(OR($B121="",$I121=""),"",$I121-IF($J121="",0,$J121))</f>
@@ -7746,7 +7746,7 @@
         <v/>
       </c>
       <c r="J127" s="4" t="n">
-        <v>642.74</v>
+        <v>642.97</v>
       </c>
       <c r="K127" s="21">
         <f>IF(OR($B127="",$I127=""),"",$I127-IF($J127="",0,$J127))</f>
@@ -7848,7 +7848,7 @@
         <v/>
       </c>
       <c r="J129" s="4" t="n">
-        <v>638.59</v>
+        <v>638.8200000000001</v>
       </c>
       <c r="K129" s="21">
         <f>IF(OR($B129="",$I129=""),"",$I129-IF($J129="",0,$J129))</f>
@@ -7950,7 +7950,7 @@
         <v/>
       </c>
       <c r="J131" s="4" t="n">
-        <v>654.36</v>
+        <v>654.5700000000001</v>
       </c>
       <c r="K131" s="21">
         <f>IF(OR($B131="",$I131=""),"",$I131-IF($J131="",0,$J131))</f>
@@ -8052,7 +8052,7 @@
         <v/>
       </c>
       <c r="J133" s="4" t="n">
-        <v>564.41</v>
+        <v>564.64</v>
       </c>
       <c r="K133" s="21">
         <f>IF(OR($B133="",$I133=""),"",$I133-IF($J133="",0,$J133))</f>
@@ -8103,7 +8103,7 @@
         <v/>
       </c>
       <c r="J134" s="4" t="n">
-        <v>632.37</v>
+        <v>632.6</v>
       </c>
       <c r="K134" s="21">
         <f>IF(OR($B134="",$I134=""),"",$I134-IF($J134="",0,$J134))</f>
@@ -8154,7 +8154,7 @@
         <v/>
       </c>
       <c r="J135" s="4" t="n">
-        <v>498.25</v>
+        <v>498.61</v>
       </c>
       <c r="K135" s="21">
         <f>IF(OR($B135="",$I135=""),"",$I135-IF($J135="",0,$J135))</f>
@@ -8307,7 +8307,7 @@
         <v/>
       </c>
       <c r="J138" s="4" t="n">
-        <v>494.99</v>
+        <v>495.35</v>
       </c>
       <c r="K138" s="21">
         <f>IF(OR($B138="",$I138=""),"",$I138-IF($J138="",0,$J138))</f>
@@ -8409,7 +8409,7 @@
         <v/>
       </c>
       <c r="J140" s="4" t="n">
-        <v>504.92</v>
+        <v>504.65</v>
       </c>
       <c r="K140" s="21">
         <f>IF(OR($B140="",$I140=""),"",$I140-IF($J140="",0,$J140))</f>
@@ -8460,7 +8460,7 @@
         <v/>
       </c>
       <c r="J141" s="4" t="n">
-        <v>491.81</v>
+        <v>492.34</v>
       </c>
       <c r="K141" s="21">
         <f>IF(OR($B141="",$I141=""),"",$I141-IF($J141="",0,$J141))</f>
@@ -8511,7 +8511,7 @@
         <v/>
       </c>
       <c r="J142" s="4" t="n">
-        <v>467.6</v>
+        <v>467.9</v>
       </c>
       <c r="K142" s="21">
         <f>IF(OR($B142="",$I142=""),"",$I142-IF($J142="",0,$J142))</f>
@@ -8664,7 +8664,7 @@
         <v/>
       </c>
       <c r="J145" s="4" t="n">
-        <v>543.27</v>
+        <v>542.99</v>
       </c>
       <c r="K145" s="21">
         <f>IF(OR($B145="",$I145=""),"",$I145-IF($J145="",0,$J145))</f>
@@ -9225,7 +9225,7 @@
         <v/>
       </c>
       <c r="J156" s="4" t="n">
-        <v>460.1</v>
+        <v>435.16</v>
       </c>
       <c r="K156" s="21">
         <f>IF(OR($B156="",$I156=""),"",$I156-IF($J156="",0,$J156))</f>
@@ -9480,7 +9480,7 @@
         <v/>
       </c>
       <c r="J161" s="4" t="n">
-        <v>461.81</v>
+        <v>461.82</v>
       </c>
       <c r="K161" s="21">
         <f>IF(OR($B161="",$I161=""),"",$I161-IF($J161="",0,$J161))</f>
@@ -9837,7 +9837,7 @@
         <v/>
       </c>
       <c r="J168" s="4" t="n">
-        <v>588.5</v>
+        <v>626.4400000000001</v>
       </c>
       <c r="K168" s="21">
         <f>IF(OR($B168="",$I168=""),"",$I168-IF($J168="",0,$J168))</f>
@@ -9888,7 +9888,7 @@
         <v/>
       </c>
       <c r="J169" s="4" t="n">
-        <v>596.58</v>
+        <v>634.4299999999999</v>
       </c>
       <c r="K169" s="21">
         <f>IF(OR($B169="",$I169=""),"",$I169-IF($J169="",0,$J169))</f>
@@ -9928,14 +9928,18 @@
       <c r="F170" s="26" t="n">
         <v>1726</v>
       </c>
-      <c r="G170" s="24" t="inlineStr"/>
-      <c r="H170" s="25" t="inlineStr"/>
+      <c r="G170" s="24" t="n">
+        <v>46286</v>
+      </c>
+      <c r="H170" s="25" t="n">
+        <v>85.17</v>
+      </c>
       <c r="I170" s="21">
         <f>IF(OR($B170="",$H170=""),"",IF($C170="LONG",($H170-$E170)*$F170,($E170-$H170)*$F170))</f>
         <v/>
       </c>
       <c r="J170" s="4" t="n">
-        <v>14.75</v>
+        <v>192.79</v>
       </c>
       <c r="K170" s="21">
         <f>IF(OR($B170="",$I170=""),"",$I170-IF($J170="",0,$J170))</f>
@@ -9975,14 +9979,18 @@
       <c r="F171" s="26" t="n">
         <v>263</v>
       </c>
-      <c r="G171" s="24" t="inlineStr"/>
-      <c r="H171" s="25" t="inlineStr"/>
+      <c r="G171" s="24" t="n">
+        <v>46286</v>
+      </c>
+      <c r="H171" s="25" t="n">
+        <v>1139.97</v>
+      </c>
       <c r="I171" s="21">
         <f>IF(OR($B171="",$H171=""),"",IF($C171="LONG",($H171-$E171)*$F171,($E171-$H171)*$F171))</f>
         <v/>
       </c>
       <c r="J171" s="4" t="n">
-        <v>50.15</v>
+        <v>627.5599999999999</v>
       </c>
       <c r="K171" s="21">
         <f>IF(OR($B171="",$I171=""),"",$I171-IF($J171="",0,$J171))</f>
@@ -10022,14 +10030,18 @@
       <c r="F172" s="26" t="n">
         <v>568</v>
       </c>
-      <c r="G172" s="24" t="inlineStr"/>
-      <c r="H172" s="25" t="inlineStr"/>
+      <c r="G172" s="24" t="n">
+        <v>46286</v>
+      </c>
+      <c r="H172" s="25" t="n">
+        <v>533.65</v>
+      </c>
       <c r="I172" s="21">
         <f>IF(OR($B172="",$H172=""),"",IF($C172="LONG",($H172-$E172)*$F172,($E172-$H172)*$F172))</f>
         <v/>
       </c>
       <c r="J172" s="4" t="n">
-        <v>50.15</v>
+        <v>612.35</v>
       </c>
       <c r="K172" s="21">
         <f>IF(OR($B172="",$I172=""),"",$I172-IF($J172="",0,$J172))</f>
@@ -10069,14 +10081,18 @@
       <c r="F173" s="26" t="n">
         <v>2021</v>
       </c>
-      <c r="G173" s="24" t="inlineStr"/>
-      <c r="H173" s="25" t="inlineStr"/>
+      <c r="G173" s="24" t="n">
+        <v>46286</v>
+      </c>
+      <c r="H173" s="25" t="n">
+        <v>155.57</v>
+      </c>
       <c r="I173" s="21">
         <f>IF(OR($B173="",$H173=""),"",IF($C173="LONG",($H173-$E173)*$F173,($E173-$H173)*$F173))</f>
         <v/>
       </c>
       <c r="J173" s="4" t="n">
-        <v>50.15</v>
+        <v>629.67</v>
       </c>
       <c r="K173" s="21">
         <f>IF(OR($B173="",$I173=""),"",$I173-IF($J173="",0,$J173))</f>
@@ -10127,7 +10143,7 @@
         <v/>
       </c>
       <c r="J174" s="4" t="n">
-        <v>0</v>
+        <v>548.39</v>
       </c>
       <c r="K174" s="21">
         <f>IF(OR($B174="",$I174=""),"",$I174-IF($J174="",0,$J174))</f>
@@ -10167,14 +10183,18 @@
       <c r="F175" s="26" t="n">
         <v>632</v>
       </c>
-      <c r="G175" s="24" t="inlineStr"/>
-      <c r="H175" s="25" t="inlineStr"/>
+      <c r="G175" s="24" t="n">
+        <v>46286</v>
+      </c>
+      <c r="H175" s="25" t="n">
+        <v>477.78</v>
+      </c>
       <c r="I175" s="21">
         <f>IF(OR($B175="",$H175=""),"",IF($C175="LONG",($H175-$E175)*$F175,($E175-$H175)*$F175))</f>
         <v/>
       </c>
       <c r="J175" s="4" t="n">
-        <v>50.15</v>
+        <v>614.6</v>
       </c>
       <c r="K175" s="21">
         <f>IF(OR($B175="",$I175=""),"",$I175-IF($J175="",0,$J175))</f>
@@ -10225,7 +10245,7 @@
         <v/>
       </c>
       <c r="J176" s="4" t="n">
-        <v>0</v>
+        <v>550.84</v>
       </c>
       <c r="K176" s="21">
         <f>IF(OR($B176="",$I176=""),"",$I176-IF($J176="",0,$J176))</f>
@@ -10241,19 +10261,43 @@
       </c>
     </row>
     <row r="177">
-      <c r="A177" s="23" t="n"/>
-      <c r="B177" s="23" t="n"/>
-      <c r="C177" s="23" t="n"/>
-      <c r="D177" s="24" t="n"/>
-      <c r="E177" s="25" t="n"/>
-      <c r="F177" s="26" t="n"/>
-      <c r="G177" s="24" t="n"/>
-      <c r="H177" s="25" t="n"/>
+      <c r="A177" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-321260921417509</t>
+        </is>
+      </c>
+      <c r="B177" s="23" t="inlineStr">
+        <is>
+          <t>GRAUWEIL</t>
+        </is>
+      </c>
+      <c r="C177" s="23" t="inlineStr">
+        <is>
+          <t>SHORT</t>
+        </is>
+      </c>
+      <c r="D177" s="24" t="n">
+        <v>46286</v>
+      </c>
+      <c r="E177" s="25" t="n">
+        <v>85.12</v>
+      </c>
+      <c r="F177" s="26" t="n">
+        <v>1726</v>
+      </c>
+      <c r="G177" s="24" t="n">
+        <v>46286</v>
+      </c>
+      <c r="H177" s="25" t="n">
+        <v>84.69</v>
+      </c>
       <c r="I177" s="21">
         <f>IF(OR($B177="",$H177=""),"",IF($C177="LONG",($H177-$E177)*$F177,($E177-$H177)*$F177))</f>
         <v/>
       </c>
-      <c r="J177" s="4" t="n"/>
+      <c r="J177" s="4" t="n">
+        <v>0</v>
+      </c>
       <c r="K177" s="21">
         <f>IF(OR($B177="",$I177=""),"",$I177-IF($J177="",0,$J177))</f>
         <v/>
@@ -10268,19 +10312,43 @@
       </c>
     </row>
     <row r="178">
-      <c r="A178" s="23" t="n"/>
-      <c r="B178" s="23" t="n"/>
-      <c r="C178" s="23" t="n"/>
-      <c r="D178" s="24" t="n"/>
-      <c r="E178" s="25" t="n"/>
-      <c r="F178" s="26" t="n"/>
-      <c r="G178" s="24" t="n"/>
-      <c r="H178" s="25" t="n"/>
+      <c r="A178" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-23126092113309</t>
+        </is>
+      </c>
+      <c r="B178" s="23" t="inlineStr">
+        <is>
+          <t>LUXIND</t>
+        </is>
+      </c>
+      <c r="C178" s="23" t="inlineStr">
+        <is>
+          <t>SHORT</t>
+        </is>
+      </c>
+      <c r="D178" s="24" t="n">
+        <v>46286</v>
+      </c>
+      <c r="E178" s="25" t="n">
+        <v>1142.1</v>
+      </c>
+      <c r="F178" s="26" t="n">
+        <v>263</v>
+      </c>
+      <c r="G178" s="24" t="n">
+        <v>46286</v>
+      </c>
+      <c r="H178" s="25" t="n">
+        <v>1197.67</v>
+      </c>
       <c r="I178" s="21">
         <f>IF(OR($B178="",$H178=""),"",IF($C178="LONG",($H178-$E178)*$F178,($E178-$H178)*$F178))</f>
         <v/>
       </c>
-      <c r="J178" s="4" t="n"/>
+      <c r="J178" s="4" t="n">
+        <v>0</v>
+      </c>
       <c r="K178" s="21">
         <f>IF(OR($B178="",$I178=""),"",$I178-IF($J178="",0,$J178))</f>
         <v/>
@@ -10295,19 +10363,43 @@
       </c>
     </row>
     <row r="179">
-      <c r="A179" s="23" t="n"/>
-      <c r="B179" s="23" t="n"/>
-      <c r="C179" s="23" t="n"/>
-      <c r="D179" s="24" t="n"/>
-      <c r="E179" s="25" t="n"/>
-      <c r="F179" s="26" t="n"/>
-      <c r="G179" s="24" t="n"/>
-      <c r="H179" s="25" t="n"/>
+      <c r="A179" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-22126092158309</t>
+        </is>
+      </c>
+      <c r="B179" s="23" t="inlineStr">
+        <is>
+          <t>NRBBEARING</t>
+        </is>
+      </c>
+      <c r="C179" s="23" t="inlineStr">
+        <is>
+          <t>SHORT</t>
+        </is>
+      </c>
+      <c r="D179" s="24" t="n">
+        <v>46286</v>
+      </c>
+      <c r="E179" s="25" t="n">
+        <v>535.51</v>
+      </c>
+      <c r="F179" s="26" t="n">
+        <v>568</v>
+      </c>
+      <c r="G179" s="24" t="n">
+        <v>46286</v>
+      </c>
+      <c r="H179" s="25" t="n">
+        <v>531.6799999999999</v>
+      </c>
       <c r="I179" s="21">
         <f>IF(OR($B179="",$H179=""),"",IF($C179="LONG",($H179-$E179)*$F179,($E179-$H179)*$F179))</f>
         <v/>
       </c>
-      <c r="J179" s="4" t="n"/>
+      <c r="J179" s="4" t="n">
+        <v>0</v>
+      </c>
       <c r="K179" s="21">
         <f>IF(OR($B179="",$I179=""),"",$I179-IF($J179="",0,$J179))</f>
         <v/>
@@ -10322,19 +10414,43 @@
       </c>
     </row>
     <row r="180">
-      <c r="A180" s="23" t="n"/>
-      <c r="B180" s="23" t="n"/>
-      <c r="C180" s="23" t="n"/>
-      <c r="D180" s="24" t="n"/>
-      <c r="E180" s="25" t="n"/>
-      <c r="F180" s="26" t="n"/>
-      <c r="G180" s="24" t="n"/>
-      <c r="H180" s="25" t="n"/>
+      <c r="A180" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-32126092161209</t>
+        </is>
+      </c>
+      <c r="B180" s="23" t="inlineStr">
+        <is>
+          <t>SAMBHV</t>
+        </is>
+      </c>
+      <c r="C180" s="23" t="inlineStr">
+        <is>
+          <t>SHORT</t>
+        </is>
+      </c>
+      <c r="D180" s="24" t="n">
+        <v>46286</v>
+      </c>
+      <c r="E180" s="25" t="n">
+        <v>156.2</v>
+      </c>
+      <c r="F180" s="26" t="n">
+        <v>2021</v>
+      </c>
+      <c r="G180" s="24" t="n">
+        <v>46286</v>
+      </c>
+      <c r="H180" s="25" t="n">
+        <v>153.42</v>
+      </c>
       <c r="I180" s="21">
         <f>IF(OR($B180="",$H180=""),"",IF($C180="LONG",($H180-$E180)*$F180,($E180-$H180)*$F180))</f>
         <v/>
       </c>
-      <c r="J180" s="4" t="n"/>
+      <c r="J180" s="4" t="n">
+        <v>0</v>
+      </c>
       <c r="K180" s="21">
         <f>IF(OR($B180="",$I180=""),"",$I180-IF($J180="",0,$J180))</f>
         <v/>
@@ -10349,19 +10465,43 @@
       </c>
     </row>
     <row r="181">
-      <c r="A181" s="23" t="n"/>
-      <c r="B181" s="23" t="n"/>
-      <c r="C181" s="23" t="n"/>
-      <c r="D181" s="24" t="n"/>
-      <c r="E181" s="25" t="n"/>
-      <c r="F181" s="26" t="n"/>
-      <c r="G181" s="24" t="n"/>
-      <c r="H181" s="25" t="n"/>
+      <c r="A181" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-23126092113209</t>
+        </is>
+      </c>
+      <c r="B181" s="23" t="inlineStr">
+        <is>
+          <t>TALBROAUTO</t>
+        </is>
+      </c>
+      <c r="C181" s="23" t="inlineStr">
+        <is>
+          <t>SHORT</t>
+        </is>
+      </c>
+      <c r="D181" s="24" t="n">
+        <v>46286</v>
+      </c>
+      <c r="E181" s="25" t="n">
+        <v>478.39</v>
+      </c>
+      <c r="F181" s="26" t="n">
+        <v>632</v>
+      </c>
+      <c r="G181" s="24" t="n">
+        <v>46286</v>
+      </c>
+      <c r="H181" s="25" t="n">
+        <v>465.51</v>
+      </c>
       <c r="I181" s="21">
         <f>IF(OR($B181="",$H181=""),"",IF($C181="LONG",($H181-$E181)*$F181,($E181-$H181)*$F181))</f>
         <v/>
       </c>
-      <c r="J181" s="4" t="n"/>
+      <c r="J181" s="4" t="n">
+        <v>0</v>
+      </c>
       <c r="K181" s="21">
         <f>IF(OR($B181="",$I181=""),"",$I181-IF($J181="",0,$J181))</f>
         <v/>

</xml_diff>

<commit_message>
Reconcile 6 manual trades from 2026-09-21 into position tracking
ASHIANA, INDORAMA, JASH, JAYKAY, KROSS, REFEX were bought manually via the
Dhan app/web today (correlationId=NA, algoId=0, MARKET/LIMIT order type,
zero footprint in dhan_trades.log -- same fingerprint as the RML/INDNIPPON
external-order cases), unrelated to run_entry_321's own 3:21pm attempt,
which separately skipped all 11 of today's real signals for insufficient
balance. KROSS's order shows orderStatus=CANCELLED but filledQty=233 -- a
genuine partial fill, not a clean zero-fill cancel.

Added to positions_dhan_long.json as status=open so tomorrow's
place_targets_915/check_exit_916/force_exit_1159 pick them up like any
other position. strategy_pnl_simple.xlsx regenerated via the existing
_sync_pnl_workbook() to include them.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/results/strategy_pnl_simple.xlsx
+++ b/results/strategy_pnl_simple.xlsx
@@ -4941,7 +4941,7 @@
         <v/>
       </c>
       <c r="J72" s="4" t="n">
-        <v>376.9</v>
+        <v>411.21</v>
       </c>
       <c r="K72" s="21">
         <f>IF(OR($B72="",$I72=""),"",$I72-IF($J72="",0,$J72))</f>
@@ -5043,7 +5043,7 @@
         <v/>
       </c>
       <c r="J74" s="4" t="n">
-        <v>356.06</v>
+        <v>355.78</v>
       </c>
       <c r="K74" s="21">
         <f>IF(OR($B74="",$I74=""),"",$I74-IF($J74="",0,$J74))</f>
@@ -5094,7 +5094,7 @@
         <v/>
       </c>
       <c r="J75" s="4" t="n">
-        <v>364.64</v>
+        <v>364.3</v>
       </c>
       <c r="K75" s="21">
         <f>IF(OR($B75="",$I75=""),"",$I75-IF($J75="",0,$J75))</f>
@@ -5196,7 +5196,7 @@
         <v/>
       </c>
       <c r="J77" s="4" t="n">
-        <v>411.85</v>
+        <v>411.49</v>
       </c>
       <c r="K77" s="21">
         <f>IF(OR($B77="",$I77=""),"",$I77-IF($J77="",0,$J77))</f>
@@ -5298,7 +5298,7 @@
         <v/>
       </c>
       <c r="J79" s="4" t="n">
-        <v>344.09</v>
+        <v>343.88</v>
       </c>
       <c r="K79" s="21">
         <f>IF(OR($B79="",$I79=""),"",$I79-IF($J79="",0,$J79))</f>
@@ -5349,7 +5349,7 @@
         <v/>
       </c>
       <c r="J80" s="4" t="n">
-        <v>345.53</v>
+        <v>345.32</v>
       </c>
       <c r="K80" s="21">
         <f>IF(OR($B80="",$I80=""),"",$I80-IF($J80="",0,$J80))</f>
@@ -5859,7 +5859,7 @@
         <v/>
       </c>
       <c r="J90" s="4" t="n">
-        <v>894.61</v>
+        <v>891.87</v>
       </c>
       <c r="K90" s="21">
         <f>IF(OR($B90="",$I90=""),"",$I90-IF($J90="",0,$J90))</f>
@@ -5961,7 +5961,7 @@
         <v/>
       </c>
       <c r="J92" s="4" t="n">
-        <v>800.62</v>
+        <v>797.89</v>
       </c>
       <c r="K92" s="21">
         <f>IF(OR($B92="",$I92=""),"",$I92-IF($J92="",0,$J92))</f>
@@ -6012,7 +6012,7 @@
         <v/>
       </c>
       <c r="J93" s="4" t="n">
-        <v>827.97</v>
+        <v>825.22</v>
       </c>
       <c r="K93" s="21">
         <f>IF(OR($B93="",$I93=""),"",$I93-IF($J93="",0,$J93))</f>
@@ -6063,7 +6063,7 @@
         <v/>
       </c>
       <c r="J94" s="4" t="n">
-        <v>480.84</v>
+        <v>479.87</v>
       </c>
       <c r="K94" s="21">
         <f>IF(OR($B94="",$I94=""),"",$I94-IF($J94="",0,$J94))</f>
@@ -6165,7 +6165,7 @@
         <v/>
       </c>
       <c r="J96" s="4" t="n">
-        <v>474.96</v>
+        <v>474.05</v>
       </c>
       <c r="K96" s="21">
         <f>IF(OR($B96="",$I96=""),"",$I96-IF($J96="",0,$J96))</f>
@@ -6267,7 +6267,7 @@
         <v/>
       </c>
       <c r="J98" s="4" t="n">
-        <v>531.74</v>
+        <v>530.83</v>
       </c>
       <c r="K98" s="21">
         <f>IF(OR($B98="",$I98=""),"",$I98-IF($J98="",0,$J98))</f>
@@ -6471,7 +6471,7 @@
         <v/>
       </c>
       <c r="J102" s="4" t="n">
-        <v>531.95</v>
+        <v>531.04</v>
       </c>
       <c r="K102" s="21">
         <f>IF(OR($B102="",$I102=""),"",$I102-IF($J102="",0,$J102))</f>
@@ -6879,7 +6879,7 @@
         <v/>
       </c>
       <c r="J110" s="4" t="n">
-        <v>481.18</v>
+        <v>480.28</v>
       </c>
       <c r="K110" s="21">
         <f>IF(OR($B110="",$I110=""),"",$I110-IF($J110="",0,$J110))</f>
@@ -6981,7 +6981,7 @@
         <v/>
       </c>
       <c r="J112" s="4" t="n">
-        <v>420.46</v>
+        <v>419.68</v>
       </c>
       <c r="K112" s="21">
         <f>IF(OR($B112="",$I112=""),"",$I112-IF($J112="",0,$J112))</f>
@@ -7185,7 +7185,7 @@
         <v/>
       </c>
       <c r="J116" s="4" t="n">
-        <v>428.94</v>
+        <v>428.22</v>
       </c>
       <c r="K116" s="21">
         <f>IF(OR($B116="",$I116=""),"",$I116-IF($J116="",0,$J116))</f>
@@ -7236,7 +7236,7 @@
         <v/>
       </c>
       <c r="J117" s="4" t="n">
-        <v>546.78</v>
+        <v>545.7</v>
       </c>
       <c r="K117" s="21">
         <f>IF(OR($B117="",$I117=""),"",$I117-IF($J117="",0,$J117))</f>
@@ -7389,7 +7389,7 @@
         <v/>
       </c>
       <c r="J120" s="4" t="n">
-        <v>425.16</v>
+        <v>424.46</v>
       </c>
       <c r="K120" s="21">
         <f>IF(OR($B120="",$I120=""),"",$I120-IF($J120="",0,$J120))</f>
@@ -7440,7 +7440,7 @@
         <v/>
       </c>
       <c r="J121" s="4" t="n">
-        <v>371.83</v>
+        <v>371.24</v>
       </c>
       <c r="K121" s="21">
         <f>IF(OR($B121="",$I121=""),"",$I121-IF($J121="",0,$J121))</f>
@@ -7746,7 +7746,7 @@
         <v/>
       </c>
       <c r="J127" s="4" t="n">
-        <v>642.97</v>
+        <v>641.84</v>
       </c>
       <c r="K127" s="21">
         <f>IF(OR($B127="",$I127=""),"",$I127-IF($J127="",0,$J127))</f>
@@ -7848,7 +7848,7 @@
         <v/>
       </c>
       <c r="J129" s="4" t="n">
-        <v>638.8200000000001</v>
+        <v>637.6799999999999</v>
       </c>
       <c r="K129" s="21">
         <f>IF(OR($B129="",$I129=""),"",$I129-IF($J129="",0,$J129))</f>
@@ -7950,7 +7950,7 @@
         <v/>
       </c>
       <c r="J131" s="4" t="n">
-        <v>654.5700000000001</v>
+        <v>653.29</v>
       </c>
       <c r="K131" s="21">
         <f>IF(OR($B131="",$I131=""),"",$I131-IF($J131="",0,$J131))</f>
@@ -8052,7 +8052,7 @@
         <v/>
       </c>
       <c r="J133" s="4" t="n">
-        <v>564.64</v>
+        <v>563.51</v>
       </c>
       <c r="K133" s="21">
         <f>IF(OR($B133="",$I133=""),"",$I133-IF($J133="",0,$J133))</f>
@@ -8103,7 +8103,7 @@
         <v/>
       </c>
       <c r="J134" s="4" t="n">
-        <v>632.6</v>
+        <v>631.48</v>
       </c>
       <c r="K134" s="21">
         <f>IF(OR($B134="",$I134=""),"",$I134-IF($J134="",0,$J134))</f>
@@ -8154,7 +8154,7 @@
         <v/>
       </c>
       <c r="J135" s="4" t="n">
-        <v>498.61</v>
+        <v>496.84</v>
       </c>
       <c r="K135" s="21">
         <f>IF(OR($B135="",$I135=""),"",$I135-IF($J135="",0,$J135))</f>
@@ -8307,7 +8307,7 @@
         <v/>
       </c>
       <c r="J138" s="4" t="n">
-        <v>495.35</v>
+        <v>493.59</v>
       </c>
       <c r="K138" s="21">
         <f>IF(OR($B138="",$I138=""),"",$I138-IF($J138="",0,$J138))</f>
@@ -8409,7 +8409,7 @@
         <v/>
       </c>
       <c r="J140" s="4" t="n">
-        <v>504.65</v>
+        <v>502.8</v>
       </c>
       <c r="K140" s="21">
         <f>IF(OR($B140="",$I140=""),"",$I140-IF($J140="",0,$J140))</f>
@@ -8460,7 +8460,7 @@
         <v/>
       </c>
       <c r="J141" s="4" t="n">
-        <v>492.34</v>
+        <v>490.63</v>
       </c>
       <c r="K141" s="21">
         <f>IF(OR($B141="",$I141=""),"",$I141-IF($J141="",0,$J141))</f>
@@ -8511,7 +8511,7 @@
         <v/>
       </c>
       <c r="J142" s="4" t="n">
-        <v>467.9</v>
+        <v>466.42</v>
       </c>
       <c r="K142" s="21">
         <f>IF(OR($B142="",$I142=""),"",$I142-IF($J142="",0,$J142))</f>
@@ -8664,7 +8664,7 @@
         <v/>
       </c>
       <c r="J145" s="4" t="n">
-        <v>542.99</v>
+        <v>541.16</v>
       </c>
       <c r="K145" s="21">
         <f>IF(OR($B145="",$I145=""),"",$I145-IF($J145="",0,$J145))</f>
@@ -10263,40 +10263,36 @@
     <row r="177">
       <c r="A177" s="23" t="inlineStr">
         <is>
-          <t>DHAN-321260921417509</t>
+          <t>DHAN-241260921697209</t>
         </is>
       </c>
       <c r="B177" s="23" t="inlineStr">
         <is>
-          <t>GRAUWEIL</t>
+          <t>ASHIANA</t>
         </is>
       </c>
       <c r="C177" s="23" t="inlineStr">
         <is>
-          <t>SHORT</t>
+          <t>LONG</t>
         </is>
       </c>
       <c r="D177" s="24" t="n">
         <v>46286</v>
       </c>
       <c r="E177" s="25" t="n">
-        <v>85.12</v>
+        <v>406.58957</v>
       </c>
       <c r="F177" s="26" t="n">
-        <v>1726</v>
-      </c>
-      <c r="G177" s="24" t="n">
-        <v>46286</v>
-      </c>
-      <c r="H177" s="25" t="n">
-        <v>84.69</v>
-      </c>
+        <v>340</v>
+      </c>
+      <c r="G177" s="24" t="inlineStr"/>
+      <c r="H177" s="25" t="inlineStr"/>
       <c r="I177" s="21">
         <f>IF(OR($B177="",$H177=""),"",IF($C177="LONG",($H177-$E177)*$F177,($E177-$H177)*$F177))</f>
         <v/>
       </c>
       <c r="J177" s="4" t="n">
-        <v>0</v>
+        <v>50.15</v>
       </c>
       <c r="K177" s="21">
         <f>IF(OR($B177="",$I177=""),"",$I177-IF($J177="",0,$J177))</f>
@@ -10314,12 +10310,12 @@
     <row r="178">
       <c r="A178" s="23" t="inlineStr">
         <is>
-          <t>DHAN-23126092113309</t>
+          <t>DHAN-321260921417509</t>
         </is>
       </c>
       <c r="B178" s="23" t="inlineStr">
         <is>
-          <t>LUXIND</t>
+          <t>GRAUWEIL</t>
         </is>
       </c>
       <c r="C178" s="23" t="inlineStr">
@@ -10331,16 +10327,16 @@
         <v>46286</v>
       </c>
       <c r="E178" s="25" t="n">
-        <v>1142.1</v>
+        <v>85.12</v>
       </c>
       <c r="F178" s="26" t="n">
-        <v>263</v>
+        <v>1726</v>
       </c>
       <c r="G178" s="24" t="n">
         <v>46286</v>
       </c>
       <c r="H178" s="25" t="n">
-        <v>1197.67</v>
+        <v>84.69</v>
       </c>
       <c r="I178" s="21">
         <f>IF(OR($B178="",$H178=""),"",IF($C178="LONG",($H178-$E178)*$F178,($E178-$H178)*$F178))</f>
@@ -10365,40 +10361,36 @@
     <row r="179">
       <c r="A179" s="23" t="inlineStr">
         <is>
-          <t>DHAN-22126092158309</t>
+          <t>DHAN-241260921699009</t>
         </is>
       </c>
       <c r="B179" s="23" t="inlineStr">
         <is>
-          <t>NRBBEARING</t>
+          <t>INDORAMA</t>
         </is>
       </c>
       <c r="C179" s="23" t="inlineStr">
         <is>
-          <t>SHORT</t>
+          <t>LONG</t>
         </is>
       </c>
       <c r="D179" s="24" t="n">
         <v>46286</v>
       </c>
       <c r="E179" s="25" t="n">
-        <v>535.51</v>
+        <v>105.67</v>
       </c>
       <c r="F179" s="26" t="n">
-        <v>568</v>
-      </c>
-      <c r="G179" s="24" t="n">
-        <v>46286</v>
-      </c>
-      <c r="H179" s="25" t="n">
-        <v>531.6799999999999</v>
-      </c>
+        <v>1300</v>
+      </c>
+      <c r="G179" s="24" t="inlineStr"/>
+      <c r="H179" s="25" t="inlineStr"/>
       <c r="I179" s="21">
         <f>IF(OR($B179="",$H179=""),"",IF($C179="LONG",($H179-$E179)*$F179,($E179-$H179)*$F179))</f>
         <v/>
       </c>
       <c r="J179" s="4" t="n">
-        <v>0</v>
+        <v>50.15</v>
       </c>
       <c r="K179" s="21">
         <f>IF(OR($B179="",$I179=""),"",$I179-IF($J179="",0,$J179))</f>
@@ -10416,40 +10408,36 @@
     <row r="180">
       <c r="A180" s="23" t="inlineStr">
         <is>
-          <t>DHAN-32126092161209</t>
+          <t>DHAN-351260921486209</t>
         </is>
       </c>
       <c r="B180" s="23" t="inlineStr">
         <is>
-          <t>SAMBHV</t>
+          <t>JASH</t>
         </is>
       </c>
       <c r="C180" s="23" t="inlineStr">
         <is>
-          <t>SHORT</t>
+          <t>LONG</t>
         </is>
       </c>
       <c r="D180" s="24" t="n">
         <v>46286</v>
       </c>
       <c r="E180" s="25" t="n">
-        <v>156.2</v>
+        <v>580.8</v>
       </c>
       <c r="F180" s="26" t="n">
-        <v>2021</v>
-      </c>
-      <c r="G180" s="24" t="n">
-        <v>46286</v>
-      </c>
-      <c r="H180" s="25" t="n">
-        <v>153.42</v>
-      </c>
+        <v>244</v>
+      </c>
+      <c r="G180" s="24" t="inlineStr"/>
+      <c r="H180" s="25" t="inlineStr"/>
       <c r="I180" s="21">
         <f>IF(OR($B180="",$H180=""),"",IF($C180="LONG",($H180-$E180)*$F180,($E180-$H180)*$F180))</f>
         <v/>
       </c>
       <c r="J180" s="4" t="n">
-        <v>0</v>
+        <v>50.15</v>
       </c>
       <c r="K180" s="21">
         <f>IF(OR($B180="",$I180=""),"",$I180-IF($J180="",0,$J180))</f>
@@ -10467,40 +10455,36 @@
     <row r="181">
       <c r="A181" s="23" t="inlineStr">
         <is>
-          <t>DHAN-23126092113209</t>
+          <t>DHAN-211260921155609</t>
         </is>
       </c>
       <c r="B181" s="23" t="inlineStr">
         <is>
-          <t>TALBROAUTO</t>
+          <t>JAYKAY</t>
         </is>
       </c>
       <c r="C181" s="23" t="inlineStr">
         <is>
-          <t>SHORT</t>
+          <t>LONG</t>
         </is>
       </c>
       <c r="D181" s="24" t="n">
         <v>46286</v>
       </c>
       <c r="E181" s="25" t="n">
-        <v>478.39</v>
+        <v>188.91</v>
       </c>
       <c r="F181" s="26" t="n">
-        <v>632</v>
-      </c>
-      <c r="G181" s="24" t="n">
-        <v>46286</v>
-      </c>
-      <c r="H181" s="25" t="n">
-        <v>465.51</v>
-      </c>
+        <v>750</v>
+      </c>
+      <c r="G181" s="24" t="inlineStr"/>
+      <c r="H181" s="25" t="inlineStr"/>
       <c r="I181" s="21">
         <f>IF(OR($B181="",$H181=""),"",IF($C181="LONG",($H181-$E181)*$F181,($E181-$H181)*$F181))</f>
         <v/>
       </c>
       <c r="J181" s="4" t="n">
-        <v>0</v>
+        <v>50.15</v>
       </c>
       <c r="K181" s="21">
         <f>IF(OR($B181="",$I181=""),"",$I181-IF($J181="",0,$J181))</f>
@@ -10516,19 +10500,39 @@
       </c>
     </row>
     <row r="182">
-      <c r="A182" s="23" t="n"/>
-      <c r="B182" s="23" t="n"/>
-      <c r="C182" s="23" t="n"/>
-      <c r="D182" s="24" t="n"/>
-      <c r="E182" s="25" t="n"/>
-      <c r="F182" s="26" t="n"/>
-      <c r="G182" s="24" t="n"/>
-      <c r="H182" s="25" t="n"/>
+      <c r="A182" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-241260921702409</t>
+        </is>
+      </c>
+      <c r="B182" s="23" t="inlineStr">
+        <is>
+          <t>KROSS</t>
+        </is>
+      </c>
+      <c r="C182" s="23" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="D182" s="24" t="n">
+        <v>46286</v>
+      </c>
+      <c r="E182" s="25" t="n">
+        <v>257.49</v>
+      </c>
+      <c r="F182" s="26" t="n">
+        <v>233</v>
+      </c>
+      <c r="G182" s="24" t="inlineStr"/>
+      <c r="H182" s="25" t="inlineStr"/>
       <c r="I182" s="21">
         <f>IF(OR($B182="",$H182=""),"",IF($C182="LONG",($H182-$E182)*$F182,($E182-$H182)*$F182))</f>
         <v/>
       </c>
-      <c r="J182" s="4" t="n"/>
+      <c r="J182" s="4" t="n">
+        <v>50.15</v>
+      </c>
       <c r="K182" s="21">
         <f>IF(OR($B182="",$I182=""),"",$I182-IF($J182="",0,$J182))</f>
         <v/>
@@ -10543,19 +10547,43 @@
       </c>
     </row>
     <row r="183">
-      <c r="A183" s="23" t="n"/>
-      <c r="B183" s="23" t="n"/>
-      <c r="C183" s="23" t="n"/>
-      <c r="D183" s="24" t="n"/>
-      <c r="E183" s="25" t="n"/>
-      <c r="F183" s="26" t="n"/>
-      <c r="G183" s="24" t="n"/>
-      <c r="H183" s="25" t="n"/>
+      <c r="A183" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-23126092113309</t>
+        </is>
+      </c>
+      <c r="B183" s="23" t="inlineStr">
+        <is>
+          <t>LUXIND</t>
+        </is>
+      </c>
+      <c r="C183" s="23" t="inlineStr">
+        <is>
+          <t>SHORT</t>
+        </is>
+      </c>
+      <c r="D183" s="24" t="n">
+        <v>46286</v>
+      </c>
+      <c r="E183" s="25" t="n">
+        <v>1142.1</v>
+      </c>
+      <c r="F183" s="26" t="n">
+        <v>263</v>
+      </c>
+      <c r="G183" s="24" t="n">
+        <v>46286</v>
+      </c>
+      <c r="H183" s="25" t="n">
+        <v>1197.67</v>
+      </c>
       <c r="I183" s="21">
         <f>IF(OR($B183="",$H183=""),"",IF($C183="LONG",($H183-$E183)*$F183,($E183-$H183)*$F183))</f>
         <v/>
       </c>
-      <c r="J183" s="4" t="n"/>
+      <c r="J183" s="4" t="n">
+        <v>0</v>
+      </c>
       <c r="K183" s="21">
         <f>IF(OR($B183="",$I183=""),"",$I183-IF($J183="",0,$J183))</f>
         <v/>
@@ -10570,19 +10598,43 @@
       </c>
     </row>
     <row r="184">
-      <c r="A184" s="23" t="n"/>
-      <c r="B184" s="23" t="n"/>
-      <c r="C184" s="23" t="n"/>
-      <c r="D184" s="24" t="n"/>
-      <c r="E184" s="25" t="n"/>
-      <c r="F184" s="26" t="n"/>
-      <c r="G184" s="24" t="n"/>
-      <c r="H184" s="25" t="n"/>
+      <c r="A184" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-22126092158309</t>
+        </is>
+      </c>
+      <c r="B184" s="23" t="inlineStr">
+        <is>
+          <t>NRBBEARING</t>
+        </is>
+      </c>
+      <c r="C184" s="23" t="inlineStr">
+        <is>
+          <t>SHORT</t>
+        </is>
+      </c>
+      <c r="D184" s="24" t="n">
+        <v>46286</v>
+      </c>
+      <c r="E184" s="25" t="n">
+        <v>535.51</v>
+      </c>
+      <c r="F184" s="26" t="n">
+        <v>568</v>
+      </c>
+      <c r="G184" s="24" t="n">
+        <v>46286</v>
+      </c>
+      <c r="H184" s="25" t="n">
+        <v>531.6799999999999</v>
+      </c>
       <c r="I184" s="21">
         <f>IF(OR($B184="",$H184=""),"",IF($C184="LONG",($H184-$E184)*$F184,($E184-$H184)*$F184))</f>
         <v/>
       </c>
-      <c r="J184" s="4" t="n"/>
+      <c r="J184" s="4" t="n">
+        <v>0</v>
+      </c>
       <c r="K184" s="21">
         <f>IF(OR($B184="",$I184=""),"",$I184-IF($J184="",0,$J184))</f>
         <v/>
@@ -10597,19 +10649,39 @@
       </c>
     </row>
     <row r="185">
-      <c r="A185" s="23" t="n"/>
-      <c r="B185" s="23" t="n"/>
-      <c r="C185" s="23" t="n"/>
-      <c r="D185" s="24" t="n"/>
-      <c r="E185" s="25" t="n"/>
-      <c r="F185" s="26" t="n"/>
-      <c r="G185" s="24" t="n"/>
-      <c r="H185" s="25" t="n"/>
+      <c r="A185" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-221260921659609</t>
+        </is>
+      </c>
+      <c r="B185" s="23" t="inlineStr">
+        <is>
+          <t>REFEX</t>
+        </is>
+      </c>
+      <c r="C185" s="23" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="D185" s="24" t="n">
+        <v>46286</v>
+      </c>
+      <c r="E185" s="25" t="n">
+        <v>293.2</v>
+      </c>
+      <c r="F185" s="26" t="n">
+        <v>470</v>
+      </c>
+      <c r="G185" s="24" t="inlineStr"/>
+      <c r="H185" s="25" t="inlineStr"/>
       <c r="I185" s="21">
         <f>IF(OR($B185="",$H185=""),"",IF($C185="LONG",($H185-$E185)*$F185,($E185-$H185)*$F185))</f>
         <v/>
       </c>
-      <c r="J185" s="4" t="n"/>
+      <c r="J185" s="4" t="n">
+        <v>50.15</v>
+      </c>
       <c r="K185" s="21">
         <f>IF(OR($B185="",$I185=""),"",$I185-IF($J185="",0,$J185))</f>
         <v/>
@@ -10624,19 +10696,43 @@
       </c>
     </row>
     <row r="186">
-      <c r="A186" s="23" t="n"/>
-      <c r="B186" s="23" t="n"/>
-      <c r="C186" s="23" t="n"/>
-      <c r="D186" s="24" t="n"/>
-      <c r="E186" s="25" t="n"/>
-      <c r="F186" s="26" t="n"/>
-      <c r="G186" s="24" t="n"/>
-      <c r="H186" s="25" t="n"/>
+      <c r="A186" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-32126092161209</t>
+        </is>
+      </c>
+      <c r="B186" s="23" t="inlineStr">
+        <is>
+          <t>SAMBHV</t>
+        </is>
+      </c>
+      <c r="C186" s="23" t="inlineStr">
+        <is>
+          <t>SHORT</t>
+        </is>
+      </c>
+      <c r="D186" s="24" t="n">
+        <v>46286</v>
+      </c>
+      <c r="E186" s="25" t="n">
+        <v>156.2</v>
+      </c>
+      <c r="F186" s="26" t="n">
+        <v>2021</v>
+      </c>
+      <c r="G186" s="24" t="n">
+        <v>46286</v>
+      </c>
+      <c r="H186" s="25" t="n">
+        <v>153.42</v>
+      </c>
       <c r="I186" s="21">
         <f>IF(OR($B186="",$H186=""),"",IF($C186="LONG",($H186-$E186)*$F186,($E186-$H186)*$F186))</f>
         <v/>
       </c>
-      <c r="J186" s="4" t="n"/>
+      <c r="J186" s="4" t="n">
+        <v>0</v>
+      </c>
       <c r="K186" s="21">
         <f>IF(OR($B186="",$I186=""),"",$I186-IF($J186="",0,$J186))</f>
         <v/>
@@ -10651,19 +10747,43 @@
       </c>
     </row>
     <row r="187">
-      <c r="A187" s="23" t="n"/>
-      <c r="B187" s="23" t="n"/>
-      <c r="C187" s="23" t="n"/>
-      <c r="D187" s="24" t="n"/>
-      <c r="E187" s="25" t="n"/>
-      <c r="F187" s="26" t="n"/>
-      <c r="G187" s="24" t="n"/>
-      <c r="H187" s="25" t="n"/>
+      <c r="A187" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-23126092113209</t>
+        </is>
+      </c>
+      <c r="B187" s="23" t="inlineStr">
+        <is>
+          <t>TALBROAUTO</t>
+        </is>
+      </c>
+      <c r="C187" s="23" t="inlineStr">
+        <is>
+          <t>SHORT</t>
+        </is>
+      </c>
+      <c r="D187" s="24" t="n">
+        <v>46286</v>
+      </c>
+      <c r="E187" s="25" t="n">
+        <v>478.39</v>
+      </c>
+      <c r="F187" s="26" t="n">
+        <v>632</v>
+      </c>
+      <c r="G187" s="24" t="n">
+        <v>46286</v>
+      </c>
+      <c r="H187" s="25" t="n">
+        <v>465.51</v>
+      </c>
       <c r="I187" s="21">
         <f>IF(OR($B187="",$H187=""),"",IF($C187="LONG",($H187-$E187)*$F187,($E187-$H187)*$F187))</f>
         <v/>
       </c>
-      <c r="J187" s="4" t="n"/>
+      <c r="J187" s="4" t="n">
+        <v>0</v>
+      </c>
       <c r="K187" s="21">
         <f>IF(OR($B187="",$I187=""),"",$I187-IF($J187="",0,$J187))</f>
         <v/>
@@ -33140,7 +33260,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J86"/>
+  <dimension ref="A1:J91"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -33310,7 +33430,7 @@
     <row r="6">
       <c r="A6" s="27" t="inlineStr">
         <is>
-          <t>ASHOKA</t>
+          <t>ASHIANA</t>
         </is>
       </c>
       <c r="B6" s="20">
@@ -33353,7 +33473,7 @@
     <row r="7">
       <c r="A7" s="27" t="inlineStr">
         <is>
-          <t>AWFIS</t>
+          <t>ASHOKA</t>
         </is>
       </c>
       <c r="B7" s="20">
@@ -33396,7 +33516,7 @@
     <row r="8">
       <c r="A8" s="27" t="inlineStr">
         <is>
-          <t>BAJAJHIND</t>
+          <t>AWFIS</t>
         </is>
       </c>
       <c r="B8" s="20">
@@ -33439,7 +33559,7 @@
     <row r="9">
       <c r="A9" s="27" t="inlineStr">
         <is>
-          <t>BANARISUG</t>
+          <t>BAJAJHIND</t>
         </is>
       </c>
       <c r="B9" s="20">
@@ -33482,7 +33602,7 @@
     <row r="10">
       <c r="A10" s="27" t="inlineStr">
         <is>
-          <t>BCG</t>
+          <t>BANARISUG</t>
         </is>
       </c>
       <c r="B10" s="20">
@@ -33525,7 +33645,7 @@
     <row r="11">
       <c r="A11" s="27" t="inlineStr">
         <is>
-          <t>BFUTILITIE</t>
+          <t>BCG</t>
         </is>
       </c>
       <c r="B11" s="20">
@@ -33568,7 +33688,7 @@
     <row r="12">
       <c r="A12" s="27" t="inlineStr">
         <is>
-          <t>BOMDYEING</t>
+          <t>BFUTILITIE</t>
         </is>
       </c>
       <c r="B12" s="20">
@@ -33611,7 +33731,7 @@
     <row r="13">
       <c r="A13" s="27" t="inlineStr">
         <is>
-          <t>CHEMPLASTS</t>
+          <t>BOMDYEING</t>
         </is>
       </c>
       <c r="B13" s="20">
@@ -33654,7 +33774,7 @@
     <row r="14">
       <c r="A14" s="27" t="inlineStr">
         <is>
-          <t>EIEL</t>
+          <t>CHEMPLASTS</t>
         </is>
       </c>
       <c r="B14" s="20">
@@ -33697,7 +33817,7 @@
     <row r="15">
       <c r="A15" s="27" t="inlineStr">
         <is>
-          <t>EMUDHRA</t>
+          <t>EIEL</t>
         </is>
       </c>
       <c r="B15" s="20">
@@ -33740,7 +33860,7 @@
     <row r="16">
       <c r="A16" s="27" t="inlineStr">
         <is>
-          <t>FILATEX</t>
+          <t>EMUDHRA</t>
         </is>
       </c>
       <c r="B16" s="20">
@@ -33783,7 +33903,7 @@
     <row r="17">
       <c r="A17" s="27" t="inlineStr">
         <is>
-          <t>FMGOETZE</t>
+          <t>FILATEX</t>
         </is>
       </c>
       <c r="B17" s="20">
@@ -33826,7 +33946,7 @@
     <row r="18">
       <c r="A18" s="27" t="inlineStr">
         <is>
-          <t>FOSECOIND</t>
+          <t>FMGOETZE</t>
         </is>
       </c>
       <c r="B18" s="20">
@@ -33869,7 +33989,7 @@
     <row r="19">
       <c r="A19" s="27" t="inlineStr">
         <is>
-          <t>GKENERGY</t>
+          <t>FOSECOIND</t>
         </is>
       </c>
       <c r="B19" s="20">
@@ -33912,7 +34032,7 @@
     <row r="20">
       <c r="A20" s="27" t="inlineStr">
         <is>
-          <t>GNRL</t>
+          <t>GKENERGY</t>
         </is>
       </c>
       <c r="B20" s="20">
@@ -33955,7 +34075,7 @@
     <row r="21">
       <c r="A21" s="27" t="inlineStr">
         <is>
-          <t>GOCLCORP</t>
+          <t>GNRL</t>
         </is>
       </c>
       <c r="B21" s="20">
@@ -33998,7 +34118,7 @@
     <row r="22">
       <c r="A22" s="27" t="inlineStr">
         <is>
-          <t>GOPAL</t>
+          <t>GOCLCORP</t>
         </is>
       </c>
       <c r="B22" s="20">
@@ -34041,7 +34161,7 @@
     <row r="23">
       <c r="A23" s="27" t="inlineStr">
         <is>
-          <t>GRAUWEIL</t>
+          <t>GOPAL</t>
         </is>
       </c>
       <c r="B23" s="20">
@@ -34084,7 +34204,7 @@
     <row r="24">
       <c r="A24" s="27" t="inlineStr">
         <is>
-          <t>GUJTHEM</t>
+          <t>GRAUWEIL</t>
         </is>
       </c>
       <c r="B24" s="20">
@@ -34127,7 +34247,7 @@
     <row r="25">
       <c r="A25" s="27" t="inlineStr">
         <is>
-          <t>HERITGFOOD</t>
+          <t>GUJTHEM</t>
         </is>
       </c>
       <c r="B25" s="20">
@@ -34170,7 +34290,7 @@
     <row r="26">
       <c r="A26" s="27" t="inlineStr">
         <is>
-          <t>HIKAL</t>
+          <t>HERITGFOOD</t>
         </is>
       </c>
       <c r="B26" s="20">
@@ -34213,7 +34333,7 @@
     <row r="27">
       <c r="A27" s="27" t="inlineStr">
         <is>
-          <t>HINDOILEXP</t>
+          <t>HIKAL</t>
         </is>
       </c>
       <c r="B27" s="20">
@@ -34256,7 +34376,7 @@
     <row r="28">
       <c r="A28" s="27" t="inlineStr">
         <is>
-          <t>HUBTOWN</t>
+          <t>HINDOILEXP</t>
         </is>
       </c>
       <c r="B28" s="20">
@@ -34299,7 +34419,7 @@
     <row r="29">
       <c r="A29" s="27" t="inlineStr">
         <is>
-          <t>INDNIPPON</t>
+          <t>HUBTOWN</t>
         </is>
       </c>
       <c r="B29" s="20">
@@ -34342,7 +34462,7 @@
     <row r="30">
       <c r="A30" s="27" t="inlineStr">
         <is>
-          <t>INDOCO</t>
+          <t>INDNIPPON</t>
         </is>
       </c>
       <c r="B30" s="20">
@@ -34385,7 +34505,7 @@
     <row r="31">
       <c r="A31" s="27" t="inlineStr">
         <is>
-          <t>INDORAMA</t>
+          <t>INDOCO</t>
         </is>
       </c>
       <c r="B31" s="20">
@@ -34428,7 +34548,7 @@
     <row r="32">
       <c r="A32" s="27" t="inlineStr">
         <is>
-          <t>IPL</t>
+          <t>INDORAMA</t>
         </is>
       </c>
       <c r="B32" s="20">
@@ -34471,7 +34591,7 @@
     <row r="33">
       <c r="A33" s="27" t="inlineStr">
         <is>
-          <t>JGCHEM</t>
+          <t>IPL</t>
         </is>
       </c>
       <c r="B33" s="20">
@@ -34514,7 +34634,7 @@
     <row r="34">
       <c r="A34" s="27" t="inlineStr">
         <is>
-          <t>KCP</t>
+          <t>JASH</t>
         </is>
       </c>
       <c r="B34" s="20">
@@ -34557,7 +34677,7 @@
     <row r="35">
       <c r="A35" s="27" t="inlineStr">
         <is>
-          <t>KIRIINDUS</t>
+          <t>JAYKAY</t>
         </is>
       </c>
       <c r="B35" s="20">
@@ -34600,7 +34720,7 @@
     <row r="36">
       <c r="A36" s="27" t="inlineStr">
         <is>
-          <t>KIRLOSIND</t>
+          <t>JGCHEM</t>
         </is>
       </c>
       <c r="B36" s="20">
@@ -34643,7 +34763,7 @@
     <row r="37">
       <c r="A37" s="27" t="inlineStr">
         <is>
-          <t>KLBRENG-B</t>
+          <t>KCP</t>
         </is>
       </c>
       <c r="B37" s="20">
@@ -34686,7 +34806,7 @@
     <row r="38">
       <c r="A38" s="27" t="inlineStr">
         <is>
-          <t>KSL</t>
+          <t>KIRIINDUS</t>
         </is>
       </c>
       <c r="B38" s="20">
@@ -34729,7 +34849,7 @@
     <row r="39">
       <c r="A39" s="27" t="inlineStr">
         <is>
-          <t>LUXIND</t>
+          <t>KIRLOSIND</t>
         </is>
       </c>
       <c r="B39" s="20">
@@ -34772,7 +34892,7 @@
     <row r="40">
       <c r="A40" s="27" t="inlineStr">
         <is>
-          <t>MAITHANALL</t>
+          <t>KLBRENG-B</t>
         </is>
       </c>
       <c r="B40" s="20">
@@ -34815,7 +34935,7 @@
     <row r="41">
       <c r="A41" s="27" t="inlineStr">
         <is>
-          <t>MANGLMCEM</t>
+          <t>KROSS</t>
         </is>
       </c>
       <c r="B41" s="20">
@@ -34858,7 +34978,7 @@
     <row r="42">
       <c r="A42" s="27" t="inlineStr">
         <is>
-          <t>MASTEK</t>
+          <t>KSL</t>
         </is>
       </c>
       <c r="B42" s="20">
@@ -34901,7 +35021,7 @@
     <row r="43">
       <c r="A43" s="27" t="inlineStr">
         <is>
-          <t>MOBIKWIK</t>
+          <t>LUXIND</t>
         </is>
       </c>
       <c r="B43" s="20">
@@ -34944,7 +35064,7 @@
     <row r="44">
       <c r="A44" s="27" t="inlineStr">
         <is>
-          <t>NETWORK18</t>
+          <t>MAITHANALL</t>
         </is>
       </c>
       <c r="B44" s="20">
@@ -34987,7 +35107,7 @@
     <row r="45">
       <c r="A45" s="27" t="inlineStr">
         <is>
-          <t>NILKAMAL</t>
+          <t>MANGLMCEM</t>
         </is>
       </c>
       <c r="B45" s="20">
@@ -35030,7 +35150,7 @@
     <row r="46">
       <c r="A46" s="27" t="inlineStr">
         <is>
-          <t>NORTHARC</t>
+          <t>MASTEK</t>
         </is>
       </c>
       <c r="B46" s="20">
@@ -35073,7 +35193,7 @@
     <row r="47">
       <c r="A47" s="27" t="inlineStr">
         <is>
-          <t>NOVARTIND</t>
+          <t>MOBIKWIK</t>
         </is>
       </c>
       <c r="B47" s="20">
@@ -35116,7 +35236,7 @@
     <row r="48">
       <c r="A48" s="27" t="inlineStr">
         <is>
-          <t>NPST</t>
+          <t>NETWORK18</t>
         </is>
       </c>
       <c r="B48" s="20">
@@ -35159,7 +35279,7 @@
     <row r="49">
       <c r="A49" s="27" t="inlineStr">
         <is>
-          <t>NRBBEARING</t>
+          <t>NILKAMAL</t>
         </is>
       </c>
       <c r="B49" s="20">
@@ -35202,7 +35322,7 @@
     <row r="50">
       <c r="A50" s="27" t="inlineStr">
         <is>
-          <t>OMAXE</t>
+          <t>NORTHARC</t>
         </is>
       </c>
       <c r="B50" s="20">
@@ -35245,7 +35365,7 @@
     <row r="51">
       <c r="A51" s="27" t="inlineStr">
         <is>
-          <t>OPTIEMUS</t>
+          <t>NOVARTIND</t>
         </is>
       </c>
       <c r="B51" s="20">
@@ -35288,7 +35408,7 @@
     <row r="52">
       <c r="A52" s="27" t="inlineStr">
         <is>
-          <t>ORIENTHOT</t>
+          <t>NPST</t>
         </is>
       </c>
       <c r="B52" s="20">
@@ -35331,7 +35451,7 @@
     <row r="53">
       <c r="A53" s="27" t="inlineStr">
         <is>
-          <t>PITTIENG</t>
+          <t>NRBBEARING</t>
         </is>
       </c>
       <c r="B53" s="20">
@@ -35374,7 +35494,7 @@
     <row r="54">
       <c r="A54" s="27" t="inlineStr">
         <is>
-          <t>QUADFUTURE</t>
+          <t>OMAXE</t>
         </is>
       </c>
       <c r="B54" s="20">
@@ -35417,7 +35537,7 @@
     <row r="55">
       <c r="A55" s="27" t="inlineStr">
         <is>
-          <t>RACLGEAR</t>
+          <t>OPTIEMUS</t>
         </is>
       </c>
       <c r="B55" s="20">
@@ -35460,7 +35580,7 @@
     <row r="56">
       <c r="A56" s="27" t="inlineStr">
         <is>
-          <t>RAMRAT</t>
+          <t>ORIENTHOT</t>
         </is>
       </c>
       <c r="B56" s="20">
@@ -35503,7 +35623,7 @@
     <row r="57">
       <c r="A57" s="27" t="inlineStr">
         <is>
-          <t>RAYMOND</t>
+          <t>PITTIENG</t>
         </is>
       </c>
       <c r="B57" s="20">
@@ -35546,7 +35666,7 @@
     <row r="58">
       <c r="A58" s="27" t="inlineStr">
         <is>
-          <t>RESPONIND</t>
+          <t>QUADFUTURE</t>
         </is>
       </c>
       <c r="B58" s="20">
@@ -35589,7 +35709,7 @@
     <row r="59">
       <c r="A59" s="27" t="inlineStr">
         <is>
-          <t>RML</t>
+          <t>RACLGEAR</t>
         </is>
       </c>
       <c r="B59" s="20">
@@ -35632,7 +35752,7 @@
     <row r="60">
       <c r="A60" s="27" t="inlineStr">
         <is>
-          <t>ROSSTECH</t>
+          <t>RAMRAT</t>
         </is>
       </c>
       <c r="B60" s="20">
@@ -35675,7 +35795,7 @@
     <row r="61">
       <c r="A61" s="27" t="inlineStr">
         <is>
-          <t>SAATVIKGL</t>
+          <t>RAYMOND</t>
         </is>
       </c>
       <c r="B61" s="20">
@@ -35718,7 +35838,7 @@
     <row r="62">
       <c r="A62" s="27" t="inlineStr">
         <is>
-          <t>SAKAR</t>
+          <t>REFEX</t>
         </is>
       </c>
       <c r="B62" s="20">
@@ -35761,7 +35881,7 @@
     <row r="63">
       <c r="A63" s="27" t="inlineStr">
         <is>
-          <t>SAMBHV</t>
+          <t>RESPONIND</t>
         </is>
       </c>
       <c r="B63" s="20">
@@ -35804,7 +35924,7 @@
     <row r="64">
       <c r="A64" s="27" t="inlineStr">
         <is>
-          <t>SAMHI</t>
+          <t>RML</t>
         </is>
       </c>
       <c r="B64" s="20">
@@ -35847,7 +35967,7 @@
     <row r="65">
       <c r="A65" s="27" t="inlineStr">
         <is>
-          <t>SHAREINDIA</t>
+          <t>ROSSTECH</t>
         </is>
       </c>
       <c r="B65" s="20">
@@ -35890,7 +36010,7 @@
     <row r="66">
       <c r="A66" s="27" t="inlineStr">
         <is>
-          <t>SIKA</t>
+          <t>SAATVIKGL</t>
         </is>
       </c>
       <c r="B66" s="20">
@@ -35933,7 +36053,7 @@
     <row r="67">
       <c r="A67" s="27" t="inlineStr">
         <is>
-          <t>SINDHUTRAD</t>
+          <t>SAKAR</t>
         </is>
       </c>
       <c r="B67" s="20">
@@ -35976,7 +36096,7 @@
     <row r="68">
       <c r="A68" s="27" t="inlineStr">
         <is>
-          <t>SMSPHARMA</t>
+          <t>SAMBHV</t>
         </is>
       </c>
       <c r="B68" s="20">
@@ -36019,7 +36139,7 @@
     <row r="69">
       <c r="A69" s="27" t="inlineStr">
         <is>
-          <t>SOLARA</t>
+          <t>SAMHI</t>
         </is>
       </c>
       <c r="B69" s="20">
@@ -36062,7 +36182,7 @@
     <row r="70">
       <c r="A70" s="27" t="inlineStr">
         <is>
-          <t>SOTL</t>
+          <t>SHAREINDIA</t>
         </is>
       </c>
       <c r="B70" s="20">
@@ -36105,7 +36225,7 @@
     <row r="71">
       <c r="A71" s="27" t="inlineStr">
         <is>
-          <t>SSWL</t>
+          <t>SIKA</t>
         </is>
       </c>
       <c r="B71" s="20">
@@ -36148,7 +36268,7 @@
     <row r="72">
       <c r="A72" s="27" t="inlineStr">
         <is>
-          <t>SYMPHONY</t>
+          <t>SINDHUTRAD</t>
         </is>
       </c>
       <c r="B72" s="20">
@@ -36191,7 +36311,7 @@
     <row r="73">
       <c r="A73" s="27" t="inlineStr">
         <is>
-          <t>SYNCOMF</t>
+          <t>SMSPHARMA</t>
         </is>
       </c>
       <c r="B73" s="20">
@@ -36234,7 +36354,7 @@
     <row r="74">
       <c r="A74" s="27" t="inlineStr">
         <is>
-          <t>TALBROAUTO</t>
+          <t>SOLARA</t>
         </is>
       </c>
       <c r="B74" s="20">
@@ -36277,7 +36397,7 @@
     <row r="75">
       <c r="A75" s="27" t="inlineStr">
         <is>
-          <t>TBZ</t>
+          <t>SOTL</t>
         </is>
       </c>
       <c r="B75" s="20">
@@ -36320,7 +36440,7 @@
     <row r="76">
       <c r="A76" s="27" t="inlineStr">
         <is>
-          <t>THOMASCOOK</t>
+          <t>SSWL</t>
         </is>
       </c>
       <c r="B76" s="20">
@@ -36363,7 +36483,7 @@
     <row r="77">
       <c r="A77" s="27" t="inlineStr">
         <is>
-          <t>VENKEYS</t>
+          <t>SYMPHONY</t>
         </is>
       </c>
       <c r="B77" s="20">
@@ -36406,7 +36526,7 @@
     <row r="78">
       <c r="A78" s="27" t="inlineStr">
         <is>
-          <t>VENUSPIPES</t>
+          <t>SYNCOMF</t>
         </is>
       </c>
       <c r="B78" s="20">
@@ -36449,7 +36569,7 @@
     <row r="79">
       <c r="A79" s="27" t="inlineStr">
         <is>
-          <t>VERANDA</t>
+          <t>TALBROAUTO</t>
         </is>
       </c>
       <c r="B79" s="20">
@@ -36492,7 +36612,7 @@
     <row r="80">
       <c r="A80" s="27" t="inlineStr">
         <is>
-          <t>VSSL</t>
+          <t>TBZ</t>
         </is>
       </c>
       <c r="B80" s="20">
@@ -36535,7 +36655,7 @@
     <row r="81">
       <c r="A81" s="27" t="inlineStr">
         <is>
-          <t>WELSPLSOL</t>
+          <t>THOMASCOOK</t>
         </is>
       </c>
       <c r="B81" s="20">
@@ -36578,7 +36698,7 @@
     <row r="82">
       <c r="A82" s="27" t="inlineStr">
         <is>
-          <t>WENDT</t>
+          <t>VENKEYS</t>
         </is>
       </c>
       <c r="B82" s="20">
@@ -36621,7 +36741,7 @@
     <row r="83">
       <c r="A83" s="27" t="inlineStr">
         <is>
-          <t>WINDLAS</t>
+          <t>VENUSPIPES</t>
         </is>
       </c>
       <c r="B83" s="20">
@@ -36664,7 +36784,7 @@
     <row r="84">
       <c r="A84" s="27" t="inlineStr">
         <is>
-          <t>XPROINDIA</t>
+          <t>VERANDA</t>
         </is>
       </c>
       <c r="B84" s="20">
@@ -36707,7 +36827,7 @@
     <row r="85">
       <c r="A85" s="27" t="inlineStr">
         <is>
-          <t>ZAGGLE</t>
+          <t>VSSL</t>
         </is>
       </c>
       <c r="B85" s="20">
@@ -36748,37 +36868,252 @@
       </c>
     </row>
     <row r="86">
-      <c r="A86" s="3" t="inlineStr">
+      <c r="A86" s="27" t="inlineStr">
+        <is>
+          <t>WELSPLSOL</t>
+        </is>
+      </c>
+      <c r="B86" s="20">
+        <f>COUNTIF('Trade Log'!$B$4:$B$503,$A86)</f>
+        <v/>
+      </c>
+      <c r="C86" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A86,'Trade Log'!$K$4:$K$503,"&gt;0")</f>
+        <v/>
+      </c>
+      <c r="D86" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A86,'Trade Log'!$K$4:$K$503,"&lt;0")</f>
+        <v/>
+      </c>
+      <c r="E86" s="29">
+        <f>IFERROR($C86/$B86,"")</f>
+        <v/>
+      </c>
+      <c r="F86" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A86,'Trade Log'!$I$4:$I$503)</f>
+        <v/>
+      </c>
+      <c r="G86" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A86,'Trade Log'!$K$4:$K$503)</f>
+        <v/>
+      </c>
+      <c r="H86" s="21">
+        <f>IFERROR($G86/$B86,"")</f>
+        <v/>
+      </c>
+      <c r="I86" s="21">
+        <f>IFERROR(_xlfn.MAXIFS('Trade Log'!$K$4:$K$503,'Trade Log'!$B$4:$B$503,$A86),"")</f>
+        <v/>
+      </c>
+      <c r="J86" s="21">
+        <f>IFERROR(_xlfn.MINIFS('Trade Log'!$K$4:$K$503,'Trade Log'!$B$4:$B$503,$A86),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="27" t="inlineStr">
+        <is>
+          <t>WENDT</t>
+        </is>
+      </c>
+      <c r="B87" s="20">
+        <f>COUNTIF('Trade Log'!$B$4:$B$503,$A87)</f>
+        <v/>
+      </c>
+      <c r="C87" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A87,'Trade Log'!$K$4:$K$503,"&gt;0")</f>
+        <v/>
+      </c>
+      <c r="D87" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A87,'Trade Log'!$K$4:$K$503,"&lt;0")</f>
+        <v/>
+      </c>
+      <c r="E87" s="29">
+        <f>IFERROR($C87/$B87,"")</f>
+        <v/>
+      </c>
+      <c r="F87" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A87,'Trade Log'!$I$4:$I$503)</f>
+        <v/>
+      </c>
+      <c r="G87" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A87,'Trade Log'!$K$4:$K$503)</f>
+        <v/>
+      </c>
+      <c r="H87" s="21">
+        <f>IFERROR($G87/$B87,"")</f>
+        <v/>
+      </c>
+      <c r="I87" s="21">
+        <f>IFERROR(_xlfn.MAXIFS('Trade Log'!$K$4:$K$503,'Trade Log'!$B$4:$B$503,$A87),"")</f>
+        <v/>
+      </c>
+      <c r="J87" s="21">
+        <f>IFERROR(_xlfn.MINIFS('Trade Log'!$K$4:$K$503,'Trade Log'!$B$4:$B$503,$A87),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="27" t="inlineStr">
+        <is>
+          <t>WINDLAS</t>
+        </is>
+      </c>
+      <c r="B88" s="20">
+        <f>COUNTIF('Trade Log'!$B$4:$B$503,$A88)</f>
+        <v/>
+      </c>
+      <c r="C88" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A88,'Trade Log'!$K$4:$K$503,"&gt;0")</f>
+        <v/>
+      </c>
+      <c r="D88" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A88,'Trade Log'!$K$4:$K$503,"&lt;0")</f>
+        <v/>
+      </c>
+      <c r="E88" s="29">
+        <f>IFERROR($C88/$B88,"")</f>
+        <v/>
+      </c>
+      <c r="F88" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A88,'Trade Log'!$I$4:$I$503)</f>
+        <v/>
+      </c>
+      <c r="G88" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A88,'Trade Log'!$K$4:$K$503)</f>
+        <v/>
+      </c>
+      <c r="H88" s="21">
+        <f>IFERROR($G88/$B88,"")</f>
+        <v/>
+      </c>
+      <c r="I88" s="21">
+        <f>IFERROR(_xlfn.MAXIFS('Trade Log'!$K$4:$K$503,'Trade Log'!$B$4:$B$503,$A88),"")</f>
+        <v/>
+      </c>
+      <c r="J88" s="21">
+        <f>IFERROR(_xlfn.MINIFS('Trade Log'!$K$4:$K$503,'Trade Log'!$B$4:$B$503,$A88),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="27" t="inlineStr">
+        <is>
+          <t>XPROINDIA</t>
+        </is>
+      </c>
+      <c r="B89" s="20">
+        <f>COUNTIF('Trade Log'!$B$4:$B$503,$A89)</f>
+        <v/>
+      </c>
+      <c r="C89" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A89,'Trade Log'!$K$4:$K$503,"&gt;0")</f>
+        <v/>
+      </c>
+      <c r="D89" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A89,'Trade Log'!$K$4:$K$503,"&lt;0")</f>
+        <v/>
+      </c>
+      <c r="E89" s="29">
+        <f>IFERROR($C89/$B89,"")</f>
+        <v/>
+      </c>
+      <c r="F89" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A89,'Trade Log'!$I$4:$I$503)</f>
+        <v/>
+      </c>
+      <c r="G89" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A89,'Trade Log'!$K$4:$K$503)</f>
+        <v/>
+      </c>
+      <c r="H89" s="21">
+        <f>IFERROR($G89/$B89,"")</f>
+        <v/>
+      </c>
+      <c r="I89" s="21">
+        <f>IFERROR(_xlfn.MAXIFS('Trade Log'!$K$4:$K$503,'Trade Log'!$B$4:$B$503,$A89),"")</f>
+        <v/>
+      </c>
+      <c r="J89" s="21">
+        <f>IFERROR(_xlfn.MINIFS('Trade Log'!$K$4:$K$503,'Trade Log'!$B$4:$B$503,$A89),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="27" t="inlineStr">
+        <is>
+          <t>ZAGGLE</t>
+        </is>
+      </c>
+      <c r="B90" s="20">
+        <f>COUNTIF('Trade Log'!$B$4:$B$503,$A90)</f>
+        <v/>
+      </c>
+      <c r="C90" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A90,'Trade Log'!$K$4:$K$503,"&gt;0")</f>
+        <v/>
+      </c>
+      <c r="D90" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A90,'Trade Log'!$K$4:$K$503,"&lt;0")</f>
+        <v/>
+      </c>
+      <c r="E90" s="29">
+        <f>IFERROR($C90/$B90,"")</f>
+        <v/>
+      </c>
+      <c r="F90" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A90,'Trade Log'!$I$4:$I$503)</f>
+        <v/>
+      </c>
+      <c r="G90" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A90,'Trade Log'!$K$4:$K$503)</f>
+        <v/>
+      </c>
+      <c r="H90" s="21">
+        <f>IFERROR($G90/$B90,"")</f>
+        <v/>
+      </c>
+      <c r="I90" s="21">
+        <f>IFERROR(_xlfn.MAXIFS('Trade Log'!$K$4:$K$503,'Trade Log'!$B$4:$B$503,$A90),"")</f>
+        <v/>
+      </c>
+      <c r="J90" s="21">
+        <f>IFERROR(_xlfn.MINIFS('Trade Log'!$K$4:$K$503,'Trade Log'!$B$4:$B$503,$A90),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="3" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="B86" s="30">
-        <f>SUM(B4:B85)</f>
-        <v/>
-      </c>
-      <c r="C86" s="30">
-        <f>SUM(C4:C85)</f>
-        <v/>
-      </c>
-      <c r="D86" s="30">
-        <f>SUM(D4:D85)</f>
-        <v/>
-      </c>
-      <c r="E86" s="31">
-        <f>IFERROR(C86/B86,"")</f>
-        <v/>
-      </c>
-      <c r="F86" s="32">
-        <f>SUM(F4:F85)</f>
-        <v/>
-      </c>
-      <c r="G86" s="32">
-        <f>SUM(G4:G85)</f>
-        <v/>
-      </c>
-      <c r="H86" s="32">
-        <f>IFERROR(G86/B86,"")</f>
+      <c r="B91" s="30">
+        <f>SUM(B4:B90)</f>
+        <v/>
+      </c>
+      <c r="C91" s="30">
+        <f>SUM(C4:C90)</f>
+        <v/>
+      </c>
+      <c r="D91" s="30">
+        <f>SUM(D4:D90)</f>
+        <v/>
+      </c>
+      <c r="E91" s="31">
+        <f>IFERROR(C91/B91,"")</f>
+        <v/>
+      </c>
+      <c r="F91" s="32">
+        <f>SUM(F4:F90)</f>
+        <v/>
+      </c>
+      <c r="G91" s="32">
+        <f>SUM(G4:G90)</f>
+        <v/>
+      </c>
+      <c r="H91" s="32">
+        <f>IFERROR(G91/B91,"")</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Data update — 2026-09-22 candle + results refresh
</commit_message>
<xml_diff>
--- a/results/strategy_pnl_simple.xlsx
+++ b/results/strategy_pnl_simple.xlsx
@@ -1473,7 +1473,7 @@
         <v/>
       </c>
       <c r="J4" s="4" t="n">
-        <v>571.78</v>
+        <v>464.09</v>
       </c>
       <c r="K4" s="21">
         <f>IF(OR($B4="",$I4=""),"",$I4-IF($J4="",0,$J4))</f>
@@ -1524,7 +1524,7 @@
         <v/>
       </c>
       <c r="J5" s="4" t="n">
-        <v>688.87</v>
+        <v>538.4</v>
       </c>
       <c r="K5" s="21">
         <f>IF(OR($B5="",$I5=""),"",$I5-IF($J5="",0,$J5))</f>
@@ -1575,7 +1575,7 @@
         <v/>
       </c>
       <c r="J6" s="4" t="n">
-        <v>570.63</v>
+        <v>514.1900000000001</v>
       </c>
       <c r="K6" s="21">
         <f>IF(OR($B6="",$I6=""),"",$I6-IF($J6="",0,$J6))</f>
@@ -1626,7 +1626,7 @@
         <v/>
       </c>
       <c r="J7" s="4" t="n">
-        <v>663.03</v>
+        <v>595.38</v>
       </c>
       <c r="K7" s="21">
         <f>IF(OR($B7="",$I7=""),"",$I7-IF($J7="",0,$J7))</f>
@@ -1677,7 +1677,7 @@
         <v/>
       </c>
       <c r="J8" s="4" t="n">
-        <v>591.04</v>
+        <v>525.1900000000001</v>
       </c>
       <c r="K8" s="21">
         <f>IF(OR($B8="",$I8=""),"",$I8-IF($J8="",0,$J8))</f>
@@ -1779,7 +1779,7 @@
         <v/>
       </c>
       <c r="J10" s="4" t="n">
-        <v>398.61</v>
+        <v>367.34</v>
       </c>
       <c r="K10" s="21">
         <f>IF(OR($B10="",$I10=""),"",$I10-IF($J10="",0,$J10))</f>
@@ -1881,7 +1881,7 @@
         <v/>
       </c>
       <c r="J12" s="4" t="n">
-        <v>414.15</v>
+        <v>376.36</v>
       </c>
       <c r="K12" s="21">
         <f>IF(OR($B12="",$I12=""),"",$I12-IF($J12="",0,$J12))</f>
@@ -1932,7 +1932,7 @@
         <v/>
       </c>
       <c r="J13" s="4" t="n">
-        <v>345.07</v>
+        <v>322.36</v>
       </c>
       <c r="K13" s="21">
         <f>IF(OR($B13="",$I13=""),"",$I13-IF($J13="",0,$J13))</f>
@@ -1983,7 +1983,7 @@
         <v/>
       </c>
       <c r="J14" s="4" t="n">
-        <v>414.48</v>
+        <v>376.81</v>
       </c>
       <c r="K14" s="21">
         <f>IF(OR($B14="",$I14=""),"",$I14-IF($J14="",0,$J14))</f>
@@ -2034,7 +2034,7 @@
         <v/>
       </c>
       <c r="J15" s="4" t="n">
-        <v>380.41</v>
+        <v>339.07</v>
       </c>
       <c r="K15" s="21">
         <f>IF(OR($B15="",$I15=""),"",$I15-IF($J15="",0,$J15))</f>
@@ -2187,7 +2187,7 @@
         <v/>
       </c>
       <c r="J18" s="4" t="n">
-        <v>413.91</v>
+        <v>376.04</v>
       </c>
       <c r="K18" s="21">
         <f>IF(OR($B18="",$I18=""),"",$I18-IF($J18="",0,$J18))</f>
@@ -2238,7 +2238,7 @@
         <v/>
       </c>
       <c r="J19" s="4" t="n">
-        <v>406.45</v>
+        <v>374.18</v>
       </c>
       <c r="K19" s="21">
         <f>IF(OR($B19="",$I19=""),"",$I19-IF($J19="",0,$J19))</f>
@@ -2697,7 +2697,7 @@
         <v/>
       </c>
       <c r="J28" s="4" t="n">
-        <v>870.41</v>
+        <v>801.17</v>
       </c>
       <c r="K28" s="21">
         <f>IF(OR($B28="",$I28=""),"",$I28-IF($J28="",0,$J28))</f>
@@ -2850,7 +2850,7 @@
         <v/>
       </c>
       <c r="J31" s="4" t="n">
-        <v>391.16</v>
+        <v>377.89</v>
       </c>
       <c r="K31" s="21">
         <f>IF(OR($B31="",$I31=""),"",$I31-IF($J31="",0,$J31))</f>
@@ -2901,7 +2901,7 @@
         <v/>
       </c>
       <c r="J32" s="4" t="n">
-        <v>349.77</v>
+        <v>336.52</v>
       </c>
       <c r="K32" s="21">
         <f>IF(OR($B32="",$I32=""),"",$I32-IF($J32="",0,$J32))</f>
@@ -3003,7 +3003,7 @@
         <v/>
       </c>
       <c r="J34" s="4" t="n">
-        <v>349.8</v>
+        <v>336.28</v>
       </c>
       <c r="K34" s="21">
         <f>IF(OR($B34="",$I34=""),"",$I34-IF($J34="",0,$J34))</f>
@@ -3054,7 +3054,7 @@
         <v/>
       </c>
       <c r="J35" s="4" t="n">
-        <v>386.15</v>
+        <v>373.48</v>
       </c>
       <c r="K35" s="21">
         <f>IF(OR($B35="",$I35=""),"",$I35-IF($J35="",0,$J35))</f>
@@ -3411,7 +3411,7 @@
         <v/>
       </c>
       <c r="J42" s="4" t="n">
-        <v>978.27</v>
+        <v>950.51</v>
       </c>
       <c r="K42" s="21">
         <f>IF(OR($B42="",$I42=""),"",$I42-IF($J42="",0,$J42))</f>
@@ -3462,7 +3462,7 @@
         <v/>
       </c>
       <c r="J43" s="4" t="n">
-        <v>957.67</v>
+        <v>934.51</v>
       </c>
       <c r="K43" s="21">
         <f>IF(OR($B43="",$I43=""),"",$I43-IF($J43="",0,$J43))</f>
@@ -3513,7 +3513,7 @@
         <v/>
       </c>
       <c r="J44" s="4" t="n">
-        <v>992.26</v>
+        <v>964.38</v>
       </c>
       <c r="K44" s="21">
         <f>IF(OR($B44="",$I44=""),"",$I44-IF($J44="",0,$J44))</f>
@@ -3564,7 +3564,7 @@
         <v/>
       </c>
       <c r="J45" s="4" t="n">
-        <v>599.6799999999999</v>
+        <v>612.7</v>
       </c>
       <c r="K45" s="21">
         <f>IF(OR($B45="",$I45=""),"",$I45-IF($J45="",0,$J45))</f>
@@ -3615,7 +3615,7 @@
         <v/>
       </c>
       <c r="J46" s="4" t="n">
-        <v>600.79</v>
+        <v>613.84</v>
       </c>
       <c r="K46" s="21">
         <f>IF(OR($B46="",$I46=""),"",$I46-IF($J46="",0,$J46))</f>
@@ -3666,7 +3666,7 @@
         <v/>
       </c>
       <c r="J47" s="4" t="n">
-        <v>678.95</v>
+        <v>693.27</v>
       </c>
       <c r="K47" s="21">
         <f>IF(OR($B47="",$I47=""),"",$I47-IF($J47="",0,$J47))</f>
@@ -3717,7 +3717,7 @@
         <v/>
       </c>
       <c r="J48" s="4" t="n">
-        <v>672.4299999999999</v>
+        <v>685.47</v>
       </c>
       <c r="K48" s="21">
         <f>IF(OR($B48="",$I48=""),"",$I48-IF($J48="",0,$J48))</f>
@@ -3768,7 +3768,7 @@
         <v/>
       </c>
       <c r="J49" s="4" t="n">
-        <v>538.67</v>
+        <v>546.53</v>
       </c>
       <c r="K49" s="21">
         <f>IF(OR($B49="",$I49=""),"",$I49-IF($J49="",0,$J49))</f>
@@ -3819,7 +3819,7 @@
         <v/>
       </c>
       <c r="J50" s="4" t="n">
-        <v>627.9400000000001</v>
+        <v>609.98</v>
       </c>
       <c r="K50" s="21">
         <f>IF(OR($B50="",$I50=""),"",$I50-IF($J50="",0,$J50))</f>
@@ -4023,7 +4023,7 @@
         <v/>
       </c>
       <c r="J54" s="4" t="n">
-        <v>619.09</v>
+        <v>601.39</v>
       </c>
       <c r="K54" s="21">
         <f>IF(OR($B54="",$I54=""),"",$I54-IF($J54="",0,$J54))</f>
@@ -4176,7 +4176,7 @@
         <v/>
       </c>
       <c r="J57" s="4" t="n">
-        <v>612.28</v>
+        <v>596.23</v>
       </c>
       <c r="K57" s="21">
         <f>IF(OR($B57="",$I57=""),"",$I57-IF($J57="",0,$J57))</f>
@@ -4380,7 +4380,7 @@
         <v/>
       </c>
       <c r="J61" s="4" t="n">
-        <v>692.14</v>
+        <v>687.71</v>
       </c>
       <c r="K61" s="21">
         <f>IF(OR($B61="",$I61=""),"",$I61-IF($J61="",0,$J61))</f>
@@ -4431,7 +4431,7 @@
         <v/>
       </c>
       <c r="J62" s="4" t="n">
-        <v>615.15</v>
+        <v>610.26</v>
       </c>
       <c r="K62" s="21">
         <f>IF(OR($B62="",$I62=""),"",$I62-IF($J62="",0,$J62))</f>
@@ -4533,7 +4533,7 @@
         <v/>
       </c>
       <c r="J64" s="4" t="n">
-        <v>440.43</v>
+        <v>437.62</v>
       </c>
       <c r="K64" s="21">
         <f>IF(OR($B64="",$I64=""),"",$I64-IF($J64="",0,$J64))</f>
@@ -4584,7 +4584,7 @@
         <v/>
       </c>
       <c r="J65" s="4" t="n">
-        <v>386.62</v>
+        <v>384.09</v>
       </c>
       <c r="K65" s="21">
         <f>IF(OR($B65="",$I65=""),"",$I65-IF($J65="",0,$J65))</f>
@@ -4839,7 +4839,7 @@
         <v/>
       </c>
       <c r="J70" s="4" t="n">
-        <v>385.22</v>
+        <v>382.7</v>
       </c>
       <c r="K70" s="21">
         <f>IF(OR($B70="",$I70=""),"",$I70-IF($J70="",0,$J70))</f>
@@ -4890,7 +4890,7 @@
         <v/>
       </c>
       <c r="J71" s="4" t="n">
-        <v>434.29</v>
+        <v>431.78</v>
       </c>
       <c r="K71" s="21">
         <f>IF(OR($B71="",$I71=""),"",$I71-IF($J71="",0,$J71))</f>
@@ -4941,7 +4941,7 @@
         <v/>
       </c>
       <c r="J72" s="4" t="n">
-        <v>411.21</v>
+        <v>393.8</v>
       </c>
       <c r="K72" s="21">
         <f>IF(OR($B72="",$I72=""),"",$I72-IF($J72="",0,$J72))</f>
@@ -5043,7 +5043,7 @@
         <v/>
       </c>
       <c r="J74" s="4" t="n">
-        <v>355.78</v>
+        <v>341.34</v>
       </c>
       <c r="K74" s="21">
         <f>IF(OR($B74="",$I74=""),"",$I74-IF($J74="",0,$J74))</f>
@@ -5094,7 +5094,7 @@
         <v/>
       </c>
       <c r="J75" s="4" t="n">
-        <v>364.3</v>
+        <v>346.98</v>
       </c>
       <c r="K75" s="21">
         <f>IF(OR($B75="",$I75=""),"",$I75-IF($J75="",0,$J75))</f>
@@ -5196,7 +5196,7 @@
         <v/>
       </c>
       <c r="J77" s="4" t="n">
-        <v>411.49</v>
+        <v>393.05</v>
       </c>
       <c r="K77" s="21">
         <f>IF(OR($B77="",$I77=""),"",$I77-IF($J77="",0,$J77))</f>
@@ -5298,7 +5298,7 @@
         <v/>
       </c>
       <c r="J79" s="4" t="n">
-        <v>343.88</v>
+        <v>333.47</v>
       </c>
       <c r="K79" s="21">
         <f>IF(OR($B79="",$I79=""),"",$I79-IF($J79="",0,$J79))</f>
@@ -5349,7 +5349,7 @@
         <v/>
       </c>
       <c r="J80" s="4" t="n">
-        <v>345.32</v>
+        <v>334.83</v>
       </c>
       <c r="K80" s="21">
         <f>IF(OR($B80="",$I80=""),"",$I80-IF($J80="",0,$J80))</f>
@@ -5859,7 +5859,7 @@
         <v/>
       </c>
       <c r="J90" s="4" t="n">
-        <v>891.87</v>
+        <v>833.8200000000001</v>
       </c>
       <c r="K90" s="21">
         <f>IF(OR($B90="",$I90=""),"",$I90-IF($J90="",0,$J90))</f>
@@ -5961,7 +5961,7 @@
         <v/>
       </c>
       <c r="J92" s="4" t="n">
-        <v>797.89</v>
+        <v>739.8200000000001</v>
       </c>
       <c r="K92" s="21">
         <f>IF(OR($B92="",$I92=""),"",$I92-IF($J92="",0,$J92))</f>
@@ -6012,7 +6012,7 @@
         <v/>
       </c>
       <c r="J93" s="4" t="n">
-        <v>825.22</v>
+        <v>766.78</v>
       </c>
       <c r="K93" s="21">
         <f>IF(OR($B93="",$I93=""),"",$I93-IF($J93="",0,$J93))</f>
@@ -6063,7 +6063,7 @@
         <v/>
       </c>
       <c r="J94" s="4" t="n">
-        <v>479.87</v>
+        <v>433.61</v>
       </c>
       <c r="K94" s="21">
         <f>IF(OR($B94="",$I94=""),"",$I94-IF($J94="",0,$J94))</f>
@@ -6165,7 +6165,7 @@
         <v/>
       </c>
       <c r="J96" s="4" t="n">
-        <v>474.05</v>
+        <v>430.76</v>
       </c>
       <c r="K96" s="21">
         <f>IF(OR($B96="",$I96=""),"",$I96-IF($J96="",0,$J96))</f>
@@ -6267,7 +6267,7 @@
         <v/>
       </c>
       <c r="J98" s="4" t="n">
-        <v>530.83</v>
+        <v>487.6</v>
       </c>
       <c r="K98" s="21">
         <f>IF(OR($B98="",$I98=""),"",$I98-IF($J98="",0,$J98))</f>
@@ -6471,7 +6471,7 @@
         <v/>
       </c>
       <c r="J102" s="4" t="n">
-        <v>531.04</v>
+        <v>487.69</v>
       </c>
       <c r="K102" s="21">
         <f>IF(OR($B102="",$I102=""),"",$I102-IF($J102="",0,$J102))</f>
@@ -6879,7 +6879,7 @@
         <v/>
       </c>
       <c r="J110" s="4" t="n">
-        <v>480.28</v>
+        <v>437.6</v>
       </c>
       <c r="K110" s="21">
         <f>IF(OR($B110="",$I110=""),"",$I110-IF($J110="",0,$J110))</f>
@@ -6981,7 +6981,7 @@
         <v/>
       </c>
       <c r="J112" s="4" t="n">
-        <v>419.68</v>
+        <v>382.63</v>
       </c>
       <c r="K112" s="21">
         <f>IF(OR($B112="",$I112=""),"",$I112-IF($J112="",0,$J112))</f>
@@ -7185,7 +7185,7 @@
         <v/>
       </c>
       <c r="J116" s="4" t="n">
-        <v>428.22</v>
+        <v>394.21</v>
       </c>
       <c r="K116" s="21">
         <f>IF(OR($B116="",$I116=""),"",$I116-IF($J116="",0,$J116))</f>
@@ -7236,7 +7236,7 @@
         <v/>
       </c>
       <c r="J117" s="4" t="n">
-        <v>545.7</v>
+        <v>494.15</v>
       </c>
       <c r="K117" s="21">
         <f>IF(OR($B117="",$I117=""),"",$I117-IF($J117="",0,$J117))</f>
@@ -7389,7 +7389,7 @@
         <v/>
       </c>
       <c r="J120" s="4" t="n">
-        <v>424.46</v>
+        <v>391.31</v>
       </c>
       <c r="K120" s="21">
         <f>IF(OR($B120="",$I120=""),"",$I120-IF($J120="",0,$J120))</f>
@@ -7440,7 +7440,7 @@
         <v/>
       </c>
       <c r="J121" s="4" t="n">
-        <v>371.24</v>
+        <v>343.5</v>
       </c>
       <c r="K121" s="21">
         <f>IF(OR($B121="",$I121=""),"",$I121-IF($J121="",0,$J121))</f>
@@ -7746,7 +7746,7 @@
         <v/>
       </c>
       <c r="J127" s="4" t="n">
-        <v>641.84</v>
+        <v>587.9400000000001</v>
       </c>
       <c r="K127" s="21">
         <f>IF(OR($B127="",$I127=""),"",$I127-IF($J127="",0,$J127))</f>
@@ -7848,7 +7848,7 @@
         <v/>
       </c>
       <c r="J129" s="4" t="n">
-        <v>637.6799999999999</v>
+        <v>583.85</v>
       </c>
       <c r="K129" s="21">
         <f>IF(OR($B129="",$I129=""),"",$I129-IF($J129="",0,$J129))</f>
@@ -7950,7 +7950,7 @@
         <v/>
       </c>
       <c r="J131" s="4" t="n">
-        <v>653.29</v>
+        <v>592.6900000000001</v>
       </c>
       <c r="K131" s="21">
         <f>IF(OR($B131="",$I131=""),"",$I131-IF($J131="",0,$J131))</f>
@@ -8052,7 +8052,7 @@
         <v/>
       </c>
       <c r="J133" s="4" t="n">
-        <v>563.51</v>
+        <v>509.91</v>
       </c>
       <c r="K133" s="21">
         <f>IF(OR($B133="",$I133=""),"",$I133-IF($J133="",0,$J133))</f>
@@ -8103,7 +8103,7 @@
         <v/>
       </c>
       <c r="J134" s="4" t="n">
-        <v>631.48</v>
+        <v>578.39</v>
       </c>
       <c r="K134" s="21">
         <f>IF(OR($B134="",$I134=""),"",$I134-IF($J134="",0,$J134))</f>
@@ -8154,7 +8154,7 @@
         <v/>
       </c>
       <c r="J135" s="4" t="n">
-        <v>496.84</v>
+        <v>468.38</v>
       </c>
       <c r="K135" s="21">
         <f>IF(OR($B135="",$I135=""),"",$I135-IF($J135="",0,$J135))</f>
@@ -8307,7 +8307,7 @@
         <v/>
       </c>
       <c r="J138" s="4" t="n">
-        <v>493.59</v>
+        <v>465.39</v>
       </c>
       <c r="K138" s="21">
         <f>IF(OR($B138="",$I138=""),"",$I138-IF($J138="",0,$J138))</f>
@@ -8409,7 +8409,7 @@
         <v/>
       </c>
       <c r="J140" s="4" t="n">
-        <v>502.8</v>
+        <v>473.31</v>
       </c>
       <c r="K140" s="21">
         <f>IF(OR($B140="",$I140=""),"",$I140-IF($J140="",0,$J140))</f>
@@ -8460,7 +8460,7 @@
         <v/>
       </c>
       <c r="J141" s="4" t="n">
-        <v>490.63</v>
+        <v>463.42</v>
       </c>
       <c r="K141" s="21">
         <f>IF(OR($B141="",$I141=""),"",$I141-IF($J141="",0,$J141))</f>
@@ -8511,7 +8511,7 @@
         <v/>
       </c>
       <c r="J142" s="4" t="n">
-        <v>466.42</v>
+        <v>442.78</v>
       </c>
       <c r="K142" s="21">
         <f>IF(OR($B142="",$I142=""),"",$I142-IF($J142="",0,$J142))</f>
@@ -8664,7 +8664,7 @@
         <v/>
       </c>
       <c r="J145" s="4" t="n">
-        <v>541.16</v>
+        <v>511.54</v>
       </c>
       <c r="K145" s="21">
         <f>IF(OR($B145="",$I145=""),"",$I145-IF($J145="",0,$J145))</f>
@@ -9480,7 +9480,7 @@
         <v/>
       </c>
       <c r="J161" s="4" t="n">
-        <v>461.82</v>
+        <v>461.7</v>
       </c>
       <c r="K161" s="21">
         <f>IF(OR($B161="",$I161=""),"",$I161-IF($J161="",0,$J161))</f>
@@ -9939,7 +9939,7 @@
         <v/>
       </c>
       <c r="J170" s="4" t="n">
-        <v>192.79</v>
+        <v>258.56</v>
       </c>
       <c r="K170" s="21">
         <f>IF(OR($B170="",$I170=""),"",$I170-IF($J170="",0,$J170))</f>
@@ -9990,7 +9990,7 @@
         <v/>
       </c>
       <c r="J171" s="4" t="n">
-        <v>627.5599999999999</v>
+        <v>662.13</v>
       </c>
       <c r="K171" s="21">
         <f>IF(OR($B171="",$I171=""),"",$I171-IF($J171="",0,$J171))</f>
@@ -10041,7 +10041,7 @@
         <v/>
       </c>
       <c r="J172" s="4" t="n">
-        <v>612.35</v>
+        <v>647.29</v>
       </c>
       <c r="K172" s="21">
         <f>IF(OR($B172="",$I172=""),"",$I172-IF($J172="",0,$J172))</f>
@@ -10092,7 +10092,7 @@
         <v/>
       </c>
       <c r="J173" s="4" t="n">
-        <v>629.67</v>
+        <v>665.03</v>
       </c>
       <c r="K173" s="21">
         <f>IF(OR($B173="",$I173=""),"",$I173-IF($J173="",0,$J173))</f>
@@ -10194,7 +10194,7 @@
         <v/>
       </c>
       <c r="J175" s="4" t="n">
-        <v>614.6</v>
+        <v>649.5</v>
       </c>
       <c r="K175" s="21">
         <f>IF(OR($B175="",$I175=""),"",$I175-IF($J175="",0,$J175))</f>
@@ -10285,14 +10285,18 @@
       <c r="F177" s="26" t="n">
         <v>340</v>
       </c>
-      <c r="G177" s="24" t="inlineStr"/>
-      <c r="H177" s="25" t="inlineStr"/>
+      <c r="G177" s="24" t="n">
+        <v>46287</v>
+      </c>
+      <c r="H177" s="25" t="n">
+        <v>392.12</v>
+      </c>
       <c r="I177" s="21">
         <f>IF(OR($B177="",$H177=""),"",IF($C177="LONG",($H177-$E177)*$F177,($E177-$H177)*$F177))</f>
         <v/>
       </c>
       <c r="J177" s="4" t="n">
-        <v>50.15</v>
+        <v>266.27</v>
       </c>
       <c r="K177" s="21">
         <f>IF(OR($B177="",$I177=""),"",$I177-IF($J177="",0,$J177))</f>
@@ -10343,7 +10347,7 @@
         <v/>
       </c>
       <c r="J178" s="4" t="n">
-        <v>0</v>
+        <v>185.64</v>
       </c>
       <c r="K178" s="21">
         <f>IF(OR($B178="",$I178=""),"",$I178-IF($J178="",0,$J178))</f>
@@ -10383,14 +10387,18 @@
       <c r="F179" s="26" t="n">
         <v>1300</v>
       </c>
-      <c r="G179" s="24" t="inlineStr"/>
-      <c r="H179" s="25" t="inlineStr"/>
+      <c r="G179" s="24" t="n">
+        <v>46287</v>
+      </c>
+      <c r="H179" s="25" t="n">
+        <v>107.2</v>
+      </c>
       <c r="I179" s="21">
         <f>IF(OR($B179="",$H179=""),"",IF($C179="LONG",($H179-$E179)*$F179,($E179-$H179)*$F179))</f>
         <v/>
       </c>
       <c r="J179" s="4" t="n">
-        <v>50.15</v>
+        <v>236.87</v>
       </c>
       <c r="K179" s="21">
         <f>IF(OR($B179="",$I179=""),"",$I179-IF($J179="",0,$J179))</f>
@@ -10430,14 +10438,18 @@
       <c r="F180" s="26" t="n">
         <v>244</v>
       </c>
-      <c r="G180" s="24" t="inlineStr"/>
-      <c r="H180" s="25" t="inlineStr"/>
+      <c r="G180" s="24" t="n">
+        <v>46287</v>
+      </c>
+      <c r="H180" s="25" t="n">
+        <v>593.59</v>
+      </c>
       <c r="I180" s="21">
         <f>IF(OR($B180="",$H180=""),"",IF($C180="LONG",($H180-$E180)*$F180,($E180-$H180)*$F180))</f>
         <v/>
       </c>
       <c r="J180" s="4" t="n">
-        <v>50.15</v>
+        <v>271.55</v>
       </c>
       <c r="K180" s="21">
         <f>IF(OR($B180="",$I180=""),"",$I180-IF($J180="",0,$J180))</f>
@@ -10477,14 +10489,18 @@
       <c r="F181" s="26" t="n">
         <v>750</v>
       </c>
-      <c r="G181" s="24" t="inlineStr"/>
-      <c r="H181" s="25" t="inlineStr"/>
+      <c r="G181" s="24" t="n">
+        <v>46287</v>
+      </c>
+      <c r="H181" s="25" t="n">
+        <v>191.21</v>
+      </c>
       <c r="I181" s="21">
         <f>IF(OR($B181="",$H181=""),"",IF($C181="LONG",($H181-$E181)*$F181,($E181-$H181)*$F181))</f>
         <v/>
       </c>
       <c r="J181" s="4" t="n">
-        <v>50.15</v>
+        <v>269.7</v>
       </c>
       <c r="K181" s="21">
         <f>IF(OR($B181="",$I181=""),"",$I181-IF($J181="",0,$J181))</f>
@@ -10524,14 +10540,18 @@
       <c r="F182" s="26" t="n">
         <v>233</v>
       </c>
-      <c r="G182" s="24" t="inlineStr"/>
-      <c r="H182" s="25" t="inlineStr"/>
+      <c r="G182" s="24" t="n">
+        <v>46287</v>
+      </c>
+      <c r="H182" s="25" t="n">
+        <v>260.01</v>
+      </c>
       <c r="I182" s="21">
         <f>IF(OR($B182="",$H182=""),"",IF($C182="LONG",($H182-$E182)*$F182,($E182-$H182)*$F182))</f>
         <v/>
       </c>
       <c r="J182" s="4" t="n">
-        <v>50.15</v>
+        <v>152.88</v>
       </c>
       <c r="K182" s="21">
         <f>IF(OR($B182="",$I182=""),"",$I182-IF($J182="",0,$J182))</f>
@@ -10582,7 +10602,7 @@
         <v/>
       </c>
       <c r="J183" s="4" t="n">
-        <v>0</v>
+        <v>436.71</v>
       </c>
       <c r="K183" s="21">
         <f>IF(OR($B183="",$I183=""),"",$I183-IF($J183="",0,$J183))</f>
@@ -10633,7 +10653,7 @@
         <v/>
       </c>
       <c r="J184" s="4" t="n">
-        <v>0</v>
+        <v>434.19</v>
       </c>
       <c r="K184" s="21">
         <f>IF(OR($B184="",$I184=""),"",$I184-IF($J184="",0,$J184))</f>
@@ -10673,14 +10693,18 @@
       <c r="F185" s="26" t="n">
         <v>470</v>
       </c>
-      <c r="G185" s="24" t="inlineStr"/>
-      <c r="H185" s="25" t="inlineStr"/>
+      <c r="G185" s="24" t="n">
+        <v>46287</v>
+      </c>
+      <c r="H185" s="25" t="n">
+        <v>292.43</v>
+      </c>
       <c r="I185" s="21">
         <f>IF(OR($B185="",$H185=""),"",IF($C185="LONG",($H185-$E185)*$F185,($E185-$H185)*$F185))</f>
         <v/>
       </c>
       <c r="J185" s="4" t="n">
-        <v>50.15</v>
+        <v>266.46</v>
       </c>
       <c r="K185" s="21">
         <f>IF(OR($B185="",$I185=""),"",$I185-IF($J185="",0,$J185))</f>
@@ -10731,7 +10755,7 @@
         <v/>
       </c>
       <c r="J186" s="4" t="n">
-        <v>0</v>
+        <v>447.15</v>
       </c>
       <c r="K186" s="21">
         <f>IF(OR($B186="",$I186=""),"",$I186-IF($J186="",0,$J186))</f>
@@ -10782,7 +10806,7 @@
         <v/>
       </c>
       <c r="J187" s="4" t="n">
-        <v>0</v>
+        <v>429.11</v>
       </c>
       <c r="K187" s="21">
         <f>IF(OR($B187="",$I187=""),"",$I187-IF($J187="",0,$J187))</f>
@@ -10798,19 +10822,43 @@
       </c>
     </row>
     <row r="188">
-      <c r="A188" s="23" t="n"/>
-      <c r="B188" s="23" t="n"/>
-      <c r="C188" s="23" t="n"/>
-      <c r="D188" s="24" t="n"/>
-      <c r="E188" s="25" t="n"/>
-      <c r="F188" s="26" t="n"/>
-      <c r="G188" s="24" t="n"/>
-      <c r="H188" s="25" t="n"/>
+      <c r="A188" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-34126092243009</t>
+        </is>
+      </c>
+      <c r="B188" s="23" t="inlineStr">
+        <is>
+          <t>ASHIANA</t>
+        </is>
+      </c>
+      <c r="C188" s="23" t="inlineStr">
+        <is>
+          <t>SHORT</t>
+        </is>
+      </c>
+      <c r="D188" s="24" t="n">
+        <v>46287</v>
+      </c>
+      <c r="E188" s="25" t="n">
+        <v>391.52</v>
+      </c>
+      <c r="F188" s="26" t="n">
+        <v>340</v>
+      </c>
+      <c r="G188" s="24" t="n">
+        <v>46287</v>
+      </c>
+      <c r="H188" s="25" t="n">
+        <v>386.54</v>
+      </c>
       <c r="I188" s="21">
         <f>IF(OR($B188="",$H188=""),"",IF($C188="LONG",($H188-$E188)*$F188,($E188-$H188)*$F188))</f>
         <v/>
       </c>
-      <c r="J188" s="4" t="n"/>
+      <c r="J188" s="4" t="n">
+        <v>0</v>
+      </c>
       <c r="K188" s="21">
         <f>IF(OR($B188="",$I188=""),"",$I188-IF($J188="",0,$J188))</f>
         <v/>
@@ -10825,19 +10873,39 @@
       </c>
     </row>
     <row r="189">
-      <c r="A189" s="23" t="n"/>
-      <c r="B189" s="23" t="n"/>
-      <c r="C189" s="23" t="n"/>
-      <c r="D189" s="24" t="n"/>
-      <c r="E189" s="25" t="n"/>
-      <c r="F189" s="26" t="n"/>
-      <c r="G189" s="24" t="n"/>
-      <c r="H189" s="25" t="n"/>
+      <c r="A189" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-limit_entry_multi</t>
+        </is>
+      </c>
+      <c r="B189" s="23" t="inlineStr">
+        <is>
+          <t>ASTEC</t>
+        </is>
+      </c>
+      <c r="C189" s="23" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="D189" s="24" t="n">
+        <v>46287</v>
+      </c>
+      <c r="E189" s="25" t="n">
+        <v>794.5626999999999</v>
+      </c>
+      <c r="F189" s="26" t="n">
+        <v>315</v>
+      </c>
+      <c r="G189" s="24" t="inlineStr"/>
+      <c r="H189" s="25" t="inlineStr"/>
       <c r="I189" s="21">
         <f>IF(OR($B189="",$H189=""),"",IF($C189="LONG",($H189-$E189)*$F189,($E189-$H189)*$F189))</f>
         <v/>
       </c>
-      <c r="J189" s="4" t="n"/>
+      <c r="J189" s="4" t="n">
+        <v>50.15</v>
+      </c>
       <c r="K189" s="21">
         <f>IF(OR($B189="",$I189=""),"",$I189-IF($J189="",0,$J189))</f>
         <v/>
@@ -10852,19 +10920,39 @@
       </c>
     </row>
     <row r="190">
-      <c r="A190" s="23" t="n"/>
-      <c r="B190" s="23" t="n"/>
-      <c r="C190" s="23" t="n"/>
-      <c r="D190" s="24" t="n"/>
-      <c r="E190" s="25" t="n"/>
-      <c r="F190" s="26" t="n"/>
-      <c r="G190" s="24" t="n"/>
-      <c r="H190" s="25" t="n"/>
+      <c r="A190" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-23126092274109</t>
+        </is>
+      </c>
+      <c r="B190" s="23" t="inlineStr">
+        <is>
+          <t>CHEMPLASTS</t>
+        </is>
+      </c>
+      <c r="C190" s="23" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="D190" s="24" t="n">
+        <v>46287</v>
+      </c>
+      <c r="E190" s="25" t="n">
+        <v>200.3954</v>
+      </c>
+      <c r="F190" s="26" t="n">
+        <v>1255</v>
+      </c>
+      <c r="G190" s="24" t="inlineStr"/>
+      <c r="H190" s="25" t="inlineStr"/>
       <c r="I190" s="21">
         <f>IF(OR($B190="",$H190=""),"",IF($C190="LONG",($H190-$E190)*$F190,($E190-$H190)*$F190))</f>
         <v/>
       </c>
-      <c r="J190" s="4" t="n"/>
+      <c r="J190" s="4" t="n">
+        <v>50.15</v>
+      </c>
       <c r="K190" s="21">
         <f>IF(OR($B190="",$I190=""),"",$I190-IF($J190="",0,$J190))</f>
         <v/>
@@ -10879,19 +10967,43 @@
       </c>
     </row>
     <row r="191">
-      <c r="A191" s="23" t="n"/>
-      <c r="B191" s="23" t="n"/>
-      <c r="C191" s="23" t="n"/>
-      <c r="D191" s="24" t="n"/>
-      <c r="E191" s="25" t="n"/>
-      <c r="F191" s="26" t="n"/>
-      <c r="G191" s="24" t="n"/>
-      <c r="H191" s="25" t="n"/>
+      <c r="A191" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-23126092251309</t>
+        </is>
+      </c>
+      <c r="B191" s="23" t="inlineStr">
+        <is>
+          <t>INDORAMA</t>
+        </is>
+      </c>
+      <c r="C191" s="23" t="inlineStr">
+        <is>
+          <t>SHORT</t>
+        </is>
+      </c>
+      <c r="D191" s="24" t="n">
+        <v>46287</v>
+      </c>
+      <c r="E191" s="25" t="n">
+        <v>107.16</v>
+      </c>
+      <c r="F191" s="26" t="n">
+        <v>1300</v>
+      </c>
+      <c r="G191" s="24" t="n">
+        <v>46287</v>
+      </c>
+      <c r="H191" s="25" t="n">
+        <v>105.33</v>
+      </c>
       <c r="I191" s="21">
         <f>IF(OR($B191="",$H191=""),"",IF($C191="LONG",($H191-$E191)*$F191,($E191-$H191)*$F191))</f>
         <v/>
       </c>
-      <c r="J191" s="4" t="n"/>
+      <c r="J191" s="4" t="n">
+        <v>0</v>
+      </c>
       <c r="K191" s="21">
         <f>IF(OR($B191="",$I191=""),"",$I191-IF($J191="",0,$J191))</f>
         <v/>
@@ -10906,19 +11018,43 @@
       </c>
     </row>
     <row r="192">
-      <c r="A192" s="23" t="n"/>
-      <c r="B192" s="23" t="n"/>
-      <c r="C192" s="23" t="n"/>
-      <c r="D192" s="24" t="n"/>
-      <c r="E192" s="25" t="n"/>
-      <c r="F192" s="26" t="n"/>
-      <c r="G192" s="24" t="n"/>
-      <c r="H192" s="25" t="n"/>
+      <c r="A192" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-34126092213209</t>
+        </is>
+      </c>
+      <c r="B192" s="23" t="inlineStr">
+        <is>
+          <t>JASH</t>
+        </is>
+      </c>
+      <c r="C192" s="23" t="inlineStr">
+        <is>
+          <t>SHORT</t>
+        </is>
+      </c>
+      <c r="D192" s="24" t="n">
+        <v>46287</v>
+      </c>
+      <c r="E192" s="25" t="n">
+        <v>595.99</v>
+      </c>
+      <c r="F192" s="26" t="n">
+        <v>244</v>
+      </c>
+      <c r="G192" s="24" t="n">
+        <v>46287</v>
+      </c>
+      <c r="H192" s="25" t="n">
+        <v>584.99</v>
+      </c>
       <c r="I192" s="21">
         <f>IF(OR($B192="",$H192=""),"",IF($C192="LONG",($H192-$E192)*$F192,($E192-$H192)*$F192))</f>
         <v/>
       </c>
-      <c r="J192" s="4" t="n"/>
+      <c r="J192" s="4" t="n">
+        <v>0</v>
+      </c>
       <c r="K192" s="21">
         <f>IF(OR($B192="",$I192=""),"",$I192-IF($J192="",0,$J192))</f>
         <v/>
@@ -10933,19 +11069,43 @@
       </c>
     </row>
     <row r="193">
-      <c r="A193" s="23" t="n"/>
-      <c r="B193" s="23" t="n"/>
-      <c r="C193" s="23" t="n"/>
-      <c r="D193" s="24" t="n"/>
-      <c r="E193" s="25" t="n"/>
-      <c r="F193" s="26" t="n"/>
-      <c r="G193" s="24" t="n"/>
-      <c r="H193" s="25" t="n"/>
+      <c r="A193" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-32126092252109</t>
+        </is>
+      </c>
+      <c r="B193" s="23" t="inlineStr">
+        <is>
+          <t>JAYKAY</t>
+        </is>
+      </c>
+      <c r="C193" s="23" t="inlineStr">
+        <is>
+          <t>SHORT</t>
+        </is>
+      </c>
+      <c r="D193" s="24" t="n">
+        <v>46287</v>
+      </c>
+      <c r="E193" s="25" t="n">
+        <v>190.59</v>
+      </c>
+      <c r="F193" s="26" t="n">
+        <v>750</v>
+      </c>
+      <c r="G193" s="24" t="n">
+        <v>46287</v>
+      </c>
+      <c r="H193" s="25" t="n">
+        <v>188.34</v>
+      </c>
       <c r="I193" s="21">
         <f>IF(OR($B193="",$H193=""),"",IF($C193="LONG",($H193-$E193)*$F193,($E193-$H193)*$F193))</f>
         <v/>
       </c>
-      <c r="J193" s="4" t="n"/>
+      <c r="J193" s="4" t="n">
+        <v>0</v>
+      </c>
       <c r="K193" s="21">
         <f>IF(OR($B193="",$I193=""),"",$I193-IF($J193="",0,$J193))</f>
         <v/>
@@ -10960,19 +11120,43 @@
       </c>
     </row>
     <row r="194">
-      <c r="A194" s="23" t="n"/>
-      <c r="B194" s="23" t="n"/>
-      <c r="C194" s="23" t="n"/>
-      <c r="D194" s="24" t="n"/>
-      <c r="E194" s="25" t="n"/>
-      <c r="F194" s="26" t="n"/>
-      <c r="G194" s="24" t="n"/>
-      <c r="H194" s="25" t="n"/>
+      <c r="A194" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-22126092254109</t>
+        </is>
+      </c>
+      <c r="B194" s="23" t="inlineStr">
+        <is>
+          <t>KROSS</t>
+        </is>
+      </c>
+      <c r="C194" s="23" t="inlineStr">
+        <is>
+          <t>SHORT</t>
+        </is>
+      </c>
+      <c r="D194" s="24" t="n">
+        <v>46287</v>
+      </c>
+      <c r="E194" s="25" t="n">
+        <v>259</v>
+      </c>
+      <c r="F194" s="26" t="n">
+        <v>233</v>
+      </c>
+      <c r="G194" s="24" t="n">
+        <v>46287</v>
+      </c>
+      <c r="H194" s="25" t="n">
+        <v>256.71</v>
+      </c>
       <c r="I194" s="21">
         <f>IF(OR($B194="",$H194=""),"",IF($C194="LONG",($H194-$E194)*$F194,($E194-$H194)*$F194))</f>
         <v/>
       </c>
-      <c r="J194" s="4" t="n"/>
+      <c r="J194" s="4" t="n">
+        <v>0</v>
+      </c>
       <c r="K194" s="21">
         <f>IF(OR($B194="",$I194=""),"",$I194-IF($J194="",0,$J194))</f>
         <v/>
@@ -10987,19 +11171,39 @@
       </c>
     </row>
     <row r="195">
-      <c r="A195" s="23" t="n"/>
-      <c r="B195" s="23" t="n"/>
-      <c r="C195" s="23" t="n"/>
-      <c r="D195" s="24" t="n"/>
-      <c r="E195" s="25" t="n"/>
-      <c r="F195" s="26" t="n"/>
-      <c r="G195" s="24" t="n"/>
-      <c r="H195" s="25" t="n"/>
+      <c r="A195" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-221260922659909</t>
+        </is>
+      </c>
+      <c r="B195" s="23" t="inlineStr">
+        <is>
+          <t>PACEDIGITK</t>
+        </is>
+      </c>
+      <c r="C195" s="23" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="D195" s="24" t="n">
+        <v>46287</v>
+      </c>
+      <c r="E195" s="25" t="n">
+        <v>168.7</v>
+      </c>
+      <c r="F195" s="26" t="n">
+        <v>1482</v>
+      </c>
+      <c r="G195" s="24" t="inlineStr"/>
+      <c r="H195" s="25" t="inlineStr"/>
       <c r="I195" s="21">
         <f>IF(OR($B195="",$H195=""),"",IF($C195="LONG",($H195-$E195)*$F195,($E195-$H195)*$F195))</f>
         <v/>
       </c>
-      <c r="J195" s="4" t="n"/>
+      <c r="J195" s="4" t="n">
+        <v>50.15</v>
+      </c>
       <c r="K195" s="21">
         <f>IF(OR($B195="",$I195=""),"",$I195-IF($J195="",0,$J195))</f>
         <v/>
@@ -11014,19 +11218,39 @@
       </c>
     </row>
     <row r="196">
-      <c r="A196" s="23" t="n"/>
-      <c r="B196" s="23" t="n"/>
-      <c r="C196" s="23" t="n"/>
-      <c r="D196" s="24" t="n"/>
-      <c r="E196" s="25" t="n"/>
-      <c r="F196" s="26" t="n"/>
-      <c r="G196" s="24" t="n"/>
-      <c r="H196" s="25" t="n"/>
+      <c r="A196" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-23126092274009</t>
+        </is>
+      </c>
+      <c r="B196" s="23" t="inlineStr">
+        <is>
+          <t>PROTEAN</t>
+        </is>
+      </c>
+      <c r="C196" s="23" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="D196" s="24" t="n">
+        <v>46287</v>
+      </c>
+      <c r="E196" s="25" t="n">
+        <v>620.9959</v>
+      </c>
+      <c r="F196" s="26" t="n">
+        <v>403</v>
+      </c>
+      <c r="G196" s="24" t="inlineStr"/>
+      <c r="H196" s="25" t="inlineStr"/>
       <c r="I196" s="21">
         <f>IF(OR($B196="",$H196=""),"",IF($C196="LONG",($H196-$E196)*$F196,($E196-$H196)*$F196))</f>
         <v/>
       </c>
-      <c r="J196" s="4" t="n"/>
+      <c r="J196" s="4" t="n">
+        <v>50.15</v>
+      </c>
       <c r="K196" s="21">
         <f>IF(OR($B196="",$I196=""),"",$I196-IF($J196="",0,$J196))</f>
         <v/>
@@ -11041,19 +11265,43 @@
       </c>
     </row>
     <row r="197">
-      <c r="A197" s="23" t="n"/>
-      <c r="B197" s="23" t="n"/>
-      <c r="C197" s="23" t="n"/>
-      <c r="D197" s="24" t="n"/>
-      <c r="E197" s="25" t="n"/>
-      <c r="F197" s="26" t="n"/>
-      <c r="G197" s="24" t="n"/>
-      <c r="H197" s="25" t="n"/>
+      <c r="A197" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-23126092251409</t>
+        </is>
+      </c>
+      <c r="B197" s="23" t="inlineStr">
+        <is>
+          <t>REFEX</t>
+        </is>
+      </c>
+      <c r="C197" s="23" t="inlineStr">
+        <is>
+          <t>SHORT</t>
+        </is>
+      </c>
+      <c r="D197" s="24" t="n">
+        <v>46287</v>
+      </c>
+      <c r="E197" s="25" t="n">
+        <v>292.4</v>
+      </c>
+      <c r="F197" s="26" t="n">
+        <v>470</v>
+      </c>
+      <c r="G197" s="24" t="n">
+        <v>46287</v>
+      </c>
+      <c r="H197" s="25" t="n">
+        <v>292</v>
+      </c>
       <c r="I197" s="21">
         <f>IF(OR($B197="",$H197=""),"",IF($C197="LONG",($H197-$E197)*$F197,($E197-$H197)*$F197))</f>
         <v/>
       </c>
-      <c r="J197" s="4" t="n"/>
+      <c r="J197" s="4" t="n">
+        <v>0</v>
+      </c>
       <c r="K197" s="21">
         <f>IF(OR($B197="",$I197=""),"",$I197-IF($J197="",0,$J197))</f>
         <v/>
@@ -11068,19 +11316,39 @@
       </c>
     </row>
     <row r="198">
-      <c r="A198" s="23" t="n"/>
-      <c r="B198" s="23" t="n"/>
-      <c r="C198" s="23" t="n"/>
-      <c r="D198" s="24" t="n"/>
-      <c r="E198" s="25" t="n"/>
-      <c r="F198" s="26" t="n"/>
-      <c r="G198" s="24" t="n"/>
-      <c r="H198" s="25" t="n"/>
+      <c r="A198" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-321260922627909</t>
+        </is>
+      </c>
+      <c r="B198" s="23" t="inlineStr">
+        <is>
+          <t>STEELCAS</t>
+        </is>
+      </c>
+      <c r="C198" s="23" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="D198" s="24" t="n">
+        <v>46287</v>
+      </c>
+      <c r="E198" s="25" t="n">
+        <v>349.9038</v>
+      </c>
+      <c r="F198" s="26" t="n">
+        <v>715</v>
+      </c>
+      <c r="G198" s="24" t="inlineStr"/>
+      <c r="H198" s="25" t="inlineStr"/>
       <c r="I198" s="21">
         <f>IF(OR($B198="",$H198=""),"",IF($C198="LONG",($H198-$E198)*$F198,($E198-$H198)*$F198))</f>
         <v/>
       </c>
-      <c r="J198" s="4" t="n"/>
+      <c r="J198" s="4" t="n">
+        <v>50.15</v>
+      </c>
       <c r="K198" s="21">
         <f>IF(OR($B198="",$I198=""),"",$I198-IF($J198="",0,$J198))</f>
         <v/>
@@ -11095,19 +11363,39 @@
       </c>
     </row>
     <row r="199">
-      <c r="A199" s="23" t="n"/>
-      <c r="B199" s="23" t="n"/>
-      <c r="C199" s="23" t="n"/>
-      <c r="D199" s="24" t="n"/>
-      <c r="E199" s="25" t="n"/>
-      <c r="F199" s="26" t="n"/>
-      <c r="G199" s="24" t="n"/>
-      <c r="H199" s="25" t="n"/>
+      <c r="A199" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-34126092267009</t>
+        </is>
+      </c>
+      <c r="B199" s="23" t="inlineStr">
+        <is>
+          <t>ZOTA</t>
+        </is>
+      </c>
+      <c r="C199" s="23" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="D199" s="24" t="n">
+        <v>46287</v>
+      </c>
+      <c r="E199" s="25" t="n">
+        <v>1359.8431</v>
+      </c>
+      <c r="F199" s="26" t="n">
+        <v>183</v>
+      </c>
+      <c r="G199" s="24" t="inlineStr"/>
+      <c r="H199" s="25" t="inlineStr"/>
       <c r="I199" s="21">
         <f>IF(OR($B199="",$H199=""),"",IF($C199="LONG",($H199-$E199)*$F199,($E199-$H199)*$F199))</f>
         <v/>
       </c>
-      <c r="J199" s="4" t="n"/>
+      <c r="J199" s="4" t="n">
+        <v>50.15</v>
+      </c>
       <c r="K199" s="21">
         <f>IF(OR($B199="",$I199=""),"",$I199-IF($J199="",0,$J199))</f>
         <v/>
@@ -33260,7 +33548,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J91"/>
+  <dimension ref="A1:J96"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -33516,7 +33804,7 @@
     <row r="8">
       <c r="A8" s="27" t="inlineStr">
         <is>
-          <t>AWFIS</t>
+          <t>ASTEC</t>
         </is>
       </c>
       <c r="B8" s="20">
@@ -33559,7 +33847,7 @@
     <row r="9">
       <c r="A9" s="27" t="inlineStr">
         <is>
-          <t>BAJAJHIND</t>
+          <t>AWFIS</t>
         </is>
       </c>
       <c r="B9" s="20">
@@ -33602,7 +33890,7 @@
     <row r="10">
       <c r="A10" s="27" t="inlineStr">
         <is>
-          <t>BANARISUG</t>
+          <t>BAJAJHIND</t>
         </is>
       </c>
       <c r="B10" s="20">
@@ -33645,7 +33933,7 @@
     <row r="11">
       <c r="A11" s="27" t="inlineStr">
         <is>
-          <t>BCG</t>
+          <t>BANARISUG</t>
         </is>
       </c>
       <c r="B11" s="20">
@@ -33688,7 +33976,7 @@
     <row r="12">
       <c r="A12" s="27" t="inlineStr">
         <is>
-          <t>BFUTILITIE</t>
+          <t>BCG</t>
         </is>
       </c>
       <c r="B12" s="20">
@@ -33731,7 +34019,7 @@
     <row r="13">
       <c r="A13" s="27" t="inlineStr">
         <is>
-          <t>BOMDYEING</t>
+          <t>BFUTILITIE</t>
         </is>
       </c>
       <c r="B13" s="20">
@@ -33774,7 +34062,7 @@
     <row r="14">
       <c r="A14" s="27" t="inlineStr">
         <is>
-          <t>CHEMPLASTS</t>
+          <t>BOMDYEING</t>
         </is>
       </c>
       <c r="B14" s="20">
@@ -33817,7 +34105,7 @@
     <row r="15">
       <c r="A15" s="27" t="inlineStr">
         <is>
-          <t>EIEL</t>
+          <t>CHEMPLASTS</t>
         </is>
       </c>
       <c r="B15" s="20">
@@ -33860,7 +34148,7 @@
     <row r="16">
       <c r="A16" s="27" t="inlineStr">
         <is>
-          <t>EMUDHRA</t>
+          <t>EIEL</t>
         </is>
       </c>
       <c r="B16" s="20">
@@ -33903,7 +34191,7 @@
     <row r="17">
       <c r="A17" s="27" t="inlineStr">
         <is>
-          <t>FILATEX</t>
+          <t>EMUDHRA</t>
         </is>
       </c>
       <c r="B17" s="20">
@@ -33946,7 +34234,7 @@
     <row r="18">
       <c r="A18" s="27" t="inlineStr">
         <is>
-          <t>FMGOETZE</t>
+          <t>FILATEX</t>
         </is>
       </c>
       <c r="B18" s="20">
@@ -33989,7 +34277,7 @@
     <row r="19">
       <c r="A19" s="27" t="inlineStr">
         <is>
-          <t>FOSECOIND</t>
+          <t>FMGOETZE</t>
         </is>
       </c>
       <c r="B19" s="20">
@@ -34032,7 +34320,7 @@
     <row r="20">
       <c r="A20" s="27" t="inlineStr">
         <is>
-          <t>GKENERGY</t>
+          <t>FOSECOIND</t>
         </is>
       </c>
       <c r="B20" s="20">
@@ -34075,7 +34363,7 @@
     <row r="21">
       <c r="A21" s="27" t="inlineStr">
         <is>
-          <t>GNRL</t>
+          <t>GKENERGY</t>
         </is>
       </c>
       <c r="B21" s="20">
@@ -34118,7 +34406,7 @@
     <row r="22">
       <c r="A22" s="27" t="inlineStr">
         <is>
-          <t>GOCLCORP</t>
+          <t>GNRL</t>
         </is>
       </c>
       <c r="B22" s="20">
@@ -34161,7 +34449,7 @@
     <row r="23">
       <c r="A23" s="27" t="inlineStr">
         <is>
-          <t>GOPAL</t>
+          <t>GOCLCORP</t>
         </is>
       </c>
       <c r="B23" s="20">
@@ -34204,7 +34492,7 @@
     <row r="24">
       <c r="A24" s="27" t="inlineStr">
         <is>
-          <t>GRAUWEIL</t>
+          <t>GOPAL</t>
         </is>
       </c>
       <c r="B24" s="20">
@@ -34247,7 +34535,7 @@
     <row r="25">
       <c r="A25" s="27" t="inlineStr">
         <is>
-          <t>GUJTHEM</t>
+          <t>GRAUWEIL</t>
         </is>
       </c>
       <c r="B25" s="20">
@@ -34290,7 +34578,7 @@
     <row r="26">
       <c r="A26" s="27" t="inlineStr">
         <is>
-          <t>HERITGFOOD</t>
+          <t>GUJTHEM</t>
         </is>
       </c>
       <c r="B26" s="20">
@@ -34333,7 +34621,7 @@
     <row r="27">
       <c r="A27" s="27" t="inlineStr">
         <is>
-          <t>HIKAL</t>
+          <t>HERITGFOOD</t>
         </is>
       </c>
       <c r="B27" s="20">
@@ -34376,7 +34664,7 @@
     <row r="28">
       <c r="A28" s="27" t="inlineStr">
         <is>
-          <t>HINDOILEXP</t>
+          <t>HIKAL</t>
         </is>
       </c>
       <c r="B28" s="20">
@@ -34419,7 +34707,7 @@
     <row r="29">
       <c r="A29" s="27" t="inlineStr">
         <is>
-          <t>HUBTOWN</t>
+          <t>HINDOILEXP</t>
         </is>
       </c>
       <c r="B29" s="20">
@@ -34462,7 +34750,7 @@
     <row r="30">
       <c r="A30" s="27" t="inlineStr">
         <is>
-          <t>INDNIPPON</t>
+          <t>HUBTOWN</t>
         </is>
       </c>
       <c r="B30" s="20">
@@ -34505,7 +34793,7 @@
     <row r="31">
       <c r="A31" s="27" t="inlineStr">
         <is>
-          <t>INDOCO</t>
+          <t>INDNIPPON</t>
         </is>
       </c>
       <c r="B31" s="20">
@@ -34548,7 +34836,7 @@
     <row r="32">
       <c r="A32" s="27" t="inlineStr">
         <is>
-          <t>INDORAMA</t>
+          <t>INDOCO</t>
         </is>
       </c>
       <c r="B32" s="20">
@@ -34591,7 +34879,7 @@
     <row r="33">
       <c r="A33" s="27" t="inlineStr">
         <is>
-          <t>IPL</t>
+          <t>INDORAMA</t>
         </is>
       </c>
       <c r="B33" s="20">
@@ -34634,7 +34922,7 @@
     <row r="34">
       <c r="A34" s="27" t="inlineStr">
         <is>
-          <t>JASH</t>
+          <t>IPL</t>
         </is>
       </c>
       <c r="B34" s="20">
@@ -34677,7 +34965,7 @@
     <row r="35">
       <c r="A35" s="27" t="inlineStr">
         <is>
-          <t>JAYKAY</t>
+          <t>JASH</t>
         </is>
       </c>
       <c r="B35" s="20">
@@ -34720,7 +35008,7 @@
     <row r="36">
       <c r="A36" s="27" t="inlineStr">
         <is>
-          <t>JGCHEM</t>
+          <t>JAYKAY</t>
         </is>
       </c>
       <c r="B36" s="20">
@@ -34763,7 +35051,7 @@
     <row r="37">
       <c r="A37" s="27" t="inlineStr">
         <is>
-          <t>KCP</t>
+          <t>JGCHEM</t>
         </is>
       </c>
       <c r="B37" s="20">
@@ -34806,7 +35094,7 @@
     <row r="38">
       <c r="A38" s="27" t="inlineStr">
         <is>
-          <t>KIRIINDUS</t>
+          <t>KCP</t>
         </is>
       </c>
       <c r="B38" s="20">
@@ -34849,7 +35137,7 @@
     <row r="39">
       <c r="A39" s="27" t="inlineStr">
         <is>
-          <t>KIRLOSIND</t>
+          <t>KIRIINDUS</t>
         </is>
       </c>
       <c r="B39" s="20">
@@ -34892,7 +35180,7 @@
     <row r="40">
       <c r="A40" s="27" t="inlineStr">
         <is>
-          <t>KLBRENG-B</t>
+          <t>KIRLOSIND</t>
         </is>
       </c>
       <c r="B40" s="20">
@@ -34935,7 +35223,7 @@
     <row r="41">
       <c r="A41" s="27" t="inlineStr">
         <is>
-          <t>KROSS</t>
+          <t>KLBRENG-B</t>
         </is>
       </c>
       <c r="B41" s="20">
@@ -34978,7 +35266,7 @@
     <row r="42">
       <c r="A42" s="27" t="inlineStr">
         <is>
-          <t>KSL</t>
+          <t>KROSS</t>
         </is>
       </c>
       <c r="B42" s="20">
@@ -35021,7 +35309,7 @@
     <row r="43">
       <c r="A43" s="27" t="inlineStr">
         <is>
-          <t>LUXIND</t>
+          <t>KSL</t>
         </is>
       </c>
       <c r="B43" s="20">
@@ -35064,7 +35352,7 @@
     <row r="44">
       <c r="A44" s="27" t="inlineStr">
         <is>
-          <t>MAITHANALL</t>
+          <t>LUXIND</t>
         </is>
       </c>
       <c r="B44" s="20">
@@ -35107,7 +35395,7 @@
     <row r="45">
       <c r="A45" s="27" t="inlineStr">
         <is>
-          <t>MANGLMCEM</t>
+          <t>MAITHANALL</t>
         </is>
       </c>
       <c r="B45" s="20">
@@ -35150,7 +35438,7 @@
     <row r="46">
       <c r="A46" s="27" t="inlineStr">
         <is>
-          <t>MASTEK</t>
+          <t>MANGLMCEM</t>
         </is>
       </c>
       <c r="B46" s="20">
@@ -35193,7 +35481,7 @@
     <row r="47">
       <c r="A47" s="27" t="inlineStr">
         <is>
-          <t>MOBIKWIK</t>
+          <t>MASTEK</t>
         </is>
       </c>
       <c r="B47" s="20">
@@ -35236,7 +35524,7 @@
     <row r="48">
       <c r="A48" s="27" t="inlineStr">
         <is>
-          <t>NETWORK18</t>
+          <t>MOBIKWIK</t>
         </is>
       </c>
       <c r="B48" s="20">
@@ -35279,7 +35567,7 @@
     <row r="49">
       <c r="A49" s="27" t="inlineStr">
         <is>
-          <t>NILKAMAL</t>
+          <t>NETWORK18</t>
         </is>
       </c>
       <c r="B49" s="20">
@@ -35322,7 +35610,7 @@
     <row r="50">
       <c r="A50" s="27" t="inlineStr">
         <is>
-          <t>NORTHARC</t>
+          <t>NILKAMAL</t>
         </is>
       </c>
       <c r="B50" s="20">
@@ -35365,7 +35653,7 @@
     <row r="51">
       <c r="A51" s="27" t="inlineStr">
         <is>
-          <t>NOVARTIND</t>
+          <t>NORTHARC</t>
         </is>
       </c>
       <c r="B51" s="20">
@@ -35408,7 +35696,7 @@
     <row r="52">
       <c r="A52" s="27" t="inlineStr">
         <is>
-          <t>NPST</t>
+          <t>NOVARTIND</t>
         </is>
       </c>
       <c r="B52" s="20">
@@ -35451,7 +35739,7 @@
     <row r="53">
       <c r="A53" s="27" t="inlineStr">
         <is>
-          <t>NRBBEARING</t>
+          <t>NPST</t>
         </is>
       </c>
       <c r="B53" s="20">
@@ -35494,7 +35782,7 @@
     <row r="54">
       <c r="A54" s="27" t="inlineStr">
         <is>
-          <t>OMAXE</t>
+          <t>NRBBEARING</t>
         </is>
       </c>
       <c r="B54" s="20">
@@ -35537,7 +35825,7 @@
     <row r="55">
       <c r="A55" s="27" t="inlineStr">
         <is>
-          <t>OPTIEMUS</t>
+          <t>OMAXE</t>
         </is>
       </c>
       <c r="B55" s="20">
@@ -35580,7 +35868,7 @@
     <row r="56">
       <c r="A56" s="27" t="inlineStr">
         <is>
-          <t>ORIENTHOT</t>
+          <t>OPTIEMUS</t>
         </is>
       </c>
       <c r="B56" s="20">
@@ -35623,7 +35911,7 @@
     <row r="57">
       <c r="A57" s="27" t="inlineStr">
         <is>
-          <t>PITTIENG</t>
+          <t>ORIENTHOT</t>
         </is>
       </c>
       <c r="B57" s="20">
@@ -35666,7 +35954,7 @@
     <row r="58">
       <c r="A58" s="27" t="inlineStr">
         <is>
-          <t>QUADFUTURE</t>
+          <t>PACEDIGITK</t>
         </is>
       </c>
       <c r="B58" s="20">
@@ -35709,7 +35997,7 @@
     <row r="59">
       <c r="A59" s="27" t="inlineStr">
         <is>
-          <t>RACLGEAR</t>
+          <t>PITTIENG</t>
         </is>
       </c>
       <c r="B59" s="20">
@@ -35752,7 +36040,7 @@
     <row r="60">
       <c r="A60" s="27" t="inlineStr">
         <is>
-          <t>RAMRAT</t>
+          <t>PROTEAN</t>
         </is>
       </c>
       <c r="B60" s="20">
@@ -35795,7 +36083,7 @@
     <row r="61">
       <c r="A61" s="27" t="inlineStr">
         <is>
-          <t>RAYMOND</t>
+          <t>QUADFUTURE</t>
         </is>
       </c>
       <c r="B61" s="20">
@@ -35838,7 +36126,7 @@
     <row r="62">
       <c r="A62" s="27" t="inlineStr">
         <is>
-          <t>REFEX</t>
+          <t>RACLGEAR</t>
         </is>
       </c>
       <c r="B62" s="20">
@@ -35881,7 +36169,7 @@
     <row r="63">
       <c r="A63" s="27" t="inlineStr">
         <is>
-          <t>RESPONIND</t>
+          <t>RAMRAT</t>
         </is>
       </c>
       <c r="B63" s="20">
@@ -35924,7 +36212,7 @@
     <row r="64">
       <c r="A64" s="27" t="inlineStr">
         <is>
-          <t>RML</t>
+          <t>RAYMOND</t>
         </is>
       </c>
       <c r="B64" s="20">
@@ -35967,7 +36255,7 @@
     <row r="65">
       <c r="A65" s="27" t="inlineStr">
         <is>
-          <t>ROSSTECH</t>
+          <t>REFEX</t>
         </is>
       </c>
       <c r="B65" s="20">
@@ -36010,7 +36298,7 @@
     <row r="66">
       <c r="A66" s="27" t="inlineStr">
         <is>
-          <t>SAATVIKGL</t>
+          <t>RESPONIND</t>
         </is>
       </c>
       <c r="B66" s="20">
@@ -36053,7 +36341,7 @@
     <row r="67">
       <c r="A67" s="27" t="inlineStr">
         <is>
-          <t>SAKAR</t>
+          <t>RML</t>
         </is>
       </c>
       <c r="B67" s="20">
@@ -36096,7 +36384,7 @@
     <row r="68">
       <c r="A68" s="27" t="inlineStr">
         <is>
-          <t>SAMBHV</t>
+          <t>ROSSTECH</t>
         </is>
       </c>
       <c r="B68" s="20">
@@ -36139,7 +36427,7 @@
     <row r="69">
       <c r="A69" s="27" t="inlineStr">
         <is>
-          <t>SAMHI</t>
+          <t>SAATVIKGL</t>
         </is>
       </c>
       <c r="B69" s="20">
@@ -36182,7 +36470,7 @@
     <row r="70">
       <c r="A70" s="27" t="inlineStr">
         <is>
-          <t>SHAREINDIA</t>
+          <t>SAKAR</t>
         </is>
       </c>
       <c r="B70" s="20">
@@ -36225,7 +36513,7 @@
     <row r="71">
       <c r="A71" s="27" t="inlineStr">
         <is>
-          <t>SIKA</t>
+          <t>SAMBHV</t>
         </is>
       </c>
       <c r="B71" s="20">
@@ -36268,7 +36556,7 @@
     <row r="72">
       <c r="A72" s="27" t="inlineStr">
         <is>
-          <t>SINDHUTRAD</t>
+          <t>SAMHI</t>
         </is>
       </c>
       <c r="B72" s="20">
@@ -36311,7 +36599,7 @@
     <row r="73">
       <c r="A73" s="27" t="inlineStr">
         <is>
-          <t>SMSPHARMA</t>
+          <t>SHAREINDIA</t>
         </is>
       </c>
       <c r="B73" s="20">
@@ -36354,7 +36642,7 @@
     <row r="74">
       <c r="A74" s="27" t="inlineStr">
         <is>
-          <t>SOLARA</t>
+          <t>SIKA</t>
         </is>
       </c>
       <c r="B74" s="20">
@@ -36397,7 +36685,7 @@
     <row r="75">
       <c r="A75" s="27" t="inlineStr">
         <is>
-          <t>SOTL</t>
+          <t>SINDHUTRAD</t>
         </is>
       </c>
       <c r="B75" s="20">
@@ -36440,7 +36728,7 @@
     <row r="76">
       <c r="A76" s="27" t="inlineStr">
         <is>
-          <t>SSWL</t>
+          <t>SMSPHARMA</t>
         </is>
       </c>
       <c r="B76" s="20">
@@ -36483,7 +36771,7 @@
     <row r="77">
       <c r="A77" s="27" t="inlineStr">
         <is>
-          <t>SYMPHONY</t>
+          <t>SOLARA</t>
         </is>
       </c>
       <c r="B77" s="20">
@@ -36526,7 +36814,7 @@
     <row r="78">
       <c r="A78" s="27" t="inlineStr">
         <is>
-          <t>SYNCOMF</t>
+          <t>SOTL</t>
         </is>
       </c>
       <c r="B78" s="20">
@@ -36569,7 +36857,7 @@
     <row r="79">
       <c r="A79" s="27" t="inlineStr">
         <is>
-          <t>TALBROAUTO</t>
+          <t>SSWL</t>
         </is>
       </c>
       <c r="B79" s="20">
@@ -36612,7 +36900,7 @@
     <row r="80">
       <c r="A80" s="27" t="inlineStr">
         <is>
-          <t>TBZ</t>
+          <t>STEELCAS</t>
         </is>
       </c>
       <c r="B80" s="20">
@@ -36655,7 +36943,7 @@
     <row r="81">
       <c r="A81" s="27" t="inlineStr">
         <is>
-          <t>THOMASCOOK</t>
+          <t>SYMPHONY</t>
         </is>
       </c>
       <c r="B81" s="20">
@@ -36698,7 +36986,7 @@
     <row r="82">
       <c r="A82" s="27" t="inlineStr">
         <is>
-          <t>VENKEYS</t>
+          <t>SYNCOMF</t>
         </is>
       </c>
       <c r="B82" s="20">
@@ -36741,7 +37029,7 @@
     <row r="83">
       <c r="A83" s="27" t="inlineStr">
         <is>
-          <t>VENUSPIPES</t>
+          <t>TALBROAUTO</t>
         </is>
       </c>
       <c r="B83" s="20">
@@ -36784,7 +37072,7 @@
     <row r="84">
       <c r="A84" s="27" t="inlineStr">
         <is>
-          <t>VERANDA</t>
+          <t>TBZ</t>
         </is>
       </c>
       <c r="B84" s="20">
@@ -36827,7 +37115,7 @@
     <row r="85">
       <c r="A85" s="27" t="inlineStr">
         <is>
-          <t>VSSL</t>
+          <t>THOMASCOOK</t>
         </is>
       </c>
       <c r="B85" s="20">
@@ -36870,7 +37158,7 @@
     <row r="86">
       <c r="A86" s="27" t="inlineStr">
         <is>
-          <t>WELSPLSOL</t>
+          <t>VENKEYS</t>
         </is>
       </c>
       <c r="B86" s="20">
@@ -36913,7 +37201,7 @@
     <row r="87">
       <c r="A87" s="27" t="inlineStr">
         <is>
-          <t>WENDT</t>
+          <t>VENUSPIPES</t>
         </is>
       </c>
       <c r="B87" s="20">
@@ -36956,7 +37244,7 @@
     <row r="88">
       <c r="A88" s="27" t="inlineStr">
         <is>
-          <t>WINDLAS</t>
+          <t>VERANDA</t>
         </is>
       </c>
       <c r="B88" s="20">
@@ -36999,7 +37287,7 @@
     <row r="89">
       <c r="A89" s="27" t="inlineStr">
         <is>
-          <t>XPROINDIA</t>
+          <t>VSSL</t>
         </is>
       </c>
       <c r="B89" s="20">
@@ -37042,7 +37330,7 @@
     <row r="90">
       <c r="A90" s="27" t="inlineStr">
         <is>
-          <t>ZAGGLE</t>
+          <t>WELSPLSOL</t>
         </is>
       </c>
       <c r="B90" s="20">
@@ -37083,37 +37371,252 @@
       </c>
     </row>
     <row r="91">
-      <c r="A91" s="3" t="inlineStr">
+      <c r="A91" s="27" t="inlineStr">
+        <is>
+          <t>WENDT</t>
+        </is>
+      </c>
+      <c r="B91" s="20">
+        <f>COUNTIF('Trade Log'!$B$4:$B$503,$A91)</f>
+        <v/>
+      </c>
+      <c r="C91" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A91,'Trade Log'!$K$4:$K$503,"&gt;0")</f>
+        <v/>
+      </c>
+      <c r="D91" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A91,'Trade Log'!$K$4:$K$503,"&lt;0")</f>
+        <v/>
+      </c>
+      <c r="E91" s="29">
+        <f>IFERROR($C91/$B91,"")</f>
+        <v/>
+      </c>
+      <c r="F91" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A91,'Trade Log'!$I$4:$I$503)</f>
+        <v/>
+      </c>
+      <c r="G91" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A91,'Trade Log'!$K$4:$K$503)</f>
+        <v/>
+      </c>
+      <c r="H91" s="21">
+        <f>IFERROR($G91/$B91,"")</f>
+        <v/>
+      </c>
+      <c r="I91" s="21">
+        <f>IFERROR(_xlfn.MAXIFS('Trade Log'!$K$4:$K$503,'Trade Log'!$B$4:$B$503,$A91),"")</f>
+        <v/>
+      </c>
+      <c r="J91" s="21">
+        <f>IFERROR(_xlfn.MINIFS('Trade Log'!$K$4:$K$503,'Trade Log'!$B$4:$B$503,$A91),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="27" t="inlineStr">
+        <is>
+          <t>WINDLAS</t>
+        </is>
+      </c>
+      <c r="B92" s="20">
+        <f>COUNTIF('Trade Log'!$B$4:$B$503,$A92)</f>
+        <v/>
+      </c>
+      <c r="C92" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A92,'Trade Log'!$K$4:$K$503,"&gt;0")</f>
+        <v/>
+      </c>
+      <c r="D92" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A92,'Trade Log'!$K$4:$K$503,"&lt;0")</f>
+        <v/>
+      </c>
+      <c r="E92" s="29">
+        <f>IFERROR($C92/$B92,"")</f>
+        <v/>
+      </c>
+      <c r="F92" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A92,'Trade Log'!$I$4:$I$503)</f>
+        <v/>
+      </c>
+      <c r="G92" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A92,'Trade Log'!$K$4:$K$503)</f>
+        <v/>
+      </c>
+      <c r="H92" s="21">
+        <f>IFERROR($G92/$B92,"")</f>
+        <v/>
+      </c>
+      <c r="I92" s="21">
+        <f>IFERROR(_xlfn.MAXIFS('Trade Log'!$K$4:$K$503,'Trade Log'!$B$4:$B$503,$A92),"")</f>
+        <v/>
+      </c>
+      <c r="J92" s="21">
+        <f>IFERROR(_xlfn.MINIFS('Trade Log'!$K$4:$K$503,'Trade Log'!$B$4:$B$503,$A92),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="27" t="inlineStr">
+        <is>
+          <t>XPROINDIA</t>
+        </is>
+      </c>
+      <c r="B93" s="20">
+        <f>COUNTIF('Trade Log'!$B$4:$B$503,$A93)</f>
+        <v/>
+      </c>
+      <c r="C93" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A93,'Trade Log'!$K$4:$K$503,"&gt;0")</f>
+        <v/>
+      </c>
+      <c r="D93" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A93,'Trade Log'!$K$4:$K$503,"&lt;0")</f>
+        <v/>
+      </c>
+      <c r="E93" s="29">
+        <f>IFERROR($C93/$B93,"")</f>
+        <v/>
+      </c>
+      <c r="F93" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A93,'Trade Log'!$I$4:$I$503)</f>
+        <v/>
+      </c>
+      <c r="G93" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A93,'Trade Log'!$K$4:$K$503)</f>
+        <v/>
+      </c>
+      <c r="H93" s="21">
+        <f>IFERROR($G93/$B93,"")</f>
+        <v/>
+      </c>
+      <c r="I93" s="21">
+        <f>IFERROR(_xlfn.MAXIFS('Trade Log'!$K$4:$K$503,'Trade Log'!$B$4:$B$503,$A93),"")</f>
+        <v/>
+      </c>
+      <c r="J93" s="21">
+        <f>IFERROR(_xlfn.MINIFS('Trade Log'!$K$4:$K$503,'Trade Log'!$B$4:$B$503,$A93),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="27" t="inlineStr">
+        <is>
+          <t>ZAGGLE</t>
+        </is>
+      </c>
+      <c r="B94" s="20">
+        <f>COUNTIF('Trade Log'!$B$4:$B$503,$A94)</f>
+        <v/>
+      </c>
+      <c r="C94" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A94,'Trade Log'!$K$4:$K$503,"&gt;0")</f>
+        <v/>
+      </c>
+      <c r="D94" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A94,'Trade Log'!$K$4:$K$503,"&lt;0")</f>
+        <v/>
+      </c>
+      <c r="E94" s="29">
+        <f>IFERROR($C94/$B94,"")</f>
+        <v/>
+      </c>
+      <c r="F94" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A94,'Trade Log'!$I$4:$I$503)</f>
+        <v/>
+      </c>
+      <c r="G94" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A94,'Trade Log'!$K$4:$K$503)</f>
+        <v/>
+      </c>
+      <c r="H94" s="21">
+        <f>IFERROR($G94/$B94,"")</f>
+        <v/>
+      </c>
+      <c r="I94" s="21">
+        <f>IFERROR(_xlfn.MAXIFS('Trade Log'!$K$4:$K$503,'Trade Log'!$B$4:$B$503,$A94),"")</f>
+        <v/>
+      </c>
+      <c r="J94" s="21">
+        <f>IFERROR(_xlfn.MINIFS('Trade Log'!$K$4:$K$503,'Trade Log'!$B$4:$B$503,$A94),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="27" t="inlineStr">
+        <is>
+          <t>ZOTA</t>
+        </is>
+      </c>
+      <c r="B95" s="20">
+        <f>COUNTIF('Trade Log'!$B$4:$B$503,$A95)</f>
+        <v/>
+      </c>
+      <c r="C95" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A95,'Trade Log'!$K$4:$K$503,"&gt;0")</f>
+        <v/>
+      </c>
+      <c r="D95" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A95,'Trade Log'!$K$4:$K$503,"&lt;0")</f>
+        <v/>
+      </c>
+      <c r="E95" s="29">
+        <f>IFERROR($C95/$B95,"")</f>
+        <v/>
+      </c>
+      <c r="F95" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A95,'Trade Log'!$I$4:$I$503)</f>
+        <v/>
+      </c>
+      <c r="G95" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A95,'Trade Log'!$K$4:$K$503)</f>
+        <v/>
+      </c>
+      <c r="H95" s="21">
+        <f>IFERROR($G95/$B95,"")</f>
+        <v/>
+      </c>
+      <c r="I95" s="21">
+        <f>IFERROR(_xlfn.MAXIFS('Trade Log'!$K$4:$K$503,'Trade Log'!$B$4:$B$503,$A95),"")</f>
+        <v/>
+      </c>
+      <c r="J95" s="21">
+        <f>IFERROR(_xlfn.MINIFS('Trade Log'!$K$4:$K$503,'Trade Log'!$B$4:$B$503,$A95),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" s="3" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="B91" s="30">
-        <f>SUM(B4:B90)</f>
-        <v/>
-      </c>
-      <c r="C91" s="30">
-        <f>SUM(C4:C90)</f>
-        <v/>
-      </c>
-      <c r="D91" s="30">
-        <f>SUM(D4:D90)</f>
-        <v/>
-      </c>
-      <c r="E91" s="31">
-        <f>IFERROR(C91/B91,"")</f>
-        <v/>
-      </c>
-      <c r="F91" s="32">
-        <f>SUM(F4:F90)</f>
-        <v/>
-      </c>
-      <c r="G91" s="32">
-        <f>SUM(G4:G90)</f>
-        <v/>
-      </c>
-      <c r="H91" s="32">
-        <f>IFERROR(G91/B91,"")</f>
+      <c r="B96" s="30">
+        <f>SUM(B4:B95)</f>
+        <v/>
+      </c>
+      <c r="C96" s="30">
+        <f>SUM(C4:C95)</f>
+        <v/>
+      </c>
+      <c r="D96" s="30">
+        <f>SUM(D4:D95)</f>
+        <v/>
+      </c>
+      <c r="E96" s="31">
+        <f>IFERROR(C96/B96,"")</f>
+        <v/>
+      </c>
+      <c r="F96" s="32">
+        <f>SUM(F4:F95)</f>
+        <v/>
+      </c>
+      <c r="G96" s="32">
+        <f>SUM(G4:G95)</f>
+        <v/>
+      </c>
+      <c r="H96" s="32">
+        <f>IFERROR(G96/B96,"")</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Data update — 2026-09-23 candle + results refresh
</commit_message>
<xml_diff>
--- a/results/strategy_pnl_simple.xlsx
+++ b/results/strategy_pnl_simple.xlsx
@@ -1473,7 +1473,7 @@
         <v/>
       </c>
       <c r="J4" s="4" t="n">
-        <v>464.09</v>
+        <v>50.15</v>
       </c>
       <c r="K4" s="21">
         <f>IF(OR($B4="",$I4=""),"",$I4-IF($J4="",0,$J4))</f>
@@ -1524,7 +1524,7 @@
         <v/>
       </c>
       <c r="J5" s="4" t="n">
-        <v>538.4</v>
+        <v>50.15</v>
       </c>
       <c r="K5" s="21">
         <f>IF(OR($B5="",$I5=""),"",$I5-IF($J5="",0,$J5))</f>
@@ -1575,7 +1575,7 @@
         <v/>
       </c>
       <c r="J6" s="4" t="n">
-        <v>514.1900000000001</v>
+        <v>101.22</v>
       </c>
       <c r="K6" s="21">
         <f>IF(OR($B6="",$I6=""),"",$I6-IF($J6="",0,$J6))</f>
@@ -1626,7 +1626,7 @@
         <v/>
       </c>
       <c r="J7" s="4" t="n">
-        <v>595.38</v>
+        <v>111.37</v>
       </c>
       <c r="K7" s="21">
         <f>IF(OR($B7="",$I7=""),"",$I7-IF($J7="",0,$J7))</f>
@@ -1677,7 +1677,7 @@
         <v/>
       </c>
       <c r="J8" s="4" t="n">
-        <v>525.1900000000001</v>
+        <v>109.94</v>
       </c>
       <c r="K8" s="21">
         <f>IF(OR($B8="",$I8=""),"",$I8-IF($J8="",0,$J8))</f>
@@ -1728,7 +1728,7 @@
         <v/>
       </c>
       <c r="J9" s="4" t="n">
-        <v>451.6</v>
+        <v>0</v>
       </c>
       <c r="K9" s="21">
         <f>IF(OR($B9="",$I9=""),"",$I9-IF($J9="",0,$J9))</f>
@@ -1779,7 +1779,7 @@
         <v/>
       </c>
       <c r="J10" s="4" t="n">
-        <v>367.34</v>
+        <v>78.45</v>
       </c>
       <c r="K10" s="21">
         <f>IF(OR($B10="",$I10=""),"",$I10-IF($J10="",0,$J10))</f>
@@ -1830,7 +1830,7 @@
         <v/>
       </c>
       <c r="J11" s="4" t="n">
-        <v>346.76</v>
+        <v>0</v>
       </c>
       <c r="K11" s="21">
         <f>IF(OR($B11="",$I11=""),"",$I11-IF($J11="",0,$J11))</f>
@@ -1881,7 +1881,7 @@
         <v/>
       </c>
       <c r="J12" s="4" t="n">
-        <v>376.36</v>
+        <v>84.34999999999999</v>
       </c>
       <c r="K12" s="21">
         <f>IF(OR($B12="",$I12=""),"",$I12-IF($J12="",0,$J12))</f>
@@ -1932,7 +1932,7 @@
         <v/>
       </c>
       <c r="J13" s="4" t="n">
-        <v>322.36</v>
+        <v>70.7</v>
       </c>
       <c r="K13" s="21">
         <f>IF(OR($B13="",$I13=""),"",$I13-IF($J13="",0,$J13))</f>
@@ -1983,7 +1983,7 @@
         <v/>
       </c>
       <c r="J14" s="4" t="n">
-        <v>376.81</v>
+        <v>84.23999999999999</v>
       </c>
       <c r="K14" s="21">
         <f>IF(OR($B14="",$I14=""),"",$I14-IF($J14="",0,$J14))</f>
@@ -2034,7 +2034,7 @@
         <v/>
       </c>
       <c r="J15" s="4" t="n">
-        <v>339.07</v>
+        <v>87.63</v>
       </c>
       <c r="K15" s="21">
         <f>IF(OR($B15="",$I15=""),"",$I15-IF($J15="",0,$J15))</f>
@@ -2085,7 +2085,7 @@
         <v/>
       </c>
       <c r="J16" s="4" t="n">
-        <v>427.19</v>
+        <v>0</v>
       </c>
       <c r="K16" s="21">
         <f>IF(OR($B16="",$I16=""),"",$I16-IF($J16="",0,$J16))</f>
@@ -2136,7 +2136,7 @@
         <v/>
       </c>
       <c r="J17" s="4" t="n">
-        <v>341.04</v>
+        <v>0</v>
       </c>
       <c r="K17" s="21">
         <f>IF(OR($B17="",$I17=""),"",$I17-IF($J17="",0,$J17))</f>
@@ -2187,7 +2187,7 @@
         <v/>
       </c>
       <c r="J18" s="4" t="n">
-        <v>376.04</v>
+        <v>84.42</v>
       </c>
       <c r="K18" s="21">
         <f>IF(OR($B18="",$I18=""),"",$I18-IF($J18="",0,$J18))</f>
@@ -2238,7 +2238,7 @@
         <v/>
       </c>
       <c r="J19" s="4" t="n">
-        <v>374.18</v>
+        <v>79.34999999999999</v>
       </c>
       <c r="K19" s="21">
         <f>IF(OR($B19="",$I19=""),"",$I19-IF($J19="",0,$J19))</f>
@@ -2289,7 +2289,7 @@
         <v/>
       </c>
       <c r="J20" s="4" t="n">
-        <v>444.79</v>
+        <v>0</v>
       </c>
       <c r="K20" s="21">
         <f>IF(OR($B20="",$I20=""),"",$I20-IF($J20="",0,$J20))</f>
@@ -2340,7 +2340,7 @@
         <v/>
       </c>
       <c r="J21" s="4" t="n">
-        <v>197.25</v>
+        <v>0</v>
       </c>
       <c r="K21" s="21">
         <f>IF(OR($B21="",$I21=""),"",$I21-IF($J21="",0,$J21))</f>
@@ -2391,7 +2391,7 @@
         <v/>
       </c>
       <c r="J22" s="4" t="n">
-        <v>203.83</v>
+        <v>0</v>
       </c>
       <c r="K22" s="21">
         <f>IF(OR($B22="",$I22=""),"",$I22-IF($J22="",0,$J22))</f>
@@ -2442,7 +2442,7 @@
         <v/>
       </c>
       <c r="J23" s="4" t="n">
-        <v>251.98</v>
+        <v>0</v>
       </c>
       <c r="K23" s="21">
         <f>IF(OR($B23="",$I23=""),"",$I23-IF($J23="",0,$J23))</f>
@@ -2493,7 +2493,7 @@
         <v/>
       </c>
       <c r="J24" s="4" t="n">
-        <v>534.25</v>
+        <v>14.75</v>
       </c>
       <c r="K24" s="21">
         <f>IF(OR($B24="",$I24=""),"",$I24-IF($J24="",0,$J24))</f>
@@ -2544,7 +2544,7 @@
         <v/>
       </c>
       <c r="J25" s="4" t="n">
-        <v>208.81</v>
+        <v>0</v>
       </c>
       <c r="K25" s="21">
         <f>IF(OR($B25="",$I25=""),"",$I25-IF($J25="",0,$J25))</f>
@@ -2595,7 +2595,7 @@
         <v/>
       </c>
       <c r="J26" s="4" t="n">
-        <v>248.04</v>
+        <v>0</v>
       </c>
       <c r="K26" s="21">
         <f>IF(OR($B26="",$I26=""),"",$I26-IF($J26="",0,$J26))</f>
@@ -2646,7 +2646,7 @@
         <v/>
       </c>
       <c r="J27" s="4" t="n">
-        <v>200.87</v>
+        <v>0</v>
       </c>
       <c r="K27" s="21">
         <f>IF(OR($B27="",$I27=""),"",$I27-IF($J27="",0,$J27))</f>
@@ -2697,7 +2697,7 @@
         <v/>
       </c>
       <c r="J28" s="4" t="n">
-        <v>801.17</v>
+        <v>295.22</v>
       </c>
       <c r="K28" s="21">
         <f>IF(OR($B28="",$I28=""),"",$I28-IF($J28="",0,$J28))</f>
@@ -2748,7 +2748,7 @@
         <v/>
       </c>
       <c r="J29" s="4" t="n">
-        <v>210.52</v>
+        <v>0</v>
       </c>
       <c r="K29" s="21">
         <f>IF(OR($B29="",$I29=""),"",$I29-IF($J29="",0,$J29))</f>
@@ -2799,7 +2799,7 @@
         <v/>
       </c>
       <c r="J30" s="4" t="n">
-        <v>517.89</v>
+        <v>14.75</v>
       </c>
       <c r="K30" s="21">
         <f>IF(OR($B30="",$I30=""),"",$I30-IF($J30="",0,$J30))</f>
@@ -2850,7 +2850,7 @@
         <v/>
       </c>
       <c r="J31" s="4" t="n">
-        <v>377.89</v>
+        <v>84.45</v>
       </c>
       <c r="K31" s="21">
         <f>IF(OR($B31="",$I31=""),"",$I31-IF($J31="",0,$J31))</f>
@@ -2901,7 +2901,7 @@
         <v/>
       </c>
       <c r="J32" s="4" t="n">
-        <v>336.52</v>
+        <v>84.44</v>
       </c>
       <c r="K32" s="21">
         <f>IF(OR($B32="",$I32=""),"",$I32-IF($J32="",0,$J32))</f>
@@ -2952,7 +2952,7 @@
         <v/>
       </c>
       <c r="J33" s="4" t="n">
-        <v>526.1799999999999</v>
+        <v>0</v>
       </c>
       <c r="K33" s="21">
         <f>IF(OR($B33="",$I33=""),"",$I33-IF($J33="",0,$J33))</f>
@@ -3003,7 +3003,7 @@
         <v/>
       </c>
       <c r="J34" s="4" t="n">
-        <v>336.28</v>
+        <v>84.20999999999999</v>
       </c>
       <c r="K34" s="21">
         <f>IF(OR($B34="",$I34=""),"",$I34-IF($J34="",0,$J34))</f>
@@ -3054,7 +3054,7 @@
         <v/>
       </c>
       <c r="J35" s="4" t="n">
-        <v>373.48</v>
+        <v>83.05</v>
       </c>
       <c r="K35" s="21">
         <f>IF(OR($B35="",$I35=""),"",$I35-IF($J35="",0,$J35))</f>
@@ -3105,7 +3105,7 @@
         <v/>
       </c>
       <c r="J36" s="4" t="n">
-        <v>536.1</v>
+        <v>0</v>
       </c>
       <c r="K36" s="21">
         <f>IF(OR($B36="",$I36=""),"",$I36-IF($J36="",0,$J36))</f>
@@ -3156,7 +3156,7 @@
         <v/>
       </c>
       <c r="J37" s="4" t="n">
-        <v>529.84</v>
+        <v>0</v>
       </c>
       <c r="K37" s="21">
         <f>IF(OR($B37="",$I37=""),"",$I37-IF($J37="",0,$J37))</f>
@@ -3207,7 +3207,7 @@
         <v/>
       </c>
       <c r="J38" s="4" t="n">
-        <v>207.3</v>
+        <v>0</v>
       </c>
       <c r="K38" s="21">
         <f>IF(OR($B38="",$I38=""),"",$I38-IF($J38="",0,$J38))</f>
@@ -3258,7 +3258,7 @@
         <v/>
       </c>
       <c r="J39" s="4" t="n">
-        <v>246.41</v>
+        <v>0</v>
       </c>
       <c r="K39" s="21">
         <f>IF(OR($B39="",$I39=""),"",$I39-IF($J39="",0,$J39))</f>
@@ -3309,7 +3309,7 @@
         <v/>
       </c>
       <c r="J40" s="4" t="n">
-        <v>251.07</v>
+        <v>0</v>
       </c>
       <c r="K40" s="21">
         <f>IF(OR($B40="",$I40=""),"",$I40-IF($J40="",0,$J40))</f>
@@ -3360,7 +3360,7 @@
         <v/>
       </c>
       <c r="J41" s="4" t="n">
-        <v>198.63</v>
+        <v>0</v>
       </c>
       <c r="K41" s="21">
         <f>IF(OR($B41="",$I41=""),"",$I41-IF($J41="",0,$J41))</f>
@@ -3411,7 +3411,7 @@
         <v/>
       </c>
       <c r="J42" s="4" t="n">
-        <v>950.51</v>
+        <v>121.96</v>
       </c>
       <c r="K42" s="21">
         <f>IF(OR($B42="",$I42=""),"",$I42-IF($J42="",0,$J42))</f>
@@ -3462,7 +3462,7 @@
         <v/>
       </c>
       <c r="J43" s="4" t="n">
-        <v>934.51</v>
+        <v>110.04</v>
       </c>
       <c r="K43" s="21">
         <f>IF(OR($B43="",$I43=""),"",$I43-IF($J43="",0,$J43))</f>
@@ -3513,7 +3513,7 @@
         <v/>
       </c>
       <c r="J44" s="4" t="n">
-        <v>964.38</v>
+        <v>122.26</v>
       </c>
       <c r="K44" s="21">
         <f>IF(OR($B44="",$I44=""),"",$I44-IF($J44="",0,$J44))</f>
@@ -3564,7 +3564,7 @@
         <v/>
       </c>
       <c r="J45" s="4" t="n">
-        <v>612.7</v>
+        <v>222.4</v>
       </c>
       <c r="K45" s="21">
         <f>IF(OR($B45="",$I45=""),"",$I45-IF($J45="",0,$J45))</f>
@@ -3615,7 +3615,7 @@
         <v/>
       </c>
       <c r="J46" s="4" t="n">
-        <v>613.84</v>
+        <v>222.89</v>
       </c>
       <c r="K46" s="21">
         <f>IF(OR($B46="",$I46=""),"",$I46-IF($J46="",0,$J46))</f>
@@ -3666,7 +3666,7 @@
         <v/>
       </c>
       <c r="J47" s="4" t="n">
-        <v>693.27</v>
+        <v>237.84</v>
       </c>
       <c r="K47" s="21">
         <f>IF(OR($B47="",$I47=""),"",$I47-IF($J47="",0,$J47))</f>
@@ -3717,7 +3717,7 @@
         <v/>
       </c>
       <c r="J48" s="4" t="n">
-        <v>685.47</v>
+        <v>222.06</v>
       </c>
       <c r="K48" s="21">
         <f>IF(OR($B48="",$I48=""),"",$I48-IF($J48="",0,$J48))</f>
@@ -3768,7 +3768,7 @@
         <v/>
       </c>
       <c r="J49" s="4" t="n">
-        <v>546.53</v>
+        <v>154.21</v>
       </c>
       <c r="K49" s="21">
         <f>IF(OR($B49="",$I49=""),"",$I49-IF($J49="",0,$J49))</f>
@@ -3819,7 +3819,7 @@
         <v/>
       </c>
       <c r="J50" s="4" t="n">
-        <v>609.98</v>
+        <v>130.61</v>
       </c>
       <c r="K50" s="21">
         <f>IF(OR($B50="",$I50=""),"",$I50-IF($J50="",0,$J50))</f>
@@ -3870,7 +3870,7 @@
         <v/>
       </c>
       <c r="J51" s="4" t="n">
-        <v>415.51</v>
+        <v>0</v>
       </c>
       <c r="K51" s="21">
         <f>IF(OR($B51="",$I51=""),"",$I51-IF($J51="",0,$J51))</f>
@@ -3921,7 +3921,7 @@
         <v/>
       </c>
       <c r="J52" s="4" t="n">
-        <v>397.84</v>
+        <v>0</v>
       </c>
       <c r="K52" s="21">
         <f>IF(OR($B52="",$I52=""),"",$I52-IF($J52="",0,$J52))</f>
@@ -3972,7 +3972,7 @@
         <v/>
       </c>
       <c r="J53" s="4" t="n">
-        <v>312.31</v>
+        <v>0</v>
       </c>
       <c r="K53" s="21">
         <f>IF(OR($B53="",$I53=""),"",$I53-IF($J53="",0,$J53))</f>
@@ -4023,7 +4023,7 @@
         <v/>
       </c>
       <c r="J54" s="4" t="n">
-        <v>601.39</v>
+        <v>129.27</v>
       </c>
       <c r="K54" s="21">
         <f>IF(OR($B54="",$I54=""),"",$I54-IF($J54="",0,$J54))</f>
@@ -4074,7 +4074,7 @@
         <v/>
       </c>
       <c r="J55" s="4" t="n">
-        <v>332.07</v>
+        <v>0</v>
       </c>
       <c r="K55" s="21">
         <f>IF(OR($B55="",$I55=""),"",$I55-IF($J55="",0,$J55))</f>
@@ -4125,7 +4125,7 @@
         <v/>
       </c>
       <c r="J56" s="4" t="n">
-        <v>407.39</v>
+        <v>0</v>
       </c>
       <c r="K56" s="21">
         <f>IF(OR($B56="",$I56=""),"",$I56-IF($J56="",0,$J56))</f>
@@ -4176,7 +4176,7 @@
         <v/>
       </c>
       <c r="J57" s="4" t="n">
-        <v>596.23</v>
+        <v>121.78</v>
       </c>
       <c r="K57" s="21">
         <f>IF(OR($B57="",$I57=""),"",$I57-IF($J57="",0,$J57))</f>
@@ -4227,7 +4227,7 @@
         <v/>
       </c>
       <c r="J58" s="4" t="n">
-        <v>508.65</v>
+        <v>0</v>
       </c>
       <c r="K58" s="21">
         <f>IF(OR($B58="",$I58=""),"",$I58-IF($J58="",0,$J58))</f>
@@ -4278,7 +4278,7 @@
         <v/>
       </c>
       <c r="J59" s="4" t="n">
-        <v>480.12</v>
+        <v>0</v>
       </c>
       <c r="K59" s="21">
         <f>IF(OR($B59="",$I59=""),"",$I59-IF($J59="",0,$J59))</f>
@@ -4329,7 +4329,7 @@
         <v/>
       </c>
       <c r="J60" s="4" t="n">
-        <v>296.33</v>
+        <v>14.75</v>
       </c>
       <c r="K60" s="21">
         <f>IF(OR($B60="",$I60=""),"",$I60-IF($J60="",0,$J60))</f>
@@ -4380,7 +4380,7 @@
         <v/>
       </c>
       <c r="J61" s="4" t="n">
-        <v>687.71</v>
+        <v>122.24</v>
       </c>
       <c r="K61" s="21">
         <f>IF(OR($B61="",$I61=""),"",$I61-IF($J61="",0,$J61))</f>
@@ -4431,7 +4431,7 @@
         <v/>
       </c>
       <c r="J62" s="4" t="n">
-        <v>610.26</v>
+        <v>129.45</v>
       </c>
       <c r="K62" s="21">
         <f>IF(OR($B62="",$I62=""),"",$I62-IF($J62="",0,$J62))</f>
@@ -4482,7 +4482,7 @@
         <v/>
       </c>
       <c r="J63" s="4" t="n">
-        <v>484.3</v>
+        <v>0</v>
       </c>
       <c r="K63" s="21">
         <f>IF(OR($B63="",$I63=""),"",$I63-IF($J63="",0,$J63))</f>
@@ -4533,7 +4533,7 @@
         <v/>
       </c>
       <c r="J64" s="4" t="n">
-        <v>437.62</v>
+        <v>96.40000000000001</v>
       </c>
       <c r="K64" s="21">
         <f>IF(OR($B64="",$I64=""),"",$I64-IF($J64="",0,$J64))</f>
@@ -4584,7 +4584,7 @@
         <v/>
       </c>
       <c r="J65" s="4" t="n">
-        <v>384.09</v>
+        <v>91.26000000000001</v>
       </c>
       <c r="K65" s="21">
         <f>IF(OR($B65="",$I65=""),"",$I65-IF($J65="",0,$J65))</f>
@@ -4635,7 +4635,7 @@
         <v/>
       </c>
       <c r="J66" s="4" t="n">
-        <v>220.84</v>
+        <v>0</v>
       </c>
       <c r="K66" s="21">
         <f>IF(OR($B66="",$I66=""),"",$I66-IF($J66="",0,$J66))</f>
@@ -4686,7 +4686,7 @@
         <v/>
       </c>
       <c r="J67" s="4" t="n">
-        <v>411.42</v>
+        <v>0</v>
       </c>
       <c r="K67" s="21">
         <f>IF(OR($B67="",$I67=""),"",$I67-IF($J67="",0,$J67))</f>
@@ -4737,7 +4737,7 @@
         <v/>
       </c>
       <c r="J68" s="4" t="n">
-        <v>478.28</v>
+        <v>0</v>
       </c>
       <c r="K68" s="21">
         <f>IF(OR($B68="",$I68=""),"",$I68-IF($J68="",0,$J68))</f>
@@ -4788,7 +4788,7 @@
         <v/>
       </c>
       <c r="J69" s="4" t="n">
-        <v>161.82</v>
+        <v>14.75</v>
       </c>
       <c r="K69" s="21">
         <f>IF(OR($B69="",$I69=""),"",$I69-IF($J69="",0,$J69))</f>
@@ -4839,7 +4839,7 @@
         <v/>
       </c>
       <c r="J70" s="4" t="n">
-        <v>382.7</v>
+        <v>91.06</v>
       </c>
       <c r="K70" s="21">
         <f>IF(OR($B70="",$I70=""),"",$I70-IF($J70="",0,$J70))</f>
@@ -4890,7 +4890,7 @@
         <v/>
       </c>
       <c r="J71" s="4" t="n">
-        <v>431.78</v>
+        <v>90.95999999999999</v>
       </c>
       <c r="K71" s="21">
         <f>IF(OR($B71="",$I71=""),"",$I71-IF($J71="",0,$J71))</f>
@@ -4941,7 +4941,7 @@
         <v/>
       </c>
       <c r="J72" s="4" t="n">
-        <v>393.8</v>
+        <v>86.16</v>
       </c>
       <c r="K72" s="21">
         <f>IF(OR($B72="",$I72=""),"",$I72-IF($J72="",0,$J72))</f>
@@ -4992,7 +4992,7 @@
         <v/>
       </c>
       <c r="J73" s="4" t="n">
-        <v>166.41</v>
+        <v>14.75</v>
       </c>
       <c r="K73" s="21">
         <f>IF(OR($B73="",$I73=""),"",$I73-IF($J73="",0,$J73))</f>
@@ -5043,7 +5043,7 @@
         <v/>
       </c>
       <c r="J74" s="4" t="n">
-        <v>341.34</v>
+        <v>80.02</v>
       </c>
       <c r="K74" s="21">
         <f>IF(OR($B74="",$I74=""),"",$I74-IF($J74="",0,$J74))</f>
@@ -5094,7 +5094,7 @@
         <v/>
       </c>
       <c r="J75" s="4" t="n">
-        <v>346.98</v>
+        <v>85.95999999999999</v>
       </c>
       <c r="K75" s="21">
         <f>IF(OR($B75="",$I75=""),"",$I75-IF($J75="",0,$J75))</f>
@@ -5145,7 +5145,7 @@
         <v/>
       </c>
       <c r="J76" s="4" t="n">
-        <v>241.15</v>
+        <v>0</v>
       </c>
       <c r="K76" s="21">
         <f>IF(OR($B76="",$I76=""),"",$I76-IF($J76="",0,$J76))</f>
@@ -5196,7 +5196,7 @@
         <v/>
       </c>
       <c r="J77" s="4" t="n">
-        <v>393.05</v>
+        <v>88.37</v>
       </c>
       <c r="K77" s="21">
         <f>IF(OR($B77="",$I77=""),"",$I77-IF($J77="",0,$J77))</f>
@@ -5247,7 +5247,7 @@
         <v/>
       </c>
       <c r="J78" s="4" t="n">
-        <v>296.69</v>
+        <v>0</v>
       </c>
       <c r="K78" s="21">
         <f>IF(OR($B78="",$I78=""),"",$I78-IF($J78="",0,$J78))</f>
@@ -5298,7 +5298,7 @@
         <v/>
       </c>
       <c r="J79" s="4" t="n">
-        <v>333.47</v>
+        <v>71.69</v>
       </c>
       <c r="K79" s="21">
         <f>IF(OR($B79="",$I79=""),"",$I79-IF($J79="",0,$J79))</f>
@@ -5349,7 +5349,7 @@
         <v/>
       </c>
       <c r="J80" s="4" t="n">
-        <v>334.83</v>
+        <v>50.15</v>
       </c>
       <c r="K80" s="21">
         <f>IF(OR($B80="",$I80=""),"",$I80-IF($J80="",0,$J80))</f>
@@ -5400,7 +5400,7 @@
         <v/>
       </c>
       <c r="J81" s="4" t="n">
-        <v>162.41</v>
+        <v>0</v>
       </c>
       <c r="K81" s="21">
         <f>IF(OR($B81="",$I81=""),"",$I81-IF($J81="",0,$J81))</f>
@@ -5451,7 +5451,7 @@
         <v/>
       </c>
       <c r="J82" s="4" t="n">
-        <v>302.18</v>
+        <v>0</v>
       </c>
       <c r="K82" s="21">
         <f>IF(OR($B82="",$I82=""),"",$I82-IF($J82="",0,$J82))</f>
@@ -5502,7 +5502,7 @@
         <v/>
       </c>
       <c r="J83" s="4" t="n">
-        <v>244.39</v>
+        <v>0</v>
       </c>
       <c r="K83" s="21">
         <f>IF(OR($B83="",$I83=""),"",$I83-IF($J83="",0,$J83))</f>
@@ -5553,7 +5553,7 @@
         <v/>
       </c>
       <c r="J84" s="4" t="n">
-        <v>223.48</v>
+        <v>0</v>
       </c>
       <c r="K84" s="21">
         <f>IF(OR($B84="",$I84=""),"",$I84-IF($J84="",0,$J84))</f>
@@ -5604,7 +5604,7 @@
         <v/>
       </c>
       <c r="J85" s="4" t="n">
-        <v>118.41</v>
+        <v>0</v>
       </c>
       <c r="K85" s="21">
         <f>IF(OR($B85="",$I85=""),"",$I85-IF($J85="",0,$J85))</f>
@@ -5655,7 +5655,7 @@
         <v/>
       </c>
       <c r="J86" s="4" t="n">
-        <v>264.5</v>
+        <v>0</v>
       </c>
       <c r="K86" s="21">
         <f>IF(OR($B86="",$I86=""),"",$I86-IF($J86="",0,$J86))</f>
@@ -5706,7 +5706,7 @@
         <v/>
       </c>
       <c r="J87" s="4" t="n">
-        <v>262.49</v>
+        <v>0</v>
       </c>
       <c r="K87" s="21">
         <f>IF(OR($B87="",$I87=""),"",$I87-IF($J87="",0,$J87))</f>
@@ -5757,7 +5757,7 @@
         <v/>
       </c>
       <c r="J88" s="4" t="n">
-        <v>214.74</v>
+        <v>0</v>
       </c>
       <c r="K88" s="21">
         <f>IF(OR($B88="",$I88=""),"",$I88-IF($J88="",0,$J88))</f>
@@ -5808,7 +5808,7 @@
         <v/>
       </c>
       <c r="J89" s="4" t="n">
-        <v>261.3</v>
+        <v>0</v>
       </c>
       <c r="K89" s="21">
         <f>IF(OR($B89="",$I89=""),"",$I89-IF($J89="",0,$J89))</f>
@@ -5859,7 +5859,7 @@
         <v/>
       </c>
       <c r="J90" s="4" t="n">
-        <v>833.8200000000001</v>
+        <v>264.84</v>
       </c>
       <c r="K90" s="21">
         <f>IF(OR($B90="",$I90=""),"",$I90-IF($J90="",0,$J90))</f>
@@ -5910,7 +5910,7 @@
         <v/>
       </c>
       <c r="J91" s="4" t="n">
-        <v>257.68</v>
+        <v>0</v>
       </c>
       <c r="K91" s="21">
         <f>IF(OR($B91="",$I91=""),"",$I91-IF($J91="",0,$J91))</f>
@@ -5961,7 +5961,7 @@
         <v/>
       </c>
       <c r="J92" s="4" t="n">
-        <v>739.8200000000001</v>
+        <v>264.89</v>
       </c>
       <c r="K92" s="21">
         <f>IF(OR($B92="",$I92=""),"",$I92-IF($J92="",0,$J92))</f>
@@ -6012,7 +6012,7 @@
         <v/>
       </c>
       <c r="J93" s="4" t="n">
-        <v>766.78</v>
+        <v>266.26</v>
       </c>
       <c r="K93" s="21">
         <f>IF(OR($B93="",$I93=""),"",$I93-IF($J93="",0,$J93))</f>
@@ -6063,7 +6063,7 @@
         <v/>
       </c>
       <c r="J94" s="4" t="n">
-        <v>433.61</v>
+        <v>100.63</v>
       </c>
       <c r="K94" s="21">
         <f>IF(OR($B94="",$I94=""),"",$I94-IF($J94="",0,$J94))</f>
@@ -6114,7 +6114,7 @@
         <v/>
       </c>
       <c r="J95" s="4" t="n">
-        <v>181.46</v>
+        <v>14.75</v>
       </c>
       <c r="K95" s="21">
         <f>IF(OR($B95="",$I95=""),"",$I95-IF($J95="",0,$J95))</f>
@@ -6165,7 +6165,7 @@
         <v/>
       </c>
       <c r="J96" s="4" t="n">
-        <v>430.76</v>
+        <v>97.95999999999999</v>
       </c>
       <c r="K96" s="21">
         <f>IF(OR($B96="",$I96=""),"",$I96-IF($J96="",0,$J96))</f>
@@ -6216,7 +6216,7 @@
         <v/>
       </c>
       <c r="J97" s="4" t="n">
-        <v>437.06</v>
+        <v>0</v>
       </c>
       <c r="K97" s="21">
         <f>IF(OR($B97="",$I97=""),"",$I97-IF($J97="",0,$J97))</f>
@@ -6267,7 +6267,7 @@
         <v/>
       </c>
       <c r="J98" s="4" t="n">
-        <v>487.6</v>
+        <v>97.89</v>
       </c>
       <c r="K98" s="21">
         <f>IF(OR($B98="",$I98=""),"",$I98-IF($J98="",0,$J98))</f>
@@ -6318,7 +6318,7 @@
         <v/>
       </c>
       <c r="J99" s="4" t="n">
-        <v>311.54</v>
+        <v>14.75</v>
       </c>
       <c r="K99" s="21">
         <f>IF(OR($B99="",$I99=""),"",$I99-IF($J99="",0,$J99))</f>
@@ -6369,7 +6369,7 @@
         <v/>
       </c>
       <c r="J100" s="4" t="n">
-        <v>380.66</v>
+        <v>0</v>
       </c>
       <c r="K100" s="21">
         <f>IF(OR($B100="",$I100=""),"",$I100-IF($J100="",0,$J100))</f>
@@ -6420,7 +6420,7 @@
         <v/>
       </c>
       <c r="J101" s="4" t="n">
-        <v>516.37</v>
+        <v>0</v>
       </c>
       <c r="K101" s="21">
         <f>IF(OR($B101="",$I101=""),"",$I101-IF($J101="",0,$J101))</f>
@@ -6471,7 +6471,7 @@
         <v/>
       </c>
       <c r="J102" s="4" t="n">
-        <v>487.69</v>
+        <v>98.01000000000001</v>
       </c>
       <c r="K102" s="21">
         <f>IF(OR($B102="",$I102=""),"",$I102-IF($J102="",0,$J102))</f>
@@ -6522,7 +6522,7 @@
         <v/>
       </c>
       <c r="J103" s="4" t="n">
-        <v>161.36</v>
+        <v>14.75</v>
       </c>
       <c r="K103" s="21">
         <f>IF(OR($B103="",$I103=""),"",$I103-IF($J103="",0,$J103))</f>
@@ -6573,7 +6573,7 @@
         <v/>
       </c>
       <c r="J104" s="4" t="n">
-        <v>185.66</v>
+        <v>14.75</v>
       </c>
       <c r="K104" s="21">
         <f>IF(OR($B104="",$I104=""),"",$I104-IF($J104="",0,$J104))</f>
@@ -6624,7 +6624,7 @@
         <v/>
       </c>
       <c r="J105" s="4" t="n">
-        <v>337.14</v>
+        <v>0</v>
       </c>
       <c r="K105" s="21">
         <f>IF(OR($B105="",$I105=""),"",$I105-IF($J105="",0,$J105))</f>
@@ -6675,7 +6675,7 @@
         <v/>
       </c>
       <c r="J106" s="4" t="n">
-        <v>172.01</v>
+        <v>0</v>
       </c>
       <c r="K106" s="21">
         <f>IF(OR($B106="",$I106=""),"",$I106-IF($J106="",0,$J106))</f>
@@ -6726,7 +6726,7 @@
         <v/>
       </c>
       <c r="J107" s="4" t="n">
-        <v>343.41</v>
+        <v>0</v>
       </c>
       <c r="K107" s="21">
         <f>IF(OR($B107="",$I107=""),"",$I107-IF($J107="",0,$J107))</f>
@@ -6777,7 +6777,7 @@
         <v/>
       </c>
       <c r="J108" s="4" t="n">
-        <v>187.34</v>
+        <v>14.75</v>
       </c>
       <c r="K108" s="21">
         <f>IF(OR($B108="",$I108=""),"",$I108-IF($J108="",0,$J108))</f>
@@ -6828,7 +6828,7 @@
         <v/>
       </c>
       <c r="J109" s="4" t="n">
-        <v>278.06</v>
+        <v>0</v>
       </c>
       <c r="K109" s="21">
         <f>IF(OR($B109="",$I109=""),"",$I109-IF($J109="",0,$J109))</f>
@@ -6879,7 +6879,7 @@
         <v/>
       </c>
       <c r="J110" s="4" t="n">
-        <v>437.6</v>
+        <v>97.34999999999999</v>
       </c>
       <c r="K110" s="21">
         <f>IF(OR($B110="",$I110=""),"",$I110-IF($J110="",0,$J110))</f>
@@ -6930,7 +6930,7 @@
         <v/>
       </c>
       <c r="J111" s="4" t="n">
-        <v>275.39</v>
+        <v>0</v>
       </c>
       <c r="K111" s="21">
         <f>IF(OR($B111="",$I111=""),"",$I111-IF($J111="",0,$J111))</f>
@@ -6981,7 +6981,7 @@
         <v/>
       </c>
       <c r="J112" s="4" t="n">
-        <v>382.63</v>
+        <v>91.06999999999999</v>
       </c>
       <c r="K112" s="21">
         <f>IF(OR($B112="",$I112=""),"",$I112-IF($J112="",0,$J112))</f>
@@ -7032,7 +7032,7 @@
         <v/>
       </c>
       <c r="J113" s="4" t="n">
-        <v>68.40000000000001</v>
+        <v>14.75</v>
       </c>
       <c r="K113" s="21">
         <f>IF(OR($B113="",$I113=""),"",$I113-IF($J113="",0,$J113))</f>
@@ -7083,7 +7083,7 @@
         <v/>
       </c>
       <c r="J114" s="4" t="n">
-        <v>126.99</v>
+        <v>0</v>
       </c>
       <c r="K114" s="21">
         <f>IF(OR($B114="",$I114=""),"",$I114-IF($J114="",0,$J114))</f>
@@ -7134,7 +7134,7 @@
         <v/>
       </c>
       <c r="J115" s="4" t="n">
-        <v>133.49</v>
+        <v>0</v>
       </c>
       <c r="K115" s="21">
         <f>IF(OR($B115="",$I115=""),"",$I115-IF($J115="",0,$J115))</f>
@@ -7185,7 +7185,7 @@
         <v/>
       </c>
       <c r="J116" s="4" t="n">
-        <v>394.21</v>
+        <v>87.77</v>
       </c>
       <c r="K116" s="21">
         <f>IF(OR($B116="",$I116=""),"",$I116-IF($J116="",0,$J116))</f>
@@ -7236,7 +7236,7 @@
         <v/>
       </c>
       <c r="J117" s="4" t="n">
-        <v>494.15</v>
+        <v>107.07</v>
       </c>
       <c r="K117" s="21">
         <f>IF(OR($B117="",$I117=""),"",$I117-IF($J117="",0,$J117))</f>
@@ -7287,7 +7287,7 @@
         <v/>
       </c>
       <c r="J118" s="4" t="n">
-        <v>145.41</v>
+        <v>14.75</v>
       </c>
       <c r="K118" s="21">
         <f>IF(OR($B118="",$I118=""),"",$I118-IF($J118="",0,$J118))</f>
@@ -7338,7 +7338,7 @@
         <v/>
       </c>
       <c r="J119" s="4" t="n">
-        <v>145.85</v>
+        <v>0</v>
       </c>
       <c r="K119" s="21">
         <f>IF(OR($B119="",$I119=""),"",$I119-IF($J119="",0,$J119))</f>
@@ -7389,7 +7389,7 @@
         <v/>
       </c>
       <c r="J120" s="4" t="n">
-        <v>391.31</v>
+        <v>86.84</v>
       </c>
       <c r="K120" s="21">
         <f>IF(OR($B120="",$I120=""),"",$I120-IF($J120="",0,$J120))</f>
@@ -7440,7 +7440,7 @@
         <v/>
       </c>
       <c r="J121" s="4" t="n">
-        <v>343.5</v>
+        <v>80.79000000000001</v>
       </c>
       <c r="K121" s="21">
         <f>IF(OR($B121="",$I121=""),"",$I121-IF($J121="",0,$J121))</f>
@@ -7491,7 +7491,7 @@
         <v/>
       </c>
       <c r="J122" s="4" t="n">
-        <v>243.77</v>
+        <v>0</v>
       </c>
       <c r="K122" s="21">
         <f>IF(OR($B122="",$I122=""),"",$I122-IF($J122="",0,$J122))</f>
@@ -7542,7 +7542,7 @@
         <v/>
       </c>
       <c r="J123" s="4" t="n">
-        <v>296.19</v>
+        <v>0</v>
       </c>
       <c r="K123" s="21">
         <f>IF(OR($B123="",$I123=""),"",$I123-IF($J123="",0,$J123))</f>
@@ -7593,7 +7593,7 @@
         <v/>
       </c>
       <c r="J124" s="4" t="n">
-        <v>139.07</v>
+        <v>0</v>
       </c>
       <c r="K124" s="21">
         <f>IF(OR($B124="",$I124=""),"",$I124-IF($J124="",0,$J124))</f>
@@ -7644,7 +7644,7 @@
         <v/>
       </c>
       <c r="J125" s="4" t="n">
-        <v>223.4</v>
+        <v>0</v>
       </c>
       <c r="K125" s="21">
         <f>IF(OR($B125="",$I125=""),"",$I125-IF($J125="",0,$J125))</f>
@@ -7695,7 +7695,7 @@
         <v/>
       </c>
       <c r="J126" s="4" t="n">
-        <v>442.09</v>
+        <v>0</v>
       </c>
       <c r="K126" s="21">
         <f>IF(OR($B126="",$I126=""),"",$I126-IF($J126="",0,$J126))</f>
@@ -7746,7 +7746,7 @@
         <v/>
       </c>
       <c r="J127" s="4" t="n">
-        <v>587.9400000000001</v>
+        <v>109.66</v>
       </c>
       <c r="K127" s="21">
         <f>IF(OR($B127="",$I127=""),"",$I127-IF($J127="",0,$J127))</f>
@@ -7797,7 +7797,7 @@
         <v/>
       </c>
       <c r="J128" s="4" t="n">
-        <v>143.17</v>
+        <v>0</v>
       </c>
       <c r="K128" s="21">
         <f>IF(OR($B128="",$I128=""),"",$I128-IF($J128="",0,$J128))</f>
@@ -7848,7 +7848,7 @@
         <v/>
       </c>
       <c r="J129" s="4" t="n">
-        <v>583.85</v>
+        <v>109.59</v>
       </c>
       <c r="K129" s="21">
         <f>IF(OR($B129="",$I129=""),"",$I129-IF($J129="",0,$J129))</f>
@@ -7899,7 +7899,7 @@
         <v/>
       </c>
       <c r="J130" s="4" t="n">
-        <v>218.38</v>
+        <v>0</v>
       </c>
       <c r="K130" s="21">
         <f>IF(OR($B130="",$I130=""),"",$I130-IF($J130="",0,$J130))</f>
@@ -7950,7 +7950,7 @@
         <v/>
       </c>
       <c r="J131" s="4" t="n">
-        <v>592.6900000000001</v>
+        <v>117.16</v>
       </c>
       <c r="K131" s="21">
         <f>IF(OR($B131="",$I131=""),"",$I131-IF($J131="",0,$J131))</f>
@@ -8001,7 +8001,7 @@
         <v/>
       </c>
       <c r="J132" s="4" t="n">
-        <v>276.97</v>
+        <v>0</v>
       </c>
       <c r="K132" s="21">
         <f>IF(OR($B132="",$I132=""),"",$I132-IF($J132="",0,$J132))</f>
@@ -8052,7 +8052,7 @@
         <v/>
       </c>
       <c r="J133" s="4" t="n">
-        <v>509.91</v>
+        <v>109.33</v>
       </c>
       <c r="K133" s="21">
         <f>IF(OR($B133="",$I133=""),"",$I133-IF($J133="",0,$J133))</f>
@@ -8103,7 +8103,7 @@
         <v/>
       </c>
       <c r="J134" s="4" t="n">
-        <v>578.39</v>
+        <v>108.78</v>
       </c>
       <c r="K134" s="21">
         <f>IF(OR($B134="",$I134=""),"",$I134-IF($J134="",0,$J134))</f>
@@ -8154,7 +8154,7 @@
         <v/>
       </c>
       <c r="J135" s="4" t="n">
-        <v>468.38</v>
+        <v>199.14</v>
       </c>
       <c r="K135" s="21">
         <f>IF(OR($B135="",$I135=""),"",$I135-IF($J135="",0,$J135))</f>
@@ -8205,7 +8205,7 @@
         <v/>
       </c>
       <c r="J136" s="4" t="n">
-        <v>149.82</v>
+        <v>14.75</v>
       </c>
       <c r="K136" s="21">
         <f>IF(OR($B136="",$I136=""),"",$I136-IF($J136="",0,$J136))</f>
@@ -8256,7 +8256,7 @@
         <v/>
       </c>
       <c r="J137" s="4" t="n">
-        <v>357.16</v>
+        <v>0</v>
       </c>
       <c r="K137" s="21">
         <f>IF(OR($B137="",$I137=""),"",$I137-IF($J137="",0,$J137))</f>
@@ -8307,7 +8307,7 @@
         <v/>
       </c>
       <c r="J138" s="4" t="n">
-        <v>465.39</v>
+        <v>197.77</v>
       </c>
       <c r="K138" s="21">
         <f>IF(OR($B138="",$I138=""),"",$I138-IF($J138="",0,$J138))</f>
@@ -8358,7 +8358,7 @@
         <v/>
       </c>
       <c r="J139" s="4" t="n">
-        <v>342.92</v>
+        <v>0</v>
       </c>
       <c r="K139" s="21">
         <f>IF(OR($B139="",$I139=""),"",$I139-IF($J139="",0,$J139))</f>
@@ -8409,7 +8409,7 @@
         <v/>
       </c>
       <c r="J140" s="4" t="n">
-        <v>473.31</v>
+        <v>205.28</v>
       </c>
       <c r="K140" s="21">
         <f>IF(OR($B140="",$I140=""),"",$I140-IF($J140="",0,$J140))</f>
@@ -8460,7 +8460,7 @@
         <v/>
       </c>
       <c r="J141" s="4" t="n">
-        <v>463.42</v>
+        <v>193.64</v>
       </c>
       <c r="K141" s="21">
         <f>IF(OR($B141="",$I141=""),"",$I141-IF($J141="",0,$J141))</f>
@@ -8511,7 +8511,7 @@
         <v/>
       </c>
       <c r="J142" s="4" t="n">
-        <v>442.78</v>
+        <v>173.91</v>
       </c>
       <c r="K142" s="21">
         <f>IF(OR($B142="",$I142=""),"",$I142-IF($J142="",0,$J142))</f>
@@ -8562,7 +8562,7 @@
         <v/>
       </c>
       <c r="J143" s="4" t="n">
-        <v>339.3</v>
+        <v>0</v>
       </c>
       <c r="K143" s="21">
         <f>IF(OR($B143="",$I143=""),"",$I143-IF($J143="",0,$J143))</f>
@@ -8613,7 +8613,7 @@
         <v/>
       </c>
       <c r="J144" s="4" t="n">
-        <v>148.71</v>
+        <v>14.75</v>
       </c>
       <c r="K144" s="21">
         <f>IF(OR($B144="",$I144=""),"",$I144-IF($J144="",0,$J144))</f>
@@ -8664,7 +8664,7 @@
         <v/>
       </c>
       <c r="J145" s="4" t="n">
-        <v>511.54</v>
+        <v>203.6</v>
       </c>
       <c r="K145" s="21">
         <f>IF(OR($B145="",$I145=""),"",$I145-IF($J145="",0,$J145))</f>
@@ -8715,7 +8715,7 @@
         <v/>
       </c>
       <c r="J146" s="4" t="n">
-        <v>421.14</v>
+        <v>0</v>
       </c>
       <c r="K146" s="21">
         <f>IF(OR($B146="",$I146=""),"",$I146-IF($J146="",0,$J146))</f>
@@ -8766,7 +8766,7 @@
         <v/>
       </c>
       <c r="J147" s="4" t="n">
-        <v>343.65</v>
+        <v>0</v>
       </c>
       <c r="K147" s="21">
         <f>IF(OR($B147="",$I147=""),"",$I147-IF($J147="",0,$J147))</f>
@@ -8817,7 +8817,7 @@
         <v/>
       </c>
       <c r="J148" s="4" t="n">
-        <v>257.03</v>
+        <v>0</v>
       </c>
       <c r="K148" s="21">
         <f>IF(OR($B148="",$I148=""),"",$I148-IF($J148="",0,$J148))</f>
@@ -8868,7 +8868,7 @@
         <v/>
       </c>
       <c r="J149" s="4" t="n">
-        <v>145.39</v>
+        <v>0</v>
       </c>
       <c r="K149" s="21">
         <f>IF(OR($B149="",$I149=""),"",$I149-IF($J149="",0,$J149))</f>
@@ -8919,7 +8919,7 @@
         <v/>
       </c>
       <c r="J150" s="4" t="n">
-        <v>270.28</v>
+        <v>0</v>
       </c>
       <c r="K150" s="21">
         <f>IF(OR($B150="",$I150=""),"",$I150-IF($J150="",0,$J150))</f>
@@ -8970,7 +8970,7 @@
         <v/>
       </c>
       <c r="J151" s="4" t="n">
-        <v>262.28</v>
+        <v>0</v>
       </c>
       <c r="K151" s="21">
         <f>IF(OR($B151="",$I151=""),"",$I151-IF($J151="",0,$J151))</f>
@@ -9021,7 +9021,7 @@
         <v/>
       </c>
       <c r="J152" s="4" t="n">
-        <v>276.22</v>
+        <v>0</v>
       </c>
       <c r="K152" s="21">
         <f>IF(OR($B152="",$I152=""),"",$I152-IF($J152="",0,$J152))</f>
@@ -9072,7 +9072,7 @@
         <v/>
       </c>
       <c r="J153" s="4" t="n">
-        <v>266.93</v>
+        <v>0</v>
       </c>
       <c r="K153" s="21">
         <f>IF(OR($B153="",$I153=""),"",$I153-IF($J153="",0,$J153))</f>
@@ -9123,7 +9123,7 @@
         <v/>
       </c>
       <c r="J154" s="4" t="n">
-        <v>140.35</v>
+        <v>0</v>
       </c>
       <c r="K154" s="21">
         <f>IF(OR($B154="",$I154=""),"",$I154-IF($J154="",0,$J154))</f>
@@ -9174,7 +9174,7 @@
         <v/>
       </c>
       <c r="J155" s="4" t="n">
-        <v>200.3</v>
+        <v>0</v>
       </c>
       <c r="K155" s="21">
         <f>IF(OR($B155="",$I155=""),"",$I155-IF($J155="",0,$J155))</f>
@@ -9225,7 +9225,7 @@
         <v/>
       </c>
       <c r="J156" s="4" t="n">
-        <v>435.16</v>
+        <v>81.05</v>
       </c>
       <c r="K156" s="21">
         <f>IF(OR($B156="",$I156=""),"",$I156-IF($J156="",0,$J156))</f>
@@ -9276,7 +9276,7 @@
         <v/>
       </c>
       <c r="J157" s="4" t="n">
-        <v>524.72</v>
+        <v>105.91</v>
       </c>
       <c r="K157" s="21">
         <f>IF(OR($B157="",$I157=""),"",$I157-IF($J157="",0,$J157))</f>
@@ -9327,7 +9327,7 @@
         <v/>
       </c>
       <c r="J158" s="4" t="n">
-        <v>519.0599999999999</v>
+        <v>101.6</v>
       </c>
       <c r="K158" s="21">
         <f>IF(OR($B158="",$I158=""),"",$I158-IF($J158="",0,$J158))</f>
@@ -9378,7 +9378,7 @@
         <v/>
       </c>
       <c r="J159" s="4" t="n">
-        <v>517.4400000000001</v>
+        <v>101.35</v>
       </c>
       <c r="K159" s="21">
         <f>IF(OR($B159="",$I159=""),"",$I159-IF($J159="",0,$J159))</f>
@@ -9429,7 +9429,7 @@
         <v/>
       </c>
       <c r="J160" s="4" t="n">
-        <v>445.64</v>
+        <v>92.8</v>
       </c>
       <c r="K160" s="21">
         <f>IF(OR($B160="",$I160=""),"",$I160-IF($J160="",0,$J160))</f>
@@ -9480,7 +9480,7 @@
         <v/>
       </c>
       <c r="J161" s="4" t="n">
-        <v>461.7</v>
+        <v>108.61</v>
       </c>
       <c r="K161" s="21">
         <f>IF(OR($B161="",$I161=""),"",$I161-IF($J161="",0,$J161))</f>
@@ -9531,7 +9531,7 @@
         <v/>
       </c>
       <c r="J162" s="4" t="n">
-        <v>365.55</v>
+        <v>0</v>
       </c>
       <c r="K162" s="21">
         <f>IF(OR($B162="",$I162=""),"",$I162-IF($J162="",0,$J162))</f>
@@ -9582,7 +9582,7 @@
         <v/>
       </c>
       <c r="J163" s="4" t="n">
-        <v>306.98</v>
+        <v>0</v>
       </c>
       <c r="K163" s="21">
         <f>IF(OR($B163="",$I163=""),"",$I163-IF($J163="",0,$J163))</f>
@@ -9633,7 +9633,7 @@
         <v/>
       </c>
       <c r="J164" s="4" t="n">
-        <v>302.7</v>
+        <v>0</v>
       </c>
       <c r="K164" s="21">
         <f>IF(OR($B164="",$I164=""),"",$I164-IF($J164="",0,$J164))</f>
@@ -9684,7 +9684,7 @@
         <v/>
       </c>
       <c r="J165" s="4" t="n">
-        <v>302.56</v>
+        <v>0</v>
       </c>
       <c r="K165" s="21">
         <f>IF(OR($B165="",$I165=""),"",$I165-IF($J165="",0,$J165))</f>
@@ -9735,7 +9735,7 @@
         <v/>
       </c>
       <c r="J166" s="4" t="n">
-        <v>367.56</v>
+        <v>0</v>
       </c>
       <c r="K166" s="21">
         <f>IF(OR($B166="",$I166=""),"",$I166-IF($J166="",0,$J166))</f>
@@ -9786,7 +9786,7 @@
         <v/>
       </c>
       <c r="J167" s="4" t="n">
-        <v>355.64</v>
+        <v>0</v>
       </c>
       <c r="K167" s="21">
         <f>IF(OR($B167="",$I167=""),"",$I167-IF($J167="",0,$J167))</f>
@@ -9837,7 +9837,7 @@
         <v/>
       </c>
       <c r="J168" s="4" t="n">
-        <v>626.4400000000001</v>
+        <v>116.08</v>
       </c>
       <c r="K168" s="21">
         <f>IF(OR($B168="",$I168=""),"",$I168-IF($J168="",0,$J168))</f>
@@ -9888,7 +9888,7 @@
         <v/>
       </c>
       <c r="J169" s="4" t="n">
-        <v>634.4299999999999</v>
+        <v>127.24</v>
       </c>
       <c r="K169" s="21">
         <f>IF(OR($B169="",$I169=""),"",$I169-IF($J169="",0,$J169))</f>
@@ -9939,7 +9939,7 @@
         <v/>
       </c>
       <c r="J170" s="4" t="n">
-        <v>258.56</v>
+        <v>14.75</v>
       </c>
       <c r="K170" s="21">
         <f>IF(OR($B170="",$I170=""),"",$I170-IF($J170="",0,$J170))</f>
@@ -9990,7 +9990,7 @@
         <v/>
       </c>
       <c r="J171" s="4" t="n">
-        <v>662.13</v>
+        <v>247.73</v>
       </c>
       <c r="K171" s="21">
         <f>IF(OR($B171="",$I171=""),"",$I171-IF($J171="",0,$J171))</f>
@@ -10041,7 +10041,7 @@
         <v/>
       </c>
       <c r="J172" s="4" t="n">
-        <v>647.29</v>
+        <v>234.09</v>
       </c>
       <c r="K172" s="21">
         <f>IF(OR($B172="",$I172=""),"",$I172-IF($J172="",0,$J172))</f>
@@ -10092,7 +10092,7 @@
         <v/>
       </c>
       <c r="J173" s="4" t="n">
-        <v>665.03</v>
+        <v>250.09</v>
       </c>
       <c r="K173" s="21">
         <f>IF(OR($B173="",$I173=""),"",$I173-IF($J173="",0,$J173))</f>
@@ -10143,7 +10143,7 @@
         <v/>
       </c>
       <c r="J174" s="4" t="n">
-        <v>548.39</v>
+        <v>0</v>
       </c>
       <c r="K174" s="21">
         <f>IF(OR($B174="",$I174=""),"",$I174-IF($J174="",0,$J174))</f>
@@ -10194,7 +10194,7 @@
         <v/>
       </c>
       <c r="J175" s="4" t="n">
-        <v>649.5</v>
+        <v>234.81</v>
       </c>
       <c r="K175" s="21">
         <f>IF(OR($B175="",$I175=""),"",$I175-IF($J175="",0,$J175))</f>
@@ -10245,7 +10245,7 @@
         <v/>
       </c>
       <c r="J176" s="4" t="n">
-        <v>550.84</v>
+        <v>0</v>
       </c>
       <c r="K176" s="21">
         <f>IF(OR($B176="",$I176=""),"",$I176-IF($J176="",0,$J176))</f>
@@ -10296,7 +10296,7 @@
         <v/>
       </c>
       <c r="J177" s="4" t="n">
-        <v>266.27</v>
+        <v>78.52</v>
       </c>
       <c r="K177" s="21">
         <f>IF(OR($B177="",$I177=""),"",$I177-IF($J177="",0,$J177))</f>
@@ -10347,7 +10347,7 @@
         <v/>
       </c>
       <c r="J178" s="4" t="n">
-        <v>185.64</v>
+        <v>0</v>
       </c>
       <c r="K178" s="21">
         <f>IF(OR($B178="",$I178=""),"",$I178-IF($J178="",0,$J178))</f>
@@ -10398,7 +10398,7 @@
         <v/>
       </c>
       <c r="J179" s="4" t="n">
-        <v>236.87</v>
+        <v>50.15</v>
       </c>
       <c r="K179" s="21">
         <f>IF(OR($B179="",$I179=""),"",$I179-IF($J179="",0,$J179))</f>
@@ -10449,7 +10449,7 @@
         <v/>
       </c>
       <c r="J180" s="4" t="n">
-        <v>271.55</v>
+        <v>79.23</v>
       </c>
       <c r="K180" s="21">
         <f>IF(OR($B180="",$I180=""),"",$I180-IF($J180="",0,$J180))</f>
@@ -10500,7 +10500,7 @@
         <v/>
       </c>
       <c r="J181" s="4" t="n">
-        <v>269.7</v>
+        <v>77.90000000000001</v>
       </c>
       <c r="K181" s="21">
         <f>IF(OR($B181="",$I181=""),"",$I181-IF($J181="",0,$J181))</f>
@@ -10551,7 +10551,7 @@
         <v/>
       </c>
       <c r="J182" s="4" t="n">
-        <v>152.88</v>
+        <v>60.41</v>
       </c>
       <c r="K182" s="21">
         <f>IF(OR($B182="",$I182=""),"",$I182-IF($J182="",0,$J182))</f>
@@ -10602,7 +10602,7 @@
         <v/>
       </c>
       <c r="J183" s="4" t="n">
-        <v>436.71</v>
+        <v>0</v>
       </c>
       <c r="K183" s="21">
         <f>IF(OR($B183="",$I183=""),"",$I183-IF($J183="",0,$J183))</f>
@@ -10653,7 +10653,7 @@
         <v/>
       </c>
       <c r="J184" s="4" t="n">
-        <v>434.19</v>
+        <v>0</v>
       </c>
       <c r="K184" s="21">
         <f>IF(OR($B184="",$I184=""),"",$I184-IF($J184="",0,$J184))</f>
@@ -10704,7 +10704,7 @@
         <v/>
       </c>
       <c r="J185" s="4" t="n">
-        <v>266.46</v>
+        <v>79.26000000000001</v>
       </c>
       <c r="K185" s="21">
         <f>IF(OR($B185="",$I185=""),"",$I185-IF($J185="",0,$J185))</f>
@@ -10755,7 +10755,7 @@
         <v/>
       </c>
       <c r="J186" s="4" t="n">
-        <v>447.15</v>
+        <v>0</v>
       </c>
       <c r="K186" s="21">
         <f>IF(OR($B186="",$I186=""),"",$I186-IF($J186="",0,$J186))</f>
@@ -10806,7 +10806,7 @@
         <v/>
       </c>
       <c r="J187" s="4" t="n">
-        <v>429.11</v>
+        <v>0</v>
       </c>
       <c r="K187" s="21">
         <f>IF(OR($B187="",$I187=""),"",$I187-IF($J187="",0,$J187))</f>
@@ -10897,14 +10897,18 @@
       <c r="F189" s="26" t="n">
         <v>315</v>
       </c>
-      <c r="G189" s="24" t="inlineStr"/>
-      <c r="H189" s="25" t="inlineStr"/>
+      <c r="G189" s="24" t="n">
+        <v>46288</v>
+      </c>
+      <c r="H189" s="25" t="n">
+        <v>775.9299999999999</v>
+      </c>
       <c r="I189" s="21">
         <f>IF(OR($B189="",$H189=""),"",IF($C189="LONG",($H189-$E189)*$F189,($E189-$H189)*$F189))</f>
         <v/>
       </c>
       <c r="J189" s="4" t="n">
-        <v>50.15</v>
+        <v>99.33</v>
       </c>
       <c r="K189" s="21">
         <f>IF(OR($B189="",$I189=""),"",$I189-IF($J189="",0,$J189))</f>
@@ -10944,14 +10948,18 @@
       <c r="F190" s="26" t="n">
         <v>1255</v>
       </c>
-      <c r="G190" s="24" t="inlineStr"/>
-      <c r="H190" s="25" t="inlineStr"/>
+      <c r="G190" s="24" t="n">
+        <v>46288</v>
+      </c>
+      <c r="H190" s="25" t="n">
+        <v>196.71</v>
+      </c>
       <c r="I190" s="21">
         <f>IF(OR($B190="",$H190=""),"",IF($C190="LONG",($H190-$E190)*$F190,($E190-$H190)*$F190))</f>
         <v/>
       </c>
       <c r="J190" s="4" t="n">
-        <v>50.15</v>
+        <v>104.63</v>
       </c>
       <c r="K190" s="21">
         <f>IF(OR($B190="",$I190=""),"",$I190-IF($J190="",0,$J190))</f>
@@ -11195,14 +11203,18 @@
       <c r="F195" s="26" t="n">
         <v>1482</v>
       </c>
-      <c r="G195" s="24" t="inlineStr"/>
-      <c r="H195" s="25" t="inlineStr"/>
+      <c r="G195" s="24" t="n">
+        <v>46288</v>
+      </c>
+      <c r="H195" s="25" t="n">
+        <v>170.47</v>
+      </c>
       <c r="I195" s="21">
         <f>IF(OR($B195="",$H195=""),"",IF($C195="LONG",($H195-$E195)*$F195,($E195-$H195)*$F195))</f>
         <v/>
       </c>
       <c r="J195" s="4" t="n">
-        <v>50.15</v>
+        <v>108.26</v>
       </c>
       <c r="K195" s="21">
         <f>IF(OR($B195="",$I195=""),"",$I195-IF($J195="",0,$J195))</f>
@@ -11242,14 +11254,18 @@
       <c r="F196" s="26" t="n">
         <v>403</v>
       </c>
-      <c r="G196" s="24" t="inlineStr"/>
-      <c r="H196" s="25" t="inlineStr"/>
+      <c r="G196" s="24" t="n">
+        <v>46288</v>
+      </c>
+      <c r="H196" s="25" t="n">
+        <v>607.61</v>
+      </c>
       <c r="I196" s="21">
         <f>IF(OR($B196="",$H196=""),"",IF($C196="LONG",($H196-$E196)*$F196,($E196-$H196)*$F196))</f>
         <v/>
       </c>
       <c r="J196" s="4" t="n">
-        <v>50.15</v>
+        <v>101.5</v>
       </c>
       <c r="K196" s="21">
         <f>IF(OR($B196="",$I196=""),"",$I196-IF($J196="",0,$J196))</f>
@@ -11340,14 +11356,18 @@
       <c r="F198" s="26" t="n">
         <v>715</v>
       </c>
-      <c r="G198" s="24" t="inlineStr"/>
-      <c r="H198" s="25" t="inlineStr"/>
+      <c r="G198" s="24" t="n">
+        <v>46288</v>
+      </c>
+      <c r="H198" s="25" t="n">
+        <v>357.47</v>
+      </c>
       <c r="I198" s="21">
         <f>IF(OR($B198="",$H198=""),"",IF($C198="LONG",($H198-$E198)*$F198,($E198-$H198)*$F198))</f>
         <v/>
       </c>
       <c r="J198" s="4" t="n">
-        <v>50.15</v>
+        <v>101.49</v>
       </c>
       <c r="K198" s="21">
         <f>IF(OR($B198="",$I198=""),"",$I198-IF($J198="",0,$J198))</f>
@@ -11387,14 +11407,18 @@
       <c r="F199" s="26" t="n">
         <v>183</v>
       </c>
-      <c r="G199" s="24" t="inlineStr"/>
-      <c r="H199" s="25" t="inlineStr"/>
+      <c r="G199" s="24" t="n">
+        <v>46288</v>
+      </c>
+      <c r="H199" s="25" t="n">
+        <v>1372.32</v>
+      </c>
       <c r="I199" s="21">
         <f>IF(OR($B199="",$H199=""),"",IF($C199="LONG",($H199-$E199)*$F199,($E199-$H199)*$F199))</f>
         <v/>
       </c>
       <c r="J199" s="4" t="n">
-        <v>50.15</v>
+        <v>104.5</v>
       </c>
       <c r="K199" s="21">
         <f>IF(OR($B199="",$I199=""),"",$I199-IF($J199="",0,$J199))</f>
@@ -11410,19 +11434,39 @@
       </c>
     </row>
     <row r="200">
-      <c r="A200" s="23" t="n"/>
-      <c r="B200" s="23" t="n"/>
-      <c r="C200" s="23" t="n"/>
-      <c r="D200" s="24" t="n"/>
-      <c r="E200" s="25" t="n"/>
-      <c r="F200" s="26" t="n"/>
-      <c r="G200" s="24" t="n"/>
-      <c r="H200" s="25" t="n"/>
+      <c r="A200" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-limit_entry_multi</t>
+        </is>
+      </c>
+      <c r="B200" s="23" t="inlineStr">
+        <is>
+          <t>ARVSMART</t>
+        </is>
+      </c>
+      <c r="C200" s="23" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="D200" s="24" t="n">
+        <v>46288</v>
+      </c>
+      <c r="E200" s="25" t="n">
+        <v>635.6889</v>
+      </c>
+      <c r="F200" s="26" t="n">
+        <v>262</v>
+      </c>
+      <c r="G200" s="24" t="inlineStr"/>
+      <c r="H200" s="25" t="inlineStr"/>
       <c r="I200" s="21">
         <f>IF(OR($B200="",$H200=""),"",IF($C200="LONG",($H200-$E200)*$F200,($E200-$H200)*$F200))</f>
         <v/>
       </c>
-      <c r="J200" s="4" t="n"/>
+      <c r="J200" s="4" t="n">
+        <v>50.15</v>
+      </c>
       <c r="K200" s="21">
         <f>IF(OR($B200="",$I200=""),"",$I200-IF($J200="",0,$J200))</f>
         <v/>
@@ -11437,19 +11481,43 @@
       </c>
     </row>
     <row r="201">
-      <c r="A201" s="23" t="n"/>
-      <c r="B201" s="23" t="n"/>
-      <c r="C201" s="23" t="n"/>
-      <c r="D201" s="24" t="n"/>
-      <c r="E201" s="25" t="n"/>
-      <c r="F201" s="26" t="n"/>
-      <c r="G201" s="24" t="n"/>
-      <c r="H201" s="25" t="n"/>
+      <c r="A201" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-221260923445309</t>
+        </is>
+      </c>
+      <c r="B201" s="23" t="inlineStr">
+        <is>
+          <t>ASTEC</t>
+        </is>
+      </c>
+      <c r="C201" s="23" t="inlineStr">
+        <is>
+          <t>SHORT</t>
+        </is>
+      </c>
+      <c r="D201" s="24" t="n">
+        <v>46288</v>
+      </c>
+      <c r="E201" s="25" t="n">
+        <v>775.25</v>
+      </c>
+      <c r="F201" s="26" t="n">
+        <v>315</v>
+      </c>
+      <c r="G201" s="24" t="n">
+        <v>46288</v>
+      </c>
+      <c r="H201" s="25" t="n">
+        <v>764.5</v>
+      </c>
       <c r="I201" s="21">
         <f>IF(OR($B201="",$H201=""),"",IF($C201="LONG",($H201-$E201)*$F201,($E201-$H201)*$F201))</f>
         <v/>
       </c>
-      <c r="J201" s="4" t="n"/>
+      <c r="J201" s="4" t="n">
+        <v>0</v>
+      </c>
       <c r="K201" s="21">
         <f>IF(OR($B201="",$I201=""),"",$I201-IF($J201="",0,$J201))</f>
         <v/>
@@ -11464,19 +11532,43 @@
       </c>
     </row>
     <row r="202">
-      <c r="A202" s="23" t="n"/>
-      <c r="B202" s="23" t="n"/>
-      <c r="C202" s="23" t="n"/>
-      <c r="D202" s="24" t="n"/>
-      <c r="E202" s="25" t="n"/>
-      <c r="F202" s="26" t="n"/>
-      <c r="G202" s="24" t="n"/>
-      <c r="H202" s="25" t="n"/>
+      <c r="A202" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-34126092354709</t>
+        </is>
+      </c>
+      <c r="B202" s="23" t="inlineStr">
+        <is>
+          <t>CHEMPLASTS</t>
+        </is>
+      </c>
+      <c r="C202" s="23" t="inlineStr">
+        <is>
+          <t>SHORT</t>
+        </is>
+      </c>
+      <c r="D202" s="24" t="n">
+        <v>46288</v>
+      </c>
+      <c r="E202" s="25" t="n">
+        <v>196.53</v>
+      </c>
+      <c r="F202" s="26" t="n">
+        <v>1255</v>
+      </c>
+      <c r="G202" s="24" t="n">
+        <v>46288</v>
+      </c>
+      <c r="H202" s="25" t="n">
+        <v>199.17</v>
+      </c>
       <c r="I202" s="21">
         <f>IF(OR($B202="",$H202=""),"",IF($C202="LONG",($H202-$E202)*$F202,($E202-$H202)*$F202))</f>
         <v/>
       </c>
-      <c r="J202" s="4" t="n"/>
+      <c r="J202" s="4" t="n">
+        <v>0</v>
+      </c>
       <c r="K202" s="21">
         <f>IF(OR($B202="",$I202=""),"",$I202-IF($J202="",0,$J202))</f>
         <v/>
@@ -11491,19 +11583,39 @@
       </c>
     </row>
     <row r="203">
-      <c r="A203" s="23" t="n"/>
-      <c r="B203" s="23" t="n"/>
-      <c r="C203" s="23" t="n"/>
-      <c r="D203" s="24" t="n"/>
-      <c r="E203" s="25" t="n"/>
-      <c r="F203" s="26" t="n"/>
-      <c r="G203" s="24" t="n"/>
-      <c r="H203" s="25" t="n"/>
+      <c r="A203" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-limit_entry_multi</t>
+        </is>
+      </c>
+      <c r="B203" s="23" t="inlineStr">
+        <is>
+          <t>DELTACORP</t>
+        </is>
+      </c>
+      <c r="C203" s="23" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="D203" s="24" t="n">
+        <v>46288</v>
+      </c>
+      <c r="E203" s="25" t="n">
+        <v>68.7423</v>
+      </c>
+      <c r="F203" s="26" t="n">
+        <v>2426</v>
+      </c>
+      <c r="G203" s="24" t="inlineStr"/>
+      <c r="H203" s="25" t="inlineStr"/>
       <c r="I203" s="21">
         <f>IF(OR($B203="",$H203=""),"",IF($C203="LONG",($H203-$E203)*$F203,($E203-$H203)*$F203))</f>
         <v/>
       </c>
-      <c r="J203" s="4" t="n"/>
+      <c r="J203" s="4" t="n">
+        <v>50.15</v>
+      </c>
       <c r="K203" s="21">
         <f>IF(OR($B203="",$I203=""),"",$I203-IF($J203="",0,$J203))</f>
         <v/>
@@ -11518,19 +11630,39 @@
       </c>
     </row>
     <row r="204">
-      <c r="A204" s="23" t="n"/>
-      <c r="B204" s="23" t="n"/>
-      <c r="C204" s="23" t="n"/>
-      <c r="D204" s="24" t="n"/>
-      <c r="E204" s="25" t="n"/>
-      <c r="F204" s="26" t="n"/>
-      <c r="G204" s="24" t="n"/>
-      <c r="H204" s="25" t="n"/>
+      <c r="A204" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-limit_entry_multi</t>
+        </is>
+      </c>
+      <c r="B204" s="23" t="inlineStr">
+        <is>
+          <t>GNA</t>
+        </is>
+      </c>
+      <c r="C204" s="23" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="D204" s="24" t="n">
+        <v>46288</v>
+      </c>
+      <c r="E204" s="25" t="n">
+        <v>596.2712</v>
+      </c>
+      <c r="F204" s="26" t="n">
+        <v>139</v>
+      </c>
+      <c r="G204" s="24" t="inlineStr"/>
+      <c r="H204" s="25" t="inlineStr"/>
       <c r="I204" s="21">
         <f>IF(OR($B204="",$H204=""),"",IF($C204="LONG",($H204-$E204)*$F204,($E204-$H204)*$F204))</f>
         <v/>
       </c>
-      <c r="J204" s="4" t="n"/>
+      <c r="J204" s="4" t="n">
+        <v>14.75</v>
+      </c>
       <c r="K204" s="21">
         <f>IF(OR($B204="",$I204=""),"",$I204-IF($J204="",0,$J204))</f>
         <v/>
@@ -11545,19 +11677,39 @@
       </c>
     </row>
     <row r="205">
-      <c r="A205" s="23" t="n"/>
-      <c r="B205" s="23" t="n"/>
-      <c r="C205" s="23" t="n"/>
-      <c r="D205" s="24" t="n"/>
-      <c r="E205" s="25" t="n"/>
-      <c r="F205" s="26" t="n"/>
-      <c r="G205" s="24" t="n"/>
-      <c r="H205" s="25" t="n"/>
+      <c r="A205" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-limit_entry_multi</t>
+        </is>
+      </c>
+      <c r="B205" s="23" t="inlineStr">
+        <is>
+          <t>JAYKAY</t>
+        </is>
+      </c>
+      <c r="C205" s="23" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="D205" s="24" t="n">
+        <v>46288</v>
+      </c>
+      <c r="E205" s="25" t="n">
+        <v>212.4728</v>
+      </c>
+      <c r="F205" s="26" t="n">
+        <v>780</v>
+      </c>
+      <c r="G205" s="24" t="inlineStr"/>
+      <c r="H205" s="25" t="inlineStr"/>
       <c r="I205" s="21">
         <f>IF(OR($B205="",$H205=""),"",IF($C205="LONG",($H205-$E205)*$F205,($E205-$H205)*$F205))</f>
         <v/>
       </c>
-      <c r="J205" s="4" t="n"/>
+      <c r="J205" s="4" t="n">
+        <v>50.15</v>
+      </c>
       <c r="K205" s="21">
         <f>IF(OR($B205="",$I205=""),"",$I205-IF($J205="",0,$J205))</f>
         <v/>
@@ -11572,19 +11724,39 @@
       </c>
     </row>
     <row r="206">
-      <c r="A206" s="23" t="n"/>
-      <c r="B206" s="23" t="n"/>
-      <c r="C206" s="23" t="n"/>
-      <c r="D206" s="24" t="n"/>
-      <c r="E206" s="25" t="n"/>
-      <c r="F206" s="26" t="n"/>
-      <c r="G206" s="24" t="n"/>
-      <c r="H206" s="25" t="n"/>
+      <c r="A206" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-23126092396409</t>
+        </is>
+      </c>
+      <c r="B206" s="23" t="inlineStr">
+        <is>
+          <t>KROSS</t>
+        </is>
+      </c>
+      <c r="C206" s="23" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="D206" s="24" t="n">
+        <v>46288</v>
+      </c>
+      <c r="E206" s="25" t="n">
+        <v>278.5987</v>
+      </c>
+      <c r="F206" s="26" t="n">
+        <v>597</v>
+      </c>
+      <c r="G206" s="24" t="inlineStr"/>
+      <c r="H206" s="25" t="inlineStr"/>
       <c r="I206" s="21">
         <f>IF(OR($B206="",$H206=""),"",IF($C206="LONG",($H206-$E206)*$F206,($E206-$H206)*$F206))</f>
         <v/>
       </c>
-      <c r="J206" s="4" t="n"/>
+      <c r="J206" s="4" t="n">
+        <v>50.15</v>
+      </c>
       <c r="K206" s="21">
         <f>IF(OR($B206="",$I206=""),"",$I206-IF($J206="",0,$J206))</f>
         <v/>
@@ -11599,19 +11771,39 @@
       </c>
     </row>
     <row r="207">
-      <c r="A207" s="23" t="n"/>
-      <c r="B207" s="23" t="n"/>
-      <c r="C207" s="23" t="n"/>
-      <c r="D207" s="24" t="n"/>
-      <c r="E207" s="25" t="n"/>
-      <c r="F207" s="26" t="n"/>
-      <c r="G207" s="24" t="n"/>
-      <c r="H207" s="25" t="n"/>
+      <c r="A207" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-221260923710209</t>
+        </is>
+      </c>
+      <c r="B207" s="23" t="inlineStr">
+        <is>
+          <t>MUKANDLTD</t>
+        </is>
+      </c>
+      <c r="C207" s="23" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="D207" s="24" t="n">
+        <v>46288</v>
+      </c>
+      <c r="E207" s="25" t="n">
+        <v>156.9292</v>
+      </c>
+      <c r="F207" s="26" t="n">
+        <v>1059</v>
+      </c>
+      <c r="G207" s="24" t="inlineStr"/>
+      <c r="H207" s="25" t="inlineStr"/>
       <c r="I207" s="21">
         <f>IF(OR($B207="",$H207=""),"",IF($C207="LONG",($H207-$E207)*$F207,($E207-$H207)*$F207))</f>
         <v/>
       </c>
-      <c r="J207" s="4" t="n"/>
+      <c r="J207" s="4" t="n">
+        <v>50.15</v>
+      </c>
       <c r="K207" s="21">
         <f>IF(OR($B207="",$I207=""),"",$I207-IF($J207="",0,$J207))</f>
         <v/>
@@ -11626,19 +11818,39 @@
       </c>
     </row>
     <row r="208">
-      <c r="A208" s="23" t="n"/>
-      <c r="B208" s="23" t="n"/>
-      <c r="C208" s="23" t="n"/>
-      <c r="D208" s="24" t="n"/>
-      <c r="E208" s="25" t="n"/>
-      <c r="F208" s="26" t="n"/>
-      <c r="G208" s="24" t="n"/>
-      <c r="H208" s="25" t="n"/>
+      <c r="A208" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-34126092398809</t>
+        </is>
+      </c>
+      <c r="B208" s="23" t="inlineStr">
+        <is>
+          <t>ONEPOINT</t>
+        </is>
+      </c>
+      <c r="C208" s="23" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="D208" s="24" t="n">
+        <v>46288</v>
+      </c>
+      <c r="E208" s="25" t="n">
+        <v>68.3674</v>
+      </c>
+      <c r="F208" s="26" t="n">
+        <v>2439</v>
+      </c>
+      <c r="G208" s="24" t="inlineStr"/>
+      <c r="H208" s="25" t="inlineStr"/>
       <c r="I208" s="21">
         <f>IF(OR($B208="",$H208=""),"",IF($C208="LONG",($H208-$E208)*$F208,($E208-$H208)*$F208))</f>
         <v/>
       </c>
-      <c r="J208" s="4" t="n"/>
+      <c r="J208" s="4" t="n">
+        <v>50.15</v>
+      </c>
       <c r="K208" s="21">
         <f>IF(OR($B208="",$I208=""),"",$I208-IF($J208="",0,$J208))</f>
         <v/>
@@ -11653,19 +11865,43 @@
       </c>
     </row>
     <row r="209">
-      <c r="A209" s="23" t="n"/>
-      <c r="B209" s="23" t="n"/>
-      <c r="C209" s="23" t="n"/>
-      <c r="D209" s="24" t="n"/>
-      <c r="E209" s="25" t="n"/>
-      <c r="F209" s="26" t="n"/>
-      <c r="G209" s="24" t="n"/>
-      <c r="H209" s="25" t="n"/>
+      <c r="A209" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-22126092353109</t>
+        </is>
+      </c>
+      <c r="B209" s="23" t="inlineStr">
+        <is>
+          <t>PACEDIGITK</t>
+        </is>
+      </c>
+      <c r="C209" s="23" t="inlineStr">
+        <is>
+          <t>SHORT</t>
+        </is>
+      </c>
+      <c r="D209" s="24" t="n">
+        <v>46288</v>
+      </c>
+      <c r="E209" s="25" t="n">
+        <v>170.48</v>
+      </c>
+      <c r="F209" s="26" t="n">
+        <v>1482</v>
+      </c>
+      <c r="G209" s="24" t="n">
+        <v>46288</v>
+      </c>
+      <c r="H209" s="25" t="n">
+        <v>169.7</v>
+      </c>
       <c r="I209" s="21">
         <f>IF(OR($B209="",$H209=""),"",IF($C209="LONG",($H209-$E209)*$F209,($E209-$H209)*$F209))</f>
         <v/>
       </c>
-      <c r="J209" s="4" t="n"/>
+      <c r="J209" s="4" t="n">
+        <v>0</v>
+      </c>
       <c r="K209" s="21">
         <f>IF(OR($B209="",$I209=""),"",$I209-IF($J209="",0,$J209))</f>
         <v/>
@@ -11680,19 +11916,43 @@
       </c>
     </row>
     <row r="210">
-      <c r="A210" s="23" t="n"/>
-      <c r="B210" s="23" t="n"/>
-      <c r="C210" s="23" t="n"/>
-      <c r="D210" s="24" t="n"/>
-      <c r="E210" s="25" t="n"/>
-      <c r="F210" s="26" t="n"/>
-      <c r="G210" s="24" t="n"/>
-      <c r="H210" s="25" t="n"/>
+      <c r="A210" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-321260923455309</t>
+        </is>
+      </c>
+      <c r="B210" s="23" t="inlineStr">
+        <is>
+          <t>PROTEAN</t>
+        </is>
+      </c>
+      <c r="C210" s="23" t="inlineStr">
+        <is>
+          <t>SHORT</t>
+        </is>
+      </c>
+      <c r="D210" s="24" t="n">
+        <v>46288</v>
+      </c>
+      <c r="E210" s="25" t="n">
+        <v>607.0599999999999</v>
+      </c>
+      <c r="F210" s="26" t="n">
+        <v>403</v>
+      </c>
+      <c r="G210" s="24" t="n">
+        <v>46288</v>
+      </c>
+      <c r="H210" s="25" t="n">
+        <v>633.91</v>
+      </c>
       <c r="I210" s="21">
         <f>IF(OR($B210="",$H210=""),"",IF($C210="LONG",($H210-$E210)*$F210,($E210-$H210)*$F210))</f>
         <v/>
       </c>
-      <c r="J210" s="4" t="n"/>
+      <c r="J210" s="4" t="n">
+        <v>0</v>
+      </c>
       <c r="K210" s="21">
         <f>IF(OR($B210="",$I210=""),"",$I210-IF($J210="",0,$J210))</f>
         <v/>
@@ -11707,19 +11967,39 @@
       </c>
     </row>
     <row r="211">
-      <c r="A211" s="23" t="n"/>
-      <c r="B211" s="23" t="n"/>
-      <c r="C211" s="23" t="n"/>
-      <c r="D211" s="24" t="n"/>
-      <c r="E211" s="25" t="n"/>
-      <c r="F211" s="26" t="n"/>
-      <c r="G211" s="24" t="n"/>
-      <c r="H211" s="25" t="n"/>
+      <c r="A211" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-221260923710309</t>
+        </is>
+      </c>
+      <c r="B211" s="23" t="inlineStr">
+        <is>
+          <t>RAYMONDREL</t>
+        </is>
+      </c>
+      <c r="C211" s="23" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="D211" s="24" t="n">
+        <v>46288</v>
+      </c>
+      <c r="E211" s="25" t="n">
+        <v>669.9376</v>
+      </c>
+      <c r="F211" s="26" t="n">
+        <v>246</v>
+      </c>
+      <c r="G211" s="24" t="inlineStr"/>
+      <c r="H211" s="25" t="inlineStr"/>
       <c r="I211" s="21">
         <f>IF(OR($B211="",$H211=""),"",IF($C211="LONG",($H211-$E211)*$F211,($E211-$H211)*$F211))</f>
         <v/>
       </c>
-      <c r="J211" s="4" t="n"/>
+      <c r="J211" s="4" t="n">
+        <v>50.15</v>
+      </c>
       <c r="K211" s="21">
         <f>IF(OR($B211="",$I211=""),"",$I211-IF($J211="",0,$J211))</f>
         <v/>
@@ -11734,19 +12014,39 @@
       </c>
     </row>
     <row r="212">
-      <c r="A212" s="23" t="n"/>
-      <c r="B212" s="23" t="n"/>
-      <c r="C212" s="23" t="n"/>
-      <c r="D212" s="24" t="n"/>
-      <c r="E212" s="25" t="n"/>
-      <c r="F212" s="26" t="n"/>
-      <c r="G212" s="24" t="n"/>
-      <c r="H212" s="25" t="n"/>
+      <c r="A212" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-34126092398909</t>
+        </is>
+      </c>
+      <c r="B212" s="23" t="inlineStr">
+        <is>
+          <t>RPGLIFE</t>
+        </is>
+      </c>
+      <c r="C212" s="23" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="D212" s="24" t="n">
+        <v>46288</v>
+      </c>
+      <c r="E212" s="25" t="n">
+        <v>3034.4072</v>
+      </c>
+      <c r="F212" s="26" t="n">
+        <v>55</v>
+      </c>
+      <c r="G212" s="24" t="inlineStr"/>
+      <c r="H212" s="25" t="inlineStr"/>
       <c r="I212" s="21">
         <f>IF(OR($B212="",$H212=""),"",IF($C212="LONG",($H212-$E212)*$F212,($E212-$H212)*$F212))</f>
         <v/>
       </c>
-      <c r="J212" s="4" t="n"/>
+      <c r="J212" s="4" t="n">
+        <v>50.15</v>
+      </c>
       <c r="K212" s="21">
         <f>IF(OR($B212="",$I212=""),"",$I212-IF($J212="",0,$J212))</f>
         <v/>
@@ -11761,19 +12061,43 @@
       </c>
     </row>
     <row r="213">
-      <c r="A213" s="23" t="n"/>
-      <c r="B213" s="23" t="n"/>
-      <c r="C213" s="23" t="n"/>
-      <c r="D213" s="24" t="n"/>
-      <c r="E213" s="25" t="n"/>
-      <c r="F213" s="26" t="n"/>
-      <c r="G213" s="24" t="n"/>
-      <c r="H213" s="25" t="n"/>
+      <c r="A213" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-23126092351809</t>
+        </is>
+      </c>
+      <c r="B213" s="23" t="inlineStr">
+        <is>
+          <t>STEELCAS</t>
+        </is>
+      </c>
+      <c r="C213" s="23" t="inlineStr">
+        <is>
+          <t>SHORT</t>
+        </is>
+      </c>
+      <c r="D213" s="24" t="n">
+        <v>46288</v>
+      </c>
+      <c r="E213" s="25" t="n">
+        <v>356.89</v>
+      </c>
+      <c r="F213" s="26" t="n">
+        <v>715</v>
+      </c>
+      <c r="G213" s="24" t="n">
+        <v>46288</v>
+      </c>
+      <c r="H213" s="25" t="n">
+        <v>356.99</v>
+      </c>
       <c r="I213" s="21">
         <f>IF(OR($B213="",$H213=""),"",IF($C213="LONG",($H213-$E213)*$F213,($E213-$H213)*$F213))</f>
         <v/>
       </c>
-      <c r="J213" s="4" t="n"/>
+      <c r="J213" s="4" t="n">
+        <v>0</v>
+      </c>
       <c r="K213" s="21">
         <f>IF(OR($B213="",$I213=""),"",$I213-IF($J213="",0,$J213))</f>
         <v/>
@@ -11788,19 +12112,43 @@
       </c>
     </row>
     <row r="214">
-      <c r="A214" s="23" t="n"/>
-      <c r="B214" s="23" t="n"/>
-      <c r="C214" s="23" t="n"/>
-      <c r="D214" s="24" t="n"/>
-      <c r="E214" s="25" t="n"/>
-      <c r="F214" s="26" t="n"/>
-      <c r="G214" s="24" t="n"/>
-      <c r="H214" s="25" t="n"/>
+      <c r="A214" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-23126092351709</t>
+        </is>
+      </c>
+      <c r="B214" s="23" t="inlineStr">
+        <is>
+          <t>ZOTA</t>
+        </is>
+      </c>
+      <c r="C214" s="23" t="inlineStr">
+        <is>
+          <t>SHORT</t>
+        </is>
+      </c>
+      <c r="D214" s="24" t="n">
+        <v>46288</v>
+      </c>
+      <c r="E214" s="25" t="n">
+        <v>1372.09</v>
+      </c>
+      <c r="F214" s="26" t="n">
+        <v>183</v>
+      </c>
+      <c r="G214" s="24" t="n">
+        <v>46288</v>
+      </c>
+      <c r="H214" s="25" t="n">
+        <v>1392.4</v>
+      </c>
       <c r="I214" s="21">
         <f>IF(OR($B214="",$H214=""),"",IF($C214="LONG",($H214-$E214)*$F214,($E214-$H214)*$F214))</f>
         <v/>
       </c>
-      <c r="J214" s="4" t="n"/>
+      <c r="J214" s="4" t="n">
+        <v>0</v>
+      </c>
       <c r="K214" s="21">
         <f>IF(OR($B214="",$I214=""),"",$I214-IF($J214="",0,$J214))</f>
         <v/>
@@ -33548,7 +33896,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J96"/>
+  <dimension ref="A1:J103"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -33718,7 +34066,7 @@
     <row r="6">
       <c r="A6" s="27" t="inlineStr">
         <is>
-          <t>ASHIANA</t>
+          <t>ARVSMART</t>
         </is>
       </c>
       <c r="B6" s="20">
@@ -33761,7 +34109,7 @@
     <row r="7">
       <c r="A7" s="27" t="inlineStr">
         <is>
-          <t>ASHOKA</t>
+          <t>ASHIANA</t>
         </is>
       </c>
       <c r="B7" s="20">
@@ -33804,7 +34152,7 @@
     <row r="8">
       <c r="A8" s="27" t="inlineStr">
         <is>
-          <t>ASTEC</t>
+          <t>ASHOKA</t>
         </is>
       </c>
       <c r="B8" s="20">
@@ -33847,7 +34195,7 @@
     <row r="9">
       <c r="A9" s="27" t="inlineStr">
         <is>
-          <t>AWFIS</t>
+          <t>ASTEC</t>
         </is>
       </c>
       <c r="B9" s="20">
@@ -33890,7 +34238,7 @@
     <row r="10">
       <c r="A10" s="27" t="inlineStr">
         <is>
-          <t>BAJAJHIND</t>
+          <t>AWFIS</t>
         </is>
       </c>
       <c r="B10" s="20">
@@ -33933,7 +34281,7 @@
     <row r="11">
       <c r="A11" s="27" t="inlineStr">
         <is>
-          <t>BANARISUG</t>
+          <t>BAJAJHIND</t>
         </is>
       </c>
       <c r="B11" s="20">
@@ -33976,7 +34324,7 @@
     <row r="12">
       <c r="A12" s="27" t="inlineStr">
         <is>
-          <t>BCG</t>
+          <t>BANARISUG</t>
         </is>
       </c>
       <c r="B12" s="20">
@@ -34019,7 +34367,7 @@
     <row r="13">
       <c r="A13" s="27" t="inlineStr">
         <is>
-          <t>BFUTILITIE</t>
+          <t>BCG</t>
         </is>
       </c>
       <c r="B13" s="20">
@@ -34062,7 +34410,7 @@
     <row r="14">
       <c r="A14" s="27" t="inlineStr">
         <is>
-          <t>BOMDYEING</t>
+          <t>BFUTILITIE</t>
         </is>
       </c>
       <c r="B14" s="20">
@@ -34105,7 +34453,7 @@
     <row r="15">
       <c r="A15" s="27" t="inlineStr">
         <is>
-          <t>CHEMPLASTS</t>
+          <t>BOMDYEING</t>
         </is>
       </c>
       <c r="B15" s="20">
@@ -34148,7 +34496,7 @@
     <row r="16">
       <c r="A16" s="27" t="inlineStr">
         <is>
-          <t>EIEL</t>
+          <t>CHEMPLASTS</t>
         </is>
       </c>
       <c r="B16" s="20">
@@ -34191,7 +34539,7 @@
     <row r="17">
       <c r="A17" s="27" t="inlineStr">
         <is>
-          <t>EMUDHRA</t>
+          <t>DELTACORP</t>
         </is>
       </c>
       <c r="B17" s="20">
@@ -34234,7 +34582,7 @@
     <row r="18">
       <c r="A18" s="27" t="inlineStr">
         <is>
-          <t>FILATEX</t>
+          <t>EIEL</t>
         </is>
       </c>
       <c r="B18" s="20">
@@ -34277,7 +34625,7 @@
     <row r="19">
       <c r="A19" s="27" t="inlineStr">
         <is>
-          <t>FMGOETZE</t>
+          <t>EMUDHRA</t>
         </is>
       </c>
       <c r="B19" s="20">
@@ -34320,7 +34668,7 @@
     <row r="20">
       <c r="A20" s="27" t="inlineStr">
         <is>
-          <t>FOSECOIND</t>
+          <t>FILATEX</t>
         </is>
       </c>
       <c r="B20" s="20">
@@ -34363,7 +34711,7 @@
     <row r="21">
       <c r="A21" s="27" t="inlineStr">
         <is>
-          <t>GKENERGY</t>
+          <t>FMGOETZE</t>
         </is>
       </c>
       <c r="B21" s="20">
@@ -34406,7 +34754,7 @@
     <row r="22">
       <c r="A22" s="27" t="inlineStr">
         <is>
-          <t>GNRL</t>
+          <t>FOSECOIND</t>
         </is>
       </c>
       <c r="B22" s="20">
@@ -34449,7 +34797,7 @@
     <row r="23">
       <c r="A23" s="27" t="inlineStr">
         <is>
-          <t>GOCLCORP</t>
+          <t>GKENERGY</t>
         </is>
       </c>
       <c r="B23" s="20">
@@ -34492,7 +34840,7 @@
     <row r="24">
       <c r="A24" s="27" t="inlineStr">
         <is>
-          <t>GOPAL</t>
+          <t>GNA</t>
         </is>
       </c>
       <c r="B24" s="20">
@@ -34535,7 +34883,7 @@
     <row r="25">
       <c r="A25" s="27" t="inlineStr">
         <is>
-          <t>GRAUWEIL</t>
+          <t>GNRL</t>
         </is>
       </c>
       <c r="B25" s="20">
@@ -34578,7 +34926,7 @@
     <row r="26">
       <c r="A26" s="27" t="inlineStr">
         <is>
-          <t>GUJTHEM</t>
+          <t>GOCLCORP</t>
         </is>
       </c>
       <c r="B26" s="20">
@@ -34621,7 +34969,7 @@
     <row r="27">
       <c r="A27" s="27" t="inlineStr">
         <is>
-          <t>HERITGFOOD</t>
+          <t>GOPAL</t>
         </is>
       </c>
       <c r="B27" s="20">
@@ -34664,7 +35012,7 @@
     <row r="28">
       <c r="A28" s="27" t="inlineStr">
         <is>
-          <t>HIKAL</t>
+          <t>GRAUWEIL</t>
         </is>
       </c>
       <c r="B28" s="20">
@@ -34707,7 +35055,7 @@
     <row r="29">
       <c r="A29" s="27" t="inlineStr">
         <is>
-          <t>HINDOILEXP</t>
+          <t>GUJTHEM</t>
         </is>
       </c>
       <c r="B29" s="20">
@@ -34750,7 +35098,7 @@
     <row r="30">
       <c r="A30" s="27" t="inlineStr">
         <is>
-          <t>HUBTOWN</t>
+          <t>HERITGFOOD</t>
         </is>
       </c>
       <c r="B30" s="20">
@@ -34793,7 +35141,7 @@
     <row r="31">
       <c r="A31" s="27" t="inlineStr">
         <is>
-          <t>INDNIPPON</t>
+          <t>HIKAL</t>
         </is>
       </c>
       <c r="B31" s="20">
@@ -34836,7 +35184,7 @@
     <row r="32">
       <c r="A32" s="27" t="inlineStr">
         <is>
-          <t>INDOCO</t>
+          <t>HINDOILEXP</t>
         </is>
       </c>
       <c r="B32" s="20">
@@ -34879,7 +35227,7 @@
     <row r="33">
       <c r="A33" s="27" t="inlineStr">
         <is>
-          <t>INDORAMA</t>
+          <t>HUBTOWN</t>
         </is>
       </c>
       <c r="B33" s="20">
@@ -34922,7 +35270,7 @@
     <row r="34">
       <c r="A34" s="27" t="inlineStr">
         <is>
-          <t>IPL</t>
+          <t>INDNIPPON</t>
         </is>
       </c>
       <c r="B34" s="20">
@@ -34965,7 +35313,7 @@
     <row r="35">
       <c r="A35" s="27" t="inlineStr">
         <is>
-          <t>JASH</t>
+          <t>INDOCO</t>
         </is>
       </c>
       <c r="B35" s="20">
@@ -35008,7 +35356,7 @@
     <row r="36">
       <c r="A36" s="27" t="inlineStr">
         <is>
-          <t>JAYKAY</t>
+          <t>INDORAMA</t>
         </is>
       </c>
       <c r="B36" s="20">
@@ -35051,7 +35399,7 @@
     <row r="37">
       <c r="A37" s="27" t="inlineStr">
         <is>
-          <t>JGCHEM</t>
+          <t>IPL</t>
         </is>
       </c>
       <c r="B37" s="20">
@@ -35094,7 +35442,7 @@
     <row r="38">
       <c r="A38" s="27" t="inlineStr">
         <is>
-          <t>KCP</t>
+          <t>JASH</t>
         </is>
       </c>
       <c r="B38" s="20">
@@ -35137,7 +35485,7 @@
     <row r="39">
       <c r="A39" s="27" t="inlineStr">
         <is>
-          <t>KIRIINDUS</t>
+          <t>JAYKAY</t>
         </is>
       </c>
       <c r="B39" s="20">
@@ -35180,7 +35528,7 @@
     <row r="40">
       <c r="A40" s="27" t="inlineStr">
         <is>
-          <t>KIRLOSIND</t>
+          <t>JGCHEM</t>
         </is>
       </c>
       <c r="B40" s="20">
@@ -35223,7 +35571,7 @@
     <row r="41">
       <c r="A41" s="27" t="inlineStr">
         <is>
-          <t>KLBRENG-B</t>
+          <t>KCP</t>
         </is>
       </c>
       <c r="B41" s="20">
@@ -35266,7 +35614,7 @@
     <row r="42">
       <c r="A42" s="27" t="inlineStr">
         <is>
-          <t>KROSS</t>
+          <t>KIRIINDUS</t>
         </is>
       </c>
       <c r="B42" s="20">
@@ -35309,7 +35657,7 @@
     <row r="43">
       <c r="A43" s="27" t="inlineStr">
         <is>
-          <t>KSL</t>
+          <t>KIRLOSIND</t>
         </is>
       </c>
       <c r="B43" s="20">
@@ -35352,7 +35700,7 @@
     <row r="44">
       <c r="A44" s="27" t="inlineStr">
         <is>
-          <t>LUXIND</t>
+          <t>KLBRENG-B</t>
         </is>
       </c>
       <c r="B44" s="20">
@@ -35395,7 +35743,7 @@
     <row r="45">
       <c r="A45" s="27" t="inlineStr">
         <is>
-          <t>MAITHANALL</t>
+          <t>KROSS</t>
         </is>
       </c>
       <c r="B45" s="20">
@@ -35438,7 +35786,7 @@
     <row r="46">
       <c r="A46" s="27" t="inlineStr">
         <is>
-          <t>MANGLMCEM</t>
+          <t>KSL</t>
         </is>
       </c>
       <c r="B46" s="20">
@@ -35481,7 +35829,7 @@
     <row r="47">
       <c r="A47" s="27" t="inlineStr">
         <is>
-          <t>MASTEK</t>
+          <t>LUXIND</t>
         </is>
       </c>
       <c r="B47" s="20">
@@ -35524,7 +35872,7 @@
     <row r="48">
       <c r="A48" s="27" t="inlineStr">
         <is>
-          <t>MOBIKWIK</t>
+          <t>MAITHANALL</t>
         </is>
       </c>
       <c r="B48" s="20">
@@ -35567,7 +35915,7 @@
     <row r="49">
       <c r="A49" s="27" t="inlineStr">
         <is>
-          <t>NETWORK18</t>
+          <t>MANGLMCEM</t>
         </is>
       </c>
       <c r="B49" s="20">
@@ -35610,7 +35958,7 @@
     <row r="50">
       <c r="A50" s="27" t="inlineStr">
         <is>
-          <t>NILKAMAL</t>
+          <t>MASTEK</t>
         </is>
       </c>
       <c r="B50" s="20">
@@ -35653,7 +36001,7 @@
     <row r="51">
       <c r="A51" s="27" t="inlineStr">
         <is>
-          <t>NORTHARC</t>
+          <t>MOBIKWIK</t>
         </is>
       </c>
       <c r="B51" s="20">
@@ -35696,7 +36044,7 @@
     <row r="52">
       <c r="A52" s="27" t="inlineStr">
         <is>
-          <t>NOVARTIND</t>
+          <t>MUKANDLTD</t>
         </is>
       </c>
       <c r="B52" s="20">
@@ -35739,7 +36087,7 @@
     <row r="53">
       <c r="A53" s="27" t="inlineStr">
         <is>
-          <t>NPST</t>
+          <t>NETWORK18</t>
         </is>
       </c>
       <c r="B53" s="20">
@@ -35782,7 +36130,7 @@
     <row r="54">
       <c r="A54" s="27" t="inlineStr">
         <is>
-          <t>NRBBEARING</t>
+          <t>NILKAMAL</t>
         </is>
       </c>
       <c r="B54" s="20">
@@ -35825,7 +36173,7 @@
     <row r="55">
       <c r="A55" s="27" t="inlineStr">
         <is>
-          <t>OMAXE</t>
+          <t>NORTHARC</t>
         </is>
       </c>
       <c r="B55" s="20">
@@ -35868,7 +36216,7 @@
     <row r="56">
       <c r="A56" s="27" t="inlineStr">
         <is>
-          <t>OPTIEMUS</t>
+          <t>NOVARTIND</t>
         </is>
       </c>
       <c r="B56" s="20">
@@ -35911,7 +36259,7 @@
     <row r="57">
       <c r="A57" s="27" t="inlineStr">
         <is>
-          <t>ORIENTHOT</t>
+          <t>NPST</t>
         </is>
       </c>
       <c r="B57" s="20">
@@ -35954,7 +36302,7 @@
     <row r="58">
       <c r="A58" s="27" t="inlineStr">
         <is>
-          <t>PACEDIGITK</t>
+          <t>NRBBEARING</t>
         </is>
       </c>
       <c r="B58" s="20">
@@ -35997,7 +36345,7 @@
     <row r="59">
       <c r="A59" s="27" t="inlineStr">
         <is>
-          <t>PITTIENG</t>
+          <t>OMAXE</t>
         </is>
       </c>
       <c r="B59" s="20">
@@ -36040,7 +36388,7 @@
     <row r="60">
       <c r="A60" s="27" t="inlineStr">
         <is>
-          <t>PROTEAN</t>
+          <t>ONEPOINT</t>
         </is>
       </c>
       <c r="B60" s="20">
@@ -36083,7 +36431,7 @@
     <row r="61">
       <c r="A61" s="27" t="inlineStr">
         <is>
-          <t>QUADFUTURE</t>
+          <t>OPTIEMUS</t>
         </is>
       </c>
       <c r="B61" s="20">
@@ -36126,7 +36474,7 @@
     <row r="62">
       <c r="A62" s="27" t="inlineStr">
         <is>
-          <t>RACLGEAR</t>
+          <t>ORIENTHOT</t>
         </is>
       </c>
       <c r="B62" s="20">
@@ -36169,7 +36517,7 @@
     <row r="63">
       <c r="A63" s="27" t="inlineStr">
         <is>
-          <t>RAMRAT</t>
+          <t>PACEDIGITK</t>
         </is>
       </c>
       <c r="B63" s="20">
@@ -36212,7 +36560,7 @@
     <row r="64">
       <c r="A64" s="27" t="inlineStr">
         <is>
-          <t>RAYMOND</t>
+          <t>PITTIENG</t>
         </is>
       </c>
       <c r="B64" s="20">
@@ -36255,7 +36603,7 @@
     <row r="65">
       <c r="A65" s="27" t="inlineStr">
         <is>
-          <t>REFEX</t>
+          <t>PROTEAN</t>
         </is>
       </c>
       <c r="B65" s="20">
@@ -36298,7 +36646,7 @@
     <row r="66">
       <c r="A66" s="27" t="inlineStr">
         <is>
-          <t>RESPONIND</t>
+          <t>QUADFUTURE</t>
         </is>
       </c>
       <c r="B66" s="20">
@@ -36341,7 +36689,7 @@
     <row r="67">
       <c r="A67" s="27" t="inlineStr">
         <is>
-          <t>RML</t>
+          <t>RACLGEAR</t>
         </is>
       </c>
       <c r="B67" s="20">
@@ -36384,7 +36732,7 @@
     <row r="68">
       <c r="A68" s="27" t="inlineStr">
         <is>
-          <t>ROSSTECH</t>
+          <t>RAMRAT</t>
         </is>
       </c>
       <c r="B68" s="20">
@@ -36427,7 +36775,7 @@
     <row r="69">
       <c r="A69" s="27" t="inlineStr">
         <is>
-          <t>SAATVIKGL</t>
+          <t>RAYMOND</t>
         </is>
       </c>
       <c r="B69" s="20">
@@ -36470,7 +36818,7 @@
     <row r="70">
       <c r="A70" s="27" t="inlineStr">
         <is>
-          <t>SAKAR</t>
+          <t>RAYMONDREL</t>
         </is>
       </c>
       <c r="B70" s="20">
@@ -36513,7 +36861,7 @@
     <row r="71">
       <c r="A71" s="27" t="inlineStr">
         <is>
-          <t>SAMBHV</t>
+          <t>REFEX</t>
         </is>
       </c>
       <c r="B71" s="20">
@@ -36556,7 +36904,7 @@
     <row r="72">
       <c r="A72" s="27" t="inlineStr">
         <is>
-          <t>SAMHI</t>
+          <t>RESPONIND</t>
         </is>
       </c>
       <c r="B72" s="20">
@@ -36599,7 +36947,7 @@
     <row r="73">
       <c r="A73" s="27" t="inlineStr">
         <is>
-          <t>SHAREINDIA</t>
+          <t>RML</t>
         </is>
       </c>
       <c r="B73" s="20">
@@ -36642,7 +36990,7 @@
     <row r="74">
       <c r="A74" s="27" t="inlineStr">
         <is>
-          <t>SIKA</t>
+          <t>ROSSTECH</t>
         </is>
       </c>
       <c r="B74" s="20">
@@ -36685,7 +37033,7 @@
     <row r="75">
       <c r="A75" s="27" t="inlineStr">
         <is>
-          <t>SINDHUTRAD</t>
+          <t>RPGLIFE</t>
         </is>
       </c>
       <c r="B75" s="20">
@@ -36728,7 +37076,7 @@
     <row r="76">
       <c r="A76" s="27" t="inlineStr">
         <is>
-          <t>SMSPHARMA</t>
+          <t>SAATVIKGL</t>
         </is>
       </c>
       <c r="B76" s="20">
@@ -36771,7 +37119,7 @@
     <row r="77">
       <c r="A77" s="27" t="inlineStr">
         <is>
-          <t>SOLARA</t>
+          <t>SAKAR</t>
         </is>
       </c>
       <c r="B77" s="20">
@@ -36814,7 +37162,7 @@
     <row r="78">
       <c r="A78" s="27" t="inlineStr">
         <is>
-          <t>SOTL</t>
+          <t>SAMBHV</t>
         </is>
       </c>
       <c r="B78" s="20">
@@ -36857,7 +37205,7 @@
     <row r="79">
       <c r="A79" s="27" t="inlineStr">
         <is>
-          <t>SSWL</t>
+          <t>SAMHI</t>
         </is>
       </c>
       <c r="B79" s="20">
@@ -36900,7 +37248,7 @@
     <row r="80">
       <c r="A80" s="27" t="inlineStr">
         <is>
-          <t>STEELCAS</t>
+          <t>SHAREINDIA</t>
         </is>
       </c>
       <c r="B80" s="20">
@@ -36943,7 +37291,7 @@
     <row r="81">
       <c r="A81" s="27" t="inlineStr">
         <is>
-          <t>SYMPHONY</t>
+          <t>SIKA</t>
         </is>
       </c>
       <c r="B81" s="20">
@@ -36986,7 +37334,7 @@
     <row r="82">
       <c r="A82" s="27" t="inlineStr">
         <is>
-          <t>SYNCOMF</t>
+          <t>SINDHUTRAD</t>
         </is>
       </c>
       <c r="B82" s="20">
@@ -37029,7 +37377,7 @@
     <row r="83">
       <c r="A83" s="27" t="inlineStr">
         <is>
-          <t>TALBROAUTO</t>
+          <t>SMSPHARMA</t>
         </is>
       </c>
       <c r="B83" s="20">
@@ -37072,7 +37420,7 @@
     <row r="84">
       <c r="A84" s="27" t="inlineStr">
         <is>
-          <t>TBZ</t>
+          <t>SOLARA</t>
         </is>
       </c>
       <c r="B84" s="20">
@@ -37115,7 +37463,7 @@
     <row r="85">
       <c r="A85" s="27" t="inlineStr">
         <is>
-          <t>THOMASCOOK</t>
+          <t>SOTL</t>
         </is>
       </c>
       <c r="B85" s="20">
@@ -37158,7 +37506,7 @@
     <row r="86">
       <c r="A86" s="27" t="inlineStr">
         <is>
-          <t>VENKEYS</t>
+          <t>SSWL</t>
         </is>
       </c>
       <c r="B86" s="20">
@@ -37201,7 +37549,7 @@
     <row r="87">
       <c r="A87" s="27" t="inlineStr">
         <is>
-          <t>VENUSPIPES</t>
+          <t>STEELCAS</t>
         </is>
       </c>
       <c r="B87" s="20">
@@ -37244,7 +37592,7 @@
     <row r="88">
       <c r="A88" s="27" t="inlineStr">
         <is>
-          <t>VERANDA</t>
+          <t>SYMPHONY</t>
         </is>
       </c>
       <c r="B88" s="20">
@@ -37287,7 +37635,7 @@
     <row r="89">
       <c r="A89" s="27" t="inlineStr">
         <is>
-          <t>VSSL</t>
+          <t>SYNCOMF</t>
         </is>
       </c>
       <c r="B89" s="20">
@@ -37330,7 +37678,7 @@
     <row r="90">
       <c r="A90" s="27" t="inlineStr">
         <is>
-          <t>WELSPLSOL</t>
+          <t>TALBROAUTO</t>
         </is>
       </c>
       <c r="B90" s="20">
@@ -37373,7 +37721,7 @@
     <row r="91">
       <c r="A91" s="27" t="inlineStr">
         <is>
-          <t>WENDT</t>
+          <t>TBZ</t>
         </is>
       </c>
       <c r="B91" s="20">
@@ -37416,7 +37764,7 @@
     <row r="92">
       <c r="A92" s="27" t="inlineStr">
         <is>
-          <t>WINDLAS</t>
+          <t>THOMASCOOK</t>
         </is>
       </c>
       <c r="B92" s="20">
@@ -37459,7 +37807,7 @@
     <row r="93">
       <c r="A93" s="27" t="inlineStr">
         <is>
-          <t>XPROINDIA</t>
+          <t>VENKEYS</t>
         </is>
       </c>
       <c r="B93" s="20">
@@ -37502,7 +37850,7 @@
     <row r="94">
       <c r="A94" s="27" t="inlineStr">
         <is>
-          <t>ZAGGLE</t>
+          <t>VENUSPIPES</t>
         </is>
       </c>
       <c r="B94" s="20">
@@ -37545,7 +37893,7 @@
     <row r="95">
       <c r="A95" s="27" t="inlineStr">
         <is>
-          <t>ZOTA</t>
+          <t>VERANDA</t>
         </is>
       </c>
       <c r="B95" s="20">
@@ -37586,37 +37934,338 @@
       </c>
     </row>
     <row r="96">
-      <c r="A96" s="3" t="inlineStr">
+      <c r="A96" s="27" t="inlineStr">
+        <is>
+          <t>VSSL</t>
+        </is>
+      </c>
+      <c r="B96" s="20">
+        <f>COUNTIF('Trade Log'!$B$4:$B$503,$A96)</f>
+        <v/>
+      </c>
+      <c r="C96" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A96,'Trade Log'!$K$4:$K$503,"&gt;0")</f>
+        <v/>
+      </c>
+      <c r="D96" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A96,'Trade Log'!$K$4:$K$503,"&lt;0")</f>
+        <v/>
+      </c>
+      <c r="E96" s="29">
+        <f>IFERROR($C96/$B96,"")</f>
+        <v/>
+      </c>
+      <c r="F96" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A96,'Trade Log'!$I$4:$I$503)</f>
+        <v/>
+      </c>
+      <c r="G96" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A96,'Trade Log'!$K$4:$K$503)</f>
+        <v/>
+      </c>
+      <c r="H96" s="21">
+        <f>IFERROR($G96/$B96,"")</f>
+        <v/>
+      </c>
+      <c r="I96" s="21">
+        <f>IFERROR(_xlfn.MAXIFS('Trade Log'!$K$4:$K$503,'Trade Log'!$B$4:$B$503,$A96),"")</f>
+        <v/>
+      </c>
+      <c r="J96" s="21">
+        <f>IFERROR(_xlfn.MINIFS('Trade Log'!$K$4:$K$503,'Trade Log'!$B$4:$B$503,$A96),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" s="27" t="inlineStr">
+        <is>
+          <t>WELSPLSOL</t>
+        </is>
+      </c>
+      <c r="B97" s="20">
+        <f>COUNTIF('Trade Log'!$B$4:$B$503,$A97)</f>
+        <v/>
+      </c>
+      <c r="C97" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A97,'Trade Log'!$K$4:$K$503,"&gt;0")</f>
+        <v/>
+      </c>
+      <c r="D97" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A97,'Trade Log'!$K$4:$K$503,"&lt;0")</f>
+        <v/>
+      </c>
+      <c r="E97" s="29">
+        <f>IFERROR($C97/$B97,"")</f>
+        <v/>
+      </c>
+      <c r="F97" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A97,'Trade Log'!$I$4:$I$503)</f>
+        <v/>
+      </c>
+      <c r="G97" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A97,'Trade Log'!$K$4:$K$503)</f>
+        <v/>
+      </c>
+      <c r="H97" s="21">
+        <f>IFERROR($G97/$B97,"")</f>
+        <v/>
+      </c>
+      <c r="I97" s="21">
+        <f>IFERROR(_xlfn.MAXIFS('Trade Log'!$K$4:$K$503,'Trade Log'!$B$4:$B$503,$A97),"")</f>
+        <v/>
+      </c>
+      <c r="J97" s="21">
+        <f>IFERROR(_xlfn.MINIFS('Trade Log'!$K$4:$K$503,'Trade Log'!$B$4:$B$503,$A97),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" s="27" t="inlineStr">
+        <is>
+          <t>WENDT</t>
+        </is>
+      </c>
+      <c r="B98" s="20">
+        <f>COUNTIF('Trade Log'!$B$4:$B$503,$A98)</f>
+        <v/>
+      </c>
+      <c r="C98" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A98,'Trade Log'!$K$4:$K$503,"&gt;0")</f>
+        <v/>
+      </c>
+      <c r="D98" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A98,'Trade Log'!$K$4:$K$503,"&lt;0")</f>
+        <v/>
+      </c>
+      <c r="E98" s="29">
+        <f>IFERROR($C98/$B98,"")</f>
+        <v/>
+      </c>
+      <c r="F98" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A98,'Trade Log'!$I$4:$I$503)</f>
+        <v/>
+      </c>
+      <c r="G98" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A98,'Trade Log'!$K$4:$K$503)</f>
+        <v/>
+      </c>
+      <c r="H98" s="21">
+        <f>IFERROR($G98/$B98,"")</f>
+        <v/>
+      </c>
+      <c r="I98" s="21">
+        <f>IFERROR(_xlfn.MAXIFS('Trade Log'!$K$4:$K$503,'Trade Log'!$B$4:$B$503,$A98),"")</f>
+        <v/>
+      </c>
+      <c r="J98" s="21">
+        <f>IFERROR(_xlfn.MINIFS('Trade Log'!$K$4:$K$503,'Trade Log'!$B$4:$B$503,$A98),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" s="27" t="inlineStr">
+        <is>
+          <t>WINDLAS</t>
+        </is>
+      </c>
+      <c r="B99" s="20">
+        <f>COUNTIF('Trade Log'!$B$4:$B$503,$A99)</f>
+        <v/>
+      </c>
+      <c r="C99" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A99,'Trade Log'!$K$4:$K$503,"&gt;0")</f>
+        <v/>
+      </c>
+      <c r="D99" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A99,'Trade Log'!$K$4:$K$503,"&lt;0")</f>
+        <v/>
+      </c>
+      <c r="E99" s="29">
+        <f>IFERROR($C99/$B99,"")</f>
+        <v/>
+      </c>
+      <c r="F99" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A99,'Trade Log'!$I$4:$I$503)</f>
+        <v/>
+      </c>
+      <c r="G99" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A99,'Trade Log'!$K$4:$K$503)</f>
+        <v/>
+      </c>
+      <c r="H99" s="21">
+        <f>IFERROR($G99/$B99,"")</f>
+        <v/>
+      </c>
+      <c r="I99" s="21">
+        <f>IFERROR(_xlfn.MAXIFS('Trade Log'!$K$4:$K$503,'Trade Log'!$B$4:$B$503,$A99),"")</f>
+        <v/>
+      </c>
+      <c r="J99" s="21">
+        <f>IFERROR(_xlfn.MINIFS('Trade Log'!$K$4:$K$503,'Trade Log'!$B$4:$B$503,$A99),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" s="27" t="inlineStr">
+        <is>
+          <t>XPROINDIA</t>
+        </is>
+      </c>
+      <c r="B100" s="20">
+        <f>COUNTIF('Trade Log'!$B$4:$B$503,$A100)</f>
+        <v/>
+      </c>
+      <c r="C100" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A100,'Trade Log'!$K$4:$K$503,"&gt;0")</f>
+        <v/>
+      </c>
+      <c r="D100" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A100,'Trade Log'!$K$4:$K$503,"&lt;0")</f>
+        <v/>
+      </c>
+      <c r="E100" s="29">
+        <f>IFERROR($C100/$B100,"")</f>
+        <v/>
+      </c>
+      <c r="F100" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A100,'Trade Log'!$I$4:$I$503)</f>
+        <v/>
+      </c>
+      <c r="G100" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A100,'Trade Log'!$K$4:$K$503)</f>
+        <v/>
+      </c>
+      <c r="H100" s="21">
+        <f>IFERROR($G100/$B100,"")</f>
+        <v/>
+      </c>
+      <c r="I100" s="21">
+        <f>IFERROR(_xlfn.MAXIFS('Trade Log'!$K$4:$K$503,'Trade Log'!$B$4:$B$503,$A100),"")</f>
+        <v/>
+      </c>
+      <c r="J100" s="21">
+        <f>IFERROR(_xlfn.MINIFS('Trade Log'!$K$4:$K$503,'Trade Log'!$B$4:$B$503,$A100),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" s="27" t="inlineStr">
+        <is>
+          <t>ZAGGLE</t>
+        </is>
+      </c>
+      <c r="B101" s="20">
+        <f>COUNTIF('Trade Log'!$B$4:$B$503,$A101)</f>
+        <v/>
+      </c>
+      <c r="C101" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A101,'Trade Log'!$K$4:$K$503,"&gt;0")</f>
+        <v/>
+      </c>
+      <c r="D101" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A101,'Trade Log'!$K$4:$K$503,"&lt;0")</f>
+        <v/>
+      </c>
+      <c r="E101" s="29">
+        <f>IFERROR($C101/$B101,"")</f>
+        <v/>
+      </c>
+      <c r="F101" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A101,'Trade Log'!$I$4:$I$503)</f>
+        <v/>
+      </c>
+      <c r="G101" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A101,'Trade Log'!$K$4:$K$503)</f>
+        <v/>
+      </c>
+      <c r="H101" s="21">
+        <f>IFERROR($G101/$B101,"")</f>
+        <v/>
+      </c>
+      <c r="I101" s="21">
+        <f>IFERROR(_xlfn.MAXIFS('Trade Log'!$K$4:$K$503,'Trade Log'!$B$4:$B$503,$A101),"")</f>
+        <v/>
+      </c>
+      <c r="J101" s="21">
+        <f>IFERROR(_xlfn.MINIFS('Trade Log'!$K$4:$K$503,'Trade Log'!$B$4:$B$503,$A101),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" s="27" t="inlineStr">
+        <is>
+          <t>ZOTA</t>
+        </is>
+      </c>
+      <c r="B102" s="20">
+        <f>COUNTIF('Trade Log'!$B$4:$B$503,$A102)</f>
+        <v/>
+      </c>
+      <c r="C102" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A102,'Trade Log'!$K$4:$K$503,"&gt;0")</f>
+        <v/>
+      </c>
+      <c r="D102" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A102,'Trade Log'!$K$4:$K$503,"&lt;0")</f>
+        <v/>
+      </c>
+      <c r="E102" s="29">
+        <f>IFERROR($C102/$B102,"")</f>
+        <v/>
+      </c>
+      <c r="F102" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A102,'Trade Log'!$I$4:$I$503)</f>
+        <v/>
+      </c>
+      <c r="G102" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A102,'Trade Log'!$K$4:$K$503)</f>
+        <v/>
+      </c>
+      <c r="H102" s="21">
+        <f>IFERROR($G102/$B102,"")</f>
+        <v/>
+      </c>
+      <c r="I102" s="21">
+        <f>IFERROR(_xlfn.MAXIFS('Trade Log'!$K$4:$K$503,'Trade Log'!$B$4:$B$503,$A102),"")</f>
+        <v/>
+      </c>
+      <c r="J102" s="21">
+        <f>IFERROR(_xlfn.MINIFS('Trade Log'!$K$4:$K$503,'Trade Log'!$B$4:$B$503,$A102),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" s="3" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="B96" s="30">
-        <f>SUM(B4:B95)</f>
-        <v/>
-      </c>
-      <c r="C96" s="30">
-        <f>SUM(C4:C95)</f>
-        <v/>
-      </c>
-      <c r="D96" s="30">
-        <f>SUM(D4:D95)</f>
-        <v/>
-      </c>
-      <c r="E96" s="31">
-        <f>IFERROR(C96/B96,"")</f>
-        <v/>
-      </c>
-      <c r="F96" s="32">
-        <f>SUM(F4:F95)</f>
-        <v/>
-      </c>
-      <c r="G96" s="32">
-        <f>SUM(G4:G95)</f>
-        <v/>
-      </c>
-      <c r="H96" s="32">
-        <f>IFERROR(G96/B96,"")</f>
+      <c r="B103" s="30">
+        <f>SUM(B4:B102)</f>
+        <v/>
+      </c>
+      <c r="C103" s="30">
+        <f>SUM(C4:C102)</f>
+        <v/>
+      </c>
+      <c r="D103" s="30">
+        <f>SUM(D4:D102)</f>
+        <v/>
+      </c>
+      <c r="E103" s="31">
+        <f>IFERROR(C103/B103,"")</f>
+        <v/>
+      </c>
+      <c r="F103" s="32">
+        <f>SUM(F4:F102)</f>
+        <v/>
+      </c>
+      <c r="G103" s="32">
+        <f>SUM(G4:G102)</f>
+        <v/>
+      </c>
+      <c r="H103" s="32">
+        <f>IFERROR(G103/B103,"")</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Data update — 2026-09-24 candle + results refresh
</commit_message>
<xml_diff>
--- a/results/strategy_pnl_simple.xlsx
+++ b/results/strategy_pnl_simple.xlsx
@@ -1473,7 +1473,7 @@
         <v/>
       </c>
       <c r="J4" s="4" t="n">
-        <v>571.72</v>
+        <v>571.6900000000001</v>
       </c>
       <c r="K4" s="21">
         <f>IF(OR($B4="",$I4=""),"",$I4-IF($J4="",0,$J4))</f>
@@ -1575,7 +1575,7 @@
         <v/>
       </c>
       <c r="J6" s="4" t="n">
-        <v>570.5700000000001</v>
+        <v>570.54</v>
       </c>
       <c r="K6" s="21">
         <f>IF(OR($B6="",$I6=""),"",$I6-IF($J6="",0,$J6))</f>
@@ -1626,7 +1626,7 @@
         <v/>
       </c>
       <c r="J7" s="4" t="n">
-        <v>662.96</v>
+        <v>662.9299999999999</v>
       </c>
       <c r="K7" s="21">
         <f>IF(OR($B7="",$I7=""),"",$I7-IF($J7="",0,$J7))</f>
@@ -1677,7 +1677,7 @@
         <v/>
       </c>
       <c r="J8" s="4" t="n">
-        <v>591.26</v>
+        <v>591.38</v>
       </c>
       <c r="K8" s="21">
         <f>IF(OR($B8="",$I8=""),"",$I8-IF($J8="",0,$J8))</f>
@@ -1779,7 +1779,7 @@
         <v/>
       </c>
       <c r="J10" s="4" t="n">
-        <v>398.58</v>
+        <v>398.57</v>
       </c>
       <c r="K10" s="21">
         <f>IF(OR($B10="",$I10=""),"",$I10-IF($J10="",0,$J10))</f>
@@ -1881,7 +1881,7 @@
         <v/>
       </c>
       <c r="J12" s="4" t="n">
-        <v>414.11</v>
+        <v>414.1</v>
       </c>
       <c r="K12" s="21">
         <f>IF(OR($B12="",$I12=""),"",$I12-IF($J12="",0,$J12))</f>
@@ -1932,7 +1932,7 @@
         <v/>
       </c>
       <c r="J13" s="4" t="n">
-        <v>345.04</v>
+        <v>345.03</v>
       </c>
       <c r="K13" s="21">
         <f>IF(OR($B13="",$I13=""),"",$I13-IF($J13="",0,$J13))</f>
@@ -1983,7 +1983,7 @@
         <v/>
       </c>
       <c r="J14" s="4" t="n">
-        <v>414.44</v>
+        <v>414.43</v>
       </c>
       <c r="K14" s="21">
         <f>IF(OR($B14="",$I14=""),"",$I14-IF($J14="",0,$J14))</f>
@@ -2034,7 +2034,7 @@
         <v/>
       </c>
       <c r="J15" s="4" t="n">
-        <v>380.46</v>
+        <v>380.49</v>
       </c>
       <c r="K15" s="21">
         <f>IF(OR($B15="",$I15=""),"",$I15-IF($J15="",0,$J15))</f>
@@ -2187,7 +2187,7 @@
         <v/>
       </c>
       <c r="J18" s="4" t="n">
-        <v>413.88</v>
+        <v>413.86</v>
       </c>
       <c r="K18" s="21">
         <f>IF(OR($B18="",$I18=""),"",$I18-IF($J18="",0,$J18))</f>
@@ -2238,7 +2238,7 @@
         <v/>
       </c>
       <c r="J19" s="4" t="n">
-        <v>406.42</v>
+        <v>406.4</v>
       </c>
       <c r="K19" s="21">
         <f>IF(OR($B19="",$I19=""),"",$I19-IF($J19="",0,$J19))</f>
@@ -2697,7 +2697,7 @@
         <v/>
       </c>
       <c r="J28" s="4" t="n">
-        <v>870.79</v>
+        <v>869.5700000000001</v>
       </c>
       <c r="K28" s="21">
         <f>IF(OR($B28="",$I28=""),"",$I28-IF($J28="",0,$J28))</f>
@@ -2850,7 +2850,7 @@
         <v/>
       </c>
       <c r="J31" s="4" t="n">
-        <v>391.18</v>
+        <v>390</v>
       </c>
       <c r="K31" s="21">
         <f>IF(OR($B31="",$I31=""),"",$I31-IF($J31="",0,$J31))</f>
@@ -2901,7 +2901,7 @@
         <v/>
       </c>
       <c r="J32" s="4" t="n">
-        <v>349.8</v>
+        <v>348.62</v>
       </c>
       <c r="K32" s="21">
         <f>IF(OR($B32="",$I32=""),"",$I32-IF($J32="",0,$J32))</f>
@@ -3003,7 +3003,7 @@
         <v/>
       </c>
       <c r="J34" s="4" t="n">
-        <v>348.45</v>
+        <v>346.34</v>
       </c>
       <c r="K34" s="21">
         <f>IF(OR($B34="",$I34=""),"",$I34-IF($J34="",0,$J34))</f>
@@ -3054,7 +3054,7 @@
         <v/>
       </c>
       <c r="J35" s="4" t="n">
-        <v>386.25</v>
+        <v>385.16</v>
       </c>
       <c r="K35" s="21">
         <f>IF(OR($B35="",$I35=""),"",$I35-IF($J35="",0,$J35))</f>
@@ -3411,7 +3411,7 @@
         <v/>
       </c>
       <c r="J42" s="4" t="n">
-        <v>978.3200000000001</v>
+        <v>975.85</v>
       </c>
       <c r="K42" s="21">
         <f>IF(OR($B42="",$I42=""),"",$I42-IF($J42="",0,$J42))</f>
@@ -3462,7 +3462,7 @@
         <v/>
       </c>
       <c r="J43" s="4" t="n">
-        <v>957.71</v>
+        <v>955.65</v>
       </c>
       <c r="K43" s="21">
         <f>IF(OR($B43="",$I43=""),"",$I43-IF($J43="",0,$J43))</f>
@@ -3513,7 +3513,7 @@
         <v/>
       </c>
       <c r="J44" s="4" t="n">
-        <v>992.3099999999999</v>
+        <v>989.83</v>
       </c>
       <c r="K44" s="21">
         <f>IF(OR($B44="",$I44=""),"",$I44-IF($J44="",0,$J44))</f>
@@ -3564,7 +3564,7 @@
         <v/>
       </c>
       <c r="J45" s="4" t="n">
-        <v>599.76</v>
+        <v>595.8099999999999</v>
       </c>
       <c r="K45" s="21">
         <f>IF(OR($B45="",$I45=""),"",$I45-IF($J45="",0,$J45))</f>
@@ -3615,7 +3615,7 @@
         <v/>
       </c>
       <c r="J46" s="4" t="n">
-        <v>600.87</v>
+        <v>596.91</v>
       </c>
       <c r="K46" s="21">
         <f>IF(OR($B46="",$I46=""),"",$I46-IF($J46="",0,$J46))</f>
@@ -3666,7 +3666,7 @@
         <v/>
       </c>
       <c r="J47" s="4" t="n">
-        <v>679.25</v>
+        <v>675.08</v>
       </c>
       <c r="K47" s="21">
         <f>IF(OR($B47="",$I47=""),"",$I47-IF($J47="",0,$J47))</f>
@@ -3717,7 +3717,7 @@
         <v/>
       </c>
       <c r="J48" s="4" t="n">
-        <v>672.67</v>
+        <v>668.47</v>
       </c>
       <c r="K48" s="21">
         <f>IF(OR($B48="",$I48=""),"",$I48-IF($J48="",0,$J48))</f>
@@ -3768,7 +3768,7 @@
         <v/>
       </c>
       <c r="J49" s="4" t="n">
-        <v>538.72</v>
+        <v>572.83</v>
       </c>
       <c r="K49" s="21">
         <f>IF(OR($B49="",$I49=""),"",$I49-IF($J49="",0,$J49))</f>
@@ -3819,7 +3819,7 @@
         <v/>
       </c>
       <c r="J50" s="4" t="n">
-        <v>628.96</v>
+        <v>627.63</v>
       </c>
       <c r="K50" s="21">
         <f>IF(OR($B50="",$I50=""),"",$I50-IF($J50="",0,$J50))</f>
@@ -4023,7 +4023,7 @@
         <v/>
       </c>
       <c r="J54" s="4" t="n">
-        <v>620.05</v>
+        <v>618.74</v>
       </c>
       <c r="K54" s="21">
         <f>IF(OR($B54="",$I54=""),"",$I54-IF($J54="",0,$J54))</f>
@@ -4176,7 +4176,7 @@
         <v/>
       </c>
       <c r="J57" s="4" t="n">
-        <v>613.09</v>
+        <v>611.85</v>
       </c>
       <c r="K57" s="21">
         <f>IF(OR($B57="",$I57=""),"",$I57-IF($J57="",0,$J57))</f>
@@ -4380,7 +4380,7 @@
         <v/>
       </c>
       <c r="J61" s="4" t="n">
-        <v>693.72</v>
+        <v>693.71</v>
       </c>
       <c r="K61" s="21">
         <f>IF(OR($B61="",$I61=""),"",$I61-IF($J61="",0,$J61))</f>
@@ -4431,7 +4431,7 @@
         <v/>
       </c>
       <c r="J62" s="4" t="n">
-        <v>616.92</v>
+        <v>616.9299999999999</v>
       </c>
       <c r="K62" s="21">
         <f>IF(OR($B62="",$I62=""),"",$I62-IF($J62="",0,$J62))</f>
@@ -4533,7 +4533,7 @@
         <v/>
       </c>
       <c r="J64" s="4" t="n">
-        <v>441.49</v>
+        <v>441.48</v>
       </c>
       <c r="K64" s="21">
         <f>IF(OR($B64="",$I64=""),"",$I64-IF($J64="",0,$J64))</f>
@@ -4584,7 +4584,7 @@
         <v/>
       </c>
       <c r="J65" s="4" t="n">
-        <v>387.52</v>
+        <v>387.51</v>
       </c>
       <c r="K65" s="21">
         <f>IF(OR($B65="",$I65=""),"",$I65-IF($J65="",0,$J65))</f>
@@ -4839,7 +4839,7 @@
         <v/>
       </c>
       <c r="J70" s="4" t="n">
-        <v>386.12</v>
+        <v>386.11</v>
       </c>
       <c r="K70" s="21">
         <f>IF(OR($B70="",$I70=""),"",$I70-IF($J70="",0,$J70))</f>
@@ -4890,7 +4890,7 @@
         <v/>
       </c>
       <c r="J71" s="4" t="n">
-        <v>435.19</v>
+        <v>435.18</v>
       </c>
       <c r="K71" s="21">
         <f>IF(OR($B71="",$I71=""),"",$I71-IF($J71="",0,$J71))</f>
@@ -4941,7 +4941,7 @@
         <v/>
       </c>
       <c r="J72" s="4" t="n">
-        <v>411.82</v>
+        <v>411.81</v>
       </c>
       <c r="K72" s="21">
         <f>IF(OR($B72="",$I72=""),"",$I72-IF($J72="",0,$J72))</f>
@@ -5043,7 +5043,7 @@
         <v/>
       </c>
       <c r="J74" s="4" t="n">
-        <v>356.28</v>
+        <v>356.27</v>
       </c>
       <c r="K74" s="21">
         <f>IF(OR($B74="",$I74=""),"",$I74-IF($J74="",0,$J74))</f>
@@ -5094,7 +5094,7 @@
         <v/>
       </c>
       <c r="J75" s="4" t="n">
-        <v>364.9</v>
+        <v>364.89</v>
       </c>
       <c r="K75" s="21">
         <f>IF(OR($B75="",$I75=""),"",$I75-IF($J75="",0,$J75))</f>
@@ -5196,7 +5196,7 @@
         <v/>
       </c>
       <c r="J77" s="4" t="n">
-        <v>412.19</v>
+        <v>412.23</v>
       </c>
       <c r="K77" s="21">
         <f>IF(OR($B77="",$I77=""),"",$I77-IF($J77="",0,$J77))</f>
@@ -5859,7 +5859,7 @@
         <v/>
       </c>
       <c r="J90" s="4" t="n">
-        <v>893.53</v>
+        <v>893.48</v>
       </c>
       <c r="K90" s="21">
         <f>IF(OR($B90="",$I90=""),"",$I90-IF($J90="",0,$J90))</f>
@@ -5961,7 +5961,7 @@
         <v/>
       </c>
       <c r="J92" s="4" t="n">
-        <v>799.55</v>
+        <v>799.5</v>
       </c>
       <c r="K92" s="21">
         <f>IF(OR($B92="",$I92=""),"",$I92-IF($J92="",0,$J92))</f>
@@ -6012,7 +6012,7 @@
         <v/>
       </c>
       <c r="J93" s="4" t="n">
-        <v>826.89</v>
+        <v>826.84</v>
       </c>
       <c r="K93" s="21">
         <f>IF(OR($B93="",$I93=""),"",$I93-IF($J93="",0,$J93))</f>
@@ -6063,7 +6063,7 @@
         <v/>
       </c>
       <c r="J94" s="4" t="n">
-        <v>479.53</v>
+        <v>479.59</v>
       </c>
       <c r="K94" s="21">
         <f>IF(OR($B94="",$I94=""),"",$I94-IF($J94="",0,$J94))</f>
@@ -6165,7 +6165,7 @@
         <v/>
       </c>
       <c r="J96" s="4" t="n">
-        <v>474.61</v>
+        <v>474.59</v>
       </c>
       <c r="K96" s="21">
         <f>IF(OR($B96="",$I96=""),"",$I96-IF($J96="",0,$J96))</f>
@@ -6267,7 +6267,7 @@
         <v/>
       </c>
       <c r="J98" s="4" t="n">
-        <v>531.38</v>
+        <v>531.36</v>
       </c>
       <c r="K98" s="21">
         <f>IF(OR($B98="",$I98=""),"",$I98-IF($J98="",0,$J98))</f>
@@ -6471,7 +6471,7 @@
         <v/>
       </c>
       <c r="J102" s="4" t="n">
-        <v>531.59</v>
+        <v>531.58</v>
       </c>
       <c r="K102" s="21">
         <f>IF(OR($B102="",$I102=""),"",$I102-IF($J102="",0,$J102))</f>
@@ -6879,7 +6879,7 @@
         <v/>
       </c>
       <c r="J110" s="4" t="n">
-        <v>480.91</v>
+        <v>480.93</v>
       </c>
       <c r="K110" s="21">
         <f>IF(OR($B110="",$I110=""),"",$I110-IF($J110="",0,$J110))</f>
@@ -6981,7 +6981,7 @@
         <v/>
       </c>
       <c r="J112" s="4" t="n">
-        <v>420.16</v>
+        <v>420.14</v>
       </c>
       <c r="K112" s="21">
         <f>IF(OR($B112="",$I112=""),"",$I112-IF($J112="",0,$J112))</f>
@@ -7185,7 +7185,7 @@
         <v/>
       </c>
       <c r="J116" s="4" t="n">
-        <v>428.75</v>
+        <v>428.78</v>
       </c>
       <c r="K116" s="21">
         <f>IF(OR($B116="",$I116=""),"",$I116-IF($J116="",0,$J116))</f>
@@ -7236,7 +7236,7 @@
         <v/>
       </c>
       <c r="J117" s="4" t="n">
-        <v>546.36</v>
+        <v>546.34</v>
       </c>
       <c r="K117" s="21">
         <f>IF(OR($B117="",$I117=""),"",$I117-IF($J117="",0,$J117))</f>
@@ -7389,7 +7389,7 @@
         <v/>
       </c>
       <c r="J120" s="4" t="n">
-        <v>424.99</v>
+        <v>424.98</v>
       </c>
       <c r="K120" s="21">
         <f>IF(OR($B120="",$I120=""),"",$I120-IF($J120="",0,$J120))</f>
@@ -7440,7 +7440,7 @@
         <v/>
       </c>
       <c r="J121" s="4" t="n">
-        <v>371.6</v>
+        <v>371.59</v>
       </c>
       <c r="K121" s="21">
         <f>IF(OR($B121="",$I121=""),"",$I121-IF($J121="",0,$J121))</f>
@@ -7746,7 +7746,7 @@
         <v/>
       </c>
       <c r="J127" s="4" t="n">
-        <v>642.53</v>
+        <v>642.51</v>
       </c>
       <c r="K127" s="21">
         <f>IF(OR($B127="",$I127=""),"",$I127-IF($J127="",0,$J127))</f>
@@ -7848,7 +7848,7 @@
         <v/>
       </c>
       <c r="J129" s="4" t="n">
-        <v>638.37</v>
+        <v>638.35</v>
       </c>
       <c r="K129" s="21">
         <f>IF(OR($B129="",$I129=""),"",$I129-IF($J129="",0,$J129))</f>
@@ -7950,7 +7950,7 @@
         <v/>
       </c>
       <c r="J131" s="4" t="n">
-        <v>654.2</v>
+        <v>654.25</v>
       </c>
       <c r="K131" s="21">
         <f>IF(OR($B131="",$I131=""),"",$I131-IF($J131="",0,$J131))</f>
@@ -8052,7 +8052,7 @@
         <v/>
       </c>
       <c r="J133" s="4" t="n">
-        <v>564.2</v>
+        <v>564.1799999999999</v>
       </c>
       <c r="K133" s="21">
         <f>IF(OR($B133="",$I133=""),"",$I133-IF($J133="",0,$J133))</f>
@@ -8103,7 +8103,7 @@
         <v/>
       </c>
       <c r="J134" s="4" t="n">
-        <v>632.16</v>
+        <v>632.14</v>
       </c>
       <c r="K134" s="21">
         <f>IF(OR($B134="",$I134=""),"",$I134-IF($J134="",0,$J134))</f>
@@ -8154,7 +8154,7 @@
         <v/>
       </c>
       <c r="J135" s="4" t="n">
-        <v>497.92</v>
+        <v>497.88</v>
       </c>
       <c r="K135" s="21">
         <f>IF(OR($B135="",$I135=""),"",$I135-IF($J135="",0,$J135))</f>
@@ -8307,7 +8307,7 @@
         <v/>
       </c>
       <c r="J138" s="4" t="n">
-        <v>494.66</v>
+        <v>494.63</v>
       </c>
       <c r="K138" s="21">
         <f>IF(OR($B138="",$I138=""),"",$I138-IF($J138="",0,$J138))</f>
@@ -8409,7 +8409,7 @@
         <v/>
       </c>
       <c r="J140" s="4" t="n">
-        <v>504.22</v>
+        <v>504.18</v>
       </c>
       <c r="K140" s="21">
         <f>IF(OR($B140="",$I140=""),"",$I140-IF($J140="",0,$J140))</f>
@@ -8460,7 +8460,7 @@
         <v/>
       </c>
       <c r="J141" s="4" t="n">
-        <v>491.96</v>
+        <v>492.11</v>
       </c>
       <c r="K141" s="21">
         <f>IF(OR($B141="",$I141=""),"",$I141-IF($J141="",0,$J141))</f>
@@ -8511,7 +8511,7 @@
         <v/>
       </c>
       <c r="J142" s="4" t="n">
-        <v>467.32</v>
+        <v>467.29</v>
       </c>
       <c r="K142" s="21">
         <f>IF(OR($B142="",$I142=""),"",$I142-IF($J142="",0,$J142))</f>
@@ -8664,7 +8664,7 @@
         <v/>
       </c>
       <c r="J145" s="4" t="n">
-        <v>541.92</v>
+        <v>542.0599999999999</v>
       </c>
       <c r="K145" s="21">
         <f>IF(OR($B145="",$I145=""),"",$I145-IF($J145="",0,$J145))</f>
@@ -9480,7 +9480,7 @@
         <v/>
       </c>
       <c r="J161" s="4" t="n">
-        <v>461.65</v>
+        <v>461.69</v>
       </c>
       <c r="K161" s="21">
         <f>IF(OR($B161="",$I161=""),"",$I161-IF($J161="",0,$J161))</f>
@@ -9990,7 +9990,7 @@
         <v/>
       </c>
       <c r="J171" s="4" t="n">
-        <v>662.1</v>
+        <v>662.13</v>
       </c>
       <c r="K171" s="21">
         <f>IF(OR($B171="",$I171=""),"",$I171-IF($J171="",0,$J171))</f>
@@ -10500,7 +10500,7 @@
         <v/>
       </c>
       <c r="J181" s="4" t="n">
-        <v>298.69</v>
+        <v>298.41</v>
       </c>
       <c r="K181" s="21">
         <f>IF(OR($B181="",$I181=""),"",$I181-IF($J181="",0,$J181))</f>
@@ -10704,7 +10704,7 @@
         <v/>
       </c>
       <c r="J185" s="4" t="n">
-        <v>295.23</v>
+        <v>295.25</v>
       </c>
       <c r="K185" s="21">
         <f>IF(OR($B185="",$I185=""),"",$I185-IF($J185="",0,$J185))</f>
@@ -10908,7 +10908,7 @@
         <v/>
       </c>
       <c r="J189" s="4" t="n">
-        <v>99.33</v>
+        <v>132.03</v>
       </c>
       <c r="K189" s="21">
         <f>IF(OR($B189="",$I189=""),"",$I189-IF($J189="",0,$J189))</f>
@@ -10959,7 +10959,7 @@
         <v/>
       </c>
       <c r="J190" s="4" t="n">
-        <v>426.86</v>
+        <v>459.73</v>
       </c>
       <c r="K190" s="21">
         <f>IF(OR($B190="",$I190=""),"",$I190-IF($J190="",0,$J190))</f>
@@ -11214,7 +11214,7 @@
         <v/>
       </c>
       <c r="J195" s="4" t="n">
-        <v>429.45</v>
+        <v>462.53</v>
       </c>
       <c r="K195" s="21">
         <f>IF(OR($B195="",$I195=""),"",$I195-IF($J195="",0,$J195))</f>
@@ -11265,7 +11265,7 @@
         <v/>
       </c>
       <c r="J196" s="4" t="n">
-        <v>422.26</v>
+        <v>517.1</v>
       </c>
       <c r="K196" s="21">
         <f>IF(OR($B196="",$I196=""),"",$I196-IF($J196="",0,$J196))</f>
@@ -11367,7 +11367,7 @@
         <v/>
       </c>
       <c r="J198" s="4" t="n">
-        <v>422.16</v>
+        <v>519.16</v>
       </c>
       <c r="K198" s="21">
         <f>IF(OR($B198="",$I198=""),"",$I198-IF($J198="",0,$J198))</f>
@@ -11418,7 +11418,7 @@
         <v/>
       </c>
       <c r="J199" s="4" t="n">
-        <v>423.59</v>
+        <v>456.59</v>
       </c>
       <c r="K199" s="21">
         <f>IF(OR($B199="",$I199=""),"",$I199-IF($J199="",0,$J199))</f>
@@ -11458,14 +11458,18 @@
       <c r="F200" s="26" t="n">
         <v>262</v>
       </c>
-      <c r="G200" s="24" t="inlineStr"/>
-      <c r="H200" s="25" t="inlineStr"/>
+      <c r="G200" s="24" t="n">
+        <v>46289</v>
+      </c>
+      <c r="H200" s="25" t="n">
+        <v>627.8200000000001</v>
+      </c>
       <c r="I200" s="21">
         <f>IF(OR($B200="",$H200=""),"",IF($C200="LONG",($H200-$E200)*$F200,($E200-$H200)*$F200))</f>
         <v/>
       </c>
       <c r="J200" s="4" t="n">
-        <v>50.15</v>
+        <v>84.33</v>
       </c>
       <c r="K200" s="21">
         <f>IF(OR($B200="",$I200=""),"",$I200-IF($J200="",0,$J200))</f>
@@ -11516,7 +11520,7 @@
         <v/>
       </c>
       <c r="J201" s="4" t="n">
-        <v>0</v>
+        <v>352.9</v>
       </c>
       <c r="K201" s="21">
         <f>IF(OR($B201="",$I201=""),"",$I201-IF($J201="",0,$J201))</f>
@@ -11567,7 +11571,7 @@
         <v/>
       </c>
       <c r="J202" s="4" t="n">
-        <v>0</v>
+        <v>359.46</v>
       </c>
       <c r="K202" s="21">
         <f>IF(OR($B202="",$I202=""),"",$I202-IF($J202="",0,$J202))</f>
@@ -11607,14 +11611,18 @@
       <c r="F203" s="26" t="n">
         <v>2426</v>
       </c>
-      <c r="G203" s="24" t="inlineStr"/>
-      <c r="H203" s="25" t="inlineStr"/>
+      <c r="G203" s="24" t="n">
+        <v>46289</v>
+      </c>
+      <c r="H203" s="25" t="n">
+        <v>71</v>
+      </c>
       <c r="I203" s="21">
         <f>IF(OR($B203="",$H203=""),"",IF($C203="LONG",($H203-$E203)*$F203,($E203-$H203)*$F203))</f>
         <v/>
       </c>
       <c r="J203" s="4" t="n">
-        <v>50.15</v>
+        <v>86.05</v>
       </c>
       <c r="K203" s="21">
         <f>IF(OR($B203="",$I203=""),"",$I203-IF($J203="",0,$J203))</f>
@@ -11654,8 +11662,12 @@
       <c r="F204" s="26" t="n">
         <v>139</v>
       </c>
-      <c r="G204" s="24" t="inlineStr"/>
-      <c r="H204" s="25" t="inlineStr"/>
+      <c r="G204" s="24" t="n">
+        <v>46289</v>
+      </c>
+      <c r="H204" s="25" t="n">
+        <v>634.15</v>
+      </c>
       <c r="I204" s="21">
         <f>IF(OR($B204="",$H204=""),"",IF($C204="LONG",($H204-$E204)*$F204,($E204-$H204)*$F204))</f>
         <v/>
@@ -11701,14 +11713,18 @@
       <c r="F205" s="26" t="n">
         <v>780</v>
       </c>
-      <c r="G205" s="24" t="inlineStr"/>
-      <c r="H205" s="25" t="inlineStr"/>
+      <c r="G205" s="24" t="n">
+        <v>46289</v>
+      </c>
+      <c r="H205" s="25" t="n">
+        <v>205.69</v>
+      </c>
       <c r="I205" s="21">
         <f>IF(OR($B205="",$H205=""),"",IF($C205="LONG",($H205-$E205)*$F205,($E205-$H205)*$F205))</f>
         <v/>
       </c>
       <c r="J205" s="4" t="n">
-        <v>50.15</v>
+        <v>82.28</v>
       </c>
       <c r="K205" s="21">
         <f>IF(OR($B205="",$I205=""),"",$I205-IF($J205="",0,$J205))</f>
@@ -11748,14 +11764,18 @@
       <c r="F206" s="26" t="n">
         <v>597</v>
       </c>
-      <c r="G206" s="24" t="inlineStr"/>
-      <c r="H206" s="25" t="inlineStr"/>
+      <c r="G206" s="24" t="n">
+        <v>46289</v>
+      </c>
+      <c r="H206" s="25" t="n">
+        <v>273.19</v>
+      </c>
       <c r="I206" s="21">
         <f>IF(OR($B206="",$H206=""),"",IF($C206="LONG",($H206-$E206)*$F206,($E206-$H206)*$F206))</f>
         <v/>
       </c>
       <c r="J206" s="4" t="n">
-        <v>50.15</v>
+        <v>299.68</v>
       </c>
       <c r="K206" s="21">
         <f>IF(OR($B206="",$I206=""),"",$I206-IF($J206="",0,$J206))</f>
@@ -11795,14 +11815,18 @@
       <c r="F207" s="26" t="n">
         <v>1059</v>
       </c>
-      <c r="G207" s="24" t="inlineStr"/>
-      <c r="H207" s="25" t="inlineStr"/>
+      <c r="G207" s="24" t="n">
+        <v>46289</v>
+      </c>
+      <c r="H207" s="25" t="n">
+        <v>156.75</v>
+      </c>
       <c r="I207" s="21">
         <f>IF(OR($B207="",$H207=""),"",IF($C207="LONG",($H207-$E207)*$F207,($E207-$H207)*$F207))</f>
         <v/>
       </c>
       <c r="J207" s="4" t="n">
-        <v>50.15</v>
+        <v>305.04</v>
       </c>
       <c r="K207" s="21">
         <f>IF(OR($B207="",$I207=""),"",$I207-IF($J207="",0,$J207))</f>
@@ -11842,14 +11866,18 @@
       <c r="F208" s="26" t="n">
         <v>2439</v>
       </c>
-      <c r="G208" s="24" t="inlineStr"/>
-      <c r="H208" s="25" t="inlineStr"/>
+      <c r="G208" s="24" t="n">
+        <v>46289</v>
+      </c>
+      <c r="H208" s="25" t="n">
+        <v>71.39</v>
+      </c>
       <c r="I208" s="21">
         <f>IF(OR($B208="",$H208=""),"",IF($C208="LONG",($H208-$E208)*$F208,($E208-$H208)*$F208))</f>
         <v/>
       </c>
       <c r="J208" s="4" t="n">
-        <v>50.15</v>
+        <v>300.26</v>
       </c>
       <c r="K208" s="21">
         <f>IF(OR($B208="",$I208=""),"",$I208-IF($J208="",0,$J208))</f>
@@ -11900,7 +11928,7 @@
         <v/>
       </c>
       <c r="J209" s="4" t="n">
-        <v>0</v>
+        <v>365.31</v>
       </c>
       <c r="K209" s="21">
         <f>IF(OR($B209="",$I209=""),"",$I209-IF($J209="",0,$J209))</f>
@@ -11951,7 +11979,7 @@
         <v/>
       </c>
       <c r="J210" s="4" t="n">
-        <v>0</v>
+        <v>298.29</v>
       </c>
       <c r="K210" s="21">
         <f>IF(OR($B210="",$I210=""),"",$I210-IF($J210="",0,$J210))</f>
@@ -11991,14 +12019,18 @@
       <c r="F211" s="26" t="n">
         <v>246</v>
       </c>
-      <c r="G211" s="24" t="inlineStr"/>
-      <c r="H211" s="25" t="inlineStr"/>
+      <c r="G211" s="24" t="n">
+        <v>46289</v>
+      </c>
+      <c r="H211" s="25" t="n">
+        <v>677.5</v>
+      </c>
       <c r="I211" s="21">
         <f>IF(OR($B211="",$H211=""),"",IF($C211="LONG",($H211-$E211)*$F211,($E211-$H211)*$F211))</f>
         <v/>
       </c>
       <c r="J211" s="4" t="n">
-        <v>50.15</v>
+        <v>303.26</v>
       </c>
       <c r="K211" s="21">
         <f>IF(OR($B211="",$I211=""),"",$I211-IF($J211="",0,$J211))</f>
@@ -12038,14 +12070,18 @@
       <c r="F212" s="26" t="n">
         <v>55</v>
       </c>
-      <c r="G212" s="24" t="inlineStr"/>
-      <c r="H212" s="25" t="inlineStr"/>
+      <c r="G212" s="24" t="n">
+        <v>46289</v>
+      </c>
+      <c r="H212" s="25" t="n">
+        <v>2940.33</v>
+      </c>
       <c r="I212" s="21">
         <f>IF(OR($B212="",$H212=""),"",IF($C212="LONG",($H212-$E212)*$F212,($E212-$H212)*$F212))</f>
         <v/>
       </c>
       <c r="J212" s="4" t="n">
-        <v>50.15</v>
+        <v>309.33</v>
       </c>
       <c r="K212" s="21">
         <f>IF(OR($B212="",$I212=""),"",$I212-IF($J212="",0,$J212))</f>
@@ -12096,7 +12132,7 @@
         <v/>
       </c>
       <c r="J213" s="4" t="n">
-        <v>0</v>
+        <v>305.76</v>
       </c>
       <c r="K213" s="21">
         <f>IF(OR($B213="",$I213=""),"",$I213-IF($J213="",0,$J213))</f>
@@ -12147,7 +12183,7 @@
         <v/>
       </c>
       <c r="J214" s="4" t="n">
-        <v>0</v>
+        <v>365.6</v>
       </c>
       <c r="K214" s="21">
         <f>IF(OR($B214="",$I214=""),"",$I214-IF($J214="",0,$J214))</f>
@@ -12163,19 +12199,43 @@
       </c>
     </row>
     <row r="215">
-      <c r="A215" s="23" t="n"/>
-      <c r="B215" s="23" t="n"/>
-      <c r="C215" s="23" t="n"/>
-      <c r="D215" s="24" t="n"/>
-      <c r="E215" s="25" t="n"/>
-      <c r="F215" s="26" t="n"/>
-      <c r="G215" s="24" t="n"/>
-      <c r="H215" s="25" t="n"/>
+      <c r="A215" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-221260924489209</t>
+        </is>
+      </c>
+      <c r="B215" s="23" t="inlineStr">
+        <is>
+          <t>ARVSMART</t>
+        </is>
+      </c>
+      <c r="C215" s="23" t="inlineStr">
+        <is>
+          <t>SHORT</t>
+        </is>
+      </c>
+      <c r="D215" s="24" t="n">
+        <v>46289</v>
+      </c>
+      <c r="E215" s="25" t="n">
+        <v>627.33</v>
+      </c>
+      <c r="F215" s="26" t="n">
+        <v>262</v>
+      </c>
+      <c r="G215" s="24" t="n">
+        <v>46289</v>
+      </c>
+      <c r="H215" s="25" t="n">
+        <v>624.98</v>
+      </c>
       <c r="I215" s="21">
         <f>IF(OR($B215="",$H215=""),"",IF($C215="LONG",($H215-$E215)*$F215,($E215-$H215)*$F215))</f>
         <v/>
       </c>
-      <c r="J215" s="4" t="n"/>
+      <c r="J215" s="4" t="n">
+        <v>0</v>
+      </c>
       <c r="K215" s="21">
         <f>IF(OR($B215="",$I215=""),"",$I215-IF($J215="",0,$J215))</f>
         <v/>
@@ -12190,19 +12250,39 @@
       </c>
     </row>
     <row r="216">
-      <c r="A216" s="23" t="n"/>
-      <c r="B216" s="23" t="n"/>
-      <c r="C216" s="23" t="n"/>
-      <c r="D216" s="24" t="n"/>
-      <c r="E216" s="25" t="n"/>
-      <c r="F216" s="26" t="n"/>
-      <c r="G216" s="24" t="n"/>
-      <c r="H216" s="25" t="n"/>
+      <c r="A216" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-34126092474909</t>
+        </is>
+      </c>
+      <c r="B216" s="23" t="inlineStr">
+        <is>
+          <t>AVANTEL</t>
+        </is>
+      </c>
+      <c r="C216" s="23" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="D216" s="24" t="n">
+        <v>46289</v>
+      </c>
+      <c r="E216" s="25" t="n">
+        <v>155.3422</v>
+      </c>
+      <c r="F216" s="26" t="n">
+        <v>1614</v>
+      </c>
+      <c r="G216" s="24" t="inlineStr"/>
+      <c r="H216" s="25" t="inlineStr"/>
       <c r="I216" s="21">
         <f>IF(OR($B216="",$H216=""),"",IF($C216="LONG",($H216-$E216)*$F216,($E216-$H216)*$F216))</f>
         <v/>
       </c>
-      <c r="J216" s="4" t="n"/>
+      <c r="J216" s="4" t="n">
+        <v>50.15</v>
+      </c>
       <c r="K216" s="21">
         <f>IF(OR($B216="",$I216=""),"",$I216-IF($J216="",0,$J216))</f>
         <v/>
@@ -12217,19 +12297,43 @@
       </c>
     </row>
     <row r="217">
-      <c r="A217" s="23" t="n"/>
-      <c r="B217" s="23" t="n"/>
-      <c r="C217" s="23" t="n"/>
-      <c r="D217" s="24" t="n"/>
-      <c r="E217" s="25" t="n"/>
-      <c r="F217" s="26" t="n"/>
-      <c r="G217" s="24" t="n"/>
-      <c r="H217" s="25" t="n"/>
+      <c r="A217" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-23126092413009</t>
+        </is>
+      </c>
+      <c r="B217" s="23" t="inlineStr">
+        <is>
+          <t>DELTACORP</t>
+        </is>
+      </c>
+      <c r="C217" s="23" t="inlineStr">
+        <is>
+          <t>SHORT</t>
+        </is>
+      </c>
+      <c r="D217" s="24" t="n">
+        <v>46289</v>
+      </c>
+      <c r="E217" s="25" t="n">
+        <v>71.06999999999999</v>
+      </c>
+      <c r="F217" s="26" t="n">
+        <v>2426</v>
+      </c>
+      <c r="G217" s="24" t="n">
+        <v>46289</v>
+      </c>
+      <c r="H217" s="25" t="n">
+        <v>72.55</v>
+      </c>
       <c r="I217" s="21">
         <f>IF(OR($B217="",$H217=""),"",IF($C217="LONG",($H217-$E217)*$F217,($E217-$H217)*$F217))</f>
         <v/>
       </c>
-      <c r="J217" s="4" t="n"/>
+      <c r="J217" s="4" t="n">
+        <v>0</v>
+      </c>
       <c r="K217" s="21">
         <f>IF(OR($B217="",$I217=""),"",$I217-IF($J217="",0,$J217))</f>
         <v/>
@@ -12244,19 +12348,39 @@
       </c>
     </row>
     <row r="218">
-      <c r="A218" s="23" t="n"/>
-      <c r="B218" s="23" t="n"/>
-      <c r="C218" s="23" t="n"/>
-      <c r="D218" s="24" t="n"/>
-      <c r="E218" s="25" t="n"/>
-      <c r="F218" s="26" t="n"/>
-      <c r="G218" s="24" t="n"/>
-      <c r="H218" s="25" t="n"/>
+      <c r="A218" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-limit_entry_multi</t>
+        </is>
+      </c>
+      <c r="B218" s="23" t="inlineStr">
+        <is>
+          <t>FRONTSP</t>
+        </is>
+      </c>
+      <c r="C218" s="23" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="D218" s="24" t="n">
+        <v>46289</v>
+      </c>
+      <c r="E218" s="25" t="n">
+        <v>1515.4085</v>
+      </c>
+      <c r="F218" s="26" t="n">
+        <v>82</v>
+      </c>
+      <c r="G218" s="24" t="inlineStr"/>
+      <c r="H218" s="25" t="inlineStr"/>
       <c r="I218" s="21">
         <f>IF(OR($B218="",$H218=""),"",IF($C218="LONG",($H218-$E218)*$F218,($E218-$H218)*$F218))</f>
         <v/>
       </c>
-      <c r="J218" s="4" t="n"/>
+      <c r="J218" s="4" t="n">
+        <v>14.75</v>
+      </c>
       <c r="K218" s="21">
         <f>IF(OR($B218="",$I218=""),"",$I218-IF($J218="",0,$J218))</f>
         <v/>
@@ -12271,19 +12395,43 @@
       </c>
     </row>
     <row r="219">
-      <c r="A219" s="23" t="n"/>
-      <c r="B219" s="23" t="n"/>
-      <c r="C219" s="23" t="n"/>
-      <c r="D219" s="24" t="n"/>
-      <c r="E219" s="25" t="n"/>
-      <c r="F219" s="26" t="n"/>
-      <c r="G219" s="24" t="n"/>
-      <c r="H219" s="25" t="n"/>
+      <c r="A219" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-321260924470909</t>
+        </is>
+      </c>
+      <c r="B219" s="23" t="inlineStr">
+        <is>
+          <t>GNA</t>
+        </is>
+      </c>
+      <c r="C219" s="23" t="inlineStr">
+        <is>
+          <t>SHORT</t>
+        </is>
+      </c>
+      <c r="D219" s="24" t="n">
+        <v>46289</v>
+      </c>
+      <c r="E219" s="25" t="n">
+        <v>634.42</v>
+      </c>
+      <c r="F219" s="26" t="n">
+        <v>139</v>
+      </c>
+      <c r="G219" s="24" t="n">
+        <v>46289</v>
+      </c>
+      <c r="H219" s="25" t="n">
+        <v>622.92</v>
+      </c>
       <c r="I219" s="21">
         <f>IF(OR($B219="",$H219=""),"",IF($C219="LONG",($H219-$E219)*$F219,($E219-$H219)*$F219))</f>
         <v/>
       </c>
-      <c r="J219" s="4" t="n"/>
+      <c r="J219" s="4" t="n">
+        <v>0</v>
+      </c>
       <c r="K219" s="21">
         <f>IF(OR($B219="",$I219=""),"",$I219-IF($J219="",0,$J219))</f>
         <v/>
@@ -12298,19 +12446,39 @@
       </c>
     </row>
     <row r="220">
-      <c r="A220" s="23" t="n"/>
-      <c r="B220" s="23" t="n"/>
-      <c r="C220" s="23" t="n"/>
-      <c r="D220" s="24" t="n"/>
-      <c r="E220" s="25" t="n"/>
-      <c r="F220" s="26" t="n"/>
-      <c r="G220" s="24" t="n"/>
-      <c r="H220" s="25" t="n"/>
+      <c r="A220" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-321260924764809</t>
+        </is>
+      </c>
+      <c r="B220" s="23" t="inlineStr">
+        <is>
+          <t>GREAVESCOT</t>
+        </is>
+      </c>
+      <c r="C220" s="23" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="D220" s="24" t="n">
+        <v>46289</v>
+      </c>
+      <c r="E220" s="25" t="n">
+        <v>221.6698</v>
+      </c>
+      <c r="F220" s="26" t="n">
+        <v>1128</v>
+      </c>
+      <c r="G220" s="24" t="inlineStr"/>
+      <c r="H220" s="25" t="inlineStr"/>
       <c r="I220" s="21">
         <f>IF(OR($B220="",$H220=""),"",IF($C220="LONG",($H220-$E220)*$F220,($E220-$H220)*$F220))</f>
         <v/>
       </c>
-      <c r="J220" s="4" t="n"/>
+      <c r="J220" s="4" t="n">
+        <v>50.15</v>
+      </c>
       <c r="K220" s="21">
         <f>IF(OR($B220="",$I220=""),"",$I220-IF($J220="",0,$J220))</f>
         <v/>
@@ -12325,19 +12493,39 @@
       </c>
     </row>
     <row r="221">
-      <c r="A221" s="23" t="n"/>
-      <c r="B221" s="23" t="n"/>
-      <c r="C221" s="23" t="n"/>
-      <c r="D221" s="24" t="n"/>
-      <c r="E221" s="25" t="n"/>
-      <c r="F221" s="26" t="n"/>
-      <c r="G221" s="24" t="n"/>
-      <c r="H221" s="25" t="n"/>
+      <c r="A221" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-221260924781709</t>
+        </is>
+      </c>
+      <c r="B221" s="23" t="inlineStr">
+        <is>
+          <t>INDIAGLYCO</t>
+        </is>
+      </c>
+      <c r="C221" s="23" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="D221" s="24" t="n">
+        <v>46289</v>
+      </c>
+      <c r="E221" s="25" t="n">
+        <v>304.3391</v>
+      </c>
+      <c r="F221" s="26" t="n">
+        <v>409</v>
+      </c>
+      <c r="G221" s="24" t="inlineStr"/>
+      <c r="H221" s="25" t="inlineStr"/>
       <c r="I221" s="21">
         <f>IF(OR($B221="",$H221=""),"",IF($C221="LONG",($H221-$E221)*$F221,($E221-$H221)*$F221))</f>
         <v/>
       </c>
-      <c r="J221" s="4" t="n"/>
+      <c r="J221" s="4" t="n">
+        <v>14.75</v>
+      </c>
       <c r="K221" s="21">
         <f>IF(OR($B221="",$I221=""),"",$I221-IF($J221="",0,$J221))</f>
         <v/>
@@ -12352,19 +12540,43 @@
       </c>
     </row>
     <row r="222">
-      <c r="A222" s="23" t="n"/>
-      <c r="B222" s="23" t="n"/>
-      <c r="C222" s="23" t="n"/>
-      <c r="D222" s="24" t="n"/>
-      <c r="E222" s="25" t="n"/>
-      <c r="F222" s="26" t="n"/>
-      <c r="G222" s="24" t="n"/>
-      <c r="H222" s="25" t="n"/>
+      <c r="A222" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-34126092446309</t>
+        </is>
+      </c>
+      <c r="B222" s="23" t="inlineStr">
+        <is>
+          <t>JAYKAY</t>
+        </is>
+      </c>
+      <c r="C222" s="23" t="inlineStr">
+        <is>
+          <t>SHORT</t>
+        </is>
+      </c>
+      <c r="D222" s="24" t="n">
+        <v>46289</v>
+      </c>
+      <c r="E222" s="25" t="n">
+        <v>205.66</v>
+      </c>
+      <c r="F222" s="26" t="n">
+        <v>780</v>
+      </c>
+      <c r="G222" s="24" t="n">
+        <v>46289</v>
+      </c>
+      <c r="H222" s="25" t="n">
+        <v>203.27</v>
+      </c>
       <c r="I222" s="21">
         <f>IF(OR($B222="",$H222=""),"",IF($C222="LONG",($H222-$E222)*$F222,($E222-$H222)*$F222))</f>
         <v/>
       </c>
-      <c r="J222" s="4" t="n"/>
+      <c r="J222" s="4" t="n">
+        <v>0</v>
+      </c>
       <c r="K222" s="21">
         <f>IF(OR($B222="",$I222=""),"",$I222-IF($J222="",0,$J222))</f>
         <v/>
@@ -12379,19 +12591,43 @@
       </c>
     </row>
     <row r="223">
-      <c r="A223" s="23" t="n"/>
-      <c r="B223" s="23" t="n"/>
-      <c r="C223" s="23" t="n"/>
-      <c r="D223" s="24" t="n"/>
-      <c r="E223" s="25" t="n"/>
-      <c r="F223" s="26" t="n"/>
-      <c r="G223" s="24" t="n"/>
-      <c r="H223" s="25" t="n"/>
+      <c r="A223" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-34126092446409</t>
+        </is>
+      </c>
+      <c r="B223" s="23" t="inlineStr">
+        <is>
+          <t>KROSS</t>
+        </is>
+      </c>
+      <c r="C223" s="23" t="inlineStr">
+        <is>
+          <t>SHORT</t>
+        </is>
+      </c>
+      <c r="D223" s="24" t="n">
+        <v>46289</v>
+      </c>
+      <c r="E223" s="25" t="n">
+        <v>273.1</v>
+      </c>
+      <c r="F223" s="26" t="n">
+        <v>597</v>
+      </c>
+      <c r="G223" s="24" t="n">
+        <v>46289</v>
+      </c>
+      <c r="H223" s="25" t="n">
+        <v>270.06</v>
+      </c>
       <c r="I223" s="21">
         <f>IF(OR($B223="",$H223=""),"",IF($C223="LONG",($H223-$E223)*$F223,($E223-$H223)*$F223))</f>
         <v/>
       </c>
-      <c r="J223" s="4" t="n"/>
+      <c r="J223" s="4" t="n">
+        <v>0</v>
+      </c>
       <c r="K223" s="21">
         <f>IF(OR($B223="",$I223=""),"",$I223-IF($J223="",0,$J223))</f>
         <v/>
@@ -12406,19 +12642,39 @@
       </c>
     </row>
     <row r="224">
-      <c r="A224" s="23" t="n"/>
-      <c r="B224" s="23" t="n"/>
-      <c r="C224" s="23" t="n"/>
-      <c r="D224" s="24" t="n"/>
-      <c r="E224" s="25" t="n"/>
-      <c r="F224" s="26" t="n"/>
-      <c r="G224" s="24" t="n"/>
-      <c r="H224" s="25" t="n"/>
+      <c r="A224" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-321260924764909</t>
+        </is>
+      </c>
+      <c r="B224" s="23" t="inlineStr">
+        <is>
+          <t>KSCL</t>
+        </is>
+      </c>
+      <c r="C224" s="23" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="D224" s="24" t="n">
+        <v>46289</v>
+      </c>
+      <c r="E224" s="25" t="n">
+        <v>783.6132</v>
+      </c>
+      <c r="F224" s="26" t="n">
+        <v>319</v>
+      </c>
+      <c r="G224" s="24" t="inlineStr"/>
+      <c r="H224" s="25" t="inlineStr"/>
       <c r="I224" s="21">
         <f>IF(OR($B224="",$H224=""),"",IF($C224="LONG",($H224-$E224)*$F224,($E224-$H224)*$F224))</f>
         <v/>
       </c>
-      <c r="J224" s="4" t="n"/>
+      <c r="J224" s="4" t="n">
+        <v>50.15</v>
+      </c>
       <c r="K224" s="21">
         <f>IF(OR($B224="",$I224=""),"",$I224-IF($J224="",0,$J224))</f>
         <v/>
@@ -12433,19 +12689,43 @@
       </c>
     </row>
     <row r="225">
-      <c r="A225" s="23" t="n"/>
-      <c r="B225" s="23" t="n"/>
-      <c r="C225" s="23" t="n"/>
-      <c r="D225" s="24" t="n"/>
-      <c r="E225" s="25" t="n"/>
-      <c r="F225" s="26" t="n"/>
-      <c r="G225" s="24" t="n"/>
-      <c r="H225" s="25" t="n"/>
+      <c r="A225" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-32126092463309</t>
+        </is>
+      </c>
+      <c r="B225" s="23" t="inlineStr">
+        <is>
+          <t>MUKANDLTD</t>
+        </is>
+      </c>
+      <c r="C225" s="23" t="inlineStr">
+        <is>
+          <t>SHORT</t>
+        </is>
+      </c>
+      <c r="D225" s="24" t="n">
+        <v>46289</v>
+      </c>
+      <c r="E225" s="25" t="n">
+        <v>157.54</v>
+      </c>
+      <c r="F225" s="26" t="n">
+        <v>1059</v>
+      </c>
+      <c r="G225" s="24" t="n">
+        <v>46289</v>
+      </c>
+      <c r="H225" s="25" t="n">
+        <v>155.92</v>
+      </c>
       <c r="I225" s="21">
         <f>IF(OR($B225="",$H225=""),"",IF($C225="LONG",($H225-$E225)*$F225,($E225-$H225)*$F225))</f>
         <v/>
       </c>
-      <c r="J225" s="4" t="n"/>
+      <c r="J225" s="4" t="n">
+        <v>0</v>
+      </c>
       <c r="K225" s="21">
         <f>IF(OR($B225="",$I225=""),"",$I225-IF($J225="",0,$J225))</f>
         <v/>
@@ -12460,19 +12740,43 @@
       </c>
     </row>
     <row r="226">
-      <c r="A226" s="23" t="n"/>
-      <c r="B226" s="23" t="n"/>
-      <c r="C226" s="23" t="n"/>
-      <c r="D226" s="24" t="n"/>
-      <c r="E226" s="25" t="n"/>
-      <c r="F226" s="26" t="n"/>
-      <c r="G226" s="24" t="n"/>
-      <c r="H226" s="25" t="n"/>
+      <c r="A226" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-34126092413109</t>
+        </is>
+      </c>
+      <c r="B226" s="23" t="inlineStr">
+        <is>
+          <t>ONEPOINT</t>
+        </is>
+      </c>
+      <c r="C226" s="23" t="inlineStr">
+        <is>
+          <t>SHORT</t>
+        </is>
+      </c>
+      <c r="D226" s="24" t="n">
+        <v>46289</v>
+      </c>
+      <c r="E226" s="25" t="n">
+        <v>71.53</v>
+      </c>
+      <c r="F226" s="26" t="n">
+        <v>2439</v>
+      </c>
+      <c r="G226" s="24" t="n">
+        <v>46289</v>
+      </c>
+      <c r="H226" s="25" t="n">
+        <v>69.06999999999999</v>
+      </c>
       <c r="I226" s="21">
         <f>IF(OR($B226="",$H226=""),"",IF($C226="LONG",($H226-$E226)*$F226,($E226-$H226)*$F226))</f>
         <v/>
       </c>
-      <c r="J226" s="4" t="n"/>
+      <c r="J226" s="4" t="n">
+        <v>0</v>
+      </c>
       <c r="K226" s="21">
         <f>IF(OR($B226="",$I226=""),"",$I226-IF($J226="",0,$J226))</f>
         <v/>
@@ -12487,19 +12791,39 @@
       </c>
     </row>
     <row r="227">
-      <c r="A227" s="23" t="n"/>
-      <c r="B227" s="23" t="n"/>
-      <c r="C227" s="23" t="n"/>
-      <c r="D227" s="24" t="n"/>
-      <c r="E227" s="25" t="n"/>
-      <c r="F227" s="26" t="n"/>
-      <c r="G227" s="24" t="n"/>
-      <c r="H227" s="25" t="n"/>
+      <c r="A227" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-34126092475009</t>
+        </is>
+      </c>
+      <c r="B227" s="23" t="inlineStr">
+        <is>
+          <t>RAYMONDREL</t>
+        </is>
+      </c>
+      <c r="C227" s="23" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="D227" s="24" t="n">
+        <v>46289</v>
+      </c>
+      <c r="E227" s="25" t="n">
+        <v>708.4741</v>
+      </c>
+      <c r="F227" s="26" t="n">
+        <v>176</v>
+      </c>
+      <c r="G227" s="24" t="inlineStr"/>
+      <c r="H227" s="25" t="inlineStr"/>
       <c r="I227" s="21">
         <f>IF(OR($B227="",$H227=""),"",IF($C227="LONG",($H227-$E227)*$F227,($E227-$H227)*$F227))</f>
         <v/>
       </c>
-      <c r="J227" s="4" t="n"/>
+      <c r="J227" s="4" t="n">
+        <v>14.75</v>
+      </c>
       <c r="K227" s="21">
         <f>IF(OR($B227="",$I227=""),"",$I227-IF($J227="",0,$J227))</f>
         <v/>
@@ -12514,19 +12838,43 @@
       </c>
     </row>
     <row r="228">
-      <c r="A228" s="23" t="n"/>
-      <c r="B228" s="23" t="n"/>
-      <c r="C228" s="23" t="n"/>
-      <c r="D228" s="24" t="n"/>
-      <c r="E228" s="25" t="n"/>
-      <c r="F228" s="26" t="n"/>
-      <c r="G228" s="24" t="n"/>
-      <c r="H228" s="25" t="n"/>
+      <c r="A228" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-23126092413109</t>
+        </is>
+      </c>
+      <c r="B228" s="23" t="inlineStr">
+        <is>
+          <t>RAYMONDREL</t>
+        </is>
+      </c>
+      <c r="C228" s="23" t="inlineStr">
+        <is>
+          <t>SHORT</t>
+        </is>
+      </c>
+      <c r="D228" s="24" t="n">
+        <v>46289</v>
+      </c>
+      <c r="E228" s="25" t="n">
+        <v>677.0599999999999</v>
+      </c>
+      <c r="F228" s="26" t="n">
+        <v>246</v>
+      </c>
+      <c r="G228" s="24" t="n">
+        <v>46289</v>
+      </c>
+      <c r="H228" s="25" t="n">
+        <v>704</v>
+      </c>
       <c r="I228" s="21">
         <f>IF(OR($B228="",$H228=""),"",IF($C228="LONG",($H228-$E228)*$F228,($E228-$H228)*$F228))</f>
         <v/>
       </c>
-      <c r="J228" s="4" t="n"/>
+      <c r="J228" s="4" t="n">
+        <v>0</v>
+      </c>
       <c r="K228" s="21">
         <f>IF(OR($B228="",$I228=""),"",$I228-IF($J228="",0,$J228))</f>
         <v/>
@@ -12541,19 +12889,43 @@
       </c>
     </row>
     <row r="229">
-      <c r="A229" s="23" t="n"/>
-      <c r="B229" s="23" t="n"/>
-      <c r="C229" s="23" t="n"/>
-      <c r="D229" s="24" t="n"/>
-      <c r="E229" s="25" t="n"/>
-      <c r="F229" s="26" t="n"/>
-      <c r="G229" s="24" t="n"/>
-      <c r="H229" s="25" t="n"/>
+      <c r="A229" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-221260924489309</t>
+        </is>
+      </c>
+      <c r="B229" s="23" t="inlineStr">
+        <is>
+          <t>RPGLIFE</t>
+        </is>
+      </c>
+      <c r="C229" s="23" t="inlineStr">
+        <is>
+          <t>SHORT</t>
+        </is>
+      </c>
+      <c r="D229" s="24" t="n">
+        <v>46289</v>
+      </c>
+      <c r="E229" s="25" t="n">
+        <v>2938.97</v>
+      </c>
+      <c r="F229" s="26" t="n">
+        <v>55</v>
+      </c>
+      <c r="G229" s="24" t="n">
+        <v>46289</v>
+      </c>
+      <c r="H229" s="25" t="n">
+        <v>2914.96</v>
+      </c>
       <c r="I229" s="21">
         <f>IF(OR($B229="",$H229=""),"",IF($C229="LONG",($H229-$E229)*$F229,($E229-$H229)*$F229))</f>
         <v/>
       </c>
-      <c r="J229" s="4" t="n"/>
+      <c r="J229" s="4" t="n">
+        <v>0</v>
+      </c>
       <c r="K229" s="21">
         <f>IF(OR($B229="",$I229=""),"",$I229-IF($J229="",0,$J229))</f>
         <v/>
@@ -33896,7 +34268,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J103"/>
+  <dimension ref="A1:J108"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -34238,7 +34610,7 @@
     <row r="10">
       <c r="A10" s="27" t="inlineStr">
         <is>
-          <t>AWFIS</t>
+          <t>AVANTEL</t>
         </is>
       </c>
       <c r="B10" s="20">
@@ -34281,7 +34653,7 @@
     <row r="11">
       <c r="A11" s="27" t="inlineStr">
         <is>
-          <t>BAJAJHIND</t>
+          <t>AWFIS</t>
         </is>
       </c>
       <c r="B11" s="20">
@@ -34324,7 +34696,7 @@
     <row r="12">
       <c r="A12" s="27" t="inlineStr">
         <is>
-          <t>BANARISUG</t>
+          <t>BAJAJHIND</t>
         </is>
       </c>
       <c r="B12" s="20">
@@ -34367,7 +34739,7 @@
     <row r="13">
       <c r="A13" s="27" t="inlineStr">
         <is>
-          <t>BCG</t>
+          <t>BANARISUG</t>
         </is>
       </c>
       <c r="B13" s="20">
@@ -34410,7 +34782,7 @@
     <row r="14">
       <c r="A14" s="27" t="inlineStr">
         <is>
-          <t>BFUTILITIE</t>
+          <t>BCG</t>
         </is>
       </c>
       <c r="B14" s="20">
@@ -34453,7 +34825,7 @@
     <row r="15">
       <c r="A15" s="27" t="inlineStr">
         <is>
-          <t>BOMDYEING</t>
+          <t>BFUTILITIE</t>
         </is>
       </c>
       <c r="B15" s="20">
@@ -34496,7 +34868,7 @@
     <row r="16">
       <c r="A16" s="27" t="inlineStr">
         <is>
-          <t>CHEMPLASTS</t>
+          <t>BOMDYEING</t>
         </is>
       </c>
       <c r="B16" s="20">
@@ -34539,7 +34911,7 @@
     <row r="17">
       <c r="A17" s="27" t="inlineStr">
         <is>
-          <t>DELTACORP</t>
+          <t>CHEMPLASTS</t>
         </is>
       </c>
       <c r="B17" s="20">
@@ -34582,7 +34954,7 @@
     <row r="18">
       <c r="A18" s="27" t="inlineStr">
         <is>
-          <t>EIEL</t>
+          <t>DELTACORP</t>
         </is>
       </c>
       <c r="B18" s="20">
@@ -34625,7 +34997,7 @@
     <row r="19">
       <c r="A19" s="27" t="inlineStr">
         <is>
-          <t>EMUDHRA</t>
+          <t>EIEL</t>
         </is>
       </c>
       <c r="B19" s="20">
@@ -34668,7 +35040,7 @@
     <row r="20">
       <c r="A20" s="27" t="inlineStr">
         <is>
-          <t>FILATEX</t>
+          <t>EMUDHRA</t>
         </is>
       </c>
       <c r="B20" s="20">
@@ -34711,7 +35083,7 @@
     <row r="21">
       <c r="A21" s="27" t="inlineStr">
         <is>
-          <t>FMGOETZE</t>
+          <t>FILATEX</t>
         </is>
       </c>
       <c r="B21" s="20">
@@ -34754,7 +35126,7 @@
     <row r="22">
       <c r="A22" s="27" t="inlineStr">
         <is>
-          <t>FOSECOIND</t>
+          <t>FMGOETZE</t>
         </is>
       </c>
       <c r="B22" s="20">
@@ -34797,7 +35169,7 @@
     <row r="23">
       <c r="A23" s="27" t="inlineStr">
         <is>
-          <t>GKENERGY</t>
+          <t>FOSECOIND</t>
         </is>
       </c>
       <c r="B23" s="20">
@@ -34840,7 +35212,7 @@
     <row r="24">
       <c r="A24" s="27" t="inlineStr">
         <is>
-          <t>GNA</t>
+          <t>FRONTSP</t>
         </is>
       </c>
       <c r="B24" s="20">
@@ -34883,7 +35255,7 @@
     <row r="25">
       <c r="A25" s="27" t="inlineStr">
         <is>
-          <t>GNRL</t>
+          <t>GKENERGY</t>
         </is>
       </c>
       <c r="B25" s="20">
@@ -34926,7 +35298,7 @@
     <row r="26">
       <c r="A26" s="27" t="inlineStr">
         <is>
-          <t>GOCLCORP</t>
+          <t>GNA</t>
         </is>
       </c>
       <c r="B26" s="20">
@@ -34969,7 +35341,7 @@
     <row r="27">
       <c r="A27" s="27" t="inlineStr">
         <is>
-          <t>GOPAL</t>
+          <t>GNRL</t>
         </is>
       </c>
       <c r="B27" s="20">
@@ -35012,7 +35384,7 @@
     <row r="28">
       <c r="A28" s="27" t="inlineStr">
         <is>
-          <t>GRAUWEIL</t>
+          <t>GOCLCORP</t>
         </is>
       </c>
       <c r="B28" s="20">
@@ -35055,7 +35427,7 @@
     <row r="29">
       <c r="A29" s="27" t="inlineStr">
         <is>
-          <t>GUJTHEM</t>
+          <t>GOPAL</t>
         </is>
       </c>
       <c r="B29" s="20">
@@ -35098,7 +35470,7 @@
     <row r="30">
       <c r="A30" s="27" t="inlineStr">
         <is>
-          <t>HERITGFOOD</t>
+          <t>GRAUWEIL</t>
         </is>
       </c>
       <c r="B30" s="20">
@@ -35141,7 +35513,7 @@
     <row r="31">
       <c r="A31" s="27" t="inlineStr">
         <is>
-          <t>HIKAL</t>
+          <t>GREAVESCOT</t>
         </is>
       </c>
       <c r="B31" s="20">
@@ -35184,7 +35556,7 @@
     <row r="32">
       <c r="A32" s="27" t="inlineStr">
         <is>
-          <t>HINDOILEXP</t>
+          <t>GUJTHEM</t>
         </is>
       </c>
       <c r="B32" s="20">
@@ -35227,7 +35599,7 @@
     <row r="33">
       <c r="A33" s="27" t="inlineStr">
         <is>
-          <t>HUBTOWN</t>
+          <t>HERITGFOOD</t>
         </is>
       </c>
       <c r="B33" s="20">
@@ -35270,7 +35642,7 @@
     <row r="34">
       <c r="A34" s="27" t="inlineStr">
         <is>
-          <t>INDNIPPON</t>
+          <t>HIKAL</t>
         </is>
       </c>
       <c r="B34" s="20">
@@ -35313,7 +35685,7 @@
     <row r="35">
       <c r="A35" s="27" t="inlineStr">
         <is>
-          <t>INDOCO</t>
+          <t>HINDOILEXP</t>
         </is>
       </c>
       <c r="B35" s="20">
@@ -35356,7 +35728,7 @@
     <row r="36">
       <c r="A36" s="27" t="inlineStr">
         <is>
-          <t>INDORAMA</t>
+          <t>HUBTOWN</t>
         </is>
       </c>
       <c r="B36" s="20">
@@ -35399,7 +35771,7 @@
     <row r="37">
       <c r="A37" s="27" t="inlineStr">
         <is>
-          <t>IPL</t>
+          <t>INDIAGLYCO</t>
         </is>
       </c>
       <c r="B37" s="20">
@@ -35442,7 +35814,7 @@
     <row r="38">
       <c r="A38" s="27" t="inlineStr">
         <is>
-          <t>JASH</t>
+          <t>INDNIPPON</t>
         </is>
       </c>
       <c r="B38" s="20">
@@ -35485,7 +35857,7 @@
     <row r="39">
       <c r="A39" s="27" t="inlineStr">
         <is>
-          <t>JAYKAY</t>
+          <t>INDOCO</t>
         </is>
       </c>
       <c r="B39" s="20">
@@ -35528,7 +35900,7 @@
     <row r="40">
       <c r="A40" s="27" t="inlineStr">
         <is>
-          <t>JGCHEM</t>
+          <t>INDORAMA</t>
         </is>
       </c>
       <c r="B40" s="20">
@@ -35571,7 +35943,7 @@
     <row r="41">
       <c r="A41" s="27" t="inlineStr">
         <is>
-          <t>KCP</t>
+          <t>IPL</t>
         </is>
       </c>
       <c r="B41" s="20">
@@ -35614,7 +35986,7 @@
     <row r="42">
       <c r="A42" s="27" t="inlineStr">
         <is>
-          <t>KIRIINDUS</t>
+          <t>JASH</t>
         </is>
       </c>
       <c r="B42" s="20">
@@ -35657,7 +36029,7 @@
     <row r="43">
       <c r="A43" s="27" t="inlineStr">
         <is>
-          <t>KIRLOSIND</t>
+          <t>JAYKAY</t>
         </is>
       </c>
       <c r="B43" s="20">
@@ -35700,7 +36072,7 @@
     <row r="44">
       <c r="A44" s="27" t="inlineStr">
         <is>
-          <t>KLBRENG-B</t>
+          <t>JGCHEM</t>
         </is>
       </c>
       <c r="B44" s="20">
@@ -35743,7 +36115,7 @@
     <row r="45">
       <c r="A45" s="27" t="inlineStr">
         <is>
-          <t>KROSS</t>
+          <t>KCP</t>
         </is>
       </c>
       <c r="B45" s="20">
@@ -35786,7 +36158,7 @@
     <row r="46">
       <c r="A46" s="27" t="inlineStr">
         <is>
-          <t>KSL</t>
+          <t>KIRIINDUS</t>
         </is>
       </c>
       <c r="B46" s="20">
@@ -35829,7 +36201,7 @@
     <row r="47">
       <c r="A47" s="27" t="inlineStr">
         <is>
-          <t>LUXIND</t>
+          <t>KIRLOSIND</t>
         </is>
       </c>
       <c r="B47" s="20">
@@ -35872,7 +36244,7 @@
     <row r="48">
       <c r="A48" s="27" t="inlineStr">
         <is>
-          <t>MAITHANALL</t>
+          <t>KLBRENG-B</t>
         </is>
       </c>
       <c r="B48" s="20">
@@ -35915,7 +36287,7 @@
     <row r="49">
       <c r="A49" s="27" t="inlineStr">
         <is>
-          <t>MANGLMCEM</t>
+          <t>KROSS</t>
         </is>
       </c>
       <c r="B49" s="20">
@@ -35958,7 +36330,7 @@
     <row r="50">
       <c r="A50" s="27" t="inlineStr">
         <is>
-          <t>MASTEK</t>
+          <t>KSCL</t>
         </is>
       </c>
       <c r="B50" s="20">
@@ -36001,7 +36373,7 @@
     <row r="51">
       <c r="A51" s="27" t="inlineStr">
         <is>
-          <t>MOBIKWIK</t>
+          <t>KSL</t>
         </is>
       </c>
       <c r="B51" s="20">
@@ -36044,7 +36416,7 @@
     <row r="52">
       <c r="A52" s="27" t="inlineStr">
         <is>
-          <t>MUKANDLTD</t>
+          <t>LUXIND</t>
         </is>
       </c>
       <c r="B52" s="20">
@@ -36087,7 +36459,7 @@
     <row r="53">
       <c r="A53" s="27" t="inlineStr">
         <is>
-          <t>NETWORK18</t>
+          <t>MAITHANALL</t>
         </is>
       </c>
       <c r="B53" s="20">
@@ -36130,7 +36502,7 @@
     <row r="54">
       <c r="A54" s="27" t="inlineStr">
         <is>
-          <t>NILKAMAL</t>
+          <t>MANGLMCEM</t>
         </is>
       </c>
       <c r="B54" s="20">
@@ -36173,7 +36545,7 @@
     <row r="55">
       <c r="A55" s="27" t="inlineStr">
         <is>
-          <t>NORTHARC</t>
+          <t>MASTEK</t>
         </is>
       </c>
       <c r="B55" s="20">
@@ -36216,7 +36588,7 @@
     <row r="56">
       <c r="A56" s="27" t="inlineStr">
         <is>
-          <t>NOVARTIND</t>
+          <t>MOBIKWIK</t>
         </is>
       </c>
       <c r="B56" s="20">
@@ -36259,7 +36631,7 @@
     <row r="57">
       <c r="A57" s="27" t="inlineStr">
         <is>
-          <t>NPST</t>
+          <t>MUKANDLTD</t>
         </is>
       </c>
       <c r="B57" s="20">
@@ -36302,7 +36674,7 @@
     <row r="58">
       <c r="A58" s="27" t="inlineStr">
         <is>
-          <t>NRBBEARING</t>
+          <t>NETWORK18</t>
         </is>
       </c>
       <c r="B58" s="20">
@@ -36345,7 +36717,7 @@
     <row r="59">
       <c r="A59" s="27" t="inlineStr">
         <is>
-          <t>OMAXE</t>
+          <t>NILKAMAL</t>
         </is>
       </c>
       <c r="B59" s="20">
@@ -36388,7 +36760,7 @@
     <row r="60">
       <c r="A60" s="27" t="inlineStr">
         <is>
-          <t>ONEPOINT</t>
+          <t>NORTHARC</t>
         </is>
       </c>
       <c r="B60" s="20">
@@ -36431,7 +36803,7 @@
     <row r="61">
       <c r="A61" s="27" t="inlineStr">
         <is>
-          <t>OPTIEMUS</t>
+          <t>NOVARTIND</t>
         </is>
       </c>
       <c r="B61" s="20">
@@ -36474,7 +36846,7 @@
     <row r="62">
       <c r="A62" s="27" t="inlineStr">
         <is>
-          <t>ORIENTHOT</t>
+          <t>NPST</t>
         </is>
       </c>
       <c r="B62" s="20">
@@ -36517,7 +36889,7 @@
     <row r="63">
       <c r="A63" s="27" t="inlineStr">
         <is>
-          <t>PACEDIGITK</t>
+          <t>NRBBEARING</t>
         </is>
       </c>
       <c r="B63" s="20">
@@ -36560,7 +36932,7 @@
     <row r="64">
       <c r="A64" s="27" t="inlineStr">
         <is>
-          <t>PITTIENG</t>
+          <t>OMAXE</t>
         </is>
       </c>
       <c r="B64" s="20">
@@ -36603,7 +36975,7 @@
     <row r="65">
       <c r="A65" s="27" t="inlineStr">
         <is>
-          <t>PROTEAN</t>
+          <t>ONEPOINT</t>
         </is>
       </c>
       <c r="B65" s="20">
@@ -36646,7 +37018,7 @@
     <row r="66">
       <c r="A66" s="27" t="inlineStr">
         <is>
-          <t>QUADFUTURE</t>
+          <t>OPTIEMUS</t>
         </is>
       </c>
       <c r="B66" s="20">
@@ -36689,7 +37061,7 @@
     <row r="67">
       <c r="A67" s="27" t="inlineStr">
         <is>
-          <t>RACLGEAR</t>
+          <t>ORIENTHOT</t>
         </is>
       </c>
       <c r="B67" s="20">
@@ -36732,7 +37104,7 @@
     <row r="68">
       <c r="A68" s="27" t="inlineStr">
         <is>
-          <t>RAMRAT</t>
+          <t>PACEDIGITK</t>
         </is>
       </c>
       <c r="B68" s="20">
@@ -36775,7 +37147,7 @@
     <row r="69">
       <c r="A69" s="27" t="inlineStr">
         <is>
-          <t>RAYMOND</t>
+          <t>PITTIENG</t>
         </is>
       </c>
       <c r="B69" s="20">
@@ -36818,7 +37190,7 @@
     <row r="70">
       <c r="A70" s="27" t="inlineStr">
         <is>
-          <t>RAYMONDREL</t>
+          <t>PROTEAN</t>
         </is>
       </c>
       <c r="B70" s="20">
@@ -36861,7 +37233,7 @@
     <row r="71">
       <c r="A71" s="27" t="inlineStr">
         <is>
-          <t>REFEX</t>
+          <t>QUADFUTURE</t>
         </is>
       </c>
       <c r="B71" s="20">
@@ -36904,7 +37276,7 @@
     <row r="72">
       <c r="A72" s="27" t="inlineStr">
         <is>
-          <t>RESPONIND</t>
+          <t>RACLGEAR</t>
         </is>
       </c>
       <c r="B72" s="20">
@@ -36947,7 +37319,7 @@
     <row r="73">
       <c r="A73" s="27" t="inlineStr">
         <is>
-          <t>RML</t>
+          <t>RAMRAT</t>
         </is>
       </c>
       <c r="B73" s="20">
@@ -36990,7 +37362,7 @@
     <row r="74">
       <c r="A74" s="27" t="inlineStr">
         <is>
-          <t>ROSSTECH</t>
+          <t>RAYMOND</t>
         </is>
       </c>
       <c r="B74" s="20">
@@ -37033,7 +37405,7 @@
     <row r="75">
       <c r="A75" s="27" t="inlineStr">
         <is>
-          <t>RPGLIFE</t>
+          <t>RAYMONDREL</t>
         </is>
       </c>
       <c r="B75" s="20">
@@ -37076,7 +37448,7 @@
     <row r="76">
       <c r="A76" s="27" t="inlineStr">
         <is>
-          <t>SAATVIKGL</t>
+          <t>REFEX</t>
         </is>
       </c>
       <c r="B76" s="20">
@@ -37119,7 +37491,7 @@
     <row r="77">
       <c r="A77" s="27" t="inlineStr">
         <is>
-          <t>SAKAR</t>
+          <t>RESPONIND</t>
         </is>
       </c>
       <c r="B77" s="20">
@@ -37162,7 +37534,7 @@
     <row r="78">
       <c r="A78" s="27" t="inlineStr">
         <is>
-          <t>SAMBHV</t>
+          <t>RML</t>
         </is>
       </c>
       <c r="B78" s="20">
@@ -37205,7 +37577,7 @@
     <row r="79">
       <c r="A79" s="27" t="inlineStr">
         <is>
-          <t>SAMHI</t>
+          <t>ROSSTECH</t>
         </is>
       </c>
       <c r="B79" s="20">
@@ -37248,7 +37620,7 @@
     <row r="80">
       <c r="A80" s="27" t="inlineStr">
         <is>
-          <t>SHAREINDIA</t>
+          <t>RPGLIFE</t>
         </is>
       </c>
       <c r="B80" s="20">
@@ -37291,7 +37663,7 @@
     <row r="81">
       <c r="A81" s="27" t="inlineStr">
         <is>
-          <t>SIKA</t>
+          <t>SAATVIKGL</t>
         </is>
       </c>
       <c r="B81" s="20">
@@ -37334,7 +37706,7 @@
     <row r="82">
       <c r="A82" s="27" t="inlineStr">
         <is>
-          <t>SINDHUTRAD</t>
+          <t>SAKAR</t>
         </is>
       </c>
       <c r="B82" s="20">
@@ -37377,7 +37749,7 @@
     <row r="83">
       <c r="A83" s="27" t="inlineStr">
         <is>
-          <t>SMSPHARMA</t>
+          <t>SAMBHV</t>
         </is>
       </c>
       <c r="B83" s="20">
@@ -37420,7 +37792,7 @@
     <row r="84">
       <c r="A84" s="27" t="inlineStr">
         <is>
-          <t>SOLARA</t>
+          <t>SAMHI</t>
         </is>
       </c>
       <c r="B84" s="20">
@@ -37463,7 +37835,7 @@
     <row r="85">
       <c r="A85" s="27" t="inlineStr">
         <is>
-          <t>SOTL</t>
+          <t>SHAREINDIA</t>
         </is>
       </c>
       <c r="B85" s="20">
@@ -37506,7 +37878,7 @@
     <row r="86">
       <c r="A86" s="27" t="inlineStr">
         <is>
-          <t>SSWL</t>
+          <t>SIKA</t>
         </is>
       </c>
       <c r="B86" s="20">
@@ -37549,7 +37921,7 @@
     <row r="87">
       <c r="A87" s="27" t="inlineStr">
         <is>
-          <t>STEELCAS</t>
+          <t>SINDHUTRAD</t>
         </is>
       </c>
       <c r="B87" s="20">
@@ -37592,7 +37964,7 @@
     <row r="88">
       <c r="A88" s="27" t="inlineStr">
         <is>
-          <t>SYMPHONY</t>
+          <t>SMSPHARMA</t>
         </is>
       </c>
       <c r="B88" s="20">
@@ -37635,7 +38007,7 @@
     <row r="89">
       <c r="A89" s="27" t="inlineStr">
         <is>
-          <t>SYNCOMF</t>
+          <t>SOLARA</t>
         </is>
       </c>
       <c r="B89" s="20">
@@ -37678,7 +38050,7 @@
     <row r="90">
       <c r="A90" s="27" t="inlineStr">
         <is>
-          <t>TALBROAUTO</t>
+          <t>SOTL</t>
         </is>
       </c>
       <c r="B90" s="20">
@@ -37721,7 +38093,7 @@
     <row r="91">
       <c r="A91" s="27" t="inlineStr">
         <is>
-          <t>TBZ</t>
+          <t>SSWL</t>
         </is>
       </c>
       <c r="B91" s="20">
@@ -37764,7 +38136,7 @@
     <row r="92">
       <c r="A92" s="27" t="inlineStr">
         <is>
-          <t>THOMASCOOK</t>
+          <t>STEELCAS</t>
         </is>
       </c>
       <c r="B92" s="20">
@@ -37807,7 +38179,7 @@
     <row r="93">
       <c r="A93" s="27" t="inlineStr">
         <is>
-          <t>VENKEYS</t>
+          <t>SYMPHONY</t>
         </is>
       </c>
       <c r="B93" s="20">
@@ -37850,7 +38222,7 @@
     <row r="94">
       <c r="A94" s="27" t="inlineStr">
         <is>
-          <t>VENUSPIPES</t>
+          <t>SYNCOMF</t>
         </is>
       </c>
       <c r="B94" s="20">
@@ -37893,7 +38265,7 @@
     <row r="95">
       <c r="A95" s="27" t="inlineStr">
         <is>
-          <t>VERANDA</t>
+          <t>TALBROAUTO</t>
         </is>
       </c>
       <c r="B95" s="20">
@@ -37936,7 +38308,7 @@
     <row r="96">
       <c r="A96" s="27" t="inlineStr">
         <is>
-          <t>VSSL</t>
+          <t>TBZ</t>
         </is>
       </c>
       <c r="B96" s="20">
@@ -37979,7 +38351,7 @@
     <row r="97">
       <c r="A97" s="27" t="inlineStr">
         <is>
-          <t>WELSPLSOL</t>
+          <t>THOMASCOOK</t>
         </is>
       </c>
       <c r="B97" s="20">
@@ -38022,7 +38394,7 @@
     <row r="98">
       <c r="A98" s="27" t="inlineStr">
         <is>
-          <t>WENDT</t>
+          <t>VENKEYS</t>
         </is>
       </c>
       <c r="B98" s="20">
@@ -38065,7 +38437,7 @@
     <row r="99">
       <c r="A99" s="27" t="inlineStr">
         <is>
-          <t>WINDLAS</t>
+          <t>VENUSPIPES</t>
         </is>
       </c>
       <c r="B99" s="20">
@@ -38108,7 +38480,7 @@
     <row r="100">
       <c r="A100" s="27" t="inlineStr">
         <is>
-          <t>XPROINDIA</t>
+          <t>VERANDA</t>
         </is>
       </c>
       <c r="B100" s="20">
@@ -38151,7 +38523,7 @@
     <row r="101">
       <c r="A101" s="27" t="inlineStr">
         <is>
-          <t>ZAGGLE</t>
+          <t>VSSL</t>
         </is>
       </c>
       <c r="B101" s="20">
@@ -38194,7 +38566,7 @@
     <row r="102">
       <c r="A102" s="27" t="inlineStr">
         <is>
-          <t>ZOTA</t>
+          <t>WELSPLSOL</t>
         </is>
       </c>
       <c r="B102" s="20">
@@ -38235,37 +38607,252 @@
       </c>
     </row>
     <row r="103">
-      <c r="A103" s="3" t="inlineStr">
+      <c r="A103" s="27" t="inlineStr">
+        <is>
+          <t>WENDT</t>
+        </is>
+      </c>
+      <c r="B103" s="20">
+        <f>COUNTIF('Trade Log'!$B$4:$B$503,$A103)</f>
+        <v/>
+      </c>
+      <c r="C103" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A103,'Trade Log'!$K$4:$K$503,"&gt;0")</f>
+        <v/>
+      </c>
+      <c r="D103" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A103,'Trade Log'!$K$4:$K$503,"&lt;0")</f>
+        <v/>
+      </c>
+      <c r="E103" s="29">
+        <f>IFERROR($C103/$B103,"")</f>
+        <v/>
+      </c>
+      <c r="F103" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A103,'Trade Log'!$I$4:$I$503)</f>
+        <v/>
+      </c>
+      <c r="G103" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A103,'Trade Log'!$K$4:$K$503)</f>
+        <v/>
+      </c>
+      <c r="H103" s="21">
+        <f>IFERROR($G103/$B103,"")</f>
+        <v/>
+      </c>
+      <c r="I103" s="21">
+        <f>IFERROR(_xlfn.MAXIFS('Trade Log'!$K$4:$K$503,'Trade Log'!$B$4:$B$503,$A103),"")</f>
+        <v/>
+      </c>
+      <c r="J103" s="21">
+        <f>IFERROR(_xlfn.MINIFS('Trade Log'!$K$4:$K$503,'Trade Log'!$B$4:$B$503,$A103),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" s="27" t="inlineStr">
+        <is>
+          <t>WINDLAS</t>
+        </is>
+      </c>
+      <c r="B104" s="20">
+        <f>COUNTIF('Trade Log'!$B$4:$B$503,$A104)</f>
+        <v/>
+      </c>
+      <c r="C104" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A104,'Trade Log'!$K$4:$K$503,"&gt;0")</f>
+        <v/>
+      </c>
+      <c r="D104" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A104,'Trade Log'!$K$4:$K$503,"&lt;0")</f>
+        <v/>
+      </c>
+      <c r="E104" s="29">
+        <f>IFERROR($C104/$B104,"")</f>
+        <v/>
+      </c>
+      <c r="F104" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A104,'Trade Log'!$I$4:$I$503)</f>
+        <v/>
+      </c>
+      <c r="G104" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A104,'Trade Log'!$K$4:$K$503)</f>
+        <v/>
+      </c>
+      <c r="H104" s="21">
+        <f>IFERROR($G104/$B104,"")</f>
+        <v/>
+      </c>
+      <c r="I104" s="21">
+        <f>IFERROR(_xlfn.MAXIFS('Trade Log'!$K$4:$K$503,'Trade Log'!$B$4:$B$503,$A104),"")</f>
+        <v/>
+      </c>
+      <c r="J104" s="21">
+        <f>IFERROR(_xlfn.MINIFS('Trade Log'!$K$4:$K$503,'Trade Log'!$B$4:$B$503,$A104),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" s="27" t="inlineStr">
+        <is>
+          <t>XPROINDIA</t>
+        </is>
+      </c>
+      <c r="B105" s="20">
+        <f>COUNTIF('Trade Log'!$B$4:$B$503,$A105)</f>
+        <v/>
+      </c>
+      <c r="C105" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A105,'Trade Log'!$K$4:$K$503,"&gt;0")</f>
+        <v/>
+      </c>
+      <c r="D105" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A105,'Trade Log'!$K$4:$K$503,"&lt;0")</f>
+        <v/>
+      </c>
+      <c r="E105" s="29">
+        <f>IFERROR($C105/$B105,"")</f>
+        <v/>
+      </c>
+      <c r="F105" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A105,'Trade Log'!$I$4:$I$503)</f>
+        <v/>
+      </c>
+      <c r="G105" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A105,'Trade Log'!$K$4:$K$503)</f>
+        <v/>
+      </c>
+      <c r="H105" s="21">
+        <f>IFERROR($G105/$B105,"")</f>
+        <v/>
+      </c>
+      <c r="I105" s="21">
+        <f>IFERROR(_xlfn.MAXIFS('Trade Log'!$K$4:$K$503,'Trade Log'!$B$4:$B$503,$A105),"")</f>
+        <v/>
+      </c>
+      <c r="J105" s="21">
+        <f>IFERROR(_xlfn.MINIFS('Trade Log'!$K$4:$K$503,'Trade Log'!$B$4:$B$503,$A105),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" s="27" t="inlineStr">
+        <is>
+          <t>ZAGGLE</t>
+        </is>
+      </c>
+      <c r="B106" s="20">
+        <f>COUNTIF('Trade Log'!$B$4:$B$503,$A106)</f>
+        <v/>
+      </c>
+      <c r="C106" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A106,'Trade Log'!$K$4:$K$503,"&gt;0")</f>
+        <v/>
+      </c>
+      <c r="D106" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A106,'Trade Log'!$K$4:$K$503,"&lt;0")</f>
+        <v/>
+      </c>
+      <c r="E106" s="29">
+        <f>IFERROR($C106/$B106,"")</f>
+        <v/>
+      </c>
+      <c r="F106" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A106,'Trade Log'!$I$4:$I$503)</f>
+        <v/>
+      </c>
+      <c r="G106" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A106,'Trade Log'!$K$4:$K$503)</f>
+        <v/>
+      </c>
+      <c r="H106" s="21">
+        <f>IFERROR($G106/$B106,"")</f>
+        <v/>
+      </c>
+      <c r="I106" s="21">
+        <f>IFERROR(_xlfn.MAXIFS('Trade Log'!$K$4:$K$503,'Trade Log'!$B$4:$B$503,$A106),"")</f>
+        <v/>
+      </c>
+      <c r="J106" s="21">
+        <f>IFERROR(_xlfn.MINIFS('Trade Log'!$K$4:$K$503,'Trade Log'!$B$4:$B$503,$A106),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" s="27" t="inlineStr">
+        <is>
+          <t>ZOTA</t>
+        </is>
+      </c>
+      <c r="B107" s="20">
+        <f>COUNTIF('Trade Log'!$B$4:$B$503,$A107)</f>
+        <v/>
+      </c>
+      <c r="C107" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A107,'Trade Log'!$K$4:$K$503,"&gt;0")</f>
+        <v/>
+      </c>
+      <c r="D107" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A107,'Trade Log'!$K$4:$K$503,"&lt;0")</f>
+        <v/>
+      </c>
+      <c r="E107" s="29">
+        <f>IFERROR($C107/$B107,"")</f>
+        <v/>
+      </c>
+      <c r="F107" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A107,'Trade Log'!$I$4:$I$503)</f>
+        <v/>
+      </c>
+      <c r="G107" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A107,'Trade Log'!$K$4:$K$503)</f>
+        <v/>
+      </c>
+      <c r="H107" s="21">
+        <f>IFERROR($G107/$B107,"")</f>
+        <v/>
+      </c>
+      <c r="I107" s="21">
+        <f>IFERROR(_xlfn.MAXIFS('Trade Log'!$K$4:$K$503,'Trade Log'!$B$4:$B$503,$A107),"")</f>
+        <v/>
+      </c>
+      <c r="J107" s="21">
+        <f>IFERROR(_xlfn.MINIFS('Trade Log'!$K$4:$K$503,'Trade Log'!$B$4:$B$503,$A107),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" s="3" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="B103" s="30">
-        <f>SUM(B4:B102)</f>
-        <v/>
-      </c>
-      <c r="C103" s="30">
-        <f>SUM(C4:C102)</f>
-        <v/>
-      </c>
-      <c r="D103" s="30">
-        <f>SUM(D4:D102)</f>
-        <v/>
-      </c>
-      <c r="E103" s="31">
-        <f>IFERROR(C103/B103,"")</f>
-        <v/>
-      </c>
-      <c r="F103" s="32">
-        <f>SUM(F4:F102)</f>
-        <v/>
-      </c>
-      <c r="G103" s="32">
-        <f>SUM(G4:G102)</f>
-        <v/>
-      </c>
-      <c r="H103" s="32">
-        <f>IFERROR(G103/B103,"")</f>
+      <c r="B108" s="30">
+        <f>SUM(B4:B107)</f>
+        <v/>
+      </c>
+      <c r="C108" s="30">
+        <f>SUM(C4:C107)</f>
+        <v/>
+      </c>
+      <c r="D108" s="30">
+        <f>SUM(D4:D107)</f>
+        <v/>
+      </c>
+      <c r="E108" s="31">
+        <f>IFERROR(C108/B108,"")</f>
+        <v/>
+      </c>
+      <c r="F108" s="32">
+        <f>SUM(F4:F107)</f>
+        <v/>
+      </c>
+      <c r="G108" s="32">
+        <f>SUM(G4:G107)</f>
+        <v/>
+      </c>
+      <c r="H108" s="32">
+        <f>IFERROR(G108/B108,"")</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Data update — 2026-09-25 candle + results refresh
</commit_message>
<xml_diff>
--- a/results/strategy_pnl_simple.xlsx
+++ b/results/strategy_pnl_simple.xlsx
@@ -1473,7 +1473,7 @@
         <v/>
       </c>
       <c r="J4" s="4" t="n">
-        <v>571.6900000000001</v>
+        <v>571.67</v>
       </c>
       <c r="K4" s="21">
         <f>IF(OR($B4="",$I4=""),"",$I4-IF($J4="",0,$J4))</f>
@@ -1524,7 +1524,7 @@
         <v/>
       </c>
       <c r="J5" s="4" t="n">
-        <v>688.92</v>
+        <v>688.95</v>
       </c>
       <c r="K5" s="21">
         <f>IF(OR($B5="",$I5=""),"",$I5-IF($J5="",0,$J5))</f>
@@ -1575,7 +1575,7 @@
         <v/>
       </c>
       <c r="J6" s="4" t="n">
-        <v>570.54</v>
+        <v>570.52</v>
       </c>
       <c r="K6" s="21">
         <f>IF(OR($B6="",$I6=""),"",$I6-IF($J6="",0,$J6))</f>
@@ -1626,7 +1626,7 @@
         <v/>
       </c>
       <c r="J7" s="4" t="n">
-        <v>662.9299999999999</v>
+        <v>662.9</v>
       </c>
       <c r="K7" s="21">
         <f>IF(OR($B7="",$I7=""),"",$I7-IF($J7="",0,$J7))</f>
@@ -1677,7 +1677,7 @@
         <v/>
       </c>
       <c r="J8" s="4" t="n">
-        <v>591.38</v>
+        <v>591.48</v>
       </c>
       <c r="K8" s="21">
         <f>IF(OR($B8="",$I8=""),"",$I8-IF($J8="",0,$J8))</f>
@@ -1779,7 +1779,7 @@
         <v/>
       </c>
       <c r="J10" s="4" t="n">
-        <v>398.57</v>
+        <v>398.55</v>
       </c>
       <c r="K10" s="21">
         <f>IF(OR($B10="",$I10=""),"",$I10-IF($J10="",0,$J10))</f>
@@ -1881,7 +1881,7 @@
         <v/>
       </c>
       <c r="J12" s="4" t="n">
-        <v>414.1</v>
+        <v>414.08</v>
       </c>
       <c r="K12" s="21">
         <f>IF(OR($B12="",$I12=""),"",$I12-IF($J12="",0,$J12))</f>
@@ -1932,7 +1932,7 @@
         <v/>
       </c>
       <c r="J13" s="4" t="n">
-        <v>345.03</v>
+        <v>345.02</v>
       </c>
       <c r="K13" s="21">
         <f>IF(OR($B13="",$I13=""),"",$I13-IF($J13="",0,$J13))</f>
@@ -1983,7 +1983,7 @@
         <v/>
       </c>
       <c r="J14" s="4" t="n">
-        <v>414.43</v>
+        <v>414.41</v>
       </c>
       <c r="K14" s="21">
         <f>IF(OR($B14="",$I14=""),"",$I14-IF($J14="",0,$J14))</f>
@@ -2034,7 +2034,7 @@
         <v/>
       </c>
       <c r="J15" s="4" t="n">
-        <v>380.49</v>
+        <v>380.52</v>
       </c>
       <c r="K15" s="21">
         <f>IF(OR($B15="",$I15=""),"",$I15-IF($J15="",0,$J15))</f>
@@ -2187,7 +2187,7 @@
         <v/>
       </c>
       <c r="J18" s="4" t="n">
-        <v>413.86</v>
+        <v>413.84</v>
       </c>
       <c r="K18" s="21">
         <f>IF(OR($B18="",$I18=""),"",$I18-IF($J18="",0,$J18))</f>
@@ -2238,7 +2238,7 @@
         <v/>
       </c>
       <c r="J19" s="4" t="n">
-        <v>406.4</v>
+        <v>406.39</v>
       </c>
       <c r="K19" s="21">
         <f>IF(OR($B19="",$I19=""),"",$I19-IF($J19="",0,$J19))</f>
@@ -2697,7 +2697,7 @@
         <v/>
       </c>
       <c r="J28" s="4" t="n">
-        <v>869.5700000000001</v>
+        <v>869.71</v>
       </c>
       <c r="K28" s="21">
         <f>IF(OR($B28="",$I28=""),"",$I28-IF($J28="",0,$J28))</f>
@@ -2850,7 +2850,7 @@
         <v/>
       </c>
       <c r="J31" s="4" t="n">
-        <v>390</v>
+        <v>390.01</v>
       </c>
       <c r="K31" s="21">
         <f>IF(OR($B31="",$I31=""),"",$I31-IF($J31="",0,$J31))</f>
@@ -3003,7 +3003,7 @@
         <v/>
       </c>
       <c r="J34" s="4" t="n">
-        <v>346.34</v>
+        <v>346.26</v>
       </c>
       <c r="K34" s="21">
         <f>IF(OR($B34="",$I34=""),"",$I34-IF($J34="",0,$J34))</f>
@@ -3054,7 +3054,7 @@
         <v/>
       </c>
       <c r="J35" s="4" t="n">
-        <v>385.16</v>
+        <v>385.12</v>
       </c>
       <c r="K35" s="21">
         <f>IF(OR($B35="",$I35=""),"",$I35-IF($J35="",0,$J35))</f>
@@ -3411,7 +3411,7 @@
         <v/>
       </c>
       <c r="J42" s="4" t="n">
-        <v>975.85</v>
+        <v>975.86</v>
       </c>
       <c r="K42" s="21">
         <f>IF(OR($B42="",$I42=""),"",$I42-IF($J42="",0,$J42))</f>
@@ -3462,7 +3462,7 @@
         <v/>
       </c>
       <c r="J43" s="4" t="n">
-        <v>955.65</v>
+        <v>955.66</v>
       </c>
       <c r="K43" s="21">
         <f>IF(OR($B43="",$I43=""),"",$I43-IF($J43="",0,$J43))</f>
@@ -3513,7 +3513,7 @@
         <v/>
       </c>
       <c r="J44" s="4" t="n">
-        <v>989.83</v>
+        <v>989.84</v>
       </c>
       <c r="K44" s="21">
         <f>IF(OR($B44="",$I44=""),"",$I44-IF($J44="",0,$J44))</f>
@@ -3564,7 +3564,7 @@
         <v/>
       </c>
       <c r="J45" s="4" t="n">
-        <v>595.8099999999999</v>
+        <v>595.83</v>
       </c>
       <c r="K45" s="21">
         <f>IF(OR($B45="",$I45=""),"",$I45-IF($J45="",0,$J45))</f>
@@ -3615,7 +3615,7 @@
         <v/>
       </c>
       <c r="J46" s="4" t="n">
-        <v>596.91</v>
+        <v>596.9299999999999</v>
       </c>
       <c r="K46" s="21">
         <f>IF(OR($B46="",$I46=""),"",$I46-IF($J46="",0,$J46))</f>
@@ -3666,7 +3666,7 @@
         <v/>
       </c>
       <c r="J47" s="4" t="n">
-        <v>675.08</v>
+        <v>675.15</v>
       </c>
       <c r="K47" s="21">
         <f>IF(OR($B47="",$I47=""),"",$I47-IF($J47="",0,$J47))</f>
@@ -3717,7 +3717,7 @@
         <v/>
       </c>
       <c r="J48" s="4" t="n">
-        <v>668.47</v>
+        <v>668.38</v>
       </c>
       <c r="K48" s="21">
         <f>IF(OR($B48="",$I48=""),"",$I48-IF($J48="",0,$J48))</f>
@@ -3768,7 +3768,7 @@
         <v/>
       </c>
       <c r="J49" s="4" t="n">
-        <v>572.83</v>
+        <v>572.84</v>
       </c>
       <c r="K49" s="21">
         <f>IF(OR($B49="",$I49=""),"",$I49-IF($J49="",0,$J49))</f>
@@ -3819,7 +3819,7 @@
         <v/>
       </c>
       <c r="J50" s="4" t="n">
-        <v>627.63</v>
+        <v>627.6900000000001</v>
       </c>
       <c r="K50" s="21">
         <f>IF(OR($B50="",$I50=""),"",$I50-IF($J50="",0,$J50))</f>
@@ -4023,7 +4023,7 @@
         <v/>
       </c>
       <c r="J54" s="4" t="n">
-        <v>618.74</v>
+        <v>618.6900000000001</v>
       </c>
       <c r="K54" s="21">
         <f>IF(OR($B54="",$I54=""),"",$I54-IF($J54="",0,$J54))</f>
@@ -4380,7 +4380,7 @@
         <v/>
       </c>
       <c r="J61" s="4" t="n">
-        <v>693.71</v>
+        <v>693.7</v>
       </c>
       <c r="K61" s="21">
         <f>IF(OR($B61="",$I61=""),"",$I61-IF($J61="",0,$J61))</f>
@@ -4431,7 +4431,7 @@
         <v/>
       </c>
       <c r="J62" s="4" t="n">
-        <v>616.9299999999999</v>
+        <v>616.97</v>
       </c>
       <c r="K62" s="21">
         <f>IF(OR($B62="",$I62=""),"",$I62-IF($J62="",0,$J62))</f>
@@ -4584,7 +4584,7 @@
         <v/>
       </c>
       <c r="J65" s="4" t="n">
-        <v>387.51</v>
+        <v>387.5</v>
       </c>
       <c r="K65" s="21">
         <f>IF(OR($B65="",$I65=""),"",$I65-IF($J65="",0,$J65))</f>
@@ -4941,7 +4941,7 @@
         <v/>
       </c>
       <c r="J72" s="4" t="n">
-        <v>411.81</v>
+        <v>411.8</v>
       </c>
       <c r="K72" s="21">
         <f>IF(OR($B72="",$I72=""),"",$I72-IF($J72="",0,$J72))</f>
@@ -5196,7 +5196,7 @@
         <v/>
       </c>
       <c r="J77" s="4" t="n">
-        <v>412.23</v>
+        <v>412.27</v>
       </c>
       <c r="K77" s="21">
         <f>IF(OR($B77="",$I77=""),"",$I77-IF($J77="",0,$J77))</f>
@@ -5859,7 +5859,7 @@
         <v/>
       </c>
       <c r="J90" s="4" t="n">
-        <v>893.48</v>
+        <v>893.47</v>
       </c>
       <c r="K90" s="21">
         <f>IF(OR($B90="",$I90=""),"",$I90-IF($J90="",0,$J90))</f>
@@ -5961,7 +5961,7 @@
         <v/>
       </c>
       <c r="J92" s="4" t="n">
-        <v>799.5</v>
+        <v>799.48</v>
       </c>
       <c r="K92" s="21">
         <f>IF(OR($B92="",$I92=""),"",$I92-IF($J92="",0,$J92))</f>
@@ -6012,7 +6012,7 @@
         <v/>
       </c>
       <c r="J93" s="4" t="n">
-        <v>826.84</v>
+        <v>826.8200000000001</v>
       </c>
       <c r="K93" s="21">
         <f>IF(OR($B93="",$I93=""),"",$I93-IF($J93="",0,$J93))</f>
@@ -6063,7 +6063,7 @@
         <v/>
       </c>
       <c r="J94" s="4" t="n">
-        <v>479.59</v>
+        <v>479.55</v>
       </c>
       <c r="K94" s="21">
         <f>IF(OR($B94="",$I94=""),"",$I94-IF($J94="",0,$J94))</f>
@@ -6165,7 +6165,7 @@
         <v/>
       </c>
       <c r="J96" s="4" t="n">
-        <v>474.59</v>
+        <v>474.58</v>
       </c>
       <c r="K96" s="21">
         <f>IF(OR($B96="",$I96=""),"",$I96-IF($J96="",0,$J96))</f>
@@ -6471,7 +6471,7 @@
         <v/>
       </c>
       <c r="J102" s="4" t="n">
-        <v>531.58</v>
+        <v>531.5700000000001</v>
       </c>
       <c r="K102" s="21">
         <f>IF(OR($B102="",$I102=""),"",$I102-IF($J102="",0,$J102))</f>
@@ -6879,7 +6879,7 @@
         <v/>
       </c>
       <c r="J110" s="4" t="n">
-        <v>480.93</v>
+        <v>480.9</v>
       </c>
       <c r="K110" s="21">
         <f>IF(OR($B110="",$I110=""),"",$I110-IF($J110="",0,$J110))</f>
@@ -7185,7 +7185,7 @@
         <v/>
       </c>
       <c r="J116" s="4" t="n">
-        <v>428.78</v>
+        <v>428.83</v>
       </c>
       <c r="K116" s="21">
         <f>IF(OR($B116="",$I116=""),"",$I116-IF($J116="",0,$J116))</f>
@@ -7236,7 +7236,7 @@
         <v/>
       </c>
       <c r="J117" s="4" t="n">
-        <v>546.34</v>
+        <v>546.33</v>
       </c>
       <c r="K117" s="21">
         <f>IF(OR($B117="",$I117=""),"",$I117-IF($J117="",0,$J117))</f>
@@ -7389,7 +7389,7 @@
         <v/>
       </c>
       <c r="J120" s="4" t="n">
-        <v>424.98</v>
+        <v>425</v>
       </c>
       <c r="K120" s="21">
         <f>IF(OR($B120="",$I120=""),"",$I120-IF($J120="",0,$J120))</f>
@@ -7440,7 +7440,7 @@
         <v/>
       </c>
       <c r="J121" s="4" t="n">
-        <v>371.59</v>
+        <v>371.58</v>
       </c>
       <c r="K121" s="21">
         <f>IF(OR($B121="",$I121=""),"",$I121-IF($J121="",0,$J121))</f>
@@ -7746,7 +7746,7 @@
         <v/>
       </c>
       <c r="J127" s="4" t="n">
-        <v>642.51</v>
+        <v>642.5</v>
       </c>
       <c r="K127" s="21">
         <f>IF(OR($B127="",$I127=""),"",$I127-IF($J127="",0,$J127))</f>
@@ -7848,7 +7848,7 @@
         <v/>
       </c>
       <c r="J129" s="4" t="n">
-        <v>638.35</v>
+        <v>638.34</v>
       </c>
       <c r="K129" s="21">
         <f>IF(OR($B129="",$I129=""),"",$I129-IF($J129="",0,$J129))</f>
@@ -7950,7 +7950,7 @@
         <v/>
       </c>
       <c r="J131" s="4" t="n">
-        <v>654.25</v>
+        <v>654.3200000000001</v>
       </c>
       <c r="K131" s="21">
         <f>IF(OR($B131="",$I131=""),"",$I131-IF($J131="",0,$J131))</f>
@@ -8052,7 +8052,7 @@
         <v/>
       </c>
       <c r="J133" s="4" t="n">
-        <v>564.1799999999999</v>
+        <v>564.17</v>
       </c>
       <c r="K133" s="21">
         <f>IF(OR($B133="",$I133=""),"",$I133-IF($J133="",0,$J133))</f>
@@ -8103,7 +8103,7 @@
         <v/>
       </c>
       <c r="J134" s="4" t="n">
-        <v>632.14</v>
+        <v>632.13</v>
       </c>
       <c r="K134" s="21">
         <f>IF(OR($B134="",$I134=""),"",$I134-IF($J134="",0,$J134))</f>
@@ -8154,7 +8154,7 @@
         <v/>
       </c>
       <c r="J135" s="4" t="n">
-        <v>497.88</v>
+        <v>497.87</v>
       </c>
       <c r="K135" s="21">
         <f>IF(OR($B135="",$I135=""),"",$I135-IF($J135="",0,$J135))</f>
@@ -8307,7 +8307,7 @@
         <v/>
       </c>
       <c r="J138" s="4" t="n">
-        <v>494.63</v>
+        <v>494.62</v>
       </c>
       <c r="K138" s="21">
         <f>IF(OR($B138="",$I138=""),"",$I138-IF($J138="",0,$J138))</f>
@@ -8409,7 +8409,7 @@
         <v/>
       </c>
       <c r="J140" s="4" t="n">
-        <v>504.18</v>
+        <v>504.32</v>
       </c>
       <c r="K140" s="21">
         <f>IF(OR($B140="",$I140=""),"",$I140-IF($J140="",0,$J140))</f>
@@ -8460,7 +8460,7 @@
         <v/>
       </c>
       <c r="J141" s="4" t="n">
-        <v>492.11</v>
+        <v>491.92</v>
       </c>
       <c r="K141" s="21">
         <f>IF(OR($B141="",$I141=""),"",$I141-IF($J141="",0,$J141))</f>
@@ -8511,7 +8511,7 @@
         <v/>
       </c>
       <c r="J142" s="4" t="n">
-        <v>467.29</v>
+        <v>467.28</v>
       </c>
       <c r="K142" s="21">
         <f>IF(OR($B142="",$I142=""),"",$I142-IF($J142="",0,$J142))</f>
@@ -8664,7 +8664,7 @@
         <v/>
       </c>
       <c r="J145" s="4" t="n">
-        <v>542.0599999999999</v>
+        <v>542.14</v>
       </c>
       <c r="K145" s="21">
         <f>IF(OR($B145="",$I145=""),"",$I145-IF($J145="",0,$J145))</f>
@@ -9225,7 +9225,7 @@
         <v/>
       </c>
       <c r="J156" s="4" t="n">
-        <v>435.16</v>
+        <v>437.61</v>
       </c>
       <c r="K156" s="21">
         <f>IF(OR($B156="",$I156=""),"",$I156-IF($J156="",0,$J156))</f>
@@ -9276,7 +9276,7 @@
         <v/>
       </c>
       <c r="J157" s="4" t="n">
-        <v>524.72</v>
+        <v>529.13</v>
       </c>
       <c r="K157" s="21">
         <f>IF(OR($B157="",$I157=""),"",$I157-IF($J157="",0,$J157))</f>
@@ -9327,7 +9327,7 @@
         <v/>
       </c>
       <c r="J158" s="4" t="n">
-        <v>519.0599999999999</v>
+        <v>523.14</v>
       </c>
       <c r="K158" s="21">
         <f>IF(OR($B158="",$I158=""),"",$I158-IF($J158="",0,$J158))</f>
@@ -9378,7 +9378,7 @@
         <v/>
       </c>
       <c r="J159" s="4" t="n">
-        <v>517.4400000000001</v>
+        <v>521.5</v>
       </c>
       <c r="K159" s="21">
         <f>IF(OR($B159="",$I159=""),"",$I159-IF($J159="",0,$J159))</f>
@@ -9429,7 +9429,7 @@
         <v/>
       </c>
       <c r="J160" s="4" t="n">
-        <v>445.64</v>
+        <v>449.02</v>
       </c>
       <c r="K160" s="21">
         <f>IF(OR($B160="",$I160=""),"",$I160-IF($J160="",0,$J160))</f>
@@ -9480,7 +9480,7 @@
         <v/>
       </c>
       <c r="J161" s="4" t="n">
-        <v>461.69</v>
+        <v>466.32</v>
       </c>
       <c r="K161" s="21">
         <f>IF(OR($B161="",$I161=""),"",$I161-IF($J161="",0,$J161))</f>
@@ -9837,7 +9837,7 @@
         <v/>
       </c>
       <c r="J168" s="4" t="n">
-        <v>626.4400000000001</v>
+        <v>631.66</v>
       </c>
       <c r="K168" s="21">
         <f>IF(OR($B168="",$I168=""),"",$I168-IF($J168="",0,$J168))</f>
@@ -9888,7 +9888,7 @@
         <v/>
       </c>
       <c r="J169" s="4" t="n">
-        <v>634.4299999999999</v>
+        <v>640.53</v>
       </c>
       <c r="K169" s="21">
         <f>IF(OR($B169="",$I169=""),"",$I169-IF($J169="",0,$J169))</f>
@@ -9990,7 +9990,7 @@
         <v/>
       </c>
       <c r="J171" s="4" t="n">
-        <v>662.13</v>
+        <v>606.78</v>
       </c>
       <c r="K171" s="21">
         <f>IF(OR($B171="",$I171=""),"",$I171-IF($J171="",0,$J171))</f>
@@ -10041,7 +10041,7 @@
         <v/>
       </c>
       <c r="J172" s="4" t="n">
-        <v>647.29</v>
+        <v>595.6900000000001</v>
       </c>
       <c r="K172" s="21">
         <f>IF(OR($B172="",$I172=""),"",$I172-IF($J172="",0,$J172))</f>
@@ -10092,7 +10092,7 @@
         <v/>
       </c>
       <c r="J173" s="4" t="n">
-        <v>665.03</v>
+        <v>608.9400000000001</v>
       </c>
       <c r="K173" s="21">
         <f>IF(OR($B173="",$I173=""),"",$I173-IF($J173="",0,$J173))</f>
@@ -10194,7 +10194,7 @@
         <v/>
       </c>
       <c r="J175" s="4" t="n">
-        <v>649.5</v>
+        <v>597.7</v>
       </c>
       <c r="K175" s="21">
         <f>IF(OR($B175="",$I175=""),"",$I175-IF($J175="",0,$J175))</f>
@@ -10296,7 +10296,7 @@
         <v/>
       </c>
       <c r="J177" s="4" t="n">
-        <v>294.85</v>
+        <v>297.1</v>
       </c>
       <c r="K177" s="21">
         <f>IF(OR($B177="",$I177=""),"",$I177-IF($J177="",0,$J177))</f>
@@ -10449,7 +10449,7 @@
         <v/>
       </c>
       <c r="J180" s="4" t="n">
-        <v>336.65</v>
+        <v>338.95</v>
       </c>
       <c r="K180" s="21">
         <f>IF(OR($B180="",$I180=""),"",$I180-IF($J180="",0,$J180))</f>
@@ -10500,7 +10500,7 @@
         <v/>
       </c>
       <c r="J181" s="4" t="n">
-        <v>298.41</v>
+        <v>300.56</v>
       </c>
       <c r="K181" s="21">
         <f>IF(OR($B181="",$I181=""),"",$I181-IF($J181="",0,$J181))</f>
@@ -10551,7 +10551,7 @@
         <v/>
       </c>
       <c r="J182" s="4" t="n">
-        <v>191.65</v>
+        <v>192.46</v>
       </c>
       <c r="K182" s="21">
         <f>IF(OR($B182="",$I182=""),"",$I182-IF($J182="",0,$J182))</f>
@@ -10704,7 +10704,7 @@
         <v/>
       </c>
       <c r="J185" s="4" t="n">
-        <v>295.25</v>
+        <v>297.58</v>
       </c>
       <c r="K185" s="21">
         <f>IF(OR($B185="",$I185=""),"",$I185-IF($J185="",0,$J185))</f>
@@ -10908,7 +10908,7 @@
         <v/>
       </c>
       <c r="J189" s="4" t="n">
-        <v>132.03</v>
+        <v>100.21</v>
       </c>
       <c r="K189" s="21">
         <f>IF(OR($B189="",$I189=""),"",$I189-IF($J189="",0,$J189))</f>
@@ -10959,7 +10959,7 @@
         <v/>
       </c>
       <c r="J190" s="4" t="n">
-        <v>459.73</v>
+        <v>464.03</v>
       </c>
       <c r="K190" s="21">
         <f>IF(OR($B190="",$I190=""),"",$I190-IF($J190="",0,$J190))</f>
@@ -11214,7 +11214,7 @@
         <v/>
       </c>
       <c r="J195" s="4" t="n">
-        <v>462.53</v>
+        <v>467.16</v>
       </c>
       <c r="K195" s="21">
         <f>IF(OR($B195="",$I195=""),"",$I195-IF($J195="",0,$J195))</f>
@@ -11265,7 +11265,7 @@
         <v/>
       </c>
       <c r="J196" s="4" t="n">
-        <v>517.1</v>
+        <v>499</v>
       </c>
       <c r="K196" s="21">
         <f>IF(OR($B196="",$I196=""),"",$I196-IF($J196="",0,$J196))</f>
@@ -11367,7 +11367,7 @@
         <v/>
       </c>
       <c r="J198" s="4" t="n">
-        <v>519.16</v>
+        <v>523.22</v>
       </c>
       <c r="K198" s="21">
         <f>IF(OR($B198="",$I198=""),"",$I198-IF($J198="",0,$J198))</f>
@@ -11418,7 +11418,7 @@
         <v/>
       </c>
       <c r="J199" s="4" t="n">
-        <v>456.59</v>
+        <v>460.88</v>
       </c>
       <c r="K199" s="21">
         <f>IF(OR($B199="",$I199=""),"",$I199-IF($J199="",0,$J199))</f>
@@ -11469,7 +11469,7 @@
         <v/>
       </c>
       <c r="J200" s="4" t="n">
-        <v>84.33</v>
+        <v>138.27</v>
       </c>
       <c r="K200" s="21">
         <f>IF(OR($B200="",$I200=""),"",$I200-IF($J200="",0,$J200))</f>
@@ -11622,7 +11622,7 @@
         <v/>
       </c>
       <c r="J203" s="4" t="n">
-        <v>86.05</v>
+        <v>97.51000000000001</v>
       </c>
       <c r="K203" s="21">
         <f>IF(OR($B203="",$I203=""),"",$I203-IF($J203="",0,$J203))</f>
@@ -11673,7 +11673,7 @@
         <v/>
       </c>
       <c r="J204" s="4" t="n">
-        <v>14.75</v>
+        <v>63.56</v>
       </c>
       <c r="K204" s="21">
         <f>IF(OR($B204="",$I204=""),"",$I204-IF($J204="",0,$J204))</f>
@@ -11724,7 +11724,7 @@
         <v/>
       </c>
       <c r="J205" s="4" t="n">
-        <v>82.28</v>
+        <v>137.02</v>
       </c>
       <c r="K205" s="21">
         <f>IF(OR($B205="",$I205=""),"",$I205-IF($J205="",0,$J205))</f>
@@ -11775,7 +11775,7 @@
         <v/>
       </c>
       <c r="J206" s="4" t="n">
-        <v>299.68</v>
+        <v>316.29</v>
       </c>
       <c r="K206" s="21">
         <f>IF(OR($B206="",$I206=""),"",$I206-IF($J206="",0,$J206))</f>
@@ -11826,7 +11826,7 @@
         <v/>
       </c>
       <c r="J207" s="4" t="n">
-        <v>305.04</v>
+        <v>319.15</v>
       </c>
       <c r="K207" s="21">
         <f>IF(OR($B207="",$I207=""),"",$I207-IF($J207="",0,$J207))</f>
@@ -11877,7 +11877,7 @@
         <v/>
       </c>
       <c r="J208" s="4" t="n">
-        <v>300.26</v>
+        <v>360.34</v>
       </c>
       <c r="K208" s="21">
         <f>IF(OR($B208="",$I208=""),"",$I208-IF($J208="",0,$J208))</f>
@@ -12030,7 +12030,7 @@
         <v/>
       </c>
       <c r="J211" s="4" t="n">
-        <v>303.26</v>
+        <v>317.53</v>
       </c>
       <c r="K211" s="21">
         <f>IF(OR($B211="",$I211=""),"",$I211-IF($J211="",0,$J211))</f>
@@ -12081,7 +12081,7 @@
         <v/>
       </c>
       <c r="J212" s="4" t="n">
-        <v>309.33</v>
+        <v>362.04</v>
       </c>
       <c r="K212" s="21">
         <f>IF(OR($B212="",$I212=""),"",$I212-IF($J212="",0,$J212))</f>
@@ -12234,7 +12234,7 @@
         <v/>
       </c>
       <c r="J215" s="4" t="n">
-        <v>0</v>
+        <v>204.98</v>
       </c>
       <c r="K215" s="21">
         <f>IF(OR($B215="",$I215=""),"",$I215-IF($J215="",0,$J215))</f>
@@ -12274,14 +12274,18 @@
       <c r="F216" s="26" t="n">
         <v>1614</v>
       </c>
-      <c r="G216" s="24" t="inlineStr"/>
-      <c r="H216" s="25" t="inlineStr"/>
+      <c r="G216" s="24" t="n">
+        <v>46290</v>
+      </c>
+      <c r="H216" s="25" t="n">
+        <v>157.11</v>
+      </c>
       <c r="I216" s="21">
         <f>IF(OR($B216="",$H216=""),"",IF($C216="LONG",($H216-$E216)*$F216,($E216-$H216)*$F216))</f>
         <v/>
       </c>
       <c r="J216" s="4" t="n">
-        <v>50.15</v>
+        <v>426.08</v>
       </c>
       <c r="K216" s="21">
         <f>IF(OR($B216="",$I216=""),"",$I216-IF($J216="",0,$J216))</f>
@@ -12332,7 +12336,7 @@
         <v/>
       </c>
       <c r="J217" s="4" t="n">
-        <v>0</v>
+        <v>258.86</v>
       </c>
       <c r="K217" s="21">
         <f>IF(OR($B217="",$I217=""),"",$I217-IF($J217="",0,$J217))</f>
@@ -12372,8 +12376,12 @@
       <c r="F218" s="26" t="n">
         <v>82</v>
       </c>
-      <c r="G218" s="24" t="inlineStr"/>
-      <c r="H218" s="25" t="inlineStr"/>
+      <c r="G218" s="24" t="n">
+        <v>46290</v>
+      </c>
+      <c r="H218" s="25" t="n">
+        <v>1533.8</v>
+      </c>
       <c r="I218" s="21">
         <f>IF(OR($B218="",$H218=""),"",IF($C218="LONG",($H218-$E218)*$F218,($E218-$H218)*$F218))</f>
         <v/>
@@ -12430,7 +12438,7 @@
         <v/>
       </c>
       <c r="J219" s="4" t="n">
-        <v>0</v>
+        <v>120.38</v>
       </c>
       <c r="K219" s="21">
         <f>IF(OR($B219="",$I219=""),"",$I219-IF($J219="",0,$J219))</f>
@@ -12470,14 +12478,18 @@
       <c r="F220" s="26" t="n">
         <v>1128</v>
       </c>
-      <c r="G220" s="24" t="inlineStr"/>
-      <c r="H220" s="25" t="inlineStr"/>
+      <c r="G220" s="24" t="n">
+        <v>46290</v>
+      </c>
+      <c r="H220" s="25" t="n">
+        <v>223.36</v>
+      </c>
       <c r="I220" s="21">
         <f>IF(OR($B220="",$H220=""),"",IF($C220="LONG",($H220-$E220)*$F220,($E220-$H220)*$F220))</f>
         <v/>
       </c>
       <c r="J220" s="4" t="n">
-        <v>50.15</v>
+        <v>424.67</v>
       </c>
       <c r="K220" s="21">
         <f>IF(OR($B220="",$I220=""),"",$I220-IF($J220="",0,$J220))</f>
@@ -12517,14 +12529,18 @@
       <c r="F221" s="26" t="n">
         <v>409</v>
       </c>
-      <c r="G221" s="24" t="inlineStr"/>
-      <c r="H221" s="25" t="inlineStr"/>
+      <c r="G221" s="24" t="n">
+        <v>46290</v>
+      </c>
+      <c r="H221" s="25" t="n">
+        <v>308.29</v>
+      </c>
       <c r="I221" s="21">
         <f>IF(OR($B221="",$H221=""),"",IF($C221="LONG",($H221-$E221)*$F221,($E221-$H221)*$F221))</f>
         <v/>
       </c>
       <c r="J221" s="4" t="n">
-        <v>14.75</v>
+        <v>162.56</v>
       </c>
       <c r="K221" s="21">
         <f>IF(OR($B221="",$I221=""),"",$I221-IF($J221="",0,$J221))</f>
@@ -12575,7 +12591,7 @@
         <v/>
       </c>
       <c r="J222" s="4" t="n">
-        <v>0</v>
+        <v>200.09</v>
       </c>
       <c r="K222" s="21">
         <f>IF(OR($B222="",$I222=""),"",$I222-IF($J222="",0,$J222))</f>
@@ -12626,7 +12642,7 @@
         <v/>
       </c>
       <c r="J223" s="4" t="n">
-        <v>0</v>
+        <v>243.64</v>
       </c>
       <c r="K223" s="21">
         <f>IF(OR($B223="",$I223=""),"",$I223-IF($J223="",0,$J223))</f>
@@ -12666,14 +12682,18 @@
       <c r="F224" s="26" t="n">
         <v>319</v>
       </c>
-      <c r="G224" s="24" t="inlineStr"/>
-      <c r="H224" s="25" t="inlineStr"/>
+      <c r="G224" s="24" t="n">
+        <v>46290</v>
+      </c>
+      <c r="H224" s="25" t="n">
+        <v>824.01</v>
+      </c>
       <c r="I224" s="21">
         <f>IF(OR($B224="",$H224=""),"",IF($C224="LONG",($H224-$E224)*$F224,($E224-$H224)*$F224))</f>
         <v/>
       </c>
       <c r="J224" s="4" t="n">
-        <v>50.15</v>
+        <v>427.89</v>
       </c>
       <c r="K224" s="21">
         <f>IF(OR($B224="",$I224=""),"",$I224-IF($J224="",0,$J224))</f>
@@ -12724,7 +12744,7 @@
         <v/>
       </c>
       <c r="J225" s="4" t="n">
-        <v>0</v>
+        <v>248.07</v>
       </c>
       <c r="K225" s="21">
         <f>IF(OR($B225="",$I225=""),"",$I225-IF($J225="",0,$J225))</f>
@@ -12775,7 +12795,7 @@
         <v/>
       </c>
       <c r="J226" s="4" t="n">
-        <v>0</v>
+        <v>213.84</v>
       </c>
       <c r="K226" s="21">
         <f>IF(OR($B226="",$I226=""),"",$I226-IF($J226="",0,$J226))</f>
@@ -12822,7 +12842,7 @@
         <v/>
       </c>
       <c r="J227" s="4" t="n">
-        <v>14.75</v>
+        <v>43.01</v>
       </c>
       <c r="K227" s="21">
         <f>IF(OR($B227="",$I227=""),"",$I227-IF($J227="",0,$J227))</f>
@@ -12873,7 +12893,7 @@
         <v/>
       </c>
       <c r="J228" s="4" t="n">
-        <v>0</v>
+        <v>190.03</v>
       </c>
       <c r="K228" s="21">
         <f>IF(OR($B228="",$I228=""),"",$I228-IF($J228="",0,$J228))</f>
@@ -12924,7 +12944,7 @@
         <v/>
       </c>
       <c r="J229" s="4" t="n">
-        <v>0</v>
+        <v>201.68</v>
       </c>
       <c r="K229" s="21">
         <f>IF(OR($B229="",$I229=""),"",$I229-IF($J229="",0,$J229))</f>
@@ -12940,19 +12960,43 @@
       </c>
     </row>
     <row r="230">
-      <c r="A230" s="23" t="n"/>
-      <c r="B230" s="23" t="n"/>
-      <c r="C230" s="23" t="n"/>
-      <c r="D230" s="24" t="n"/>
-      <c r="E230" s="25" t="n"/>
-      <c r="F230" s="26" t="n"/>
-      <c r="G230" s="24" t="n"/>
-      <c r="H230" s="25" t="n"/>
+      <c r="A230" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-34126092552909</t>
+        </is>
+      </c>
+      <c r="B230" s="23" t="inlineStr">
+        <is>
+          <t>AVANTEL</t>
+        </is>
+      </c>
+      <c r="C230" s="23" t="inlineStr">
+        <is>
+          <t>SHORT</t>
+        </is>
+      </c>
+      <c r="D230" s="24" t="n">
+        <v>46290</v>
+      </c>
+      <c r="E230" s="25" t="n">
+        <v>157.03</v>
+      </c>
+      <c r="F230" s="26" t="n">
+        <v>1614</v>
+      </c>
+      <c r="G230" s="24" t="n">
+        <v>46290</v>
+      </c>
+      <c r="H230" s="25" t="n">
+        <v>156.4</v>
+      </c>
       <c r="I230" s="21">
         <f>IF(OR($B230="",$H230=""),"",IF($C230="LONG",($H230-$E230)*$F230,($E230-$H230)*$F230))</f>
         <v/>
       </c>
-      <c r="J230" s="4" t="n"/>
+      <c r="J230" s="4" t="n">
+        <v>0</v>
+      </c>
       <c r="K230" s="21">
         <f>IF(OR($B230="",$I230=""),"",$I230-IF($J230="",0,$J230))</f>
         <v/>
@@ -12967,19 +13011,39 @@
       </c>
     </row>
     <row r="231">
-      <c r="A231" s="23" t="n"/>
-      <c r="B231" s="23" t="n"/>
-      <c r="C231" s="23" t="n"/>
-      <c r="D231" s="24" t="n"/>
-      <c r="E231" s="25" t="n"/>
-      <c r="F231" s="26" t="n"/>
-      <c r="G231" s="24" t="n"/>
-      <c r="H231" s="25" t="n"/>
+      <c r="A231" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-limit_entry_multi</t>
+        </is>
+      </c>
+      <c r="B231" s="23" t="inlineStr">
+        <is>
+          <t>BHAGERIA</t>
+        </is>
+      </c>
+      <c r="C231" s="23" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="D231" s="24" t="n">
+        <v>46290</v>
+      </c>
+      <c r="E231" s="25" t="n">
+        <v>394.528</v>
+      </c>
+      <c r="F231" s="26" t="n">
+        <v>316</v>
+      </c>
+      <c r="G231" s="24" t="inlineStr"/>
+      <c r="H231" s="25" t="inlineStr"/>
       <c r="I231" s="21">
         <f>IF(OR($B231="",$H231=""),"",IF($C231="LONG",($H231-$E231)*$F231,($E231-$H231)*$F231))</f>
         <v/>
       </c>
-      <c r="J231" s="4" t="n"/>
+      <c r="J231" s="4" t="n">
+        <v>14.75</v>
+      </c>
       <c r="K231" s="21">
         <f>IF(OR($B231="",$I231=""),"",$I231-IF($J231="",0,$J231))</f>
         <v/>
@@ -12994,19 +13058,39 @@
       </c>
     </row>
     <row r="232">
-      <c r="A232" s="23" t="n"/>
-      <c r="B232" s="23" t="n"/>
-      <c r="C232" s="23" t="n"/>
-      <c r="D232" s="24" t="n"/>
-      <c r="E232" s="25" t="n"/>
-      <c r="F232" s="26" t="n"/>
-      <c r="G232" s="24" t="n"/>
-      <c r="H232" s="25" t="n"/>
+      <c r="A232" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-321260925638609</t>
+        </is>
+      </c>
+      <c r="B232" s="23" t="inlineStr">
+        <is>
+          <t>DELTACORP</t>
+        </is>
+      </c>
+      <c r="C232" s="23" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="D232" s="24" t="n">
+        <v>46290</v>
+      </c>
+      <c r="E232" s="25" t="n">
+        <v>76.9342</v>
+      </c>
+      <c r="F232" s="26" t="n">
+        <v>3254</v>
+      </c>
+      <c r="G232" s="24" t="inlineStr"/>
+      <c r="H232" s="25" t="inlineStr"/>
       <c r="I232" s="21">
         <f>IF(OR($B232="",$H232=""),"",IF($C232="LONG",($H232-$E232)*$F232,($E232-$H232)*$F232))</f>
         <v/>
       </c>
-      <c r="J232" s="4" t="n"/>
+      <c r="J232" s="4" t="n">
+        <v>50.15</v>
+      </c>
       <c r="K232" s="21">
         <f>IF(OR($B232="",$I232=""),"",$I232-IF($J232="",0,$J232))</f>
         <v/>
@@ -13021,19 +13105,43 @@
       </c>
     </row>
     <row r="233">
-      <c r="A233" s="23" t="n"/>
-      <c r="B233" s="23" t="n"/>
-      <c r="C233" s="23" t="n"/>
-      <c r="D233" s="24" t="n"/>
-      <c r="E233" s="25" t="n"/>
-      <c r="F233" s="26" t="n"/>
-      <c r="G233" s="24" t="n"/>
-      <c r="H233" s="25" t="n"/>
+      <c r="A233" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-34126092513409</t>
+        </is>
+      </c>
+      <c r="B233" s="23" t="inlineStr">
+        <is>
+          <t>FRONTSP</t>
+        </is>
+      </c>
+      <c r="C233" s="23" t="inlineStr">
+        <is>
+          <t>SHORT</t>
+        </is>
+      </c>
+      <c r="D233" s="24" t="n">
+        <v>46290</v>
+      </c>
+      <c r="E233" s="25" t="n">
+        <v>1540</v>
+      </c>
+      <c r="F233" s="26" t="n">
+        <v>82</v>
+      </c>
+      <c r="G233" s="24" t="n">
+        <v>46290</v>
+      </c>
+      <c r="H233" s="25" t="n">
+        <v>1463</v>
+      </c>
       <c r="I233" s="21">
         <f>IF(OR($B233="",$H233=""),"",IF($C233="LONG",($H233-$E233)*$F233,($E233-$H233)*$F233))</f>
         <v/>
       </c>
-      <c r="J233" s="4" t="n"/>
+      <c r="J233" s="4" t="n">
+        <v>0</v>
+      </c>
       <c r="K233" s="21">
         <f>IF(OR($B233="",$I233=""),"",$I233-IF($J233="",0,$J233))</f>
         <v/>
@@ -13048,19 +13156,43 @@
       </c>
     </row>
     <row r="234">
-      <c r="A234" s="23" t="n"/>
-      <c r="B234" s="23" t="n"/>
-      <c r="C234" s="23" t="n"/>
-      <c r="D234" s="24" t="n"/>
-      <c r="E234" s="25" t="n"/>
-      <c r="F234" s="26" t="n"/>
-      <c r="G234" s="24" t="n"/>
-      <c r="H234" s="25" t="n"/>
+      <c r="A234" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-22126092551109</t>
+        </is>
+      </c>
+      <c r="B234" s="23" t="inlineStr">
+        <is>
+          <t>GREAVESCOT</t>
+        </is>
+      </c>
+      <c r="C234" s="23" t="inlineStr">
+        <is>
+          <t>SHORT</t>
+        </is>
+      </c>
+      <c r="D234" s="24" t="n">
+        <v>46290</v>
+      </c>
+      <c r="E234" s="25" t="n">
+        <v>222.61</v>
+      </c>
+      <c r="F234" s="26" t="n">
+        <v>1128</v>
+      </c>
+      <c r="G234" s="24" t="n">
+        <v>46290</v>
+      </c>
+      <c r="H234" s="25" t="n">
+        <v>233.98</v>
+      </c>
       <c r="I234" s="21">
         <f>IF(OR($B234="",$H234=""),"",IF($C234="LONG",($H234-$E234)*$F234,($E234-$H234)*$F234))</f>
         <v/>
       </c>
-      <c r="J234" s="4" t="n"/>
+      <c r="J234" s="4" t="n">
+        <v>0</v>
+      </c>
       <c r="K234" s="21">
         <f>IF(OR($B234="",$I234=""),"",$I234-IF($J234="",0,$J234))</f>
         <v/>
@@ -13075,19 +13207,43 @@
       </c>
     </row>
     <row r="235">
-      <c r="A235" s="23" t="n"/>
-      <c r="B235" s="23" t="n"/>
-      <c r="C235" s="23" t="n"/>
-      <c r="D235" s="24" t="n"/>
-      <c r="E235" s="25" t="n"/>
-      <c r="F235" s="26" t="n"/>
-      <c r="G235" s="24" t="n"/>
-      <c r="H235" s="25" t="n"/>
+      <c r="A235" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-32126092550109</t>
+        </is>
+      </c>
+      <c r="B235" s="23" t="inlineStr">
+        <is>
+          <t>INDIAGLYCO</t>
+        </is>
+      </c>
+      <c r="C235" s="23" t="inlineStr">
+        <is>
+          <t>SHORT</t>
+        </is>
+      </c>
+      <c r="D235" s="24" t="n">
+        <v>46290</v>
+      </c>
+      <c r="E235" s="25" t="n">
+        <v>308</v>
+      </c>
+      <c r="F235" s="26" t="n">
+        <v>409</v>
+      </c>
+      <c r="G235" s="24" t="n">
+        <v>46290</v>
+      </c>
+      <c r="H235" s="25" t="n">
+        <v>308.52</v>
+      </c>
       <c r="I235" s="21">
         <f>IF(OR($B235="",$H235=""),"",IF($C235="LONG",($H235-$E235)*$F235,($E235-$H235)*$F235))</f>
         <v/>
       </c>
-      <c r="J235" s="4" t="n"/>
+      <c r="J235" s="4" t="n">
+        <v>0</v>
+      </c>
       <c r="K235" s="21">
         <f>IF(OR($B235="",$I235=""),"",$I235-IF($J235="",0,$J235))</f>
         <v/>
@@ -13102,19 +13258,43 @@
       </c>
     </row>
     <row r="236">
-      <c r="A236" s="23" t="n"/>
-      <c r="B236" s="23" t="n"/>
-      <c r="C236" s="23" t="n"/>
-      <c r="D236" s="24" t="n"/>
-      <c r="E236" s="25" t="n"/>
-      <c r="F236" s="26" t="n"/>
-      <c r="G236" s="24" t="n"/>
-      <c r="H236" s="25" t="n"/>
+      <c r="A236" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-32126092550209</t>
+        </is>
+      </c>
+      <c r="B236" s="23" t="inlineStr">
+        <is>
+          <t>KSCL</t>
+        </is>
+      </c>
+      <c r="C236" s="23" t="inlineStr">
+        <is>
+          <t>SHORT</t>
+        </is>
+      </c>
+      <c r="D236" s="24" t="n">
+        <v>46290</v>
+      </c>
+      <c r="E236" s="25" t="n">
+        <v>826.46</v>
+      </c>
+      <c r="F236" s="26" t="n">
+        <v>319</v>
+      </c>
+      <c r="G236" s="24" t="n">
+        <v>46290</v>
+      </c>
+      <c r="H236" s="25" t="n">
+        <v>785.15</v>
+      </c>
       <c r="I236" s="21">
         <f>IF(OR($B236="",$H236=""),"",IF($C236="LONG",($H236-$E236)*$F236,($E236-$H236)*$F236))</f>
         <v/>
       </c>
-      <c r="J236" s="4" t="n"/>
+      <c r="J236" s="4" t="n">
+        <v>0</v>
+      </c>
       <c r="K236" s="21">
         <f>IF(OR($B236="",$I236=""),"",$I236-IF($J236="",0,$J236))</f>
         <v/>
@@ -13129,19 +13309,39 @@
       </c>
     </row>
     <row r="237">
-      <c r="A237" s="23" t="n"/>
-      <c r="B237" s="23" t="n"/>
-      <c r="C237" s="23" t="n"/>
-      <c r="D237" s="24" t="n"/>
-      <c r="E237" s="25" t="n"/>
-      <c r="F237" s="26" t="n"/>
-      <c r="G237" s="24" t="n"/>
-      <c r="H237" s="25" t="n"/>
+      <c r="A237" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-limit_entry_multi</t>
+        </is>
+      </c>
+      <c r="B237" s="23" t="inlineStr">
+        <is>
+          <t>SANGAMIND</t>
+        </is>
+      </c>
+      <c r="C237" s="23" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="D237" s="24" t="n">
+        <v>46290</v>
+      </c>
+      <c r="E237" s="25" t="n">
+        <v>617.5682</v>
+      </c>
+      <c r="F237" s="26" t="n">
+        <v>404</v>
+      </c>
+      <c r="G237" s="24" t="inlineStr"/>
+      <c r="H237" s="25" t="inlineStr"/>
       <c r="I237" s="21">
         <f>IF(OR($B237="",$H237=""),"",IF($C237="LONG",($H237-$E237)*$F237,($E237-$H237)*$F237))</f>
         <v/>
       </c>
-      <c r="J237" s="4" t="n"/>
+      <c r="J237" s="4" t="n">
+        <v>67.47</v>
+      </c>
       <c r="K237" s="21">
         <f>IF(OR($B237="",$I237=""),"",$I237-IF($J237="",0,$J237))</f>
         <v/>
@@ -13156,19 +13356,39 @@
       </c>
     </row>
     <row r="238">
-      <c r="A238" s="23" t="n"/>
-      <c r="B238" s="23" t="n"/>
-      <c r="C238" s="23" t="n"/>
-      <c r="D238" s="24" t="n"/>
-      <c r="E238" s="25" t="n"/>
-      <c r="F238" s="26" t="n"/>
-      <c r="G238" s="24" t="n"/>
-      <c r="H238" s="25" t="n"/>
+      <c r="A238" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-23126092590809</t>
+        </is>
+      </c>
+      <c r="B238" s="23" t="inlineStr">
+        <is>
+          <t>SHANTIGOLD</t>
+        </is>
+      </c>
+      <c r="C238" s="23" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="D238" s="24" t="n">
+        <v>46290</v>
+      </c>
+      <c r="E238" s="25" t="n">
+        <v>325.9933</v>
+      </c>
+      <c r="F238" s="26" t="n">
+        <v>771</v>
+      </c>
+      <c r="G238" s="24" t="inlineStr"/>
+      <c r="H238" s="25" t="inlineStr"/>
       <c r="I238" s="21">
         <f>IF(OR($B238="",$H238=""),"",IF($C238="LONG",($H238-$E238)*$F238,($E238-$H238)*$F238))</f>
         <v/>
       </c>
-      <c r="J238" s="4" t="n"/>
+      <c r="J238" s="4" t="n">
+        <v>50.15</v>
+      </c>
       <c r="K238" s="21">
         <f>IF(OR($B238="",$I238=""),"",$I238-IF($J238="",0,$J238))</f>
         <v/>
@@ -13183,19 +13403,39 @@
       </c>
     </row>
     <row r="239">
-      <c r="A239" s="23" t="n"/>
-      <c r="B239" s="23" t="n"/>
-      <c r="C239" s="23" t="n"/>
-      <c r="D239" s="24" t="n"/>
-      <c r="E239" s="25" t="n"/>
-      <c r="F239" s="26" t="n"/>
-      <c r="G239" s="24" t="n"/>
-      <c r="H239" s="25" t="n"/>
+      <c r="A239" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-limit_entry_multi</t>
+        </is>
+      </c>
+      <c r="B239" s="23" t="inlineStr">
+        <is>
+          <t>SHOPERSTOP</t>
+        </is>
+      </c>
+      <c r="C239" s="23" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="D239" s="24" t="n">
+        <v>46290</v>
+      </c>
+      <c r="E239" s="25" t="n">
+        <v>422.7841</v>
+      </c>
+      <c r="F239" s="26" t="n">
+        <v>591</v>
+      </c>
+      <c r="G239" s="24" t="inlineStr"/>
+      <c r="H239" s="25" t="inlineStr"/>
       <c r="I239" s="21">
         <f>IF(OR($B239="",$H239=""),"",IF($C239="LONG",($H239-$E239)*$F239,($E239-$H239)*$F239))</f>
         <v/>
       </c>
-      <c r="J239" s="4" t="n"/>
+      <c r="J239" s="4" t="n">
+        <v>67.47</v>
+      </c>
       <c r="K239" s="21">
         <f>IF(OR($B239="",$I239=""),"",$I239-IF($J239="",0,$J239))</f>
         <v/>
@@ -13210,19 +13450,39 @@
       </c>
     </row>
     <row r="240">
-      <c r="A240" s="23" t="n"/>
-      <c r="B240" s="23" t="n"/>
-      <c r="C240" s="23" t="n"/>
-      <c r="D240" s="24" t="n"/>
-      <c r="E240" s="25" t="n"/>
-      <c r="F240" s="26" t="n"/>
-      <c r="G240" s="24" t="n"/>
-      <c r="H240" s="25" t="n"/>
+      <c r="A240" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-23126092590709</t>
+        </is>
+      </c>
+      <c r="B240" s="23" t="inlineStr">
+        <is>
+          <t>STEELCAS</t>
+        </is>
+      </c>
+      <c r="C240" s="23" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="D240" s="24" t="n">
+        <v>46290</v>
+      </c>
+      <c r="E240" s="25" t="n">
+        <v>375.6216</v>
+      </c>
+      <c r="F240" s="26" t="n">
+        <v>665</v>
+      </c>
+      <c r="G240" s="24" t="inlineStr"/>
+      <c r="H240" s="25" t="inlineStr"/>
       <c r="I240" s="21">
         <f>IF(OR($B240="",$H240=""),"",IF($C240="LONG",($H240-$E240)*$F240,($E240-$H240)*$F240))</f>
         <v/>
       </c>
-      <c r="J240" s="4" t="n"/>
+      <c r="J240" s="4" t="n">
+        <v>50.15</v>
+      </c>
       <c r="K240" s="21">
         <f>IF(OR($B240="",$I240=""),"",$I240-IF($J240="",0,$J240))</f>
         <v/>
@@ -34268,7 +34528,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J108"/>
+  <dimension ref="A1:J112"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -34868,7 +35128,7 @@
     <row r="16">
       <c r="A16" s="27" t="inlineStr">
         <is>
-          <t>BOMDYEING</t>
+          <t>BHAGERIA</t>
         </is>
       </c>
       <c r="B16" s="20">
@@ -34911,7 +35171,7 @@
     <row r="17">
       <c r="A17" s="27" t="inlineStr">
         <is>
-          <t>CHEMPLASTS</t>
+          <t>BOMDYEING</t>
         </is>
       </c>
       <c r="B17" s="20">
@@ -34954,7 +35214,7 @@
     <row r="18">
       <c r="A18" s="27" t="inlineStr">
         <is>
-          <t>DELTACORP</t>
+          <t>CHEMPLASTS</t>
         </is>
       </c>
       <c r="B18" s="20">
@@ -34997,7 +35257,7 @@
     <row r="19">
       <c r="A19" s="27" t="inlineStr">
         <is>
-          <t>EIEL</t>
+          <t>DELTACORP</t>
         </is>
       </c>
       <c r="B19" s="20">
@@ -35040,7 +35300,7 @@
     <row r="20">
       <c r="A20" s="27" t="inlineStr">
         <is>
-          <t>EMUDHRA</t>
+          <t>EIEL</t>
         </is>
       </c>
       <c r="B20" s="20">
@@ -35083,7 +35343,7 @@
     <row r="21">
       <c r="A21" s="27" t="inlineStr">
         <is>
-          <t>FILATEX</t>
+          <t>EMUDHRA</t>
         </is>
       </c>
       <c r="B21" s="20">
@@ -35126,7 +35386,7 @@
     <row r="22">
       <c r="A22" s="27" t="inlineStr">
         <is>
-          <t>FMGOETZE</t>
+          <t>FILATEX</t>
         </is>
       </c>
       <c r="B22" s="20">
@@ -35169,7 +35429,7 @@
     <row r="23">
       <c r="A23" s="27" t="inlineStr">
         <is>
-          <t>FOSECOIND</t>
+          <t>FMGOETZE</t>
         </is>
       </c>
       <c r="B23" s="20">
@@ -35212,7 +35472,7 @@
     <row r="24">
       <c r="A24" s="27" t="inlineStr">
         <is>
-          <t>FRONTSP</t>
+          <t>FOSECOIND</t>
         </is>
       </c>
       <c r="B24" s="20">
@@ -35255,7 +35515,7 @@
     <row r="25">
       <c r="A25" s="27" t="inlineStr">
         <is>
-          <t>GKENERGY</t>
+          <t>FRONTSP</t>
         </is>
       </c>
       <c r="B25" s="20">
@@ -35298,7 +35558,7 @@
     <row r="26">
       <c r="A26" s="27" t="inlineStr">
         <is>
-          <t>GNA</t>
+          <t>GKENERGY</t>
         </is>
       </c>
       <c r="B26" s="20">
@@ -35341,7 +35601,7 @@
     <row r="27">
       <c r="A27" s="27" t="inlineStr">
         <is>
-          <t>GNRL</t>
+          <t>GNA</t>
         </is>
       </c>
       <c r="B27" s="20">
@@ -35384,7 +35644,7 @@
     <row r="28">
       <c r="A28" s="27" t="inlineStr">
         <is>
-          <t>GOCLCORP</t>
+          <t>GNRL</t>
         </is>
       </c>
       <c r="B28" s="20">
@@ -35427,7 +35687,7 @@
     <row r="29">
       <c r="A29" s="27" t="inlineStr">
         <is>
-          <t>GOPAL</t>
+          <t>GOCLCORP</t>
         </is>
       </c>
       <c r="B29" s="20">
@@ -35470,7 +35730,7 @@
     <row r="30">
       <c r="A30" s="27" t="inlineStr">
         <is>
-          <t>GRAUWEIL</t>
+          <t>GOPAL</t>
         </is>
       </c>
       <c r="B30" s="20">
@@ -35513,7 +35773,7 @@
     <row r="31">
       <c r="A31" s="27" t="inlineStr">
         <is>
-          <t>GREAVESCOT</t>
+          <t>GRAUWEIL</t>
         </is>
       </c>
       <c r="B31" s="20">
@@ -35556,7 +35816,7 @@
     <row r="32">
       <c r="A32" s="27" t="inlineStr">
         <is>
-          <t>GUJTHEM</t>
+          <t>GREAVESCOT</t>
         </is>
       </c>
       <c r="B32" s="20">
@@ -35599,7 +35859,7 @@
     <row r="33">
       <c r="A33" s="27" t="inlineStr">
         <is>
-          <t>HERITGFOOD</t>
+          <t>GUJTHEM</t>
         </is>
       </c>
       <c r="B33" s="20">
@@ -35642,7 +35902,7 @@
     <row r="34">
       <c r="A34" s="27" t="inlineStr">
         <is>
-          <t>HIKAL</t>
+          <t>HERITGFOOD</t>
         </is>
       </c>
       <c r="B34" s="20">
@@ -35685,7 +35945,7 @@
     <row r="35">
       <c r="A35" s="27" t="inlineStr">
         <is>
-          <t>HINDOILEXP</t>
+          <t>HIKAL</t>
         </is>
       </c>
       <c r="B35" s="20">
@@ -35728,7 +35988,7 @@
     <row r="36">
       <c r="A36" s="27" t="inlineStr">
         <is>
-          <t>HUBTOWN</t>
+          <t>HINDOILEXP</t>
         </is>
       </c>
       <c r="B36" s="20">
@@ -35771,7 +36031,7 @@
     <row r="37">
       <c r="A37" s="27" t="inlineStr">
         <is>
-          <t>INDIAGLYCO</t>
+          <t>HUBTOWN</t>
         </is>
       </c>
       <c r="B37" s="20">
@@ -35814,7 +36074,7 @@
     <row r="38">
       <c r="A38" s="27" t="inlineStr">
         <is>
-          <t>INDNIPPON</t>
+          <t>INDIAGLYCO</t>
         </is>
       </c>
       <c r="B38" s="20">
@@ -35857,7 +36117,7 @@
     <row r="39">
       <c r="A39" s="27" t="inlineStr">
         <is>
-          <t>INDOCO</t>
+          <t>INDNIPPON</t>
         </is>
       </c>
       <c r="B39" s="20">
@@ -35900,7 +36160,7 @@
     <row r="40">
       <c r="A40" s="27" t="inlineStr">
         <is>
-          <t>INDORAMA</t>
+          <t>INDOCO</t>
         </is>
       </c>
       <c r="B40" s="20">
@@ -35943,7 +36203,7 @@
     <row r="41">
       <c r="A41" s="27" t="inlineStr">
         <is>
-          <t>IPL</t>
+          <t>INDORAMA</t>
         </is>
       </c>
       <c r="B41" s="20">
@@ -35986,7 +36246,7 @@
     <row r="42">
       <c r="A42" s="27" t="inlineStr">
         <is>
-          <t>JASH</t>
+          <t>IPL</t>
         </is>
       </c>
       <c r="B42" s="20">
@@ -36029,7 +36289,7 @@
     <row r="43">
       <c r="A43" s="27" t="inlineStr">
         <is>
-          <t>JAYKAY</t>
+          <t>JASH</t>
         </is>
       </c>
       <c r="B43" s="20">
@@ -36072,7 +36332,7 @@
     <row r="44">
       <c r="A44" s="27" t="inlineStr">
         <is>
-          <t>JGCHEM</t>
+          <t>JAYKAY</t>
         </is>
       </c>
       <c r="B44" s="20">
@@ -36115,7 +36375,7 @@
     <row r="45">
       <c r="A45" s="27" t="inlineStr">
         <is>
-          <t>KCP</t>
+          <t>JGCHEM</t>
         </is>
       </c>
       <c r="B45" s="20">
@@ -36158,7 +36418,7 @@
     <row r="46">
       <c r="A46" s="27" t="inlineStr">
         <is>
-          <t>KIRIINDUS</t>
+          <t>KCP</t>
         </is>
       </c>
       <c r="B46" s="20">
@@ -36201,7 +36461,7 @@
     <row r="47">
       <c r="A47" s="27" t="inlineStr">
         <is>
-          <t>KIRLOSIND</t>
+          <t>KIRIINDUS</t>
         </is>
       </c>
       <c r="B47" s="20">
@@ -36244,7 +36504,7 @@
     <row r="48">
       <c r="A48" s="27" t="inlineStr">
         <is>
-          <t>KLBRENG-B</t>
+          <t>KIRLOSIND</t>
         </is>
       </c>
       <c r="B48" s="20">
@@ -36287,7 +36547,7 @@
     <row r="49">
       <c r="A49" s="27" t="inlineStr">
         <is>
-          <t>KROSS</t>
+          <t>KLBRENG-B</t>
         </is>
       </c>
       <c r="B49" s="20">
@@ -36330,7 +36590,7 @@
     <row r="50">
       <c r="A50" s="27" t="inlineStr">
         <is>
-          <t>KSCL</t>
+          <t>KROSS</t>
         </is>
       </c>
       <c r="B50" s="20">
@@ -36373,7 +36633,7 @@
     <row r="51">
       <c r="A51" s="27" t="inlineStr">
         <is>
-          <t>KSL</t>
+          <t>KSCL</t>
         </is>
       </c>
       <c r="B51" s="20">
@@ -36416,7 +36676,7 @@
     <row r="52">
       <c r="A52" s="27" t="inlineStr">
         <is>
-          <t>LUXIND</t>
+          <t>KSL</t>
         </is>
       </c>
       <c r="B52" s="20">
@@ -36459,7 +36719,7 @@
     <row r="53">
       <c r="A53" s="27" t="inlineStr">
         <is>
-          <t>MAITHANALL</t>
+          <t>LUXIND</t>
         </is>
       </c>
       <c r="B53" s="20">
@@ -36502,7 +36762,7 @@
     <row r="54">
       <c r="A54" s="27" t="inlineStr">
         <is>
-          <t>MANGLMCEM</t>
+          <t>MAITHANALL</t>
         </is>
       </c>
       <c r="B54" s="20">
@@ -36545,7 +36805,7 @@
     <row r="55">
       <c r="A55" s="27" t="inlineStr">
         <is>
-          <t>MASTEK</t>
+          <t>MANGLMCEM</t>
         </is>
       </c>
       <c r="B55" s="20">
@@ -36588,7 +36848,7 @@
     <row r="56">
       <c r="A56" s="27" t="inlineStr">
         <is>
-          <t>MOBIKWIK</t>
+          <t>MASTEK</t>
         </is>
       </c>
       <c r="B56" s="20">
@@ -36631,7 +36891,7 @@
     <row r="57">
       <c r="A57" s="27" t="inlineStr">
         <is>
-          <t>MUKANDLTD</t>
+          <t>MOBIKWIK</t>
         </is>
       </c>
       <c r="B57" s="20">
@@ -36674,7 +36934,7 @@
     <row r="58">
       <c r="A58" s="27" t="inlineStr">
         <is>
-          <t>NETWORK18</t>
+          <t>MUKANDLTD</t>
         </is>
       </c>
       <c r="B58" s="20">
@@ -36717,7 +36977,7 @@
     <row r="59">
       <c r="A59" s="27" t="inlineStr">
         <is>
-          <t>NILKAMAL</t>
+          <t>NETWORK18</t>
         </is>
       </c>
       <c r="B59" s="20">
@@ -36760,7 +37020,7 @@
     <row r="60">
       <c r="A60" s="27" t="inlineStr">
         <is>
-          <t>NORTHARC</t>
+          <t>NILKAMAL</t>
         </is>
       </c>
       <c r="B60" s="20">
@@ -36803,7 +37063,7 @@
     <row r="61">
       <c r="A61" s="27" t="inlineStr">
         <is>
-          <t>NOVARTIND</t>
+          <t>NORTHARC</t>
         </is>
       </c>
       <c r="B61" s="20">
@@ -36846,7 +37106,7 @@
     <row r="62">
       <c r="A62" s="27" t="inlineStr">
         <is>
-          <t>NPST</t>
+          <t>NOVARTIND</t>
         </is>
       </c>
       <c r="B62" s="20">
@@ -36889,7 +37149,7 @@
     <row r="63">
       <c r="A63" s="27" t="inlineStr">
         <is>
-          <t>NRBBEARING</t>
+          <t>NPST</t>
         </is>
       </c>
       <c r="B63" s="20">
@@ -36932,7 +37192,7 @@
     <row r="64">
       <c r="A64" s="27" t="inlineStr">
         <is>
-          <t>OMAXE</t>
+          <t>NRBBEARING</t>
         </is>
       </c>
       <c r="B64" s="20">
@@ -36975,7 +37235,7 @@
     <row r="65">
       <c r="A65" s="27" t="inlineStr">
         <is>
-          <t>ONEPOINT</t>
+          <t>OMAXE</t>
         </is>
       </c>
       <c r="B65" s="20">
@@ -37018,7 +37278,7 @@
     <row r="66">
       <c r="A66" s="27" t="inlineStr">
         <is>
-          <t>OPTIEMUS</t>
+          <t>ONEPOINT</t>
         </is>
       </c>
       <c r="B66" s="20">
@@ -37061,7 +37321,7 @@
     <row r="67">
       <c r="A67" s="27" t="inlineStr">
         <is>
-          <t>ORIENTHOT</t>
+          <t>OPTIEMUS</t>
         </is>
       </c>
       <c r="B67" s="20">
@@ -37104,7 +37364,7 @@
     <row r="68">
       <c r="A68" s="27" t="inlineStr">
         <is>
-          <t>PACEDIGITK</t>
+          <t>ORIENTHOT</t>
         </is>
       </c>
       <c r="B68" s="20">
@@ -37147,7 +37407,7 @@
     <row r="69">
       <c r="A69" s="27" t="inlineStr">
         <is>
-          <t>PITTIENG</t>
+          <t>PACEDIGITK</t>
         </is>
       </c>
       <c r="B69" s="20">
@@ -37190,7 +37450,7 @@
     <row r="70">
       <c r="A70" s="27" t="inlineStr">
         <is>
-          <t>PROTEAN</t>
+          <t>PITTIENG</t>
         </is>
       </c>
       <c r="B70" s="20">
@@ -37233,7 +37493,7 @@
     <row r="71">
       <c r="A71" s="27" t="inlineStr">
         <is>
-          <t>QUADFUTURE</t>
+          <t>PROTEAN</t>
         </is>
       </c>
       <c r="B71" s="20">
@@ -37276,7 +37536,7 @@
     <row r="72">
       <c r="A72" s="27" t="inlineStr">
         <is>
-          <t>RACLGEAR</t>
+          <t>QUADFUTURE</t>
         </is>
       </c>
       <c r="B72" s="20">
@@ -37319,7 +37579,7 @@
     <row r="73">
       <c r="A73" s="27" t="inlineStr">
         <is>
-          <t>RAMRAT</t>
+          <t>RACLGEAR</t>
         </is>
       </c>
       <c r="B73" s="20">
@@ -37362,7 +37622,7 @@
     <row r="74">
       <c r="A74" s="27" t="inlineStr">
         <is>
-          <t>RAYMOND</t>
+          <t>RAMRAT</t>
         </is>
       </c>
       <c r="B74" s="20">
@@ -37405,7 +37665,7 @@
     <row r="75">
       <c r="A75" s="27" t="inlineStr">
         <is>
-          <t>RAYMONDREL</t>
+          <t>RAYMOND</t>
         </is>
       </c>
       <c r="B75" s="20">
@@ -37448,7 +37708,7 @@
     <row r="76">
       <c r="A76" s="27" t="inlineStr">
         <is>
-          <t>REFEX</t>
+          <t>RAYMONDREL</t>
         </is>
       </c>
       <c r="B76" s="20">
@@ -37491,7 +37751,7 @@
     <row r="77">
       <c r="A77" s="27" t="inlineStr">
         <is>
-          <t>RESPONIND</t>
+          <t>REFEX</t>
         </is>
       </c>
       <c r="B77" s="20">
@@ -37534,7 +37794,7 @@
     <row r="78">
       <c r="A78" s="27" t="inlineStr">
         <is>
-          <t>RML</t>
+          <t>RESPONIND</t>
         </is>
       </c>
       <c r="B78" s="20">
@@ -37577,7 +37837,7 @@
     <row r="79">
       <c r="A79" s="27" t="inlineStr">
         <is>
-          <t>ROSSTECH</t>
+          <t>RML</t>
         </is>
       </c>
       <c r="B79" s="20">
@@ -37620,7 +37880,7 @@
     <row r="80">
       <c r="A80" s="27" t="inlineStr">
         <is>
-          <t>RPGLIFE</t>
+          <t>ROSSTECH</t>
         </is>
       </c>
       <c r="B80" s="20">
@@ -37663,7 +37923,7 @@
     <row r="81">
       <c r="A81" s="27" t="inlineStr">
         <is>
-          <t>SAATVIKGL</t>
+          <t>RPGLIFE</t>
         </is>
       </c>
       <c r="B81" s="20">
@@ -37706,7 +37966,7 @@
     <row r="82">
       <c r="A82" s="27" t="inlineStr">
         <is>
-          <t>SAKAR</t>
+          <t>SAATVIKGL</t>
         </is>
       </c>
       <c r="B82" s="20">
@@ -37749,7 +38009,7 @@
     <row r="83">
       <c r="A83" s="27" t="inlineStr">
         <is>
-          <t>SAMBHV</t>
+          <t>SAKAR</t>
         </is>
       </c>
       <c r="B83" s="20">
@@ -37792,7 +38052,7 @@
     <row r="84">
       <c r="A84" s="27" t="inlineStr">
         <is>
-          <t>SAMHI</t>
+          <t>SAMBHV</t>
         </is>
       </c>
       <c r="B84" s="20">
@@ -37835,7 +38095,7 @@
     <row r="85">
       <c r="A85" s="27" t="inlineStr">
         <is>
-          <t>SHAREINDIA</t>
+          <t>SAMHI</t>
         </is>
       </c>
       <c r="B85" s="20">
@@ -37878,7 +38138,7 @@
     <row r="86">
       <c r="A86" s="27" t="inlineStr">
         <is>
-          <t>SIKA</t>
+          <t>SANGAMIND</t>
         </is>
       </c>
       <c r="B86" s="20">
@@ -37921,7 +38181,7 @@
     <row r="87">
       <c r="A87" s="27" t="inlineStr">
         <is>
-          <t>SINDHUTRAD</t>
+          <t>SHANTIGOLD</t>
         </is>
       </c>
       <c r="B87" s="20">
@@ -37964,7 +38224,7 @@
     <row r="88">
       <c r="A88" s="27" t="inlineStr">
         <is>
-          <t>SMSPHARMA</t>
+          <t>SHAREINDIA</t>
         </is>
       </c>
       <c r="B88" s="20">
@@ -38007,7 +38267,7 @@
     <row r="89">
       <c r="A89" s="27" t="inlineStr">
         <is>
-          <t>SOLARA</t>
+          <t>SHOPERSTOP</t>
         </is>
       </c>
       <c r="B89" s="20">
@@ -38050,7 +38310,7 @@
     <row r="90">
       <c r="A90" s="27" t="inlineStr">
         <is>
-          <t>SOTL</t>
+          <t>SIKA</t>
         </is>
       </c>
       <c r="B90" s="20">
@@ -38093,7 +38353,7 @@
     <row r="91">
       <c r="A91" s="27" t="inlineStr">
         <is>
-          <t>SSWL</t>
+          <t>SINDHUTRAD</t>
         </is>
       </c>
       <c r="B91" s="20">
@@ -38136,7 +38396,7 @@
     <row r="92">
       <c r="A92" s="27" t="inlineStr">
         <is>
-          <t>STEELCAS</t>
+          <t>SMSPHARMA</t>
         </is>
       </c>
       <c r="B92" s="20">
@@ -38179,7 +38439,7 @@
     <row r="93">
       <c r="A93" s="27" t="inlineStr">
         <is>
-          <t>SYMPHONY</t>
+          <t>SOLARA</t>
         </is>
       </c>
       <c r="B93" s="20">
@@ -38222,7 +38482,7 @@
     <row r="94">
       <c r="A94" s="27" t="inlineStr">
         <is>
-          <t>SYNCOMF</t>
+          <t>SOTL</t>
         </is>
       </c>
       <c r="B94" s="20">
@@ -38265,7 +38525,7 @@
     <row r="95">
       <c r="A95" s="27" t="inlineStr">
         <is>
-          <t>TALBROAUTO</t>
+          <t>SSWL</t>
         </is>
       </c>
       <c r="B95" s="20">
@@ -38308,7 +38568,7 @@
     <row r="96">
       <c r="A96" s="27" t="inlineStr">
         <is>
-          <t>TBZ</t>
+          <t>STEELCAS</t>
         </is>
       </c>
       <c r="B96" s="20">
@@ -38351,7 +38611,7 @@
     <row r="97">
       <c r="A97" s="27" t="inlineStr">
         <is>
-          <t>THOMASCOOK</t>
+          <t>SYMPHONY</t>
         </is>
       </c>
       <c r="B97" s="20">
@@ -38394,7 +38654,7 @@
     <row r="98">
       <c r="A98" s="27" t="inlineStr">
         <is>
-          <t>VENKEYS</t>
+          <t>SYNCOMF</t>
         </is>
       </c>
       <c r="B98" s="20">
@@ -38437,7 +38697,7 @@
     <row r="99">
       <c r="A99" s="27" t="inlineStr">
         <is>
-          <t>VENUSPIPES</t>
+          <t>TALBROAUTO</t>
         </is>
       </c>
       <c r="B99" s="20">
@@ -38480,7 +38740,7 @@
     <row r="100">
       <c r="A100" s="27" t="inlineStr">
         <is>
-          <t>VERANDA</t>
+          <t>TBZ</t>
         </is>
       </c>
       <c r="B100" s="20">
@@ -38523,7 +38783,7 @@
     <row r="101">
       <c r="A101" s="27" t="inlineStr">
         <is>
-          <t>VSSL</t>
+          <t>THOMASCOOK</t>
         </is>
       </c>
       <c r="B101" s="20">
@@ -38566,7 +38826,7 @@
     <row r="102">
       <c r="A102" s="27" t="inlineStr">
         <is>
-          <t>WELSPLSOL</t>
+          <t>VENKEYS</t>
         </is>
       </c>
       <c r="B102" s="20">
@@ -38609,7 +38869,7 @@
     <row r="103">
       <c r="A103" s="27" t="inlineStr">
         <is>
-          <t>WENDT</t>
+          <t>VENUSPIPES</t>
         </is>
       </c>
       <c r="B103" s="20">
@@ -38652,7 +38912,7 @@
     <row r="104">
       <c r="A104" s="27" t="inlineStr">
         <is>
-          <t>WINDLAS</t>
+          <t>VERANDA</t>
         </is>
       </c>
       <c r="B104" s="20">
@@ -38695,7 +38955,7 @@
     <row r="105">
       <c r="A105" s="27" t="inlineStr">
         <is>
-          <t>XPROINDIA</t>
+          <t>VSSL</t>
         </is>
       </c>
       <c r="B105" s="20">
@@ -38738,7 +38998,7 @@
     <row r="106">
       <c r="A106" s="27" t="inlineStr">
         <is>
-          <t>ZAGGLE</t>
+          <t>WELSPLSOL</t>
         </is>
       </c>
       <c r="B106" s="20">
@@ -38781,7 +39041,7 @@
     <row r="107">
       <c r="A107" s="27" t="inlineStr">
         <is>
-          <t>ZOTA</t>
+          <t>WENDT</t>
         </is>
       </c>
       <c r="B107" s="20">
@@ -38822,37 +39082,209 @@
       </c>
     </row>
     <row r="108">
-      <c r="A108" s="3" t="inlineStr">
+      <c r="A108" s="27" t="inlineStr">
+        <is>
+          <t>WINDLAS</t>
+        </is>
+      </c>
+      <c r="B108" s="20">
+        <f>COUNTIF('Trade Log'!$B$4:$B$503,$A108)</f>
+        <v/>
+      </c>
+      <c r="C108" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A108,'Trade Log'!$K$4:$K$503,"&gt;0")</f>
+        <v/>
+      </c>
+      <c r="D108" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A108,'Trade Log'!$K$4:$K$503,"&lt;0")</f>
+        <v/>
+      </c>
+      <c r="E108" s="29">
+        <f>IFERROR($C108/$B108,"")</f>
+        <v/>
+      </c>
+      <c r="F108" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A108,'Trade Log'!$I$4:$I$503)</f>
+        <v/>
+      </c>
+      <c r="G108" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A108,'Trade Log'!$K$4:$K$503)</f>
+        <v/>
+      </c>
+      <c r="H108" s="21">
+        <f>IFERROR($G108/$B108,"")</f>
+        <v/>
+      </c>
+      <c r="I108" s="21">
+        <f>IFERROR(_xlfn.MAXIFS('Trade Log'!$K$4:$K$503,'Trade Log'!$B$4:$B$503,$A108),"")</f>
+        <v/>
+      </c>
+      <c r="J108" s="21">
+        <f>IFERROR(_xlfn.MINIFS('Trade Log'!$K$4:$K$503,'Trade Log'!$B$4:$B$503,$A108),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" s="27" t="inlineStr">
+        <is>
+          <t>XPROINDIA</t>
+        </is>
+      </c>
+      <c r="B109" s="20">
+        <f>COUNTIF('Trade Log'!$B$4:$B$503,$A109)</f>
+        <v/>
+      </c>
+      <c r="C109" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A109,'Trade Log'!$K$4:$K$503,"&gt;0")</f>
+        <v/>
+      </c>
+      <c r="D109" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A109,'Trade Log'!$K$4:$K$503,"&lt;0")</f>
+        <v/>
+      </c>
+      <c r="E109" s="29">
+        <f>IFERROR($C109/$B109,"")</f>
+        <v/>
+      </c>
+      <c r="F109" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A109,'Trade Log'!$I$4:$I$503)</f>
+        <v/>
+      </c>
+      <c r="G109" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A109,'Trade Log'!$K$4:$K$503)</f>
+        <v/>
+      </c>
+      <c r="H109" s="21">
+        <f>IFERROR($G109/$B109,"")</f>
+        <v/>
+      </c>
+      <c r="I109" s="21">
+        <f>IFERROR(_xlfn.MAXIFS('Trade Log'!$K$4:$K$503,'Trade Log'!$B$4:$B$503,$A109),"")</f>
+        <v/>
+      </c>
+      <c r="J109" s="21">
+        <f>IFERROR(_xlfn.MINIFS('Trade Log'!$K$4:$K$503,'Trade Log'!$B$4:$B$503,$A109),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" s="27" t="inlineStr">
+        <is>
+          <t>ZAGGLE</t>
+        </is>
+      </c>
+      <c r="B110" s="20">
+        <f>COUNTIF('Trade Log'!$B$4:$B$503,$A110)</f>
+        <v/>
+      </c>
+      <c r="C110" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A110,'Trade Log'!$K$4:$K$503,"&gt;0")</f>
+        <v/>
+      </c>
+      <c r="D110" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A110,'Trade Log'!$K$4:$K$503,"&lt;0")</f>
+        <v/>
+      </c>
+      <c r="E110" s="29">
+        <f>IFERROR($C110/$B110,"")</f>
+        <v/>
+      </c>
+      <c r="F110" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A110,'Trade Log'!$I$4:$I$503)</f>
+        <v/>
+      </c>
+      <c r="G110" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A110,'Trade Log'!$K$4:$K$503)</f>
+        <v/>
+      </c>
+      <c r="H110" s="21">
+        <f>IFERROR($G110/$B110,"")</f>
+        <v/>
+      </c>
+      <c r="I110" s="21">
+        <f>IFERROR(_xlfn.MAXIFS('Trade Log'!$K$4:$K$503,'Trade Log'!$B$4:$B$503,$A110),"")</f>
+        <v/>
+      </c>
+      <c r="J110" s="21">
+        <f>IFERROR(_xlfn.MINIFS('Trade Log'!$K$4:$K$503,'Trade Log'!$B$4:$B$503,$A110),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" s="27" t="inlineStr">
+        <is>
+          <t>ZOTA</t>
+        </is>
+      </c>
+      <c r="B111" s="20">
+        <f>COUNTIF('Trade Log'!$B$4:$B$503,$A111)</f>
+        <v/>
+      </c>
+      <c r="C111" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A111,'Trade Log'!$K$4:$K$503,"&gt;0")</f>
+        <v/>
+      </c>
+      <c r="D111" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A111,'Trade Log'!$K$4:$K$503,"&lt;0")</f>
+        <v/>
+      </c>
+      <c r="E111" s="29">
+        <f>IFERROR($C111/$B111,"")</f>
+        <v/>
+      </c>
+      <c r="F111" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A111,'Trade Log'!$I$4:$I$503)</f>
+        <v/>
+      </c>
+      <c r="G111" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A111,'Trade Log'!$K$4:$K$503)</f>
+        <v/>
+      </c>
+      <c r="H111" s="21">
+        <f>IFERROR($G111/$B111,"")</f>
+        <v/>
+      </c>
+      <c r="I111" s="21">
+        <f>IFERROR(_xlfn.MAXIFS('Trade Log'!$K$4:$K$503,'Trade Log'!$B$4:$B$503,$A111),"")</f>
+        <v/>
+      </c>
+      <c r="J111" s="21">
+        <f>IFERROR(_xlfn.MINIFS('Trade Log'!$K$4:$K$503,'Trade Log'!$B$4:$B$503,$A111),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" s="3" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="B108" s="30">
-        <f>SUM(B4:B107)</f>
-        <v/>
-      </c>
-      <c r="C108" s="30">
-        <f>SUM(C4:C107)</f>
-        <v/>
-      </c>
-      <c r="D108" s="30">
-        <f>SUM(D4:D107)</f>
-        <v/>
-      </c>
-      <c r="E108" s="31">
-        <f>IFERROR(C108/B108,"")</f>
-        <v/>
-      </c>
-      <c r="F108" s="32">
-        <f>SUM(F4:F107)</f>
-        <v/>
-      </c>
-      <c r="G108" s="32">
-        <f>SUM(G4:G107)</f>
-        <v/>
-      </c>
-      <c r="H108" s="32">
-        <f>IFERROR(G108/B108,"")</f>
+      <c r="B112" s="30">
+        <f>SUM(B4:B111)</f>
+        <v/>
+      </c>
+      <c r="C112" s="30">
+        <f>SUM(C4:C111)</f>
+        <v/>
+      </c>
+      <c r="D112" s="30">
+        <f>SUM(D4:D111)</f>
+        <v/>
+      </c>
+      <c r="E112" s="31">
+        <f>IFERROR(C112/B112,"")</f>
+        <v/>
+      </c>
+      <c r="F112" s="32">
+        <f>SUM(F4:F111)</f>
+        <v/>
+      </c>
+      <c r="G112" s="32">
+        <f>SUM(G4:G111)</f>
+        <v/>
+      </c>
+      <c r="H112" s="32">
+        <f>IFERROR(G112/B112,"")</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Regenerate strategy_pnl_simple.xlsx after today's position-file corrections
build_pnl_simple.py reads positions_dhan_long.json/positions_dhan_short.json
directly for the Trade Log -- last commit's fixes (removed FRONTSP's
fictional short, corrected RAYMONDREL's manual exit) hadn't been synced
into the workbook yet. Re-ran it: FRONTSP's fictional short is gone from
the Trade Log, RAYMONDREL now shows its real manual-exit numbers
(+842.06 net) instead of sitting stuck as "open".

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/results/strategy_pnl_simple.xlsx
+++ b/results/strategy_pnl_simple.xlsx
@@ -12835,8 +12835,12 @@
       <c r="F227" s="26" t="n">
         <v>176</v>
       </c>
-      <c r="G227" s="24" t="inlineStr"/>
-      <c r="H227" s="25" t="inlineStr"/>
+      <c r="G227" s="24" t="n">
+        <v>46290</v>
+      </c>
+      <c r="H227" s="25" t="n">
+        <v>713.5029</v>
+      </c>
       <c r="I227" s="21">
         <f>IF(OR($B227="",$H227=""),"",IF($C227="LONG",($H227-$E227)*$F227,($E227-$H227)*$F227))</f>
         <v/>
@@ -13107,12 +13111,12 @@
     <row r="233">
       <c r="A233" s="23" t="inlineStr">
         <is>
-          <t>DHAN-34126092513409</t>
+          <t>DHAN-22126092551109</t>
         </is>
       </c>
       <c r="B233" s="23" t="inlineStr">
         <is>
-          <t>FRONTSP</t>
+          <t>GREAVESCOT</t>
         </is>
       </c>
       <c r="C233" s="23" t="inlineStr">
@@ -13124,16 +13128,16 @@
         <v>46290</v>
       </c>
       <c r="E233" s="25" t="n">
-        <v>1540</v>
+        <v>222.61</v>
       </c>
       <c r="F233" s="26" t="n">
-        <v>82</v>
+        <v>1128</v>
       </c>
       <c r="G233" s="24" t="n">
         <v>46290</v>
       </c>
       <c r="H233" s="25" t="n">
-        <v>1463</v>
+        <v>233.98</v>
       </c>
       <c r="I233" s="21">
         <f>IF(OR($B233="",$H233=""),"",IF($C233="LONG",($H233-$E233)*$F233,($E233-$H233)*$F233))</f>
@@ -13158,12 +13162,12 @@
     <row r="234">
       <c r="A234" s="23" t="inlineStr">
         <is>
-          <t>DHAN-22126092551109</t>
+          <t>DHAN-32126092550109</t>
         </is>
       </c>
       <c r="B234" s="23" t="inlineStr">
         <is>
-          <t>GREAVESCOT</t>
+          <t>INDIAGLYCO</t>
         </is>
       </c>
       <c r="C234" s="23" t="inlineStr">
@@ -13175,16 +13179,16 @@
         <v>46290</v>
       </c>
       <c r="E234" s="25" t="n">
-        <v>222.61</v>
+        <v>308</v>
       </c>
       <c r="F234" s="26" t="n">
-        <v>1128</v>
+        <v>409</v>
       </c>
       <c r="G234" s="24" t="n">
         <v>46290</v>
       </c>
       <c r="H234" s="25" t="n">
-        <v>233.98</v>
+        <v>308.52</v>
       </c>
       <c r="I234" s="21">
         <f>IF(OR($B234="",$H234=""),"",IF($C234="LONG",($H234-$E234)*$F234,($E234-$H234)*$F234))</f>
@@ -13209,12 +13213,12 @@
     <row r="235">
       <c r="A235" s="23" t="inlineStr">
         <is>
-          <t>DHAN-32126092550109</t>
+          <t>DHAN-32126092550209</t>
         </is>
       </c>
       <c r="B235" s="23" t="inlineStr">
         <is>
-          <t>INDIAGLYCO</t>
+          <t>KSCL</t>
         </is>
       </c>
       <c r="C235" s="23" t="inlineStr">
@@ -13226,16 +13230,16 @@
         <v>46290</v>
       </c>
       <c r="E235" s="25" t="n">
-        <v>308</v>
+        <v>826.46</v>
       </c>
       <c r="F235" s="26" t="n">
-        <v>409</v>
+        <v>319</v>
       </c>
       <c r="G235" s="24" t="n">
         <v>46290</v>
       </c>
       <c r="H235" s="25" t="n">
-        <v>308.52</v>
+        <v>785.15</v>
       </c>
       <c r="I235" s="21">
         <f>IF(OR($B235="",$H235=""),"",IF($C235="LONG",($H235-$E235)*$F235,($E235-$H235)*$F235))</f>
@@ -13260,40 +13264,36 @@
     <row r="236">
       <c r="A236" s="23" t="inlineStr">
         <is>
-          <t>DHAN-32126092550209</t>
+          <t>DHAN-limit_entry_multi</t>
         </is>
       </c>
       <c r="B236" s="23" t="inlineStr">
         <is>
-          <t>KSCL</t>
+          <t>SANGAMIND</t>
         </is>
       </c>
       <c r="C236" s="23" t="inlineStr">
         <is>
-          <t>SHORT</t>
+          <t>LONG</t>
         </is>
       </c>
       <c r="D236" s="24" t="n">
         <v>46290</v>
       </c>
       <c r="E236" s="25" t="n">
-        <v>826.46</v>
+        <v>617.5682</v>
       </c>
       <c r="F236" s="26" t="n">
-        <v>319</v>
-      </c>
-      <c r="G236" s="24" t="n">
-        <v>46290</v>
-      </c>
-      <c r="H236" s="25" t="n">
-        <v>785.15</v>
-      </c>
+        <v>404</v>
+      </c>
+      <c r="G236" s="24" t="inlineStr"/>
+      <c r="H236" s="25" t="inlineStr"/>
       <c r="I236" s="21">
         <f>IF(OR($B236="",$H236=""),"",IF($C236="LONG",($H236-$E236)*$F236,($E236-$H236)*$F236))</f>
         <v/>
       </c>
       <c r="J236" s="4" t="n">
-        <v>0</v>
+        <v>67.47</v>
       </c>
       <c r="K236" s="21">
         <f>IF(OR($B236="",$I236=""),"",$I236-IF($J236="",0,$J236))</f>
@@ -13311,12 +13311,12 @@
     <row r="237">
       <c r="A237" s="23" t="inlineStr">
         <is>
-          <t>DHAN-limit_entry_multi</t>
+          <t>DHAN-23126092590809</t>
         </is>
       </c>
       <c r="B237" s="23" t="inlineStr">
         <is>
-          <t>SANGAMIND</t>
+          <t>SHANTIGOLD</t>
         </is>
       </c>
       <c r="C237" s="23" t="inlineStr">
@@ -13328,10 +13328,10 @@
         <v>46290</v>
       </c>
       <c r="E237" s="25" t="n">
-        <v>617.5682</v>
+        <v>325.9933</v>
       </c>
       <c r="F237" s="26" t="n">
-        <v>404</v>
+        <v>771</v>
       </c>
       <c r="G237" s="24" t="inlineStr"/>
       <c r="H237" s="25" t="inlineStr"/>
@@ -13340,7 +13340,7 @@
         <v/>
       </c>
       <c r="J237" s="4" t="n">
-        <v>67.47</v>
+        <v>50.15</v>
       </c>
       <c r="K237" s="21">
         <f>IF(OR($B237="",$I237=""),"",$I237-IF($J237="",0,$J237))</f>
@@ -13358,12 +13358,12 @@
     <row r="238">
       <c r="A238" s="23" t="inlineStr">
         <is>
-          <t>DHAN-23126092590809</t>
+          <t>DHAN-limit_entry_multi</t>
         </is>
       </c>
       <c r="B238" s="23" t="inlineStr">
         <is>
-          <t>SHANTIGOLD</t>
+          <t>SHOPERSTOP</t>
         </is>
       </c>
       <c r="C238" s="23" t="inlineStr">
@@ -13375,10 +13375,10 @@
         <v>46290</v>
       </c>
       <c r="E238" s="25" t="n">
-        <v>325.9933</v>
+        <v>422.7841</v>
       </c>
       <c r="F238" s="26" t="n">
-        <v>771</v>
+        <v>591</v>
       </c>
       <c r="G238" s="24" t="inlineStr"/>
       <c r="H238" s="25" t="inlineStr"/>
@@ -13387,7 +13387,7 @@
         <v/>
       </c>
       <c r="J238" s="4" t="n">
-        <v>50.15</v>
+        <v>67.47</v>
       </c>
       <c r="K238" s="21">
         <f>IF(OR($B238="",$I238=""),"",$I238-IF($J238="",0,$J238))</f>
@@ -13405,12 +13405,12 @@
     <row r="239">
       <c r="A239" s="23" t="inlineStr">
         <is>
-          <t>DHAN-limit_entry_multi</t>
+          <t>DHAN-23126092590709</t>
         </is>
       </c>
       <c r="B239" s="23" t="inlineStr">
         <is>
-          <t>SHOPERSTOP</t>
+          <t>STEELCAS</t>
         </is>
       </c>
       <c r="C239" s="23" t="inlineStr">
@@ -13422,10 +13422,10 @@
         <v>46290</v>
       </c>
       <c r="E239" s="25" t="n">
-        <v>422.7841</v>
+        <v>375.6216</v>
       </c>
       <c r="F239" s="26" t="n">
-        <v>591</v>
+        <v>665</v>
       </c>
       <c r="G239" s="24" t="inlineStr"/>
       <c r="H239" s="25" t="inlineStr"/>
@@ -13434,7 +13434,7 @@
         <v/>
       </c>
       <c r="J239" s="4" t="n">
-        <v>67.47</v>
+        <v>50.15</v>
       </c>
       <c r="K239" s="21">
         <f>IF(OR($B239="",$I239=""),"",$I239-IF($J239="",0,$J239))</f>
@@ -13450,39 +13450,19 @@
       </c>
     </row>
     <row r="240">
-      <c r="A240" s="23" t="inlineStr">
-        <is>
-          <t>DHAN-23126092590709</t>
-        </is>
-      </c>
-      <c r="B240" s="23" t="inlineStr">
-        <is>
-          <t>STEELCAS</t>
-        </is>
-      </c>
-      <c r="C240" s="23" t="inlineStr">
-        <is>
-          <t>LONG</t>
-        </is>
-      </c>
-      <c r="D240" s="24" t="n">
-        <v>46290</v>
-      </c>
-      <c r="E240" s="25" t="n">
-        <v>375.6216</v>
-      </c>
-      <c r="F240" s="26" t="n">
-        <v>665</v>
-      </c>
-      <c r="G240" s="24" t="inlineStr"/>
-      <c r="H240" s="25" t="inlineStr"/>
+      <c r="A240" s="23" t="n"/>
+      <c r="B240" s="23" t="n"/>
+      <c r="C240" s="23" t="n"/>
+      <c r="D240" s="24" t="n"/>
+      <c r="E240" s="25" t="n"/>
+      <c r="F240" s="26" t="n"/>
+      <c r="G240" s="24" t="n"/>
+      <c r="H240" s="25" t="n"/>
       <c r="I240" s="21">
         <f>IF(OR($B240="",$H240=""),"",IF($C240="LONG",($H240-$E240)*$F240,($E240-$H240)*$F240))</f>
         <v/>
       </c>
-      <c r="J240" s="4" t="n">
-        <v>50.15</v>
-      </c>
+      <c r="J240" s="4" t="n"/>
       <c r="K240" s="21">
         <f>IF(OR($B240="",$I240=""),"",$I240-IF($J240="",0,$J240))</f>
         <v/>

</xml_diff>

<commit_message>
Resync strategy_pnl_simple.xlsx with fresh Dhan charges data
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/results/strategy_pnl_simple.xlsx
+++ b/results/strategy_pnl_simple.xlsx
@@ -13093,7 +13093,7 @@
         <v/>
       </c>
       <c r="J232" s="4" t="n">
-        <v>478.29</v>
+        <v>531.9400000000001</v>
       </c>
       <c r="K232" s="21">
         <f>IF(OR($B232="",$I232=""),"",$I232-IF($J232="",0,$J232))</f>
@@ -13340,7 +13340,7 @@
         <v/>
       </c>
       <c r="J237" s="4" t="n">
-        <v>475.34</v>
+        <v>526.92</v>
       </c>
       <c r="K237" s="21">
         <f>IF(OR($B237="",$I237=""),"",$I237-IF($J237="",0,$J237))</f>
@@ -13434,7 +13434,7 @@
         <v/>
       </c>
       <c r="J239" s="4" t="n">
-        <v>473.16</v>
+        <v>524.41</v>
       </c>
       <c r="K239" s="21">
         <f>IF(OR($B239="",$I239=""),"",$I239-IF($J239="",0,$J239))</f>

</xml_diff>

<commit_message>
Data update — 2026-09-28 candle + results refresh
</commit_message>
<xml_diff>
--- a/results/strategy_pnl_simple.xlsx
+++ b/results/strategy_pnl_simple.xlsx
@@ -18,7 +18,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Trade Log'!$A$3:$O$503</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Charges'!$A$3:$N$239</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Charges'!$A$3:$N$243</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -14879,8 +14879,12 @@
       <c r="F234" s="26" t="n">
         <v>316</v>
       </c>
-      <c r="G234" s="24" t="inlineStr"/>
-      <c r="H234" s="25" t="inlineStr"/>
+      <c r="G234" s="24" t="n">
+        <v>46293</v>
+      </c>
+      <c r="H234" s="25" t="n">
+        <v>384.93</v>
+      </c>
       <c r="I234" s="21">
         <f>IF(OR($B234="",$H234=""),"",IF($C234="LONG",($H234-$E234)*$F234,($E234-$H234)*$F234))</f>
         <v/>
@@ -14935,8 +14939,12 @@
       <c r="F235" s="26" t="n">
         <v>3254</v>
       </c>
-      <c r="G235" s="24" t="inlineStr"/>
-      <c r="H235" s="25" t="inlineStr"/>
+      <c r="G235" s="24" t="n">
+        <v>46293</v>
+      </c>
+      <c r="H235" s="25" t="n">
+        <v>79</v>
+      </c>
       <c r="I235" s="21">
         <f>IF(OR($B235="",$H235=""),"",IF($C235="LONG",($H235-$E235)*$F235,($E235-$H235)*$F235))</f>
         <v/>
@@ -14991,8 +14999,12 @@
       <c r="F236" s="26" t="n">
         <v>404</v>
       </c>
-      <c r="G236" s="24" t="inlineStr"/>
-      <c r="H236" s="25" t="inlineStr"/>
+      <c r="G236" s="24" t="n">
+        <v>46293</v>
+      </c>
+      <c r="H236" s="25" t="n">
+        <v>616.9</v>
+      </c>
       <c r="I236" s="21">
         <f>IF(OR($B236="",$H236=""),"",IF($C236="LONG",($H236-$E236)*$F236,($E236-$H236)*$F236))</f>
         <v/>
@@ -15047,8 +15059,12 @@
       <c r="F237" s="26" t="n">
         <v>771</v>
       </c>
-      <c r="G237" s="24" t="inlineStr"/>
-      <c r="H237" s="25" t="inlineStr"/>
+      <c r="G237" s="24" t="n">
+        <v>46293</v>
+      </c>
+      <c r="H237" s="25" t="n">
+        <v>310.62</v>
+      </c>
       <c r="I237" s="21">
         <f>IF(OR($B237="",$H237=""),"",IF($C237="LONG",($H237-$E237)*$F237,($E237-$H237)*$F237))</f>
         <v/>
@@ -15103,8 +15119,12 @@
       <c r="F238" s="26" t="n">
         <v>591</v>
       </c>
-      <c r="G238" s="24" t="inlineStr"/>
-      <c r="H238" s="25" t="inlineStr"/>
+      <c r="G238" s="24" t="n">
+        <v>46293</v>
+      </c>
+      <c r="H238" s="25" t="n">
+        <v>421.35</v>
+      </c>
       <c r="I238" s="21">
         <f>IF(OR($B238="",$H238=""),"",IF($C238="LONG",($H238-$E238)*$F238,($E238-$H238)*$F238))</f>
         <v/>
@@ -15159,8 +15179,12 @@
       <c r="F239" s="26" t="n">
         <v>665</v>
       </c>
-      <c r="G239" s="24" t="inlineStr"/>
-      <c r="H239" s="25" t="inlineStr"/>
+      <c r="G239" s="24" t="n">
+        <v>46293</v>
+      </c>
+      <c r="H239" s="25" t="n">
+        <v>376.65</v>
+      </c>
       <c r="I239" s="21">
         <f>IF(OR($B239="",$H239=""),"",IF($C239="LONG",($H239-$E239)*$F239,($E239-$H239)*$F239))</f>
         <v/>
@@ -15191,14 +15215,32 @@
       </c>
     </row>
     <row r="240">
-      <c r="A240" s="23" t="n"/>
-      <c r="B240" s="23" t="n"/>
-      <c r="C240" s="23" t="n"/>
-      <c r="D240" s="24" t="n"/>
-      <c r="E240" s="25" t="n"/>
-      <c r="F240" s="26" t="n"/>
-      <c r="G240" s="24" t="n"/>
-      <c r="H240" s="25" t="n"/>
+      <c r="A240" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-341260928158909</t>
+        </is>
+      </c>
+      <c r="B240" s="23" t="inlineStr">
+        <is>
+          <t>JINDRILL</t>
+        </is>
+      </c>
+      <c r="C240" s="23" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="D240" s="24" t="n">
+        <v>46293</v>
+      </c>
+      <c r="E240" s="25" t="n">
+        <v>625.9431</v>
+      </c>
+      <c r="F240" s="26" t="n">
+        <v>479</v>
+      </c>
+      <c r="G240" s="24" t="inlineStr"/>
+      <c r="H240" s="25" t="inlineStr"/>
       <c r="I240" s="21">
         <f>IF(OR($B240="",$H240=""),"",IF($C240="LONG",($H240-$E240)*$F240,($E240-$H240)*$F240))</f>
         <v/>
@@ -15207,7 +15249,9 @@
         <f>IF(OR($B240="",$I240="",$E240=0,$F240=0),"",$I240/($E240*$F240))</f>
         <v/>
       </c>
-      <c r="K240" s="4" t="n"/>
+      <c r="K240" s="4" t="n">
+        <v>50.15</v>
+      </c>
       <c r="L240" s="21">
         <f>IF(OR($B240="",$I240=""),"",$I240-IF($K240="",0,$K240))</f>
         <v/>
@@ -15220,17 +15264,39 @@
         <f>IF($B240="","",IF($H240="","Open","Closed"))</f>
         <v/>
       </c>
-      <c r="O240" s="23" t="n"/>
+      <c r="O240" s="23" t="inlineStr">
+        <is>
+          <t>5-10</t>
+        </is>
+      </c>
     </row>
     <row r="241">
-      <c r="A241" s="23" t="n"/>
-      <c r="B241" s="23" t="n"/>
-      <c r="C241" s="23" t="n"/>
-      <c r="D241" s="24" t="n"/>
-      <c r="E241" s="25" t="n"/>
-      <c r="F241" s="26" t="n"/>
-      <c r="G241" s="24" t="n"/>
-      <c r="H241" s="25" t="n"/>
+      <c r="A241" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-limit_entry_multi</t>
+        </is>
+      </c>
+      <c r="B241" s="23" t="inlineStr">
+        <is>
+          <t>SDBL</t>
+        </is>
+      </c>
+      <c r="C241" s="23" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="D241" s="24" t="n">
+        <v>46293</v>
+      </c>
+      <c r="E241" s="25" t="n">
+        <v>80.2633</v>
+      </c>
+      <c r="F241" s="26" t="n">
+        <v>3732</v>
+      </c>
+      <c r="G241" s="24" t="inlineStr"/>
+      <c r="H241" s="25" t="inlineStr"/>
       <c r="I241" s="21">
         <f>IF(OR($B241="",$H241=""),"",IF($C241="LONG",($H241-$E241)*$F241,($E241-$H241)*$F241))</f>
         <v/>
@@ -15239,7 +15305,9 @@
         <f>IF(OR($B241="",$I241="",$E241=0,$F241=0),"",$I241/($E241*$F241))</f>
         <v/>
       </c>
-      <c r="K241" s="4" t="n"/>
+      <c r="K241" s="4" t="n">
+        <v>61.09</v>
+      </c>
       <c r="L241" s="21">
         <f>IF(OR($B241="",$I241=""),"",$I241-IF($K241="",0,$K241))</f>
         <v/>
@@ -15252,17 +15320,39 @@
         <f>IF($B241="","",IF($H241="","Open","Closed"))</f>
         <v/>
       </c>
-      <c r="O241" s="23" t="n"/>
+      <c r="O241" s="23" t="inlineStr">
+        <is>
+          <t>5-10</t>
+        </is>
+      </c>
     </row>
     <row r="242">
-      <c r="A242" s="23" t="n"/>
-      <c r="B242" s="23" t="n"/>
-      <c r="C242" s="23" t="n"/>
-      <c r="D242" s="24" t="n"/>
-      <c r="E242" s="25" t="n"/>
-      <c r="F242" s="26" t="n"/>
-      <c r="G242" s="24" t="n"/>
-      <c r="H242" s="25" t="n"/>
+      <c r="A242" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-341260928159209</t>
+        </is>
+      </c>
+      <c r="B242" s="23" t="inlineStr">
+        <is>
+          <t>SMCGLOBAL</t>
+        </is>
+      </c>
+      <c r="C242" s="23" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="D242" s="24" t="n">
+        <v>46293</v>
+      </c>
+      <c r="E242" s="25" t="n">
+        <v>97.1964</v>
+      </c>
+      <c r="F242" s="26" t="n">
+        <v>3087</v>
+      </c>
+      <c r="G242" s="24" t="inlineStr"/>
+      <c r="H242" s="25" t="inlineStr"/>
       <c r="I242" s="21">
         <f>IF(OR($B242="",$H242=""),"",IF($C242="LONG",($H242-$E242)*$F242,($E242-$H242)*$F242))</f>
         <v/>
@@ -15271,7 +15361,9 @@
         <f>IF(OR($B242="",$I242="",$E242=0,$F242=0),"",$I242/($E242*$F242))</f>
         <v/>
       </c>
-      <c r="K242" s="4" t="n"/>
+      <c r="K242" s="4" t="n">
+        <v>50.15</v>
+      </c>
       <c r="L242" s="21">
         <f>IF(OR($B242="",$I242=""),"",$I242-IF($K242="",0,$K242))</f>
         <v/>
@@ -15284,17 +15376,39 @@
         <f>IF($B242="","",IF($H242="","Open","Closed"))</f>
         <v/>
       </c>
-      <c r="O242" s="23" t="n"/>
+      <c r="O242" s="23" t="inlineStr">
+        <is>
+          <t>15-20</t>
+        </is>
+      </c>
     </row>
     <row r="243">
-      <c r="A243" s="23" t="n"/>
-      <c r="B243" s="23" t="n"/>
-      <c r="C243" s="23" t="n"/>
-      <c r="D243" s="24" t="n"/>
-      <c r="E243" s="25" t="n"/>
-      <c r="F243" s="26" t="n"/>
-      <c r="G243" s="24" t="n"/>
-      <c r="H243" s="25" t="n"/>
+      <c r="A243" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-341260928159109</t>
+        </is>
+      </c>
+      <c r="B243" s="23" t="inlineStr">
+        <is>
+          <t>SYNCOMF</t>
+        </is>
+      </c>
+      <c r="C243" s="23" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="D243" s="24" t="n">
+        <v>46293</v>
+      </c>
+      <c r="E243" s="25" t="n">
+        <v>22.1897</v>
+      </c>
+      <c r="F243" s="26" t="n">
+        <v>13513</v>
+      </c>
+      <c r="G243" s="24" t="inlineStr"/>
+      <c r="H243" s="25" t="inlineStr"/>
       <c r="I243" s="21">
         <f>IF(OR($B243="",$H243=""),"",IF($C243="LONG",($H243-$E243)*$F243,($E243-$H243)*$F243))</f>
         <v/>
@@ -15303,7 +15417,9 @@
         <f>IF(OR($B243="",$I243="",$E243=0,$F243=0),"",$I243/($E243*$F243))</f>
         <v/>
       </c>
-      <c r="K243" s="4" t="n"/>
+      <c r="K243" s="4" t="n">
+        <v>50.15</v>
+      </c>
       <c r="L243" s="21">
         <f>IF(OR($B243="",$I243=""),"",$I243-IF($K243="",0,$K243))</f>
         <v/>
@@ -15316,7 +15432,11 @@
         <f>IF($B243="","",IF($H243="","Open","Closed"))</f>
         <v/>
       </c>
-      <c r="O243" s="23" t="n"/>
+      <c r="O243" s="23" t="inlineStr">
+        <is>
+          <t>10-15</t>
+        </is>
+      </c>
     </row>
     <row r="244">
       <c r="A244" s="23" t="n"/>
@@ -36313,7 +36433,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J112"/>
+  <dimension ref="A1:J115"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -38203,7 +38323,7 @@
     <row r="46">
       <c r="A46" s="27" t="inlineStr">
         <is>
-          <t>KCP</t>
+          <t>JINDRILL</t>
         </is>
       </c>
       <c r="B46" s="20">
@@ -38246,7 +38366,7 @@
     <row r="47">
       <c r="A47" s="27" t="inlineStr">
         <is>
-          <t>KIRIINDUS</t>
+          <t>KCP</t>
         </is>
       </c>
       <c r="B47" s="20">
@@ -38289,7 +38409,7 @@
     <row r="48">
       <c r="A48" s="27" t="inlineStr">
         <is>
-          <t>KIRLOSIND</t>
+          <t>KIRIINDUS</t>
         </is>
       </c>
       <c r="B48" s="20">
@@ -38332,7 +38452,7 @@
     <row r="49">
       <c r="A49" s="27" t="inlineStr">
         <is>
-          <t>KLBRENG-B</t>
+          <t>KIRLOSIND</t>
         </is>
       </c>
       <c r="B49" s="20">
@@ -38375,7 +38495,7 @@
     <row r="50">
       <c r="A50" s="27" t="inlineStr">
         <is>
-          <t>KROSS</t>
+          <t>KLBRENG-B</t>
         </is>
       </c>
       <c r="B50" s="20">
@@ -38418,7 +38538,7 @@
     <row r="51">
       <c r="A51" s="27" t="inlineStr">
         <is>
-          <t>KSCL</t>
+          <t>KROSS</t>
         </is>
       </c>
       <c r="B51" s="20">
@@ -38461,7 +38581,7 @@
     <row r="52">
       <c r="A52" s="27" t="inlineStr">
         <is>
-          <t>KSL</t>
+          <t>KSCL</t>
         </is>
       </c>
       <c r="B52" s="20">
@@ -38504,7 +38624,7 @@
     <row r="53">
       <c r="A53" s="27" t="inlineStr">
         <is>
-          <t>LUXIND</t>
+          <t>KSL</t>
         </is>
       </c>
       <c r="B53" s="20">
@@ -38547,7 +38667,7 @@
     <row r="54">
       <c r="A54" s="27" t="inlineStr">
         <is>
-          <t>MAITHANALL</t>
+          <t>LUXIND</t>
         </is>
       </c>
       <c r="B54" s="20">
@@ -38590,7 +38710,7 @@
     <row r="55">
       <c r="A55" s="27" t="inlineStr">
         <is>
-          <t>MANGLMCEM</t>
+          <t>MAITHANALL</t>
         </is>
       </c>
       <c r="B55" s="20">
@@ -38633,7 +38753,7 @@
     <row r="56">
       <c r="A56" s="27" t="inlineStr">
         <is>
-          <t>MASTEK</t>
+          <t>MANGLMCEM</t>
         </is>
       </c>
       <c r="B56" s="20">
@@ -38676,7 +38796,7 @@
     <row r="57">
       <c r="A57" s="27" t="inlineStr">
         <is>
-          <t>MOBIKWIK</t>
+          <t>MASTEK</t>
         </is>
       </c>
       <c r="B57" s="20">
@@ -38719,7 +38839,7 @@
     <row r="58">
       <c r="A58" s="27" t="inlineStr">
         <is>
-          <t>MUKANDLTD</t>
+          <t>MOBIKWIK</t>
         </is>
       </c>
       <c r="B58" s="20">
@@ -38762,7 +38882,7 @@
     <row r="59">
       <c r="A59" s="27" t="inlineStr">
         <is>
-          <t>NETWORK18</t>
+          <t>MUKANDLTD</t>
         </is>
       </c>
       <c r="B59" s="20">
@@ -38805,7 +38925,7 @@
     <row r="60">
       <c r="A60" s="27" t="inlineStr">
         <is>
-          <t>NILKAMAL</t>
+          <t>NETWORK18</t>
         </is>
       </c>
       <c r="B60" s="20">
@@ -38848,7 +38968,7 @@
     <row r="61">
       <c r="A61" s="27" t="inlineStr">
         <is>
-          <t>NORTHARC</t>
+          <t>NILKAMAL</t>
         </is>
       </c>
       <c r="B61" s="20">
@@ -38891,7 +39011,7 @@
     <row r="62">
       <c r="A62" s="27" t="inlineStr">
         <is>
-          <t>NOVARTIND</t>
+          <t>NORTHARC</t>
         </is>
       </c>
       <c r="B62" s="20">
@@ -38934,7 +39054,7 @@
     <row r="63">
       <c r="A63" s="27" t="inlineStr">
         <is>
-          <t>NPST</t>
+          <t>NOVARTIND</t>
         </is>
       </c>
       <c r="B63" s="20">
@@ -38977,7 +39097,7 @@
     <row r="64">
       <c r="A64" s="27" t="inlineStr">
         <is>
-          <t>NRBBEARING</t>
+          <t>NPST</t>
         </is>
       </c>
       <c r="B64" s="20">
@@ -39020,7 +39140,7 @@
     <row r="65">
       <c r="A65" s="27" t="inlineStr">
         <is>
-          <t>OMAXE</t>
+          <t>NRBBEARING</t>
         </is>
       </c>
       <c r="B65" s="20">
@@ -39063,7 +39183,7 @@
     <row r="66">
       <c r="A66" s="27" t="inlineStr">
         <is>
-          <t>ONEPOINT</t>
+          <t>OMAXE</t>
         </is>
       </c>
       <c r="B66" s="20">
@@ -39106,7 +39226,7 @@
     <row r="67">
       <c r="A67" s="27" t="inlineStr">
         <is>
-          <t>OPTIEMUS</t>
+          <t>ONEPOINT</t>
         </is>
       </c>
       <c r="B67" s="20">
@@ -39149,7 +39269,7 @@
     <row r="68">
       <c r="A68" s="27" t="inlineStr">
         <is>
-          <t>ORIENTHOT</t>
+          <t>OPTIEMUS</t>
         </is>
       </c>
       <c r="B68" s="20">
@@ -39192,7 +39312,7 @@
     <row r="69">
       <c r="A69" s="27" t="inlineStr">
         <is>
-          <t>PACEDIGITK</t>
+          <t>ORIENTHOT</t>
         </is>
       </c>
       <c r="B69" s="20">
@@ -39235,7 +39355,7 @@
     <row r="70">
       <c r="A70" s="27" t="inlineStr">
         <is>
-          <t>PITTIENG</t>
+          <t>PACEDIGITK</t>
         </is>
       </c>
       <c r="B70" s="20">
@@ -39278,7 +39398,7 @@
     <row r="71">
       <c r="A71" s="27" t="inlineStr">
         <is>
-          <t>PROTEAN</t>
+          <t>PITTIENG</t>
         </is>
       </c>
       <c r="B71" s="20">
@@ -39321,7 +39441,7 @@
     <row r="72">
       <c r="A72" s="27" t="inlineStr">
         <is>
-          <t>QUADFUTURE</t>
+          <t>PROTEAN</t>
         </is>
       </c>
       <c r="B72" s="20">
@@ -39364,7 +39484,7 @@
     <row r="73">
       <c r="A73" s="27" t="inlineStr">
         <is>
-          <t>RACLGEAR</t>
+          <t>QUADFUTURE</t>
         </is>
       </c>
       <c r="B73" s="20">
@@ -39407,7 +39527,7 @@
     <row r="74">
       <c r="A74" s="27" t="inlineStr">
         <is>
-          <t>RAMRAT</t>
+          <t>RACLGEAR</t>
         </is>
       </c>
       <c r="B74" s="20">
@@ -39450,7 +39570,7 @@
     <row r="75">
       <c r="A75" s="27" t="inlineStr">
         <is>
-          <t>RAYMOND</t>
+          <t>RAMRAT</t>
         </is>
       </c>
       <c r="B75" s="20">
@@ -39493,7 +39613,7 @@
     <row r="76">
       <c r="A76" s="27" t="inlineStr">
         <is>
-          <t>RAYMONDREL</t>
+          <t>RAYMOND</t>
         </is>
       </c>
       <c r="B76" s="20">
@@ -39536,7 +39656,7 @@
     <row r="77">
       <c r="A77" s="27" t="inlineStr">
         <is>
-          <t>REFEX</t>
+          <t>RAYMONDREL</t>
         </is>
       </c>
       <c r="B77" s="20">
@@ -39579,7 +39699,7 @@
     <row r="78">
       <c r="A78" s="27" t="inlineStr">
         <is>
-          <t>RESPONIND</t>
+          <t>REFEX</t>
         </is>
       </c>
       <c r="B78" s="20">
@@ -39622,7 +39742,7 @@
     <row r="79">
       <c r="A79" s="27" t="inlineStr">
         <is>
-          <t>RML</t>
+          <t>RESPONIND</t>
         </is>
       </c>
       <c r="B79" s="20">
@@ -39665,7 +39785,7 @@
     <row r="80">
       <c r="A80" s="27" t="inlineStr">
         <is>
-          <t>ROSSTECH</t>
+          <t>RML</t>
         </is>
       </c>
       <c r="B80" s="20">
@@ -39708,7 +39828,7 @@
     <row r="81">
       <c r="A81" s="27" t="inlineStr">
         <is>
-          <t>RPGLIFE</t>
+          <t>ROSSTECH</t>
         </is>
       </c>
       <c r="B81" s="20">
@@ -39751,7 +39871,7 @@
     <row r="82">
       <c r="A82" s="27" t="inlineStr">
         <is>
-          <t>SAATVIKGL</t>
+          <t>RPGLIFE</t>
         </is>
       </c>
       <c r="B82" s="20">
@@ -39794,7 +39914,7 @@
     <row r="83">
       <c r="A83" s="27" t="inlineStr">
         <is>
-          <t>SAKAR</t>
+          <t>SAATVIKGL</t>
         </is>
       </c>
       <c r="B83" s="20">
@@ -39837,7 +39957,7 @@
     <row r="84">
       <c r="A84" s="27" t="inlineStr">
         <is>
-          <t>SAMBHV</t>
+          <t>SAKAR</t>
         </is>
       </c>
       <c r="B84" s="20">
@@ -39880,7 +40000,7 @@
     <row r="85">
       <c r="A85" s="27" t="inlineStr">
         <is>
-          <t>SAMHI</t>
+          <t>SAMBHV</t>
         </is>
       </c>
       <c r="B85" s="20">
@@ -39923,7 +40043,7 @@
     <row r="86">
       <c r="A86" s="27" t="inlineStr">
         <is>
-          <t>SANGAMIND</t>
+          <t>SAMHI</t>
         </is>
       </c>
       <c r="B86" s="20">
@@ -39966,7 +40086,7 @@
     <row r="87">
       <c r="A87" s="27" t="inlineStr">
         <is>
-          <t>SHANTIGOLD</t>
+          <t>SANGAMIND</t>
         </is>
       </c>
       <c r="B87" s="20">
@@ -40009,7 +40129,7 @@
     <row r="88">
       <c r="A88" s="27" t="inlineStr">
         <is>
-          <t>SHAREINDIA</t>
+          <t>SDBL</t>
         </is>
       </c>
       <c r="B88" s="20">
@@ -40052,7 +40172,7 @@
     <row r="89">
       <c r="A89" s="27" t="inlineStr">
         <is>
-          <t>SHOPERSTOP</t>
+          <t>SHANTIGOLD</t>
         </is>
       </c>
       <c r="B89" s="20">
@@ -40095,7 +40215,7 @@
     <row r="90">
       <c r="A90" s="27" t="inlineStr">
         <is>
-          <t>SIKA</t>
+          <t>SHAREINDIA</t>
         </is>
       </c>
       <c r="B90" s="20">
@@ -40138,7 +40258,7 @@
     <row r="91">
       <c r="A91" s="27" t="inlineStr">
         <is>
-          <t>SINDHUTRAD</t>
+          <t>SHOPERSTOP</t>
         </is>
       </c>
       <c r="B91" s="20">
@@ -40181,7 +40301,7 @@
     <row r="92">
       <c r="A92" s="27" t="inlineStr">
         <is>
-          <t>SMSPHARMA</t>
+          <t>SIKA</t>
         </is>
       </c>
       <c r="B92" s="20">
@@ -40224,7 +40344,7 @@
     <row r="93">
       <c r="A93" s="27" t="inlineStr">
         <is>
-          <t>SOLARA</t>
+          <t>SINDHUTRAD</t>
         </is>
       </c>
       <c r="B93" s="20">
@@ -40267,7 +40387,7 @@
     <row r="94">
       <c r="A94" s="27" t="inlineStr">
         <is>
-          <t>SOTL</t>
+          <t>SMCGLOBAL</t>
         </is>
       </c>
       <c r="B94" s="20">
@@ -40310,7 +40430,7 @@
     <row r="95">
       <c r="A95" s="27" t="inlineStr">
         <is>
-          <t>SSWL</t>
+          <t>SMSPHARMA</t>
         </is>
       </c>
       <c r="B95" s="20">
@@ -40353,7 +40473,7 @@
     <row r="96">
       <c r="A96" s="27" t="inlineStr">
         <is>
-          <t>STEELCAS</t>
+          <t>SOLARA</t>
         </is>
       </c>
       <c r="B96" s="20">
@@ -40396,7 +40516,7 @@
     <row r="97">
       <c r="A97" s="27" t="inlineStr">
         <is>
-          <t>SYMPHONY</t>
+          <t>SOTL</t>
         </is>
       </c>
       <c r="B97" s="20">
@@ -40439,7 +40559,7 @@
     <row r="98">
       <c r="A98" s="27" t="inlineStr">
         <is>
-          <t>SYNCOMF</t>
+          <t>SSWL</t>
         </is>
       </c>
       <c r="B98" s="20">
@@ -40482,7 +40602,7 @@
     <row r="99">
       <c r="A99" s="27" t="inlineStr">
         <is>
-          <t>TALBROAUTO</t>
+          <t>STEELCAS</t>
         </is>
       </c>
       <c r="B99" s="20">
@@ -40525,7 +40645,7 @@
     <row r="100">
       <c r="A100" s="27" t="inlineStr">
         <is>
-          <t>TBZ</t>
+          <t>SYMPHONY</t>
         </is>
       </c>
       <c r="B100" s="20">
@@ -40568,7 +40688,7 @@
     <row r="101">
       <c r="A101" s="27" t="inlineStr">
         <is>
-          <t>THOMASCOOK</t>
+          <t>SYNCOMF</t>
         </is>
       </c>
       <c r="B101" s="20">
@@ -40611,7 +40731,7 @@
     <row r="102">
       <c r="A102" s="27" t="inlineStr">
         <is>
-          <t>VENKEYS</t>
+          <t>TALBROAUTO</t>
         </is>
       </c>
       <c r="B102" s="20">
@@ -40654,7 +40774,7 @@
     <row r="103">
       <c r="A103" s="27" t="inlineStr">
         <is>
-          <t>VENUSPIPES</t>
+          <t>TBZ</t>
         </is>
       </c>
       <c r="B103" s="20">
@@ -40697,7 +40817,7 @@
     <row r="104">
       <c r="A104" s="27" t="inlineStr">
         <is>
-          <t>VERANDA</t>
+          <t>THOMASCOOK</t>
         </is>
       </c>
       <c r="B104" s="20">
@@ -40740,7 +40860,7 @@
     <row r="105">
       <c r="A105" s="27" t="inlineStr">
         <is>
-          <t>VSSL</t>
+          <t>VENKEYS</t>
         </is>
       </c>
       <c r="B105" s="20">
@@ -40783,7 +40903,7 @@
     <row r="106">
       <c r="A106" s="27" t="inlineStr">
         <is>
-          <t>WELSPLSOL</t>
+          <t>VENUSPIPES</t>
         </is>
       </c>
       <c r="B106" s="20">
@@ -40826,7 +40946,7 @@
     <row r="107">
       <c r="A107" s="27" t="inlineStr">
         <is>
-          <t>WENDT</t>
+          <t>VERANDA</t>
         </is>
       </c>
       <c r="B107" s="20">
@@ -40869,7 +40989,7 @@
     <row r="108">
       <c r="A108" s="27" t="inlineStr">
         <is>
-          <t>WINDLAS</t>
+          <t>VSSL</t>
         </is>
       </c>
       <c r="B108" s="20">
@@ -40912,7 +41032,7 @@
     <row r="109">
       <c r="A109" s="27" t="inlineStr">
         <is>
-          <t>XPROINDIA</t>
+          <t>WELSPLSOL</t>
         </is>
       </c>
       <c r="B109" s="20">
@@ -40955,7 +41075,7 @@
     <row r="110">
       <c r="A110" s="27" t="inlineStr">
         <is>
-          <t>ZAGGLE</t>
+          <t>WENDT</t>
         </is>
       </c>
       <c r="B110" s="20">
@@ -40998,7 +41118,7 @@
     <row r="111">
       <c r="A111" s="27" t="inlineStr">
         <is>
-          <t>ZOTA</t>
+          <t>WINDLAS</t>
         </is>
       </c>
       <c r="B111" s="20">
@@ -41039,37 +41159,166 @@
       </c>
     </row>
     <row r="112">
-      <c r="A112" s="3" t="inlineStr">
+      <c r="A112" s="27" t="inlineStr">
+        <is>
+          <t>XPROINDIA</t>
+        </is>
+      </c>
+      <c r="B112" s="20">
+        <f>COUNTIF('Trade Log'!$B$4:$B$503,$A112)</f>
+        <v/>
+      </c>
+      <c r="C112" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A112,'Trade Log'!$L$4:$L$503,"&gt;0")</f>
+        <v/>
+      </c>
+      <c r="D112" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A112,'Trade Log'!$L$4:$L$503,"&lt;0")</f>
+        <v/>
+      </c>
+      <c r="E112" s="22">
+        <f>IFERROR($C112/$B112,"")</f>
+        <v/>
+      </c>
+      <c r="F112" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A112,'Trade Log'!$I$4:$I$503)</f>
+        <v/>
+      </c>
+      <c r="G112" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A112,'Trade Log'!$L$4:$L$503)</f>
+        <v/>
+      </c>
+      <c r="H112" s="21">
+        <f>IFERROR($G112/$B112,"")</f>
+        <v/>
+      </c>
+      <c r="I112" s="21">
+        <f>IFERROR(_xlfn.MAXIFS('Trade Log'!$L$4:$L$503,'Trade Log'!$B$4:$B$503,$A112),"")</f>
+        <v/>
+      </c>
+      <c r="J112" s="21">
+        <f>IFERROR(_xlfn.MINIFS('Trade Log'!$L$4:$L$503,'Trade Log'!$B$4:$B$503,$A112),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" s="27" t="inlineStr">
+        <is>
+          <t>ZAGGLE</t>
+        </is>
+      </c>
+      <c r="B113" s="20">
+        <f>COUNTIF('Trade Log'!$B$4:$B$503,$A113)</f>
+        <v/>
+      </c>
+      <c r="C113" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A113,'Trade Log'!$L$4:$L$503,"&gt;0")</f>
+        <v/>
+      </c>
+      <c r="D113" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A113,'Trade Log'!$L$4:$L$503,"&lt;0")</f>
+        <v/>
+      </c>
+      <c r="E113" s="22">
+        <f>IFERROR($C113/$B113,"")</f>
+        <v/>
+      </c>
+      <c r="F113" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A113,'Trade Log'!$I$4:$I$503)</f>
+        <v/>
+      </c>
+      <c r="G113" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A113,'Trade Log'!$L$4:$L$503)</f>
+        <v/>
+      </c>
+      <c r="H113" s="21">
+        <f>IFERROR($G113/$B113,"")</f>
+        <v/>
+      </c>
+      <c r="I113" s="21">
+        <f>IFERROR(_xlfn.MAXIFS('Trade Log'!$L$4:$L$503,'Trade Log'!$B$4:$B$503,$A113),"")</f>
+        <v/>
+      </c>
+      <c r="J113" s="21">
+        <f>IFERROR(_xlfn.MINIFS('Trade Log'!$L$4:$L$503,'Trade Log'!$B$4:$B$503,$A113),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" s="27" t="inlineStr">
+        <is>
+          <t>ZOTA</t>
+        </is>
+      </c>
+      <c r="B114" s="20">
+        <f>COUNTIF('Trade Log'!$B$4:$B$503,$A114)</f>
+        <v/>
+      </c>
+      <c r="C114" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A114,'Trade Log'!$L$4:$L$503,"&gt;0")</f>
+        <v/>
+      </c>
+      <c r="D114" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A114,'Trade Log'!$L$4:$L$503,"&lt;0")</f>
+        <v/>
+      </c>
+      <c r="E114" s="22">
+        <f>IFERROR($C114/$B114,"")</f>
+        <v/>
+      </c>
+      <c r="F114" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A114,'Trade Log'!$I$4:$I$503)</f>
+        <v/>
+      </c>
+      <c r="G114" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A114,'Trade Log'!$L$4:$L$503)</f>
+        <v/>
+      </c>
+      <c r="H114" s="21">
+        <f>IFERROR($G114/$B114,"")</f>
+        <v/>
+      </c>
+      <c r="I114" s="21">
+        <f>IFERROR(_xlfn.MAXIFS('Trade Log'!$L$4:$L$503,'Trade Log'!$B$4:$B$503,$A114),"")</f>
+        <v/>
+      </c>
+      <c r="J114" s="21">
+        <f>IFERROR(_xlfn.MINIFS('Trade Log'!$L$4:$L$503,'Trade Log'!$B$4:$B$503,$A114),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" s="3" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="B112" s="30">
-        <f>SUM(B4:B111)</f>
-        <v/>
-      </c>
-      <c r="C112" s="30">
-        <f>SUM(C4:C111)</f>
-        <v/>
-      </c>
-      <c r="D112" s="30">
-        <f>SUM(D4:D111)</f>
-        <v/>
-      </c>
-      <c r="E112" s="31">
-        <f>IFERROR(C112/B112,"")</f>
-        <v/>
-      </c>
-      <c r="F112" s="32">
-        <f>SUM(F4:F111)</f>
-        <v/>
-      </c>
-      <c r="G112" s="32">
-        <f>SUM(G4:G111)</f>
-        <v/>
-      </c>
-      <c r="H112" s="32">
-        <f>IFERROR(G112/B112,"")</f>
+      <c r="B115" s="30">
+        <f>SUM(B4:B114)</f>
+        <v/>
+      </c>
+      <c r="C115" s="30">
+        <f>SUM(C4:C114)</f>
+        <v/>
+      </c>
+      <c r="D115" s="30">
+        <f>SUM(D4:D114)</f>
+        <v/>
+      </c>
+      <c r="E115" s="31">
+        <f>IFERROR(C115/B115,"")</f>
+        <v/>
+      </c>
+      <c r="F115" s="32">
+        <f>SUM(F4:F114)</f>
+        <v/>
+      </c>
+      <c r="G115" s="32">
+        <f>SUM(G4:G114)</f>
+        <v/>
+      </c>
+      <c r="H115" s="32">
+        <f>IFERROR(G115/B115,"")</f>
         <v/>
       </c>
     </row>
@@ -41088,7 +41337,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N240"/>
+  <dimension ref="A1:N244"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -52939,7 +53188,9 @@
           <t>LONG</t>
         </is>
       </c>
-      <c r="D234" s="24" t="inlineStr"/>
+      <c r="D234" s="24" t="n">
+        <v>46293</v>
+      </c>
       <c r="E234" s="4" t="n">
         <v>0</v>
       </c>
@@ -52988,7 +53239,9 @@
           <t>LONG</t>
         </is>
       </c>
-      <c r="D235" s="24" t="inlineStr"/>
+      <c r="D235" s="24" t="n">
+        <v>46293</v>
+      </c>
       <c r="E235" s="4" t="n">
         <v>20</v>
       </c>
@@ -53037,7 +53290,9 @@
           <t>LONG</t>
         </is>
       </c>
-      <c r="D236" s="24" t="inlineStr"/>
+      <c r="D236" s="24" t="n">
+        <v>46293</v>
+      </c>
       <c r="E236" s="4" t="n">
         <v>0</v>
       </c>
@@ -53086,7 +53341,9 @@
           <t>LONG</t>
         </is>
       </c>
-      <c r="D237" s="24" t="inlineStr"/>
+      <c r="D237" s="24" t="n">
+        <v>46293</v>
+      </c>
       <c r="E237" s="4" t="n">
         <v>20</v>
       </c>
@@ -53135,7 +53392,9 @@
           <t>LONG</t>
         </is>
       </c>
-      <c r="D238" s="24" t="inlineStr"/>
+      <c r="D238" s="24" t="n">
+        <v>46293</v>
+      </c>
       <c r="E238" s="4" t="n">
         <v>0</v>
       </c>
@@ -53184,7 +53443,9 @@
           <t>LONG</t>
         </is>
       </c>
-      <c r="D239" s="24" t="inlineStr"/>
+      <c r="D239" s="24" t="n">
+        <v>46293</v>
+      </c>
       <c r="E239" s="4" t="n">
         <v>20</v>
       </c>
@@ -53218,54 +53479,250 @@
       </c>
     </row>
     <row r="240">
-      <c r="A240" s="3" t="inlineStr">
+      <c r="A240" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-341260928158909</t>
+        </is>
+      </c>
+      <c r="B240" s="23" t="inlineStr">
+        <is>
+          <t>JINDRILL</t>
+        </is>
+      </c>
+      <c r="C240" s="23" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="D240" s="24" t="inlineStr"/>
+      <c r="E240" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F240" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G240" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H240" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I240" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J240" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K240" s="4" t="n">
+        <v>14.75</v>
+      </c>
+      <c r="L240" s="4" t="n">
+        <v>35.4</v>
+      </c>
+      <c r="M240" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="N240" s="21">
+        <f>SUM(E240:M240)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="241">
+      <c r="A241" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-limit_entry_multi</t>
+        </is>
+      </c>
+      <c r="B241" s="23" t="inlineStr">
+        <is>
+          <t>SDBL</t>
+        </is>
+      </c>
+      <c r="C241" s="23" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="D241" s="24" t="inlineStr"/>
+      <c r="E241" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F241" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G241" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H241" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I241" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J241" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K241" s="4" t="n">
+        <v>14.75</v>
+      </c>
+      <c r="L241" s="4" t="n">
+        <v>35.4</v>
+      </c>
+      <c r="M241" s="4" t="n">
+        <v>10.94</v>
+      </c>
+      <c r="N241" s="21">
+        <f>SUM(E241:M241)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="242">
+      <c r="A242" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-341260928159209</t>
+        </is>
+      </c>
+      <c r="B242" s="23" t="inlineStr">
+        <is>
+          <t>SMCGLOBAL</t>
+        </is>
+      </c>
+      <c r="C242" s="23" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="D242" s="24" t="inlineStr"/>
+      <c r="E242" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F242" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G242" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H242" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I242" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J242" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K242" s="4" t="n">
+        <v>14.75</v>
+      </c>
+      <c r="L242" s="4" t="n">
+        <v>35.4</v>
+      </c>
+      <c r="M242" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="N242" s="21">
+        <f>SUM(E242:M242)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="243">
+      <c r="A243" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-341260928159109</t>
+        </is>
+      </c>
+      <c r="B243" s="23" t="inlineStr">
+        <is>
+          <t>SYNCOMF</t>
+        </is>
+      </c>
+      <c r="C243" s="23" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="D243" s="24" t="inlineStr"/>
+      <c r="E243" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F243" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G243" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H243" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I243" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J243" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K243" s="4" t="n">
+        <v>14.75</v>
+      </c>
+      <c r="L243" s="4" t="n">
+        <v>35.4</v>
+      </c>
+      <c r="M243" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="N243" s="21">
+        <f>SUM(E243:M243)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="244">
+      <c r="A244" s="3" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="E240" s="32">
-        <f>SUM(E4:E239)</f>
-        <v/>
-      </c>
-      <c r="F240" s="32">
-        <f>SUM(F4:F239)</f>
-        <v/>
-      </c>
-      <c r="G240" s="32">
-        <f>SUM(G4:G239)</f>
-        <v/>
-      </c>
-      <c r="H240" s="32">
-        <f>SUM(H4:H239)</f>
-        <v/>
-      </c>
-      <c r="I240" s="32">
-        <f>SUM(I4:I239)</f>
-        <v/>
-      </c>
-      <c r="J240" s="32">
-        <f>SUM(J4:J239)</f>
-        <v/>
-      </c>
-      <c r="K240" s="32">
-        <f>SUM(K4:K239)</f>
-        <v/>
-      </c>
-      <c r="L240" s="32">
-        <f>SUM(L4:L239)</f>
-        <v/>
-      </c>
-      <c r="M240" s="32">
-        <f>SUM(M4:M239)</f>
-        <v/>
-      </c>
-      <c r="N240" s="32">
-        <f>SUM(N4:N239)</f>
+      <c r="E244" s="32">
+        <f>SUM(E4:E243)</f>
+        <v/>
+      </c>
+      <c r="F244" s="32">
+        <f>SUM(F4:F243)</f>
+        <v/>
+      </c>
+      <c r="G244" s="32">
+        <f>SUM(G4:G243)</f>
+        <v/>
+      </c>
+      <c r="H244" s="32">
+        <f>SUM(H4:H243)</f>
+        <v/>
+      </c>
+      <c r="I244" s="32">
+        <f>SUM(I4:I243)</f>
+        <v/>
+      </c>
+      <c r="J244" s="32">
+        <f>SUM(J4:J243)</f>
+        <v/>
+      </c>
+      <c r="K244" s="32">
+        <f>SUM(K4:K243)</f>
+        <v/>
+      </c>
+      <c r="L244" s="32">
+        <f>SUM(L4:L243)</f>
+        <v/>
+      </c>
+      <c r="M244" s="32">
+        <f>SUM(M4:M243)</f>
+        <v/>
+      </c>
+      <c r="N244" s="32">
+        <f>SUM(N4:N243)</f>
         <v/>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A3:N239"/>
+  <autoFilter ref="A3:N243"/>
   <mergeCells count="2">
     <mergeCell ref="A2:N2"/>
     <mergeCell ref="A1:N1"/>
@@ -53280,7 +53737,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K17"/>
+  <dimension ref="A1:K18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -53842,40 +54299,85 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="3" t="inlineStr">
+      <c r="A17" s="28" t="n">
+        <v>46293</v>
+      </c>
+      <c r="B17" s="20">
+        <f>COUNTIFS('Trade Log'!$G$4:$G$503,"&gt;="&amp;DATE(2026,9,28),'Trade Log'!$G$4:$G$503,"&lt;"&amp;DATE(2026,10,5))</f>
+        <v/>
+      </c>
+      <c r="C17" s="20">
+        <f>COUNTIFS('Trade Log'!$G$4:$G$503,"&gt;="&amp;DATE(2026,9,28),'Trade Log'!$G$4:$G$503,"&lt;"&amp;DATE(2026,10,5),'Trade Log'!$L$4:$L$503,"&gt;0")</f>
+        <v/>
+      </c>
+      <c r="D17" s="20">
+        <f>COUNTIFS('Trade Log'!$G$4:$G$503,"&gt;="&amp;DATE(2026,9,28),'Trade Log'!$G$4:$G$503,"&lt;"&amp;DATE(2026,10,5),'Trade Log'!$L$4:$L$503,"&lt;0")</f>
+        <v/>
+      </c>
+      <c r="E17" s="22">
+        <f>IFERROR($C17/$B17,"")</f>
+        <v/>
+      </c>
+      <c r="F17" s="21">
+        <f>SUMIFS('Trade Log'!$I$4:$I$503,'Trade Log'!$G$4:$G$503,"&gt;="&amp;DATE(2026,9,28),'Trade Log'!$G$4:$G$503,"&lt;"&amp;DATE(2026,10,5))</f>
+        <v/>
+      </c>
+      <c r="G17" s="21">
+        <f>SUMIFS('Trade Log'!$L$4:$L$503,'Trade Log'!$G$4:$G$503,"&gt;="&amp;DATE(2026,9,28),'Trade Log'!$G$4:$G$503,"&lt;"&amp;DATE(2026,10,5))</f>
+        <v/>
+      </c>
+      <c r="H17" s="21">
+        <f>IFERROR($G17/$B17,"")</f>
+        <v/>
+      </c>
+      <c r="I17" s="21">
+        <f>IFERROR(_xlfn.MAXIFS('Trade Log'!$L$4:$L$503,'Trade Log'!$G$4:$G$503,"&gt;="&amp;DATE(2026,9,28),'Trade Log'!$G$4:$G$503,"&lt;"&amp;DATE(2026,10,5)),"")</f>
+        <v/>
+      </c>
+      <c r="J17" s="21">
+        <f>IFERROR(_xlfn.MINIFS('Trade Log'!$L$4:$L$503,'Trade Log'!$G$4:$G$503,"&gt;="&amp;DATE(2026,9,28),'Trade Log'!$G$4:$G$503,"&lt;"&amp;DATE(2026,10,5)),"")</f>
+        <v/>
+      </c>
+      <c r="K17" s="29">
+        <f>IFERROR(SUMIFS('Trade Log'!$L$4:$L$503,'Trade Log'!$G$4:$G$503,"&gt;="&amp;DATE(2026,9,28),'Trade Log'!$G$4:$G$503,"&lt;"&amp;DATE(2026,10,5),'Trade Log'!$L$4:$L$503,"&gt;0")/ABS(SUMIFS('Trade Log'!$L$4:$L$503,'Trade Log'!$G$4:$G$503,"&gt;="&amp;DATE(2026,9,28),'Trade Log'!$G$4:$G$503,"&lt;"&amp;DATE(2026,10,5),'Trade Log'!$L$4:$L$503,"&lt;0")),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="3" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="B17" s="30">
-        <f>SUM(B11:B16)</f>
-        <v/>
-      </c>
-      <c r="C17" s="30">
-        <f>SUM(C11:C16)</f>
-        <v/>
-      </c>
-      <c r="D17" s="30">
-        <f>SUM(D11:D16)</f>
-        <v/>
-      </c>
-      <c r="E17" s="31">
-        <f>IFERROR(C17/B17,"")</f>
-        <v/>
-      </c>
-      <c r="F17" s="32">
-        <f>SUM(F11:F16)</f>
-        <v/>
-      </c>
-      <c r="G17" s="32">
-        <f>SUM(G11:G16)</f>
-        <v/>
-      </c>
-      <c r="H17" s="32">
-        <f>IFERROR(G17/B17,"")</f>
-        <v/>
-      </c>
-      <c r="K17" s="33">
+      <c r="B18" s="30">
+        <f>SUM(B11:B17)</f>
+        <v/>
+      </c>
+      <c r="C18" s="30">
+        <f>SUM(C11:C17)</f>
+        <v/>
+      </c>
+      <c r="D18" s="30">
+        <f>SUM(D11:D17)</f>
+        <v/>
+      </c>
+      <c r="E18" s="31">
+        <f>IFERROR(C18/B18,"")</f>
+        <v/>
+      </c>
+      <c r="F18" s="32">
+        <f>SUM(F11:F17)</f>
+        <v/>
+      </c>
+      <c r="G18" s="32">
+        <f>SUM(G11:G17)</f>
+        <v/>
+      </c>
+      <c r="H18" s="32">
+        <f>IFERROR(G18/B18,"")</f>
+        <v/>
+      </c>
+      <c r="K18" s="33">
         <f>IFERROR(SUMIF('Trade Log'!$L$4:$L$503,"&gt;0")/ABS(SUMIF('Trade Log'!$L$4:$L$503,"&lt;0")),"")</f>
         <v/>
       </c>

</xml_diff>

<commit_message>
Data update — 2026-09-29 candle + results refresh
</commit_message>
<xml_diff>
--- a/results/strategy_pnl_simple.xlsx
+++ b/results/strategy_pnl_simple.xlsx
@@ -18,7 +18,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Trade Log'!$A$3:$O$503</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Charges'!$A$3:$N$244</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Charges'!$A$3:$N$251</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -1214,7 +1214,7 @@
         <v/>
       </c>
       <c r="K6" s="4" t="n">
-        <v>688.97</v>
+        <v>688.95</v>
       </c>
       <c r="L6" s="21">
         <f>IF(OR($B6="",$I6=""),"",$I6-IF($K6="",0,$K6))</f>
@@ -1454,7 +1454,7 @@
         <v/>
       </c>
       <c r="K10" s="4" t="n">
-        <v>662.86</v>
+        <v>662.85</v>
       </c>
       <c r="L10" s="21">
         <f>IF(OR($B10="",$I10=""),"",$I10-IF($K10="",0,$K10))</f>
@@ -1574,7 +1574,7 @@
         <v/>
       </c>
       <c r="K12" s="4" t="n">
-        <v>591.59</v>
+        <v>591.6900000000001</v>
       </c>
       <c r="L12" s="21">
         <f>IF(OR($B12="",$I12=""),"",$I12-IF($K12="",0,$K12))</f>
@@ -1814,7 +1814,7 @@
         <v/>
       </c>
       <c r="K16" s="4" t="n">
-        <v>414.06</v>
+        <v>414.05</v>
       </c>
       <c r="L16" s="21">
         <f>IF(OR($B16="",$I16=""),"",$I16-IF($K16="",0,$K16))</f>
@@ -2174,7 +2174,7 @@
         <v/>
       </c>
       <c r="K22" s="4" t="n">
-        <v>380.54</v>
+        <v>380.53</v>
       </c>
       <c r="L22" s="21">
         <f>IF(OR($B22="",$I22=""),"",$I22-IF($K22="",0,$K22))</f>
@@ -2414,7 +2414,7 @@
         <v/>
       </c>
       <c r="K26" s="4" t="n">
-        <v>406.37</v>
+        <v>406.36</v>
       </c>
       <c r="L26" s="21">
         <f>IF(OR($B26="",$I26=""),"",$I26-IF($K26="",0,$K26))</f>
@@ -2654,7 +2654,7 @@
         <v/>
       </c>
       <c r="K30" s="4" t="n">
-        <v>870.55</v>
+        <v>870.76</v>
       </c>
       <c r="L30" s="21">
         <f>IF(OR($B30="",$I30=""),"",$I30-IF($K30="",0,$K30))</f>
@@ -2894,7 +2894,7 @@
         <v/>
       </c>
       <c r="K34" s="4" t="n">
-        <v>390.57</v>
+        <v>390.59</v>
       </c>
       <c r="L34" s="21">
         <f>IF(OR($B34="",$I34=""),"",$I34-IF($K34="",0,$K34))</f>
@@ -3014,7 +3014,7 @@
         <v/>
       </c>
       <c r="K36" s="4" t="n">
-        <v>349.19</v>
+        <v>349.21</v>
       </c>
       <c r="L36" s="21">
         <f>IF(OR($B36="",$I36=""),"",$I36-IF($K36="",0,$K36))</f>
@@ -3134,7 +3134,7 @@
         <v/>
       </c>
       <c r="K38" s="4" t="n">
-        <v>329.26</v>
+        <v>329.27</v>
       </c>
       <c r="L38" s="21">
         <f>IF(OR($B38="",$I38=""),"",$I38-IF($K38="",0,$K38))</f>
@@ -3254,7 +3254,7 @@
         <v/>
       </c>
       <c r="K40" s="4" t="n">
-        <v>385.4</v>
+        <v>385.43</v>
       </c>
       <c r="L40" s="21">
         <f>IF(OR($B40="",$I40=""),"",$I40-IF($K40="",0,$K40))</f>
@@ -3374,7 +3374,7 @@
         <v/>
       </c>
       <c r="K42" s="4" t="n">
-        <v>977.05</v>
+        <v>977.08</v>
       </c>
       <c r="L42" s="21">
         <f>IF(OR($B42="",$I42=""),"",$I42-IF($K42="",0,$K42))</f>
@@ -3434,7 +3434,7 @@
         <v/>
       </c>
       <c r="K43" s="4" t="n">
-        <v>956.65</v>
+        <v>956.6799999999999</v>
       </c>
       <c r="L43" s="21">
         <f>IF(OR($B43="",$I43=""),"",$I43-IF($K43="",0,$K43))</f>
@@ -3494,7 +3494,7 @@
         <v/>
       </c>
       <c r="K44" s="4" t="n">
-        <v>991.03</v>
+        <v>991.0700000000001</v>
       </c>
       <c r="L44" s="21">
         <f>IF(OR($B44="",$I44=""),"",$I44-IF($K44="",0,$K44))</f>
@@ -3554,7 +3554,7 @@
         <v/>
       </c>
       <c r="K45" s="4" t="n">
-        <v>597.72</v>
+        <v>597.78</v>
       </c>
       <c r="L45" s="21">
         <f>IF(OR($B45="",$I45=""),"",$I45-IF($K45="",0,$K45))</f>
@@ -3674,7 +3674,7 @@
         <v/>
       </c>
       <c r="K47" s="4" t="n">
-        <v>598.83</v>
+        <v>598.88</v>
       </c>
       <c r="L47" s="21">
         <f>IF(OR($B47="",$I47=""),"",$I47-IF($K47="",0,$K47))</f>
@@ -3794,7 +3794,7 @@
         <v/>
       </c>
       <c r="K49" s="4" t="n">
-        <v>677.24</v>
+        <v>677.36</v>
       </c>
       <c r="L49" s="21">
         <f>IF(OR($B49="",$I49=""),"",$I49-IF($K49="",0,$K49))</f>
@@ -3914,7 +3914,7 @@
         <v/>
       </c>
       <c r="K51" s="4" t="n">
-        <v>670.4299999999999</v>
+        <v>669.9299999999999</v>
       </c>
       <c r="L51" s="21">
         <f>IF(OR($B51="",$I51=""),"",$I51-IF($K51="",0,$K51))</f>
@@ -4034,7 +4034,7 @@
         <v/>
       </c>
       <c r="K53" s="4" t="n">
-        <v>574.4299999999999</v>
+        <v>574.48</v>
       </c>
       <c r="L53" s="21">
         <f>IF(OR($B53="",$I53=""),"",$I53-IF($K53="",0,$K53))</f>
@@ -4274,7 +4274,7 @@
         <v/>
       </c>
       <c r="K57" s="4" t="n">
-        <v>619.39</v>
+        <v>619.35</v>
       </c>
       <c r="L57" s="21">
         <f>IF(OR($B57="",$I57=""),"",$I57-IF($K57="",0,$K57))</f>
@@ -4394,7 +4394,7 @@
         <v/>
       </c>
       <c r="K59" s="4" t="n">
-        <v>612.4299999999999</v>
+        <v>612.45</v>
       </c>
       <c r="L59" s="21">
         <f>IF(OR($B59="",$I59=""),"",$I59-IF($K59="",0,$K59))</f>
@@ -4874,7 +4874,7 @@
         <v/>
       </c>
       <c r="K67" s="4" t="n">
-        <v>441.48</v>
+        <v>441.5</v>
       </c>
       <c r="L67" s="21">
         <f>IF(OR($B67="",$I67=""),"",$I67-IF($K67="",0,$K67))</f>
@@ -5954,7 +5954,7 @@
         <v/>
       </c>
       <c r="K85" s="4" t="n">
-        <v>412.31</v>
+        <v>412.36</v>
       </c>
       <c r="L85" s="21">
         <f>IF(OR($B85="",$I85=""),"",$I85-IF($K85="",0,$K85))</f>
@@ -6434,7 +6434,7 @@
         <v/>
       </c>
       <c r="K93" s="4" t="n">
-        <v>799.53</v>
+        <v>799.52</v>
       </c>
       <c r="L93" s="21">
         <f>IF(OR($B93="",$I93=""),"",$I93-IF($K93="",0,$K93))</f>
@@ -6554,7 +6554,7 @@
         <v/>
       </c>
       <c r="K95" s="4" t="n">
-        <v>826.87</v>
+        <v>826.86</v>
       </c>
       <c r="L95" s="21">
         <f>IF(OR($B95="",$I95=""),"",$I95-IF($K95="",0,$K95))</f>
@@ -6674,7 +6674,7 @@
         <v/>
       </c>
       <c r="K97" s="4" t="n">
-        <v>479.58</v>
+        <v>479.66</v>
       </c>
       <c r="L97" s="21">
         <f>IF(OR($B97="",$I97=""),"",$I97-IF($K97="",0,$K97))</f>
@@ -7694,7 +7694,7 @@
         <v/>
       </c>
       <c r="K114" s="4" t="n">
-        <v>480.9</v>
+        <v>480.95</v>
       </c>
       <c r="L114" s="21">
         <f>IF(OR($B114="",$I114=""),"",$I114-IF($K114="",0,$K114))</f>
@@ -8414,7 +8414,7 @@
         <v/>
       </c>
       <c r="K126" s="4" t="n">
-        <v>425.04</v>
+        <v>425.11</v>
       </c>
       <c r="L126" s="21">
         <f>IF(OR($B126="",$I126=""),"",$I126-IF($K126="",0,$K126))</f>
@@ -8894,7 +8894,7 @@
         <v/>
       </c>
       <c r="K134" s="4" t="n">
-        <v>654.42</v>
+        <v>654.01</v>
       </c>
       <c r="L134" s="21">
         <f>IF(OR($B134="",$I134=""),"",$I134-IF($K134="",0,$K134))</f>
@@ -9614,7 +9614,7 @@
         <v/>
       </c>
       <c r="K146" s="4" t="n">
-        <v>504.47</v>
+        <v>504.61</v>
       </c>
       <c r="L146" s="21">
         <f>IF(OR($B146="",$I146=""),"",$I146-IF($K146="",0,$K146))</f>
@@ -9734,7 +9734,7 @@
         <v/>
       </c>
       <c r="K148" s="4" t="n">
-        <v>490.94</v>
+        <v>490.99</v>
       </c>
       <c r="L148" s="21">
         <f>IF(OR($B148="",$I148=""),"",$I148-IF($K148="",0,$K148))</f>
@@ -9854,7 +9854,7 @@
         <v/>
       </c>
       <c r="K150" s="4" t="n">
-        <v>467.31</v>
+        <v>467.3</v>
       </c>
       <c r="L150" s="21">
         <f>IF(OR($B150="",$I150=""),"",$I150-IF($K150="",0,$K150))</f>
@@ -10094,7 +10094,7 @@
         <v/>
       </c>
       <c r="K154" s="4" t="n">
-        <v>542.35</v>
+        <v>542.37</v>
       </c>
       <c r="L154" s="21">
         <f>IF(OR($B154="",$I154=""),"",$I154-IF($K154="",0,$K154))</f>
@@ -10214,7 +10214,7 @@
         <v/>
       </c>
       <c r="K156" s="4" t="n">
-        <v>461.25</v>
+        <v>461.59</v>
       </c>
       <c r="L156" s="21">
         <f>IF(OR($B156="",$I156=""),"",$I156-IF($K156="",0,$K156))</f>
@@ -10334,7 +10334,7 @@
         <v/>
       </c>
       <c r="K158" s="4" t="n">
-        <v>526.11</v>
+        <v>526.41</v>
       </c>
       <c r="L158" s="21">
         <f>IF(OR($B158="",$I158=""),"",$I158-IF($K158="",0,$K158))</f>
@@ -10454,7 +10454,7 @@
         <v/>
       </c>
       <c r="K160" s="4" t="n">
-        <v>520.35</v>
+        <v>520.62</v>
       </c>
       <c r="L160" s="21">
         <f>IF(OR($B160="",$I160=""),"",$I160-IF($K160="",0,$K160))</f>
@@ -10574,7 +10574,7 @@
         <v/>
       </c>
       <c r="K162" s="4" t="n">
-        <v>518.72</v>
+        <v>518.99</v>
       </c>
       <c r="L162" s="21">
         <f>IF(OR($B162="",$I162=""),"",$I162-IF($K162="",0,$K162))</f>
@@ -10694,7 +10694,7 @@
         <v/>
       </c>
       <c r="K164" s="4" t="n">
-        <v>446.71</v>
+        <v>446.93</v>
       </c>
       <c r="L164" s="21">
         <f>IF(OR($B164="",$I164=""),"",$I164-IF($K164="",0,$K164))</f>
@@ -10814,7 +10814,7 @@
         <v/>
       </c>
       <c r="K166" s="4" t="n">
-        <v>463.14</v>
+        <v>463.48</v>
       </c>
       <c r="L166" s="21">
         <f>IF(OR($B166="",$I166=""),"",$I166-IF($K166="",0,$K166))</f>
@@ -10934,7 +10934,7 @@
         <v/>
       </c>
       <c r="K168" s="4" t="n">
-        <v>628.09</v>
+        <v>628.4299999999999</v>
       </c>
       <c r="L168" s="21">
         <f>IF(OR($B168="",$I168=""),"",$I168-IF($K168="",0,$K168))</f>
@@ -11054,7 +11054,7 @@
         <v/>
       </c>
       <c r="K170" s="4" t="n">
-        <v>636.36</v>
+        <v>636.76</v>
       </c>
       <c r="L170" s="21">
         <f>IF(OR($B170="",$I170=""),"",$I170-IF($K170="",0,$K170))</f>
@@ -11294,7 +11294,7 @@
         <v/>
       </c>
       <c r="K174" s="4" t="n">
-        <v>599.72</v>
+        <v>600.27</v>
       </c>
       <c r="L174" s="21">
         <f>IF(OR($B174="",$I174=""),"",$I174-IF($K174="",0,$K174))</f>
@@ -11414,7 +11414,7 @@
         <v/>
       </c>
       <c r="K176" s="4" t="n">
-        <v>589.05</v>
+        <v>589.6900000000001</v>
       </c>
       <c r="L176" s="21">
         <f>IF(OR($B176="",$I176=""),"",$I176-IF($K176="",0,$K176))</f>
@@ -11534,7 +11534,7 @@
         <v/>
       </c>
       <c r="K178" s="4" t="n">
-        <v>601.72</v>
+        <v>602.4299999999999</v>
       </c>
       <c r="L178" s="21">
         <f>IF(OR($B178="",$I178=""),"",$I178-IF($K178="",0,$K178))</f>
@@ -11654,7 +11654,7 @@
         <v/>
       </c>
       <c r="K180" s="4" t="n">
-        <v>591.03</v>
+        <v>591.6799999999999</v>
       </c>
       <c r="L180" s="21">
         <f>IF(OR($B180="",$I180=""),"",$I180-IF($K180="",0,$K180))</f>
@@ -11774,7 +11774,7 @@
         <v/>
       </c>
       <c r="K182" s="4" t="n">
-        <v>295.56</v>
+        <v>295.71</v>
       </c>
       <c r="L182" s="21">
         <f>IF(OR($B182="",$I182=""),"",$I182-IF($K182="",0,$K182))</f>
@@ -12014,7 +12014,7 @@
         <v/>
       </c>
       <c r="K186" s="4" t="n">
-        <v>337.38</v>
+        <v>337.53</v>
       </c>
       <c r="L186" s="21">
         <f>IF(OR($B186="",$I186=""),"",$I186-IF($K186="",0,$K186))</f>
@@ -12134,7 +12134,7 @@
         <v/>
       </c>
       <c r="K188" s="4" t="n">
-        <v>288.82</v>
+        <v>288.92</v>
       </c>
       <c r="L188" s="21">
         <f>IF(OR($B188="",$I188=""),"",$I188-IF($K188="",0,$K188))</f>
@@ -12254,7 +12254,7 @@
         <v/>
       </c>
       <c r="K190" s="4" t="n">
-        <v>191.91</v>
+        <v>191.96</v>
       </c>
       <c r="L190" s="21">
         <f>IF(OR($B190="",$I190=""),"",$I190-IF($K190="",0,$K190))</f>
@@ -12374,7 +12374,7 @@
         <v/>
       </c>
       <c r="K192" s="4" t="n">
-        <v>296.03</v>
+        <v>296.17</v>
       </c>
       <c r="L192" s="21">
         <f>IF(OR($B192="",$I192=""),"",$I192-IF($K192="",0,$K192))</f>
@@ -12494,7 +12494,7 @@
         <v/>
       </c>
       <c r="K194" s="4" t="n">
-        <v>500.23</v>
+        <v>500.39</v>
       </c>
       <c r="L194" s="21">
         <f>IF(OR($B194="",$I194=""),"",$I194-IF($K194="",0,$K194))</f>
@@ -12614,7 +12614,7 @@
         <v/>
       </c>
       <c r="K196" s="4" t="n">
-        <v>461.09</v>
+        <v>461.42</v>
       </c>
       <c r="L196" s="21">
         <f>IF(OR($B196="",$I196=""),"",$I196-IF($K196="",0,$K196))</f>
@@ -12734,7 +12734,7 @@
         <v/>
       </c>
       <c r="K198" s="4" t="n">
-        <v>464.04</v>
+        <v>464.33</v>
       </c>
       <c r="L198" s="21">
         <f>IF(OR($B198="",$I198=""),"",$I198-IF($K198="",0,$K198))</f>
@@ -12854,7 +12854,7 @@
         <v/>
       </c>
       <c r="K200" s="4" t="n">
-        <v>497.33</v>
+        <v>497.5</v>
       </c>
       <c r="L200" s="21">
         <f>IF(OR($B200="",$I200=""),"",$I200-IF($K200="",0,$K200))</f>
@@ -12974,7 +12974,7 @@
         <v/>
       </c>
       <c r="K202" s="4" t="n">
-        <v>520.4400000000001</v>
+        <v>520.71</v>
       </c>
       <c r="L202" s="21">
         <f>IF(OR($B202="",$I202=""),"",$I202-IF($K202="",0,$K202))</f>
@@ -13094,7 +13094,7 @@
         <v/>
       </c>
       <c r="K204" s="4" t="n">
-        <v>457.98</v>
+        <v>458.31</v>
       </c>
       <c r="L204" s="21">
         <f>IF(OR($B204="",$I204=""),"",$I204-IF($K204="",0,$K204))</f>
@@ -13214,7 +13214,7 @@
         <v/>
       </c>
       <c r="K206" s="4" t="n">
-        <v>395.2</v>
+        <v>395.29</v>
       </c>
       <c r="L206" s="21">
         <f>IF(OR($B206="",$I206=""),"",$I206-IF($K206="",0,$K206))</f>
@@ -13334,7 +13334,7 @@
         <v/>
       </c>
       <c r="K208" s="4" t="n">
-        <v>355.55</v>
+        <v>347.81</v>
       </c>
       <c r="L208" s="21">
         <f>IF(OR($B208="",$I208=""),"",$I208-IF($K208="",0,$K208))</f>
@@ -13574,7 +13574,7 @@
         <v/>
       </c>
       <c r="K212" s="4" t="n">
-        <v>385.64</v>
+        <v>385.69</v>
       </c>
       <c r="L212" s="21">
         <f>IF(OR($B212="",$I212=""),"",$I212-IF($K212="",0,$K212))</f>
@@ -13694,7 +13694,7 @@
         <v/>
       </c>
       <c r="K214" s="4" t="n">
-        <v>315.52</v>
+        <v>315.59</v>
       </c>
       <c r="L214" s="21">
         <f>IF(OR($B214="",$I214=""),"",$I214-IF($K214="",0,$K214))</f>
@@ -13814,7 +13814,7 @@
         <v/>
       </c>
       <c r="K216" s="4" t="n">
-        <v>318.22</v>
+        <v>318.31</v>
       </c>
       <c r="L216" s="21">
         <f>IF(OR($B216="",$I216=""),"",$I216-IF($K216="",0,$K216))</f>
@@ -13934,7 +13934,7 @@
         <v/>
       </c>
       <c r="K218" s="4" t="n">
-        <v>359.56</v>
+        <v>359.64</v>
       </c>
       <c r="L218" s="21">
         <f>IF(OR($B218="",$I218=""),"",$I218-IF($K218="",0,$K218))</f>
@@ -14054,7 +14054,7 @@
         <v/>
       </c>
       <c r="K220" s="4" t="n">
-        <v>316.61</v>
+        <v>316.7</v>
       </c>
       <c r="L220" s="21">
         <f>IF(OR($B220="",$I220=""),"",$I220-IF($K220="",0,$K220))</f>
@@ -14174,7 +14174,7 @@
         <v/>
       </c>
       <c r="K222" s="4" t="n">
-        <v>360.99</v>
+        <v>361.08</v>
       </c>
       <c r="L222" s="21">
         <f>IF(OR($B222="",$I222=""),"",$I222-IF($K222="",0,$K222))</f>
@@ -14474,7 +14474,7 @@
         <v/>
       </c>
       <c r="K227" s="4" t="n">
-        <v>521.5</v>
+        <v>521.52</v>
       </c>
       <c r="L227" s="21">
         <f>IF(OR($B227="",$I227=""),"",$I227-IF($K227="",0,$K227))</f>
@@ -14714,7 +14714,7 @@
         <v/>
       </c>
       <c r="K231" s="4" t="n">
-        <v>461.32</v>
+        <v>461.23</v>
       </c>
       <c r="L231" s="21">
         <f>IF(OR($B231="",$I231=""),"",$I231-IF($K231="",0,$K231))</f>
@@ -14894,7 +14894,7 @@
         <v/>
       </c>
       <c r="K234" s="4" t="n">
-        <v>162.78</v>
+        <v>288.97</v>
       </c>
       <c r="L234" s="21">
         <f>IF(OR($B234="",$I234=""),"",$I234-IF($K234="",0,$K234))</f>
@@ -14954,7 +14954,7 @@
         <v/>
       </c>
       <c r="K235" s="4" t="n">
-        <v>531.9400000000001</v>
+        <v>753.75</v>
       </c>
       <c r="L235" s="21">
         <f>IF(OR($B235="",$I235=""),"",$I235-IF($K235="",0,$K235))</f>
@@ -15014,7 +15014,7 @@
         <v/>
       </c>
       <c r="K236" s="4" t="n">
-        <v>562.72</v>
+        <v>844.87</v>
       </c>
       <c r="L236" s="21">
         <f>IF(OR($B236="",$I236=""),"",$I236-IF($K236="",0,$K236))</f>
@@ -15074,7 +15074,7 @@
         <v/>
       </c>
       <c r="K237" s="4" t="n">
-        <v>526.92</v>
+        <v>798.96</v>
       </c>
       <c r="L237" s="21">
         <f>IF(OR($B237="",$I237=""),"",$I237-IF($K237="",0,$K237))</f>
@@ -15134,7 +15134,7 @@
         <v/>
       </c>
       <c r="K238" s="4" t="n">
-        <v>589.12</v>
+        <v>871.05</v>
       </c>
       <c r="L238" s="21">
         <f>IF(OR($B238="",$I238=""),"",$I238-IF($K238="",0,$K238))</f>
@@ -15194,7 +15194,7 @@
         <v/>
       </c>
       <c r="K239" s="4" t="n">
-        <v>524.41</v>
+        <v>807.85</v>
       </c>
       <c r="L239" s="21">
         <f>IF(OR($B239="",$I239=""),"",$I239-IF($K239="",0,$K239))</f>
@@ -15239,8 +15239,12 @@
       <c r="F240" s="26" t="n">
         <v>479</v>
       </c>
-      <c r="G240" s="24" t="inlineStr"/>
-      <c r="H240" s="25" t="inlineStr"/>
+      <c r="G240" s="24" t="n">
+        <v>46294</v>
+      </c>
+      <c r="H240" s="25" t="n">
+        <v>602.61</v>
+      </c>
       <c r="I240" s="21">
         <f>IF(OR($B240="",$H240=""),"",IF($C240="LONG",($H240-$E240)*$F240,($E240-$H240)*$F240))</f>
         <v/>
@@ -15250,7 +15254,7 @@
         <v/>
       </c>
       <c r="K240" s="4" t="n">
-        <v>50.15</v>
+        <v>492.69</v>
       </c>
       <c r="L240" s="21">
         <f>IF(OR($B240="",$I240=""),"",$I240-IF($K240="",0,$K240))</f>
@@ -15295,8 +15299,12 @@
       <c r="F241" s="26" t="n">
         <v>1061</v>
       </c>
-      <c r="G241" s="24" t="inlineStr"/>
-      <c r="H241" s="25" t="inlineStr"/>
+      <c r="G241" s="24" t="n">
+        <v>46294</v>
+      </c>
+      <c r="H241" s="25" t="n">
+        <v>297</v>
+      </c>
       <c r="I241" s="21">
         <f>IF(OR($B241="",$H241=""),"",IF($C241="LONG",($H241-$E241)*$F241,($E241-$H241)*$F241))</f>
         <v/>
@@ -15306,7 +15314,7 @@
         <v/>
       </c>
       <c r="K241" s="4" t="n">
-        <v>50.15</v>
+        <v>115.49</v>
       </c>
       <c r="L241" s="21">
         <f>IF(OR($B241="",$I241=""),"",$I241-IF($K241="",0,$K241))</f>
@@ -15329,30 +15337,34 @@
     <row r="242">
       <c r="A242" s="23" t="inlineStr">
         <is>
-          <t>DHAN-341260928158709+341260928158609+221260928823209+341260928158409+341260928158209+341260928158009+341260928157909+221260928821609+341260928157709+221260928820609+341260928157509</t>
+          <t>DHAN-23126092924109</t>
         </is>
       </c>
       <c r="B242" s="23" t="inlineStr">
         <is>
-          <t>SDBL</t>
+          <t>RSYSTEMS</t>
         </is>
       </c>
       <c r="C242" s="23" t="inlineStr">
         <is>
-          <t>LONG</t>
+          <t>SHORT</t>
         </is>
       </c>
       <c r="D242" s="24" t="n">
-        <v>46293</v>
+        <v>46294</v>
       </c>
       <c r="E242" s="25" t="n">
-        <v>80.2633</v>
+        <v>297.01</v>
       </c>
       <c r="F242" s="26" t="n">
-        <v>3732</v>
-      </c>
-      <c r="G242" s="24" t="inlineStr"/>
-      <c r="H242" s="25" t="inlineStr"/>
+        <v>1061</v>
+      </c>
+      <c r="G242" s="24" t="n">
+        <v>46294</v>
+      </c>
+      <c r="H242" s="25" t="n">
+        <v>298.99</v>
+      </c>
       <c r="I242" s="21">
         <f>IF(OR($B242="",$H242=""),"",IF($C242="LONG",($H242-$E242)*$F242,($E242-$H242)*$F242))</f>
         <v/>
@@ -15362,7 +15374,7 @@
         <v/>
       </c>
       <c r="K242" s="4" t="n">
-        <v>50.15</v>
+        <v>0</v>
       </c>
       <c r="L242" s="21">
         <f>IF(OR($B242="",$I242=""),"",$I242-IF($K242="",0,$K242))</f>
@@ -15378,19 +15390,19 @@
       </c>
       <c r="O242" s="23" t="inlineStr">
         <is>
-          <t>5-10</t>
+          <t>15-20</t>
         </is>
       </c>
     </row>
     <row r="243">
       <c r="A243" s="23" t="inlineStr">
         <is>
-          <t>DHAN-341260928159209</t>
+          <t>DHAN-341260928158709+341260928158609+221260928823209+341260928158409+341260928158209+341260928158009+341260928157909+221260928821609+341260928157709+221260928820609+341260928157509</t>
         </is>
       </c>
       <c r="B243" s="23" t="inlineStr">
         <is>
-          <t>SMCGLOBAL</t>
+          <t>SDBL</t>
         </is>
       </c>
       <c r="C243" s="23" t="inlineStr">
@@ -15402,13 +15414,17 @@
         <v>46293</v>
       </c>
       <c r="E243" s="25" t="n">
-        <v>97.1964</v>
+        <v>80.2633</v>
       </c>
       <c r="F243" s="26" t="n">
-        <v>3087</v>
-      </c>
-      <c r="G243" s="24" t="inlineStr"/>
-      <c r="H243" s="25" t="inlineStr"/>
+        <v>3732</v>
+      </c>
+      <c r="G243" s="24" t="n">
+        <v>46294</v>
+      </c>
+      <c r="H243" s="25" t="n">
+        <v>78.87</v>
+      </c>
       <c r="I243" s="21">
         <f>IF(OR($B243="",$H243=""),"",IF($C243="LONG",($H243-$E243)*$F243,($E243-$H243)*$F243))</f>
         <v/>
@@ -15418,7 +15434,7 @@
         <v/>
       </c>
       <c r="K243" s="4" t="n">
-        <v>50.15</v>
+        <v>574.33</v>
       </c>
       <c r="L243" s="21">
         <f>IF(OR($B243="",$I243=""),"",$I243-IF($K243="",0,$K243))</f>
@@ -15434,19 +15450,19 @@
       </c>
       <c r="O243" s="23" t="inlineStr">
         <is>
-          <t>15-20</t>
+          <t>5-10</t>
         </is>
       </c>
     </row>
     <row r="244">
       <c r="A244" s="23" t="inlineStr">
         <is>
-          <t>DHAN-341260928159109</t>
+          <t>DHAN-341260928159209</t>
         </is>
       </c>
       <c r="B244" s="23" t="inlineStr">
         <is>
-          <t>SYNCOMF</t>
+          <t>SMCGLOBAL</t>
         </is>
       </c>
       <c r="C244" s="23" t="inlineStr">
@@ -15458,13 +15474,17 @@
         <v>46293</v>
       </c>
       <c r="E244" s="25" t="n">
-        <v>22.1897</v>
+        <v>97.1964</v>
       </c>
       <c r="F244" s="26" t="n">
-        <v>13513</v>
-      </c>
-      <c r="G244" s="24" t="inlineStr"/>
-      <c r="H244" s="25" t="inlineStr"/>
+        <v>3087</v>
+      </c>
+      <c r="G244" s="24" t="n">
+        <v>46294</v>
+      </c>
+      <c r="H244" s="25" t="n">
+        <v>92.37</v>
+      </c>
       <c r="I244" s="21">
         <f>IF(OR($B244="",$H244=""),"",IF($C244="LONG",($H244-$E244)*$F244,($E244-$H244)*$F244))</f>
         <v/>
@@ -15474,7 +15494,7 @@
         <v/>
       </c>
       <c r="K244" s="4" t="n">
-        <v>50.15</v>
+        <v>481.35</v>
       </c>
       <c r="L244" s="21">
         <f>IF(OR($B244="",$I244=""),"",$I244-IF($K244="",0,$K244))</f>
@@ -15490,19 +15510,41 @@
       </c>
       <c r="O244" s="23" t="inlineStr">
         <is>
-          <t>10-15</t>
+          <t>15-20</t>
         </is>
       </c>
     </row>
     <row r="245">
-      <c r="A245" s="23" t="n"/>
-      <c r="B245" s="23" t="n"/>
-      <c r="C245" s="23" t="n"/>
-      <c r="D245" s="24" t="n"/>
-      <c r="E245" s="25" t="n"/>
-      <c r="F245" s="26" t="n"/>
-      <c r="G245" s="24" t="n"/>
-      <c r="H245" s="25" t="n"/>
+      <c r="A245" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-341260928159109</t>
+        </is>
+      </c>
+      <c r="B245" s="23" t="inlineStr">
+        <is>
+          <t>SYNCOMF</t>
+        </is>
+      </c>
+      <c r="C245" s="23" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="D245" s="24" t="n">
+        <v>46293</v>
+      </c>
+      <c r="E245" s="25" t="n">
+        <v>22.1897</v>
+      </c>
+      <c r="F245" s="26" t="n">
+        <v>13513</v>
+      </c>
+      <c r="G245" s="24" t="n">
+        <v>46294</v>
+      </c>
+      <c r="H245" s="25" t="n">
+        <v>22.65</v>
+      </c>
       <c r="I245" s="21">
         <f>IF(OR($B245="",$H245=""),"",IF($C245="LONG",($H245-$E245)*$F245,($E245-$H245)*$F245))</f>
         <v/>
@@ -15511,7 +15553,9 @@
         <f>IF(OR($B245="",$I245="",$E245=0,$F245=0),"",$I245/($E245*$F245))</f>
         <v/>
       </c>
-      <c r="K245" s="4" t="n"/>
+      <c r="K245" s="4" t="n">
+        <v>481.07</v>
+      </c>
       <c r="L245" s="21">
         <f>IF(OR($B245="",$I245=""),"",$I245-IF($K245="",0,$K245))</f>
         <v/>
@@ -15524,17 +15568,39 @@
         <f>IF($B245="","",IF($H245="","Open","Closed"))</f>
         <v/>
       </c>
-      <c r="O245" s="23" t="n"/>
+      <c r="O245" s="23" t="inlineStr">
+        <is>
+          <t>10-15</t>
+        </is>
+      </c>
     </row>
     <row r="246">
-      <c r="A246" s="23" t="n"/>
-      <c r="B246" s="23" t="n"/>
-      <c r="C246" s="23" t="n"/>
-      <c r="D246" s="24" t="n"/>
-      <c r="E246" s="25" t="n"/>
-      <c r="F246" s="26" t="n"/>
-      <c r="G246" s="24" t="n"/>
-      <c r="H246" s="25" t="n"/>
+      <c r="A246" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-221260929652409</t>
+        </is>
+      </c>
+      <c r="B246" s="23" t="inlineStr">
+        <is>
+          <t>ELECTCAST</t>
+        </is>
+      </c>
+      <c r="C246" s="23" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="D246" s="24" t="n">
+        <v>46294</v>
+      </c>
+      <c r="E246" s="25" t="n">
+        <v>76.3257</v>
+      </c>
+      <c r="F246" s="26" t="n">
+        <v>2805</v>
+      </c>
+      <c r="G246" s="24" t="inlineStr"/>
+      <c r="H246" s="25" t="inlineStr"/>
       <c r="I246" s="21">
         <f>IF(OR($B246="",$H246=""),"",IF($C246="LONG",($H246-$E246)*$F246,($E246-$H246)*$F246))</f>
         <v/>
@@ -15543,7 +15609,9 @@
         <f>IF(OR($B246="",$I246="",$E246=0,$F246=0),"",$I246/($E246*$F246))</f>
         <v/>
       </c>
-      <c r="K246" s="4" t="n"/>
+      <c r="K246" s="4" t="n">
+        <v>50.15</v>
+      </c>
       <c r="L246" s="21">
         <f>IF(OR($B246="",$I246=""),"",$I246-IF($K246="",0,$K246))</f>
         <v/>
@@ -15556,17 +15624,39 @@
         <f>IF($B246="","",IF($H246="","Open","Closed"))</f>
         <v/>
       </c>
-      <c r="O246" s="23" t="n"/>
+      <c r="O246" s="23" t="inlineStr">
+        <is>
+          <t>5-10</t>
+        </is>
+      </c>
     </row>
     <row r="247">
-      <c r="A247" s="23" t="n"/>
-      <c r="B247" s="23" t="n"/>
-      <c r="C247" s="23" t="n"/>
-      <c r="D247" s="24" t="n"/>
-      <c r="E247" s="25" t="n"/>
-      <c r="F247" s="26" t="n"/>
-      <c r="G247" s="24" t="n"/>
-      <c r="H247" s="25" t="n"/>
+      <c r="A247" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-221260929652309</t>
+        </is>
+      </c>
+      <c r="B247" s="23" t="inlineStr">
+        <is>
+          <t>INDOCO</t>
+        </is>
+      </c>
+      <c r="C247" s="23" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="D247" s="24" t="n">
+        <v>46294</v>
+      </c>
+      <c r="E247" s="25" t="n">
+        <v>272.5066</v>
+      </c>
+      <c r="F247" s="26" t="n">
+        <v>788</v>
+      </c>
+      <c r="G247" s="24" t="inlineStr"/>
+      <c r="H247" s="25" t="inlineStr"/>
       <c r="I247" s="21">
         <f>IF(OR($B247="",$H247=""),"",IF($C247="LONG",($H247-$E247)*$F247,($E247-$H247)*$F247))</f>
         <v/>
@@ -15575,7 +15665,9 @@
         <f>IF(OR($B247="",$I247="",$E247=0,$F247=0),"",$I247/($E247*$F247))</f>
         <v/>
       </c>
-      <c r="K247" s="4" t="n"/>
+      <c r="K247" s="4" t="n">
+        <v>50.15</v>
+      </c>
       <c r="L247" s="21">
         <f>IF(OR($B247="",$I247=""),"",$I247-IF($K247="",0,$K247))</f>
         <v/>
@@ -15588,17 +15680,39 @@
         <f>IF($B247="","",IF($H247="","Open","Closed"))</f>
         <v/>
       </c>
-      <c r="O247" s="23" t="n"/>
+      <c r="O247" s="23" t="inlineStr">
+        <is>
+          <t>5-10</t>
+        </is>
+      </c>
     </row>
     <row r="248">
-      <c r="A248" s="23" t="n"/>
-      <c r="B248" s="23" t="n"/>
-      <c r="C248" s="23" t="n"/>
-      <c r="D248" s="24" t="n"/>
-      <c r="E248" s="25" t="n"/>
-      <c r="F248" s="26" t="n"/>
-      <c r="G248" s="24" t="n"/>
-      <c r="H248" s="25" t="n"/>
+      <c r="A248" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-221260929652509</t>
+        </is>
+      </c>
+      <c r="B248" s="23" t="inlineStr">
+        <is>
+          <t>RSYSTEMS</t>
+        </is>
+      </c>
+      <c r="C248" s="23" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="D248" s="24" t="n">
+        <v>46294</v>
+      </c>
+      <c r="E248" s="25" t="n">
+        <v>298.4</v>
+      </c>
+      <c r="F248" s="26" t="n">
+        <v>359</v>
+      </c>
+      <c r="G248" s="24" t="inlineStr"/>
+      <c r="H248" s="25" t="inlineStr"/>
       <c r="I248" s="21">
         <f>IF(OR($B248="",$H248=""),"",IF($C248="LONG",($H248-$E248)*$F248,($E248-$H248)*$F248))</f>
         <v/>
@@ -15607,7 +15721,9 @@
         <f>IF(OR($B248="",$I248="",$E248=0,$F248=0),"",$I248/($E248*$F248))</f>
         <v/>
       </c>
-      <c r="K248" s="4" t="n"/>
+      <c r="K248" s="4" t="n">
+        <v>14.75</v>
+      </c>
       <c r="L248" s="21">
         <f>IF(OR($B248="",$I248=""),"",$I248-IF($K248="",0,$K248))</f>
         <v/>
@@ -15620,17 +15736,39 @@
         <f>IF($B248="","",IF($H248="","Open","Closed"))</f>
         <v/>
       </c>
-      <c r="O248" s="23" t="n"/>
+      <c r="O248" s="23" t="inlineStr">
+        <is>
+          <t>5-10</t>
+        </is>
+      </c>
     </row>
     <row r="249">
-      <c r="A249" s="23" t="n"/>
-      <c r="B249" s="23" t="n"/>
-      <c r="C249" s="23" t="n"/>
-      <c r="D249" s="24" t="n"/>
-      <c r="E249" s="25" t="n"/>
-      <c r="F249" s="26" t="n"/>
-      <c r="G249" s="24" t="n"/>
-      <c r="H249" s="25" t="n"/>
+      <c r="A249" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-321260929420709</t>
+        </is>
+      </c>
+      <c r="B249" s="23" t="inlineStr">
+        <is>
+          <t>SYNCOMF</t>
+        </is>
+      </c>
+      <c r="C249" s="23" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="D249" s="24" t="n">
+        <v>46294</v>
+      </c>
+      <c r="E249" s="25" t="n">
+        <v>26.45</v>
+      </c>
+      <c r="F249" s="26" t="n">
+        <v>4058</v>
+      </c>
+      <c r="G249" s="24" t="inlineStr"/>
+      <c r="H249" s="25" t="inlineStr"/>
       <c r="I249" s="21">
         <f>IF(OR($B249="",$H249=""),"",IF($C249="LONG",($H249-$E249)*$F249,($E249-$H249)*$F249))</f>
         <v/>
@@ -15639,7 +15777,9 @@
         <f>IF(OR($B249="",$I249="",$E249=0,$F249=0),"",$I249/($E249*$F249))</f>
         <v/>
       </c>
-      <c r="K249" s="4" t="n"/>
+      <c r="K249" s="4" t="n">
+        <v>14.75</v>
+      </c>
       <c r="L249" s="21">
         <f>IF(OR($B249="",$I249=""),"",$I249-IF($K249="",0,$K249))</f>
         <v/>
@@ -15652,17 +15792,39 @@
         <f>IF($B249="","",IF($H249="","Open","Closed"))</f>
         <v/>
       </c>
-      <c r="O249" s="23" t="n"/>
+      <c r="O249" s="23" t="inlineStr">
+        <is>
+          <t>15-20</t>
+        </is>
+      </c>
     </row>
     <row r="250">
-      <c r="A250" s="23" t="n"/>
-      <c r="B250" s="23" t="n"/>
-      <c r="C250" s="23" t="n"/>
-      <c r="D250" s="24" t="n"/>
-      <c r="E250" s="25" t="n"/>
-      <c r="F250" s="26" t="n"/>
-      <c r="G250" s="24" t="n"/>
-      <c r="H250" s="25" t="n"/>
+      <c r="A250" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-34126092973909+321260929416609+34126092974209+34126092974309+221260929647009+221260929647509+23126092975109+34126092974609+23126092975209+221260929648209+221260929648709+23126092975409+23126092975509+34126092974709</t>
+        </is>
+      </c>
+      <c r="B250" s="23" t="inlineStr">
+        <is>
+          <t>TCIEXP</t>
+        </is>
+      </c>
+      <c r="C250" s="23" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="D250" s="24" t="n">
+        <v>46294</v>
+      </c>
+      <c r="E250" s="25" t="n">
+        <v>526.5716</v>
+      </c>
+      <c r="F250" s="26" t="n">
+        <v>407</v>
+      </c>
+      <c r="G250" s="24" t="inlineStr"/>
+      <c r="H250" s="25" t="inlineStr"/>
       <c r="I250" s="21">
         <f>IF(OR($B250="",$H250=""),"",IF($C250="LONG",($H250-$E250)*$F250,($E250-$H250)*$F250))</f>
         <v/>
@@ -15671,7 +15833,9 @@
         <f>IF(OR($B250="",$I250="",$E250=0,$F250=0),"",$I250/($E250*$F250))</f>
         <v/>
       </c>
-      <c r="K250" s="4" t="n"/>
+      <c r="K250" s="4" t="n">
+        <v>50.15</v>
+      </c>
       <c r="L250" s="21">
         <f>IF(OR($B250="",$I250=""),"",$I250-IF($K250="",0,$K250))</f>
         <v/>
@@ -15684,17 +15848,39 @@
         <f>IF($B250="","",IF($H250="","Open","Closed"))</f>
         <v/>
       </c>
-      <c r="O250" s="23" t="n"/>
+      <c r="O250" s="23" t="inlineStr">
+        <is>
+          <t>5-10</t>
+        </is>
+      </c>
     </row>
     <row r="251">
-      <c r="A251" s="23" t="n"/>
-      <c r="B251" s="23" t="n"/>
-      <c r="C251" s="23" t="n"/>
-      <c r="D251" s="24" t="n"/>
-      <c r="E251" s="25" t="n"/>
-      <c r="F251" s="26" t="n"/>
-      <c r="G251" s="24" t="n"/>
-      <c r="H251" s="25" t="n"/>
+      <c r="A251" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-321260929416409+34126092974109+23126092974809+34126092974409+321260929417209+221260929647409+321260929417509+321260929417709+23126092975309+321260929418309+221260929648809+321260929418709+34126092974809</t>
+        </is>
+      </c>
+      <c r="B251" s="23" t="inlineStr">
+        <is>
+          <t>UNICHEMLAB</t>
+        </is>
+      </c>
+      <c r="C251" s="23" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="D251" s="24" t="n">
+        <v>46294</v>
+      </c>
+      <c r="E251" s="25" t="n">
+        <v>571.4527</v>
+      </c>
+      <c r="F251" s="26" t="n">
+        <v>375</v>
+      </c>
+      <c r="G251" s="24" t="inlineStr"/>
+      <c r="H251" s="25" t="inlineStr"/>
       <c r="I251" s="21">
         <f>IF(OR($B251="",$H251=""),"",IF($C251="LONG",($H251-$E251)*$F251,($E251-$H251)*$F251))</f>
         <v/>
@@ -15703,7 +15889,9 @@
         <f>IF(OR($B251="",$I251="",$E251=0,$F251=0),"",$I251/($E251*$F251))</f>
         <v/>
       </c>
-      <c r="K251" s="4" t="n"/>
+      <c r="K251" s="4" t="n">
+        <v>50.15</v>
+      </c>
       <c r="L251" s="21">
         <f>IF(OR($B251="",$I251=""),"",$I251-IF($K251="",0,$K251))</f>
         <v/>
@@ -15716,7 +15904,11 @@
         <f>IF($B251="","",IF($H251="","Open","Closed"))</f>
         <v/>
       </c>
-      <c r="O251" s="23" t="n"/>
+      <c r="O251" s="23" t="inlineStr">
+        <is>
+          <t>5-10</t>
+        </is>
+      </c>
     </row>
     <row r="252">
       <c r="A252" s="23" t="n"/>
@@ -36457,7 +36649,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J116"/>
+  <dimension ref="A1:J119"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -37272,7 +37464,7 @@
     <row r="21">
       <c r="A21" s="27" t="inlineStr">
         <is>
-          <t>EMUDHRA</t>
+          <t>ELECTCAST</t>
         </is>
       </c>
       <c r="B21" s="20">
@@ -37315,7 +37507,7 @@
     <row r="22">
       <c r="A22" s="27" t="inlineStr">
         <is>
-          <t>FILATEX</t>
+          <t>EMUDHRA</t>
         </is>
       </c>
       <c r="B22" s="20">
@@ -37358,7 +37550,7 @@
     <row r="23">
       <c r="A23" s="27" t="inlineStr">
         <is>
-          <t>FMGOETZE</t>
+          <t>FILATEX</t>
         </is>
       </c>
       <c r="B23" s="20">
@@ -37401,7 +37593,7 @@
     <row r="24">
       <c r="A24" s="27" t="inlineStr">
         <is>
-          <t>FOSECOIND</t>
+          <t>FMGOETZE</t>
         </is>
       </c>
       <c r="B24" s="20">
@@ -37444,7 +37636,7 @@
     <row r="25">
       <c r="A25" s="27" t="inlineStr">
         <is>
-          <t>FRONTSP</t>
+          <t>FOSECOIND</t>
         </is>
       </c>
       <c r="B25" s="20">
@@ -37487,7 +37679,7 @@
     <row r="26">
       <c r="A26" s="27" t="inlineStr">
         <is>
-          <t>GKENERGY</t>
+          <t>FRONTSP</t>
         </is>
       </c>
       <c r="B26" s="20">
@@ -37530,7 +37722,7 @@
     <row r="27">
       <c r="A27" s="27" t="inlineStr">
         <is>
-          <t>GNA</t>
+          <t>GKENERGY</t>
         </is>
       </c>
       <c r="B27" s="20">
@@ -37573,7 +37765,7 @@
     <row r="28">
       <c r="A28" s="27" t="inlineStr">
         <is>
-          <t>GNRL</t>
+          <t>GNA</t>
         </is>
       </c>
       <c r="B28" s="20">
@@ -37616,7 +37808,7 @@
     <row r="29">
       <c r="A29" s="27" t="inlineStr">
         <is>
-          <t>GOCLCORP</t>
+          <t>GNRL</t>
         </is>
       </c>
       <c r="B29" s="20">
@@ -37659,7 +37851,7 @@
     <row r="30">
       <c r="A30" s="27" t="inlineStr">
         <is>
-          <t>GOPAL</t>
+          <t>GOCLCORP</t>
         </is>
       </c>
       <c r="B30" s="20">
@@ -37702,7 +37894,7 @@
     <row r="31">
       <c r="A31" s="27" t="inlineStr">
         <is>
-          <t>GRAUWEIL</t>
+          <t>GOPAL</t>
         </is>
       </c>
       <c r="B31" s="20">
@@ -37745,7 +37937,7 @@
     <row r="32">
       <c r="A32" s="27" t="inlineStr">
         <is>
-          <t>GREAVESCOT</t>
+          <t>GRAUWEIL</t>
         </is>
       </c>
       <c r="B32" s="20">
@@ -37788,7 +37980,7 @@
     <row r="33">
       <c r="A33" s="27" t="inlineStr">
         <is>
-          <t>GUJTHEM</t>
+          <t>GREAVESCOT</t>
         </is>
       </c>
       <c r="B33" s="20">
@@ -37831,7 +38023,7 @@
     <row r="34">
       <c r="A34" s="27" t="inlineStr">
         <is>
-          <t>HERITGFOOD</t>
+          <t>GUJTHEM</t>
         </is>
       </c>
       <c r="B34" s="20">
@@ -37874,7 +38066,7 @@
     <row r="35">
       <c r="A35" s="27" t="inlineStr">
         <is>
-          <t>HIKAL</t>
+          <t>HERITGFOOD</t>
         </is>
       </c>
       <c r="B35" s="20">
@@ -37917,7 +38109,7 @@
     <row r="36">
       <c r="A36" s="27" t="inlineStr">
         <is>
-          <t>HINDOILEXP</t>
+          <t>HIKAL</t>
         </is>
       </c>
       <c r="B36" s="20">
@@ -37960,7 +38152,7 @@
     <row r="37">
       <c r="A37" s="27" t="inlineStr">
         <is>
-          <t>HUBTOWN</t>
+          <t>HINDOILEXP</t>
         </is>
       </c>
       <c r="B37" s="20">
@@ -38003,7 +38195,7 @@
     <row r="38">
       <c r="A38" s="27" t="inlineStr">
         <is>
-          <t>INDIAGLYCO</t>
+          <t>HUBTOWN</t>
         </is>
       </c>
       <c r="B38" s="20">
@@ -38046,7 +38238,7 @@
     <row r="39">
       <c r="A39" s="27" t="inlineStr">
         <is>
-          <t>INDNIPPON</t>
+          <t>INDIAGLYCO</t>
         </is>
       </c>
       <c r="B39" s="20">
@@ -38089,7 +38281,7 @@
     <row r="40">
       <c r="A40" s="27" t="inlineStr">
         <is>
-          <t>INDOCO</t>
+          <t>INDNIPPON</t>
         </is>
       </c>
       <c r="B40" s="20">
@@ -38132,7 +38324,7 @@
     <row r="41">
       <c r="A41" s="27" t="inlineStr">
         <is>
-          <t>INDORAMA</t>
+          <t>INDOCO</t>
         </is>
       </c>
       <c r="B41" s="20">
@@ -38175,7 +38367,7 @@
     <row r="42">
       <c r="A42" s="27" t="inlineStr">
         <is>
-          <t>IPL</t>
+          <t>INDORAMA</t>
         </is>
       </c>
       <c r="B42" s="20">
@@ -38218,7 +38410,7 @@
     <row r="43">
       <c r="A43" s="27" t="inlineStr">
         <is>
-          <t>JASH</t>
+          <t>IPL</t>
         </is>
       </c>
       <c r="B43" s="20">
@@ -38261,7 +38453,7 @@
     <row r="44">
       <c r="A44" s="27" t="inlineStr">
         <is>
-          <t>JAYKAY</t>
+          <t>JASH</t>
         </is>
       </c>
       <c r="B44" s="20">
@@ -38304,7 +38496,7 @@
     <row r="45">
       <c r="A45" s="27" t="inlineStr">
         <is>
-          <t>JGCHEM</t>
+          <t>JAYKAY</t>
         </is>
       </c>
       <c r="B45" s="20">
@@ -38347,7 +38539,7 @@
     <row r="46">
       <c r="A46" s="27" t="inlineStr">
         <is>
-          <t>JINDRILL</t>
+          <t>JGCHEM</t>
         </is>
       </c>
       <c r="B46" s="20">
@@ -38390,7 +38582,7 @@
     <row r="47">
       <c r="A47" s="27" t="inlineStr">
         <is>
-          <t>KCP</t>
+          <t>JINDRILL</t>
         </is>
       </c>
       <c r="B47" s="20">
@@ -38433,7 +38625,7 @@
     <row r="48">
       <c r="A48" s="27" t="inlineStr">
         <is>
-          <t>KIRIINDUS</t>
+          <t>KCP</t>
         </is>
       </c>
       <c r="B48" s="20">
@@ -38476,7 +38668,7 @@
     <row r="49">
       <c r="A49" s="27" t="inlineStr">
         <is>
-          <t>KIRLOSIND</t>
+          <t>KIRIINDUS</t>
         </is>
       </c>
       <c r="B49" s="20">
@@ -38519,7 +38711,7 @@
     <row r="50">
       <c r="A50" s="27" t="inlineStr">
         <is>
-          <t>KLBRENG-B</t>
+          <t>KIRLOSIND</t>
         </is>
       </c>
       <c r="B50" s="20">
@@ -38562,7 +38754,7 @@
     <row r="51">
       <c r="A51" s="27" t="inlineStr">
         <is>
-          <t>KROSS</t>
+          <t>KLBRENG-B</t>
         </is>
       </c>
       <c r="B51" s="20">
@@ -38605,7 +38797,7 @@
     <row r="52">
       <c r="A52" s="27" t="inlineStr">
         <is>
-          <t>KSCL</t>
+          <t>KROSS</t>
         </is>
       </c>
       <c r="B52" s="20">
@@ -38648,7 +38840,7 @@
     <row r="53">
       <c r="A53" s="27" t="inlineStr">
         <is>
-          <t>KSL</t>
+          <t>KSCL</t>
         </is>
       </c>
       <c r="B53" s="20">
@@ -38691,7 +38883,7 @@
     <row r="54">
       <c r="A54" s="27" t="inlineStr">
         <is>
-          <t>LUXIND</t>
+          <t>KSL</t>
         </is>
       </c>
       <c r="B54" s="20">
@@ -38734,7 +38926,7 @@
     <row r="55">
       <c r="A55" s="27" t="inlineStr">
         <is>
-          <t>MAITHANALL</t>
+          <t>LUXIND</t>
         </is>
       </c>
       <c r="B55" s="20">
@@ -38777,7 +38969,7 @@
     <row r="56">
       <c r="A56" s="27" t="inlineStr">
         <is>
-          <t>MANGLMCEM</t>
+          <t>MAITHANALL</t>
         </is>
       </c>
       <c r="B56" s="20">
@@ -38820,7 +39012,7 @@
     <row r="57">
       <c r="A57" s="27" t="inlineStr">
         <is>
-          <t>MASTEK</t>
+          <t>MANGLMCEM</t>
         </is>
       </c>
       <c r="B57" s="20">
@@ -38863,7 +39055,7 @@
     <row r="58">
       <c r="A58" s="27" t="inlineStr">
         <is>
-          <t>MOBIKWIK</t>
+          <t>MASTEK</t>
         </is>
       </c>
       <c r="B58" s="20">
@@ -38906,7 +39098,7 @@
     <row r="59">
       <c r="A59" s="27" t="inlineStr">
         <is>
-          <t>MUKANDLTD</t>
+          <t>MOBIKWIK</t>
         </is>
       </c>
       <c r="B59" s="20">
@@ -38949,7 +39141,7 @@
     <row r="60">
       <c r="A60" s="27" t="inlineStr">
         <is>
-          <t>NETWORK18</t>
+          <t>MUKANDLTD</t>
         </is>
       </c>
       <c r="B60" s="20">
@@ -38992,7 +39184,7 @@
     <row r="61">
       <c r="A61" s="27" t="inlineStr">
         <is>
-          <t>NILKAMAL</t>
+          <t>NETWORK18</t>
         </is>
       </c>
       <c r="B61" s="20">
@@ -39035,7 +39227,7 @@
     <row r="62">
       <c r="A62" s="27" t="inlineStr">
         <is>
-          <t>NORTHARC</t>
+          <t>NILKAMAL</t>
         </is>
       </c>
       <c r="B62" s="20">
@@ -39078,7 +39270,7 @@
     <row r="63">
       <c r="A63" s="27" t="inlineStr">
         <is>
-          <t>NOVARTIND</t>
+          <t>NORTHARC</t>
         </is>
       </c>
       <c r="B63" s="20">
@@ -39121,7 +39313,7 @@
     <row r="64">
       <c r="A64" s="27" t="inlineStr">
         <is>
-          <t>NPST</t>
+          <t>NOVARTIND</t>
         </is>
       </c>
       <c r="B64" s="20">
@@ -39164,7 +39356,7 @@
     <row r="65">
       <c r="A65" s="27" t="inlineStr">
         <is>
-          <t>NRBBEARING</t>
+          <t>NPST</t>
         </is>
       </c>
       <c r="B65" s="20">
@@ -39207,7 +39399,7 @@
     <row r="66">
       <c r="A66" s="27" t="inlineStr">
         <is>
-          <t>OMAXE</t>
+          <t>NRBBEARING</t>
         </is>
       </c>
       <c r="B66" s="20">
@@ -39250,7 +39442,7 @@
     <row r="67">
       <c r="A67" s="27" t="inlineStr">
         <is>
-          <t>ONEPOINT</t>
+          <t>OMAXE</t>
         </is>
       </c>
       <c r="B67" s="20">
@@ -39293,7 +39485,7 @@
     <row r="68">
       <c r="A68" s="27" t="inlineStr">
         <is>
-          <t>OPTIEMUS</t>
+          <t>ONEPOINT</t>
         </is>
       </c>
       <c r="B68" s="20">
@@ -39336,7 +39528,7 @@
     <row r="69">
       <c r="A69" s="27" t="inlineStr">
         <is>
-          <t>ORIENTHOT</t>
+          <t>OPTIEMUS</t>
         </is>
       </c>
       <c r="B69" s="20">
@@ -39379,7 +39571,7 @@
     <row r="70">
       <c r="A70" s="27" t="inlineStr">
         <is>
-          <t>PACEDIGITK</t>
+          <t>ORIENTHOT</t>
         </is>
       </c>
       <c r="B70" s="20">
@@ -39422,7 +39614,7 @@
     <row r="71">
       <c r="A71" s="27" t="inlineStr">
         <is>
-          <t>PITTIENG</t>
+          <t>PACEDIGITK</t>
         </is>
       </c>
       <c r="B71" s="20">
@@ -39465,7 +39657,7 @@
     <row r="72">
       <c r="A72" s="27" t="inlineStr">
         <is>
-          <t>PROTEAN</t>
+          <t>PITTIENG</t>
         </is>
       </c>
       <c r="B72" s="20">
@@ -39508,7 +39700,7 @@
     <row r="73">
       <c r="A73" s="27" t="inlineStr">
         <is>
-          <t>QUADFUTURE</t>
+          <t>PROTEAN</t>
         </is>
       </c>
       <c r="B73" s="20">
@@ -39551,7 +39743,7 @@
     <row r="74">
       <c r="A74" s="27" t="inlineStr">
         <is>
-          <t>RACLGEAR</t>
+          <t>QUADFUTURE</t>
         </is>
       </c>
       <c r="B74" s="20">
@@ -39594,7 +39786,7 @@
     <row r="75">
       <c r="A75" s="27" t="inlineStr">
         <is>
-          <t>RAMRAT</t>
+          <t>RACLGEAR</t>
         </is>
       </c>
       <c r="B75" s="20">
@@ -39637,7 +39829,7 @@
     <row r="76">
       <c r="A76" s="27" t="inlineStr">
         <is>
-          <t>RAYMOND</t>
+          <t>RAMRAT</t>
         </is>
       </c>
       <c r="B76" s="20">
@@ -39680,7 +39872,7 @@
     <row r="77">
       <c r="A77" s="27" t="inlineStr">
         <is>
-          <t>RAYMONDREL</t>
+          <t>RAYMOND</t>
         </is>
       </c>
       <c r="B77" s="20">
@@ -39723,7 +39915,7 @@
     <row r="78">
       <c r="A78" s="27" t="inlineStr">
         <is>
-          <t>REFEX</t>
+          <t>RAYMONDREL</t>
         </is>
       </c>
       <c r="B78" s="20">
@@ -39766,7 +39958,7 @@
     <row r="79">
       <c r="A79" s="27" t="inlineStr">
         <is>
-          <t>RESPONIND</t>
+          <t>REFEX</t>
         </is>
       </c>
       <c r="B79" s="20">
@@ -39809,7 +40001,7 @@
     <row r="80">
       <c r="A80" s="27" t="inlineStr">
         <is>
-          <t>RML</t>
+          <t>RESPONIND</t>
         </is>
       </c>
       <c r="B80" s="20">
@@ -39852,7 +40044,7 @@
     <row r="81">
       <c r="A81" s="27" t="inlineStr">
         <is>
-          <t>ROSSTECH</t>
+          <t>RML</t>
         </is>
       </c>
       <c r="B81" s="20">
@@ -39895,7 +40087,7 @@
     <row r="82">
       <c r="A82" s="27" t="inlineStr">
         <is>
-          <t>RPGLIFE</t>
+          <t>ROSSTECH</t>
         </is>
       </c>
       <c r="B82" s="20">
@@ -39938,7 +40130,7 @@
     <row r="83">
       <c r="A83" s="27" t="inlineStr">
         <is>
-          <t>RSYSTEMS</t>
+          <t>RPGLIFE</t>
         </is>
       </c>
       <c r="B83" s="20">
@@ -39981,7 +40173,7 @@
     <row r="84">
       <c r="A84" s="27" t="inlineStr">
         <is>
-          <t>SAATVIKGL</t>
+          <t>RSYSTEMS</t>
         </is>
       </c>
       <c r="B84" s="20">
@@ -40024,7 +40216,7 @@
     <row r="85">
       <c r="A85" s="27" t="inlineStr">
         <is>
-          <t>SAKAR</t>
+          <t>SAATVIKGL</t>
         </is>
       </c>
       <c r="B85" s="20">
@@ -40067,7 +40259,7 @@
     <row r="86">
       <c r="A86" s="27" t="inlineStr">
         <is>
-          <t>SAMBHV</t>
+          <t>SAKAR</t>
         </is>
       </c>
       <c r="B86" s="20">
@@ -40110,7 +40302,7 @@
     <row r="87">
       <c r="A87" s="27" t="inlineStr">
         <is>
-          <t>SAMHI</t>
+          <t>SAMBHV</t>
         </is>
       </c>
       <c r="B87" s="20">
@@ -40153,7 +40345,7 @@
     <row r="88">
       <c r="A88" s="27" t="inlineStr">
         <is>
-          <t>SANGAMIND</t>
+          <t>SAMHI</t>
         </is>
       </c>
       <c r="B88" s="20">
@@ -40196,7 +40388,7 @@
     <row r="89">
       <c r="A89" s="27" t="inlineStr">
         <is>
-          <t>SDBL</t>
+          <t>SANGAMIND</t>
         </is>
       </c>
       <c r="B89" s="20">
@@ -40239,7 +40431,7 @@
     <row r="90">
       <c r="A90" s="27" t="inlineStr">
         <is>
-          <t>SHANTIGOLD</t>
+          <t>SDBL</t>
         </is>
       </c>
       <c r="B90" s="20">
@@ -40282,7 +40474,7 @@
     <row r="91">
       <c r="A91" s="27" t="inlineStr">
         <is>
-          <t>SHAREINDIA</t>
+          <t>SHANTIGOLD</t>
         </is>
       </c>
       <c r="B91" s="20">
@@ -40325,7 +40517,7 @@
     <row r="92">
       <c r="A92" s="27" t="inlineStr">
         <is>
-          <t>SHOPERSTOP</t>
+          <t>SHAREINDIA</t>
         </is>
       </c>
       <c r="B92" s="20">
@@ -40368,7 +40560,7 @@
     <row r="93">
       <c r="A93" s="27" t="inlineStr">
         <is>
-          <t>SIKA</t>
+          <t>SHOPERSTOP</t>
         </is>
       </c>
       <c r="B93" s="20">
@@ -40411,7 +40603,7 @@
     <row r="94">
       <c r="A94" s="27" t="inlineStr">
         <is>
-          <t>SINDHUTRAD</t>
+          <t>SIKA</t>
         </is>
       </c>
       <c r="B94" s="20">
@@ -40454,7 +40646,7 @@
     <row r="95">
       <c r="A95" s="27" t="inlineStr">
         <is>
-          <t>SMCGLOBAL</t>
+          <t>SINDHUTRAD</t>
         </is>
       </c>
       <c r="B95" s="20">
@@ -40497,7 +40689,7 @@
     <row r="96">
       <c r="A96" s="27" t="inlineStr">
         <is>
-          <t>SMSPHARMA</t>
+          <t>SMCGLOBAL</t>
         </is>
       </c>
       <c r="B96" s="20">
@@ -40540,7 +40732,7 @@
     <row r="97">
       <c r="A97" s="27" t="inlineStr">
         <is>
-          <t>SOLARA</t>
+          <t>SMSPHARMA</t>
         </is>
       </c>
       <c r="B97" s="20">
@@ -40583,7 +40775,7 @@
     <row r="98">
       <c r="A98" s="27" t="inlineStr">
         <is>
-          <t>SOTL</t>
+          <t>SOLARA</t>
         </is>
       </c>
       <c r="B98" s="20">
@@ -40626,7 +40818,7 @@
     <row r="99">
       <c r="A99" s="27" t="inlineStr">
         <is>
-          <t>SSWL</t>
+          <t>SOTL</t>
         </is>
       </c>
       <c r="B99" s="20">
@@ -40669,7 +40861,7 @@
     <row r="100">
       <c r="A100" s="27" t="inlineStr">
         <is>
-          <t>STEELCAS</t>
+          <t>SSWL</t>
         </is>
       </c>
       <c r="B100" s="20">
@@ -40712,7 +40904,7 @@
     <row r="101">
       <c r="A101" s="27" t="inlineStr">
         <is>
-          <t>SYMPHONY</t>
+          <t>STEELCAS</t>
         </is>
       </c>
       <c r="B101" s="20">
@@ -40755,7 +40947,7 @@
     <row r="102">
       <c r="A102" s="27" t="inlineStr">
         <is>
-          <t>SYNCOMF</t>
+          <t>SYMPHONY</t>
         </is>
       </c>
       <c r="B102" s="20">
@@ -40798,7 +40990,7 @@
     <row r="103">
       <c r="A103" s="27" t="inlineStr">
         <is>
-          <t>TALBROAUTO</t>
+          <t>SYNCOMF</t>
         </is>
       </c>
       <c r="B103" s="20">
@@ -40841,7 +41033,7 @@
     <row r="104">
       <c r="A104" s="27" t="inlineStr">
         <is>
-          <t>TBZ</t>
+          <t>TALBROAUTO</t>
         </is>
       </c>
       <c r="B104" s="20">
@@ -40884,7 +41076,7 @@
     <row r="105">
       <c r="A105" s="27" t="inlineStr">
         <is>
-          <t>THOMASCOOK</t>
+          <t>TBZ</t>
         </is>
       </c>
       <c r="B105" s="20">
@@ -40927,7 +41119,7 @@
     <row r="106">
       <c r="A106" s="27" t="inlineStr">
         <is>
-          <t>VENKEYS</t>
+          <t>TCIEXP</t>
         </is>
       </c>
       <c r="B106" s="20">
@@ -40970,7 +41162,7 @@
     <row r="107">
       <c r="A107" s="27" t="inlineStr">
         <is>
-          <t>VENUSPIPES</t>
+          <t>THOMASCOOK</t>
         </is>
       </c>
       <c r="B107" s="20">
@@ -41013,7 +41205,7 @@
     <row r="108">
       <c r="A108" s="27" t="inlineStr">
         <is>
-          <t>VERANDA</t>
+          <t>UNICHEMLAB</t>
         </is>
       </c>
       <c r="B108" s="20">
@@ -41056,7 +41248,7 @@
     <row r="109">
       <c r="A109" s="27" t="inlineStr">
         <is>
-          <t>VSSL</t>
+          <t>VENKEYS</t>
         </is>
       </c>
       <c r="B109" s="20">
@@ -41099,7 +41291,7 @@
     <row r="110">
       <c r="A110" s="27" t="inlineStr">
         <is>
-          <t>WELSPLSOL</t>
+          <t>VENUSPIPES</t>
         </is>
       </c>
       <c r="B110" s="20">
@@ -41142,7 +41334,7 @@
     <row r="111">
       <c r="A111" s="27" t="inlineStr">
         <is>
-          <t>WENDT</t>
+          <t>VERANDA</t>
         </is>
       </c>
       <c r="B111" s="20">
@@ -41185,7 +41377,7 @@
     <row r="112">
       <c r="A112" s="27" t="inlineStr">
         <is>
-          <t>WINDLAS</t>
+          <t>VSSL</t>
         </is>
       </c>
       <c r="B112" s="20">
@@ -41228,7 +41420,7 @@
     <row r="113">
       <c r="A113" s="27" t="inlineStr">
         <is>
-          <t>XPROINDIA</t>
+          <t>WELSPLSOL</t>
         </is>
       </c>
       <c r="B113" s="20">
@@ -41271,7 +41463,7 @@
     <row r="114">
       <c r="A114" s="27" t="inlineStr">
         <is>
-          <t>ZAGGLE</t>
+          <t>WENDT</t>
         </is>
       </c>
       <c r="B114" s="20">
@@ -41314,7 +41506,7 @@
     <row r="115">
       <c r="A115" s="27" t="inlineStr">
         <is>
-          <t>ZOTA</t>
+          <t>WINDLAS</t>
         </is>
       </c>
       <c r="B115" s="20">
@@ -41355,37 +41547,166 @@
       </c>
     </row>
     <row r="116">
-      <c r="A116" s="3" t="inlineStr">
+      <c r="A116" s="27" t="inlineStr">
+        <is>
+          <t>XPROINDIA</t>
+        </is>
+      </c>
+      <c r="B116" s="20">
+        <f>COUNTIF('Trade Log'!$B$4:$B$503,$A116)</f>
+        <v/>
+      </c>
+      <c r="C116" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A116,'Trade Log'!$L$4:$L$503,"&gt;0")</f>
+        <v/>
+      </c>
+      <c r="D116" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A116,'Trade Log'!$L$4:$L$503,"&lt;0")</f>
+        <v/>
+      </c>
+      <c r="E116" s="22">
+        <f>IFERROR($C116/$B116,"")</f>
+        <v/>
+      </c>
+      <c r="F116" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A116,'Trade Log'!$I$4:$I$503)</f>
+        <v/>
+      </c>
+      <c r="G116" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A116,'Trade Log'!$L$4:$L$503)</f>
+        <v/>
+      </c>
+      <c r="H116" s="21">
+        <f>IFERROR($G116/$B116,"")</f>
+        <v/>
+      </c>
+      <c r="I116" s="21">
+        <f>IFERROR(_xlfn.MAXIFS('Trade Log'!$L$4:$L$503,'Trade Log'!$B$4:$B$503,$A116),"")</f>
+        <v/>
+      </c>
+      <c r="J116" s="21">
+        <f>IFERROR(_xlfn.MINIFS('Trade Log'!$L$4:$L$503,'Trade Log'!$B$4:$B$503,$A116),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" s="27" t="inlineStr">
+        <is>
+          <t>ZAGGLE</t>
+        </is>
+      </c>
+      <c r="B117" s="20">
+        <f>COUNTIF('Trade Log'!$B$4:$B$503,$A117)</f>
+        <v/>
+      </c>
+      <c r="C117" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A117,'Trade Log'!$L$4:$L$503,"&gt;0")</f>
+        <v/>
+      </c>
+      <c r="D117" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A117,'Trade Log'!$L$4:$L$503,"&lt;0")</f>
+        <v/>
+      </c>
+      <c r="E117" s="22">
+        <f>IFERROR($C117/$B117,"")</f>
+        <v/>
+      </c>
+      <c r="F117" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A117,'Trade Log'!$I$4:$I$503)</f>
+        <v/>
+      </c>
+      <c r="G117" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A117,'Trade Log'!$L$4:$L$503)</f>
+        <v/>
+      </c>
+      <c r="H117" s="21">
+        <f>IFERROR($G117/$B117,"")</f>
+        <v/>
+      </c>
+      <c r="I117" s="21">
+        <f>IFERROR(_xlfn.MAXIFS('Trade Log'!$L$4:$L$503,'Trade Log'!$B$4:$B$503,$A117),"")</f>
+        <v/>
+      </c>
+      <c r="J117" s="21">
+        <f>IFERROR(_xlfn.MINIFS('Trade Log'!$L$4:$L$503,'Trade Log'!$B$4:$B$503,$A117),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" s="27" t="inlineStr">
+        <is>
+          <t>ZOTA</t>
+        </is>
+      </c>
+      <c r="B118" s="20">
+        <f>COUNTIF('Trade Log'!$B$4:$B$503,$A118)</f>
+        <v/>
+      </c>
+      <c r="C118" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A118,'Trade Log'!$L$4:$L$503,"&gt;0")</f>
+        <v/>
+      </c>
+      <c r="D118" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A118,'Trade Log'!$L$4:$L$503,"&lt;0")</f>
+        <v/>
+      </c>
+      <c r="E118" s="22">
+        <f>IFERROR($C118/$B118,"")</f>
+        <v/>
+      </c>
+      <c r="F118" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A118,'Trade Log'!$I$4:$I$503)</f>
+        <v/>
+      </c>
+      <c r="G118" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A118,'Trade Log'!$L$4:$L$503)</f>
+        <v/>
+      </c>
+      <c r="H118" s="21">
+        <f>IFERROR($G118/$B118,"")</f>
+        <v/>
+      </c>
+      <c r="I118" s="21">
+        <f>IFERROR(_xlfn.MAXIFS('Trade Log'!$L$4:$L$503,'Trade Log'!$B$4:$B$503,$A118),"")</f>
+        <v/>
+      </c>
+      <c r="J118" s="21">
+        <f>IFERROR(_xlfn.MINIFS('Trade Log'!$L$4:$L$503,'Trade Log'!$B$4:$B$503,$A118),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" s="3" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="B116" s="30">
-        <f>SUM(B4:B115)</f>
-        <v/>
-      </c>
-      <c r="C116" s="30">
-        <f>SUM(C4:C115)</f>
-        <v/>
-      </c>
-      <c r="D116" s="30">
-        <f>SUM(D4:D115)</f>
-        <v/>
-      </c>
-      <c r="E116" s="31">
-        <f>IFERROR(C116/B116,"")</f>
-        <v/>
-      </c>
-      <c r="F116" s="32">
-        <f>SUM(F4:F115)</f>
-        <v/>
-      </c>
-      <c r="G116" s="32">
-        <f>SUM(G4:G115)</f>
-        <v/>
-      </c>
-      <c r="H116" s="32">
-        <f>IFERROR(G116/B116,"")</f>
+      <c r="B119" s="30">
+        <f>SUM(B4:B118)</f>
+        <v/>
+      </c>
+      <c r="C119" s="30">
+        <f>SUM(C4:C118)</f>
+        <v/>
+      </c>
+      <c r="D119" s="30">
+        <f>SUM(D4:D118)</f>
+        <v/>
+      </c>
+      <c r="E119" s="31">
+        <f>IFERROR(C119/B119,"")</f>
+        <v/>
+      </c>
+      <c r="F119" s="32">
+        <f>SUM(F4:F118)</f>
+        <v/>
+      </c>
+      <c r="G119" s="32">
+        <f>SUM(G4:G118)</f>
+        <v/>
+      </c>
+      <c r="H119" s="32">
+        <f>IFERROR(G119/B119,"")</f>
         <v/>
       </c>
     </row>
@@ -41404,7 +41725,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N245"/>
+  <dimension ref="A1:N252"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -41655,7 +41976,7 @@
         <v>35.4</v>
       </c>
       <c r="M6" s="4" t="n">
-        <v>150.57</v>
+        <v>150.55</v>
       </c>
       <c r="N6" s="21">
         <f>SUM(E6:M6)</f>
@@ -41859,7 +42180,7 @@
         <v>35.4</v>
       </c>
       <c r="M10" s="4" t="n">
-        <v>128.7</v>
+        <v>128.69</v>
       </c>
       <c r="N10" s="21">
         <f>SUM(E10:M10)</f>
@@ -41961,7 +42282,7 @@
         <v>35.4</v>
       </c>
       <c r="M12" s="4" t="n">
-        <v>126.13</v>
+        <v>126.23</v>
       </c>
       <c r="N12" s="21">
         <f>SUM(E12:M12)</f>
@@ -42471,7 +42792,7 @@
         <v>35.4</v>
       </c>
       <c r="M22" s="4" t="n">
-        <v>78.93000000000001</v>
+        <v>78.91</v>
       </c>
       <c r="N22" s="21">
         <f>SUM(E22:M22)</f>
@@ -42879,7 +43200,7 @@
         <v>35.4</v>
       </c>
       <c r="M30" s="4" t="n">
-        <v>314.23</v>
+        <v>314.43</v>
       </c>
       <c r="N30" s="21">
         <f>SUM(E30:M30)</f>
@@ -43083,7 +43404,7 @@
         <v>35.4</v>
       </c>
       <c r="M34" s="4" t="n">
-        <v>46.98</v>
+        <v>46.99</v>
       </c>
       <c r="N34" s="21">
         <f>SUM(E34:M34)</f>
@@ -43185,7 +43506,7 @@
         <v>35.4</v>
       </c>
       <c r="M36" s="4" t="n">
-        <v>46.96</v>
+        <v>46.98</v>
       </c>
       <c r="N36" s="21">
         <f>SUM(E36:M36)</f>
@@ -43287,7 +43608,7 @@
         <v>35.4</v>
       </c>
       <c r="M38" s="4" t="n">
-        <v>28.06</v>
+        <v>28.07</v>
       </c>
       <c r="N38" s="21">
         <f>SUM(E38:M38)</f>
@@ -43389,7 +43710,7 @@
         <v>35.4</v>
       </c>
       <c r="M40" s="4" t="n">
-        <v>44.8</v>
+        <v>44.83</v>
       </c>
       <c r="N40" s="21">
         <f>SUM(E40:M40)</f>
@@ -43491,7 +43812,7 @@
         <v>35.4</v>
       </c>
       <c r="M42" s="4" t="n">
-        <v>98.34</v>
+        <v>98.38</v>
       </c>
       <c r="N42" s="21">
         <f>SUM(E42:M42)</f>
@@ -43542,7 +43863,7 @@
         <v>35.4</v>
       </c>
       <c r="M43" s="4" t="n">
-        <v>82.03</v>
+        <v>82.05</v>
       </c>
       <c r="N43" s="21">
         <f>SUM(E43:M43)</f>
@@ -43593,7 +43914,7 @@
         <v>35.4</v>
       </c>
       <c r="M44" s="4" t="n">
-        <v>98.76000000000001</v>
+        <v>98.79000000000001</v>
       </c>
       <c r="N44" s="21">
         <f>SUM(E44:M44)</f>
@@ -43644,7 +43965,7 @@
         <v>35.4</v>
       </c>
       <c r="M45" s="4" t="n">
-        <v>157.28</v>
+        <v>157.33</v>
       </c>
       <c r="N45" s="21">
         <f>SUM(E45:M45)</f>
@@ -43746,7 +44067,7 @@
         <v>35.4</v>
       </c>
       <c r="M47" s="4" t="n">
-        <v>157.72</v>
+        <v>157.77</v>
       </c>
       <c r="N47" s="21">
         <f>SUM(E47:M47)</f>
@@ -43848,7 +44169,7 @@
         <v>35.4</v>
       </c>
       <c r="M49" s="4" t="n">
-        <v>171.58</v>
+        <v>171.7</v>
       </c>
       <c r="N49" s="21">
         <f>SUM(E49:M49)</f>
@@ -43950,7 +44271,7 @@
         <v>35.4</v>
       </c>
       <c r="M51" s="4" t="n">
-        <v>156.76</v>
+        <v>156.25</v>
       </c>
       <c r="N51" s="21">
         <f>SUM(E51:M51)</f>
@@ -44052,7 +44373,7 @@
         <v>35.4</v>
       </c>
       <c r="M53" s="4" t="n">
-        <v>131.96</v>
+        <v>132</v>
       </c>
       <c r="N53" s="21">
         <f>SUM(E53:M53)</f>
@@ -44154,7 +44475,7 @@
         <v>35.4</v>
       </c>
       <c r="M55" s="4" t="n">
-        <v>98.84999999999999</v>
+        <v>98.86</v>
       </c>
       <c r="N55" s="21">
         <f>SUM(E55:M55)</f>
@@ -44256,7 +44577,7 @@
         <v>35.4</v>
       </c>
       <c r="M57" s="4" t="n">
-        <v>97.06999999999999</v>
+        <v>97.03</v>
       </c>
       <c r="N57" s="21">
         <f>SUM(E57:M57)</f>
@@ -44358,7 +44679,7 @@
         <v>35.4</v>
       </c>
       <c r="M59" s="4" t="n">
-        <v>87.83</v>
+        <v>87.84999999999999</v>
       </c>
       <c r="N59" s="21">
         <f>SUM(E59:M59)</f>
@@ -44766,7 +45087,7 @@
         <v>35.4</v>
       </c>
       <c r="M67" s="4" t="n">
-        <v>50.1</v>
+        <v>50.12</v>
       </c>
       <c r="N67" s="21">
         <f>SUM(E67:M67)</f>
@@ -45684,7 +46005,7 @@
         <v>35.4</v>
       </c>
       <c r="M85" s="4" t="n">
-        <v>57.47</v>
+        <v>57.51</v>
       </c>
       <c r="N85" s="21">
         <f>SUM(E85:M85)</f>
@@ -45990,7 +46311,7 @@
         <v>35.4</v>
       </c>
       <c r="M91" s="4" t="n">
-        <v>274.38</v>
+        <v>274.37</v>
       </c>
       <c r="N91" s="21">
         <f>SUM(E91:M91)</f>
@@ -46296,7 +46617,7 @@
         <v>35.4</v>
       </c>
       <c r="M97" s="4" t="n">
-        <v>96.83</v>
+        <v>96.90000000000001</v>
       </c>
       <c r="N97" s="21">
         <f>SUM(E97:M97)</f>
@@ -46755,7 +47076,7 @@
         <v>35.4</v>
       </c>
       <c r="M106" s="4" t="n">
-        <v>91.76000000000001</v>
+        <v>91.75</v>
       </c>
       <c r="N106" s="21">
         <f>SUM(E106:M106)</f>
@@ -47163,7 +47484,7 @@
         <v>35.4</v>
       </c>
       <c r="M114" s="4" t="n">
-        <v>90.48999999999999</v>
+        <v>90.54000000000001</v>
       </c>
       <c r="N114" s="21">
         <f>SUM(E114:M114)</f>
@@ -47469,7 +47790,7 @@
         <v>35.4</v>
       </c>
       <c r="M120" s="4" t="n">
-        <v>72.28</v>
+        <v>72.27</v>
       </c>
       <c r="N120" s="21">
         <f>SUM(E120:M120)</f>
@@ -47571,7 +47892,7 @@
         <v>35.4</v>
       </c>
       <c r="M122" s="4" t="n">
-        <v>109.12</v>
+        <v>109.11</v>
       </c>
       <c r="N122" s="21">
         <f>SUM(E122:M122)</f>
@@ -47775,7 +48096,7 @@
         <v>35.4</v>
       </c>
       <c r="M126" s="4" t="n">
-        <v>70.40000000000001</v>
+        <v>70.45999999999999</v>
       </c>
       <c r="N126" s="21">
         <f>SUM(E126:M126)</f>
@@ -48183,7 +48504,7 @@
         <v>35.4</v>
       </c>
       <c r="M134" s="4" t="n">
-        <v>128.7</v>
+        <v>128.29</v>
       </c>
       <c r="N134" s="21">
         <f>SUM(E134:M134)</f>
@@ -48285,7 +48606,7 @@
         <v>35.4</v>
       </c>
       <c r="M136" s="4" t="n">
-        <v>113.46</v>
+        <v>113.45</v>
       </c>
       <c r="N136" s="21">
         <f>SUM(E136:M136)</f>
@@ -48795,7 +49116,7 @@
         <v>35.4</v>
       </c>
       <c r="M146" s="4" t="n">
-        <v>186.14</v>
+        <v>186.28</v>
       </c>
       <c r="N146" s="21">
         <f>SUM(E146:M146)</f>
@@ -48897,7 +49218,7 @@
         <v>35.4</v>
       </c>
       <c r="M148" s="4" t="n">
-        <v>170.92</v>
+        <v>170.97</v>
       </c>
       <c r="N148" s="21">
         <f>SUM(E148:M148)</f>
@@ -49203,7 +49524,7 @@
         <v>35.4</v>
       </c>
       <c r="M154" s="4" t="n">
-        <v>184.3</v>
+        <v>184.32</v>
       </c>
       <c r="N154" s="21">
         <f>SUM(E154:M154)</f>
@@ -49305,7 +49626,7 @@
         <v>35.4</v>
       </c>
       <c r="M156" s="4" t="n">
-        <v>56.99</v>
+        <v>57.33</v>
       </c>
       <c r="N156" s="21">
         <f>SUM(E156:M156)</f>
@@ -49407,7 +49728,7 @@
         <v>35.4</v>
       </c>
       <c r="M158" s="4" t="n">
-        <v>57.15</v>
+        <v>57.45</v>
       </c>
       <c r="N158" s="21">
         <f>SUM(E158:M158)</f>
@@ -49509,7 +49830,7 @@
         <v>35.4</v>
       </c>
       <c r="M160" s="4" t="n">
-        <v>52.74</v>
+        <v>53.01</v>
       </c>
       <c r="N160" s="21">
         <f>SUM(E160:M160)</f>
@@ -49611,7 +49932,7 @@
         <v>35.4</v>
       </c>
       <c r="M162" s="4" t="n">
-        <v>52.48</v>
+        <v>52.75</v>
       </c>
       <c r="N162" s="21">
         <f>SUM(E162:M162)</f>
@@ -49713,7 +50034,7 @@
         <v>35.4</v>
       </c>
       <c r="M164" s="4" t="n">
-        <v>43.72</v>
+        <v>43.94</v>
       </c>
       <c r="N164" s="21">
         <f>SUM(E164:M164)</f>
@@ -49815,7 +50136,7 @@
         <v>35.4</v>
       </c>
       <c r="M166" s="4" t="n">
-        <v>59.95</v>
+        <v>60.28</v>
       </c>
       <c r="N166" s="21">
         <f>SUM(E166:M166)</f>
@@ -49917,7 +50238,7 @@
         <v>35.4</v>
       </c>
       <c r="M168" s="4" t="n">
-        <v>67.58</v>
+        <v>67.93000000000001</v>
       </c>
       <c r="N168" s="21">
         <f>SUM(E168:M168)</f>
@@ -50019,7 +50340,7 @@
         <v>35.4</v>
       </c>
       <c r="M170" s="4" t="n">
-        <v>79.02</v>
+        <v>79.43000000000001</v>
       </c>
       <c r="N170" s="21">
         <f>SUM(E170:M170)</f>
@@ -50223,7 +50544,7 @@
         <v>35.4</v>
       </c>
       <c r="M174" s="4" t="n">
-        <v>135.21</v>
+        <v>135.75</v>
       </c>
       <c r="N174" s="21">
         <f>SUM(E174:M174)</f>
@@ -50325,7 +50646,7 @@
         <v>35.4</v>
       </c>
       <c r="M176" s="4" t="n">
-        <v>125.69</v>
+        <v>126.34</v>
       </c>
       <c r="N176" s="21">
         <f>SUM(E176:M176)</f>
@@ -50427,7 +50748,7 @@
         <v>35.4</v>
       </c>
       <c r="M178" s="4" t="n">
-        <v>136.63</v>
+        <v>137.33</v>
       </c>
       <c r="N178" s="21">
         <f>SUM(E178:M178)</f>
@@ -50529,7 +50850,7 @@
         <v>35.4</v>
       </c>
       <c r="M180" s="4" t="n">
-        <v>126.19</v>
+        <v>126.84</v>
       </c>
       <c r="N180" s="21">
         <f>SUM(E180:M180)</f>
@@ -50631,7 +50952,7 @@
         <v>35.4</v>
       </c>
       <c r="M182" s="4" t="n">
-        <v>29.08</v>
+        <v>29.23</v>
       </c>
       <c r="N182" s="21">
         <f>SUM(E182:M182)</f>
@@ -50835,7 +51156,7 @@
         <v>35.4</v>
       </c>
       <c r="M186" s="4" t="n">
-        <v>29.81</v>
+        <v>29.96</v>
       </c>
       <c r="N186" s="21">
         <f>SUM(E186:M186)</f>
@@ -50937,7 +51258,7 @@
         <v>35.4</v>
       </c>
       <c r="M188" s="4" t="n">
-        <v>17.88</v>
+        <v>17.97</v>
       </c>
       <c r="N188" s="21">
         <f>SUM(E188:M188)</f>
@@ -51039,7 +51360,7 @@
         <v>35.4</v>
       </c>
       <c r="M190" s="4" t="n">
-        <v>10.52</v>
+        <v>10.57</v>
       </c>
       <c r="N190" s="21">
         <f>SUM(E190:M190)</f>
@@ -51141,7 +51462,7 @@
         <v>35.4</v>
       </c>
       <c r="M192" s="4" t="n">
-        <v>29.91</v>
+        <v>30.06</v>
       </c>
       <c r="N192" s="21">
         <f>SUM(E192:M192)</f>
@@ -51243,7 +51564,7 @@
         <v>35.4</v>
       </c>
       <c r="M194" s="4" t="n">
-        <v>31.59</v>
+        <v>31.75</v>
       </c>
       <c r="N194" s="21">
         <f>SUM(E194:M194)</f>
@@ -51345,7 +51666,7 @@
         <v>35.4</v>
       </c>
       <c r="M196" s="4" t="n">
-        <v>55.88</v>
+        <v>56.21</v>
       </c>
       <c r="N196" s="21">
         <f>SUM(E196:M196)</f>
@@ -51447,7 +51768,7 @@
         <v>35.4</v>
       </c>
       <c r="M198" s="4" t="n">
-        <v>59.65</v>
+        <v>59.94</v>
       </c>
       <c r="N198" s="21">
         <f>SUM(E198:M198)</f>
@@ -51549,7 +51870,7 @@
         <v>35.4</v>
       </c>
       <c r="M200" s="4" t="n">
-        <v>31.58</v>
+        <v>31.75</v>
       </c>
       <c r="N200" s="21">
         <f>SUM(E200:M200)</f>
@@ -51651,7 +51972,7 @@
         <v>35.4</v>
       </c>
       <c r="M202" s="4" t="n">
-        <v>52.62</v>
+        <v>52.89</v>
       </c>
       <c r="N202" s="21">
         <f>SUM(E202:M202)</f>
@@ -51753,7 +52074,7 @@
         <v>35.4</v>
       </c>
       <c r="M204" s="4" t="n">
-        <v>55.75</v>
+        <v>56.08</v>
       </c>
       <c r="N204" s="21">
         <f>SUM(E204:M204)</f>
@@ -51855,7 +52176,7 @@
         <v>35.4</v>
       </c>
       <c r="M206" s="4" t="n">
-        <v>17.52</v>
+        <v>17.61</v>
       </c>
       <c r="N206" s="21">
         <f>SUM(E206:M206)</f>
@@ -51957,7 +52278,7 @@
         <v>35.4</v>
       </c>
       <c r="M208" s="4" t="n">
-        <v>18.32</v>
+        <v>10.58</v>
       </c>
       <c r="N208" s="21">
         <f>SUM(E208:M208)</f>
@@ -52161,7 +52482,7 @@
         <v>35.4</v>
       </c>
       <c r="M212" s="4" t="n">
-        <v>10.46</v>
+        <v>10.51</v>
       </c>
       <c r="N212" s="21">
         <f>SUM(E212:M212)</f>
@@ -52263,7 +52584,7 @@
         <v>35.4</v>
       </c>
       <c r="M214" s="4" t="n">
-        <v>14.58</v>
+        <v>14.65</v>
       </c>
       <c r="N214" s="21">
         <f>SUM(E214:M214)</f>
@@ -52365,7 +52686,7 @@
         <v>35.4</v>
       </c>
       <c r="M216" s="4" t="n">
-        <v>17.48</v>
+        <v>17.57</v>
       </c>
       <c r="N216" s="21">
         <f>SUM(E216:M216)</f>
@@ -52467,7 +52788,7 @@
         <v>35.4</v>
       </c>
       <c r="M218" s="4" t="n">
-        <v>14.61</v>
+        <v>14.69</v>
       </c>
       <c r="N218" s="21">
         <f>SUM(E218:M218)</f>
@@ -52569,7 +52890,7 @@
         <v>35.4</v>
       </c>
       <c r="M220" s="4" t="n">
-        <v>17.33</v>
+        <v>17.42</v>
       </c>
       <c r="N220" s="21">
         <f>SUM(E220:M220)</f>
@@ -52671,7 +52992,7 @@
         <v>35.4</v>
       </c>
       <c r="M222" s="4" t="n">
-        <v>19.12</v>
+        <v>19.21</v>
       </c>
       <c r="N222" s="21">
         <f>SUM(E222:M222)</f>
@@ -52773,7 +53094,7 @@
         <v>35.4</v>
       </c>
       <c r="M224" s="4" t="n">
-        <v>55.07</v>
+        <v>55.06</v>
       </c>
       <c r="N224" s="21">
         <f>SUM(E224:M224)</f>
@@ -52926,7 +53247,7 @@
         <v>35.4</v>
       </c>
       <c r="M227" s="4" t="n">
-        <v>53.9</v>
+        <v>53.93</v>
       </c>
       <c r="N227" s="21">
         <f>SUM(E227:M227)</f>
@@ -53130,7 +53451,7 @@
         <v>35.4</v>
       </c>
       <c r="M231" s="4" t="n">
-        <v>57.31</v>
+        <v>57.23</v>
       </c>
       <c r="N231" s="21">
         <f>SUM(E231:M231)</f>
@@ -53262,19 +53583,19 @@
         <v>0</v>
       </c>
       <c r="F234" s="4" t="n">
-        <v>124.67</v>
+        <v>246.31</v>
       </c>
       <c r="G234" s="4" t="n">
-        <v>3.83</v>
+        <v>7.56</v>
       </c>
       <c r="H234" s="4" t="n">
-        <v>0.12</v>
+        <v>0.25</v>
       </c>
       <c r="I234" s="4" t="n">
         <v>18.7</v>
       </c>
       <c r="J234" s="4" t="n">
-        <v>0.71</v>
+        <v>1.41</v>
       </c>
       <c r="K234" s="4" t="n">
         <v>14.75</v>
@@ -53310,22 +53631,22 @@
         <v>46293</v>
       </c>
       <c r="E235" s="4" t="n">
-        <v>20</v>
+        <v>40</v>
       </c>
       <c r="F235" s="4" t="n">
-        <v>250.33</v>
+        <v>507.4</v>
       </c>
       <c r="G235" s="4" t="n">
-        <v>7.69</v>
+        <v>15.58</v>
       </c>
       <c r="H235" s="4" t="n">
-        <v>0.25</v>
+        <v>0.51</v>
       </c>
       <c r="I235" s="4" t="n">
         <v>37.55</v>
       </c>
       <c r="J235" s="4" t="n">
-        <v>5.03</v>
+        <v>10.1</v>
       </c>
       <c r="K235" s="4" t="n">
         <v>14.75</v>
@@ -53334,7 +53655,7 @@
         <v>35.4</v>
       </c>
       <c r="M235" s="4" t="n">
-        <v>160.94</v>
+        <v>92.47</v>
       </c>
       <c r="N235" s="21">
         <f>SUM(E235:M235)</f>
@@ -53361,22 +53682,22 @@
         <v>46293</v>
       </c>
       <c r="E236" s="4" t="n">
-        <v>74.84999999999999</v>
+        <v>94.84999999999999</v>
       </c>
       <c r="F236" s="4" t="n">
-        <v>249.5</v>
+        <v>498.73</v>
       </c>
       <c r="G236" s="4" t="n">
-        <v>7.66</v>
+        <v>15.31</v>
       </c>
       <c r="H236" s="4" t="n">
-        <v>0.25</v>
+        <v>0.5</v>
       </c>
       <c r="I236" s="4" t="n">
         <v>37.42</v>
       </c>
       <c r="J236" s="4" t="n">
-        <v>14.9</v>
+        <v>19.92</v>
       </c>
       <c r="K236" s="4" t="n">
         <v>14.75</v>
@@ -53412,22 +53733,22 @@
         <v>46293</v>
       </c>
       <c r="E237" s="4" t="n">
-        <v>20</v>
+        <v>40</v>
       </c>
       <c r="F237" s="4" t="n">
-        <v>251.34</v>
+        <v>490.83</v>
       </c>
       <c r="G237" s="4" t="n">
-        <v>7.72</v>
+        <v>15.07</v>
       </c>
       <c r="H237" s="4" t="n">
-        <v>0.25</v>
+        <v>0.49</v>
       </c>
       <c r="I237" s="4" t="n">
         <v>37.7</v>
       </c>
       <c r="J237" s="4" t="n">
-        <v>5.03</v>
+        <v>10</v>
       </c>
       <c r="K237" s="4" t="n">
         <v>14.75</v>
@@ -53463,22 +53784,22 @@
         <v>46293</v>
       </c>
       <c r="E238" s="4" t="n">
-        <v>74.97</v>
+        <v>94.97</v>
       </c>
       <c r="F238" s="4" t="n">
-        <v>249.86</v>
+        <v>498.88</v>
       </c>
       <c r="G238" s="4" t="n">
-        <v>7.67</v>
+        <v>15.32</v>
       </c>
       <c r="H238" s="4" t="n">
-        <v>0.25</v>
+        <v>0.5</v>
       </c>
       <c r="I238" s="4" t="n">
         <v>37.48</v>
       </c>
       <c r="J238" s="4" t="n">
-        <v>14.92</v>
+        <v>19.94</v>
       </c>
       <c r="K238" s="4" t="n">
         <v>14.75</v>
@@ -53514,22 +53835,22 @@
         <v>46293</v>
       </c>
       <c r="E239" s="4" t="n">
-        <v>20</v>
+        <v>40</v>
       </c>
       <c r="F239" s="4" t="n">
-        <v>249.79</v>
+        <v>500.26</v>
       </c>
       <c r="G239" s="4" t="n">
-        <v>7.67</v>
+        <v>15.36</v>
       </c>
       <c r="H239" s="4" t="n">
-        <v>0.25</v>
+        <v>0.5</v>
       </c>
       <c r="I239" s="4" t="n">
         <v>37.76</v>
       </c>
       <c r="J239" s="4" t="n">
-        <v>5.03</v>
+        <v>10.05</v>
       </c>
       <c r="K239" s="4" t="n">
         <v>14.75</v>
@@ -53561,24 +53882,26 @@
           <t>LONG</t>
         </is>
       </c>
-      <c r="D240" s="24" t="inlineStr"/>
+      <c r="D240" s="24" t="n">
+        <v>46294</v>
+      </c>
       <c r="E240" s="4" t="n">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="F240" s="4" t="n">
-        <v>0</v>
+        <v>299.83</v>
       </c>
       <c r="G240" s="4" t="n">
-        <v>0</v>
+        <v>9.199999999999999</v>
       </c>
       <c r="H240" s="4" t="n">
-        <v>0</v>
+        <v>0.3</v>
       </c>
       <c r="I240" s="4" t="n">
-        <v>0</v>
+        <v>44.97</v>
       </c>
       <c r="J240" s="4" t="n">
-        <v>0</v>
+        <v>5.31</v>
       </c>
       <c r="K240" s="4" t="n">
         <v>14.75</v>
@@ -53587,7 +53910,7 @@
         <v>35.4</v>
       </c>
       <c r="M240" s="4" t="n">
-        <v>0</v>
+        <v>62.93</v>
       </c>
       <c r="N240" s="21">
         <f>SUM(E240:M240)</f>
@@ -53610,7 +53933,9 @@
           <t>LONG</t>
         </is>
       </c>
-      <c r="D241" s="24" t="inlineStr"/>
+      <c r="D241" s="24" t="n">
+        <v>46294</v>
+      </c>
       <c r="E241" s="4" t="n">
         <v>0</v>
       </c>
@@ -53636,7 +53961,7 @@
         <v>35.4</v>
       </c>
       <c r="M241" s="4" t="n">
-        <v>0</v>
+        <v>65.34</v>
       </c>
       <c r="N241" s="21">
         <f>SUM(E241:M241)</f>
@@ -53646,20 +53971,22 @@
     <row r="242">
       <c r="A242" s="23" t="inlineStr">
         <is>
-          <t>DHAN-341260928158709+341260928158609+221260928823209+341260928158409+341260928158209+341260928158009+341260928157909+221260928821609+341260928157709+221260928820609+341260928157509</t>
+          <t>DHAN-23126092924109</t>
         </is>
       </c>
       <c r="B242" s="23" t="inlineStr">
         <is>
-          <t>SDBL</t>
+          <t>RSYSTEMS</t>
         </is>
       </c>
       <c r="C242" s="23" t="inlineStr">
         <is>
-          <t>LONG</t>
-        </is>
-      </c>
-      <c r="D242" s="24" t="inlineStr"/>
+          <t>SHORT</t>
+        </is>
+      </c>
+      <c r="D242" s="24" t="n">
+        <v>46294</v>
+      </c>
       <c r="E242" s="4" t="n">
         <v>0</v>
       </c>
@@ -53679,10 +54006,10 @@
         <v>0</v>
       </c>
       <c r="K242" s="4" t="n">
-        <v>14.75</v>
+        <v>0</v>
       </c>
       <c r="L242" s="4" t="n">
-        <v>35.4</v>
+        <v>0</v>
       </c>
       <c r="M242" s="4" t="n">
         <v>0</v>
@@ -53695,12 +54022,12 @@
     <row r="243">
       <c r="A243" s="23" t="inlineStr">
         <is>
-          <t>DHAN-341260928159209</t>
+          <t>DHAN-341260928158709+341260928158609+221260928823209+341260928158409+341260928158209+341260928158009+341260928157909+221260928821609+341260928157709+221260928820609+341260928157509</t>
         </is>
       </c>
       <c r="B243" s="23" t="inlineStr">
         <is>
-          <t>SMCGLOBAL</t>
+          <t>SDBL</t>
         </is>
       </c>
       <c r="C243" s="23" t="inlineStr">
@@ -53708,24 +54035,26 @@
           <t>LONG</t>
         </is>
       </c>
-      <c r="D243" s="24" t="inlineStr"/>
+      <c r="D243" s="24" t="n">
+        <v>46294</v>
+      </c>
       <c r="E243" s="4" t="n">
-        <v>0</v>
+        <v>89.91</v>
       </c>
       <c r="F243" s="4" t="n">
-        <v>0</v>
+        <v>299.53</v>
       </c>
       <c r="G243" s="4" t="n">
-        <v>0</v>
+        <v>9.199999999999999</v>
       </c>
       <c r="H243" s="4" t="n">
-        <v>0</v>
+        <v>0.3</v>
       </c>
       <c r="I243" s="4" t="n">
-        <v>0</v>
+        <v>44.93</v>
       </c>
       <c r="J243" s="4" t="n">
-        <v>0</v>
+        <v>17.89</v>
       </c>
       <c r="K243" s="4" t="n">
         <v>14.75</v>
@@ -53734,7 +54063,7 @@
         <v>35.4</v>
       </c>
       <c r="M243" s="4" t="n">
-        <v>0</v>
+        <v>62.42</v>
       </c>
       <c r="N243" s="21">
         <f>SUM(E243:M243)</f>
@@ -53744,12 +54073,12 @@
     <row r="244">
       <c r="A244" s="23" t="inlineStr">
         <is>
-          <t>DHAN-341260928159109</t>
+          <t>DHAN-341260928159209</t>
         </is>
       </c>
       <c r="B244" s="23" t="inlineStr">
         <is>
-          <t>SYNCOMF</t>
+          <t>SMCGLOBAL</t>
         </is>
       </c>
       <c r="C244" s="23" t="inlineStr">
@@ -53757,24 +54086,26 @@
           <t>LONG</t>
         </is>
       </c>
-      <c r="D244" s="24" t="inlineStr"/>
+      <c r="D244" s="24" t="n">
+        <v>46294</v>
+      </c>
       <c r="E244" s="4" t="n">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="F244" s="4" t="n">
-        <v>0</v>
+        <v>300.06</v>
       </c>
       <c r="G244" s="4" t="n">
-        <v>0</v>
+        <v>9.210000000000001</v>
       </c>
       <c r="H244" s="4" t="n">
-        <v>0</v>
+        <v>0.3</v>
       </c>
       <c r="I244" s="4" t="n">
-        <v>0</v>
+        <v>45.01</v>
       </c>
       <c r="J244" s="4" t="n">
-        <v>0</v>
+        <v>5.31</v>
       </c>
       <c r="K244" s="4" t="n">
         <v>14.75</v>
@@ -53783,7 +54114,7 @@
         <v>35.4</v>
       </c>
       <c r="M244" s="4" t="n">
-        <v>0</v>
+        <v>51.31</v>
       </c>
       <c r="N244" s="21">
         <f>SUM(E244:M244)</f>
@@ -53791,54 +54122,399 @@
       </c>
     </row>
     <row r="245">
-      <c r="A245" s="3" t="inlineStr">
+      <c r="A245" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-341260928159109</t>
+        </is>
+      </c>
+      <c r="B245" s="23" t="inlineStr">
+        <is>
+          <t>SYNCOMF</t>
+        </is>
+      </c>
+      <c r="C245" s="23" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="D245" s="24" t="n">
+        <v>46294</v>
+      </c>
+      <c r="E245" s="4" t="n">
+        <v>20</v>
+      </c>
+      <c r="F245" s="4" t="n">
+        <v>299.85</v>
+      </c>
+      <c r="G245" s="4" t="n">
+        <v>9.210000000000001</v>
+      </c>
+      <c r="H245" s="4" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="I245" s="4" t="n">
+        <v>44.98</v>
+      </c>
+      <c r="J245" s="4" t="n">
+        <v>5.31</v>
+      </c>
+      <c r="K245" s="4" t="n">
+        <v>14.75</v>
+      </c>
+      <c r="L245" s="4" t="n">
+        <v>35.4</v>
+      </c>
+      <c r="M245" s="4" t="n">
+        <v>51.27</v>
+      </c>
+      <c r="N245" s="21">
+        <f>SUM(E245:M245)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="246">
+      <c r="A246" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-221260929652409</t>
+        </is>
+      </c>
+      <c r="B246" s="23" t="inlineStr">
+        <is>
+          <t>ELECTCAST</t>
+        </is>
+      </c>
+      <c r="C246" s="23" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="D246" s="24" t="inlineStr"/>
+      <c r="E246" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F246" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G246" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H246" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I246" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J246" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K246" s="4" t="n">
+        <v>14.75</v>
+      </c>
+      <c r="L246" s="4" t="n">
+        <v>35.4</v>
+      </c>
+      <c r="M246" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="N246" s="21">
+        <f>SUM(E246:M246)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="247">
+      <c r="A247" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-221260929652309</t>
+        </is>
+      </c>
+      <c r="B247" s="23" t="inlineStr">
+        <is>
+          <t>INDOCO</t>
+        </is>
+      </c>
+      <c r="C247" s="23" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="D247" s="24" t="inlineStr"/>
+      <c r="E247" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F247" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G247" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H247" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I247" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J247" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K247" s="4" t="n">
+        <v>14.75</v>
+      </c>
+      <c r="L247" s="4" t="n">
+        <v>35.4</v>
+      </c>
+      <c r="M247" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="N247" s="21">
+        <f>SUM(E247:M247)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="248">
+      <c r="A248" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-221260929652509</t>
+        </is>
+      </c>
+      <c r="B248" s="23" t="inlineStr">
+        <is>
+          <t>RSYSTEMS</t>
+        </is>
+      </c>
+      <c r="C248" s="23" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="D248" s="24" t="inlineStr"/>
+      <c r="E248" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F248" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G248" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H248" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I248" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J248" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K248" s="4" t="n">
+        <v>14.75</v>
+      </c>
+      <c r="L248" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="M248" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="N248" s="21">
+        <f>SUM(E248:M248)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="249">
+      <c r="A249" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-321260929420709</t>
+        </is>
+      </c>
+      <c r="B249" s="23" t="inlineStr">
+        <is>
+          <t>SYNCOMF</t>
+        </is>
+      </c>
+      <c r="C249" s="23" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="D249" s="24" t="inlineStr"/>
+      <c r="E249" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F249" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G249" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H249" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I249" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J249" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K249" s="4" t="n">
+        <v>14.75</v>
+      </c>
+      <c r="L249" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="M249" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="N249" s="21">
+        <f>SUM(E249:M249)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="250">
+      <c r="A250" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-34126092973909+321260929416609+34126092974209+34126092974309+221260929647009+221260929647509+23126092975109+34126092974609+23126092975209+221260929648209+221260929648709+23126092975409+23126092975509+34126092974709</t>
+        </is>
+      </c>
+      <c r="B250" s="23" t="inlineStr">
+        <is>
+          <t>TCIEXP</t>
+        </is>
+      </c>
+      <c r="C250" s="23" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="D250" s="24" t="inlineStr"/>
+      <c r="E250" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F250" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G250" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H250" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I250" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J250" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K250" s="4" t="n">
+        <v>14.75</v>
+      </c>
+      <c r="L250" s="4" t="n">
+        <v>35.4</v>
+      </c>
+      <c r="M250" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="N250" s="21">
+        <f>SUM(E250:M250)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="251">
+      <c r="A251" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-321260929416409+34126092974109+23126092974809+34126092974409+321260929417209+221260929647409+321260929417509+321260929417709+23126092975309+321260929418309+221260929648809+321260929418709+34126092974809</t>
+        </is>
+      </c>
+      <c r="B251" s="23" t="inlineStr">
+        <is>
+          <t>UNICHEMLAB</t>
+        </is>
+      </c>
+      <c r="C251" s="23" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="D251" s="24" t="inlineStr"/>
+      <c r="E251" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F251" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G251" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H251" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I251" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J251" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K251" s="4" t="n">
+        <v>14.75</v>
+      </c>
+      <c r="L251" s="4" t="n">
+        <v>35.4</v>
+      </c>
+      <c r="M251" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="N251" s="21">
+        <f>SUM(E251:M251)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="252">
+      <c r="A252" s="3" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="E245" s="32">
-        <f>SUM(E4:E244)</f>
-        <v/>
-      </c>
-      <c r="F245" s="32">
-        <f>SUM(F4:F244)</f>
-        <v/>
-      </c>
-      <c r="G245" s="32">
-        <f>SUM(G4:G244)</f>
-        <v/>
-      </c>
-      <c r="H245" s="32">
-        <f>SUM(H4:H244)</f>
-        <v/>
-      </c>
-      <c r="I245" s="32">
-        <f>SUM(I4:I244)</f>
-        <v/>
-      </c>
-      <c r="J245" s="32">
-        <f>SUM(J4:J244)</f>
-        <v/>
-      </c>
-      <c r="K245" s="32">
-        <f>SUM(K4:K244)</f>
-        <v/>
-      </c>
-      <c r="L245" s="32">
-        <f>SUM(L4:L244)</f>
-        <v/>
-      </c>
-      <c r="M245" s="32">
-        <f>SUM(M4:M244)</f>
-        <v/>
-      </c>
-      <c r="N245" s="32">
-        <f>SUM(N4:N244)</f>
+      <c r="E252" s="32">
+        <f>SUM(E4:E251)</f>
+        <v/>
+      </c>
+      <c r="F252" s="32">
+        <f>SUM(F4:F251)</f>
+        <v/>
+      </c>
+      <c r="G252" s="32">
+        <f>SUM(G4:G251)</f>
+        <v/>
+      </c>
+      <c r="H252" s="32">
+        <f>SUM(H4:H251)</f>
+        <v/>
+      </c>
+      <c r="I252" s="32">
+        <f>SUM(I4:I251)</f>
+        <v/>
+      </c>
+      <c r="J252" s="32">
+        <f>SUM(J4:J251)</f>
+        <v/>
+      </c>
+      <c r="K252" s="32">
+        <f>SUM(K4:K251)</f>
+        <v/>
+      </c>
+      <c r="L252" s="32">
+        <f>SUM(L4:L251)</f>
+        <v/>
+      </c>
+      <c r="M252" s="32">
+        <f>SUM(M4:M251)</f>
+        <v/>
+      </c>
+      <c r="N252" s="32">
+        <f>SUM(N4:N251)</f>
         <v/>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A3:N244"/>
+  <autoFilter ref="A3:N251"/>
   <mergeCells count="2">
     <mergeCell ref="A2:N2"/>
     <mergeCell ref="A1:N1"/>

</xml_diff>

<commit_message>
Data update — 2026-09-30 candle + results refresh
</commit_message>
<xml_diff>
--- a/results/strategy_pnl_simple.xlsx
+++ b/results/strategy_pnl_simple.xlsx
@@ -18,7 +18,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Trade Log'!$A$3:$O$503</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Charges'!$A$3:$N$251</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Charges'!$A$3:$N$254</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -1094,7 +1094,7 @@
         <v/>
       </c>
       <c r="K4" s="4" t="n">
-        <v>571.63</v>
+        <v>570.16</v>
       </c>
       <c r="L4" s="21">
         <f>IF(OR($B4="",$I4=""),"",$I4-IF($K4="",0,$K4))</f>
@@ -1214,7 +1214,7 @@
         <v/>
       </c>
       <c r="K6" s="4" t="n">
-        <v>688.95</v>
+        <v>686.95</v>
       </c>
       <c r="L6" s="21">
         <f>IF(OR($B6="",$I6=""),"",$I6-IF($K6="",0,$K6))</f>
@@ -1334,7 +1334,7 @@
         <v/>
       </c>
       <c r="K8" s="4" t="n">
-        <v>570.48</v>
+        <v>569.01</v>
       </c>
       <c r="L8" s="21">
         <f>IF(OR($B8="",$I8=""),"",$I8-IF($K8="",0,$K8))</f>
@@ -1454,7 +1454,7 @@
         <v/>
       </c>
       <c r="K10" s="4" t="n">
-        <v>662.85</v>
+        <v>661.09</v>
       </c>
       <c r="L10" s="21">
         <f>IF(OR($B10="",$I10=""),"",$I10-IF($K10="",0,$K10))</f>
@@ -1574,7 +1574,7 @@
         <v/>
       </c>
       <c r="K12" s="4" t="n">
-        <v>591.6900000000001</v>
+        <v>590.1</v>
       </c>
       <c r="L12" s="21">
         <f>IF(OR($B12="",$I12=""),"",$I12-IF($K12="",0,$K12))</f>
@@ -1694,7 +1694,7 @@
         <v/>
       </c>
       <c r="K14" s="4" t="n">
-        <v>398.53</v>
+        <v>397.72</v>
       </c>
       <c r="L14" s="21">
         <f>IF(OR($B14="",$I14=""),"",$I14-IF($K14="",0,$K14))</f>
@@ -1814,7 +1814,7 @@
         <v/>
       </c>
       <c r="K16" s="4" t="n">
-        <v>414.05</v>
+        <v>413.07</v>
       </c>
       <c r="L16" s="21">
         <f>IF(OR($B16="",$I16=""),"",$I16-IF($K16="",0,$K16))</f>
@@ -1934,7 +1934,7 @@
         <v/>
       </c>
       <c r="K18" s="4" t="n">
-        <v>345.01</v>
+        <v>344.42</v>
       </c>
       <c r="L18" s="21">
         <f>IF(OR($B18="",$I18=""),"",$I18-IF($K18="",0,$K18))</f>
@@ -2054,7 +2054,7 @@
         <v/>
       </c>
       <c r="K20" s="4" t="n">
-        <v>414.39</v>
+        <v>413.41</v>
       </c>
       <c r="L20" s="21">
         <f>IF(OR($B20="",$I20=""),"",$I20-IF($K20="",0,$K20))</f>
@@ -2174,7 +2174,7 @@
         <v/>
       </c>
       <c r="K22" s="4" t="n">
-        <v>380.53</v>
+        <v>379.51</v>
       </c>
       <c r="L22" s="21">
         <f>IF(OR($B22="",$I22=""),"",$I22-IF($K22="",0,$K22))</f>
@@ -2294,7 +2294,7 @@
         <v/>
       </c>
       <c r="K24" s="4" t="n">
-        <v>413.82</v>
+        <v>412.83</v>
       </c>
       <c r="L24" s="21">
         <f>IF(OR($B24="",$I24=""),"",$I24-IF($K24="",0,$K24))</f>
@@ -2414,7 +2414,7 @@
         <v/>
       </c>
       <c r="K26" s="4" t="n">
-        <v>406.36</v>
+        <v>405.53</v>
       </c>
       <c r="L26" s="21">
         <f>IF(OR($B26="",$I26=""),"",$I26-IF($K26="",0,$K26))</f>
@@ -2654,7 +2654,7 @@
         <v/>
       </c>
       <c r="K30" s="4" t="n">
-        <v>870.76</v>
+        <v>867.36</v>
       </c>
       <c r="L30" s="21">
         <f>IF(OR($B30="",$I30=""),"",$I30-IF($K30="",0,$K30))</f>
@@ -2894,7 +2894,7 @@
         <v/>
       </c>
       <c r="K34" s="4" t="n">
-        <v>390.59</v>
+        <v>390.58</v>
       </c>
       <c r="L34" s="21">
         <f>IF(OR($B34="",$I34=""),"",$I34-IF($K34="",0,$K34))</f>
@@ -3014,7 +3014,7 @@
         <v/>
       </c>
       <c r="K36" s="4" t="n">
-        <v>349.21</v>
+        <v>349.19</v>
       </c>
       <c r="L36" s="21">
         <f>IF(OR($B36="",$I36=""),"",$I36-IF($K36="",0,$K36))</f>
@@ -3254,7 +3254,7 @@
         <v/>
       </c>
       <c r="K40" s="4" t="n">
-        <v>385.43</v>
+        <v>385.46</v>
       </c>
       <c r="L40" s="21">
         <f>IF(OR($B40="",$I40=""),"",$I40-IF($K40="",0,$K40))</f>
@@ -3374,7 +3374,7 @@
         <v/>
       </c>
       <c r="K42" s="4" t="n">
-        <v>977.08</v>
+        <v>977.0599999999999</v>
       </c>
       <c r="L42" s="21">
         <f>IF(OR($B42="",$I42=""),"",$I42-IF($K42="",0,$K42))</f>
@@ -3434,7 +3434,7 @@
         <v/>
       </c>
       <c r="K43" s="4" t="n">
-        <v>956.6799999999999</v>
+        <v>956.66</v>
       </c>
       <c r="L43" s="21">
         <f>IF(OR($B43="",$I43=""),"",$I43-IF($K43="",0,$K43))</f>
@@ -3494,7 +3494,7 @@
         <v/>
       </c>
       <c r="K44" s="4" t="n">
-        <v>991.0700000000001</v>
+        <v>991.04</v>
       </c>
       <c r="L44" s="21">
         <f>IF(OR($B44="",$I44=""),"",$I44-IF($K44="",0,$K44))</f>
@@ -3554,7 +3554,7 @@
         <v/>
       </c>
       <c r="K45" s="4" t="n">
-        <v>597.78</v>
+        <v>597.74</v>
       </c>
       <c r="L45" s="21">
         <f>IF(OR($B45="",$I45=""),"",$I45-IF($K45="",0,$K45))</f>
@@ -3674,7 +3674,7 @@
         <v/>
       </c>
       <c r="K47" s="4" t="n">
-        <v>598.88</v>
+        <v>598.84</v>
       </c>
       <c r="L47" s="21">
         <f>IF(OR($B47="",$I47=""),"",$I47-IF($K47="",0,$K47))</f>
@@ -3794,7 +3794,7 @@
         <v/>
       </c>
       <c r="K49" s="4" t="n">
-        <v>677.36</v>
+        <v>677.37</v>
       </c>
       <c r="L49" s="21">
         <f>IF(OR($B49="",$I49=""),"",$I49-IF($K49="",0,$K49))</f>
@@ -3914,7 +3914,7 @@
         <v/>
       </c>
       <c r="K51" s="4" t="n">
-        <v>669.9299999999999</v>
+        <v>670.05</v>
       </c>
       <c r="L51" s="21">
         <f>IF(OR($B51="",$I51=""),"",$I51-IF($K51="",0,$K51))</f>
@@ -4034,7 +4034,7 @@
         <v/>
       </c>
       <c r="K53" s="4" t="n">
-        <v>574.48</v>
+        <v>574.45</v>
       </c>
       <c r="L53" s="21">
         <f>IF(OR($B53="",$I53=""),"",$I53-IF($K53="",0,$K53))</f>
@@ -4154,7 +4154,7 @@
         <v/>
       </c>
       <c r="K55" s="4" t="n">
-        <v>628.42</v>
+        <v>628.4400000000001</v>
       </c>
       <c r="L55" s="21">
         <f>IF(OR($B55="",$I55=""),"",$I55-IF($K55="",0,$K55))</f>
@@ -4274,7 +4274,7 @@
         <v/>
       </c>
       <c r="K57" s="4" t="n">
-        <v>619.35</v>
+        <v>619.39</v>
       </c>
       <c r="L57" s="21">
         <f>IF(OR($B57="",$I57=""),"",$I57-IF($K57="",0,$K57))</f>
@@ -4394,7 +4394,7 @@
         <v/>
       </c>
       <c r="K59" s="4" t="n">
-        <v>612.45</v>
+        <v>612.4400000000001</v>
       </c>
       <c r="L59" s="21">
         <f>IF(OR($B59="",$I59=""),"",$I59-IF($K59="",0,$K59))</f>
@@ -4634,7 +4634,7 @@
         <v/>
       </c>
       <c r="K63" s="4" t="n">
-        <v>693.6799999999999</v>
+        <v>693.67</v>
       </c>
       <c r="L63" s="21">
         <f>IF(OR($B63="",$I63=""),"",$I63-IF($K63="",0,$K63))</f>
@@ -4754,7 +4754,7 @@
         <v/>
       </c>
       <c r="K65" s="4" t="n">
-        <v>617</v>
+        <v>616.97</v>
       </c>
       <c r="L65" s="21">
         <f>IF(OR($B65="",$I65=""),"",$I65-IF($K65="",0,$K65))</f>
@@ -4874,7 +4874,7 @@
         <v/>
       </c>
       <c r="K67" s="4" t="n">
-        <v>441.5</v>
+        <v>441.52</v>
       </c>
       <c r="L67" s="21">
         <f>IF(OR($B67="",$I67=""),"",$I67-IF($K67="",0,$K67))</f>
@@ -5714,7 +5714,7 @@
         <v/>
       </c>
       <c r="K81" s="4" t="n">
-        <v>356.27</v>
+        <v>356.26</v>
       </c>
       <c r="L81" s="21">
         <f>IF(OR($B81="",$I81=""),"",$I81-IF($K81="",0,$K81))</f>
@@ -5834,7 +5834,7 @@
         <v/>
       </c>
       <c r="K83" s="4" t="n">
-        <v>364.89</v>
+        <v>364.88</v>
       </c>
       <c r="L83" s="21">
         <f>IF(OR($B83="",$I83=""),"",$I83-IF($K83="",0,$K83))</f>
@@ -5954,7 +5954,7 @@
         <v/>
       </c>
       <c r="K85" s="4" t="n">
-        <v>412.36</v>
+        <v>412.4</v>
       </c>
       <c r="L85" s="21">
         <f>IF(OR($B85="",$I85=""),"",$I85-IF($K85="",0,$K85))</f>
@@ -6074,7 +6074,7 @@
         <v/>
       </c>
       <c r="K87" s="4" t="n">
-        <v>344.24</v>
+        <v>344.23</v>
       </c>
       <c r="L87" s="21">
         <f>IF(OR($B87="",$I87=""),"",$I87-IF($K87="",0,$K87))</f>
@@ -6314,7 +6314,7 @@
         <v/>
       </c>
       <c r="K91" s="4" t="n">
-        <v>893.51</v>
+        <v>893.48</v>
       </c>
       <c r="L91" s="21">
         <f>IF(OR($B91="",$I91=""),"",$I91-IF($K91="",0,$K91))</f>
@@ -6434,7 +6434,7 @@
         <v/>
       </c>
       <c r="K93" s="4" t="n">
-        <v>799.52</v>
+        <v>799.49</v>
       </c>
       <c r="L93" s="21">
         <f>IF(OR($B93="",$I93=""),"",$I93-IF($K93="",0,$K93))</f>
@@ -6554,7 +6554,7 @@
         <v/>
       </c>
       <c r="K95" s="4" t="n">
-        <v>826.86</v>
+        <v>826.83</v>
       </c>
       <c r="L95" s="21">
         <f>IF(OR($B95="",$I95=""),"",$I95-IF($K95="",0,$K95))</f>
@@ -6674,7 +6674,7 @@
         <v/>
       </c>
       <c r="K97" s="4" t="n">
-        <v>479.66</v>
+        <v>479.69</v>
       </c>
       <c r="L97" s="21">
         <f>IF(OR($B97="",$I97=""),"",$I97-IF($K97="",0,$K97))</f>
@@ -6914,7 +6914,7 @@
         <v/>
       </c>
       <c r="K101" s="4" t="n">
-        <v>474.6</v>
+        <v>474.59</v>
       </c>
       <c r="L101" s="21">
         <f>IF(OR($B101="",$I101=""),"",$I101-IF($K101="",0,$K101))</f>
@@ -7034,7 +7034,7 @@
         <v/>
       </c>
       <c r="K103" s="4" t="n">
-        <v>531.37</v>
+        <v>531.36</v>
       </c>
       <c r="L103" s="21">
         <f>IF(OR($B103="",$I103=""),"",$I103-IF($K103="",0,$K103))</f>
@@ -7214,7 +7214,7 @@
         <v/>
       </c>
       <c r="K106" s="4" t="n">
-        <v>531.58</v>
+        <v>531.5700000000001</v>
       </c>
       <c r="L106" s="21">
         <f>IF(OR($B106="",$I106=""),"",$I106-IF($K106="",0,$K106))</f>
@@ -7694,7 +7694,7 @@
         <v/>
       </c>
       <c r="K114" s="4" t="n">
-        <v>480.95</v>
+        <v>480.98</v>
       </c>
       <c r="L114" s="21">
         <f>IF(OR($B114="",$I114=""),"",$I114-IF($K114="",0,$K114))</f>
@@ -7814,7 +7814,7 @@
         <v/>
       </c>
       <c r="K116" s="4" t="n">
-        <v>420.15</v>
+        <v>420.14</v>
       </c>
       <c r="L116" s="21">
         <f>IF(OR($B116="",$I116=""),"",$I116-IF($K116="",0,$K116))</f>
@@ -8054,7 +8054,7 @@
         <v/>
       </c>
       <c r="K120" s="4" t="n">
-        <v>428.89</v>
+        <v>428.94</v>
       </c>
       <c r="L120" s="21">
         <f>IF(OR($B120="",$I120=""),"",$I120-IF($K120="",0,$K120))</f>
@@ -8174,7 +8174,7 @@
         <v/>
       </c>
       <c r="K122" s="4" t="n">
-        <v>546.35</v>
+        <v>546.34</v>
       </c>
       <c r="L122" s="21">
         <f>IF(OR($B122="",$I122=""),"",$I122-IF($K122="",0,$K122))</f>
@@ -8414,7 +8414,7 @@
         <v/>
       </c>
       <c r="K126" s="4" t="n">
-        <v>425.11</v>
+        <v>425.06</v>
       </c>
       <c r="L126" s="21">
         <f>IF(OR($B126="",$I126=""),"",$I126-IF($K126="",0,$K126))</f>
@@ -8654,7 +8654,7 @@
         <v/>
       </c>
       <c r="K130" s="4" t="n">
-        <v>642.52</v>
+        <v>642.5</v>
       </c>
       <c r="L130" s="21">
         <f>IF(OR($B130="",$I130=""),"",$I130-IF($K130="",0,$K130))</f>
@@ -8774,7 +8774,7 @@
         <v/>
       </c>
       <c r="K132" s="4" t="n">
-        <v>638.36</v>
+        <v>638.35</v>
       </c>
       <c r="L132" s="21">
         <f>IF(OR($B132="",$I132=""),"",$I132-IF($K132="",0,$K132))</f>
@@ -8894,7 +8894,7 @@
         <v/>
       </c>
       <c r="K134" s="4" t="n">
-        <v>654.01</v>
+        <v>654.08</v>
       </c>
       <c r="L134" s="21">
         <f>IF(OR($B134="",$I134=""),"",$I134-IF($K134="",0,$K134))</f>
@@ -9014,7 +9014,7 @@
         <v/>
       </c>
       <c r="K136" s="4" t="n">
-        <v>564.1900000000001</v>
+        <v>564.17</v>
       </c>
       <c r="L136" s="21">
         <f>IF(OR($B136="",$I136=""),"",$I136-IF($K136="",0,$K136))</f>
@@ -9134,7 +9134,7 @@
         <v/>
       </c>
       <c r="K138" s="4" t="n">
-        <v>632.15</v>
+        <v>632.14</v>
       </c>
       <c r="L138" s="21">
         <f>IF(OR($B138="",$I138=""),"",$I138-IF($K138="",0,$K138))</f>
@@ -9254,7 +9254,7 @@
         <v/>
       </c>
       <c r="K140" s="4" t="n">
-        <v>497.9</v>
+        <v>497.88</v>
       </c>
       <c r="L140" s="21">
         <f>IF(OR($B140="",$I140=""),"",$I140-IF($K140="",0,$K140))</f>
@@ -9494,7 +9494,7 @@
         <v/>
       </c>
       <c r="K144" s="4" t="n">
-        <v>494.64</v>
+        <v>494.62</v>
       </c>
       <c r="L144" s="21">
         <f>IF(OR($B144="",$I144=""),"",$I144-IF($K144="",0,$K144))</f>
@@ -9614,7 +9614,7 @@
         <v/>
       </c>
       <c r="K146" s="4" t="n">
-        <v>504.61</v>
+        <v>504.68</v>
       </c>
       <c r="L146" s="21">
         <f>IF(OR($B146="",$I146=""),"",$I146-IF($K146="",0,$K146))</f>
@@ -9734,7 +9734,7 @@
         <v/>
       </c>
       <c r="K148" s="4" t="n">
-        <v>490.99</v>
+        <v>491.12</v>
       </c>
       <c r="L148" s="21">
         <f>IF(OR($B148="",$I148=""),"",$I148-IF($K148="",0,$K148))</f>
@@ -9854,7 +9854,7 @@
         <v/>
       </c>
       <c r="K150" s="4" t="n">
-        <v>467.3</v>
+        <v>467.29</v>
       </c>
       <c r="L150" s="21">
         <f>IF(OR($B150="",$I150=""),"",$I150-IF($K150="",0,$K150))</f>
@@ -10094,7 +10094,7 @@
         <v/>
       </c>
       <c r="K154" s="4" t="n">
-        <v>542.37</v>
+        <v>542.29</v>
       </c>
       <c r="L154" s="21">
         <f>IF(OR($B154="",$I154=""),"",$I154-IF($K154="",0,$K154))</f>
@@ -10214,7 +10214,7 @@
         <v/>
       </c>
       <c r="K156" s="4" t="n">
-        <v>461.59</v>
+        <v>461.56</v>
       </c>
       <c r="L156" s="21">
         <f>IF(OR($B156="",$I156=""),"",$I156-IF($K156="",0,$K156))</f>
@@ -10334,7 +10334,7 @@
         <v/>
       </c>
       <c r="K158" s="4" t="n">
-        <v>526.41</v>
+        <v>526.4</v>
       </c>
       <c r="L158" s="21">
         <f>IF(OR($B158="",$I158=""),"",$I158-IF($K158="",0,$K158))</f>
@@ -10454,7 +10454,7 @@
         <v/>
       </c>
       <c r="K160" s="4" t="n">
-        <v>520.62</v>
+        <v>520.61</v>
       </c>
       <c r="L160" s="21">
         <f>IF(OR($B160="",$I160=""),"",$I160-IF($K160="",0,$K160))</f>
@@ -11294,7 +11294,7 @@
         <v/>
       </c>
       <c r="K174" s="4" t="n">
-        <v>600.27</v>
+        <v>600.3200000000001</v>
       </c>
       <c r="L174" s="21">
         <f>IF(OR($B174="",$I174=""),"",$I174-IF($K174="",0,$K174))</f>
@@ -11414,7 +11414,7 @@
         <v/>
       </c>
       <c r="K176" s="4" t="n">
-        <v>589.6900000000001</v>
+        <v>589.6799999999999</v>
       </c>
       <c r="L176" s="21">
         <f>IF(OR($B176="",$I176=""),"",$I176-IF($K176="",0,$K176))</f>
@@ -11534,7 +11534,7 @@
         <v/>
       </c>
       <c r="K178" s="4" t="n">
-        <v>602.4299999999999</v>
+        <v>602.41</v>
       </c>
       <c r="L178" s="21">
         <f>IF(OR($B178="",$I178=""),"",$I178-IF($K178="",0,$K178))</f>
@@ -11654,7 +11654,7 @@
         <v/>
       </c>
       <c r="K180" s="4" t="n">
-        <v>591.6799999999999</v>
+        <v>591.66</v>
       </c>
       <c r="L180" s="21">
         <f>IF(OR($B180="",$I180=""),"",$I180-IF($K180="",0,$K180))</f>
@@ -12134,7 +12134,7 @@
         <v/>
       </c>
       <c r="K188" s="4" t="n">
-        <v>288.92</v>
+        <v>288.91</v>
       </c>
       <c r="L188" s="21">
         <f>IF(OR($B188="",$I188=""),"",$I188-IF($K188="",0,$K188))</f>
@@ -12374,7 +12374,7 @@
         <v/>
       </c>
       <c r="K192" s="4" t="n">
-        <v>296.17</v>
+        <v>296.19</v>
       </c>
       <c r="L192" s="21">
         <f>IF(OR($B192="",$I192=""),"",$I192-IF($K192="",0,$K192))</f>
@@ -12614,7 +12614,7 @@
         <v/>
       </c>
       <c r="K196" s="4" t="n">
-        <v>461.42</v>
+        <v>461.44</v>
       </c>
       <c r="L196" s="21">
         <f>IF(OR($B196="",$I196=""),"",$I196-IF($K196="",0,$K196))</f>
@@ -12734,7 +12734,7 @@
         <v/>
       </c>
       <c r="K198" s="4" t="n">
-        <v>464.33</v>
+        <v>464.36</v>
       </c>
       <c r="L198" s="21">
         <f>IF(OR($B198="",$I198=""),"",$I198-IF($K198="",0,$K198))</f>
@@ -12854,7 +12854,7 @@
         <v/>
       </c>
       <c r="K200" s="4" t="n">
-        <v>497.5</v>
+        <v>497.49</v>
       </c>
       <c r="L200" s="21">
         <f>IF(OR($B200="",$I200=""),"",$I200-IF($K200="",0,$K200))</f>
@@ -13094,7 +13094,7 @@
         <v/>
       </c>
       <c r="K204" s="4" t="n">
-        <v>458.31</v>
+        <v>458.33</v>
       </c>
       <c r="L204" s="21">
         <f>IF(OR($B204="",$I204=""),"",$I204-IF($K204="",0,$K204))</f>
@@ -14174,7 +14174,7 @@
         <v/>
       </c>
       <c r="K222" s="4" t="n">
-        <v>361.08</v>
+        <v>361.06</v>
       </c>
       <c r="L222" s="21">
         <f>IF(OR($B222="",$I222=""),"",$I222-IF($K222="",0,$K222))</f>
@@ -14294,7 +14294,7 @@
         <v/>
       </c>
       <c r="K224" s="4" t="n">
-        <v>459.2</v>
+        <v>459.23</v>
       </c>
       <c r="L224" s="21">
         <f>IF(OR($B224="",$I224=""),"",$I224-IF($K224="",0,$K224))</f>
@@ -14474,7 +14474,7 @@
         <v/>
       </c>
       <c r="K227" s="4" t="n">
-        <v>521.52</v>
+        <v>521.55</v>
       </c>
       <c r="L227" s="21">
         <f>IF(OR($B227="",$I227=""),"",$I227-IF($K227="",0,$K227))</f>
@@ -14714,7 +14714,7 @@
         <v/>
       </c>
       <c r="K231" s="4" t="n">
-        <v>461.23</v>
+        <v>461.19</v>
       </c>
       <c r="L231" s="21">
         <f>IF(OR($B231="",$I231=""),"",$I231-IF($K231="",0,$K231))</f>
@@ -15074,7 +15074,7 @@
         <v/>
       </c>
       <c r="K237" s="4" t="n">
-        <v>798.96</v>
+        <v>737.0700000000001</v>
       </c>
       <c r="L237" s="21">
         <f>IF(OR($B237="",$I237=""),"",$I237-IF($K237="",0,$K237))</f>
@@ -15254,7 +15254,7 @@
         <v/>
       </c>
       <c r="K240" s="4" t="n">
-        <v>492.69</v>
+        <v>815.71</v>
       </c>
       <c r="L240" s="21">
         <f>IF(OR($B240="",$I240=""),"",$I240-IF($K240="",0,$K240))</f>
@@ -15314,7 +15314,7 @@
         <v/>
       </c>
       <c r="K241" s="4" t="n">
-        <v>115.49</v>
+        <v>150.51</v>
       </c>
       <c r="L241" s="21">
         <f>IF(OR($B241="",$I241=""),"",$I241-IF($K241="",0,$K241))</f>
@@ -15374,7 +15374,7 @@
         <v/>
       </c>
       <c r="K242" s="4" t="n">
-        <v>0</v>
+        <v>398.29</v>
       </c>
       <c r="L242" s="21">
         <f>IF(OR($B242="",$I242=""),"",$I242-IF($K242="",0,$K242))</f>
@@ -15434,7 +15434,7 @@
         <v/>
       </c>
       <c r="K243" s="4" t="n">
-        <v>574.33</v>
+        <v>903.78</v>
       </c>
       <c r="L243" s="21">
         <f>IF(OR($B243="",$I243=""),"",$I243-IF($K243="",0,$K243))</f>
@@ -15494,7 +15494,7 @@
         <v/>
       </c>
       <c r="K244" s="4" t="n">
-        <v>481.35</v>
+        <v>800.77</v>
       </c>
       <c r="L244" s="21">
         <f>IF(OR($B244="",$I244=""),"",$I244-IF($K244="",0,$K244))</f>
@@ -15554,7 +15554,7 @@
         <v/>
       </c>
       <c r="K245" s="4" t="n">
-        <v>481.07</v>
+        <v>762.1</v>
       </c>
       <c r="L245" s="21">
         <f>IF(OR($B245="",$I245=""),"",$I245-IF($K245="",0,$K245))</f>
@@ -15599,8 +15599,12 @@
       <c r="F246" s="26" t="n">
         <v>2805</v>
       </c>
-      <c r="G246" s="24" t="inlineStr"/>
-      <c r="H246" s="25" t="inlineStr"/>
+      <c r="G246" s="24" t="n">
+        <v>46295</v>
+      </c>
+      <c r="H246" s="25" t="n">
+        <v>77.04000000000001</v>
+      </c>
       <c r="I246" s="21">
         <f>IF(OR($B246="",$H246=""),"",IF($C246="LONG",($H246-$E246)*$F246,($E246-$H246)*$F246))</f>
         <v/>
@@ -15610,7 +15614,7 @@
         <v/>
       </c>
       <c r="K246" s="4" t="n">
-        <v>50.15</v>
+        <v>374.49</v>
       </c>
       <c r="L246" s="21">
         <f>IF(OR($B246="",$I246=""),"",$I246-IF($K246="",0,$K246))</f>
@@ -15655,8 +15659,12 @@
       <c r="F247" s="26" t="n">
         <v>788</v>
       </c>
-      <c r="G247" s="24" t="inlineStr"/>
-      <c r="H247" s="25" t="inlineStr"/>
+      <c r="G247" s="24" t="n">
+        <v>46295</v>
+      </c>
+      <c r="H247" s="25" t="n">
+        <v>265.34</v>
+      </c>
       <c r="I247" s="21">
         <f>IF(OR($B247="",$H247=""),"",IF($C247="LONG",($H247-$E247)*$F247,($E247-$H247)*$F247))</f>
         <v/>
@@ -15666,7 +15674,7 @@
         <v/>
       </c>
       <c r="K247" s="4" t="n">
-        <v>50.15</v>
+        <v>373.24</v>
       </c>
       <c r="L247" s="21">
         <f>IF(OR($B247="",$I247=""),"",$I247-IF($K247="",0,$K247))</f>
@@ -15711,8 +15719,12 @@
       <c r="F248" s="26" t="n">
         <v>359</v>
       </c>
-      <c r="G248" s="24" t="inlineStr"/>
-      <c r="H248" s="25" t="inlineStr"/>
+      <c r="G248" s="24" t="n">
+        <v>46295</v>
+      </c>
+      <c r="H248" s="25" t="n">
+        <v>292.46</v>
+      </c>
       <c r="I248" s="21">
         <f>IF(OR($B248="",$H248=""),"",IF($C248="LONG",($H248-$E248)*$F248,($E248-$H248)*$F248))</f>
         <v/>
@@ -15722,7 +15734,7 @@
         <v/>
       </c>
       <c r="K248" s="4" t="n">
-        <v>14.75</v>
+        <v>42.36</v>
       </c>
       <c r="L248" s="21">
         <f>IF(OR($B248="",$I248=""),"",$I248-IF($K248="",0,$K248))</f>
@@ -15767,8 +15779,12 @@
       <c r="F249" s="26" t="n">
         <v>4058</v>
       </c>
-      <c r="G249" s="24" t="inlineStr"/>
-      <c r="H249" s="25" t="inlineStr"/>
+      <c r="G249" s="24" t="n">
+        <v>46295</v>
+      </c>
+      <c r="H249" s="25" t="n">
+        <v>24.94</v>
+      </c>
       <c r="I249" s="21">
         <f>IF(OR($B249="",$H249=""),"",IF($C249="LONG",($H249-$E249)*$F249,($E249-$H249)*$F249))</f>
         <v/>
@@ -15778,7 +15794,7 @@
         <v/>
       </c>
       <c r="K249" s="4" t="n">
-        <v>14.75</v>
+        <v>69.44</v>
       </c>
       <c r="L249" s="21">
         <f>IF(OR($B249="",$I249=""),"",$I249-IF($K249="",0,$K249))</f>
@@ -15823,8 +15839,12 @@
       <c r="F250" s="26" t="n">
         <v>407</v>
       </c>
-      <c r="G250" s="24" t="inlineStr"/>
-      <c r="H250" s="25" t="inlineStr"/>
+      <c r="G250" s="24" t="n">
+        <v>46295</v>
+      </c>
+      <c r="H250" s="25" t="n">
+        <v>545.84</v>
+      </c>
       <c r="I250" s="21">
         <f>IF(OR($B250="",$H250=""),"",IF($C250="LONG",($H250-$E250)*$F250,($E250-$H250)*$F250))</f>
         <v/>
@@ -15834,7 +15854,7 @@
         <v/>
       </c>
       <c r="K250" s="4" t="n">
-        <v>50.15</v>
+        <v>424.47</v>
       </c>
       <c r="L250" s="21">
         <f>IF(OR($B250="",$I250=""),"",$I250-IF($K250="",0,$K250))</f>
@@ -15857,30 +15877,34 @@
     <row r="251">
       <c r="A251" s="23" t="inlineStr">
         <is>
-          <t>DHAN-321260929416409+34126092974109+23126092974809+34126092974409+321260929417209+221260929647409+321260929417509+321260929417709+23126092975309+321260929418309+221260929648809+321260929418709+34126092974809</t>
+          <t>DHAN-32126093049609</t>
         </is>
       </c>
       <c r="B251" s="23" t="inlineStr">
         <is>
-          <t>UNICHEMLAB</t>
+          <t>TCIEXP</t>
         </is>
       </c>
       <c r="C251" s="23" t="inlineStr">
         <is>
-          <t>LONG</t>
+          <t>SHORT</t>
         </is>
       </c>
       <c r="D251" s="24" t="n">
-        <v>46294</v>
+        <v>46295</v>
       </c>
       <c r="E251" s="25" t="n">
-        <v>571.4527</v>
+        <v>547.72</v>
       </c>
       <c r="F251" s="26" t="n">
-        <v>375</v>
-      </c>
-      <c r="G251" s="24" t="inlineStr"/>
-      <c r="H251" s="25" t="inlineStr"/>
+        <v>407</v>
+      </c>
+      <c r="G251" s="24" t="n">
+        <v>46295</v>
+      </c>
+      <c r="H251" s="25" t="n">
+        <v>530.67</v>
+      </c>
       <c r="I251" s="21">
         <f>IF(OR($B251="",$H251=""),"",IF($C251="LONG",($H251-$E251)*$F251,($E251-$H251)*$F251))</f>
         <v/>
@@ -15890,7 +15914,7 @@
         <v/>
       </c>
       <c r="K251" s="4" t="n">
-        <v>50.15</v>
+        <v>0</v>
       </c>
       <c r="L251" s="21">
         <f>IF(OR($B251="",$I251=""),"",$I251-IF($K251="",0,$K251))</f>
@@ -15911,14 +15935,36 @@
       </c>
     </row>
     <row r="252">
-      <c r="A252" s="23" t="n"/>
-      <c r="B252" s="23" t="n"/>
-      <c r="C252" s="23" t="n"/>
-      <c r="D252" s="24" t="n"/>
-      <c r="E252" s="25" t="n"/>
-      <c r="F252" s="26" t="n"/>
-      <c r="G252" s="24" t="n"/>
-      <c r="H252" s="25" t="n"/>
+      <c r="A252" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-321260929416409+34126092974109+23126092974809+34126092974409+321260929417209+221260929647409+321260929417509+321260929417709+23126092975309+321260929418309+221260929648809+321260929418709+34126092974809</t>
+        </is>
+      </c>
+      <c r="B252" s="23" t="inlineStr">
+        <is>
+          <t>UNICHEMLAB</t>
+        </is>
+      </c>
+      <c r="C252" s="23" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="D252" s="24" t="n">
+        <v>46294</v>
+      </c>
+      <c r="E252" s="25" t="n">
+        <v>571.4527</v>
+      </c>
+      <c r="F252" s="26" t="n">
+        <v>375</v>
+      </c>
+      <c r="G252" s="24" t="n">
+        <v>46295</v>
+      </c>
+      <c r="H252" s="25" t="n">
+        <v>566.01</v>
+      </c>
       <c r="I252" s="21">
         <f>IF(OR($B252="",$H252=""),"",IF($C252="LONG",($H252-$E252)*$F252,($E252-$H252)*$F252))</f>
         <v/>
@@ -15927,7 +15973,9 @@
         <f>IF(OR($B252="",$I252="",$E252=0,$F252=0),"",$I252/($E252*$F252))</f>
         <v/>
       </c>
-      <c r="K252" s="4" t="n"/>
+      <c r="K252" s="4" t="n">
+        <v>424.42</v>
+      </c>
       <c r="L252" s="21">
         <f>IF(OR($B252="",$I252=""),"",$I252-IF($K252="",0,$K252))</f>
         <v/>
@@ -15940,17 +15988,39 @@
         <f>IF($B252="","",IF($H252="","Open","Closed"))</f>
         <v/>
       </c>
-      <c r="O252" s="23" t="n"/>
+      <c r="O252" s="23" t="inlineStr">
+        <is>
+          <t>5-10</t>
+        </is>
+      </c>
     </row>
     <row r="253">
-      <c r="A253" s="23" t="n"/>
-      <c r="B253" s="23" t="n"/>
-      <c r="C253" s="23" t="n"/>
-      <c r="D253" s="24" t="n"/>
-      <c r="E253" s="25" t="n"/>
-      <c r="F253" s="26" t="n"/>
-      <c r="G253" s="24" t="n"/>
-      <c r="H253" s="25" t="n"/>
+      <c r="A253" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-321260930406209+321260930406609+221260930616009+321260930406809+23126093060509+321260930407609+221260930618609+34126093061409+321260930408909+23126093060609+34126093061509</t>
+        </is>
+      </c>
+      <c r="B253" s="23" t="inlineStr">
+        <is>
+          <t>DIAMONDYD</t>
+        </is>
+      </c>
+      <c r="C253" s="23" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="D253" s="24" t="n">
+        <v>46295</v>
+      </c>
+      <c r="E253" s="25" t="n">
+        <v>1112.4101</v>
+      </c>
+      <c r="F253" s="26" t="n">
+        <v>338</v>
+      </c>
+      <c r="G253" s="24" t="inlineStr"/>
+      <c r="H253" s="25" t="inlineStr"/>
       <c r="I253" s="21">
         <f>IF(OR($B253="",$H253=""),"",IF($C253="LONG",($H253-$E253)*$F253,($E253-$H253)*$F253))</f>
         <v/>
@@ -15959,7 +16029,9 @@
         <f>IF(OR($B253="",$I253="",$E253=0,$F253=0),"",$I253/($E253*$F253))</f>
         <v/>
       </c>
-      <c r="K253" s="4" t="n"/>
+      <c r="K253" s="4" t="n">
+        <v>50.15</v>
+      </c>
       <c r="L253" s="21">
         <f>IF(OR($B253="",$I253=""),"",$I253-IF($K253="",0,$K253))</f>
         <v/>
@@ -15972,17 +16044,39 @@
         <f>IF($B253="","",IF($H253="","Open","Closed"))</f>
         <v/>
       </c>
-      <c r="O253" s="23" t="n"/>
+      <c r="O253" s="23" t="inlineStr">
+        <is>
+          <t>5-10</t>
+        </is>
+      </c>
     </row>
     <row r="254">
-      <c r="A254" s="23" t="n"/>
-      <c r="B254" s="23" t="n"/>
-      <c r="C254" s="23" t="n"/>
-      <c r="D254" s="24" t="n"/>
-      <c r="E254" s="25" t="n"/>
-      <c r="F254" s="26" t="n"/>
-      <c r="G254" s="24" t="n"/>
-      <c r="H254" s="25" t="n"/>
+      <c r="A254" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-221260930623409</t>
+        </is>
+      </c>
+      <c r="B254" s="23" t="inlineStr">
+        <is>
+          <t>DPABHUSHAN</t>
+        </is>
+      </c>
+      <c r="C254" s="23" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="D254" s="24" t="n">
+        <v>46295</v>
+      </c>
+      <c r="E254" s="25" t="n">
+        <v>1772</v>
+      </c>
+      <c r="F254" s="26" t="n">
+        <v>105</v>
+      </c>
+      <c r="G254" s="24" t="inlineStr"/>
+      <c r="H254" s="25" t="inlineStr"/>
       <c r="I254" s="21">
         <f>IF(OR($B254="",$H254=""),"",IF($C254="LONG",($H254-$E254)*$F254,($E254-$H254)*$F254))</f>
         <v/>
@@ -15991,7 +16085,9 @@
         <f>IF(OR($B254="",$I254="",$E254=0,$F254=0),"",$I254/($E254*$F254))</f>
         <v/>
       </c>
-      <c r="K254" s="4" t="n"/>
+      <c r="K254" s="4" t="n">
+        <v>14.75</v>
+      </c>
       <c r="L254" s="21">
         <f>IF(OR($B254="",$I254=""),"",$I254-IF($K254="",0,$K254))</f>
         <v/>
@@ -16004,7 +16100,11 @@
         <f>IF($B254="","",IF($H254="","Open","Closed"))</f>
         <v/>
       </c>
-      <c r="O254" s="23" t="n"/>
+      <c r="O254" s="23" t="inlineStr">
+        <is>
+          <t>5-10</t>
+        </is>
+      </c>
     </row>
     <row r="255">
       <c r="A255" s="23" t="n"/>
@@ -36649,7 +36749,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J119"/>
+  <dimension ref="A1:J121"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -37421,7 +37521,7 @@
     <row r="20">
       <c r="A20" s="27" t="inlineStr">
         <is>
-          <t>EIEL</t>
+          <t>DIAMONDYD</t>
         </is>
       </c>
       <c r="B20" s="20">
@@ -37464,7 +37564,7 @@
     <row r="21">
       <c r="A21" s="27" t="inlineStr">
         <is>
-          <t>ELECTCAST</t>
+          <t>DPABHUSHAN</t>
         </is>
       </c>
       <c r="B21" s="20">
@@ -37507,7 +37607,7 @@
     <row r="22">
       <c r="A22" s="27" t="inlineStr">
         <is>
-          <t>EMUDHRA</t>
+          <t>EIEL</t>
         </is>
       </c>
       <c r="B22" s="20">
@@ -37550,7 +37650,7 @@
     <row r="23">
       <c r="A23" s="27" t="inlineStr">
         <is>
-          <t>FILATEX</t>
+          <t>ELECTCAST</t>
         </is>
       </c>
       <c r="B23" s="20">
@@ -37593,7 +37693,7 @@
     <row r="24">
       <c r="A24" s="27" t="inlineStr">
         <is>
-          <t>FMGOETZE</t>
+          <t>EMUDHRA</t>
         </is>
       </c>
       <c r="B24" s="20">
@@ -37636,7 +37736,7 @@
     <row r="25">
       <c r="A25" s="27" t="inlineStr">
         <is>
-          <t>FOSECOIND</t>
+          <t>FILATEX</t>
         </is>
       </c>
       <c r="B25" s="20">
@@ -37679,7 +37779,7 @@
     <row r="26">
       <c r="A26" s="27" t="inlineStr">
         <is>
-          <t>FRONTSP</t>
+          <t>FMGOETZE</t>
         </is>
       </c>
       <c r="B26" s="20">
@@ -37722,7 +37822,7 @@
     <row r="27">
       <c r="A27" s="27" t="inlineStr">
         <is>
-          <t>GKENERGY</t>
+          <t>FOSECOIND</t>
         </is>
       </c>
       <c r="B27" s="20">
@@ -37765,7 +37865,7 @@
     <row r="28">
       <c r="A28" s="27" t="inlineStr">
         <is>
-          <t>GNA</t>
+          <t>FRONTSP</t>
         </is>
       </c>
       <c r="B28" s="20">
@@ -37808,7 +37908,7 @@
     <row r="29">
       <c r="A29" s="27" t="inlineStr">
         <is>
-          <t>GNRL</t>
+          <t>GKENERGY</t>
         </is>
       </c>
       <c r="B29" s="20">
@@ -37851,7 +37951,7 @@
     <row r="30">
       <c r="A30" s="27" t="inlineStr">
         <is>
-          <t>GOCLCORP</t>
+          <t>GNA</t>
         </is>
       </c>
       <c r="B30" s="20">
@@ -37894,7 +37994,7 @@
     <row r="31">
       <c r="A31" s="27" t="inlineStr">
         <is>
-          <t>GOPAL</t>
+          <t>GNRL</t>
         </is>
       </c>
       <c r="B31" s="20">
@@ -37937,7 +38037,7 @@
     <row r="32">
       <c r="A32" s="27" t="inlineStr">
         <is>
-          <t>GRAUWEIL</t>
+          <t>GOCLCORP</t>
         </is>
       </c>
       <c r="B32" s="20">
@@ -37980,7 +38080,7 @@
     <row r="33">
       <c r="A33" s="27" t="inlineStr">
         <is>
-          <t>GREAVESCOT</t>
+          <t>GOPAL</t>
         </is>
       </c>
       <c r="B33" s="20">
@@ -38023,7 +38123,7 @@
     <row r="34">
       <c r="A34" s="27" t="inlineStr">
         <is>
-          <t>GUJTHEM</t>
+          <t>GRAUWEIL</t>
         </is>
       </c>
       <c r="B34" s="20">
@@ -38066,7 +38166,7 @@
     <row r="35">
       <c r="A35" s="27" t="inlineStr">
         <is>
-          <t>HERITGFOOD</t>
+          <t>GREAVESCOT</t>
         </is>
       </c>
       <c r="B35" s="20">
@@ -38109,7 +38209,7 @@
     <row r="36">
       <c r="A36" s="27" t="inlineStr">
         <is>
-          <t>HIKAL</t>
+          <t>GUJTHEM</t>
         </is>
       </c>
       <c r="B36" s="20">
@@ -38152,7 +38252,7 @@
     <row r="37">
       <c r="A37" s="27" t="inlineStr">
         <is>
-          <t>HINDOILEXP</t>
+          <t>HERITGFOOD</t>
         </is>
       </c>
       <c r="B37" s="20">
@@ -38195,7 +38295,7 @@
     <row r="38">
       <c r="A38" s="27" t="inlineStr">
         <is>
-          <t>HUBTOWN</t>
+          <t>HIKAL</t>
         </is>
       </c>
       <c r="B38" s="20">
@@ -38238,7 +38338,7 @@
     <row r="39">
       <c r="A39" s="27" t="inlineStr">
         <is>
-          <t>INDIAGLYCO</t>
+          <t>HINDOILEXP</t>
         </is>
       </c>
       <c r="B39" s="20">
@@ -38281,7 +38381,7 @@
     <row r="40">
       <c r="A40" s="27" t="inlineStr">
         <is>
-          <t>INDNIPPON</t>
+          <t>HUBTOWN</t>
         </is>
       </c>
       <c r="B40" s="20">
@@ -38324,7 +38424,7 @@
     <row r="41">
       <c r="A41" s="27" t="inlineStr">
         <is>
-          <t>INDOCO</t>
+          <t>INDIAGLYCO</t>
         </is>
       </c>
       <c r="B41" s="20">
@@ -38367,7 +38467,7 @@
     <row r="42">
       <c r="A42" s="27" t="inlineStr">
         <is>
-          <t>INDORAMA</t>
+          <t>INDNIPPON</t>
         </is>
       </c>
       <c r="B42" s="20">
@@ -38410,7 +38510,7 @@
     <row r="43">
       <c r="A43" s="27" t="inlineStr">
         <is>
-          <t>IPL</t>
+          <t>INDOCO</t>
         </is>
       </c>
       <c r="B43" s="20">
@@ -38453,7 +38553,7 @@
     <row r="44">
       <c r="A44" s="27" t="inlineStr">
         <is>
-          <t>JASH</t>
+          <t>INDORAMA</t>
         </is>
       </c>
       <c r="B44" s="20">
@@ -38496,7 +38596,7 @@
     <row r="45">
       <c r="A45" s="27" t="inlineStr">
         <is>
-          <t>JAYKAY</t>
+          <t>IPL</t>
         </is>
       </c>
       <c r="B45" s="20">
@@ -38539,7 +38639,7 @@
     <row r="46">
       <c r="A46" s="27" t="inlineStr">
         <is>
-          <t>JGCHEM</t>
+          <t>JASH</t>
         </is>
       </c>
       <c r="B46" s="20">
@@ -38582,7 +38682,7 @@
     <row r="47">
       <c r="A47" s="27" t="inlineStr">
         <is>
-          <t>JINDRILL</t>
+          <t>JAYKAY</t>
         </is>
       </c>
       <c r="B47" s="20">
@@ -38625,7 +38725,7 @@
     <row r="48">
       <c r="A48" s="27" t="inlineStr">
         <is>
-          <t>KCP</t>
+          <t>JGCHEM</t>
         </is>
       </c>
       <c r="B48" s="20">
@@ -38668,7 +38768,7 @@
     <row r="49">
       <c r="A49" s="27" t="inlineStr">
         <is>
-          <t>KIRIINDUS</t>
+          <t>JINDRILL</t>
         </is>
       </c>
       <c r="B49" s="20">
@@ -38711,7 +38811,7 @@
     <row r="50">
       <c r="A50" s="27" t="inlineStr">
         <is>
-          <t>KIRLOSIND</t>
+          <t>KCP</t>
         </is>
       </c>
       <c r="B50" s="20">
@@ -38754,7 +38854,7 @@
     <row r="51">
       <c r="A51" s="27" t="inlineStr">
         <is>
-          <t>KLBRENG-B</t>
+          <t>KIRIINDUS</t>
         </is>
       </c>
       <c r="B51" s="20">
@@ -38797,7 +38897,7 @@
     <row r="52">
       <c r="A52" s="27" t="inlineStr">
         <is>
-          <t>KROSS</t>
+          <t>KIRLOSIND</t>
         </is>
       </c>
       <c r="B52" s="20">
@@ -38840,7 +38940,7 @@
     <row r="53">
       <c r="A53" s="27" t="inlineStr">
         <is>
-          <t>KSCL</t>
+          <t>KLBRENG-B</t>
         </is>
       </c>
       <c r="B53" s="20">
@@ -38883,7 +38983,7 @@
     <row r="54">
       <c r="A54" s="27" t="inlineStr">
         <is>
-          <t>KSL</t>
+          <t>KROSS</t>
         </is>
       </c>
       <c r="B54" s="20">
@@ -38926,7 +39026,7 @@
     <row r="55">
       <c r="A55" s="27" t="inlineStr">
         <is>
-          <t>LUXIND</t>
+          <t>KSCL</t>
         </is>
       </c>
       <c r="B55" s="20">
@@ -38969,7 +39069,7 @@
     <row r="56">
       <c r="A56" s="27" t="inlineStr">
         <is>
-          <t>MAITHANALL</t>
+          <t>KSL</t>
         </is>
       </c>
       <c r="B56" s="20">
@@ -39012,7 +39112,7 @@
     <row r="57">
       <c r="A57" s="27" t="inlineStr">
         <is>
-          <t>MANGLMCEM</t>
+          <t>LUXIND</t>
         </is>
       </c>
       <c r="B57" s="20">
@@ -39055,7 +39155,7 @@
     <row r="58">
       <c r="A58" s="27" t="inlineStr">
         <is>
-          <t>MASTEK</t>
+          <t>MAITHANALL</t>
         </is>
       </c>
       <c r="B58" s="20">
@@ -39098,7 +39198,7 @@
     <row r="59">
       <c r="A59" s="27" t="inlineStr">
         <is>
-          <t>MOBIKWIK</t>
+          <t>MANGLMCEM</t>
         </is>
       </c>
       <c r="B59" s="20">
@@ -39141,7 +39241,7 @@
     <row r="60">
       <c r="A60" s="27" t="inlineStr">
         <is>
-          <t>MUKANDLTD</t>
+          <t>MASTEK</t>
         </is>
       </c>
       <c r="B60" s="20">
@@ -39184,7 +39284,7 @@
     <row r="61">
       <c r="A61" s="27" t="inlineStr">
         <is>
-          <t>NETWORK18</t>
+          <t>MOBIKWIK</t>
         </is>
       </c>
       <c r="B61" s="20">
@@ -39227,7 +39327,7 @@
     <row r="62">
       <c r="A62" s="27" t="inlineStr">
         <is>
-          <t>NILKAMAL</t>
+          <t>MUKANDLTD</t>
         </is>
       </c>
       <c r="B62" s="20">
@@ -39270,7 +39370,7 @@
     <row r="63">
       <c r="A63" s="27" t="inlineStr">
         <is>
-          <t>NORTHARC</t>
+          <t>NETWORK18</t>
         </is>
       </c>
       <c r="B63" s="20">
@@ -39313,7 +39413,7 @@
     <row r="64">
       <c r="A64" s="27" t="inlineStr">
         <is>
-          <t>NOVARTIND</t>
+          <t>NILKAMAL</t>
         </is>
       </c>
       <c r="B64" s="20">
@@ -39356,7 +39456,7 @@
     <row r="65">
       <c r="A65" s="27" t="inlineStr">
         <is>
-          <t>NPST</t>
+          <t>NORTHARC</t>
         </is>
       </c>
       <c r="B65" s="20">
@@ -39399,7 +39499,7 @@
     <row r="66">
       <c r="A66" s="27" t="inlineStr">
         <is>
-          <t>NRBBEARING</t>
+          <t>NOVARTIND</t>
         </is>
       </c>
       <c r="B66" s="20">
@@ -39442,7 +39542,7 @@
     <row r="67">
       <c r="A67" s="27" t="inlineStr">
         <is>
-          <t>OMAXE</t>
+          <t>NPST</t>
         </is>
       </c>
       <c r="B67" s="20">
@@ -39485,7 +39585,7 @@
     <row r="68">
       <c r="A68" s="27" t="inlineStr">
         <is>
-          <t>ONEPOINT</t>
+          <t>NRBBEARING</t>
         </is>
       </c>
       <c r="B68" s="20">
@@ -39528,7 +39628,7 @@
     <row r="69">
       <c r="A69" s="27" t="inlineStr">
         <is>
-          <t>OPTIEMUS</t>
+          <t>OMAXE</t>
         </is>
       </c>
       <c r="B69" s="20">
@@ -39571,7 +39671,7 @@
     <row r="70">
       <c r="A70" s="27" t="inlineStr">
         <is>
-          <t>ORIENTHOT</t>
+          <t>ONEPOINT</t>
         </is>
       </c>
       <c r="B70" s="20">
@@ -39614,7 +39714,7 @@
     <row r="71">
       <c r="A71" s="27" t="inlineStr">
         <is>
-          <t>PACEDIGITK</t>
+          <t>OPTIEMUS</t>
         </is>
       </c>
       <c r="B71" s="20">
@@ -39657,7 +39757,7 @@
     <row r="72">
       <c r="A72" s="27" t="inlineStr">
         <is>
-          <t>PITTIENG</t>
+          <t>ORIENTHOT</t>
         </is>
       </c>
       <c r="B72" s="20">
@@ -39700,7 +39800,7 @@
     <row r="73">
       <c r="A73" s="27" t="inlineStr">
         <is>
-          <t>PROTEAN</t>
+          <t>PACEDIGITK</t>
         </is>
       </c>
       <c r="B73" s="20">
@@ -39743,7 +39843,7 @@
     <row r="74">
       <c r="A74" s="27" t="inlineStr">
         <is>
-          <t>QUADFUTURE</t>
+          <t>PITTIENG</t>
         </is>
       </c>
       <c r="B74" s="20">
@@ -39786,7 +39886,7 @@
     <row r="75">
       <c r="A75" s="27" t="inlineStr">
         <is>
-          <t>RACLGEAR</t>
+          <t>PROTEAN</t>
         </is>
       </c>
       <c r="B75" s="20">
@@ -39829,7 +39929,7 @@
     <row r="76">
       <c r="A76" s="27" t="inlineStr">
         <is>
-          <t>RAMRAT</t>
+          <t>QUADFUTURE</t>
         </is>
       </c>
       <c r="B76" s="20">
@@ -39872,7 +39972,7 @@
     <row r="77">
       <c r="A77" s="27" t="inlineStr">
         <is>
-          <t>RAYMOND</t>
+          <t>RACLGEAR</t>
         </is>
       </c>
       <c r="B77" s="20">
@@ -39915,7 +40015,7 @@
     <row r="78">
       <c r="A78" s="27" t="inlineStr">
         <is>
-          <t>RAYMONDREL</t>
+          <t>RAMRAT</t>
         </is>
       </c>
       <c r="B78" s="20">
@@ -39958,7 +40058,7 @@
     <row r="79">
       <c r="A79" s="27" t="inlineStr">
         <is>
-          <t>REFEX</t>
+          <t>RAYMOND</t>
         </is>
       </c>
       <c r="B79" s="20">
@@ -40001,7 +40101,7 @@
     <row r="80">
       <c r="A80" s="27" t="inlineStr">
         <is>
-          <t>RESPONIND</t>
+          <t>RAYMONDREL</t>
         </is>
       </c>
       <c r="B80" s="20">
@@ -40044,7 +40144,7 @@
     <row r="81">
       <c r="A81" s="27" t="inlineStr">
         <is>
-          <t>RML</t>
+          <t>REFEX</t>
         </is>
       </c>
       <c r="B81" s="20">
@@ -40087,7 +40187,7 @@
     <row r="82">
       <c r="A82" s="27" t="inlineStr">
         <is>
-          <t>ROSSTECH</t>
+          <t>RESPONIND</t>
         </is>
       </c>
       <c r="B82" s="20">
@@ -40130,7 +40230,7 @@
     <row r="83">
       <c r="A83" s="27" t="inlineStr">
         <is>
-          <t>RPGLIFE</t>
+          <t>RML</t>
         </is>
       </c>
       <c r="B83" s="20">
@@ -40173,7 +40273,7 @@
     <row r="84">
       <c r="A84" s="27" t="inlineStr">
         <is>
-          <t>RSYSTEMS</t>
+          <t>ROSSTECH</t>
         </is>
       </c>
       <c r="B84" s="20">
@@ -40216,7 +40316,7 @@
     <row r="85">
       <c r="A85" s="27" t="inlineStr">
         <is>
-          <t>SAATVIKGL</t>
+          <t>RPGLIFE</t>
         </is>
       </c>
       <c r="B85" s="20">
@@ -40259,7 +40359,7 @@
     <row r="86">
       <c r="A86" s="27" t="inlineStr">
         <is>
-          <t>SAKAR</t>
+          <t>RSYSTEMS</t>
         </is>
       </c>
       <c r="B86" s="20">
@@ -40302,7 +40402,7 @@
     <row r="87">
       <c r="A87" s="27" t="inlineStr">
         <is>
-          <t>SAMBHV</t>
+          <t>SAATVIKGL</t>
         </is>
       </c>
       <c r="B87" s="20">
@@ -40345,7 +40445,7 @@
     <row r="88">
       <c r="A88" s="27" t="inlineStr">
         <is>
-          <t>SAMHI</t>
+          <t>SAKAR</t>
         </is>
       </c>
       <c r="B88" s="20">
@@ -40388,7 +40488,7 @@
     <row r="89">
       <c r="A89" s="27" t="inlineStr">
         <is>
-          <t>SANGAMIND</t>
+          <t>SAMBHV</t>
         </is>
       </c>
       <c r="B89" s="20">
@@ -40431,7 +40531,7 @@
     <row r="90">
       <c r="A90" s="27" t="inlineStr">
         <is>
-          <t>SDBL</t>
+          <t>SAMHI</t>
         </is>
       </c>
       <c r="B90" s="20">
@@ -40474,7 +40574,7 @@
     <row r="91">
       <c r="A91" s="27" t="inlineStr">
         <is>
-          <t>SHANTIGOLD</t>
+          <t>SANGAMIND</t>
         </is>
       </c>
       <c r="B91" s="20">
@@ -40517,7 +40617,7 @@
     <row r="92">
       <c r="A92" s="27" t="inlineStr">
         <is>
-          <t>SHAREINDIA</t>
+          <t>SDBL</t>
         </is>
       </c>
       <c r="B92" s="20">
@@ -40560,7 +40660,7 @@
     <row r="93">
       <c r="A93" s="27" t="inlineStr">
         <is>
-          <t>SHOPERSTOP</t>
+          <t>SHANTIGOLD</t>
         </is>
       </c>
       <c r="B93" s="20">
@@ -40603,7 +40703,7 @@
     <row r="94">
       <c r="A94" s="27" t="inlineStr">
         <is>
-          <t>SIKA</t>
+          <t>SHAREINDIA</t>
         </is>
       </c>
       <c r="B94" s="20">
@@ -40646,7 +40746,7 @@
     <row r="95">
       <c r="A95" s="27" t="inlineStr">
         <is>
-          <t>SINDHUTRAD</t>
+          <t>SHOPERSTOP</t>
         </is>
       </c>
       <c r="B95" s="20">
@@ -40689,7 +40789,7 @@
     <row r="96">
       <c r="A96" s="27" t="inlineStr">
         <is>
-          <t>SMCGLOBAL</t>
+          <t>SIKA</t>
         </is>
       </c>
       <c r="B96" s="20">
@@ -40732,7 +40832,7 @@
     <row r="97">
       <c r="A97" s="27" t="inlineStr">
         <is>
-          <t>SMSPHARMA</t>
+          <t>SINDHUTRAD</t>
         </is>
       </c>
       <c r="B97" s="20">
@@ -40775,7 +40875,7 @@
     <row r="98">
       <c r="A98" s="27" t="inlineStr">
         <is>
-          <t>SOLARA</t>
+          <t>SMCGLOBAL</t>
         </is>
       </c>
       <c r="B98" s="20">
@@ -40818,7 +40918,7 @@
     <row r="99">
       <c r="A99" s="27" t="inlineStr">
         <is>
-          <t>SOTL</t>
+          <t>SMSPHARMA</t>
         </is>
       </c>
       <c r="B99" s="20">
@@ -40861,7 +40961,7 @@
     <row r="100">
       <c r="A100" s="27" t="inlineStr">
         <is>
-          <t>SSWL</t>
+          <t>SOLARA</t>
         </is>
       </c>
       <c r="B100" s="20">
@@ -40904,7 +41004,7 @@
     <row r="101">
       <c r="A101" s="27" t="inlineStr">
         <is>
-          <t>STEELCAS</t>
+          <t>SOTL</t>
         </is>
       </c>
       <c r="B101" s="20">
@@ -40947,7 +41047,7 @@
     <row r="102">
       <c r="A102" s="27" t="inlineStr">
         <is>
-          <t>SYMPHONY</t>
+          <t>SSWL</t>
         </is>
       </c>
       <c r="B102" s="20">
@@ -40990,7 +41090,7 @@
     <row r="103">
       <c r="A103" s="27" t="inlineStr">
         <is>
-          <t>SYNCOMF</t>
+          <t>STEELCAS</t>
         </is>
       </c>
       <c r="B103" s="20">
@@ -41033,7 +41133,7 @@
     <row r="104">
       <c r="A104" s="27" t="inlineStr">
         <is>
-          <t>TALBROAUTO</t>
+          <t>SYMPHONY</t>
         </is>
       </c>
       <c r="B104" s="20">
@@ -41076,7 +41176,7 @@
     <row r="105">
       <c r="A105" s="27" t="inlineStr">
         <is>
-          <t>TBZ</t>
+          <t>SYNCOMF</t>
         </is>
       </c>
       <c r="B105" s="20">
@@ -41119,7 +41219,7 @@
     <row r="106">
       <c r="A106" s="27" t="inlineStr">
         <is>
-          <t>TCIEXP</t>
+          <t>TALBROAUTO</t>
         </is>
       </c>
       <c r="B106" s="20">
@@ -41162,7 +41262,7 @@
     <row r="107">
       <c r="A107" s="27" t="inlineStr">
         <is>
-          <t>THOMASCOOK</t>
+          <t>TBZ</t>
         </is>
       </c>
       <c r="B107" s="20">
@@ -41205,7 +41305,7 @@
     <row r="108">
       <c r="A108" s="27" t="inlineStr">
         <is>
-          <t>UNICHEMLAB</t>
+          <t>TCIEXP</t>
         </is>
       </c>
       <c r="B108" s="20">
@@ -41248,7 +41348,7 @@
     <row r="109">
       <c r="A109" s="27" t="inlineStr">
         <is>
-          <t>VENKEYS</t>
+          <t>THOMASCOOK</t>
         </is>
       </c>
       <c r="B109" s="20">
@@ -41291,7 +41391,7 @@
     <row r="110">
       <c r="A110" s="27" t="inlineStr">
         <is>
-          <t>VENUSPIPES</t>
+          <t>UNICHEMLAB</t>
         </is>
       </c>
       <c r="B110" s="20">
@@ -41334,7 +41434,7 @@
     <row r="111">
       <c r="A111" s="27" t="inlineStr">
         <is>
-          <t>VERANDA</t>
+          <t>VENKEYS</t>
         </is>
       </c>
       <c r="B111" s="20">
@@ -41377,7 +41477,7 @@
     <row r="112">
       <c r="A112" s="27" t="inlineStr">
         <is>
-          <t>VSSL</t>
+          <t>VENUSPIPES</t>
         </is>
       </c>
       <c r="B112" s="20">
@@ -41420,7 +41520,7 @@
     <row r="113">
       <c r="A113" s="27" t="inlineStr">
         <is>
-          <t>WELSPLSOL</t>
+          <t>VERANDA</t>
         </is>
       </c>
       <c r="B113" s="20">
@@ -41463,7 +41563,7 @@
     <row r="114">
       <c r="A114" s="27" t="inlineStr">
         <is>
-          <t>WENDT</t>
+          <t>VSSL</t>
         </is>
       </c>
       <c r="B114" s="20">
@@ -41506,7 +41606,7 @@
     <row r="115">
       <c r="A115" s="27" t="inlineStr">
         <is>
-          <t>WINDLAS</t>
+          <t>WELSPLSOL</t>
         </is>
       </c>
       <c r="B115" s="20">
@@ -41549,7 +41649,7 @@
     <row r="116">
       <c r="A116" s="27" t="inlineStr">
         <is>
-          <t>XPROINDIA</t>
+          <t>WENDT</t>
         </is>
       </c>
       <c r="B116" s="20">
@@ -41592,7 +41692,7 @@
     <row r="117">
       <c r="A117" s="27" t="inlineStr">
         <is>
-          <t>ZAGGLE</t>
+          <t>WINDLAS</t>
         </is>
       </c>
       <c r="B117" s="20">
@@ -41635,7 +41735,7 @@
     <row r="118">
       <c r="A118" s="27" t="inlineStr">
         <is>
-          <t>ZOTA</t>
+          <t>XPROINDIA</t>
         </is>
       </c>
       <c r="B118" s="20">
@@ -41676,37 +41776,123 @@
       </c>
     </row>
     <row r="119">
-      <c r="A119" s="3" t="inlineStr">
+      <c r="A119" s="27" t="inlineStr">
+        <is>
+          <t>ZAGGLE</t>
+        </is>
+      </c>
+      <c r="B119" s="20">
+        <f>COUNTIF('Trade Log'!$B$4:$B$503,$A119)</f>
+        <v/>
+      </c>
+      <c r="C119" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A119,'Trade Log'!$L$4:$L$503,"&gt;0")</f>
+        <v/>
+      </c>
+      <c r="D119" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A119,'Trade Log'!$L$4:$L$503,"&lt;0")</f>
+        <v/>
+      </c>
+      <c r="E119" s="22">
+        <f>IFERROR($C119/$B119,"")</f>
+        <v/>
+      </c>
+      <c r="F119" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A119,'Trade Log'!$I$4:$I$503)</f>
+        <v/>
+      </c>
+      <c r="G119" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A119,'Trade Log'!$L$4:$L$503)</f>
+        <v/>
+      </c>
+      <c r="H119" s="21">
+        <f>IFERROR($G119/$B119,"")</f>
+        <v/>
+      </c>
+      <c r="I119" s="21">
+        <f>IFERROR(_xlfn.MAXIFS('Trade Log'!$L$4:$L$503,'Trade Log'!$B$4:$B$503,$A119),"")</f>
+        <v/>
+      </c>
+      <c r="J119" s="21">
+        <f>IFERROR(_xlfn.MINIFS('Trade Log'!$L$4:$L$503,'Trade Log'!$B$4:$B$503,$A119),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" s="27" t="inlineStr">
+        <is>
+          <t>ZOTA</t>
+        </is>
+      </c>
+      <c r="B120" s="20">
+        <f>COUNTIF('Trade Log'!$B$4:$B$503,$A120)</f>
+        <v/>
+      </c>
+      <c r="C120" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A120,'Trade Log'!$L$4:$L$503,"&gt;0")</f>
+        <v/>
+      </c>
+      <c r="D120" s="20">
+        <f>COUNTIFS('Trade Log'!$B$4:$B$503,$A120,'Trade Log'!$L$4:$L$503,"&lt;0")</f>
+        <v/>
+      </c>
+      <c r="E120" s="22">
+        <f>IFERROR($C120/$B120,"")</f>
+        <v/>
+      </c>
+      <c r="F120" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A120,'Trade Log'!$I$4:$I$503)</f>
+        <v/>
+      </c>
+      <c r="G120" s="21">
+        <f>SUMIF('Trade Log'!$B$4:$B$503,$A120,'Trade Log'!$L$4:$L$503)</f>
+        <v/>
+      </c>
+      <c r="H120" s="21">
+        <f>IFERROR($G120/$B120,"")</f>
+        <v/>
+      </c>
+      <c r="I120" s="21">
+        <f>IFERROR(_xlfn.MAXIFS('Trade Log'!$L$4:$L$503,'Trade Log'!$B$4:$B$503,$A120),"")</f>
+        <v/>
+      </c>
+      <c r="J120" s="21">
+        <f>IFERROR(_xlfn.MINIFS('Trade Log'!$L$4:$L$503,'Trade Log'!$B$4:$B$503,$A120),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" s="3" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="B119" s="30">
-        <f>SUM(B4:B118)</f>
-        <v/>
-      </c>
-      <c r="C119" s="30">
-        <f>SUM(C4:C118)</f>
-        <v/>
-      </c>
-      <c r="D119" s="30">
-        <f>SUM(D4:D118)</f>
-        <v/>
-      </c>
-      <c r="E119" s="31">
-        <f>IFERROR(C119/B119,"")</f>
-        <v/>
-      </c>
-      <c r="F119" s="32">
-        <f>SUM(F4:F118)</f>
-        <v/>
-      </c>
-      <c r="G119" s="32">
-        <f>SUM(G4:G118)</f>
-        <v/>
-      </c>
-      <c r="H119" s="32">
-        <f>IFERROR(G119/B119,"")</f>
+      <c r="B121" s="30">
+        <f>SUM(B4:B120)</f>
+        <v/>
+      </c>
+      <c r="C121" s="30">
+        <f>SUM(C4:C120)</f>
+        <v/>
+      </c>
+      <c r="D121" s="30">
+        <f>SUM(D4:D120)</f>
+        <v/>
+      </c>
+      <c r="E121" s="31">
+        <f>IFERROR(C121/B121,"")</f>
+        <v/>
+      </c>
+      <c r="F121" s="32">
+        <f>SUM(F4:F120)</f>
+        <v/>
+      </c>
+      <c r="G121" s="32">
+        <f>SUM(G4:G120)</f>
+        <v/>
+      </c>
+      <c r="H121" s="32">
+        <f>IFERROR(G121/B121,"")</f>
         <v/>
       </c>
     </row>
@@ -41725,7 +41911,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N252"/>
+  <dimension ref="A1:N255"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -41874,7 +42060,7 @@
         <v>35.4</v>
       </c>
       <c r="M4" s="4" t="n">
-        <v>107.54</v>
+        <v>106.07</v>
       </c>
       <c r="N4" s="21">
         <f>SUM(E4:M4)</f>
@@ -41976,7 +42162,7 @@
         <v>35.4</v>
       </c>
       <c r="M6" s="4" t="n">
-        <v>150.55</v>
+        <v>148.55</v>
       </c>
       <c r="N6" s="21">
         <f>SUM(E6:M6)</f>
@@ -42078,7 +42264,7 @@
         <v>35.4</v>
       </c>
       <c r="M8" s="4" t="n">
-        <v>107.37</v>
+        <v>105.9</v>
       </c>
       <c r="N8" s="21">
         <f>SUM(E8:M8)</f>
@@ -42180,7 +42366,7 @@
         <v>35.4</v>
       </c>
       <c r="M10" s="4" t="n">
-        <v>128.69</v>
+        <v>126.94</v>
       </c>
       <c r="N10" s="21">
         <f>SUM(E10:M10)</f>
@@ -42282,7 +42468,7 @@
         <v>35.4</v>
       </c>
       <c r="M12" s="4" t="n">
-        <v>126.23</v>
+        <v>124.64</v>
       </c>
       <c r="N12" s="21">
         <f>SUM(E12:M12)</f>
@@ -42384,7 +42570,7 @@
         <v>35.4</v>
       </c>
       <c r="M14" s="4" t="n">
-        <v>59.49</v>
+        <v>58.68</v>
       </c>
       <c r="N14" s="21">
         <f>SUM(E14:M14)</f>
@@ -42486,7 +42672,7 @@
         <v>35.4</v>
       </c>
       <c r="M16" s="4" t="n">
-        <v>71.89</v>
+        <v>70.91</v>
       </c>
       <c r="N16" s="21">
         <f>SUM(E16:M16)</f>
@@ -42588,7 +42774,7 @@
         <v>35.4</v>
       </c>
       <c r="M18" s="4" t="n">
-        <v>43.2</v>
+        <v>42.61</v>
       </c>
       <c r="N18" s="21">
         <f>SUM(E18:M18)</f>
@@ -42690,7 +42876,7 @@
         <v>35.4</v>
       </c>
       <c r="M20" s="4" t="n">
-        <v>71.67</v>
+        <v>70.69</v>
       </c>
       <c r="N20" s="21">
         <f>SUM(E20:M20)</f>
@@ -42792,7 +42978,7 @@
         <v>35.4</v>
       </c>
       <c r="M22" s="4" t="n">
-        <v>78.91</v>
+        <v>77.89</v>
       </c>
       <c r="N22" s="21">
         <f>SUM(E22:M22)</f>
@@ -42894,7 +43080,7 @@
         <v>35.4</v>
       </c>
       <c r="M24" s="4" t="n">
-        <v>72.04000000000001</v>
+        <v>71.06</v>
       </c>
       <c r="N24" s="21">
         <f>SUM(E24:M24)</f>
@@ -42996,7 +43182,7 @@
         <v>35.4</v>
       </c>
       <c r="M26" s="4" t="n">
-        <v>61.39</v>
+        <v>60.55</v>
       </c>
       <c r="N26" s="21">
         <f>SUM(E26:M26)</f>
@@ -43200,7 +43386,7 @@
         <v>35.4</v>
       </c>
       <c r="M30" s="4" t="n">
-        <v>314.43</v>
+        <v>311.04</v>
       </c>
       <c r="N30" s="21">
         <f>SUM(E30:M30)</f>
@@ -43404,7 +43590,7 @@
         <v>35.4</v>
       </c>
       <c r="M34" s="4" t="n">
-        <v>46.99</v>
+        <v>46.98</v>
       </c>
       <c r="N34" s="21">
         <f>SUM(E34:M34)</f>
@@ -43506,7 +43692,7 @@
         <v>35.4</v>
       </c>
       <c r="M36" s="4" t="n">
-        <v>46.98</v>
+        <v>46.97</v>
       </c>
       <c r="N36" s="21">
         <f>SUM(E36:M36)</f>
@@ -43710,7 +43896,7 @@
         <v>35.4</v>
       </c>
       <c r="M40" s="4" t="n">
-        <v>44.83</v>
+        <v>44.86</v>
       </c>
       <c r="N40" s="21">
         <f>SUM(E40:M40)</f>
@@ -43812,7 +43998,7 @@
         <v>35.4</v>
       </c>
       <c r="M42" s="4" t="n">
-        <v>98.38</v>
+        <v>98.36</v>
       </c>
       <c r="N42" s="21">
         <f>SUM(E42:M42)</f>
@@ -43863,7 +44049,7 @@
         <v>35.4</v>
       </c>
       <c r="M43" s="4" t="n">
-        <v>82.05</v>
+        <v>82.04000000000001</v>
       </c>
       <c r="N43" s="21">
         <f>SUM(E43:M43)</f>
@@ -43914,7 +44100,7 @@
         <v>35.4</v>
       </c>
       <c r="M44" s="4" t="n">
-        <v>98.79000000000001</v>
+        <v>98.77</v>
       </c>
       <c r="N44" s="21">
         <f>SUM(E44:M44)</f>
@@ -43965,7 +44151,7 @@
         <v>35.4</v>
       </c>
       <c r="M45" s="4" t="n">
-        <v>157.33</v>
+        <v>157.29</v>
       </c>
       <c r="N45" s="21">
         <f>SUM(E45:M45)</f>
@@ -44067,7 +44253,7 @@
         <v>35.4</v>
       </c>
       <c r="M47" s="4" t="n">
-        <v>157.77</v>
+        <v>157.74</v>
       </c>
       <c r="N47" s="21">
         <f>SUM(E47:M47)</f>
@@ -44169,7 +44355,7 @@
         <v>35.4</v>
       </c>
       <c r="M49" s="4" t="n">
-        <v>171.7</v>
+        <v>171.71</v>
       </c>
       <c r="N49" s="21">
         <f>SUM(E49:M49)</f>
@@ -44271,7 +44457,7 @@
         <v>35.4</v>
       </c>
       <c r="M51" s="4" t="n">
-        <v>156.25</v>
+        <v>156.38</v>
       </c>
       <c r="N51" s="21">
         <f>SUM(E51:M51)</f>
@@ -44373,7 +44559,7 @@
         <v>35.4</v>
       </c>
       <c r="M53" s="4" t="n">
-        <v>132</v>
+        <v>131.97</v>
       </c>
       <c r="N53" s="21">
         <f>SUM(E53:M53)</f>
@@ -44475,7 +44661,7 @@
         <v>35.4</v>
       </c>
       <c r="M55" s="4" t="n">
-        <v>98.86</v>
+        <v>98.87</v>
       </c>
       <c r="N55" s="21">
         <f>SUM(E55:M55)</f>
@@ -44577,7 +44763,7 @@
         <v>35.4</v>
       </c>
       <c r="M57" s="4" t="n">
-        <v>97.03</v>
+        <v>97.06999999999999</v>
       </c>
       <c r="N57" s="21">
         <f>SUM(E57:M57)</f>
@@ -44679,7 +44865,7 @@
         <v>35.4</v>
       </c>
       <c r="M59" s="4" t="n">
-        <v>87.84999999999999</v>
+        <v>87.83</v>
       </c>
       <c r="N59" s="21">
         <f>SUM(E59:M59)</f>
@@ -44883,7 +45069,7 @@
         <v>35.4</v>
       </c>
       <c r="M63" s="4" t="n">
-        <v>78.06</v>
+        <v>78.05</v>
       </c>
       <c r="N63" s="21">
         <f>SUM(E63:M63)</f>
@@ -44985,7 +45171,7 @@
         <v>35.4</v>
       </c>
       <c r="M65" s="4" t="n">
-        <v>85.98999999999999</v>
+        <v>85.97</v>
       </c>
       <c r="N65" s="21">
         <f>SUM(E65:M65)</f>
@@ -45087,7 +45273,7 @@
         <v>35.4</v>
       </c>
       <c r="M67" s="4" t="n">
-        <v>50.12</v>
+        <v>50.14</v>
       </c>
       <c r="N67" s="21">
         <f>SUM(E67:M67)</f>
@@ -45393,7 +45579,7 @@
         <v>35.4</v>
       </c>
       <c r="M73" s="4" t="n">
-        <v>44.3</v>
+        <v>44.29</v>
       </c>
       <c r="N73" s="21">
         <f>SUM(E73:M73)</f>
@@ -45903,7 +46089,7 @@
         <v>35.4</v>
       </c>
       <c r="M83" s="4" t="n">
-        <v>53.72</v>
+        <v>53.71</v>
       </c>
       <c r="N83" s="21">
         <f>SUM(E83:M83)</f>
@@ -46005,7 +46191,7 @@
         <v>35.4</v>
       </c>
       <c r="M85" s="4" t="n">
-        <v>57.51</v>
+        <v>57.55</v>
       </c>
       <c r="N85" s="21">
         <f>SUM(E85:M85)</f>
@@ -46311,7 +46497,7 @@
         <v>35.4</v>
       </c>
       <c r="M91" s="4" t="n">
-        <v>274.37</v>
+        <v>274.34</v>
       </c>
       <c r="N91" s="21">
         <f>SUM(E91:M91)</f>
@@ -46413,7 +46599,7 @@
         <v>35.4</v>
       </c>
       <c r="M93" s="4" t="n">
-        <v>274.45</v>
+        <v>274.42</v>
       </c>
       <c r="N93" s="21">
         <f>SUM(E93:M93)</f>
@@ -46515,7 +46701,7 @@
         <v>35.4</v>
       </c>
       <c r="M95" s="4" t="n">
-        <v>276.19</v>
+        <v>276.16</v>
       </c>
       <c r="N95" s="21">
         <f>SUM(E95:M95)</f>
@@ -46617,7 +46803,7 @@
         <v>35.4</v>
       </c>
       <c r="M97" s="4" t="n">
-        <v>96.90000000000001</v>
+        <v>96.94</v>
       </c>
       <c r="N97" s="21">
         <f>SUM(E97:M97)</f>
@@ -46821,7 +47007,7 @@
         <v>35.4</v>
       </c>
       <c r="M101" s="4" t="n">
-        <v>91.65000000000001</v>
+        <v>91.64</v>
       </c>
       <c r="N101" s="21">
         <f>SUM(E101:M101)</f>
@@ -46923,7 +47109,7 @@
         <v>35.4</v>
       </c>
       <c r="M103" s="4" t="n">
-        <v>91.51000000000001</v>
+        <v>91.5</v>
       </c>
       <c r="N103" s="21">
         <f>SUM(E103:M103)</f>
@@ -47076,7 +47262,7 @@
         <v>35.4</v>
       </c>
       <c r="M106" s="4" t="n">
-        <v>91.75</v>
+        <v>91.73999999999999</v>
       </c>
       <c r="N106" s="21">
         <f>SUM(E106:M106)</f>
@@ -47484,7 +47670,7 @@
         <v>35.4</v>
       </c>
       <c r="M114" s="4" t="n">
-        <v>90.54000000000001</v>
+        <v>90.56999999999999</v>
       </c>
       <c r="N114" s="21">
         <f>SUM(E114:M114)</f>
@@ -47586,7 +47772,7 @@
         <v>35.4</v>
       </c>
       <c r="M116" s="4" t="n">
-        <v>78.44</v>
+        <v>78.43000000000001</v>
       </c>
       <c r="N116" s="21">
         <f>SUM(E116:M116)</f>
@@ -47790,7 +47976,7 @@
         <v>35.4</v>
       </c>
       <c r="M120" s="4" t="n">
-        <v>72.27</v>
+        <v>72.31999999999999</v>
       </c>
       <c r="N120" s="21">
         <f>SUM(E120:M120)</f>
@@ -47892,7 +48078,7 @@
         <v>35.4</v>
       </c>
       <c r="M122" s="4" t="n">
-        <v>109.11</v>
+        <v>109.1</v>
       </c>
       <c r="N122" s="21">
         <f>SUM(E122:M122)</f>
@@ -48096,7 +48282,7 @@
         <v>35.4</v>
       </c>
       <c r="M126" s="4" t="n">
-        <v>70.45999999999999</v>
+        <v>70.41</v>
       </c>
       <c r="N126" s="21">
         <f>SUM(E126:M126)</f>
@@ -48198,7 +48384,7 @@
         <v>35.4</v>
       </c>
       <c r="M128" s="4" t="n">
-        <v>58.73</v>
+        <v>58.72</v>
       </c>
       <c r="N128" s="21">
         <f>SUM(E128:M128)</f>
@@ -48300,7 +48486,7 @@
         <v>35.4</v>
       </c>
       <c r="M130" s="4" t="n">
-        <v>114.09</v>
+        <v>114.07</v>
       </c>
       <c r="N130" s="21">
         <f>SUM(E130:M130)</f>
@@ -48402,7 +48588,7 @@
         <v>35.4</v>
       </c>
       <c r="M132" s="4" t="n">
-        <v>113.94</v>
+        <v>113.93</v>
       </c>
       <c r="N132" s="21">
         <f>SUM(E132:M132)</f>
@@ -48504,7 +48690,7 @@
         <v>35.4</v>
       </c>
       <c r="M134" s="4" t="n">
-        <v>128.29</v>
+        <v>128.36</v>
       </c>
       <c r="N134" s="21">
         <f>SUM(E134:M134)</f>
@@ -48606,7 +48792,7 @@
         <v>35.4</v>
       </c>
       <c r="M136" s="4" t="n">
-        <v>113.45</v>
+        <v>113.44</v>
       </c>
       <c r="N136" s="21">
         <f>SUM(E136:M136)</f>
@@ -48708,7 +48894,7 @@
         <v>35.4</v>
       </c>
       <c r="M138" s="4" t="n">
-        <v>112.39</v>
+        <v>112.37</v>
       </c>
       <c r="N138" s="21">
         <f>SUM(E138:M138)</f>
@@ -48810,7 +48996,7 @@
         <v>35.4</v>
       </c>
       <c r="M140" s="4" t="n">
-        <v>178.51</v>
+        <v>178.49</v>
       </c>
       <c r="N140" s="21">
         <f>SUM(E140:M140)</f>
@@ -49014,7 +49200,7 @@
         <v>35.4</v>
       </c>
       <c r="M144" s="4" t="n">
-        <v>176.87</v>
+        <v>176.85</v>
       </c>
       <c r="N144" s="21">
         <f>SUM(E144:M144)</f>
@@ -49116,7 +49302,7 @@
         <v>35.4</v>
       </c>
       <c r="M146" s="4" t="n">
-        <v>186.28</v>
+        <v>186.35</v>
       </c>
       <c r="N146" s="21">
         <f>SUM(E146:M146)</f>
@@ -49218,7 +49404,7 @@
         <v>35.4</v>
       </c>
       <c r="M148" s="4" t="n">
-        <v>170.97</v>
+        <v>171.1</v>
       </c>
       <c r="N148" s="21">
         <f>SUM(E148:M148)</f>
@@ -49320,7 +49506,7 @@
         <v>35.4</v>
       </c>
       <c r="M150" s="4" t="n">
-        <v>148.28</v>
+        <v>148.26</v>
       </c>
       <c r="N150" s="21">
         <f>SUM(E150:M150)</f>
@@ -49524,7 +49710,7 @@
         <v>35.4</v>
       </c>
       <c r="M154" s="4" t="n">
-        <v>184.32</v>
+        <v>184.24</v>
       </c>
       <c r="N154" s="21">
         <f>SUM(E154:M154)</f>
@@ -49626,7 +49812,7 @@
         <v>35.4</v>
       </c>
       <c r="M156" s="4" t="n">
-        <v>57.33</v>
+        <v>57.29</v>
       </c>
       <c r="N156" s="21">
         <f>SUM(E156:M156)</f>
@@ -49728,7 +49914,7 @@
         <v>35.4</v>
       </c>
       <c r="M158" s="4" t="n">
-        <v>57.45</v>
+        <v>57.44</v>
       </c>
       <c r="N158" s="21">
         <f>SUM(E158:M158)</f>
@@ -49830,7 +50016,7 @@
         <v>35.4</v>
       </c>
       <c r="M160" s="4" t="n">
-        <v>53.01</v>
+        <v>53</v>
       </c>
       <c r="N160" s="21">
         <f>SUM(E160:M160)</f>
@@ -50136,7 +50322,7 @@
         <v>35.4</v>
       </c>
       <c r="M166" s="4" t="n">
-        <v>60.28</v>
+        <v>60.29</v>
       </c>
       <c r="N166" s="21">
         <f>SUM(E166:M166)</f>
@@ -50238,7 +50424,7 @@
         <v>35.4</v>
       </c>
       <c r="M168" s="4" t="n">
-        <v>67.93000000000001</v>
+        <v>67.92</v>
       </c>
       <c r="N168" s="21">
         <f>SUM(E168:M168)</f>
@@ -50340,7 +50526,7 @@
         <v>35.4</v>
       </c>
       <c r="M170" s="4" t="n">
-        <v>79.43000000000001</v>
+        <v>79.42</v>
       </c>
       <c r="N170" s="21">
         <f>SUM(E170:M170)</f>
@@ -50544,7 +50730,7 @@
         <v>35.4</v>
       </c>
       <c r="M174" s="4" t="n">
-        <v>135.75</v>
+        <v>135.81</v>
       </c>
       <c r="N174" s="21">
         <f>SUM(E174:M174)</f>
@@ -50646,7 +50832,7 @@
         <v>35.4</v>
       </c>
       <c r="M176" s="4" t="n">
-        <v>126.34</v>
+        <v>126.33</v>
       </c>
       <c r="N176" s="21">
         <f>SUM(E176:M176)</f>
@@ -50748,7 +50934,7 @@
         <v>35.4</v>
       </c>
       <c r="M178" s="4" t="n">
-        <v>137.33</v>
+        <v>137.32</v>
       </c>
       <c r="N178" s="21">
         <f>SUM(E178:M178)</f>
@@ -50850,7 +51036,7 @@
         <v>35.4</v>
       </c>
       <c r="M180" s="4" t="n">
-        <v>126.84</v>
+        <v>126.83</v>
       </c>
       <c r="N180" s="21">
         <f>SUM(E180:M180)</f>
@@ -50952,7 +51138,7 @@
         <v>35.4</v>
       </c>
       <c r="M182" s="4" t="n">
-        <v>29.23</v>
+        <v>29.22</v>
       </c>
       <c r="N182" s="21">
         <f>SUM(E182:M182)</f>
@@ -51462,7 +51648,7 @@
         <v>35.4</v>
       </c>
       <c r="M192" s="4" t="n">
-        <v>30.06</v>
+        <v>30.08</v>
       </c>
       <c r="N192" s="21">
         <f>SUM(E192:M192)</f>
@@ -51666,7 +51852,7 @@
         <v>35.4</v>
       </c>
       <c r="M196" s="4" t="n">
-        <v>56.21</v>
+        <v>56.23</v>
       </c>
       <c r="N196" s="21">
         <f>SUM(E196:M196)</f>
@@ -51768,7 +51954,7 @@
         <v>35.4</v>
       </c>
       <c r="M198" s="4" t="n">
-        <v>59.94</v>
+        <v>59.97</v>
       </c>
       <c r="N198" s="21">
         <f>SUM(E198:M198)</f>
@@ -51870,7 +52056,7 @@
         <v>35.4</v>
       </c>
       <c r="M200" s="4" t="n">
-        <v>31.75</v>
+        <v>31.74</v>
       </c>
       <c r="N200" s="21">
         <f>SUM(E200:M200)</f>
@@ -52074,7 +52260,7 @@
         <v>35.4</v>
       </c>
       <c r="M204" s="4" t="n">
-        <v>56.08</v>
+        <v>56.1</v>
       </c>
       <c r="N204" s="21">
         <f>SUM(E204:M204)</f>
@@ -52176,7 +52362,7 @@
         <v>35.4</v>
       </c>
       <c r="M206" s="4" t="n">
-        <v>17.61</v>
+        <v>17.6</v>
       </c>
       <c r="N206" s="21">
         <f>SUM(E206:M206)</f>
@@ -52992,7 +53178,7 @@
         <v>35.4</v>
       </c>
       <c r="M222" s="4" t="n">
-        <v>19.21</v>
+        <v>19.19</v>
       </c>
       <c r="N222" s="21">
         <f>SUM(E222:M222)</f>
@@ -53094,7 +53280,7 @@
         <v>35.4</v>
       </c>
       <c r="M224" s="4" t="n">
-        <v>55.06</v>
+        <v>55.09</v>
       </c>
       <c r="N224" s="21">
         <f>SUM(E224:M224)</f>
@@ -53247,7 +53433,7 @@
         <v>35.4</v>
       </c>
       <c r="M227" s="4" t="n">
-        <v>53.93</v>
+        <v>53.95</v>
       </c>
       <c r="N227" s="21">
         <f>SUM(E227:M227)</f>
@@ -53451,7 +53637,7 @@
         <v>35.4</v>
       </c>
       <c r="M231" s="4" t="n">
-        <v>57.23</v>
+        <v>57.18</v>
       </c>
       <c r="N231" s="21">
         <f>SUM(E231:M231)</f>
@@ -53757,7 +53943,7 @@
         <v>35.4</v>
       </c>
       <c r="M237" s="4" t="n">
-        <v>154.73</v>
+        <v>92.84</v>
       </c>
       <c r="N237" s="21">
         <f>SUM(E237:M237)</f>
@@ -53886,22 +54072,22 @@
         <v>46294</v>
       </c>
       <c r="E240" s="4" t="n">
-        <v>20</v>
+        <v>40</v>
       </c>
       <c r="F240" s="4" t="n">
-        <v>299.83</v>
+        <v>588.48</v>
       </c>
       <c r="G240" s="4" t="n">
-        <v>9.199999999999999</v>
+        <v>18.07</v>
       </c>
       <c r="H240" s="4" t="n">
-        <v>0.3</v>
+        <v>0.59</v>
       </c>
       <c r="I240" s="4" t="n">
         <v>44.97</v>
       </c>
       <c r="J240" s="4" t="n">
-        <v>5.31</v>
+        <v>10.56</v>
       </c>
       <c r="K240" s="4" t="n">
         <v>14.75</v>
@@ -53910,7 +54096,7 @@
         <v>35.4</v>
       </c>
       <c r="M240" s="4" t="n">
-        <v>62.93</v>
+        <v>62.9</v>
       </c>
       <c r="N240" s="21">
         <f>SUM(E240:M240)</f>
@@ -53937,22 +54123,22 @@
         <v>46294</v>
       </c>
       <c r="E241" s="4" t="n">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="F241" s="4" t="n">
         <v>0</v>
       </c>
       <c r="G241" s="4" t="n">
-        <v>0</v>
+        <v>9.67</v>
       </c>
       <c r="H241" s="4" t="n">
-        <v>0</v>
+        <v>0.32</v>
       </c>
       <c r="I241" s="4" t="n">
         <v>0</v>
       </c>
       <c r="J241" s="4" t="n">
-        <v>0</v>
+        <v>5.4</v>
       </c>
       <c r="K241" s="4" t="n">
         <v>14.75</v>
@@ -53961,7 +54147,7 @@
         <v>35.4</v>
       </c>
       <c r="M241" s="4" t="n">
-        <v>65.34</v>
+        <v>64.97</v>
       </c>
       <c r="N241" s="21">
         <f>SUM(E241:M241)</f>
@@ -53988,22 +54174,22 @@
         <v>46294</v>
       </c>
       <c r="E242" s="4" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="F242" s="4" t="n">
-        <v>0</v>
+        <v>314.71</v>
       </c>
       <c r="G242" s="4" t="n">
-        <v>0</v>
+        <v>19.41</v>
       </c>
       <c r="H242" s="4" t="n">
-        <v>0</v>
+        <v>0.63</v>
       </c>
       <c r="I242" s="4" t="n">
-        <v>0</v>
+        <v>12.73</v>
       </c>
       <c r="J242" s="4" t="n">
-        <v>0</v>
+        <v>10.81</v>
       </c>
       <c r="K242" s="4" t="n">
         <v>0</v>
@@ -54039,22 +54225,22 @@
         <v>46294</v>
       </c>
       <c r="E243" s="4" t="n">
-        <v>89.91</v>
+        <v>109.91</v>
       </c>
       <c r="F243" s="4" t="n">
-        <v>299.53</v>
+        <v>594.33</v>
       </c>
       <c r="G243" s="4" t="n">
-        <v>9.199999999999999</v>
+        <v>18.23</v>
       </c>
       <c r="H243" s="4" t="n">
-        <v>0.3</v>
+        <v>0.59</v>
       </c>
       <c r="I243" s="4" t="n">
         <v>44.93</v>
       </c>
       <c r="J243" s="4" t="n">
-        <v>17.89</v>
+        <v>23.17</v>
       </c>
       <c r="K243" s="4" t="n">
         <v>14.75</v>
@@ -54063,7 +54249,7 @@
         <v>35.4</v>
       </c>
       <c r="M243" s="4" t="n">
-        <v>62.42</v>
+        <v>62.46</v>
       </c>
       <c r="N243" s="21">
         <f>SUM(E243:M243)</f>
@@ -54090,22 +54276,22 @@
         <v>46294</v>
       </c>
       <c r="E244" s="4" t="n">
-        <v>20</v>
+        <v>40</v>
       </c>
       <c r="F244" s="4" t="n">
-        <v>300.06</v>
+        <v>585.21</v>
       </c>
       <c r="G244" s="4" t="n">
-        <v>9.210000000000001</v>
+        <v>17.96</v>
       </c>
       <c r="H244" s="4" t="n">
-        <v>0.3</v>
+        <v>0.59</v>
       </c>
       <c r="I244" s="4" t="n">
         <v>45.01</v>
       </c>
       <c r="J244" s="4" t="n">
-        <v>5.31</v>
+        <v>10.54</v>
       </c>
       <c r="K244" s="4" t="n">
         <v>14.75</v>
@@ -54141,22 +54327,22 @@
         <v>46294</v>
       </c>
       <c r="E245" s="4" t="n">
-        <v>20</v>
+        <v>60</v>
       </c>
       <c r="F245" s="4" t="n">
-        <v>299.85</v>
+        <v>522.23</v>
       </c>
       <c r="G245" s="4" t="n">
-        <v>9.210000000000001</v>
+        <v>18.6</v>
       </c>
       <c r="H245" s="4" t="n">
-        <v>0.3</v>
+        <v>0.61</v>
       </c>
       <c r="I245" s="4" t="n">
         <v>44.98</v>
       </c>
       <c r="J245" s="4" t="n">
-        <v>5.31</v>
+        <v>14.26</v>
       </c>
       <c r="K245" s="4" t="n">
         <v>14.75</v>
@@ -54188,24 +54374,26 @@
           <t>LONG</t>
         </is>
       </c>
-      <c r="D246" s="24" t="inlineStr"/>
+      <c r="D246" s="24" t="n">
+        <v>46295</v>
+      </c>
       <c r="E246" s="4" t="n">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="F246" s="4" t="n">
-        <v>0</v>
+        <v>214.11</v>
       </c>
       <c r="G246" s="4" t="n">
-        <v>0</v>
+        <v>6.57</v>
       </c>
       <c r="H246" s="4" t="n">
-        <v>0</v>
+        <v>0.21</v>
       </c>
       <c r="I246" s="4" t="n">
-        <v>0</v>
+        <v>32.11</v>
       </c>
       <c r="J246" s="4" t="n">
-        <v>0</v>
+        <v>4.82</v>
       </c>
       <c r="K246" s="4" t="n">
         <v>14.75</v>
@@ -54214,7 +54402,7 @@
         <v>35.4</v>
       </c>
       <c r="M246" s="4" t="n">
-        <v>0</v>
+        <v>46.51</v>
       </c>
       <c r="N246" s="21">
         <f>SUM(E246:M246)</f>
@@ -54237,24 +54425,26 @@
           <t>LONG</t>
         </is>
       </c>
-      <c r="D247" s="24" t="inlineStr"/>
+      <c r="D247" s="24" t="n">
+        <v>46295</v>
+      </c>
       <c r="E247" s="4" t="n">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="F247" s="4" t="n">
-        <v>0</v>
+        <v>214.74</v>
       </c>
       <c r="G247" s="4" t="n">
-        <v>0</v>
+        <v>6.59</v>
       </c>
       <c r="H247" s="4" t="n">
-        <v>0</v>
+        <v>0.21</v>
       </c>
       <c r="I247" s="4" t="n">
-        <v>0</v>
+        <v>32.65</v>
       </c>
       <c r="J247" s="4" t="n">
-        <v>0</v>
+        <v>4.83</v>
       </c>
       <c r="K247" s="4" t="n">
         <v>14.75</v>
@@ -54263,7 +54453,7 @@
         <v>35.4</v>
       </c>
       <c r="M247" s="4" t="n">
-        <v>0</v>
+        <v>44.06</v>
       </c>
       <c r="N247" s="21">
         <f>SUM(E247:M247)</f>
@@ -54286,24 +54476,26 @@
           <t>LONG</t>
         </is>
       </c>
-      <c r="D248" s="24" t="inlineStr"/>
+      <c r="D248" s="24" t="n">
+        <v>46295</v>
+      </c>
       <c r="E248" s="4" t="n">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="F248" s="4" t="n">
         <v>0</v>
       </c>
       <c r="G248" s="4" t="n">
-        <v>0</v>
+        <v>3.29</v>
       </c>
       <c r="H248" s="4" t="n">
-        <v>0</v>
+        <v>0.11</v>
       </c>
       <c r="I248" s="4" t="n">
         <v>0</v>
       </c>
       <c r="J248" s="4" t="n">
-        <v>0</v>
+        <v>4.21</v>
       </c>
       <c r="K248" s="4" t="n">
         <v>14.75</v>
@@ -54335,24 +54527,26 @@
           <t>LONG</t>
         </is>
       </c>
-      <c r="D249" s="24" t="inlineStr"/>
+      <c r="D249" s="24" t="n">
+        <v>46295</v>
+      </c>
       <c r="E249" s="4" t="n">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="F249" s="4" t="n">
-        <v>0</v>
+        <v>23.86</v>
       </c>
       <c r="G249" s="4" t="n">
-        <v>0</v>
+        <v>3.29</v>
       </c>
       <c r="H249" s="4" t="n">
-        <v>0</v>
+        <v>0.11</v>
       </c>
       <c r="I249" s="4" t="n">
-        <v>0</v>
+        <v>3.22</v>
       </c>
       <c r="J249" s="4" t="n">
-        <v>0</v>
+        <v>4.21</v>
       </c>
       <c r="K249" s="4" t="n">
         <v>14.75</v>
@@ -54384,24 +54578,26 @@
           <t>LONG</t>
         </is>
       </c>
-      <c r="D250" s="24" t="inlineStr"/>
+      <c r="D250" s="24" t="n">
+        <v>46295</v>
+      </c>
       <c r="E250" s="4" t="n">
-        <v>0</v>
+        <v>64.29000000000001</v>
       </c>
       <c r="F250" s="4" t="n">
-        <v>0</v>
+        <v>214.31</v>
       </c>
       <c r="G250" s="4" t="n">
-        <v>0</v>
+        <v>6.58</v>
       </c>
       <c r="H250" s="4" t="n">
-        <v>0</v>
+        <v>0.21</v>
       </c>
       <c r="I250" s="4" t="n">
-        <v>0</v>
+        <v>32.15</v>
       </c>
       <c r="J250" s="4" t="n">
-        <v>0</v>
+        <v>12.8</v>
       </c>
       <c r="K250" s="4" t="n">
         <v>14.75</v>
@@ -54410,7 +54606,7 @@
         <v>35.4</v>
       </c>
       <c r="M250" s="4" t="n">
-        <v>0</v>
+        <v>43.98</v>
       </c>
       <c r="N250" s="21">
         <f>SUM(E250:M250)</f>
@@ -54420,20 +54616,22 @@
     <row r="251">
       <c r="A251" s="23" t="inlineStr">
         <is>
-          <t>DHAN-321260929416409+34126092974109+23126092974809+34126092974409+321260929417209+221260929647409+321260929417509+321260929417709+23126092975309+321260929418309+221260929648809+321260929418709+34126092974809</t>
+          <t>DHAN-32126093049609</t>
         </is>
       </c>
       <c r="B251" s="23" t="inlineStr">
         <is>
-          <t>UNICHEMLAB</t>
+          <t>TCIEXP</t>
         </is>
       </c>
       <c r="C251" s="23" t="inlineStr">
         <is>
-          <t>LONG</t>
-        </is>
-      </c>
-      <c r="D251" s="24" t="inlineStr"/>
+          <t>SHORT</t>
+        </is>
+      </c>
+      <c r="D251" s="24" t="n">
+        <v>46295</v>
+      </c>
       <c r="E251" s="4" t="n">
         <v>0</v>
       </c>
@@ -54453,10 +54651,10 @@
         <v>0</v>
       </c>
       <c r="K251" s="4" t="n">
-        <v>14.75</v>
+        <v>0</v>
       </c>
       <c r="L251" s="4" t="n">
-        <v>35.4</v>
+        <v>0</v>
       </c>
       <c r="M251" s="4" t="n">
         <v>0</v>
@@ -54467,54 +54665,203 @@
       </c>
     </row>
     <row r="252">
-      <c r="A252" s="3" t="inlineStr">
+      <c r="A252" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-321260929416409+34126092974109+23126092974809+34126092974409+321260929417209+221260929647409+321260929417509+321260929417709+23126092975309+321260929418309+221260929648809+321260929418709+34126092974809</t>
+        </is>
+      </c>
+      <c r="B252" s="23" t="inlineStr">
+        <is>
+          <t>UNICHEMLAB</t>
+        </is>
+      </c>
+      <c r="C252" s="23" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="D252" s="24" t="n">
+        <v>46295</v>
+      </c>
+      <c r="E252" s="4" t="n">
+        <v>64.28</v>
+      </c>
+      <c r="F252" s="4" t="n">
+        <v>214.29</v>
+      </c>
+      <c r="G252" s="4" t="n">
+        <v>6.58</v>
+      </c>
+      <c r="H252" s="4" t="n">
+        <v>0.21</v>
+      </c>
+      <c r="I252" s="4" t="n">
+        <v>32.14</v>
+      </c>
+      <c r="J252" s="4" t="n">
+        <v>12.79</v>
+      </c>
+      <c r="K252" s="4" t="n">
+        <v>14.75</v>
+      </c>
+      <c r="L252" s="4" t="n">
+        <v>35.4</v>
+      </c>
+      <c r="M252" s="4" t="n">
+        <v>43.97</v>
+      </c>
+      <c r="N252" s="21">
+        <f>SUM(E252:M252)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="253">
+      <c r="A253" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-321260930406209+321260930406609+221260930616009+321260930406809+23126093060509+321260930407609+221260930618609+34126093061409+321260930408909+23126093060609+34126093061509</t>
+        </is>
+      </c>
+      <c r="B253" s="23" t="inlineStr">
+        <is>
+          <t>DIAMONDYD</t>
+        </is>
+      </c>
+      <c r="C253" s="23" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="D253" s="24" t="inlineStr"/>
+      <c r="E253" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F253" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G253" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H253" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I253" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J253" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K253" s="4" t="n">
+        <v>14.75</v>
+      </c>
+      <c r="L253" s="4" t="n">
+        <v>35.4</v>
+      </c>
+      <c r="M253" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="N253" s="21">
+        <f>SUM(E253:M253)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="254">
+      <c r="A254" s="23" t="inlineStr">
+        <is>
+          <t>DHAN-221260930623409</t>
+        </is>
+      </c>
+      <c r="B254" s="23" t="inlineStr">
+        <is>
+          <t>DPABHUSHAN</t>
+        </is>
+      </c>
+      <c r="C254" s="23" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="D254" s="24" t="inlineStr"/>
+      <c r="E254" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F254" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G254" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H254" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I254" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J254" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K254" s="4" t="n">
+        <v>14.75</v>
+      </c>
+      <c r="L254" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="M254" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="N254" s="21">
+        <f>SUM(E254:M254)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="255">
+      <c r="A255" s="3" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="E252" s="32">
-        <f>SUM(E4:E251)</f>
-        <v/>
-      </c>
-      <c r="F252" s="32">
-        <f>SUM(F4:F251)</f>
-        <v/>
-      </c>
-      <c r="G252" s="32">
-        <f>SUM(G4:G251)</f>
-        <v/>
-      </c>
-      <c r="H252" s="32">
-        <f>SUM(H4:H251)</f>
-        <v/>
-      </c>
-      <c r="I252" s="32">
-        <f>SUM(I4:I251)</f>
-        <v/>
-      </c>
-      <c r="J252" s="32">
-        <f>SUM(J4:J251)</f>
-        <v/>
-      </c>
-      <c r="K252" s="32">
-        <f>SUM(K4:K251)</f>
-        <v/>
-      </c>
-      <c r="L252" s="32">
-        <f>SUM(L4:L251)</f>
-        <v/>
-      </c>
-      <c r="M252" s="32">
-        <f>SUM(M4:M251)</f>
-        <v/>
-      </c>
-      <c r="N252" s="32">
-        <f>SUM(N4:N251)</f>
+      <c r="E255" s="32">
+        <f>SUM(E4:E254)</f>
+        <v/>
+      </c>
+      <c r="F255" s="32">
+        <f>SUM(F4:F254)</f>
+        <v/>
+      </c>
+      <c r="G255" s="32">
+        <f>SUM(G4:G254)</f>
+        <v/>
+      </c>
+      <c r="H255" s="32">
+        <f>SUM(H4:H254)</f>
+        <v/>
+      </c>
+      <c r="I255" s="32">
+        <f>SUM(I4:I254)</f>
+        <v/>
+      </c>
+      <c r="J255" s="32">
+        <f>SUM(J4:J254)</f>
+        <v/>
+      </c>
+      <c r="K255" s="32">
+        <f>SUM(K4:K254)</f>
+        <v/>
+      </c>
+      <c r="L255" s="32">
+        <f>SUM(L4:L254)</f>
+        <v/>
+      </c>
+      <c r="M255" s="32">
+        <f>SUM(M4:M254)</f>
+        <v/>
+      </c>
+      <c r="N255" s="32">
+        <f>SUM(N4:N254)</f>
         <v/>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A3:N251"/>
+  <autoFilter ref="A3:N254"/>
   <mergeCells count="2">
     <mergeCell ref="A2:N2"/>
     <mergeCell ref="A1:N1"/>

</xml_diff>

<commit_message>
Data update — 2026-10-01 candle + results refresh
</commit_message>
<xml_diff>
--- a/results/strategy_pnl_simple.xlsx
+++ b/results/strategy_pnl_simple.xlsx
@@ -16019,8 +16019,12 @@
       <c r="F253" s="26" t="n">
         <v>338</v>
       </c>
-      <c r="G253" s="24" t="inlineStr"/>
-      <c r="H253" s="25" t="inlineStr"/>
+      <c r="G253" s="24" t="n">
+        <v>46296</v>
+      </c>
+      <c r="H253" s="25" t="n">
+        <v>1092.88</v>
+      </c>
       <c r="I253" s="21">
         <f>IF(OR($B253="",$H253=""),"",IF($C253="LONG",($H253-$E253)*$F253,($E253-$H253)*$F253))</f>
         <v/>
@@ -16075,8 +16079,12 @@
       <c r="F254" s="26" t="n">
         <v>105</v>
       </c>
-      <c r="G254" s="24" t="inlineStr"/>
-      <c r="H254" s="25" t="inlineStr"/>
+      <c r="G254" s="24" t="n">
+        <v>46296</v>
+      </c>
+      <c r="H254" s="25" t="n">
+        <v>1775.08</v>
+      </c>
       <c r="I254" s="21">
         <f>IF(OR($B254="",$H254=""),"",IF($C254="LONG",($H254-$E254)*$F254,($E254-$H254)*$F254))</f>
         <v/>
@@ -54731,7 +54739,9 @@
           <t>LONG</t>
         </is>
       </c>
-      <c r="D253" s="24" t="inlineStr"/>
+      <c r="D253" s="24" t="n">
+        <v>46296</v>
+      </c>
       <c r="E253" s="4" t="n">
         <v>82.01000000000001</v>
       </c>
@@ -54780,7 +54790,9 @@
           <t>LONG</t>
         </is>
       </c>
-      <c r="D254" s="24" t="inlineStr"/>
+      <c r="D254" s="24" t="n">
+        <v>46296</v>
+      </c>
       <c r="E254" s="4" t="n">
         <v>0</v>
       </c>
@@ -54876,7 +54888,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K18"/>
+  <dimension ref="A1:K19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -55065,167 +55077,169 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="3" t="inlineStr">
+      <c r="A7" s="27" t="inlineStr">
+        <is>
+          <t>2026-10</t>
+        </is>
+      </c>
+      <c r="B7" s="20">
+        <f>COUNTIFS('Trade Log'!$G$4:$G$503,"&gt;="&amp;DATE(2026,10,1),'Trade Log'!$G$4:$G$503,"&lt;"&amp;DATE(2026,11,1))</f>
+        <v/>
+      </c>
+      <c r="C7" s="20">
+        <f>COUNTIFS('Trade Log'!$G$4:$G$503,"&gt;="&amp;DATE(2026,10,1),'Trade Log'!$G$4:$G$503,"&lt;"&amp;DATE(2026,11,1),'Trade Log'!$L$4:$L$503,"&gt;0")</f>
+        <v/>
+      </c>
+      <c r="D7" s="20">
+        <f>COUNTIFS('Trade Log'!$G$4:$G$503,"&gt;="&amp;DATE(2026,10,1),'Trade Log'!$G$4:$G$503,"&lt;"&amp;DATE(2026,11,1),'Trade Log'!$L$4:$L$503,"&lt;0")</f>
+        <v/>
+      </c>
+      <c r="E7" s="22">
+        <f>IFERROR($C7/$B7,"")</f>
+        <v/>
+      </c>
+      <c r="F7" s="21">
+        <f>SUMIFS('Trade Log'!$I$4:$I$503,'Trade Log'!$G$4:$G$503,"&gt;="&amp;DATE(2026,10,1),'Trade Log'!$G$4:$G$503,"&lt;"&amp;DATE(2026,11,1))</f>
+        <v/>
+      </c>
+      <c r="G7" s="21">
+        <f>SUMIFS('Trade Log'!$L$4:$L$503,'Trade Log'!$G$4:$G$503,"&gt;="&amp;DATE(2026,10,1),'Trade Log'!$G$4:$G$503,"&lt;"&amp;DATE(2026,11,1))</f>
+        <v/>
+      </c>
+      <c r="H7" s="21">
+        <f>IFERROR($G7/$B7,"")</f>
+        <v/>
+      </c>
+      <c r="I7" s="21">
+        <f>IFERROR(_xlfn.MAXIFS('Trade Log'!$L$4:$L$503,'Trade Log'!$G$4:$G$503,"&gt;="&amp;DATE(2026,10,1),'Trade Log'!$G$4:$G$503,"&lt;"&amp;DATE(2026,11,1)),"")</f>
+        <v/>
+      </c>
+      <c r="J7" s="21">
+        <f>IFERROR(_xlfn.MINIFS('Trade Log'!$L$4:$L$503,'Trade Log'!$G$4:$G$503,"&gt;="&amp;DATE(2026,10,1),'Trade Log'!$G$4:$G$503,"&lt;"&amp;DATE(2026,11,1)),"")</f>
+        <v/>
+      </c>
+      <c r="K7" s="29">
+        <f>IFERROR(SUMIFS('Trade Log'!$L$4:$L$503,'Trade Log'!$G$4:$G$503,"&gt;="&amp;DATE(2026,10,1),'Trade Log'!$G$4:$G$503,"&lt;"&amp;DATE(2026,11,1),'Trade Log'!$L$4:$L$503,"&gt;0")/ABS(SUMIFS('Trade Log'!$L$4:$L$503,'Trade Log'!$G$4:$G$503,"&gt;="&amp;DATE(2026,10,1),'Trade Log'!$G$4:$G$503,"&lt;"&amp;DATE(2026,11,1),'Trade Log'!$L$4:$L$503,"&lt;0")),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="3" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="B7" s="30">
-        <f>SUM(B5:B6)</f>
-        <v/>
-      </c>
-      <c r="C7" s="30">
-        <f>SUM(C5:C6)</f>
-        <v/>
-      </c>
-      <c r="D7" s="30">
-        <f>SUM(D5:D6)</f>
-        <v/>
-      </c>
-      <c r="E7" s="31">
-        <f>IFERROR(C7/B7,"")</f>
-        <v/>
-      </c>
-      <c r="F7" s="32">
-        <f>SUM(F5:F6)</f>
-        <v/>
-      </c>
-      <c r="G7" s="32">
-        <f>SUM(G5:G6)</f>
-        <v/>
-      </c>
-      <c r="H7" s="32">
-        <f>IFERROR(G7/B7,"")</f>
-        <v/>
-      </c>
-      <c r="K7" s="33">
+      <c r="B8" s="30">
+        <f>SUM(B5:B7)</f>
+        <v/>
+      </c>
+      <c r="C8" s="30">
+        <f>SUM(C5:C7)</f>
+        <v/>
+      </c>
+      <c r="D8" s="30">
+        <f>SUM(D5:D7)</f>
+        <v/>
+      </c>
+      <c r="E8" s="31">
+        <f>IFERROR(C8/B8,"")</f>
+        <v/>
+      </c>
+      <c r="F8" s="32">
+        <f>SUM(F5:F7)</f>
+        <v/>
+      </c>
+      <c r="G8" s="32">
+        <f>SUM(G5:G7)</f>
+        <v/>
+      </c>
+      <c r="H8" s="32">
+        <f>IFERROR(G8/B8,"")</f>
+        <v/>
+      </c>
+      <c r="K8" s="33">
         <f>IFERROR(SUMIF('Trade Log'!$L$4:$L$503,"&gt;0")/ABS(SUMIF('Trade Log'!$L$4:$L$503,"&lt;0")),"")</f>
         <v/>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" s="3" t="inlineStr">
+    <row r="10">
+      <c r="A10" s="3" t="inlineStr">
         <is>
           <t>WEEKLY PnL</t>
         </is>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" s="19" t="inlineStr">
+    <row r="11">
+      <c r="A11" s="19" t="inlineStr">
         <is>
           <t>Period</t>
         </is>
       </c>
-      <c r="B10" s="19" t="inlineStr">
+      <c r="B11" s="19" t="inlineStr">
         <is>
           <t>Trades</t>
         </is>
       </c>
-      <c r="C10" s="19" t="inlineStr">
+      <c r="C11" s="19" t="inlineStr">
         <is>
           <t>Wins</t>
         </is>
       </c>
-      <c r="D10" s="19" t="inlineStr">
+      <c r="D11" s="19" t="inlineStr">
         <is>
           <t>Losses</t>
         </is>
       </c>
-      <c r="E10" s="19" t="inlineStr">
+      <c r="E11" s="19" t="inlineStr">
         <is>
           <t>Win Rate</t>
         </is>
       </c>
-      <c r="F10" s="19" t="inlineStr">
+      <c r="F11" s="19" t="inlineStr">
         <is>
           <t>Gross P&amp;L</t>
         </is>
       </c>
-      <c r="G10" s="19" t="inlineStr">
+      <c r="G11" s="19" t="inlineStr">
         <is>
           <t>Net P&amp;L</t>
         </is>
       </c>
-      <c r="H10" s="19" t="inlineStr">
+      <c r="H11" s="19" t="inlineStr">
         <is>
           <t>Avg Net P&amp;L / Trade</t>
         </is>
       </c>
-      <c r="I10" s="19" t="inlineStr">
+      <c r="I11" s="19" t="inlineStr">
         <is>
           <t>Best Trade</t>
         </is>
       </c>
-      <c r="J10" s="19" t="inlineStr">
+      <c r="J11" s="19" t="inlineStr">
         <is>
           <t>Worst Trade</t>
         </is>
       </c>
-      <c r="K10" s="19" t="inlineStr">
+      <c r="K11" s="19" t="inlineStr">
         <is>
           <t>Profit Factor</t>
         </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="28" t="n">
-        <v>46251</v>
-      </c>
-      <c r="B11" s="20">
-        <f>COUNTIFS('Trade Log'!$G$4:$G$503,"&gt;="&amp;DATE(2026,8,17),'Trade Log'!$G$4:$G$503,"&lt;"&amp;DATE(2026,8,24))</f>
-        <v/>
-      </c>
-      <c r="C11" s="20">
-        <f>COUNTIFS('Trade Log'!$G$4:$G$503,"&gt;="&amp;DATE(2026,8,17),'Trade Log'!$G$4:$G$503,"&lt;"&amp;DATE(2026,8,24),'Trade Log'!$L$4:$L$503,"&gt;0")</f>
-        <v/>
-      </c>
-      <c r="D11" s="20">
-        <f>COUNTIFS('Trade Log'!$G$4:$G$503,"&gt;="&amp;DATE(2026,8,17),'Trade Log'!$G$4:$G$503,"&lt;"&amp;DATE(2026,8,24),'Trade Log'!$L$4:$L$503,"&lt;0")</f>
-        <v/>
-      </c>
-      <c r="E11" s="22">
-        <f>IFERROR($C11/$B11,"")</f>
-        <v/>
-      </c>
-      <c r="F11" s="21">
-        <f>SUMIFS('Trade Log'!$I$4:$I$503,'Trade Log'!$G$4:$G$503,"&gt;="&amp;DATE(2026,8,17),'Trade Log'!$G$4:$G$503,"&lt;"&amp;DATE(2026,8,24))</f>
-        <v/>
-      </c>
-      <c r="G11" s="21">
-        <f>SUMIFS('Trade Log'!$L$4:$L$503,'Trade Log'!$G$4:$G$503,"&gt;="&amp;DATE(2026,8,17),'Trade Log'!$G$4:$G$503,"&lt;"&amp;DATE(2026,8,24))</f>
-        <v/>
-      </c>
-      <c r="H11" s="21">
-        <f>IFERROR($G11/$B11,"")</f>
-        <v/>
-      </c>
-      <c r="I11" s="21">
-        <f>IFERROR(_xlfn.MAXIFS('Trade Log'!$L$4:$L$503,'Trade Log'!$G$4:$G$503,"&gt;="&amp;DATE(2026,8,17),'Trade Log'!$G$4:$G$503,"&lt;"&amp;DATE(2026,8,24)),"")</f>
-        <v/>
-      </c>
-      <c r="J11" s="21">
-        <f>IFERROR(_xlfn.MINIFS('Trade Log'!$L$4:$L$503,'Trade Log'!$G$4:$G$503,"&gt;="&amp;DATE(2026,8,17),'Trade Log'!$G$4:$G$503,"&lt;"&amp;DATE(2026,8,24)),"")</f>
-        <v/>
-      </c>
-      <c r="K11" s="29">
-        <f>IFERROR(SUMIFS('Trade Log'!$L$4:$L$503,'Trade Log'!$G$4:$G$503,"&gt;="&amp;DATE(2026,8,17),'Trade Log'!$G$4:$G$503,"&lt;"&amp;DATE(2026,8,24),'Trade Log'!$L$4:$L$503,"&gt;0")/ABS(SUMIFS('Trade Log'!$L$4:$L$503,'Trade Log'!$G$4:$G$503,"&gt;="&amp;DATE(2026,8,17),'Trade Log'!$G$4:$G$503,"&lt;"&amp;DATE(2026,8,24),'Trade Log'!$L$4:$L$503,"&lt;0")),"")</f>
-        <v/>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="28" t="n">
-        <v>46258</v>
+        <v>46251</v>
       </c>
       <c r="B12" s="20">
-        <f>COUNTIFS('Trade Log'!$G$4:$G$503,"&gt;="&amp;DATE(2026,8,24),'Trade Log'!$G$4:$G$503,"&lt;"&amp;DATE(2026,8,31))</f>
+        <f>COUNTIFS('Trade Log'!$G$4:$G$503,"&gt;="&amp;DATE(2026,8,17),'Trade Log'!$G$4:$G$503,"&lt;"&amp;DATE(2026,8,24))</f>
         <v/>
       </c>
       <c r="C12" s="20">
-        <f>COUNTIFS('Trade Log'!$G$4:$G$503,"&gt;="&amp;DATE(2026,8,24),'Trade Log'!$G$4:$G$503,"&lt;"&amp;DATE(2026,8,31),'Trade Log'!$L$4:$L$503,"&gt;0")</f>
+        <f>COUNTIFS('Trade Log'!$G$4:$G$503,"&gt;="&amp;DATE(2026,8,17),'Trade Log'!$G$4:$G$503,"&lt;"&amp;DATE(2026,8,24),'Trade Log'!$L$4:$L$503,"&gt;0")</f>
         <v/>
       </c>
       <c r="D12" s="20">
-        <f>COUNTIFS('Trade Log'!$G$4:$G$503,"&gt;="&amp;DATE(2026,8,24),'Trade Log'!$G$4:$G$503,"&lt;"&amp;DATE(2026,8,31),'Trade Log'!$L$4:$L$503,"&lt;0")</f>
+        <f>COUNTIFS('Trade Log'!$G$4:$G$503,"&gt;="&amp;DATE(2026,8,17),'Trade Log'!$G$4:$G$503,"&lt;"&amp;DATE(2026,8,24),'Trade Log'!$L$4:$L$503,"&lt;0")</f>
         <v/>
       </c>
       <c r="E12" s="22">
@@ -55233,11 +55247,11 @@
         <v/>
       </c>
       <c r="F12" s="21">
-        <f>SUMIFS('Trade Log'!$I$4:$I$503,'Trade Log'!$G$4:$G$503,"&gt;="&amp;DATE(2026,8,24),'Trade Log'!$G$4:$G$503,"&lt;"&amp;DATE(2026,8,31))</f>
+        <f>SUMIFS('Trade Log'!$I$4:$I$503,'Trade Log'!$G$4:$G$503,"&gt;="&amp;DATE(2026,8,17),'Trade Log'!$G$4:$G$503,"&lt;"&amp;DATE(2026,8,24))</f>
         <v/>
       </c>
       <c r="G12" s="21">
-        <f>SUMIFS('Trade Log'!$L$4:$L$503,'Trade Log'!$G$4:$G$503,"&gt;="&amp;DATE(2026,8,24),'Trade Log'!$G$4:$G$503,"&lt;"&amp;DATE(2026,8,31))</f>
+        <f>SUMIFS('Trade Log'!$L$4:$L$503,'Trade Log'!$G$4:$G$503,"&gt;="&amp;DATE(2026,8,17),'Trade Log'!$G$4:$G$503,"&lt;"&amp;DATE(2026,8,24))</f>
         <v/>
       </c>
       <c r="H12" s="21">
@@ -55245,32 +55259,32 @@
         <v/>
       </c>
       <c r="I12" s="21">
-        <f>IFERROR(_xlfn.MAXIFS('Trade Log'!$L$4:$L$503,'Trade Log'!$G$4:$G$503,"&gt;="&amp;DATE(2026,8,24),'Trade Log'!$G$4:$G$503,"&lt;"&amp;DATE(2026,8,31)),"")</f>
+        <f>IFERROR(_xlfn.MAXIFS('Trade Log'!$L$4:$L$503,'Trade Log'!$G$4:$G$503,"&gt;="&amp;DATE(2026,8,17),'Trade Log'!$G$4:$G$503,"&lt;"&amp;DATE(2026,8,24)),"")</f>
         <v/>
       </c>
       <c r="J12" s="21">
-        <f>IFERROR(_xlfn.MINIFS('Trade Log'!$L$4:$L$503,'Trade Log'!$G$4:$G$503,"&gt;="&amp;DATE(2026,8,24),'Trade Log'!$G$4:$G$503,"&lt;"&amp;DATE(2026,8,31)),"")</f>
+        <f>IFERROR(_xlfn.MINIFS('Trade Log'!$L$4:$L$503,'Trade Log'!$G$4:$G$503,"&gt;="&amp;DATE(2026,8,17),'Trade Log'!$G$4:$G$503,"&lt;"&amp;DATE(2026,8,24)),"")</f>
         <v/>
       </c>
       <c r="K12" s="29">
-        <f>IFERROR(SUMIFS('Trade Log'!$L$4:$L$503,'Trade Log'!$G$4:$G$503,"&gt;="&amp;DATE(2026,8,24),'Trade Log'!$G$4:$G$503,"&lt;"&amp;DATE(2026,8,31),'Trade Log'!$L$4:$L$503,"&gt;0")/ABS(SUMIFS('Trade Log'!$L$4:$L$503,'Trade Log'!$G$4:$G$503,"&gt;="&amp;DATE(2026,8,24),'Trade Log'!$G$4:$G$503,"&lt;"&amp;DATE(2026,8,31),'Trade Log'!$L$4:$L$503,"&lt;0")),"")</f>
+        <f>IFERROR(SUMIFS('Trade Log'!$L$4:$L$503,'Trade Log'!$G$4:$G$503,"&gt;="&amp;DATE(2026,8,17),'Trade Log'!$G$4:$G$503,"&lt;"&amp;DATE(2026,8,24),'Trade Log'!$L$4:$L$503,"&gt;0")/ABS(SUMIFS('Trade Log'!$L$4:$L$503,'Trade Log'!$G$4:$G$503,"&gt;="&amp;DATE(2026,8,17),'Trade Log'!$G$4:$G$503,"&lt;"&amp;DATE(2026,8,24),'Trade Log'!$L$4:$L$503,"&lt;0")),"")</f>
         <v/>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="28" t="n">
-        <v>46265</v>
+        <v>46258</v>
       </c>
       <c r="B13" s="20">
-        <f>COUNTIFS('Trade Log'!$G$4:$G$503,"&gt;="&amp;DATE(2026,8,31),'Trade Log'!$G$4:$G$503,"&lt;"&amp;DATE(2026,9,7))</f>
+        <f>COUNTIFS('Trade Log'!$G$4:$G$503,"&gt;="&amp;DATE(2026,8,24),'Trade Log'!$G$4:$G$503,"&lt;"&amp;DATE(2026,8,31))</f>
         <v/>
       </c>
       <c r="C13" s="20">
-        <f>COUNTIFS('Trade Log'!$G$4:$G$503,"&gt;="&amp;DATE(2026,8,31),'Trade Log'!$G$4:$G$503,"&lt;"&amp;DATE(2026,9,7),'Trade Log'!$L$4:$L$503,"&gt;0")</f>
+        <f>COUNTIFS('Trade Log'!$G$4:$G$503,"&gt;="&amp;DATE(2026,8,24),'Trade Log'!$G$4:$G$503,"&lt;"&amp;DATE(2026,8,31),'Trade Log'!$L$4:$L$503,"&gt;0")</f>
         <v/>
       </c>
       <c r="D13" s="20">
-        <f>COUNTIFS('Trade Log'!$G$4:$G$503,"&gt;="&amp;DATE(2026,8,31),'Trade Log'!$G$4:$G$503,"&lt;"&amp;DATE(2026,9,7),'Trade Log'!$L$4:$L$503,"&lt;0")</f>
+        <f>COUNTIFS('Trade Log'!$G$4:$G$503,"&gt;="&amp;DATE(2026,8,24),'Trade Log'!$G$4:$G$503,"&lt;"&amp;DATE(2026,8,31),'Trade Log'!$L$4:$L$503,"&lt;0")</f>
         <v/>
       </c>
       <c r="E13" s="22">
@@ -55278,11 +55292,11 @@
         <v/>
       </c>
       <c r="F13" s="21">
-        <f>SUMIFS('Trade Log'!$I$4:$I$503,'Trade Log'!$G$4:$G$503,"&gt;="&amp;DATE(2026,8,31),'Trade Log'!$G$4:$G$503,"&lt;"&amp;DATE(2026,9,7))</f>
+        <f>SUMIFS('Trade Log'!$I$4:$I$503,'Trade Log'!$G$4:$G$503,"&gt;="&amp;DATE(2026,8,24),'Trade Log'!$G$4:$G$503,"&lt;"&amp;DATE(2026,8,31))</f>
         <v/>
       </c>
       <c r="G13" s="21">
-        <f>SUMIFS('Trade Log'!$L$4:$L$503,'Trade Log'!$G$4:$G$503,"&gt;="&amp;DATE(2026,8,31),'Trade Log'!$G$4:$G$503,"&lt;"&amp;DATE(2026,9,7))</f>
+        <f>SUMIFS('Trade Log'!$L$4:$L$503,'Trade Log'!$G$4:$G$503,"&gt;="&amp;DATE(2026,8,24),'Trade Log'!$G$4:$G$503,"&lt;"&amp;DATE(2026,8,31))</f>
         <v/>
       </c>
       <c r="H13" s="21">
@@ -55290,32 +55304,32 @@
         <v/>
       </c>
       <c r="I13" s="21">
-        <f>IFERROR(_xlfn.MAXIFS('Trade Log'!$L$4:$L$503,'Trade Log'!$G$4:$G$503,"&gt;="&amp;DATE(2026,8,31),'Trade Log'!$G$4:$G$503,"&lt;"&amp;DATE(2026,9,7)),"")</f>
+        <f>IFERROR(_xlfn.MAXIFS('Trade Log'!$L$4:$L$503,'Trade Log'!$G$4:$G$503,"&gt;="&amp;DATE(2026,8,24),'Trade Log'!$G$4:$G$503,"&lt;"&amp;DATE(2026,8,31)),"")</f>
         <v/>
       </c>
       <c r="J13" s="21">
-        <f>IFERROR(_xlfn.MINIFS('Trade Log'!$L$4:$L$503,'Trade Log'!$G$4:$G$503,"&gt;="&amp;DATE(2026,8,31),'Trade Log'!$G$4:$G$503,"&lt;"&amp;DATE(2026,9,7)),"")</f>
+        <f>IFERROR(_xlfn.MINIFS('Trade Log'!$L$4:$L$503,'Trade Log'!$G$4:$G$503,"&gt;="&amp;DATE(2026,8,24),'Trade Log'!$G$4:$G$503,"&lt;"&amp;DATE(2026,8,31)),"")</f>
         <v/>
       </c>
       <c r="K13" s="29">
-        <f>IFERROR(SUMIFS('Trade Log'!$L$4:$L$503,'Trade Log'!$G$4:$G$503,"&gt;="&amp;DATE(2026,8,31),'Trade Log'!$G$4:$G$503,"&lt;"&amp;DATE(2026,9,7),'Trade Log'!$L$4:$L$503,"&gt;0")/ABS(SUMIFS('Trade Log'!$L$4:$L$503,'Trade Log'!$G$4:$G$503,"&gt;="&amp;DATE(2026,8,31),'Trade Log'!$G$4:$G$503,"&lt;"&amp;DATE(2026,9,7),'Trade Log'!$L$4:$L$503,"&lt;0")),"")</f>
+        <f>IFERROR(SUMIFS('Trade Log'!$L$4:$L$503,'Trade Log'!$G$4:$G$503,"&gt;="&amp;DATE(2026,8,24),'Trade Log'!$G$4:$G$503,"&lt;"&amp;DATE(2026,8,31),'Trade Log'!$L$4:$L$503,"&gt;0")/ABS(SUMIFS('Trade Log'!$L$4:$L$503,'Trade Log'!$G$4:$G$503,"&gt;="&amp;DATE(2026,8,24),'Trade Log'!$G$4:$G$503,"&lt;"&amp;DATE(2026,8,31),'Trade Log'!$L$4:$L$503,"&lt;0")),"")</f>
         <v/>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="28" t="n">
-        <v>46272</v>
+        <v>46265</v>
       </c>
       <c r="B14" s="20">
-        <f>COUNTIFS('Trade Log'!$G$4:$G$503,"&gt;="&amp;DATE(2026,9,7),'Trade Log'!$G$4:$G$503,"&lt;"&amp;DATE(2026,9,14))</f>
+        <f>COUNTIFS('Trade Log'!$G$4:$G$503,"&gt;="&amp;DATE(2026,8,31),'Trade Log'!$G$4:$G$503,"&lt;"&amp;DATE(2026,9,7))</f>
         <v/>
       </c>
       <c r="C14" s="20">
-        <f>COUNTIFS('Trade Log'!$G$4:$G$503,"&gt;="&amp;DATE(2026,9,7),'Trade Log'!$G$4:$G$503,"&lt;"&amp;DATE(2026,9,14),'Trade Log'!$L$4:$L$503,"&gt;0")</f>
+        <f>COUNTIFS('Trade Log'!$G$4:$G$503,"&gt;="&amp;DATE(2026,8,31),'Trade Log'!$G$4:$G$503,"&lt;"&amp;DATE(2026,9,7),'Trade Log'!$L$4:$L$503,"&gt;0")</f>
         <v/>
       </c>
       <c r="D14" s="20">
-        <f>COUNTIFS('Trade Log'!$G$4:$G$503,"&gt;="&amp;DATE(2026,9,7),'Trade Log'!$G$4:$G$503,"&lt;"&amp;DATE(2026,9,14),'Trade Log'!$L$4:$L$503,"&lt;0")</f>
+        <f>COUNTIFS('Trade Log'!$G$4:$G$503,"&gt;="&amp;DATE(2026,8,31),'Trade Log'!$G$4:$G$503,"&lt;"&amp;DATE(2026,9,7),'Trade Log'!$L$4:$L$503,"&lt;0")</f>
         <v/>
       </c>
       <c r="E14" s="22">
@@ -55323,11 +55337,11 @@
         <v/>
       </c>
       <c r="F14" s="21">
-        <f>SUMIFS('Trade Log'!$I$4:$I$503,'Trade Log'!$G$4:$G$503,"&gt;="&amp;DATE(2026,9,7),'Trade Log'!$G$4:$G$503,"&lt;"&amp;DATE(2026,9,14))</f>
+        <f>SUMIFS('Trade Log'!$I$4:$I$503,'Trade Log'!$G$4:$G$503,"&gt;="&amp;DATE(2026,8,31),'Trade Log'!$G$4:$G$503,"&lt;"&amp;DATE(2026,9,7))</f>
         <v/>
       </c>
       <c r="G14" s="21">
-        <f>SUMIFS('Trade Log'!$L$4:$L$503,'Trade Log'!$G$4:$G$503,"&gt;="&amp;DATE(2026,9,7),'Trade Log'!$G$4:$G$503,"&lt;"&amp;DATE(2026,9,14))</f>
+        <f>SUMIFS('Trade Log'!$L$4:$L$503,'Trade Log'!$G$4:$G$503,"&gt;="&amp;DATE(2026,8,31),'Trade Log'!$G$4:$G$503,"&lt;"&amp;DATE(2026,9,7))</f>
         <v/>
       </c>
       <c r="H14" s="21">
@@ -55335,32 +55349,32 @@
         <v/>
       </c>
       <c r="I14" s="21">
-        <f>IFERROR(_xlfn.MAXIFS('Trade Log'!$L$4:$L$503,'Trade Log'!$G$4:$G$503,"&gt;="&amp;DATE(2026,9,7),'Trade Log'!$G$4:$G$503,"&lt;"&amp;DATE(2026,9,14)),"")</f>
+        <f>IFERROR(_xlfn.MAXIFS('Trade Log'!$L$4:$L$503,'Trade Log'!$G$4:$G$503,"&gt;="&amp;DATE(2026,8,31),'Trade Log'!$G$4:$G$503,"&lt;"&amp;DATE(2026,9,7)),"")</f>
         <v/>
       </c>
       <c r="J14" s="21">
-        <f>IFERROR(_xlfn.MINIFS('Trade Log'!$L$4:$L$503,'Trade Log'!$G$4:$G$503,"&gt;="&amp;DATE(2026,9,7),'Trade Log'!$G$4:$G$503,"&lt;"&amp;DATE(2026,9,14)),"")</f>
+        <f>IFERROR(_xlfn.MINIFS('Trade Log'!$L$4:$L$503,'Trade Log'!$G$4:$G$503,"&gt;="&amp;DATE(2026,8,31),'Trade Log'!$G$4:$G$503,"&lt;"&amp;DATE(2026,9,7)),"")</f>
         <v/>
       </c>
       <c r="K14" s="29">
-        <f>IFERROR(SUMIFS('Trade Log'!$L$4:$L$503,'Trade Log'!$G$4:$G$503,"&gt;="&amp;DATE(2026,9,7),'Trade Log'!$G$4:$G$503,"&lt;"&amp;DATE(2026,9,14),'Trade Log'!$L$4:$L$503,"&gt;0")/ABS(SUMIFS('Trade Log'!$L$4:$L$503,'Trade Log'!$G$4:$G$503,"&gt;="&amp;DATE(2026,9,7),'Trade Log'!$G$4:$G$503,"&lt;"&amp;DATE(2026,9,14),'Trade Log'!$L$4:$L$503,"&lt;0")),"")</f>
+        <f>IFERROR(SUMIFS('Trade Log'!$L$4:$L$503,'Trade Log'!$G$4:$G$503,"&gt;="&amp;DATE(2026,8,31),'Trade Log'!$G$4:$G$503,"&lt;"&amp;DATE(2026,9,7),'Trade Log'!$L$4:$L$503,"&gt;0")/ABS(SUMIFS('Trade Log'!$L$4:$L$503,'Trade Log'!$G$4:$G$503,"&gt;="&amp;DATE(2026,8,31),'Trade Log'!$G$4:$G$503,"&lt;"&amp;DATE(2026,9,7),'Trade Log'!$L$4:$L$503,"&lt;0")),"")</f>
         <v/>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="28" t="n">
-        <v>46279</v>
+        <v>46272</v>
       </c>
       <c r="B15" s="20">
-        <f>COUNTIFS('Trade Log'!$G$4:$G$503,"&gt;="&amp;DATE(2026,9,14),'Trade Log'!$G$4:$G$503,"&lt;"&amp;DATE(2026,9,21))</f>
+        <f>COUNTIFS('Trade Log'!$G$4:$G$503,"&gt;="&amp;DATE(2026,9,7),'Trade Log'!$G$4:$G$503,"&lt;"&amp;DATE(2026,9,14))</f>
         <v/>
       </c>
       <c r="C15" s="20">
-        <f>COUNTIFS('Trade Log'!$G$4:$G$503,"&gt;="&amp;DATE(2026,9,14),'Trade Log'!$G$4:$G$503,"&lt;"&amp;DATE(2026,9,21),'Trade Log'!$L$4:$L$503,"&gt;0")</f>
+        <f>COUNTIFS('Trade Log'!$G$4:$G$503,"&gt;="&amp;DATE(2026,9,7),'Trade Log'!$G$4:$G$503,"&lt;"&amp;DATE(2026,9,14),'Trade Log'!$L$4:$L$503,"&gt;0")</f>
         <v/>
       </c>
       <c r="D15" s="20">
-        <f>COUNTIFS('Trade Log'!$G$4:$G$503,"&gt;="&amp;DATE(2026,9,14),'Trade Log'!$G$4:$G$503,"&lt;"&amp;DATE(2026,9,21),'Trade Log'!$L$4:$L$503,"&lt;0")</f>
+        <f>COUNTIFS('Trade Log'!$G$4:$G$503,"&gt;="&amp;DATE(2026,9,7),'Trade Log'!$G$4:$G$503,"&lt;"&amp;DATE(2026,9,14),'Trade Log'!$L$4:$L$503,"&lt;0")</f>
         <v/>
       </c>
       <c r="E15" s="22">
@@ -55368,11 +55382,11 @@
         <v/>
       </c>
       <c r="F15" s="21">
-        <f>SUMIFS('Trade Log'!$I$4:$I$503,'Trade Log'!$G$4:$G$503,"&gt;="&amp;DATE(2026,9,14),'Trade Log'!$G$4:$G$503,"&lt;"&amp;DATE(2026,9,21))</f>
+        <f>SUMIFS('Trade Log'!$I$4:$I$503,'Trade Log'!$G$4:$G$503,"&gt;="&amp;DATE(2026,9,7),'Trade Log'!$G$4:$G$503,"&lt;"&amp;DATE(2026,9,14))</f>
         <v/>
       </c>
       <c r="G15" s="21">
-        <f>SUMIFS('Trade Log'!$L$4:$L$503,'Trade Log'!$G$4:$G$503,"&gt;="&amp;DATE(2026,9,14),'Trade Log'!$G$4:$G$503,"&lt;"&amp;DATE(2026,9,21))</f>
+        <f>SUMIFS('Trade Log'!$L$4:$L$503,'Trade Log'!$G$4:$G$503,"&gt;="&amp;DATE(2026,9,7),'Trade Log'!$G$4:$G$503,"&lt;"&amp;DATE(2026,9,14))</f>
         <v/>
       </c>
       <c r="H15" s="21">
@@ -55380,32 +55394,32 @@
         <v/>
       </c>
       <c r="I15" s="21">
-        <f>IFERROR(_xlfn.MAXIFS('Trade Log'!$L$4:$L$503,'Trade Log'!$G$4:$G$503,"&gt;="&amp;DATE(2026,9,14),'Trade Log'!$G$4:$G$503,"&lt;"&amp;DATE(2026,9,21)),"")</f>
+        <f>IFERROR(_xlfn.MAXIFS('Trade Log'!$L$4:$L$503,'Trade Log'!$G$4:$G$503,"&gt;="&amp;DATE(2026,9,7),'Trade Log'!$G$4:$G$503,"&lt;"&amp;DATE(2026,9,14)),"")</f>
         <v/>
       </c>
       <c r="J15" s="21">
-        <f>IFERROR(_xlfn.MINIFS('Trade Log'!$L$4:$L$503,'Trade Log'!$G$4:$G$503,"&gt;="&amp;DATE(2026,9,14),'Trade Log'!$G$4:$G$503,"&lt;"&amp;DATE(2026,9,21)),"")</f>
+        <f>IFERROR(_xlfn.MINIFS('Trade Log'!$L$4:$L$503,'Trade Log'!$G$4:$G$503,"&gt;="&amp;DATE(2026,9,7),'Trade Log'!$G$4:$G$503,"&lt;"&amp;DATE(2026,9,14)),"")</f>
         <v/>
       </c>
       <c r="K15" s="29">
-        <f>IFERROR(SUMIFS('Trade Log'!$L$4:$L$503,'Trade Log'!$G$4:$G$503,"&gt;="&amp;DATE(2026,9,14),'Trade Log'!$G$4:$G$503,"&lt;"&amp;DATE(2026,9,21),'Trade Log'!$L$4:$L$503,"&gt;0")/ABS(SUMIFS('Trade Log'!$L$4:$L$503,'Trade Log'!$G$4:$G$503,"&gt;="&amp;DATE(2026,9,14),'Trade Log'!$G$4:$G$503,"&lt;"&amp;DATE(2026,9,21),'Trade Log'!$L$4:$L$503,"&lt;0")),"")</f>
+        <f>IFERROR(SUMIFS('Trade Log'!$L$4:$L$503,'Trade Log'!$G$4:$G$503,"&gt;="&amp;DATE(2026,9,7),'Trade Log'!$G$4:$G$503,"&lt;"&amp;DATE(2026,9,14),'Trade Log'!$L$4:$L$503,"&gt;0")/ABS(SUMIFS('Trade Log'!$L$4:$L$503,'Trade Log'!$G$4:$G$503,"&gt;="&amp;DATE(2026,9,7),'Trade Log'!$G$4:$G$503,"&lt;"&amp;DATE(2026,9,14),'Trade Log'!$L$4:$L$503,"&lt;0")),"")</f>
         <v/>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="28" t="n">
-        <v>46286</v>
+        <v>46279</v>
       </c>
       <c r="B16" s="20">
-        <f>COUNTIFS('Trade Log'!$G$4:$G$503,"&gt;="&amp;DATE(2026,9,21),'Trade Log'!$G$4:$G$503,"&lt;"&amp;DATE(2026,9,28))</f>
+        <f>COUNTIFS('Trade Log'!$G$4:$G$503,"&gt;="&amp;DATE(2026,9,14),'Trade Log'!$G$4:$G$503,"&lt;"&amp;DATE(2026,9,21))</f>
         <v/>
       </c>
       <c r="C16" s="20">
-        <f>COUNTIFS('Trade Log'!$G$4:$G$503,"&gt;="&amp;DATE(2026,9,21),'Trade Log'!$G$4:$G$503,"&lt;"&amp;DATE(2026,9,28),'Trade Log'!$L$4:$L$503,"&gt;0")</f>
+        <f>COUNTIFS('Trade Log'!$G$4:$G$503,"&gt;="&amp;DATE(2026,9,14),'Trade Log'!$G$4:$G$503,"&lt;"&amp;DATE(2026,9,21),'Trade Log'!$L$4:$L$503,"&gt;0")</f>
         <v/>
       </c>
       <c r="D16" s="20">
-        <f>COUNTIFS('Trade Log'!$G$4:$G$503,"&gt;="&amp;DATE(2026,9,21),'Trade Log'!$G$4:$G$503,"&lt;"&amp;DATE(2026,9,28),'Trade Log'!$L$4:$L$503,"&lt;0")</f>
+        <f>COUNTIFS('Trade Log'!$G$4:$G$503,"&gt;="&amp;DATE(2026,9,14),'Trade Log'!$G$4:$G$503,"&lt;"&amp;DATE(2026,9,21),'Trade Log'!$L$4:$L$503,"&lt;0")</f>
         <v/>
       </c>
       <c r="E16" s="22">
@@ -55413,11 +55427,11 @@
         <v/>
       </c>
       <c r="F16" s="21">
-        <f>SUMIFS('Trade Log'!$I$4:$I$503,'Trade Log'!$G$4:$G$503,"&gt;="&amp;DATE(2026,9,21),'Trade Log'!$G$4:$G$503,"&lt;"&amp;DATE(2026,9,28))</f>
+        <f>SUMIFS('Trade Log'!$I$4:$I$503,'Trade Log'!$G$4:$G$503,"&gt;="&amp;DATE(2026,9,14),'Trade Log'!$G$4:$G$503,"&lt;"&amp;DATE(2026,9,21))</f>
         <v/>
       </c>
       <c r="G16" s="21">
-        <f>SUMIFS('Trade Log'!$L$4:$L$503,'Trade Log'!$G$4:$G$503,"&gt;="&amp;DATE(2026,9,21),'Trade Log'!$G$4:$G$503,"&lt;"&amp;DATE(2026,9,28))</f>
+        <f>SUMIFS('Trade Log'!$L$4:$L$503,'Trade Log'!$G$4:$G$503,"&gt;="&amp;DATE(2026,9,14),'Trade Log'!$G$4:$G$503,"&lt;"&amp;DATE(2026,9,21))</f>
         <v/>
       </c>
       <c r="H16" s="21">
@@ -55425,32 +55439,32 @@
         <v/>
       </c>
       <c r="I16" s="21">
-        <f>IFERROR(_xlfn.MAXIFS('Trade Log'!$L$4:$L$503,'Trade Log'!$G$4:$G$503,"&gt;="&amp;DATE(2026,9,21),'Trade Log'!$G$4:$G$503,"&lt;"&amp;DATE(2026,9,28)),"")</f>
+        <f>IFERROR(_xlfn.MAXIFS('Trade Log'!$L$4:$L$503,'Trade Log'!$G$4:$G$503,"&gt;="&amp;DATE(2026,9,14),'Trade Log'!$G$4:$G$503,"&lt;"&amp;DATE(2026,9,21)),"")</f>
         <v/>
       </c>
       <c r="J16" s="21">
-        <f>IFERROR(_xlfn.MINIFS('Trade Log'!$L$4:$L$503,'Trade Log'!$G$4:$G$503,"&gt;="&amp;DATE(2026,9,21),'Trade Log'!$G$4:$G$503,"&lt;"&amp;DATE(2026,9,28)),"")</f>
+        <f>IFERROR(_xlfn.MINIFS('Trade Log'!$L$4:$L$503,'Trade Log'!$G$4:$G$503,"&gt;="&amp;DATE(2026,9,14),'Trade Log'!$G$4:$G$503,"&lt;"&amp;DATE(2026,9,21)),"")</f>
         <v/>
       </c>
       <c r="K16" s="29">
-        <f>IFERROR(SUMIFS('Trade Log'!$L$4:$L$503,'Trade Log'!$G$4:$G$503,"&gt;="&amp;DATE(2026,9,21),'Trade Log'!$G$4:$G$503,"&lt;"&amp;DATE(2026,9,28),'Trade Log'!$L$4:$L$503,"&gt;0")/ABS(SUMIFS('Trade Log'!$L$4:$L$503,'Trade Log'!$G$4:$G$503,"&gt;="&amp;DATE(2026,9,21),'Trade Log'!$G$4:$G$503,"&lt;"&amp;DATE(2026,9,28),'Trade Log'!$L$4:$L$503,"&lt;0")),"")</f>
+        <f>IFERROR(SUMIFS('Trade Log'!$L$4:$L$503,'Trade Log'!$G$4:$G$503,"&gt;="&amp;DATE(2026,9,14),'Trade Log'!$G$4:$G$503,"&lt;"&amp;DATE(2026,9,21),'Trade Log'!$L$4:$L$503,"&gt;0")/ABS(SUMIFS('Trade Log'!$L$4:$L$503,'Trade Log'!$G$4:$G$503,"&gt;="&amp;DATE(2026,9,14),'Trade Log'!$G$4:$G$503,"&lt;"&amp;DATE(2026,9,21),'Trade Log'!$L$4:$L$503,"&lt;0")),"")</f>
         <v/>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="28" t="n">
-        <v>46293</v>
+        <v>46286</v>
       </c>
       <c r="B17" s="20">
-        <f>COUNTIFS('Trade Log'!$G$4:$G$503,"&gt;="&amp;DATE(2026,9,28),'Trade Log'!$G$4:$G$503,"&lt;"&amp;DATE(2026,10,5))</f>
+        <f>COUNTIFS('Trade Log'!$G$4:$G$503,"&gt;="&amp;DATE(2026,9,21),'Trade Log'!$G$4:$G$503,"&lt;"&amp;DATE(2026,9,28))</f>
         <v/>
       </c>
       <c r="C17" s="20">
-        <f>COUNTIFS('Trade Log'!$G$4:$G$503,"&gt;="&amp;DATE(2026,9,28),'Trade Log'!$G$4:$G$503,"&lt;"&amp;DATE(2026,10,5),'Trade Log'!$L$4:$L$503,"&gt;0")</f>
+        <f>COUNTIFS('Trade Log'!$G$4:$G$503,"&gt;="&amp;DATE(2026,9,21),'Trade Log'!$G$4:$G$503,"&lt;"&amp;DATE(2026,9,28),'Trade Log'!$L$4:$L$503,"&gt;0")</f>
         <v/>
       </c>
       <c r="D17" s="20">
-        <f>COUNTIFS('Trade Log'!$G$4:$G$503,"&gt;="&amp;DATE(2026,9,28),'Trade Log'!$G$4:$G$503,"&lt;"&amp;DATE(2026,10,5),'Trade Log'!$L$4:$L$503,"&lt;0")</f>
+        <f>COUNTIFS('Trade Log'!$G$4:$G$503,"&gt;="&amp;DATE(2026,9,21),'Trade Log'!$G$4:$G$503,"&lt;"&amp;DATE(2026,9,28),'Trade Log'!$L$4:$L$503,"&lt;0")</f>
         <v/>
       </c>
       <c r="E17" s="22">
@@ -55458,11 +55472,11 @@
         <v/>
       </c>
       <c r="F17" s="21">
-        <f>SUMIFS('Trade Log'!$I$4:$I$503,'Trade Log'!$G$4:$G$503,"&gt;="&amp;DATE(2026,9,28),'Trade Log'!$G$4:$G$503,"&lt;"&amp;DATE(2026,10,5))</f>
+        <f>SUMIFS('Trade Log'!$I$4:$I$503,'Trade Log'!$G$4:$G$503,"&gt;="&amp;DATE(2026,9,21),'Trade Log'!$G$4:$G$503,"&lt;"&amp;DATE(2026,9,28))</f>
         <v/>
       </c>
       <c r="G17" s="21">
-        <f>SUMIFS('Trade Log'!$L$4:$L$503,'Trade Log'!$G$4:$G$503,"&gt;="&amp;DATE(2026,9,28),'Trade Log'!$G$4:$G$503,"&lt;"&amp;DATE(2026,10,5))</f>
+        <f>SUMIFS('Trade Log'!$L$4:$L$503,'Trade Log'!$G$4:$G$503,"&gt;="&amp;DATE(2026,9,21),'Trade Log'!$G$4:$G$503,"&lt;"&amp;DATE(2026,9,28))</f>
         <v/>
       </c>
       <c r="H17" s="21">
@@ -55470,53 +55484,98 @@
         <v/>
       </c>
       <c r="I17" s="21">
+        <f>IFERROR(_xlfn.MAXIFS('Trade Log'!$L$4:$L$503,'Trade Log'!$G$4:$G$503,"&gt;="&amp;DATE(2026,9,21),'Trade Log'!$G$4:$G$503,"&lt;"&amp;DATE(2026,9,28)),"")</f>
+        <v/>
+      </c>
+      <c r="J17" s="21">
+        <f>IFERROR(_xlfn.MINIFS('Trade Log'!$L$4:$L$503,'Trade Log'!$G$4:$G$503,"&gt;="&amp;DATE(2026,9,21),'Trade Log'!$G$4:$G$503,"&lt;"&amp;DATE(2026,9,28)),"")</f>
+        <v/>
+      </c>
+      <c r="K17" s="29">
+        <f>IFERROR(SUMIFS('Trade Log'!$L$4:$L$503,'Trade Log'!$G$4:$G$503,"&gt;="&amp;DATE(2026,9,21),'Trade Log'!$G$4:$G$503,"&lt;"&amp;DATE(2026,9,28),'Trade Log'!$L$4:$L$503,"&gt;0")/ABS(SUMIFS('Trade Log'!$L$4:$L$503,'Trade Log'!$G$4:$G$503,"&gt;="&amp;DATE(2026,9,21),'Trade Log'!$G$4:$G$503,"&lt;"&amp;DATE(2026,9,28),'Trade Log'!$L$4:$L$503,"&lt;0")),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="28" t="n">
+        <v>46293</v>
+      </c>
+      <c r="B18" s="20">
+        <f>COUNTIFS('Trade Log'!$G$4:$G$503,"&gt;="&amp;DATE(2026,9,28),'Trade Log'!$G$4:$G$503,"&lt;"&amp;DATE(2026,10,5))</f>
+        <v/>
+      </c>
+      <c r="C18" s="20">
+        <f>COUNTIFS('Trade Log'!$G$4:$G$503,"&gt;="&amp;DATE(2026,9,28),'Trade Log'!$G$4:$G$503,"&lt;"&amp;DATE(2026,10,5),'Trade Log'!$L$4:$L$503,"&gt;0")</f>
+        <v/>
+      </c>
+      <c r="D18" s="20">
+        <f>COUNTIFS('Trade Log'!$G$4:$G$503,"&gt;="&amp;DATE(2026,9,28),'Trade Log'!$G$4:$G$503,"&lt;"&amp;DATE(2026,10,5),'Trade Log'!$L$4:$L$503,"&lt;0")</f>
+        <v/>
+      </c>
+      <c r="E18" s="22">
+        <f>IFERROR($C18/$B18,"")</f>
+        <v/>
+      </c>
+      <c r="F18" s="21">
+        <f>SUMIFS('Trade Log'!$I$4:$I$503,'Trade Log'!$G$4:$G$503,"&gt;="&amp;DATE(2026,9,28),'Trade Log'!$G$4:$G$503,"&lt;"&amp;DATE(2026,10,5))</f>
+        <v/>
+      </c>
+      <c r="G18" s="21">
+        <f>SUMIFS('Trade Log'!$L$4:$L$503,'Trade Log'!$G$4:$G$503,"&gt;="&amp;DATE(2026,9,28),'Trade Log'!$G$4:$G$503,"&lt;"&amp;DATE(2026,10,5))</f>
+        <v/>
+      </c>
+      <c r="H18" s="21">
+        <f>IFERROR($G18/$B18,"")</f>
+        <v/>
+      </c>
+      <c r="I18" s="21">
         <f>IFERROR(_xlfn.MAXIFS('Trade Log'!$L$4:$L$503,'Trade Log'!$G$4:$G$503,"&gt;="&amp;DATE(2026,9,28),'Trade Log'!$G$4:$G$503,"&lt;"&amp;DATE(2026,10,5)),"")</f>
         <v/>
       </c>
-      <c r="J17" s="21">
+      <c r="J18" s="21">
         <f>IFERROR(_xlfn.MINIFS('Trade Log'!$L$4:$L$503,'Trade Log'!$G$4:$G$503,"&gt;="&amp;DATE(2026,9,28),'Trade Log'!$G$4:$G$503,"&lt;"&amp;DATE(2026,10,5)),"")</f>
         <v/>
       </c>
-      <c r="K17" s="29">
+      <c r="K18" s="29">
         <f>IFERROR(SUMIFS('Trade Log'!$L$4:$L$503,'Trade Log'!$G$4:$G$503,"&gt;="&amp;DATE(2026,9,28),'Trade Log'!$G$4:$G$503,"&lt;"&amp;DATE(2026,10,5),'Trade Log'!$L$4:$L$503,"&gt;0")/ABS(SUMIFS('Trade Log'!$L$4:$L$503,'Trade Log'!$G$4:$G$503,"&gt;="&amp;DATE(2026,9,28),'Trade Log'!$G$4:$G$503,"&lt;"&amp;DATE(2026,10,5),'Trade Log'!$L$4:$L$503,"&lt;0")),"")</f>
         <v/>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" s="3" t="inlineStr">
+    <row r="19">
+      <c r="A19" s="3" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="B18" s="30">
-        <f>SUM(B11:B17)</f>
-        <v/>
-      </c>
-      <c r="C18" s="30">
-        <f>SUM(C11:C17)</f>
-        <v/>
-      </c>
-      <c r="D18" s="30">
-        <f>SUM(D11:D17)</f>
-        <v/>
-      </c>
-      <c r="E18" s="31">
-        <f>IFERROR(C18/B18,"")</f>
-        <v/>
-      </c>
-      <c r="F18" s="32">
-        <f>SUM(F11:F17)</f>
-        <v/>
-      </c>
-      <c r="G18" s="32">
-        <f>SUM(G11:G17)</f>
-        <v/>
-      </c>
-      <c r="H18" s="32">
-        <f>IFERROR(G18/B18,"")</f>
-        <v/>
-      </c>
-      <c r="K18" s="33">
+      <c r="B19" s="30">
+        <f>SUM(B12:B18)</f>
+        <v/>
+      </c>
+      <c r="C19" s="30">
+        <f>SUM(C12:C18)</f>
+        <v/>
+      </c>
+      <c r="D19" s="30">
+        <f>SUM(D12:D18)</f>
+        <v/>
+      </c>
+      <c r="E19" s="31">
+        <f>IFERROR(C19/B19,"")</f>
+        <v/>
+      </c>
+      <c r="F19" s="32">
+        <f>SUM(F12:F18)</f>
+        <v/>
+      </c>
+      <c r="G19" s="32">
+        <f>SUM(G12:G18)</f>
+        <v/>
+      </c>
+      <c r="H19" s="32">
+        <f>IFERROR(G19/B19,"")</f>
+        <v/>
+      </c>
+      <c r="K19" s="33">
         <f>IFERROR(SUMIF('Trade Log'!$L$4:$L$503,"&gt;0")/ABS(SUMIF('Trade Log'!$L$4:$L$503,"&lt;0")),"")</f>
         <v/>
       </c>

</xml_diff>

<commit_message>
Data update — 2026-10-05 candle + results refresh
</commit_message>
<xml_diff>
--- a/results/strategy_pnl_simple.xlsx
+++ b/results/strategy_pnl_simple.xlsx
@@ -1094,7 +1094,7 @@
         <v/>
       </c>
       <c r="K4" s="4" t="n">
-        <v>570.13</v>
+        <v>568.33</v>
       </c>
       <c r="L4" s="21">
         <f>IF(OR($B4="",$I4=""),"",$I4-IF($K4="",0,$K4))</f>
@@ -1214,7 +1214,7 @@
         <v/>
       </c>
       <c r="K6" s="4" t="n">
-        <v>686.97</v>
+        <v>684.47</v>
       </c>
       <c r="L6" s="21">
         <f>IF(OR($B6="",$I6=""),"",$I6-IF($K6="",0,$K6))</f>
@@ -1334,7 +1334,7 @@
         <v/>
       </c>
       <c r="K8" s="4" t="n">
-        <v>568.98</v>
+        <v>567.1900000000001</v>
       </c>
       <c r="L8" s="21">
         <f>IF(OR($B8="",$I8=""),"",$I8-IF($K8="",0,$K8))</f>
@@ -1454,7 +1454,7 @@
         <v/>
       </c>
       <c r="K10" s="4" t="n">
-        <v>661.0599999999999</v>
+        <v>658.9</v>
       </c>
       <c r="L10" s="21">
         <f>IF(OR($B10="",$I10=""),"",$I10-IF($K10="",0,$K10))</f>
@@ -1574,7 +1574,7 @@
         <v/>
       </c>
       <c r="K12" s="4" t="n">
-        <v>590.21</v>
+        <v>588.22</v>
       </c>
       <c r="L12" s="21">
         <f>IF(OR($B12="",$I12=""),"",$I12-IF($K12="",0,$K12))</f>
@@ -1694,7 +1694,7 @@
         <v/>
       </c>
       <c r="K14" s="4" t="n">
-        <v>397.7</v>
+        <v>396.71</v>
       </c>
       <c r="L14" s="21">
         <f>IF(OR($B14="",$I14=""),"",$I14-IF($K14="",0,$K14))</f>
@@ -1814,7 +1814,7 @@
         <v/>
       </c>
       <c r="K16" s="4" t="n">
-        <v>413.05</v>
+        <v>411.85</v>
       </c>
       <c r="L16" s="21">
         <f>IF(OR($B16="",$I16=""),"",$I16-IF($K16="",0,$K16))</f>
@@ -1934,7 +1934,7 @@
         <v/>
       </c>
       <c r="K18" s="4" t="n">
-        <v>344.41</v>
+        <v>374.48</v>
       </c>
       <c r="L18" s="21">
         <f>IF(OR($B18="",$I18=""),"",$I18-IF($K18="",0,$K18))</f>
@@ -2054,7 +2054,7 @@
         <v/>
       </c>
       <c r="K20" s="4" t="n">
-        <v>413.39</v>
+        <v>412.19</v>
       </c>
       <c r="L20" s="21">
         <f>IF(OR($B20="",$I20=""),"",$I20-IF($K20="",0,$K20))</f>
@@ -2174,7 +2174,7 @@
         <v/>
       </c>
       <c r="K22" s="4" t="n">
-        <v>379.54</v>
+        <v>378.25</v>
       </c>
       <c r="L22" s="21">
         <f>IF(OR($B22="",$I22=""),"",$I22-IF($K22="",0,$K22))</f>
@@ -2294,7 +2294,7 @@
         <v/>
       </c>
       <c r="K24" s="4" t="n">
-        <v>412.81</v>
+        <v>411.61</v>
       </c>
       <c r="L24" s="21">
         <f>IF(OR($B24="",$I24=""),"",$I24-IF($K24="",0,$K24))</f>
@@ -2414,7 +2414,7 @@
         <v/>
       </c>
       <c r="K26" s="4" t="n">
-        <v>405.51</v>
+        <v>404.48</v>
       </c>
       <c r="L26" s="21">
         <f>IF(OR($B26="",$I26=""),"",$I26-IF($K26="",0,$K26))</f>
@@ -2654,7 +2654,7 @@
         <v/>
       </c>
       <c r="K30" s="4" t="n">
-        <v>867.47</v>
+        <v>864.75</v>
       </c>
       <c r="L30" s="21">
         <f>IF(OR($B30="",$I30=""),"",$I30-IF($K30="",0,$K30))</f>
@@ -2894,7 +2894,7 @@
         <v/>
       </c>
       <c r="K34" s="4" t="n">
-        <v>390.57</v>
+        <v>391.79</v>
       </c>
       <c r="L34" s="21">
         <f>IF(OR($B34="",$I34=""),"",$I34-IF($K34="",0,$K34))</f>
@@ -3014,7 +3014,7 @@
         <v/>
       </c>
       <c r="K36" s="4" t="n">
-        <v>349.18</v>
+        <v>350.41</v>
       </c>
       <c r="L36" s="21">
         <f>IF(OR($B36="",$I36=""),"",$I36-IF($K36="",0,$K36))</f>
@@ -3134,7 +3134,7 @@
         <v/>
       </c>
       <c r="K38" s="4" t="n">
-        <v>329.26</v>
+        <v>329.99</v>
       </c>
       <c r="L38" s="21">
         <f>IF(OR($B38="",$I38=""),"",$I38-IF($K38="",0,$K38))</f>
@@ -3254,7 +3254,7 @@
         <v/>
       </c>
       <c r="K40" s="4" t="n">
-        <v>385.5</v>
+        <v>386.69</v>
       </c>
       <c r="L40" s="21">
         <f>IF(OR($B40="",$I40=""),"",$I40-IF($K40="",0,$K40))</f>
@@ -3374,7 +3374,7 @@
         <v/>
       </c>
       <c r="K42" s="4" t="n">
-        <v>977.03</v>
+        <v>979.6</v>
       </c>
       <c r="L42" s="21">
         <f>IF(OR($B42="",$I42=""),"",$I42-IF($K42="",0,$K42))</f>
@@ -3434,7 +3434,7 @@
         <v/>
       </c>
       <c r="K43" s="4" t="n">
-        <v>956.64</v>
+        <v>958.78</v>
       </c>
       <c r="L43" s="21">
         <f>IF(OR($B43="",$I43=""),"",$I43-IF($K43="",0,$K43))</f>
@@ -3494,7 +3494,7 @@
         <v/>
       </c>
       <c r="K44" s="4" t="n">
-        <v>991.02</v>
+        <v>993.6</v>
       </c>
       <c r="L44" s="21">
         <f>IF(OR($B44="",$I44=""),"",$I44-IF($K44="",0,$K44))</f>
@@ -3554,7 +3554,7 @@
         <v/>
       </c>
       <c r="K45" s="4" t="n">
-        <v>597.7</v>
+        <v>601.8099999999999</v>
       </c>
       <c r="L45" s="21">
         <f>IF(OR($B45="",$I45=""),"",$I45-IF($K45="",0,$K45))</f>
@@ -3674,7 +3674,7 @@
         <v/>
       </c>
       <c r="K47" s="4" t="n">
-        <v>598.8099999999999</v>
+        <v>602.9299999999999</v>
       </c>
       <c r="L47" s="21">
         <f>IF(OR($B47="",$I47=""),"",$I47-IF($K47="",0,$K47))</f>
@@ -3794,7 +3794,7 @@
         <v/>
       </c>
       <c r="K49" s="4" t="n">
-        <v>677.33</v>
+        <v>681.95</v>
       </c>
       <c r="L49" s="21">
         <f>IF(OR($B49="",$I49=""),"",$I49-IF($K49="",0,$K49))</f>
@@ -3914,7 +3914,7 @@
         <v/>
       </c>
       <c r="K51" s="4" t="n">
-        <v>670.2</v>
+        <v>674.45</v>
       </c>
       <c r="L51" s="21">
         <f>IF(OR($B51="",$I51=""),"",$I51-IF($K51="",0,$K51))</f>
@@ -4034,7 +4034,7 @@
         <v/>
       </c>
       <c r="K53" s="4" t="n">
-        <v>574.42</v>
+        <v>539.96</v>
       </c>
       <c r="L53" s="21">
         <f>IF(OR($B53="",$I53=""),"",$I53-IF($K53="",0,$K53))</f>
@@ -4154,7 +4154,7 @@
         <v/>
       </c>
       <c r="K55" s="4" t="n">
-        <v>628.47</v>
+        <v>629.28</v>
       </c>
       <c r="L55" s="21">
         <f>IF(OR($B55="",$I55=""),"",$I55-IF($K55="",0,$K55))</f>
@@ -4274,7 +4274,7 @@
         <v/>
       </c>
       <c r="K57" s="4" t="n">
-        <v>619.42</v>
+        <v>620.26</v>
       </c>
       <c r="L57" s="21">
         <f>IF(OR($B57="",$I57=""),"",$I57-IF($K57="",0,$K57))</f>
@@ -4394,7 +4394,7 @@
         <v/>
       </c>
       <c r="K59" s="4" t="n">
-        <v>612.42</v>
+        <v>613.12</v>
       </c>
       <c r="L59" s="21">
         <f>IF(OR($B59="",$I59=""),"",$I59-IF($K59="",0,$K59))</f>
@@ -4634,7 +4634,7 @@
         <v/>
       </c>
       <c r="K63" s="4" t="n">
-        <v>693.65</v>
+        <v>692.48</v>
       </c>
       <c r="L63" s="21">
         <f>IF(OR($B63="",$I63=""),"",$I63-IF($K63="",0,$K63))</f>
@@ -4754,7 +4754,7 @@
         <v/>
       </c>
       <c r="K65" s="4" t="n">
-        <v>616.98</v>
+        <v>615.59</v>
       </c>
       <c r="L65" s="21">
         <f>IF(OR($B65="",$I65=""),"",$I65-IF($K65="",0,$K65))</f>
@@ -4874,7 +4874,7 @@
         <v/>
       </c>
       <c r="K67" s="4" t="n">
-        <v>441.54</v>
+        <v>440.81</v>
       </c>
       <c r="L67" s="21">
         <f>IF(OR($B67="",$I67=""),"",$I67-IF($K67="",0,$K67))</f>
@@ -4994,7 +4994,7 @@
         <v/>
       </c>
       <c r="K69" s="4" t="n">
-        <v>387.48</v>
+        <v>386.81</v>
       </c>
       <c r="L69" s="21">
         <f>IF(OR($B69="",$I69=""),"",$I69-IF($K69="",0,$K69))</f>
@@ -5234,7 +5234,7 @@
         <v/>
       </c>
       <c r="K73" s="4" t="n">
-        <v>386.08</v>
+        <v>385.41</v>
       </c>
       <c r="L73" s="21">
         <f>IF(OR($B73="",$I73=""),"",$I73-IF($K73="",0,$K73))</f>
@@ -5354,7 +5354,7 @@
         <v/>
       </c>
       <c r="K75" s="4" t="n">
-        <v>435.15</v>
+        <v>434.49</v>
       </c>
       <c r="L75" s="21">
         <f>IF(OR($B75="",$I75=""),"",$I75-IF($K75="",0,$K75))</f>
@@ -5474,7 +5474,7 @@
         <v/>
       </c>
       <c r="K77" s="4" t="n">
-        <v>411.79</v>
+        <v>411.34</v>
       </c>
       <c r="L77" s="21">
         <f>IF(OR($B77="",$I77=""),"",$I77-IF($K77="",0,$K77))</f>
@@ -5714,7 +5714,7 @@
         <v/>
       </c>
       <c r="K81" s="4" t="n">
-        <v>356.25</v>
+        <v>355.88</v>
       </c>
       <c r="L81" s="21">
         <f>IF(OR($B81="",$I81=""),"",$I81-IF($K81="",0,$K81))</f>
@@ -5834,7 +5834,7 @@
         <v/>
       </c>
       <c r="K83" s="4" t="n">
-        <v>364.87</v>
+        <v>364.42</v>
       </c>
       <c r="L83" s="21">
         <f>IF(OR($B83="",$I83=""),"",$I83-IF($K83="",0,$K83))</f>
@@ -5954,7 +5954,7 @@
         <v/>
       </c>
       <c r="K85" s="4" t="n">
-        <v>412.42</v>
+        <v>411.95</v>
       </c>
       <c r="L85" s="21">
         <f>IF(OR($B85="",$I85=""),"",$I85-IF($K85="",0,$K85))</f>
@@ -6074,7 +6074,7 @@
         <v/>
       </c>
       <c r="K87" s="4" t="n">
-        <v>344.23</v>
+        <v>367.52</v>
       </c>
       <c r="L87" s="21">
         <f>IF(OR($B87="",$I87=""),"",$I87-IF($K87="",0,$K87))</f>
@@ -6314,7 +6314,7 @@
         <v/>
       </c>
       <c r="K91" s="4" t="n">
-        <v>893.4299999999999</v>
+        <v>892.1900000000001</v>
       </c>
       <c r="L91" s="21">
         <f>IF(OR($B91="",$I91=""),"",$I91-IF($K91="",0,$K91))</f>
@@ -6434,7 +6434,7 @@
         <v/>
       </c>
       <c r="K93" s="4" t="n">
-        <v>799.4400000000001</v>
+        <v>798.21</v>
       </c>
       <c r="L93" s="21">
         <f>IF(OR($B93="",$I93=""),"",$I93-IF($K93="",0,$K93))</f>
@@ -6554,7 +6554,7 @@
         <v/>
       </c>
       <c r="K95" s="4" t="n">
-        <v>826.78</v>
+        <v>825.54</v>
       </c>
       <c r="L95" s="21">
         <f>IF(OR($B95="",$I95=""),"",$I95-IF($K95="",0,$K95))</f>
@@ -6674,7 +6674,7 @@
         <v/>
       </c>
       <c r="K97" s="4" t="n">
-        <v>479.65</v>
+        <v>479.21</v>
       </c>
       <c r="L97" s="21">
         <f>IF(OR($B97="",$I97=""),"",$I97-IF($K97="",0,$K97))</f>
@@ -6914,7 +6914,7 @@
         <v/>
       </c>
       <c r="K101" s="4" t="n">
-        <v>474.57</v>
+        <v>474.16</v>
       </c>
       <c r="L101" s="21">
         <f>IF(OR($B101="",$I101=""),"",$I101-IF($K101="",0,$K101))</f>
@@ -7034,7 +7034,7 @@
         <v/>
       </c>
       <c r="K103" s="4" t="n">
-        <v>531.35</v>
+        <v>530.9299999999999</v>
       </c>
       <c r="L103" s="21">
         <f>IF(OR($B103="",$I103=""),"",$I103-IF($K103="",0,$K103))</f>
@@ -7214,7 +7214,7 @@
         <v/>
       </c>
       <c r="K106" s="4" t="n">
-        <v>531.5599999999999</v>
+        <v>531.14</v>
       </c>
       <c r="L106" s="21">
         <f>IF(OR($B106="",$I106=""),"",$I106-IF($K106="",0,$K106))</f>
@@ -7694,7 +7694,7 @@
         <v/>
       </c>
       <c r="K114" s="4" t="n">
-        <v>481</v>
+        <v>480.61</v>
       </c>
       <c r="L114" s="21">
         <f>IF(OR($B114="",$I114=""),"",$I114-IF($K114="",0,$K114))</f>
@@ -7814,7 +7814,7 @@
         <v/>
       </c>
       <c r="K116" s="4" t="n">
-        <v>420.13</v>
+        <v>419.77</v>
       </c>
       <c r="L116" s="21">
         <f>IF(OR($B116="",$I116=""),"",$I116-IF($K116="",0,$K116))</f>
@@ -8054,7 +8054,7 @@
         <v/>
       </c>
       <c r="K120" s="4" t="n">
-        <v>428.98</v>
+        <v>428.64</v>
       </c>
       <c r="L120" s="21">
         <f>IF(OR($B120="",$I120=""),"",$I120-IF($K120="",0,$K120))</f>
@@ -8174,7 +8174,7 @@
         <v/>
       </c>
       <c r="K122" s="4" t="n">
-        <v>546.3200000000001</v>
+        <v>545.8200000000001</v>
       </c>
       <c r="L122" s="21">
         <f>IF(OR($B122="",$I122=""),"",$I122-IF($K122="",0,$K122))</f>
@@ -8414,7 +8414,7 @@
         <v/>
       </c>
       <c r="K126" s="4" t="n">
-        <v>425.1</v>
+        <v>424.83</v>
       </c>
       <c r="L126" s="21">
         <f>IF(OR($B126="",$I126=""),"",$I126-IF($K126="",0,$K126))</f>
@@ -8534,7 +8534,7 @@
         <v/>
       </c>
       <c r="K128" s="4" t="n">
-        <v>371.58</v>
+        <v>371.31</v>
       </c>
       <c r="L128" s="21">
         <f>IF(OR($B128="",$I128=""),"",$I128-IF($K128="",0,$K128))</f>
@@ -8654,7 +8654,7 @@
         <v/>
       </c>
       <c r="K130" s="4" t="n">
-        <v>642.48</v>
+        <v>641.97</v>
       </c>
       <c r="L130" s="21">
         <f>IF(OR($B130="",$I130=""),"",$I130-IF($K130="",0,$K130))</f>
@@ -8774,7 +8774,7 @@
         <v/>
       </c>
       <c r="K132" s="4" t="n">
-        <v>638.33</v>
+        <v>637.8099999999999</v>
       </c>
       <c r="L132" s="21">
         <f>IF(OR($B132="",$I132=""),"",$I132-IF($K132="",0,$K132))</f>
@@ -8894,7 +8894,7 @@
         <v/>
       </c>
       <c r="K134" s="4" t="n">
-        <v>654.01</v>
+        <v>653.51</v>
       </c>
       <c r="L134" s="21">
         <f>IF(OR($B134="",$I134=""),"",$I134-IF($K134="",0,$K134))</f>
@@ -9014,7 +9014,7 @@
         <v/>
       </c>
       <c r="K136" s="4" t="n">
-        <v>564.15</v>
+        <v>563.64</v>
       </c>
       <c r="L136" s="21">
         <f>IF(OR($B136="",$I136=""),"",$I136-IF($K136="",0,$K136))</f>
@@ -9134,7 +9134,7 @@
         <v/>
       </c>
       <c r="K138" s="4" t="n">
-        <v>632.12</v>
+        <v>631.61</v>
       </c>
       <c r="L138" s="21">
         <f>IF(OR($B138="",$I138=""),"",$I138-IF($K138="",0,$K138))</f>
@@ -9254,7 +9254,7 @@
         <v/>
       </c>
       <c r="K140" s="4" t="n">
-        <v>497.85</v>
+        <v>497.04</v>
       </c>
       <c r="L140" s="21">
         <f>IF(OR($B140="",$I140=""),"",$I140-IF($K140="",0,$K140))</f>
@@ -9494,7 +9494,7 @@
         <v/>
       </c>
       <c r="K144" s="4" t="n">
-        <v>494.59</v>
+        <v>493.79</v>
       </c>
       <c r="L144" s="21">
         <f>IF(OR($B144="",$I144=""),"",$I144-IF($K144="",0,$K144))</f>
@@ -9614,7 +9614,7 @@
         <v/>
       </c>
       <c r="K146" s="4" t="n">
-        <v>504.8</v>
+        <v>504.1</v>
       </c>
       <c r="L146" s="21">
         <f>IF(OR($B146="",$I146=""),"",$I146-IF($K146="",0,$K146))</f>
@@ -9734,7 +9734,7 @@
         <v/>
       </c>
       <c r="K148" s="4" t="n">
-        <v>491.3</v>
+        <v>490.59</v>
       </c>
       <c r="L148" s="21">
         <f>IF(OR($B148="",$I148=""),"",$I148-IF($K148="",0,$K148))</f>
@@ -9854,7 +9854,7 @@
         <v/>
       </c>
       <c r="K150" s="4" t="n">
-        <v>467.26</v>
+        <v>466.59</v>
       </c>
       <c r="L150" s="21">
         <f>IF(OR($B150="",$I150=""),"",$I150-IF($K150="",0,$K150))</f>
@@ -10094,7 +10094,7 @@
         <v/>
       </c>
       <c r="K154" s="4" t="n">
-        <v>542.41</v>
+        <v>541.72</v>
       </c>
       <c r="L154" s="21">
         <f>IF(OR($B154="",$I154=""),"",$I154-IF($K154="",0,$K154))</f>
@@ -10214,7 +10214,7 @@
         <v/>
       </c>
       <c r="K156" s="4" t="n">
-        <v>461.72</v>
+        <v>460.93</v>
       </c>
       <c r="L156" s="21">
         <f>IF(OR($B156="",$I156=""),"",$I156-IF($K156="",0,$K156))</f>
@@ -10334,7 +10334,7 @@
         <v/>
       </c>
       <c r="K158" s="4" t="n">
-        <v>526.66</v>
+        <v>525.87</v>
       </c>
       <c r="L158" s="21">
         <f>IF(OR($B158="",$I158=""),"",$I158-IF($K158="",0,$K158))</f>
@@ -10454,7 +10454,7 @@
         <v/>
       </c>
       <c r="K160" s="4" t="n">
-        <v>520.86</v>
+        <v>520.13</v>
       </c>
       <c r="L160" s="21">
         <f>IF(OR($B160="",$I160=""),"",$I160-IF($K160="",0,$K160))</f>
@@ -10574,7 +10574,7 @@
         <v/>
       </c>
       <c r="K162" s="4" t="n">
-        <v>519.23</v>
+        <v>518.5</v>
       </c>
       <c r="L162" s="21">
         <f>IF(OR($B162="",$I162=""),"",$I162-IF($K162="",0,$K162))</f>
@@ -10694,7 +10694,7 @@
         <v/>
       </c>
       <c r="K164" s="4" t="n">
-        <v>447.13</v>
+        <v>446.52</v>
       </c>
       <c r="L164" s="21">
         <f>IF(OR($B164="",$I164=""),"",$I164-IF($K164="",0,$K164))</f>
@@ -10814,7 +10814,7 @@
         <v/>
       </c>
       <c r="K166" s="4" t="n">
-        <v>463.78</v>
+        <v>462.96</v>
       </c>
       <c r="L166" s="21">
         <f>IF(OR($B166="",$I166=""),"",$I166-IF($K166="",0,$K166))</f>
@@ -10934,7 +10934,7 @@
         <v/>
       </c>
       <c r="K168" s="4" t="n">
-        <v>628.74</v>
+        <v>627.8</v>
       </c>
       <c r="L168" s="21">
         <f>IF(OR($B168="",$I168=""),"",$I168-IF($K168="",0,$K168))</f>
@@ -11054,7 +11054,7 @@
         <v/>
       </c>
       <c r="K170" s="4" t="n">
-        <v>637.12</v>
+        <v>636.02</v>
       </c>
       <c r="L170" s="21">
         <f>IF(OR($B170="",$I170=""),"",$I170-IF($K170="",0,$K170))</f>
@@ -11294,7 +11294,7 @@
         <v/>
       </c>
       <c r="K174" s="4" t="n">
-        <v>601.05</v>
+        <v>599.26</v>
       </c>
       <c r="L174" s="21">
         <f>IF(OR($B174="",$I174=""),"",$I174-IF($K174="",0,$K174))</f>
@@ -11414,7 +11414,7 @@
         <v/>
       </c>
       <c r="K176" s="4" t="n">
-        <v>590.26</v>
+        <v>588.52</v>
       </c>
       <c r="L176" s="21">
         <f>IF(OR($B176="",$I176=""),"",$I176-IF($K176="",0,$K176))</f>
@@ -11534,7 +11534,7 @@
         <v/>
       </c>
       <c r="K178" s="4" t="n">
-        <v>603.04</v>
+        <v>601.14</v>
       </c>
       <c r="L178" s="21">
         <f>IF(OR($B178="",$I178=""),"",$I178-IF($K178="",0,$K178))</f>
@@ -11654,7 +11654,7 @@
         <v/>
       </c>
       <c r="K180" s="4" t="n">
-        <v>592.24</v>
+        <v>590.49</v>
       </c>
       <c r="L180" s="21">
         <f>IF(OR($B180="",$I180=""),"",$I180-IF($K180="",0,$K180))</f>
@@ -11774,7 +11774,7 @@
         <v/>
       </c>
       <c r="K182" s="4" t="n">
-        <v>295.85</v>
+        <v>295.44</v>
       </c>
       <c r="L182" s="21">
         <f>IF(OR($B182="",$I182=""),"",$I182-IF($K182="",0,$K182))</f>
@@ -12014,7 +12014,7 @@
         <v/>
       </c>
       <c r="K186" s="4" t="n">
-        <v>337.66</v>
+        <v>337.25</v>
       </c>
       <c r="L186" s="21">
         <f>IF(OR($B186="",$I186=""),"",$I186-IF($K186="",0,$K186))</f>
@@ -12134,7 +12134,7 @@
         <v/>
       </c>
       <c r="K188" s="4" t="n">
-        <v>289</v>
+        <v>288.75</v>
       </c>
       <c r="L188" s="21">
         <f>IF(OR($B188="",$I188=""),"",$I188-IF($K188="",0,$K188))</f>
@@ -12254,7 +12254,7 @@
         <v/>
       </c>
       <c r="K190" s="4" t="n">
-        <v>192.01</v>
+        <v>191.86</v>
       </c>
       <c r="L190" s="21">
         <f>IF(OR($B190="",$I190=""),"",$I190-IF($K190="",0,$K190))</f>
@@ -12374,7 +12374,7 @@
         <v/>
       </c>
       <c r="K192" s="4" t="n">
-        <v>296.34</v>
+        <v>295.94</v>
       </c>
       <c r="L192" s="21">
         <f>IF(OR($B192="",$I192=""),"",$I192-IF($K192="",0,$K192))</f>
@@ -12494,7 +12494,7 @@
         <v/>
       </c>
       <c r="K194" s="4" t="n">
-        <v>500.53</v>
+        <v>500.1</v>
       </c>
       <c r="L194" s="21">
         <f>IF(OR($B194="",$I194=""),"",$I194-IF($K194="",0,$K194))</f>
@@ -12614,7 +12614,7 @@
         <v/>
       </c>
       <c r="K196" s="4" t="n">
-        <v>461.68</v>
+        <v>460.91</v>
       </c>
       <c r="L196" s="21">
         <f>IF(OR($B196="",$I196=""),"",$I196-IF($K196="",0,$K196))</f>
@@ -12734,7 +12734,7 @@
         <v/>
       </c>
       <c r="K198" s="4" t="n">
-        <v>464.65</v>
+        <v>463.72</v>
       </c>
       <c r="L198" s="21">
         <f>IF(OR($B198="",$I198=""),"",$I198-IF($K198="",0,$K198))</f>
@@ -12854,7 +12854,7 @@
         <v/>
       </c>
       <c r="K200" s="4" t="n">
-        <v>497.64</v>
+        <v>518.17</v>
       </c>
       <c r="L200" s="21">
         <f>IF(OR($B200="",$I200=""),"",$I200-IF($K200="",0,$K200))</f>
@@ -12974,7 +12974,7 @@
         <v/>
       </c>
       <c r="K202" s="4" t="n">
-        <v>520.95</v>
+        <v>520.22</v>
       </c>
       <c r="L202" s="21">
         <f>IF(OR($B202="",$I202=""),"",$I202-IF($K202="",0,$K202))</f>
@@ -13094,7 +13094,7 @@
         <v/>
       </c>
       <c r="K204" s="4" t="n">
-        <v>458.63</v>
+        <v>457.87</v>
       </c>
       <c r="L204" s="21">
         <f>IF(OR($B204="",$I204=""),"",$I204-IF($K204="",0,$K204))</f>
@@ -13214,7 +13214,7 @@
         <v/>
       </c>
       <c r="K206" s="4" t="n">
-        <v>395.37</v>
+        <v>395.13</v>
       </c>
       <c r="L206" s="21">
         <f>IF(OR($B206="",$I206=""),"",$I206-IF($K206="",0,$K206))</f>
@@ -13334,7 +13334,7 @@
         <v/>
       </c>
       <c r="K208" s="4" t="n">
-        <v>347.86</v>
+        <v>347.71</v>
       </c>
       <c r="L208" s="21">
         <f>IF(OR($B208="",$I208=""),"",$I208-IF($K208="",0,$K208))</f>
@@ -13574,7 +13574,7 @@
         <v/>
       </c>
       <c r="K212" s="4" t="n">
-        <v>385.74</v>
+        <v>385.6</v>
       </c>
       <c r="L212" s="21">
         <f>IF(OR($B212="",$I212=""),"",$I212-IF($K212="",0,$K212))</f>
@@ -13694,7 +13694,7 @@
         <v/>
       </c>
       <c r="K214" s="4" t="n">
-        <v>315.66</v>
+        <v>315.46</v>
       </c>
       <c r="L214" s="21">
         <f>IF(OR($B214="",$I214=""),"",$I214-IF($K214="",0,$K214))</f>
@@ -13814,7 +13814,7 @@
         <v/>
       </c>
       <c r="K216" s="4" t="n">
-        <v>311.33</v>
+        <v>311.19</v>
       </c>
       <c r="L216" s="21">
         <f>IF(OR($B216="",$I216=""),"",$I216-IF($K216="",0,$K216))</f>
@@ -13934,7 +13934,7 @@
         <v/>
       </c>
       <c r="K218" s="4" t="n">
-        <v>359.7</v>
+        <v>359.5</v>
       </c>
       <c r="L218" s="21">
         <f>IF(OR($B218="",$I218=""),"",$I218-IF($K218="",0,$K218))</f>
@@ -14054,7 +14054,7 @@
         <v/>
       </c>
       <c r="K220" s="4" t="n">
-        <v>316.78</v>
+        <v>316.54</v>
       </c>
       <c r="L220" s="21">
         <f>IF(OR($B220="",$I220=""),"",$I220-IF($K220="",0,$K220))</f>
@@ -14174,7 +14174,7 @@
         <v/>
       </c>
       <c r="K222" s="4" t="n">
-        <v>361.15</v>
+        <v>360.88</v>
       </c>
       <c r="L222" s="21">
         <f>IF(OR($B222="",$I222=""),"",$I222-IF($K222="",0,$K222))</f>
@@ -14294,7 +14294,7 @@
         <v/>
       </c>
       <c r="K224" s="4" t="n">
-        <v>459.21</v>
+        <v>459.22</v>
       </c>
       <c r="L224" s="21">
         <f>IF(OR($B224="",$I224=""),"",$I224-IF($K224="",0,$K224))</f>
@@ -14474,7 +14474,7 @@
         <v/>
       </c>
       <c r="K227" s="4" t="n">
-        <v>521.5700000000001</v>
+        <v>521.6</v>
       </c>
       <c r="L227" s="21">
         <f>IF(OR($B227="",$I227=""),"",$I227-IF($K227="",0,$K227))</f>
@@ -14714,7 +14714,7 @@
         <v/>
       </c>
       <c r="K231" s="4" t="n">
-        <v>461.19</v>
+        <v>461.21</v>
       </c>
       <c r="L231" s="21">
         <f>IF(OR($B231="",$I231=""),"",$I231-IF($K231="",0,$K231))</f>
@@ -15254,7 +15254,7 @@
         <v/>
       </c>
       <c r="K240" s="4" t="n">
-        <v>815.77</v>
+        <v>815.8</v>
       </c>
       <c r="L240" s="21">
         <f>IF(OR($B240="",$I240=""),"",$I240-IF($K240="",0,$K240))</f>
@@ -15434,7 +15434,7 @@
         <v/>
       </c>
       <c r="K243" s="4" t="n">
-        <v>903.83</v>
+        <v>903.79</v>
       </c>
       <c r="L243" s="21">
         <f>IF(OR($B243="",$I243=""),"",$I243-IF($K243="",0,$K243))</f>
@@ -15554,7 +15554,7 @@
         <v/>
       </c>
       <c r="K245" s="4" t="n">
-        <v>762.1</v>
+        <v>747.74</v>
       </c>
       <c r="L245" s="21">
         <f>IF(OR($B245="",$I245=""),"",$I245-IF($K245="",0,$K245))</f>
@@ -15614,7 +15614,7 @@
         <v/>
       </c>
       <c r="K246" s="4" t="n">
-        <v>622.27</v>
+        <v>622.3099999999999</v>
       </c>
       <c r="L246" s="21">
         <f>IF(OR($B246="",$I246=""),"",$I246-IF($K246="",0,$K246))</f>
@@ -42068,7 +42068,7 @@
         <v>35.4</v>
       </c>
       <c r="M4" s="4" t="n">
-        <v>106.04</v>
+        <v>104.24</v>
       </c>
       <c r="N4" s="21">
         <f>SUM(E4:M4)</f>
@@ -42170,7 +42170,7 @@
         <v>35.4</v>
       </c>
       <c r="M6" s="4" t="n">
-        <v>148.58</v>
+        <v>146.08</v>
       </c>
       <c r="N6" s="21">
         <f>SUM(E6:M6)</f>
@@ -42272,7 +42272,7 @@
         <v>35.4</v>
       </c>
       <c r="M8" s="4" t="n">
-        <v>105.87</v>
+        <v>104.07</v>
       </c>
       <c r="N8" s="21">
         <f>SUM(E8:M8)</f>
@@ -42374,7 +42374,7 @@
         <v>35.4</v>
       </c>
       <c r="M10" s="4" t="n">
-        <v>126.9</v>
+        <v>124.75</v>
       </c>
       <c r="N10" s="21">
         <f>SUM(E10:M10)</f>
@@ -42476,7 +42476,7 @@
         <v>35.4</v>
       </c>
       <c r="M12" s="4" t="n">
-        <v>124.75</v>
+        <v>122.76</v>
       </c>
       <c r="N12" s="21">
         <f>SUM(E12:M12)</f>
@@ -42578,7 +42578,7 @@
         <v>35.4</v>
       </c>
       <c r="M14" s="4" t="n">
-        <v>58.66</v>
+        <v>57.67</v>
       </c>
       <c r="N14" s="21">
         <f>SUM(E14:M14)</f>
@@ -42680,7 +42680,7 @@
         <v>35.4</v>
       </c>
       <c r="M16" s="4" t="n">
-        <v>70.89</v>
+        <v>69.69</v>
       </c>
       <c r="N16" s="21">
         <f>SUM(E16:M16)</f>
@@ -42782,7 +42782,7 @@
         <v>35.4</v>
       </c>
       <c r="M18" s="4" t="n">
-        <v>42.6</v>
+        <v>72.68000000000001</v>
       </c>
       <c r="N18" s="21">
         <f>SUM(E18:M18)</f>
@@ -42884,7 +42884,7 @@
         <v>35.4</v>
       </c>
       <c r="M20" s="4" t="n">
-        <v>70.67</v>
+        <v>69.47</v>
       </c>
       <c r="N20" s="21">
         <f>SUM(E20:M20)</f>
@@ -42986,7 +42986,7 @@
         <v>35.4</v>
       </c>
       <c r="M22" s="4" t="n">
-        <v>77.92</v>
+        <v>76.63</v>
       </c>
       <c r="N22" s="21">
         <f>SUM(E22:M22)</f>
@@ -43088,7 +43088,7 @@
         <v>35.4</v>
       </c>
       <c r="M24" s="4" t="n">
-        <v>71.04000000000001</v>
+        <v>69.83</v>
       </c>
       <c r="N24" s="21">
         <f>SUM(E24:M24)</f>
@@ -43190,7 +43190,7 @@
         <v>35.4</v>
       </c>
       <c r="M26" s="4" t="n">
-        <v>60.54</v>
+        <v>59.51</v>
       </c>
       <c r="N26" s="21">
         <f>SUM(E26:M26)</f>
@@ -43394,7 +43394,7 @@
         <v>35.4</v>
       </c>
       <c r="M30" s="4" t="n">
-        <v>311.14</v>
+        <v>308.43</v>
       </c>
       <c r="N30" s="21">
         <f>SUM(E30:M30)</f>
@@ -43598,7 +43598,7 @@
         <v>35.4</v>
       </c>
       <c r="M34" s="4" t="n">
-        <v>46.97</v>
+        <v>48.2</v>
       </c>
       <c r="N34" s="21">
         <f>SUM(E34:M34)</f>
@@ -43700,7 +43700,7 @@
         <v>35.4</v>
       </c>
       <c r="M36" s="4" t="n">
-        <v>46.95</v>
+        <v>48.18</v>
       </c>
       <c r="N36" s="21">
         <f>SUM(E36:M36)</f>
@@ -43802,7 +43802,7 @@
         <v>35.4</v>
       </c>
       <c r="M38" s="4" t="n">
-        <v>28.06</v>
+        <v>28.79</v>
       </c>
       <c r="N38" s="21">
         <f>SUM(E38:M38)</f>
@@ -43904,7 +43904,7 @@
         <v>35.4</v>
       </c>
       <c r="M40" s="4" t="n">
-        <v>44.9</v>
+        <v>46.09</v>
       </c>
       <c r="N40" s="21">
         <f>SUM(E40:M40)</f>
@@ -44006,7 +44006,7 @@
         <v>35.4</v>
       </c>
       <c r="M42" s="4" t="n">
-        <v>98.33</v>
+        <v>100.9</v>
       </c>
       <c r="N42" s="21">
         <f>SUM(E42:M42)</f>
@@ -44057,7 +44057,7 @@
         <v>35.4</v>
       </c>
       <c r="M43" s="4" t="n">
-        <v>82.02</v>
+        <v>84.16</v>
       </c>
       <c r="N43" s="21">
         <f>SUM(E43:M43)</f>
@@ -44108,7 +44108,7 @@
         <v>35.4</v>
       </c>
       <c r="M44" s="4" t="n">
-        <v>98.73999999999999</v>
+        <v>101.32</v>
       </c>
       <c r="N44" s="21">
         <f>SUM(E44:M44)</f>
@@ -44159,7 +44159,7 @@
         <v>35.4</v>
       </c>
       <c r="M45" s="4" t="n">
-        <v>157.26</v>
+        <v>161.37</v>
       </c>
       <c r="N45" s="21">
         <f>SUM(E45:M45)</f>
@@ -44261,7 +44261,7 @@
         <v>35.4</v>
       </c>
       <c r="M47" s="4" t="n">
-        <v>157.7</v>
+        <v>161.82</v>
       </c>
       <c r="N47" s="21">
         <f>SUM(E47:M47)</f>
@@ -44363,7 +44363,7 @@
         <v>35.4</v>
       </c>
       <c r="M49" s="4" t="n">
-        <v>171.67</v>
+        <v>176.29</v>
       </c>
       <c r="N49" s="21">
         <f>SUM(E49:M49)</f>
@@ -44465,7 +44465,7 @@
         <v>35.4</v>
       </c>
       <c r="M51" s="4" t="n">
-        <v>156.53</v>
+        <v>160.78</v>
       </c>
       <c r="N51" s="21">
         <f>SUM(E51:M51)</f>
@@ -44567,7 +44567,7 @@
         <v>35.4</v>
       </c>
       <c r="M53" s="4" t="n">
-        <v>131.94</v>
+        <v>97.48</v>
       </c>
       <c r="N53" s="21">
         <f>SUM(E53:M53)</f>
@@ -44669,7 +44669,7 @@
         <v>35.4</v>
       </c>
       <c r="M55" s="4" t="n">
-        <v>98.90000000000001</v>
+        <v>99.70999999999999</v>
       </c>
       <c r="N55" s="21">
         <f>SUM(E55:M55)</f>
@@ -44771,7 +44771,7 @@
         <v>35.4</v>
       </c>
       <c r="M57" s="4" t="n">
-        <v>97.11</v>
+        <v>97.94</v>
       </c>
       <c r="N57" s="21">
         <f>SUM(E57:M57)</f>
@@ -44873,7 +44873,7 @@
         <v>35.4</v>
       </c>
       <c r="M59" s="4" t="n">
-        <v>87.81</v>
+        <v>88.51000000000001</v>
       </c>
       <c r="N59" s="21">
         <f>SUM(E59:M59)</f>
@@ -45077,7 +45077,7 @@
         <v>35.4</v>
       </c>
       <c r="M63" s="4" t="n">
-        <v>78.03</v>
+        <v>76.86</v>
       </c>
       <c r="N63" s="21">
         <f>SUM(E63:M63)</f>
@@ -45179,7 +45179,7 @@
         <v>35.4</v>
       </c>
       <c r="M65" s="4" t="n">
-        <v>85.98</v>
+        <v>84.58</v>
       </c>
       <c r="N65" s="21">
         <f>SUM(E65:M65)</f>
@@ -45281,7 +45281,7 @@
         <v>35.4</v>
       </c>
       <c r="M67" s="4" t="n">
-        <v>50.16</v>
+        <v>49.43</v>
       </c>
       <c r="N67" s="21">
         <f>SUM(E67:M67)</f>
@@ -45383,7 +45383,7 @@
         <v>35.4</v>
       </c>
       <c r="M69" s="4" t="n">
-        <v>44.5</v>
+        <v>43.83</v>
       </c>
       <c r="N69" s="21">
         <f>SUM(E69:M69)</f>
@@ -45587,7 +45587,7 @@
         <v>35.4</v>
       </c>
       <c r="M73" s="4" t="n">
-        <v>44.28</v>
+        <v>43.62</v>
       </c>
       <c r="N73" s="21">
         <f>SUM(E73:M73)</f>
@@ -45689,7 +45689,7 @@
         <v>35.4</v>
       </c>
       <c r="M75" s="4" t="n">
-        <v>44.18</v>
+        <v>43.52</v>
       </c>
       <c r="N75" s="21">
         <f>SUM(E75:M75)</f>
@@ -45791,7 +45791,7 @@
         <v>35.4</v>
       </c>
       <c r="M77" s="4" t="n">
-        <v>54</v>
+        <v>53.55</v>
       </c>
       <c r="N77" s="21">
         <f>SUM(E77:M77)</f>
@@ -45995,7 +45995,7 @@
         <v>35.4</v>
       </c>
       <c r="M81" s="4" t="n">
-        <v>44.79</v>
+        <v>44.42</v>
       </c>
       <c r="N81" s="21">
         <f>SUM(E81:M81)</f>
@@ -46097,7 +46097,7 @@
         <v>35.4</v>
       </c>
       <c r="M83" s="4" t="n">
-        <v>53.7</v>
+        <v>53.26</v>
       </c>
       <c r="N83" s="21">
         <f>SUM(E83:M83)</f>
@@ -46199,7 +46199,7 @@
         <v>35.4</v>
       </c>
       <c r="M85" s="4" t="n">
-        <v>57.57</v>
+        <v>57.1</v>
       </c>
       <c r="N85" s="21">
         <f>SUM(E85:M85)</f>
@@ -46301,7 +46301,7 @@
         <v>35.4</v>
       </c>
       <c r="M87" s="4" t="n">
-        <v>32.3</v>
+        <v>55.6</v>
       </c>
       <c r="N87" s="21">
         <f>SUM(E87:M87)</f>
@@ -46505,7 +46505,7 @@
         <v>35.4</v>
       </c>
       <c r="M91" s="4" t="n">
-        <v>274.29</v>
+        <v>273.06</v>
       </c>
       <c r="N91" s="21">
         <f>SUM(E91:M91)</f>
@@ -46607,7 +46607,7 @@
         <v>35.4</v>
       </c>
       <c r="M93" s="4" t="n">
-        <v>274.37</v>
+        <v>273.13</v>
       </c>
       <c r="N93" s="21">
         <f>SUM(E93:M93)</f>
@@ -46709,7 +46709,7 @@
         <v>35.4</v>
       </c>
       <c r="M95" s="4" t="n">
-        <v>276.11</v>
+        <v>274.86</v>
       </c>
       <c r="N95" s="21">
         <f>SUM(E95:M95)</f>
@@ -46811,7 +46811,7 @@
         <v>35.4</v>
       </c>
       <c r="M97" s="4" t="n">
-        <v>96.89</v>
+        <v>96.45</v>
       </c>
       <c r="N97" s="21">
         <f>SUM(E97:M97)</f>
@@ -47015,7 +47015,7 @@
         <v>35.4</v>
       </c>
       <c r="M101" s="4" t="n">
-        <v>91.62</v>
+        <v>91.20999999999999</v>
       </c>
       <c r="N101" s="21">
         <f>SUM(E101:M101)</f>
@@ -47117,7 +47117,7 @@
         <v>35.4</v>
       </c>
       <c r="M103" s="4" t="n">
-        <v>91.48</v>
+        <v>91.06999999999999</v>
       </c>
       <c r="N103" s="21">
         <f>SUM(E103:M103)</f>
@@ -47270,7 +47270,7 @@
         <v>35.4</v>
       </c>
       <c r="M106" s="4" t="n">
-        <v>91.73</v>
+        <v>91.31</v>
       </c>
       <c r="N106" s="21">
         <f>SUM(E106:M106)</f>
@@ -47678,7 +47678,7 @@
         <v>35.4</v>
       </c>
       <c r="M114" s="4" t="n">
-        <v>90.59</v>
+        <v>90.2</v>
       </c>
       <c r="N114" s="21">
         <f>SUM(E114:M114)</f>
@@ -47780,7 +47780,7 @@
         <v>35.4</v>
       </c>
       <c r="M116" s="4" t="n">
-        <v>78.42</v>
+        <v>78.06</v>
       </c>
       <c r="N116" s="21">
         <f>SUM(E116:M116)</f>
@@ -47984,7 +47984,7 @@
         <v>35.4</v>
       </c>
       <c r="M120" s="4" t="n">
-        <v>72.37</v>
+        <v>72.03</v>
       </c>
       <c r="N120" s="21">
         <f>SUM(E120:M120)</f>
@@ -48086,7 +48086,7 @@
         <v>35.4</v>
       </c>
       <c r="M122" s="4" t="n">
-        <v>109.08</v>
+        <v>108.59</v>
       </c>
       <c r="N122" s="21">
         <f>SUM(E122:M122)</f>
@@ -48290,7 +48290,7 @@
         <v>35.4</v>
       </c>
       <c r="M126" s="4" t="n">
-        <v>70.45</v>
+        <v>70.18000000000001</v>
       </c>
       <c r="N126" s="21">
         <f>SUM(E126:M126)</f>
@@ -48392,7 +48392,7 @@
         <v>35.4</v>
       </c>
       <c r="M128" s="4" t="n">
-        <v>58.71</v>
+        <v>58.45</v>
       </c>
       <c r="N128" s="21">
         <f>SUM(E128:M128)</f>
@@ -48494,7 +48494,7 @@
         <v>35.4</v>
       </c>
       <c r="M130" s="4" t="n">
-        <v>114.05</v>
+        <v>113.54</v>
       </c>
       <c r="N130" s="21">
         <f>SUM(E130:M130)</f>
@@ -48596,7 +48596,7 @@
         <v>35.4</v>
       </c>
       <c r="M132" s="4" t="n">
-        <v>113.91</v>
+        <v>113.39</v>
       </c>
       <c r="N132" s="21">
         <f>SUM(E132:M132)</f>
@@ -48698,7 +48698,7 @@
         <v>35.4</v>
       </c>
       <c r="M134" s="4" t="n">
-        <v>128.29</v>
+        <v>127.79</v>
       </c>
       <c r="N134" s="21">
         <f>SUM(E134:M134)</f>
@@ -48800,7 +48800,7 @@
         <v>35.4</v>
       </c>
       <c r="M136" s="4" t="n">
-        <v>113.42</v>
+        <v>112.91</v>
       </c>
       <c r="N136" s="21">
         <f>SUM(E136:M136)</f>
@@ -48902,7 +48902,7 @@
         <v>35.4</v>
       </c>
       <c r="M138" s="4" t="n">
-        <v>112.35</v>
+        <v>111.85</v>
       </c>
       <c r="N138" s="21">
         <f>SUM(E138:M138)</f>
@@ -49004,7 +49004,7 @@
         <v>35.4</v>
       </c>
       <c r="M140" s="4" t="n">
-        <v>178.46</v>
+        <v>177.66</v>
       </c>
       <c r="N140" s="21">
         <f>SUM(E140:M140)</f>
@@ -49208,7 +49208,7 @@
         <v>35.4</v>
       </c>
       <c r="M144" s="4" t="n">
-        <v>176.82</v>
+        <v>176.02</v>
       </c>
       <c r="N144" s="21">
         <f>SUM(E144:M144)</f>
@@ -49310,7 +49310,7 @@
         <v>35.4</v>
       </c>
       <c r="M146" s="4" t="n">
-        <v>186.47</v>
+        <v>185.77</v>
       </c>
       <c r="N146" s="21">
         <f>SUM(E146:M146)</f>
@@ -49412,7 +49412,7 @@
         <v>35.4</v>
       </c>
       <c r="M148" s="4" t="n">
-        <v>171.28</v>
+        <v>170.57</v>
       </c>
       <c r="N148" s="21">
         <f>SUM(E148:M148)</f>
@@ -49514,7 +49514,7 @@
         <v>35.4</v>
       </c>
       <c r="M150" s="4" t="n">
-        <v>148.23</v>
+        <v>147.56</v>
       </c>
       <c r="N150" s="21">
         <f>SUM(E150:M150)</f>
@@ -49718,7 +49718,7 @@
         <v>35.4</v>
       </c>
       <c r="M154" s="4" t="n">
-        <v>184.36</v>
+        <v>183.68</v>
       </c>
       <c r="N154" s="21">
         <f>SUM(E154:M154)</f>
@@ -49820,7 +49820,7 @@
         <v>35.4</v>
       </c>
       <c r="M156" s="4" t="n">
-        <v>57.45</v>
+        <v>56.66</v>
       </c>
       <c r="N156" s="21">
         <f>SUM(E156:M156)</f>
@@ -49922,7 +49922,7 @@
         <v>35.4</v>
       </c>
       <c r="M158" s="4" t="n">
-        <v>57.7</v>
+        <v>56.91</v>
       </c>
       <c r="N158" s="21">
         <f>SUM(E158:M158)</f>
@@ -50024,7 +50024,7 @@
         <v>35.4</v>
       </c>
       <c r="M160" s="4" t="n">
-        <v>53.25</v>
+        <v>52.51</v>
       </c>
       <c r="N160" s="21">
         <f>SUM(E160:M160)</f>
@@ -50126,7 +50126,7 @@
         <v>35.4</v>
       </c>
       <c r="M162" s="4" t="n">
-        <v>52.99</v>
+        <v>52.26</v>
       </c>
       <c r="N162" s="21">
         <f>SUM(E162:M162)</f>
@@ -50228,7 +50228,7 @@
         <v>35.4</v>
       </c>
       <c r="M164" s="4" t="n">
-        <v>44.14</v>
+        <v>43.53</v>
       </c>
       <c r="N164" s="21">
         <f>SUM(E164:M164)</f>
@@ -50330,7 +50330,7 @@
         <v>35.4</v>
       </c>
       <c r="M166" s="4" t="n">
-        <v>60.59</v>
+        <v>59.77</v>
       </c>
       <c r="N166" s="21">
         <f>SUM(E166:M166)</f>
@@ -50432,7 +50432,7 @@
         <v>35.4</v>
       </c>
       <c r="M168" s="4" t="n">
-        <v>68.23</v>
+        <v>67.29000000000001</v>
       </c>
       <c r="N168" s="21">
         <f>SUM(E168:M168)</f>
@@ -50534,7 +50534,7 @@
         <v>35.4</v>
       </c>
       <c r="M170" s="4" t="n">
-        <v>79.79000000000001</v>
+        <v>78.69</v>
       </c>
       <c r="N170" s="21">
         <f>SUM(E170:M170)</f>
@@ -50738,7 +50738,7 @@
         <v>35.4</v>
       </c>
       <c r="M174" s="4" t="n">
-        <v>136.53</v>
+        <v>134.74</v>
       </c>
       <c r="N174" s="21">
         <f>SUM(E174:M174)</f>
@@ -50840,7 +50840,7 @@
         <v>35.4</v>
       </c>
       <c r="M176" s="4" t="n">
-        <v>126.91</v>
+        <v>125.16</v>
       </c>
       <c r="N176" s="21">
         <f>SUM(E176:M176)</f>
@@ -50942,7 +50942,7 @@
         <v>35.4</v>
       </c>
       <c r="M178" s="4" t="n">
-        <v>137.95</v>
+        <v>136.05</v>
       </c>
       <c r="N178" s="21">
         <f>SUM(E178:M178)</f>
@@ -51044,7 +51044,7 @@
         <v>35.4</v>
       </c>
       <c r="M180" s="4" t="n">
-        <v>127.41</v>
+        <v>125.66</v>
       </c>
       <c r="N180" s="21">
         <f>SUM(E180:M180)</f>
@@ -51146,7 +51146,7 @@
         <v>35.4</v>
       </c>
       <c r="M182" s="4" t="n">
-        <v>29.36</v>
+        <v>28.95</v>
       </c>
       <c r="N182" s="21">
         <f>SUM(E182:M182)</f>
@@ -51350,7 +51350,7 @@
         <v>35.4</v>
       </c>
       <c r="M186" s="4" t="n">
-        <v>30.1</v>
+        <v>29.68</v>
       </c>
       <c r="N186" s="21">
         <f>SUM(E186:M186)</f>
@@ -51452,7 +51452,7 @@
         <v>35.4</v>
       </c>
       <c r="M188" s="4" t="n">
-        <v>18.05</v>
+        <v>17.81</v>
       </c>
       <c r="N188" s="21">
         <f>SUM(E188:M188)</f>
@@ -51554,7 +51554,7 @@
         <v>35.4</v>
       </c>
       <c r="M190" s="4" t="n">
-        <v>10.62</v>
+        <v>10.47</v>
       </c>
       <c r="N190" s="21">
         <f>SUM(E190:M190)</f>
@@ -51656,7 +51656,7 @@
         <v>35.4</v>
       </c>
       <c r="M192" s="4" t="n">
-        <v>30.23</v>
+        <v>29.83</v>
       </c>
       <c r="N192" s="21">
         <f>SUM(E192:M192)</f>
@@ -51758,7 +51758,7 @@
         <v>35.4</v>
       </c>
       <c r="M194" s="4" t="n">
-        <v>31.89</v>
+        <v>31.45</v>
       </c>
       <c r="N194" s="21">
         <f>SUM(E194:M194)</f>
@@ -51860,7 +51860,7 @@
         <v>35.4</v>
       </c>
       <c r="M196" s="4" t="n">
-        <v>56.47</v>
+        <v>55.7</v>
       </c>
       <c r="N196" s="21">
         <f>SUM(E196:M196)</f>
@@ -51962,7 +51962,7 @@
         <v>35.4</v>
       </c>
       <c r="M198" s="4" t="n">
-        <v>60.26</v>
+        <v>59.33</v>
       </c>
       <c r="N198" s="21">
         <f>SUM(E198:M198)</f>
@@ -52064,7 +52064,7 @@
         <v>35.4</v>
       </c>
       <c r="M200" s="4" t="n">
-        <v>31.89</v>
+        <v>52.42</v>
       </c>
       <c r="N200" s="21">
         <f>SUM(E200:M200)</f>
@@ -52166,7 +52166,7 @@
         <v>35.4</v>
       </c>
       <c r="M202" s="4" t="n">
-        <v>53.13</v>
+        <v>52.4</v>
       </c>
       <c r="N202" s="21">
         <f>SUM(E202:M202)</f>
@@ -52268,7 +52268,7 @@
         <v>35.4</v>
       </c>
       <c r="M204" s="4" t="n">
-        <v>56.4</v>
+        <v>55.64</v>
       </c>
       <c r="N204" s="21">
         <f>SUM(E204:M204)</f>
@@ -52370,7 +52370,7 @@
         <v>35.4</v>
       </c>
       <c r="M206" s="4" t="n">
-        <v>17.68</v>
+        <v>17.44</v>
       </c>
       <c r="N206" s="21">
         <f>SUM(E206:M206)</f>
@@ -52472,7 +52472,7 @@
         <v>35.4</v>
       </c>
       <c r="M208" s="4" t="n">
-        <v>10.62</v>
+        <v>10.48</v>
       </c>
       <c r="N208" s="21">
         <f>SUM(E208:M208)</f>
@@ -52676,7 +52676,7 @@
         <v>35.4</v>
       </c>
       <c r="M212" s="4" t="n">
-        <v>10.56</v>
+        <v>10.41</v>
       </c>
       <c r="N212" s="21">
         <f>SUM(E212:M212)</f>
@@ -52778,7 +52778,7 @@
         <v>35.4</v>
       </c>
       <c r="M214" s="4" t="n">
-        <v>14.72</v>
+        <v>14.52</v>
       </c>
       <c r="N214" s="21">
         <f>SUM(E214:M214)</f>
@@ -52880,7 +52880,7 @@
         <v>35.4</v>
       </c>
       <c r="M216" s="4" t="n">
-        <v>10.59</v>
+        <v>10.44</v>
       </c>
       <c r="N216" s="21">
         <f>SUM(E216:M216)</f>
@@ -52982,7 +52982,7 @@
         <v>35.4</v>
       </c>
       <c r="M218" s="4" t="n">
-        <v>14.75</v>
+        <v>14.55</v>
       </c>
       <c r="N218" s="21">
         <f>SUM(E218:M218)</f>
@@ -53084,7 +53084,7 @@
         <v>35.4</v>
       </c>
       <c r="M220" s="4" t="n">
-        <v>17.5</v>
+        <v>17.26</v>
       </c>
       <c r="N220" s="21">
         <f>SUM(E220:M220)</f>
@@ -53186,7 +53186,7 @@
         <v>35.4</v>
       </c>
       <c r="M222" s="4" t="n">
-        <v>19.28</v>
+        <v>19.01</v>
       </c>
       <c r="N222" s="21">
         <f>SUM(E222:M222)</f>
@@ -53441,7 +53441,7 @@
         <v>35.4</v>
       </c>
       <c r="M227" s="4" t="n">
-        <v>53.98</v>
+        <v>54</v>
       </c>
       <c r="N227" s="21">
         <f>SUM(E227:M227)</f>
@@ -53645,7 +53645,7 @@
         <v>35.4</v>
       </c>
       <c r="M231" s="4" t="n">
-        <v>57.18</v>
+        <v>57.21</v>
       </c>
       <c r="N231" s="21">
         <f>SUM(E231:M231)</f>
@@ -54104,7 +54104,7 @@
         <v>35.4</v>
       </c>
       <c r="M240" s="4" t="n">
-        <v>62.96</v>
+        <v>62.99</v>
       </c>
       <c r="N240" s="21">
         <f>SUM(E240:M240)</f>
@@ -54257,7 +54257,7 @@
         <v>35.4</v>
       </c>
       <c r="M243" s="4" t="n">
-        <v>62.51</v>
+        <v>62.47</v>
       </c>
       <c r="N243" s="21">
         <f>SUM(E243:M243)</f>
@@ -54359,7 +54359,7 @@
         <v>35.4</v>
       </c>
       <c r="M245" s="4" t="n">
-        <v>51.27</v>
+        <v>36.92</v>
       </c>
       <c r="N245" s="21">
         <f>SUM(E245:M245)</f>
@@ -54410,7 +54410,7 @@
         <v>35.4</v>
       </c>
       <c r="M246" s="4" t="n">
-        <v>46.51</v>
+        <v>46.55</v>
       </c>
       <c r="N246" s="21">
         <f>SUM(E246:M246)</f>

</xml_diff>